<commit_message>
Improve output planning fallbacks and transfers
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Macro\SqlAnalyzerFormatter-feature\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85FAE87A-140A-4A9E-B9E7-38C137417D13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59EEC7B3-565F-457D-895E-E2B3A55614E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{41A826B0-B2A2-4DC8-9B04-8EFBE807DC37}"/>
   </bookViews>
@@ -902,18 +902,10 @@
     <phoneticPr fontId="3"/>
   </si>
   <si>
-    <t>@status</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
     <t>更新日時</t>
     <rPh sb="0" eb="4">
       <t>コウシンニチジ</t>
     </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>sysdatetime()</t>
     <phoneticPr fontId="3"/>
   </si>
   <si>
@@ -922,6 +914,12 @@
       <t>ジョウタイ</t>
     </rPh>
     <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>@status</t>
+  </si>
+  <si>
+    <t>sysdatetime()</t>
   </si>
 </sst>
 </file>
@@ -2059,9 +2057,7 @@
       <c r="P4" s="16"/>
       <c r="Q4" s="16"/>
       <c r="R4" s="16"/>
-      <c r="S4" s="55" t="s">
-        <v>184</v>
-      </c>
+      <c r="S4" s="55"/>
       <c r="T4" s="16"/>
       <c r="U4" s="16"/>
       <c r="V4" s="16"/>
@@ -2079,7 +2075,9 @@
       <c r="AH4" s="16"/>
       <c r="AI4" s="16"/>
       <c r="AJ4" s="16"/>
-      <c r="AK4" s="54"/>
+      <c r="AK4" s="54" t="s">
+        <v>186</v>
+      </c>
       <c r="AL4" s="16"/>
       <c r="AM4" s="16"/>
       <c r="AN4" s="16"/>
@@ -2136,7 +2134,7 @@
     </row>
     <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="23" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -2155,9 +2153,7 @@
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
       <c r="R5" s="1"/>
-      <c r="S5" s="23" t="s">
-        <v>186</v>
-      </c>
+      <c r="S5" s="23"/>
       <c r="T5" s="1"/>
       <c r="U5" s="1"/>
       <c r="V5" s="1"/>
@@ -2175,7 +2171,9 @@
       <c r="AH5" s="1"/>
       <c r="AI5" s="1"/>
       <c r="AJ5" s="1"/>
-      <c r="AK5" s="23"/>
+      <c r="AK5" s="23" t="s">
+        <v>187</v>
+      </c>
       <c r="AL5" s="1"/>
       <c r="AM5" s="1"/>
       <c r="AN5" s="1"/>
@@ -2440,7 +2438,7 @@
       <c r="O8" s="10"/>
       <c r="P8" s="10"/>
       <c r="Q8" s="10" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="R8" s="10"/>
       <c r="S8" s="16"/>

</xml_diff>

<commit_message>
feat: indent compound CASE conditions
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Macro\SqlAnalyzerFormatter-feature\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7990AA4-0BB3-4452-A0A2-2124EB6FA650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06717DE8-126A-42B7-982D-E9DE3F05EB86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="63" activeTab="69" xr2:uid="{41A826B0-B2A2-4DC8-9B04-8EFBE807DC37}"/>
   </bookViews>
@@ -99,7 +99,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1275" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1279" uniqueCount="279">
   <si>
     <t>ソートキー2</t>
   </si>
@@ -683,12 +683,6 @@
     <t>tb1.ユーザーID IN (SQ1)</t>
   </si>
   <si>
-    <t>AND tb1.削除日時 IS NULL → 1</t>
-  </si>
-  <si>
-    <t>AND tb1.作成日時 &gt;= DATEADD(day, -7, @base_date) → 1</t>
-  </si>
-  <si>
     <t>paid_amount</t>
   </si>
   <si>
@@ -717,9 +711,6 @@
   </si>
   <si>
     <t>tb1.削除日時 IS NULL</t>
-  </si>
-  <si>
-    <t>AND tb1.有効区分 = 1 → 'ACTIVE'</t>
   </si>
   <si>
     <t>それ以外 → 'INACTIVE'</t>
@@ -936,6 +927,15 @@
   </si>
   <si>
     <t>参照テーブル: ユーザー[tb1]、注文[tb2]、SQ1</t>
+  </si>
+  <si>
+    <t>tb1.削除日時 IS NULL → 1</t>
+  </si>
+  <si>
+    <t>tb1.作成日時 &gt;= DATEADD(day, -7, @base_date) → 1</t>
+  </si>
+  <si>
+    <t>tb1.有効区分 = 1 → 'ACTIVE'</t>
   </si>
 </sst>
 </file>
@@ -4786,7 +4786,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -5575,7 +5575,7 @@
     </row>
     <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="24" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -5689,7 +5689,7 @@
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
       <c r="Q6" s="25" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="R6" s="6"/>
       <c r="S6" s="6"/>
@@ -5879,7 +5879,7 @@
       <c r="O8" s="18"/>
       <c r="P8" s="18"/>
       <c r="Q8" s="29" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="R8" s="18"/>
       <c r="S8" s="18"/>
@@ -6178,7 +6178,7 @@
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -6274,7 +6274,7 @@
       <c r="O4" s="14"/>
       <c r="P4" s="14"/>
       <c r="Q4" s="30" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="R4" s="14"/>
       <c r="S4" s="14"/>
@@ -6461,7 +6461,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -6849,7 +6849,7 @@
     </row>
     <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="25" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -6965,7 +6965,7 @@
       </c>
       <c r="P7" s="6"/>
       <c r="Q7" s="25" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="R7" s="6"/>
       <c r="S7" s="6"/>
@@ -7063,7 +7063,7 @@
       </c>
       <c r="P8" s="3"/>
       <c r="Q8" s="27" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="R8" s="3"/>
       <c r="S8" s="3"/>
@@ -7159,7 +7159,7 @@
       <c r="O9" s="18"/>
       <c r="P9" s="18"/>
       <c r="Q9" s="29" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="R9" s="18"/>
       <c r="S9" s="18"/>
@@ -7252,7 +7252,7 @@
   <sheetData>
     <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="22" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7656,7 +7656,7 @@
       <c r="O5" s="18"/>
       <c r="P5" s="18"/>
       <c r="Q5" s="29" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="R5" s="18"/>
       <c r="S5" s="18"/>
@@ -7920,7 +7920,7 @@
     </row>
     <row r="8" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="22" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -8036,7 +8036,7 @@
       </c>
       <c r="P9" s="6"/>
       <c r="Q9" s="25" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="R9" s="6"/>
       <c r="S9" s="6"/>
@@ -8134,7 +8134,7 @@
       </c>
       <c r="P10" s="14"/>
       <c r="Q10" s="30" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="R10" s="14"/>
       <c r="S10" s="14"/>
@@ -8533,7 +8533,7 @@
       <c r="O4" s="18"/>
       <c r="P4" s="18"/>
       <c r="Q4" s="29" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="R4" s="18"/>
       <c r="S4" s="18"/>
@@ -9606,7 +9606,7 @@
       <c r="O5" s="6"/>
       <c r="P5" s="6"/>
       <c r="Q5" s="25" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="R5" s="6"/>
       <c r="S5" s="6"/>
@@ -9702,7 +9702,7 @@
       </c>
       <c r="P6" s="3"/>
       <c r="Q6" s="27" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="R6" s="3"/>
       <c r="S6" s="3"/>
@@ -9894,7 +9894,7 @@
       </c>
       <c r="P8" s="3"/>
       <c r="Q8" s="27" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="R8" s="3"/>
       <c r="S8" s="3"/>
@@ -9990,7 +9990,7 @@
       </c>
       <c r="P9" s="3"/>
       <c r="Q9" s="27" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="R9" s="3"/>
       <c r="S9" s="3"/>
@@ -11750,7 +11750,7 @@
       </c>
       <c r="P4" s="3"/>
       <c r="Q4" s="27" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
@@ -11769,7 +11769,7 @@
         <v>7</v>
       </c>
       <c r="AF4" s="27" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -12268,7 +12268,7 @@
         <v>7</v>
       </c>
       <c r="AF4" s="27" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -12449,7 +12449,7 @@
       <c r="O6" s="18"/>
       <c r="P6" s="18"/>
       <c r="Q6" s="29" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="R6" s="18"/>
       <c r="S6" s="18"/>
@@ -12869,7 +12869,7 @@
         <v>7</v>
       </c>
       <c r="AF4" s="27" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -19228,7 +19228,7 @@
       </c>
       <c r="P5" s="3"/>
       <c r="Q5" s="27" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
@@ -19612,7 +19612,7 @@
       <c r="O9" s="14"/>
       <c r="P9" s="14"/>
       <c r="Q9" s="30" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="R9" s="14"/>
       <c r="S9" s="14"/>
@@ -25497,7 +25497,7 @@
         <v>7</v>
       </c>
       <c r="AF4" s="27" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -25580,7 +25580,7 @@
       </c>
       <c r="P5" s="14"/>
       <c r="Q5" s="30" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="R5" s="14"/>
       <c r="S5" s="14"/>
@@ -25599,7 +25599,7 @@
         <v>7</v>
       </c>
       <c r="AF5" s="30" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="AG5" s="14"/>
       <c r="AH5" s="14"/>
@@ -25985,7 +25985,7 @@
       </c>
       <c r="P4" s="3"/>
       <c r="Q4" s="27" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
@@ -26004,7 +26004,7 @@
         <v>7</v>
       </c>
       <c r="AF4" s="27" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -26087,7 +26087,7 @@
       </c>
       <c r="P5" s="14"/>
       <c r="Q5" s="30" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="R5" s="14"/>
       <c r="S5" s="14"/>
@@ -26106,7 +26106,7 @@
         <v>7</v>
       </c>
       <c r="AF5" s="30" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="AG5" s="14"/>
       <c r="AH5" s="14"/>
@@ -26492,7 +26492,7 @@
       </c>
       <c r="P4" s="14"/>
       <c r="Q4" s="30" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="R4" s="14"/>
       <c r="S4" s="14"/>
@@ -26511,7 +26511,7 @@
         <v>7</v>
       </c>
       <c r="AF4" s="30" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="AG4" s="14"/>
       <c r="AH4" s="14"/>
@@ -26993,7 +26993,7 @@
       <c r="O5" s="18"/>
       <c r="P5" s="18"/>
       <c r="Q5" s="29" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="R5" s="18"/>
       <c r="S5" s="18"/>
@@ -27296,7 +27296,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -27315,7 +27315,7 @@
         <v>7</v>
       </c>
       <c r="AF3" s="25" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="AG3" s="6"/>
       <c r="AH3" s="6"/>
@@ -27701,7 +27701,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -27720,7 +27720,7 @@
         <v>7</v>
       </c>
       <c r="AF3" s="25" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="AG3" s="6"/>
       <c r="AH3" s="6"/>
@@ -28489,7 +28489,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -28801,7 +28801,7 @@
       </c>
       <c r="P5" s="3"/>
       <c r="Q5" s="27" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
@@ -28897,7 +28897,7 @@
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
       <c r="Q6" s="25" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="R6" s="6"/>
       <c r="S6" s="6"/>
@@ -28991,7 +28991,7 @@
       <c r="O7" s="14"/>
       <c r="P7" s="14"/>
       <c r="Q7" s="30" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="R7" s="14"/>
       <c r="S7" s="14"/>
@@ -29178,7 +29178,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -29392,7 +29392,7 @@
       </c>
       <c r="P4" s="3"/>
       <c r="Q4" s="27" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
@@ -29490,7 +29490,7 @@
       </c>
       <c r="P5" s="3"/>
       <c r="Q5" s="27" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
@@ -29586,7 +29586,7 @@
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
       <c r="Q6" s="25" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="R6" s="6"/>
       <c r="S6" s="6"/>
@@ -29774,7 +29774,7 @@
       <c r="O8" s="3"/>
       <c r="P8" s="3"/>
       <c r="Q8" s="27" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="R8" s="3"/>
       <c r="S8" s="3"/>
@@ -29868,7 +29868,7 @@
       <c r="O9" s="14"/>
       <c r="P9" s="14"/>
       <c r="Q9" s="30" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="R9" s="14"/>
       <c r="S9" s="14"/>
@@ -30367,7 +30367,7 @@
       </c>
       <c r="P5" s="3"/>
       <c r="Q5" s="27" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
@@ -31056,7 +31056,7 @@
       </c>
       <c r="P5" s="3"/>
       <c r="Q5" s="27" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
@@ -31152,7 +31152,7 @@
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
       <c r="Q6" s="25" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="R6" s="6"/>
       <c r="S6" s="6"/>
@@ -31845,7 +31845,7 @@
       </c>
       <c r="P6" s="14"/>
       <c r="Q6" s="30" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="R6" s="14"/>
       <c r="S6" s="14"/>
@@ -33344,7 +33344,7 @@
       <c r="O5" s="6"/>
       <c r="P5" s="6"/>
       <c r="Q5" s="25" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="R5" s="6"/>
       <c r="S5" s="6"/>
@@ -33440,7 +33440,7 @@
       <c r="O6" s="14"/>
       <c r="P6" s="14"/>
       <c r="Q6" s="30" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="R6" s="14"/>
       <c r="S6" s="14"/>
@@ -33937,7 +33937,7 @@
       <c r="O5" s="18"/>
       <c r="P5" s="18"/>
       <c r="Q5" s="29" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="R5" s="18"/>
       <c r="S5" s="18"/>
@@ -34525,7 +34525,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -35001,7 +35001,7 @@
     </row>
     <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="22" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -39503,11 +39503,11 @@
       <c r="AE6" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="AF6" s="25" t="s">
+      <c r="AF6" s="6"/>
+      <c r="AG6" s="6"/>
+      <c r="AH6" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="AG6" s="6"/>
-      <c r="AH6" s="6"/>
       <c r="AI6" s="6"/>
       <c r="AJ6" s="6"/>
       <c r="AK6" s="6"/>
@@ -39598,10 +39598,12 @@
       <c r="AD7" s="3"/>
       <c r="AE7" s="3"/>
       <c r="AF7" s="27" t="s">
-        <v>194</v>
+        <v>86</v>
       </c>
       <c r="AG7" s="3"/>
-      <c r="AH7" s="3"/>
+      <c r="AH7" s="27" t="s">
+        <v>276</v>
+      </c>
       <c r="AI7" s="3"/>
       <c r="AJ7" s="3"/>
       <c r="AK7" s="3"/>
@@ -39691,11 +39693,11 @@
       <c r="AC8" s="3"/>
       <c r="AD8" s="3"/>
       <c r="AE8" s="3"/>
-      <c r="AF8" s="27" t="s">
+      <c r="AF8" s="3"/>
+      <c r="AG8" s="3"/>
+      <c r="AH8" s="27" t="s">
         <v>132</v>
       </c>
-      <c r="AG8" s="3"/>
-      <c r="AH8" s="3"/>
       <c r="AI8" s="3"/>
       <c r="AJ8" s="3"/>
       <c r="AK8" s="3"/>
@@ -39786,10 +39788,12 @@
       <c r="AD9" s="3"/>
       <c r="AE9" s="3"/>
       <c r="AF9" s="27" t="s">
-        <v>195</v>
+        <v>86</v>
       </c>
       <c r="AG9" s="3"/>
-      <c r="AH9" s="3"/>
+      <c r="AH9" s="27" t="s">
+        <v>277</v>
+      </c>
       <c r="AI9" s="3"/>
       <c r="AJ9" s="3"/>
       <c r="AK9" s="3"/>
@@ -40168,7 +40172,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -40187,11 +40191,11 @@
         <v>7</v>
       </c>
       <c r="AF3" s="25" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="AG3" s="6"/>
       <c r="AH3" s="25" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="AI3" s="6"/>
       <c r="AJ3" s="6"/>
@@ -40571,7 +40575,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -40590,7 +40594,7 @@
         <v>7</v>
       </c>
       <c r="AF3" s="25" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="AG3" s="6"/>
       <c r="AH3" s="6"/>
@@ -40684,7 +40688,7 @@
       <c r="AD4" s="3"/>
       <c r="AE4" s="3"/>
       <c r="AF4" s="27" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -40780,7 +40784,7 @@
       <c r="AF5" s="3"/>
       <c r="AG5" s="3"/>
       <c r="AH5" s="27" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="AI5" s="3"/>
       <c r="AJ5" s="3"/>
@@ -40874,7 +40878,7 @@
       <c r="AF6" s="14"/>
       <c r="AG6" s="14"/>
       <c r="AH6" s="30" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="AI6" s="14"/>
       <c r="AJ6" s="14"/>
@@ -40942,7 +40946,7 @@
 <file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13E13F0B-BD68-436F-AC4B-0DE79A71FA29}">
   <sheetPr codeName="Sheet70"/>
-  <dimension ref="A1:CL5"/>
+  <dimension ref="A1:CL10"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="90" width="1.75" customWidth="1"/>
@@ -41160,7 +41164,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -41178,11 +41182,11 @@
       <c r="AE3" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="AF3" s="25" t="s">
+      <c r="AF3" s="6"/>
+      <c r="AG3" s="6"/>
+      <c r="AH3" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="AG3" s="6"/>
-      <c r="AH3" s="6"/>
       <c r="AI3" s="6"/>
       <c r="AJ3" s="6"/>
       <c r="AK3" s="6"/>
@@ -41273,10 +41277,12 @@
       <c r="AD4" s="3"/>
       <c r="AE4" s="3"/>
       <c r="AF4" s="27" t="s">
-        <v>194</v>
+        <v>86</v>
       </c>
       <c r="AG4" s="3"/>
-      <c r="AH4" s="3"/>
+      <c r="AH4" s="27" t="s">
+        <v>276</v>
+      </c>
       <c r="AI4" s="3"/>
       <c r="AJ4" s="3"/>
       <c r="AK4" s="3"/>
@@ -41428,6 +41434,11 @@
       <c r="CK5" s="14"/>
       <c r="CL5" s="15"/>
     </row>
+    <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="8" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="9" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="10" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -41437,7 +41448,7 @@
 <file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30AB51C2-4CAF-40D2-90C0-05BD312EBAB8}">
   <sheetPr codeName="Sheet71"/>
-  <dimension ref="A1:CL6"/>
+  <dimension ref="A1:CL10"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="90" width="1.75" customWidth="1"/>
@@ -41772,11 +41783,11 @@
         <v>7</v>
       </c>
       <c r="AJ4" s="14"/>
-      <c r="AK4" s="31" t="s">
-        <v>205</v>
-      </c>
+      <c r="AK4" s="13"/>
       <c r="AL4" s="14"/>
-      <c r="AM4" s="14"/>
+      <c r="AM4" s="30" t="s">
+        <v>203</v>
+      </c>
       <c r="AN4" s="14"/>
       <c r="AO4" s="14"/>
       <c r="AP4" s="14"/>
@@ -41867,10 +41878,12 @@
       <c r="AI5" s="18"/>
       <c r="AJ5" s="18"/>
       <c r="AK5" s="20" t="s">
-        <v>206</v>
+        <v>86</v>
       </c>
       <c r="AL5" s="18"/>
-      <c r="AM5" s="18"/>
+      <c r="AM5" s="29" t="s">
+        <v>278</v>
+      </c>
       <c r="AN5" s="18"/>
       <c r="AO5" s="18"/>
       <c r="AP5" s="18"/>
@@ -41961,7 +41974,7 @@
       <c r="AI6" s="18"/>
       <c r="AJ6" s="18"/>
       <c r="AK6" s="20" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="AL6" s="18"/>
       <c r="AM6" s="18"/>
@@ -42017,6 +42030,10 @@
       <c r="CK6" s="18"/>
       <c r="CL6" s="19"/>
     </row>
+    <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="8" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="9" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="10" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -42362,7 +42379,7 @@
       </c>
       <c r="AJ4" s="14"/>
       <c r="AK4" s="31" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="AL4" s="14"/>
       <c r="AM4" s="14"/>
@@ -42456,7 +42473,7 @@
       <c r="AI5" s="18"/>
       <c r="AJ5" s="18"/>
       <c r="AK5" s="20" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="AL5" s="18"/>
       <c r="AM5" s="18"/>
@@ -42739,7 +42756,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -42833,7 +42850,7 @@
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="27" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
@@ -43353,7 +43370,7 @@
         <v>7</v>
       </c>
       <c r="AF4" s="27" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -43436,7 +43453,7 @@
       </c>
       <c r="P5" s="3"/>
       <c r="Q5" s="27" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
@@ -43455,7 +43472,7 @@
         <v>7</v>
       </c>
       <c r="AF5" s="27" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="AG5" s="3"/>
       <c r="AH5" s="3"/>
@@ -43536,7 +43553,7 @@
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
       <c r="Q6" s="25" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="R6" s="6"/>
       <c r="S6" s="6"/>
@@ -43732,7 +43749,7 @@
       <c r="O8" s="18"/>
       <c r="P8" s="18"/>
       <c r="Q8" s="29" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="R8" s="18"/>
       <c r="S8" s="18"/>
@@ -44308,7 +44325,7 @@
       </c>
       <c r="P14" s="3"/>
       <c r="Q14" s="27" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="R14" s="3"/>
       <c r="S14" s="3"/>
@@ -44406,7 +44423,7 @@
       </c>
       <c r="P15" s="3"/>
       <c r="Q15" s="27" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="R15" s="3"/>
       <c r="S15" s="3"/>
@@ -44692,7 +44709,7 @@
       <c r="O18" s="3"/>
       <c r="P18" s="3"/>
       <c r="Q18" s="27" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="R18" s="3"/>
       <c r="S18" s="3"/>
@@ -44888,7 +44905,7 @@
       </c>
       <c r="P20" s="18"/>
       <c r="Q20" s="29" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="R20" s="18"/>
       <c r="S20" s="18"/>
@@ -46927,7 +46944,7 @@
     </row>
     <row r="21" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A21" s="22" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -48474,7 +48491,7 @@
     </row>
     <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="22" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -50521,7 +50538,7 @@
     </row>
     <row r="18" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="22" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -51974,7 +51991,7 @@
     </row>
     <row r="9" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="22" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -52698,7 +52715,7 @@
         <v>7</v>
       </c>
       <c r="AF3" s="25" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="AG3" s="6"/>
       <c r="AH3" s="6"/>
@@ -53066,7 +53083,7 @@
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="24" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
@@ -53080,7 +53097,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -53875,7 +53892,7 @@
       </c>
       <c r="P5" s="6"/>
       <c r="Q5" s="25" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="R5" s="6"/>
       <c r="S5" s="6"/>
@@ -53973,7 +53990,7 @@
       </c>
       <c r="R6" s="3"/>
       <c r="S6" s="27" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="T6" s="3"/>
       <c r="U6" s="3"/>
@@ -54263,7 +54280,7 @@
       </c>
       <c r="T9" s="3"/>
       <c r="U9" s="27" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="V9" s="3"/>
       <c r="W9" s="3"/>

</xml_diff>

<commit_message>
feat: align UPDATE CASE transfer layout
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Macro\SqlAnalyzerFormatter-feature\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06717DE8-126A-42B7-982D-E9DE3F05EB86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50AB106C-FE30-4410-8F28-9CD23F9819AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="63" activeTab="69" xr2:uid="{41A826B0-B2A2-4DC8-9B04-8EFBE807DC37}"/>
+    <workbookView xWindow="20370" yWindow="-8340" windowWidth="29040" windowHeight="15720" firstSheet="58" activeTab="59" xr2:uid="{41A826B0-B2A2-4DC8-9B04-8EFBE807DC37}"/>
   </bookViews>
   <sheets>
     <sheet name="SEL-064" sheetId="66" r:id="rId1"/>
@@ -76,12 +76,12 @@
     <sheet name="SEL-066" sheetId="68" r:id="rId61"/>
     <sheet name="SEL-067" sheetId="69" r:id="rId62"/>
     <sheet name="SEL-057" sheetId="70" r:id="rId63"/>
-    <sheet name="SEL-068" sheetId="71" r:id="rId64"/>
-    <sheet name="SEL-069" sheetId="72" r:id="rId65"/>
-    <sheet name="SEL-070" sheetId="73" r:id="rId66"/>
-    <sheet name="SEL-071" sheetId="74" r:id="rId67"/>
-    <sheet name="SEL-072" sheetId="75" r:id="rId68"/>
-    <sheet name="SEL-073" sheetId="76" r:id="rId69"/>
+    <sheet name="SEL-073" sheetId="76" r:id="rId64"/>
+    <sheet name="SEL-072" sheetId="75" r:id="rId65"/>
+    <sheet name="SEL-071" sheetId="74" r:id="rId66"/>
+    <sheet name="SEL-070" sheetId="73" r:id="rId67"/>
+    <sheet name="SEL-069" sheetId="72" r:id="rId68"/>
+    <sheet name="SEL-068" sheetId="71" r:id="rId69"/>
     <sheet name="SEL-061" sheetId="82" r:id="rId70"/>
     <sheet name="SEL-059" sheetId="81" r:id="rId71"/>
     <sheet name="SEL-056" sheetId="80" r:id="rId72"/>
@@ -942,7 +942,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -965,6 +965,21 @@
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="游ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="游ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -986,7 +1001,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -1111,13 +1126,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1221,6 +1245,39 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -39952,9 +40009,9 @@
 </file>
 
 <file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98123E36-DEC7-4BA3-914F-651666C56468}">
-  <sheetPr codeName="Sheet68"/>
-  <dimension ref="A1:CL4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{956EFD9A-0444-473E-BD83-6FED68498CDD}">
+  <sheetPr codeName="Sheet73"/>
+  <dimension ref="A1:CL5"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="90" width="1.75" customWidth="1"/>
@@ -40056,7 +40113,1958 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>2</v>
+        <v>21</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1"/>
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+      <c r="AC2" s="1"/>
+      <c r="AD2" s="1"/>
+      <c r="AE2" s="1"/>
+      <c r="AF2" s="1"/>
+      <c r="AG2" s="1"/>
+      <c r="AH2" s="1"/>
+      <c r="AI2" s="1"/>
+      <c r="AJ2" s="1"/>
+      <c r="AK2" s="1"/>
+      <c r="AL2" s="1"/>
+      <c r="AM2" s="1"/>
+      <c r="AN2" s="1"/>
+      <c r="AO2" s="1"/>
+      <c r="AP2" s="1"/>
+      <c r="AQ2" s="1"/>
+      <c r="AR2" s="1"/>
+      <c r="AS2" s="1"/>
+      <c r="AT2" s="1"/>
+      <c r="AU2" s="1"/>
+      <c r="AV2" s="1"/>
+      <c r="AW2" s="1"/>
+      <c r="AX2" s="1"/>
+      <c r="AY2" s="1"/>
+      <c r="AZ2" s="1"/>
+      <c r="BA2" s="1"/>
+      <c r="BB2" s="1"/>
+      <c r="BC2" s="1"/>
+      <c r="BD2" s="1"/>
+      <c r="BE2" s="1"/>
+      <c r="BF2" s="1"/>
+      <c r="BG2" s="1"/>
+      <c r="BH2" s="1"/>
+      <c r="BI2" s="1"/>
+      <c r="BJ2" s="1"/>
+      <c r="BK2" s="1"/>
+      <c r="BL2" s="1"/>
+      <c r="BM2" s="1"/>
+      <c r="BN2" s="1"/>
+      <c r="BO2" s="1"/>
+      <c r="BP2" s="1"/>
+      <c r="BQ2" s="1"/>
+      <c r="BR2" s="1"/>
+      <c r="BS2" s="1"/>
+      <c r="BT2" s="1"/>
+      <c r="BU2" s="1"/>
+      <c r="BV2" s="1"/>
+      <c r="BW2" s="1"/>
+      <c r="BX2" s="1"/>
+      <c r="BY2" s="1"/>
+      <c r="BZ2" s="1"/>
+      <c r="CA2" s="1"/>
+      <c r="CB2" s="1"/>
+      <c r="CC2" s="1"/>
+      <c r="CD2" s="1"/>
+      <c r="CE2" s="1"/>
+      <c r="CF2" s="1"/>
+      <c r="CG2" s="1"/>
+      <c r="CH2" s="1"/>
+      <c r="CI2" s="1"/>
+      <c r="CJ2" s="1"/>
+      <c r="CK2" s="1"/>
+      <c r="CL2" s="1"/>
+    </row>
+    <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="25" t="s">
+        <v>206</v>
+      </c>
+      <c r="R3" s="6"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
+      <c r="AA3" s="6"/>
+      <c r="AB3" s="6"/>
+      <c r="AC3" s="6"/>
+      <c r="AD3" s="6"/>
+      <c r="AE3" s="6"/>
+      <c r="AF3" s="6"/>
+      <c r="AG3" s="6"/>
+      <c r="AH3" s="6"/>
+      <c r="AI3" s="6"/>
+      <c r="AJ3" s="6"/>
+      <c r="AK3" s="6"/>
+      <c r="AL3" s="6"/>
+      <c r="AM3" s="6"/>
+      <c r="AN3" s="6"/>
+      <c r="AO3" s="6"/>
+      <c r="AP3" s="6"/>
+      <c r="AQ3" s="6"/>
+      <c r="AR3" s="6"/>
+      <c r="AS3" s="6"/>
+      <c r="AT3" s="6"/>
+      <c r="AU3" s="6"/>
+      <c r="AV3" s="6"/>
+      <c r="AW3" s="6"/>
+      <c r="AX3" s="6"/>
+      <c r="AY3" s="6"/>
+      <c r="AZ3" s="6"/>
+      <c r="BA3" s="6"/>
+      <c r="BB3" s="6"/>
+      <c r="BC3" s="6"/>
+      <c r="BD3" s="6"/>
+      <c r="BE3" s="6"/>
+      <c r="BF3" s="6"/>
+      <c r="BG3" s="6"/>
+      <c r="BH3" s="6"/>
+      <c r="BI3" s="6"/>
+      <c r="BJ3" s="6"/>
+      <c r="BK3" s="6"/>
+      <c r="BL3" s="6"/>
+      <c r="BM3" s="6"/>
+      <c r="BN3" s="6"/>
+      <c r="BO3" s="6"/>
+      <c r="BP3" s="6"/>
+      <c r="BQ3" s="6"/>
+      <c r="BR3" s="6"/>
+      <c r="BS3" s="6"/>
+      <c r="BT3" s="6"/>
+      <c r="BU3" s="6"/>
+      <c r="BV3" s="6"/>
+      <c r="BW3" s="6"/>
+      <c r="BX3" s="6"/>
+      <c r="BY3" s="6"/>
+      <c r="BZ3" s="6"/>
+      <c r="CA3" s="6"/>
+      <c r="CB3" s="6"/>
+      <c r="CC3" s="6"/>
+      <c r="CD3" s="6"/>
+      <c r="CE3" s="6"/>
+      <c r="CF3" s="6"/>
+      <c r="CG3" s="6"/>
+      <c r="CH3" s="6"/>
+      <c r="CI3" s="6"/>
+      <c r="CJ3" s="6"/>
+      <c r="CK3" s="6"/>
+      <c r="CL3" s="7"/>
+    </row>
+    <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="8"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="27" t="s">
+        <v>207</v>
+      </c>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="Y4" s="3"/>
+      <c r="Z4" s="3"/>
+      <c r="AA4" s="3"/>
+      <c r="AB4" s="3"/>
+      <c r="AC4" s="3"/>
+      <c r="AD4" s="3"/>
+      <c r="AE4" s="3"/>
+      <c r="AF4" s="3"/>
+      <c r="AG4" s="3"/>
+      <c r="AH4" s="3"/>
+      <c r="AI4" s="3"/>
+      <c r="AJ4" s="3"/>
+      <c r="AK4" s="3"/>
+      <c r="AL4" s="3"/>
+      <c r="AM4" s="3"/>
+      <c r="AN4" s="3"/>
+      <c r="AO4" s="3"/>
+      <c r="AP4" s="3"/>
+      <c r="AQ4" s="3"/>
+      <c r="AR4" s="3"/>
+      <c r="AS4" s="3"/>
+      <c r="AT4" s="3"/>
+      <c r="AU4" s="3"/>
+      <c r="AV4" s="3"/>
+      <c r="AW4" s="3"/>
+      <c r="AX4" s="3"/>
+      <c r="AY4" s="3"/>
+      <c r="AZ4" s="3"/>
+      <c r="BA4" s="3"/>
+      <c r="BB4" s="3"/>
+      <c r="BC4" s="3"/>
+      <c r="BD4" s="3"/>
+      <c r="BE4" s="3"/>
+      <c r="BF4" s="3"/>
+      <c r="BG4" s="3"/>
+      <c r="BH4" s="3"/>
+      <c r="BI4" s="3"/>
+      <c r="BJ4" s="3"/>
+      <c r="BK4" s="3"/>
+      <c r="BL4" s="3"/>
+      <c r="BM4" s="3"/>
+      <c r="BN4" s="3"/>
+      <c r="BO4" s="3"/>
+      <c r="BP4" s="3"/>
+      <c r="BQ4" s="3"/>
+      <c r="BR4" s="3"/>
+      <c r="BS4" s="3"/>
+      <c r="BT4" s="3"/>
+      <c r="BU4" s="3"/>
+      <c r="BV4" s="3"/>
+      <c r="BW4" s="3"/>
+      <c r="BX4" s="3"/>
+      <c r="BY4" s="3"/>
+      <c r="BZ4" s="3"/>
+      <c r="CA4" s="3"/>
+      <c r="CB4" s="3"/>
+      <c r="CC4" s="3"/>
+      <c r="CD4" s="3"/>
+      <c r="CE4" s="3"/>
+      <c r="CF4" s="3"/>
+      <c r="CG4" s="3"/>
+      <c r="CH4" s="3"/>
+      <c r="CI4" s="3"/>
+      <c r="CJ4" s="3"/>
+      <c r="CK4" s="3"/>
+      <c r="CL4" s="10"/>
+    </row>
+    <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="H5" s="18"/>
+      <c r="I5" s="18"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="18"/>
+      <c r="M5" s="18"/>
+      <c r="N5" s="18"/>
+      <c r="O5" s="29" t="s">
+        <v>5</v>
+      </c>
+      <c r="P5" s="18"/>
+      <c r="Q5" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="R5" s="18"/>
+      <c r="S5" s="18"/>
+      <c r="T5" s="18"/>
+      <c r="U5" s="18"/>
+      <c r="V5" s="18"/>
+      <c r="W5" s="18"/>
+      <c r="X5" s="18"/>
+      <c r="Y5" s="18"/>
+      <c r="Z5" s="18"/>
+      <c r="AA5" s="18"/>
+      <c r="AB5" s="18"/>
+      <c r="AC5" s="18"/>
+      <c r="AD5" s="18"/>
+      <c r="AE5" s="18"/>
+      <c r="AF5" s="18"/>
+      <c r="AG5" s="18"/>
+      <c r="AH5" s="18"/>
+      <c r="AI5" s="18"/>
+      <c r="AJ5" s="18"/>
+      <c r="AK5" s="18"/>
+      <c r="AL5" s="18"/>
+      <c r="AM5" s="18"/>
+      <c r="AN5" s="18"/>
+      <c r="AO5" s="18"/>
+      <c r="AP5" s="18"/>
+      <c r="AQ5" s="18"/>
+      <c r="AR5" s="18"/>
+      <c r="AS5" s="18"/>
+      <c r="AT5" s="18"/>
+      <c r="AU5" s="18"/>
+      <c r="AV5" s="18"/>
+      <c r="AW5" s="18"/>
+      <c r="AX5" s="18"/>
+      <c r="AY5" s="18"/>
+      <c r="AZ5" s="18"/>
+      <c r="BA5" s="18"/>
+      <c r="BB5" s="18"/>
+      <c r="BC5" s="18"/>
+      <c r="BD5" s="18"/>
+      <c r="BE5" s="18"/>
+      <c r="BF5" s="18"/>
+      <c r="BG5" s="18"/>
+      <c r="BH5" s="18"/>
+      <c r="BI5" s="18"/>
+      <c r="BJ5" s="18"/>
+      <c r="BK5" s="18"/>
+      <c r="BL5" s="18"/>
+      <c r="BM5" s="18"/>
+      <c r="BN5" s="18"/>
+      <c r="BO5" s="18"/>
+      <c r="BP5" s="18"/>
+      <c r="BQ5" s="18"/>
+      <c r="BR5" s="18"/>
+      <c r="BS5" s="18"/>
+      <c r="BT5" s="18"/>
+      <c r="BU5" s="18"/>
+      <c r="BV5" s="18"/>
+      <c r="BW5" s="18"/>
+      <c r="BX5" s="18"/>
+      <c r="BY5" s="18"/>
+      <c r="BZ5" s="18"/>
+      <c r="CA5" s="18"/>
+      <c r="CB5" s="18"/>
+      <c r="CC5" s="18"/>
+      <c r="CD5" s="18"/>
+      <c r="CE5" s="18"/>
+      <c r="CF5" s="18"/>
+      <c r="CG5" s="18"/>
+      <c r="CH5" s="18"/>
+      <c r="CI5" s="18"/>
+      <c r="CJ5" s="18"/>
+      <c r="CK5" s="18"/>
+      <c r="CL5" s="19"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A2358E7-8911-407D-AA94-1AF2EC7340FC}">
+  <sheetPr codeName="Sheet72"/>
+  <dimension ref="A1:CL5"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="90" width="1.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
+      <c r="AH1" s="1"/>
+      <c r="AI1" s="1"/>
+      <c r="AJ1" s="1"/>
+      <c r="AK1" s="1"/>
+      <c r="AL1" s="1"/>
+      <c r="AM1" s="1"/>
+      <c r="AN1" s="1"/>
+      <c r="AO1" s="1"/>
+      <c r="AP1" s="1"/>
+      <c r="AQ1" s="1"/>
+      <c r="AR1" s="1"/>
+      <c r="AS1" s="1"/>
+      <c r="AT1" s="1"/>
+      <c r="AU1" s="1"/>
+      <c r="AV1" s="1"/>
+      <c r="AW1" s="1"/>
+      <c r="AX1" s="1"/>
+      <c r="AY1" s="1"/>
+      <c r="AZ1" s="1"/>
+      <c r="BA1" s="1"/>
+      <c r="BB1" s="1"/>
+      <c r="BC1" s="1"/>
+      <c r="BD1" s="1"/>
+      <c r="BE1" s="1"/>
+      <c r="BF1" s="1"/>
+      <c r="BG1" s="1"/>
+      <c r="BH1" s="1"/>
+      <c r="BI1" s="1"/>
+      <c r="BJ1" s="1"/>
+      <c r="BK1" s="1"/>
+      <c r="BL1" s="1"/>
+      <c r="BM1" s="1"/>
+      <c r="BN1" s="1"/>
+      <c r="BO1" s="1"/>
+      <c r="BP1" s="1"/>
+      <c r="BQ1" s="1"/>
+      <c r="BR1" s="1"/>
+      <c r="BS1" s="1"/>
+      <c r="BT1" s="1"/>
+      <c r="BU1" s="1"/>
+      <c r="BV1" s="1"/>
+      <c r="BW1" s="1"/>
+      <c r="BX1" s="1"/>
+      <c r="BY1" s="1"/>
+      <c r="BZ1" s="1"/>
+      <c r="CA1" s="1"/>
+      <c r="CB1" s="1"/>
+      <c r="CC1" s="1"/>
+      <c r="CD1" s="1"/>
+      <c r="CE1" s="1"/>
+      <c r="CF1" s="1"/>
+      <c r="CG1" s="1"/>
+      <c r="CH1" s="1"/>
+      <c r="CI1" s="1"/>
+      <c r="CJ1" s="1"/>
+      <c r="CK1" s="1"/>
+      <c r="CL1" s="1"/>
+    </row>
+    <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1"/>
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+      <c r="AC2" s="1"/>
+      <c r="AD2" s="1"/>
+      <c r="AE2" s="1"/>
+      <c r="AF2" s="1"/>
+      <c r="AG2" s="1"/>
+      <c r="AH2" s="1"/>
+      <c r="AI2" s="1"/>
+      <c r="AJ2" s="1"/>
+      <c r="AK2" s="1"/>
+      <c r="AL2" s="1"/>
+      <c r="AM2" s="1"/>
+      <c r="AN2" s="1"/>
+      <c r="AO2" s="1"/>
+      <c r="AP2" s="1"/>
+      <c r="AQ2" s="1"/>
+      <c r="AR2" s="1"/>
+      <c r="AS2" s="1"/>
+      <c r="AT2" s="1"/>
+      <c r="AU2" s="1"/>
+      <c r="AV2" s="1"/>
+      <c r="AW2" s="1"/>
+      <c r="AX2" s="1"/>
+      <c r="AY2" s="1"/>
+      <c r="AZ2" s="1"/>
+      <c r="BA2" s="1"/>
+      <c r="BB2" s="1"/>
+      <c r="BC2" s="1"/>
+      <c r="BD2" s="1"/>
+      <c r="BE2" s="1"/>
+      <c r="BF2" s="1"/>
+      <c r="BG2" s="1"/>
+      <c r="BH2" s="1"/>
+      <c r="BI2" s="1"/>
+      <c r="BJ2" s="1"/>
+      <c r="BK2" s="1"/>
+      <c r="BL2" s="1"/>
+      <c r="BM2" s="1"/>
+      <c r="BN2" s="1"/>
+      <c r="BO2" s="1"/>
+      <c r="BP2" s="1"/>
+      <c r="BQ2" s="1"/>
+      <c r="BR2" s="1"/>
+      <c r="BS2" s="1"/>
+      <c r="BT2" s="1"/>
+      <c r="BU2" s="1"/>
+      <c r="BV2" s="1"/>
+      <c r="BW2" s="1"/>
+      <c r="BX2" s="1"/>
+      <c r="BY2" s="1"/>
+      <c r="BZ2" s="1"/>
+      <c r="CA2" s="1"/>
+      <c r="CB2" s="1"/>
+      <c r="CC2" s="1"/>
+      <c r="CD2" s="1"/>
+      <c r="CE2" s="1"/>
+      <c r="CF2" s="1"/>
+      <c r="CG2" s="1"/>
+      <c r="CH2" s="1"/>
+      <c r="CI2" s="1"/>
+      <c r="CJ2" s="1"/>
+      <c r="CK2" s="1"/>
+      <c r="CL2" s="1"/>
+    </row>
+    <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="28" t="s">
+        <v>91</v>
+      </c>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="16"/>
+      <c r="N3" s="16"/>
+      <c r="O3" s="16"/>
+      <c r="P3" s="16"/>
+      <c r="Q3" s="16"/>
+      <c r="R3" s="16"/>
+      <c r="S3" s="28" t="s">
+        <v>92</v>
+      </c>
+      <c r="T3" s="16"/>
+      <c r="U3" s="16"/>
+      <c r="V3" s="16"/>
+      <c r="W3" s="16"/>
+      <c r="X3" s="16"/>
+      <c r="Y3" s="16"/>
+      <c r="Z3" s="16"/>
+      <c r="AA3" s="16"/>
+      <c r="AB3" s="16"/>
+      <c r="AC3" s="16"/>
+      <c r="AD3" s="16"/>
+      <c r="AE3" s="16"/>
+      <c r="AF3" s="16"/>
+      <c r="AG3" s="16"/>
+      <c r="AH3" s="16"/>
+      <c r="AI3" s="16"/>
+      <c r="AJ3" s="16"/>
+      <c r="AK3" s="28" t="s">
+        <v>93</v>
+      </c>
+      <c r="AL3" s="16"/>
+      <c r="AM3" s="16"/>
+      <c r="AN3" s="16"/>
+      <c r="AO3" s="16"/>
+      <c r="AP3" s="16"/>
+      <c r="AQ3" s="16"/>
+      <c r="AR3" s="16"/>
+      <c r="AS3" s="16"/>
+      <c r="AT3" s="16"/>
+      <c r="AU3" s="16"/>
+      <c r="AV3" s="16"/>
+      <c r="AW3" s="16"/>
+      <c r="AX3" s="16"/>
+      <c r="AY3" s="16"/>
+      <c r="AZ3" s="16"/>
+      <c r="BA3" s="16"/>
+      <c r="BB3" s="16"/>
+      <c r="BC3" s="16"/>
+      <c r="BD3" s="16"/>
+      <c r="BE3" s="16"/>
+      <c r="BF3" s="16"/>
+      <c r="BG3" s="16"/>
+      <c r="BH3" s="16"/>
+      <c r="BI3" s="16"/>
+      <c r="BJ3" s="16"/>
+      <c r="BK3" s="16"/>
+      <c r="BL3" s="16"/>
+      <c r="BM3" s="16"/>
+      <c r="BN3" s="16"/>
+      <c r="BO3" s="16"/>
+      <c r="BP3" s="16"/>
+      <c r="BQ3" s="16"/>
+      <c r="BR3" s="16"/>
+      <c r="BS3" s="16"/>
+      <c r="BT3" s="16"/>
+      <c r="BU3" s="16"/>
+      <c r="BV3" s="16"/>
+      <c r="BW3" s="16"/>
+      <c r="BX3" s="16"/>
+      <c r="BY3" s="16"/>
+      <c r="BZ3" s="16"/>
+      <c r="CA3" s="16"/>
+      <c r="CB3" s="16"/>
+      <c r="CC3" s="16"/>
+      <c r="CD3" s="16"/>
+      <c r="CE3" s="16"/>
+      <c r="CF3" s="16"/>
+      <c r="CG3" s="16"/>
+      <c r="CH3" s="16"/>
+      <c r="CI3" s="16"/>
+      <c r="CJ3" s="16"/>
+      <c r="CK3" s="16"/>
+      <c r="CL3" s="21"/>
+    </row>
+    <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="31" t="s">
+        <v>159</v>
+      </c>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14"/>
+      <c r="K4" s="14"/>
+      <c r="L4" s="14"/>
+      <c r="M4" s="14"/>
+      <c r="N4" s="14"/>
+      <c r="O4" s="14"/>
+      <c r="P4" s="14"/>
+      <c r="Q4" s="14"/>
+      <c r="R4" s="14"/>
+      <c r="S4" s="31" t="s">
+        <v>124</v>
+      </c>
+      <c r="T4" s="14"/>
+      <c r="U4" s="14"/>
+      <c r="V4" s="14"/>
+      <c r="W4" s="14"/>
+      <c r="X4" s="14"/>
+      <c r="Y4" s="14"/>
+      <c r="Z4" s="14"/>
+      <c r="AA4" s="14"/>
+      <c r="AB4" s="14"/>
+      <c r="AC4" s="14"/>
+      <c r="AD4" s="14"/>
+      <c r="AE4" s="14"/>
+      <c r="AF4" s="14"/>
+      <c r="AG4" s="14"/>
+      <c r="AH4" s="14"/>
+      <c r="AI4" s="30" t="s">
+        <v>7</v>
+      </c>
+      <c r="AJ4" s="14"/>
+      <c r="AK4" s="31" t="s">
+        <v>205</v>
+      </c>
+      <c r="AL4" s="14"/>
+      <c r="AM4" s="14"/>
+      <c r="AN4" s="14"/>
+      <c r="AO4" s="14"/>
+      <c r="AP4" s="14"/>
+      <c r="AQ4" s="14"/>
+      <c r="AR4" s="14"/>
+      <c r="AS4" s="14"/>
+      <c r="AT4" s="14"/>
+      <c r="AU4" s="14"/>
+      <c r="AV4" s="14"/>
+      <c r="AW4" s="14"/>
+      <c r="AX4" s="14"/>
+      <c r="AY4" s="14"/>
+      <c r="AZ4" s="14"/>
+      <c r="BA4" s="14"/>
+      <c r="BB4" s="14"/>
+      <c r="BC4" s="14"/>
+      <c r="BD4" s="14"/>
+      <c r="BE4" s="14"/>
+      <c r="BF4" s="14"/>
+      <c r="BG4" s="14"/>
+      <c r="BH4" s="14"/>
+      <c r="BI4" s="14"/>
+      <c r="BJ4" s="14"/>
+      <c r="BK4" s="14"/>
+      <c r="BL4" s="14"/>
+      <c r="BM4" s="14"/>
+      <c r="BN4" s="14"/>
+      <c r="BO4" s="14"/>
+      <c r="BP4" s="14"/>
+      <c r="BQ4" s="14"/>
+      <c r="BR4" s="14"/>
+      <c r="BS4" s="14"/>
+      <c r="BT4" s="14"/>
+      <c r="BU4" s="14"/>
+      <c r="BV4" s="14"/>
+      <c r="BW4" s="14"/>
+      <c r="BX4" s="14"/>
+      <c r="BY4" s="14"/>
+      <c r="BZ4" s="14"/>
+      <c r="CA4" s="14"/>
+      <c r="CB4" s="14"/>
+      <c r="CC4" s="14"/>
+      <c r="CD4" s="14"/>
+      <c r="CE4" s="14"/>
+      <c r="CF4" s="14"/>
+      <c r="CG4" s="14"/>
+      <c r="CH4" s="14"/>
+      <c r="CI4" s="14"/>
+      <c r="CJ4" s="14"/>
+      <c r="CK4" s="14"/>
+      <c r="CL4" s="15"/>
+    </row>
+    <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="17"/>
+      <c r="B5" s="18"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="18"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="18"/>
+      <c r="M5" s="18"/>
+      <c r="N5" s="18"/>
+      <c r="O5" s="18"/>
+      <c r="P5" s="18"/>
+      <c r="Q5" s="18"/>
+      <c r="R5" s="18"/>
+      <c r="S5" s="17"/>
+      <c r="T5" s="18"/>
+      <c r="U5" s="18"/>
+      <c r="V5" s="18"/>
+      <c r="W5" s="18"/>
+      <c r="X5" s="18"/>
+      <c r="Y5" s="18"/>
+      <c r="Z5" s="18"/>
+      <c r="AA5" s="18"/>
+      <c r="AB5" s="18"/>
+      <c r="AC5" s="18"/>
+      <c r="AD5" s="18"/>
+      <c r="AE5" s="18"/>
+      <c r="AF5" s="18"/>
+      <c r="AG5" s="18"/>
+      <c r="AH5" s="18"/>
+      <c r="AI5" s="18"/>
+      <c r="AJ5" s="18"/>
+      <c r="AK5" s="20" t="s">
+        <v>204</v>
+      </c>
+      <c r="AL5" s="18"/>
+      <c r="AM5" s="18"/>
+      <c r="AN5" s="18"/>
+      <c r="AO5" s="18"/>
+      <c r="AP5" s="18"/>
+      <c r="AQ5" s="18"/>
+      <c r="AR5" s="18"/>
+      <c r="AS5" s="18"/>
+      <c r="AT5" s="18"/>
+      <c r="AU5" s="18"/>
+      <c r="AV5" s="18"/>
+      <c r="AW5" s="18"/>
+      <c r="AX5" s="18"/>
+      <c r="AY5" s="18"/>
+      <c r="AZ5" s="18"/>
+      <c r="BA5" s="18"/>
+      <c r="BB5" s="18"/>
+      <c r="BC5" s="18"/>
+      <c r="BD5" s="18"/>
+      <c r="BE5" s="18"/>
+      <c r="BF5" s="18"/>
+      <c r="BG5" s="18"/>
+      <c r="BH5" s="18"/>
+      <c r="BI5" s="18"/>
+      <c r="BJ5" s="18"/>
+      <c r="BK5" s="18"/>
+      <c r="BL5" s="18"/>
+      <c r="BM5" s="18"/>
+      <c r="BN5" s="18"/>
+      <c r="BO5" s="18"/>
+      <c r="BP5" s="18"/>
+      <c r="BQ5" s="18"/>
+      <c r="BR5" s="18"/>
+      <c r="BS5" s="18"/>
+      <c r="BT5" s="18"/>
+      <c r="BU5" s="18"/>
+      <c r="BV5" s="18"/>
+      <c r="BW5" s="18"/>
+      <c r="BX5" s="18"/>
+      <c r="BY5" s="18"/>
+      <c r="BZ5" s="18"/>
+      <c r="CA5" s="18"/>
+      <c r="CB5" s="18"/>
+      <c r="CC5" s="18"/>
+      <c r="CD5" s="18"/>
+      <c r="CE5" s="18"/>
+      <c r="CF5" s="18"/>
+      <c r="CG5" s="18"/>
+      <c r="CH5" s="18"/>
+      <c r="CI5" s="18"/>
+      <c r="CJ5" s="18"/>
+      <c r="CK5" s="18"/>
+      <c r="CL5" s="19"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30AB51C2-4CAF-40D2-90C0-05BD312EBAB8}">
+  <sheetPr codeName="Sheet71"/>
+  <dimension ref="A1:CL10"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="90" width="1.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
+      <c r="AH1" s="1"/>
+      <c r="AI1" s="1"/>
+      <c r="AJ1" s="1"/>
+      <c r="AK1" s="1"/>
+      <c r="AL1" s="1"/>
+      <c r="AM1" s="1"/>
+      <c r="AN1" s="1"/>
+      <c r="AO1" s="1"/>
+      <c r="AP1" s="1"/>
+      <c r="AQ1" s="1"/>
+      <c r="AR1" s="1"/>
+      <c r="AS1" s="1"/>
+      <c r="AT1" s="1"/>
+      <c r="AU1" s="1"/>
+      <c r="AV1" s="1"/>
+      <c r="AW1" s="1"/>
+      <c r="AX1" s="1"/>
+      <c r="AY1" s="1"/>
+      <c r="AZ1" s="1"/>
+      <c r="BA1" s="1"/>
+      <c r="BB1" s="1"/>
+      <c r="BC1" s="1"/>
+      <c r="BD1" s="1"/>
+      <c r="BE1" s="1"/>
+      <c r="BF1" s="1"/>
+      <c r="BG1" s="1"/>
+      <c r="BH1" s="1"/>
+      <c r="BI1" s="1"/>
+      <c r="BJ1" s="1"/>
+      <c r="BK1" s="1"/>
+      <c r="BL1" s="1"/>
+      <c r="BM1" s="1"/>
+      <c r="BN1" s="1"/>
+      <c r="BO1" s="1"/>
+      <c r="BP1" s="1"/>
+      <c r="BQ1" s="1"/>
+      <c r="BR1" s="1"/>
+      <c r="BS1" s="1"/>
+      <c r="BT1" s="1"/>
+      <c r="BU1" s="1"/>
+      <c r="BV1" s="1"/>
+      <c r="BW1" s="1"/>
+      <c r="BX1" s="1"/>
+      <c r="BY1" s="1"/>
+      <c r="BZ1" s="1"/>
+      <c r="CA1" s="1"/>
+      <c r="CB1" s="1"/>
+      <c r="CC1" s="1"/>
+      <c r="CD1" s="1"/>
+      <c r="CE1" s="1"/>
+      <c r="CF1" s="1"/>
+      <c r="CG1" s="1"/>
+      <c r="CH1" s="1"/>
+      <c r="CI1" s="1"/>
+      <c r="CJ1" s="1"/>
+      <c r="CK1" s="1"/>
+      <c r="CL1" s="1"/>
+    </row>
+    <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1"/>
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+      <c r="AC2" s="1"/>
+      <c r="AD2" s="1"/>
+      <c r="AE2" s="1"/>
+      <c r="AF2" s="1"/>
+      <c r="AG2" s="1"/>
+      <c r="AH2" s="1"/>
+      <c r="AI2" s="1"/>
+      <c r="AJ2" s="1"/>
+      <c r="AK2" s="1"/>
+      <c r="AL2" s="1"/>
+      <c r="AM2" s="1"/>
+      <c r="AN2" s="1"/>
+      <c r="AO2" s="1"/>
+      <c r="AP2" s="1"/>
+      <c r="AQ2" s="1"/>
+      <c r="AR2" s="1"/>
+      <c r="AS2" s="1"/>
+      <c r="AT2" s="1"/>
+      <c r="AU2" s="1"/>
+      <c r="AV2" s="1"/>
+      <c r="AW2" s="1"/>
+      <c r="AX2" s="1"/>
+      <c r="AY2" s="1"/>
+      <c r="AZ2" s="1"/>
+      <c r="BA2" s="1"/>
+      <c r="BB2" s="1"/>
+      <c r="BC2" s="1"/>
+      <c r="BD2" s="1"/>
+      <c r="BE2" s="1"/>
+      <c r="BF2" s="1"/>
+      <c r="BG2" s="1"/>
+      <c r="BH2" s="1"/>
+      <c r="BI2" s="1"/>
+      <c r="BJ2" s="1"/>
+      <c r="BK2" s="1"/>
+      <c r="BL2" s="1"/>
+      <c r="BM2" s="1"/>
+      <c r="BN2" s="1"/>
+      <c r="BO2" s="1"/>
+      <c r="BP2" s="1"/>
+      <c r="BQ2" s="1"/>
+      <c r="BR2" s="1"/>
+      <c r="BS2" s="1"/>
+      <c r="BT2" s="1"/>
+      <c r="BU2" s="1"/>
+      <c r="BV2" s="1"/>
+      <c r="BW2" s="1"/>
+      <c r="BX2" s="1"/>
+      <c r="BY2" s="1"/>
+      <c r="BZ2" s="1"/>
+      <c r="CA2" s="1"/>
+      <c r="CB2" s="1"/>
+      <c r="CC2" s="1"/>
+      <c r="CD2" s="1"/>
+      <c r="CE2" s="1"/>
+      <c r="CF2" s="1"/>
+      <c r="CG2" s="1"/>
+      <c r="CH2" s="1"/>
+      <c r="CI2" s="1"/>
+      <c r="CJ2" s="1"/>
+      <c r="CK2" s="1"/>
+      <c r="CL2" s="1"/>
+    </row>
+    <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="28" t="s">
+        <v>91</v>
+      </c>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="16"/>
+      <c r="N3" s="16"/>
+      <c r="O3" s="16"/>
+      <c r="P3" s="16"/>
+      <c r="Q3" s="16"/>
+      <c r="R3" s="16"/>
+      <c r="S3" s="28" t="s">
+        <v>92</v>
+      </c>
+      <c r="T3" s="16"/>
+      <c r="U3" s="16"/>
+      <c r="V3" s="16"/>
+      <c r="W3" s="16"/>
+      <c r="X3" s="16"/>
+      <c r="Y3" s="16"/>
+      <c r="Z3" s="16"/>
+      <c r="AA3" s="16"/>
+      <c r="AB3" s="16"/>
+      <c r="AC3" s="16"/>
+      <c r="AD3" s="16"/>
+      <c r="AE3" s="16"/>
+      <c r="AF3" s="16"/>
+      <c r="AG3" s="16"/>
+      <c r="AH3" s="16"/>
+      <c r="AI3" s="16"/>
+      <c r="AJ3" s="16"/>
+      <c r="AK3" s="28" t="s">
+        <v>93</v>
+      </c>
+      <c r="AL3" s="16"/>
+      <c r="AM3" s="16"/>
+      <c r="AN3" s="16"/>
+      <c r="AO3" s="16"/>
+      <c r="AP3" s="16"/>
+      <c r="AQ3" s="16"/>
+      <c r="AR3" s="16"/>
+      <c r="AS3" s="16"/>
+      <c r="AT3" s="16"/>
+      <c r="AU3" s="16"/>
+      <c r="AV3" s="16"/>
+      <c r="AW3" s="16"/>
+      <c r="AX3" s="16"/>
+      <c r="AY3" s="16"/>
+      <c r="AZ3" s="16"/>
+      <c r="BA3" s="16"/>
+      <c r="BB3" s="16"/>
+      <c r="BC3" s="16"/>
+      <c r="BD3" s="16"/>
+      <c r="BE3" s="16"/>
+      <c r="BF3" s="16"/>
+      <c r="BG3" s="16"/>
+      <c r="BH3" s="16"/>
+      <c r="BI3" s="16"/>
+      <c r="BJ3" s="16"/>
+      <c r="BK3" s="16"/>
+      <c r="BL3" s="16"/>
+      <c r="BM3" s="16"/>
+      <c r="BN3" s="16"/>
+      <c r="BO3" s="16"/>
+      <c r="BP3" s="16"/>
+      <c r="BQ3" s="16"/>
+      <c r="BR3" s="16"/>
+      <c r="BS3" s="16"/>
+      <c r="BT3" s="16"/>
+      <c r="BU3" s="16"/>
+      <c r="BV3" s="16"/>
+      <c r="BW3" s="16"/>
+      <c r="BX3" s="16"/>
+      <c r="BY3" s="16"/>
+      <c r="BZ3" s="16"/>
+      <c r="CA3" s="16"/>
+      <c r="CB3" s="16"/>
+      <c r="CC3" s="16"/>
+      <c r="CD3" s="16"/>
+      <c r="CE3" s="16"/>
+      <c r="CF3" s="16"/>
+      <c r="CG3" s="16"/>
+      <c r="CH3" s="16"/>
+      <c r="CI3" s="16"/>
+      <c r="CJ3" s="16"/>
+      <c r="CK3" s="16"/>
+      <c r="CL3" s="21"/>
+    </row>
+    <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="35"/>
+      <c r="T4" s="6"/>
+      <c r="U4" s="6"/>
+      <c r="V4" s="6"/>
+      <c r="W4" s="6"/>
+      <c r="X4" s="6"/>
+      <c r="Y4" s="6"/>
+      <c r="Z4" s="6"/>
+      <c r="AA4" s="6"/>
+      <c r="AB4" s="6"/>
+      <c r="AC4" s="6"/>
+      <c r="AD4" s="6"/>
+      <c r="AE4" s="6"/>
+      <c r="AF4" s="6"/>
+      <c r="AG4" s="6"/>
+      <c r="AH4" s="6"/>
+      <c r="AI4" s="36"/>
+      <c r="AJ4" s="7"/>
+      <c r="AK4" s="27" t="s">
+        <v>124</v>
+      </c>
+      <c r="AL4" s="1"/>
+      <c r="AM4" s="1"/>
+      <c r="AN4" s="1"/>
+      <c r="AO4" s="1"/>
+      <c r="AP4" s="1"/>
+      <c r="AQ4" s="1"/>
+      <c r="AR4" s="1"/>
+      <c r="AS4" s="1"/>
+      <c r="AT4" s="1"/>
+      <c r="AU4" s="3"/>
+      <c r="AV4" s="3"/>
+      <c r="AW4" s="1"/>
+      <c r="AX4" s="1"/>
+      <c r="AY4" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="AZ4" s="3"/>
+      <c r="BA4" s="3"/>
+      <c r="BB4" s="27" t="s">
+        <v>203</v>
+      </c>
+      <c r="BC4" s="3"/>
+      <c r="BD4" s="3"/>
+      <c r="BE4" s="3"/>
+      <c r="BF4" s="3"/>
+      <c r="BG4" s="3"/>
+      <c r="BH4" s="3"/>
+      <c r="BI4" s="3"/>
+      <c r="BJ4" s="3"/>
+      <c r="BK4" s="3"/>
+      <c r="BL4" s="3"/>
+      <c r="BM4" s="3"/>
+      <c r="BN4" s="3"/>
+      <c r="BO4" s="3"/>
+      <c r="BP4" s="3"/>
+      <c r="BQ4" s="3"/>
+      <c r="BR4" s="3"/>
+      <c r="BS4" s="1"/>
+      <c r="BT4" s="1"/>
+      <c r="BU4" s="1"/>
+      <c r="BV4" s="1"/>
+      <c r="BW4" s="1"/>
+      <c r="BX4" s="1"/>
+      <c r="BY4" s="1"/>
+      <c r="BZ4" s="1"/>
+      <c r="CA4" s="1"/>
+      <c r="CB4" s="3"/>
+      <c r="CC4" s="3"/>
+      <c r="CD4" s="3"/>
+      <c r="CE4" s="3"/>
+      <c r="CF4" s="3"/>
+      <c r="CG4" s="3"/>
+      <c r="CH4" s="3"/>
+      <c r="CI4" s="3"/>
+      <c r="CJ4" s="3"/>
+      <c r="CK4" s="3"/>
+      <c r="CL4" s="10"/>
+    </row>
+    <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="9"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="9"/>
+      <c r="T5" s="3"/>
+      <c r="U5" s="3"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="3"/>
+      <c r="X5" s="3"/>
+      <c r="Y5" s="3"/>
+      <c r="Z5" s="3"/>
+      <c r="AA5" s="3"/>
+      <c r="AB5" s="3"/>
+      <c r="AC5" s="3"/>
+      <c r="AD5" s="3"/>
+      <c r="AE5" s="3"/>
+      <c r="AF5" s="3"/>
+      <c r="AG5" s="3"/>
+      <c r="AH5" s="3"/>
+      <c r="AI5" s="3"/>
+      <c r="AJ5" s="10"/>
+      <c r="AK5" s="37"/>
+      <c r="AL5" s="1"/>
+      <c r="AM5" s="1"/>
+      <c r="AN5" s="1"/>
+      <c r="AO5" s="1"/>
+      <c r="AP5" s="1"/>
+      <c r="AQ5" s="1"/>
+      <c r="AR5" s="1"/>
+      <c r="AS5" s="1"/>
+      <c r="AT5" s="1"/>
+      <c r="AU5" s="3"/>
+      <c r="AV5" s="3"/>
+      <c r="AW5" s="1"/>
+      <c r="AX5" s="1"/>
+      <c r="AY5" s="3"/>
+      <c r="AZ5" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="BA5" s="3"/>
+      <c r="BB5" s="27" t="s">
+        <v>278</v>
+      </c>
+      <c r="BC5" s="3"/>
+      <c r="BD5" s="3"/>
+      <c r="BE5" s="3"/>
+      <c r="BF5" s="3"/>
+      <c r="BG5" s="3"/>
+      <c r="BH5" s="3"/>
+      <c r="BI5" s="3"/>
+      <c r="BJ5" s="3"/>
+      <c r="BK5" s="3"/>
+      <c r="BL5" s="3"/>
+      <c r="BM5" s="3"/>
+      <c r="BN5" s="3"/>
+      <c r="BO5" s="3"/>
+      <c r="BP5" s="3"/>
+      <c r="BQ5" s="3"/>
+      <c r="BR5" s="3"/>
+      <c r="BS5" s="1"/>
+      <c r="BT5" s="1"/>
+      <c r="BU5" s="1"/>
+      <c r="BV5" s="1"/>
+      <c r="BW5" s="1"/>
+      <c r="BX5" s="1"/>
+      <c r="BY5" s="1"/>
+      <c r="BZ5" s="1"/>
+      <c r="CA5" s="1"/>
+      <c r="CB5" s="3"/>
+      <c r="CC5" s="3"/>
+      <c r="CD5" s="3"/>
+      <c r="CE5" s="3"/>
+      <c r="CF5" s="3"/>
+      <c r="CG5" s="3"/>
+      <c r="CH5" s="3"/>
+      <c r="CI5" s="3"/>
+      <c r="CJ5" s="3"/>
+      <c r="CK5" s="3"/>
+      <c r="CL5" s="10"/>
+    </row>
+    <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="13"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="14"/>
+      <c r="M6" s="14"/>
+      <c r="N6" s="14"/>
+      <c r="O6" s="14"/>
+      <c r="P6" s="14"/>
+      <c r="Q6" s="14"/>
+      <c r="R6" s="14"/>
+      <c r="S6" s="13"/>
+      <c r="T6" s="14"/>
+      <c r="U6" s="14"/>
+      <c r="V6" s="14"/>
+      <c r="W6" s="14"/>
+      <c r="X6" s="14"/>
+      <c r="Y6" s="14"/>
+      <c r="Z6" s="14"/>
+      <c r="AA6" s="14"/>
+      <c r="AB6" s="14"/>
+      <c r="AC6" s="14"/>
+      <c r="AD6" s="14"/>
+      <c r="AE6" s="14"/>
+      <c r="AF6" s="14"/>
+      <c r="AG6" s="14"/>
+      <c r="AH6" s="14"/>
+      <c r="AI6" s="14"/>
+      <c r="AJ6" s="15"/>
+      <c r="AK6" s="38"/>
+      <c r="AL6" s="39"/>
+      <c r="AM6" s="39"/>
+      <c r="AN6" s="39"/>
+      <c r="AO6" s="39"/>
+      <c r="AP6" s="39"/>
+      <c r="AQ6" s="39"/>
+      <c r="AR6" s="39"/>
+      <c r="AS6" s="39"/>
+      <c r="AT6" s="39"/>
+      <c r="AU6" s="40"/>
+      <c r="AV6" s="40"/>
+      <c r="AW6" s="41"/>
+      <c r="AX6" s="41"/>
+      <c r="AY6" s="40"/>
+      <c r="AZ6" s="42" t="s">
+        <v>204</v>
+      </c>
+      <c r="BA6" s="40"/>
+      <c r="BB6" s="40"/>
+      <c r="BC6" s="14"/>
+      <c r="BD6" s="14"/>
+      <c r="BE6" s="14"/>
+      <c r="BF6" s="14"/>
+      <c r="BG6" s="14"/>
+      <c r="BH6" s="14"/>
+      <c r="BI6" s="14"/>
+      <c r="BJ6" s="14"/>
+      <c r="BK6" s="14"/>
+      <c r="BL6" s="14"/>
+      <c r="BM6" s="14"/>
+      <c r="BN6" s="14"/>
+      <c r="BO6" s="14"/>
+      <c r="BP6" s="14"/>
+      <c r="BQ6" s="14"/>
+      <c r="BR6" s="14"/>
+      <c r="BS6" s="41"/>
+      <c r="BT6" s="41"/>
+      <c r="BU6" s="41"/>
+      <c r="BV6" s="41"/>
+      <c r="BW6" s="41"/>
+      <c r="BX6" s="41"/>
+      <c r="BY6" s="41"/>
+      <c r="BZ6" s="41"/>
+      <c r="CA6" s="41"/>
+      <c r="CB6" s="40"/>
+      <c r="CC6" s="40"/>
+      <c r="CD6" s="14"/>
+      <c r="CE6" s="14"/>
+      <c r="CF6" s="14"/>
+      <c r="CG6" s="14"/>
+      <c r="CH6" s="14"/>
+      <c r="CI6" s="14"/>
+      <c r="CJ6" s="14"/>
+      <c r="CK6" s="14"/>
+      <c r="CL6" s="15"/>
+    </row>
+    <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="43"/>
+      <c r="B7" s="43"/>
+      <c r="C7" s="43"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="43"/>
+      <c r="I7" s="43"/>
+      <c r="J7" s="43"/>
+      <c r="K7" s="43"/>
+      <c r="L7" s="43"/>
+      <c r="M7" s="43"/>
+      <c r="N7" s="43"/>
+      <c r="O7" s="43"/>
+      <c r="P7" s="43"/>
+      <c r="Q7" s="43"/>
+      <c r="R7" s="43"/>
+      <c r="S7" s="43"/>
+      <c r="T7" s="43"/>
+      <c r="U7" s="43"/>
+      <c r="V7" s="43"/>
+      <c r="W7" s="43"/>
+      <c r="X7" s="43"/>
+      <c r="Y7" s="43"/>
+      <c r="Z7" s="43"/>
+      <c r="AA7" s="43"/>
+      <c r="AB7" s="43"/>
+      <c r="AC7" s="43"/>
+      <c r="AD7" s="43"/>
+      <c r="AE7" s="43"/>
+      <c r="AF7" s="43"/>
+      <c r="AG7" s="43"/>
+      <c r="AH7" s="43"/>
+      <c r="AI7" s="43"/>
+      <c r="AJ7" s="43"/>
+      <c r="AK7" s="44"/>
+      <c r="AL7" s="45"/>
+      <c r="AM7" s="45"/>
+      <c r="AN7" s="45"/>
+      <c r="AO7" s="45"/>
+      <c r="AP7" s="45"/>
+      <c r="AQ7" s="45"/>
+      <c r="AR7" s="45"/>
+      <c r="AS7" s="45"/>
+      <c r="AT7" s="45"/>
+      <c r="AU7" s="45"/>
+      <c r="AV7" s="45"/>
+      <c r="AW7" s="45"/>
+      <c r="AX7" s="45"/>
+      <c r="AY7" s="44"/>
+      <c r="AZ7" s="44"/>
+      <c r="BA7" s="45"/>
+      <c r="BB7" s="43"/>
+      <c r="BC7" s="43"/>
+      <c r="BD7" s="43"/>
+      <c r="BE7" s="43"/>
+      <c r="BF7" s="43"/>
+      <c r="BG7" s="43"/>
+      <c r="BH7" s="43"/>
+      <c r="BI7" s="43"/>
+      <c r="BJ7" s="43"/>
+      <c r="BK7" s="43"/>
+      <c r="BL7" s="43"/>
+      <c r="BM7" s="43"/>
+      <c r="BN7" s="43"/>
+      <c r="BO7" s="43"/>
+      <c r="BP7" s="43"/>
+      <c r="BQ7" s="43"/>
+      <c r="BR7" s="43"/>
+      <c r="BS7" s="43"/>
+      <c r="BT7" s="43"/>
+      <c r="BU7" s="43"/>
+      <c r="BV7" s="43"/>
+      <c r="BW7" s="43"/>
+      <c r="BX7" s="43"/>
+      <c r="BY7" s="43"/>
+      <c r="BZ7" s="43"/>
+      <c r="CA7" s="43"/>
+      <c r="CB7" s="43"/>
+      <c r="CC7" s="43"/>
+      <c r="CD7" s="43"/>
+      <c r="CE7" s="43"/>
+      <c r="CF7" s="43"/>
+      <c r="CG7" s="43"/>
+      <c r="CH7" s="43"/>
+      <c r="CI7" s="43"/>
+      <c r="CJ7" s="43"/>
+      <c r="CK7" s="43"/>
+      <c r="CL7" s="43"/>
+    </row>
+    <row r="8" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="43"/>
+      <c r="B8" s="43"/>
+      <c r="C8" s="43"/>
+      <c r="D8" s="43"/>
+      <c r="E8" s="43"/>
+      <c r="F8" s="43"/>
+      <c r="G8" s="43"/>
+      <c r="H8" s="43"/>
+      <c r="I8" s="43"/>
+      <c r="J8" s="43"/>
+      <c r="K8" s="43"/>
+      <c r="L8" s="43"/>
+      <c r="M8" s="43"/>
+      <c r="N8" s="43"/>
+      <c r="O8" s="43"/>
+      <c r="P8" s="43"/>
+      <c r="Q8" s="43"/>
+      <c r="R8" s="43"/>
+      <c r="S8" s="43"/>
+      <c r="T8" s="43"/>
+      <c r="U8" s="43"/>
+      <c r="V8" s="43"/>
+      <c r="W8" s="43"/>
+      <c r="X8" s="43"/>
+      <c r="Y8" s="43"/>
+      <c r="Z8" s="43"/>
+      <c r="AA8" s="43"/>
+      <c r="AB8" s="43"/>
+      <c r="AC8" s="43"/>
+      <c r="AD8" s="43"/>
+      <c r="AE8" s="43"/>
+      <c r="AF8" s="43"/>
+      <c r="AG8" s="43"/>
+      <c r="AH8" s="43"/>
+      <c r="AI8" s="43"/>
+      <c r="AJ8" s="43"/>
+      <c r="AK8" s="43"/>
+      <c r="AL8" s="43"/>
+      <c r="AM8" s="43"/>
+      <c r="AN8" s="43"/>
+      <c r="AO8" s="43"/>
+      <c r="AP8" s="43"/>
+      <c r="AQ8" s="43"/>
+      <c r="AR8" s="43"/>
+      <c r="AS8" s="43"/>
+      <c r="AT8" s="43"/>
+      <c r="AU8" s="43"/>
+      <c r="AV8" s="43"/>
+      <c r="AW8" s="43"/>
+      <c r="AX8" s="43"/>
+      <c r="AY8" s="43"/>
+      <c r="AZ8" s="43"/>
+      <c r="BA8" s="43"/>
+      <c r="BB8" s="43"/>
+      <c r="BC8" s="43"/>
+      <c r="BD8" s="43"/>
+      <c r="BE8" s="43"/>
+      <c r="BF8" s="43"/>
+      <c r="BG8" s="43"/>
+      <c r="BH8" s="43"/>
+      <c r="BI8" s="43"/>
+      <c r="BJ8" s="43"/>
+      <c r="BK8" s="43"/>
+      <c r="BL8" s="43"/>
+      <c r="BM8" s="43"/>
+      <c r="BN8" s="43"/>
+      <c r="BO8" s="43"/>
+      <c r="BP8" s="43"/>
+      <c r="BQ8" s="43"/>
+      <c r="BR8" s="43"/>
+      <c r="BS8" s="43"/>
+      <c r="BT8" s="43"/>
+      <c r="BU8" s="43"/>
+      <c r="BV8" s="43"/>
+      <c r="BW8" s="43"/>
+      <c r="BX8" s="43"/>
+      <c r="BY8" s="43"/>
+      <c r="BZ8" s="43"/>
+      <c r="CA8" s="43"/>
+      <c r="CB8" s="43"/>
+      <c r="CC8" s="43"/>
+      <c r="CD8" s="43"/>
+      <c r="CE8" s="43"/>
+      <c r="CF8" s="43"/>
+      <c r="CG8" s="43"/>
+      <c r="CH8" s="43"/>
+      <c r="CI8" s="43"/>
+      <c r="CJ8" s="43"/>
+      <c r="CK8" s="43"/>
+      <c r="CL8" s="43"/>
+    </row>
+    <row r="9" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="43"/>
+      <c r="B9" s="43"/>
+      <c r="C9" s="43"/>
+      <c r="D9" s="43"/>
+      <c r="E9" s="43"/>
+      <c r="F9" s="43"/>
+      <c r="G9" s="43"/>
+      <c r="H9" s="43"/>
+      <c r="I9" s="43"/>
+      <c r="J9" s="43"/>
+      <c r="K9" s="43"/>
+      <c r="L9" s="43"/>
+      <c r="M9" s="43"/>
+      <c r="N9" s="43"/>
+      <c r="O9" s="43"/>
+      <c r="P9" s="43"/>
+      <c r="Q9" s="43"/>
+      <c r="R9" s="43"/>
+      <c r="S9" s="43"/>
+      <c r="T9" s="43"/>
+      <c r="U9" s="43"/>
+      <c r="V9" s="43"/>
+      <c r="W9" s="43"/>
+      <c r="X9" s="43"/>
+      <c r="Y9" s="43"/>
+      <c r="Z9" s="43"/>
+      <c r="AA9" s="43"/>
+      <c r="AB9" s="43"/>
+      <c r="AC9" s="43"/>
+      <c r="AD9" s="43"/>
+      <c r="AE9" s="43"/>
+      <c r="AF9" s="43"/>
+      <c r="AG9" s="43"/>
+      <c r="AH9" s="43"/>
+      <c r="AI9" s="43"/>
+      <c r="AJ9" s="43"/>
+      <c r="AK9" s="43"/>
+      <c r="AL9" s="43"/>
+      <c r="AM9" s="43"/>
+      <c r="AN9" s="43"/>
+      <c r="AO9" s="43"/>
+      <c r="AP9" s="43"/>
+      <c r="AQ9" s="43"/>
+      <c r="AR9" s="43"/>
+      <c r="AS9" s="43"/>
+      <c r="AT9" s="43"/>
+      <c r="AU9" s="43"/>
+      <c r="AV9" s="43"/>
+      <c r="AW9" s="43"/>
+      <c r="AX9" s="43"/>
+      <c r="AY9" s="43"/>
+      <c r="AZ9" s="43"/>
+      <c r="BA9" s="43"/>
+      <c r="BB9" s="43"/>
+      <c r="BC9" s="43"/>
+      <c r="BD9" s="43"/>
+      <c r="BE9" s="43"/>
+      <c r="BF9" s="43"/>
+      <c r="BG9" s="43"/>
+      <c r="BH9" s="43"/>
+      <c r="BI9" s="43"/>
+      <c r="BJ9" s="43"/>
+      <c r="BK9" s="43"/>
+      <c r="BL9" s="43"/>
+      <c r="BM9" s="43"/>
+      <c r="BN9" s="43"/>
+      <c r="BO9" s="43"/>
+      <c r="BP9" s="43"/>
+      <c r="BQ9" s="43"/>
+      <c r="BR9" s="43"/>
+      <c r="BS9" s="43"/>
+      <c r="BT9" s="43"/>
+      <c r="BU9" s="43"/>
+      <c r="BV9" s="43"/>
+      <c r="BW9" s="43"/>
+      <c r="BX9" s="43"/>
+      <c r="BY9" s="43"/>
+      <c r="BZ9" s="43"/>
+      <c r="CA9" s="43"/>
+      <c r="CB9" s="43"/>
+      <c r="CC9" s="43"/>
+      <c r="CD9" s="43"/>
+      <c r="CE9" s="43"/>
+      <c r="CF9" s="43"/>
+      <c r="CG9" s="43"/>
+      <c r="CH9" s="43"/>
+      <c r="CI9" s="43"/>
+      <c r="CJ9" s="43"/>
+      <c r="CK9" s="43"/>
+      <c r="CL9" s="43"/>
+    </row>
+    <row r="10" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="43"/>
+      <c r="B10" s="43"/>
+      <c r="C10" s="43"/>
+      <c r="D10" s="43"/>
+      <c r="E10" s="43"/>
+      <c r="F10" s="43"/>
+      <c r="G10" s="43"/>
+      <c r="H10" s="43"/>
+      <c r="I10" s="43"/>
+      <c r="J10" s="43"/>
+      <c r="K10" s="43"/>
+      <c r="L10" s="43"/>
+      <c r="M10" s="43"/>
+      <c r="N10" s="43"/>
+      <c r="O10" s="43"/>
+      <c r="P10" s="43"/>
+      <c r="Q10" s="43"/>
+      <c r="R10" s="43"/>
+      <c r="S10" s="43"/>
+      <c r="T10" s="43"/>
+      <c r="U10" s="43"/>
+      <c r="V10" s="43"/>
+      <c r="W10" s="43"/>
+      <c r="X10" s="43"/>
+      <c r="Y10" s="43"/>
+      <c r="Z10" s="43"/>
+      <c r="AA10" s="43"/>
+      <c r="AB10" s="43"/>
+      <c r="AC10" s="43"/>
+      <c r="AD10" s="43"/>
+      <c r="AE10" s="43"/>
+      <c r="AF10" s="43"/>
+      <c r="AG10" s="43"/>
+      <c r="AH10" s="43"/>
+      <c r="AI10" s="43"/>
+      <c r="AJ10" s="43"/>
+      <c r="AK10" s="43"/>
+      <c r="AL10" s="43"/>
+      <c r="AM10" s="43"/>
+      <c r="AN10" s="43"/>
+      <c r="AO10" s="43"/>
+      <c r="AP10" s="43"/>
+      <c r="AQ10" s="43"/>
+      <c r="AR10" s="43"/>
+      <c r="AS10" s="43"/>
+      <c r="AT10" s="43"/>
+      <c r="AU10" s="43"/>
+      <c r="AV10" s="43"/>
+      <c r="AW10" s="43"/>
+      <c r="AX10" s="43"/>
+      <c r="AY10" s="43"/>
+      <c r="AZ10" s="43"/>
+      <c r="BA10" s="43"/>
+      <c r="BB10" s="43"/>
+      <c r="BC10" s="43"/>
+      <c r="BD10" s="43"/>
+      <c r="BE10" s="43"/>
+      <c r="BF10" s="43"/>
+      <c r="BG10" s="43"/>
+      <c r="BH10" s="43"/>
+      <c r="BI10" s="43"/>
+      <c r="BJ10" s="43"/>
+      <c r="BK10" s="43"/>
+      <c r="BL10" s="43"/>
+      <c r="BM10" s="43"/>
+      <c r="BN10" s="43"/>
+      <c r="BO10" s="43"/>
+      <c r="BP10" s="43"/>
+      <c r="BQ10" s="43"/>
+      <c r="BR10" s="43"/>
+      <c r="BS10" s="43"/>
+      <c r="BT10" s="43"/>
+      <c r="BU10" s="43"/>
+      <c r="BV10" s="43"/>
+      <c r="BW10" s="43"/>
+      <c r="BX10" s="43"/>
+      <c r="BY10" s="43"/>
+      <c r="BZ10" s="43"/>
+      <c r="CA10" s="43"/>
+      <c r="CB10" s="43"/>
+      <c r="CC10" s="43"/>
+      <c r="CD10" s="43"/>
+      <c r="CE10" s="43"/>
+      <c r="CF10" s="43"/>
+      <c r="CG10" s="43"/>
+      <c r="CH10" s="43"/>
+      <c r="CI10" s="43"/>
+      <c r="CJ10" s="43"/>
+      <c r="CK10" s="43"/>
+      <c r="CL10" s="43"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13E13F0B-BD68-436F-AC4B-0DE79A71FA29}">
+  <sheetPr codeName="Sheet70"/>
+  <dimension ref="A1:CL10"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="90" width="1.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
+      <c r="AH1" s="1"/>
+      <c r="AI1" s="1"/>
+      <c r="AJ1" s="1"/>
+      <c r="AK1" s="1"/>
+      <c r="AL1" s="1"/>
+      <c r="AM1" s="1"/>
+      <c r="AN1" s="1"/>
+      <c r="AO1" s="1"/>
+      <c r="AP1" s="1"/>
+      <c r="AQ1" s="1"/>
+      <c r="AR1" s="1"/>
+      <c r="AS1" s="1"/>
+      <c r="AT1" s="1"/>
+      <c r="AU1" s="1"/>
+      <c r="AV1" s="1"/>
+      <c r="AW1" s="1"/>
+      <c r="AX1" s="1"/>
+      <c r="AY1" s="1"/>
+      <c r="AZ1" s="1"/>
+      <c r="BA1" s="1"/>
+      <c r="BB1" s="1"/>
+      <c r="BC1" s="1"/>
+      <c r="BD1" s="1"/>
+      <c r="BE1" s="1"/>
+      <c r="BF1" s="1"/>
+      <c r="BG1" s="1"/>
+      <c r="BH1" s="1"/>
+      <c r="BI1" s="1"/>
+      <c r="BJ1" s="1"/>
+      <c r="BK1" s="1"/>
+      <c r="BL1" s="1"/>
+      <c r="BM1" s="1"/>
+      <c r="BN1" s="1"/>
+      <c r="BO1" s="1"/>
+      <c r="BP1" s="1"/>
+      <c r="BQ1" s="1"/>
+      <c r="BR1" s="1"/>
+      <c r="BS1" s="1"/>
+      <c r="BT1" s="1"/>
+      <c r="BU1" s="1"/>
+      <c r="BV1" s="1"/>
+      <c r="BW1" s="1"/>
+      <c r="BX1" s="1"/>
+      <c r="BY1" s="1"/>
+      <c r="BZ1" s="1"/>
+      <c r="CA1" s="1"/>
+      <c r="CB1" s="1"/>
+      <c r="CC1" s="1"/>
+      <c r="CD1" s="1"/>
+      <c r="CE1" s="1"/>
+      <c r="CF1" s="1"/>
+      <c r="CG1" s="1"/>
+      <c r="CH1" s="1"/>
+      <c r="CI1" s="1"/>
+      <c r="CJ1" s="1"/>
+      <c r="CK1" s="1"/>
+      <c r="CL1" s="1"/>
+    </row>
+    <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="22" t="s">
+        <v>21</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -40172,7 +42180,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -40190,12 +42198,10 @@
       <c r="AE3" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="AF3" s="25" t="s">
-        <v>195</v>
-      </c>
+      <c r="AF3" s="6"/>
       <c r="AG3" s="6"/>
       <c r="AH3" s="25" t="s">
-        <v>196</v>
+        <v>80</v>
       </c>
       <c r="AI3" s="6"/>
       <c r="AJ3" s="6"/>
@@ -40255,106 +42261,207 @@
       <c r="CL3" s="7"/>
     </row>
     <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="11"/>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
-      <c r="L4" s="14"/>
-      <c r="M4" s="14"/>
-      <c r="N4" s="14"/>
-      <c r="O4" s="14"/>
-      <c r="P4" s="14"/>
-      <c r="Q4" s="14"/>
-      <c r="R4" s="14"/>
-      <c r="S4" s="14"/>
-      <c r="T4" s="14"/>
-      <c r="U4" s="14"/>
-      <c r="V4" s="14"/>
-      <c r="W4" s="14"/>
-      <c r="X4" s="14"/>
-      <c r="Y4" s="14"/>
-      <c r="Z4" s="14"/>
-      <c r="AA4" s="14"/>
-      <c r="AB4" s="14"/>
-      <c r="AC4" s="14"/>
-      <c r="AD4" s="14"/>
-      <c r="AE4" s="14"/>
-      <c r="AF4" s="14"/>
-      <c r="AG4" s="14"/>
-      <c r="AH4" s="30" t="s">
+      <c r="A4" s="8"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="Y4" s="3"/>
+      <c r="Z4" s="3"/>
+      <c r="AA4" s="3"/>
+      <c r="AB4" s="3"/>
+      <c r="AC4" s="3"/>
+      <c r="AD4" s="3"/>
+      <c r="AE4" s="3"/>
+      <c r="AF4" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="AG4" s="3"/>
+      <c r="AH4" s="27" t="s">
+        <v>276</v>
+      </c>
+      <c r="AI4" s="3"/>
+      <c r="AJ4" s="3"/>
+      <c r="AK4" s="3"/>
+      <c r="AL4" s="3"/>
+      <c r="AM4" s="3"/>
+      <c r="AN4" s="3"/>
+      <c r="AO4" s="3"/>
+      <c r="AP4" s="3"/>
+      <c r="AQ4" s="3"/>
+      <c r="AR4" s="3"/>
+      <c r="AS4" s="3"/>
+      <c r="AT4" s="3"/>
+      <c r="AU4" s="3"/>
+      <c r="AV4" s="3"/>
+      <c r="AW4" s="3"/>
+      <c r="AX4" s="3"/>
+      <c r="AY4" s="3"/>
+      <c r="AZ4" s="3"/>
+      <c r="BA4" s="3"/>
+      <c r="BB4" s="3"/>
+      <c r="BC4" s="3"/>
+      <c r="BD4" s="3"/>
+      <c r="BE4" s="3"/>
+      <c r="BF4" s="3"/>
+      <c r="BG4" s="3"/>
+      <c r="BH4" s="3"/>
+      <c r="BI4" s="3"/>
+      <c r="BJ4" s="3"/>
+      <c r="BK4" s="3"/>
+      <c r="BL4" s="3"/>
+      <c r="BM4" s="3"/>
+      <c r="BN4" s="3"/>
+      <c r="BO4" s="3"/>
+      <c r="BP4" s="3"/>
+      <c r="BQ4" s="3"/>
+      <c r="BR4" s="3"/>
+      <c r="BS4" s="3"/>
+      <c r="BT4" s="3"/>
+      <c r="BU4" s="3"/>
+      <c r="BV4" s="3"/>
+      <c r="BW4" s="3"/>
+      <c r="BX4" s="3"/>
+      <c r="BY4" s="3"/>
+      <c r="BZ4" s="3"/>
+      <c r="CA4" s="3"/>
+      <c r="CB4" s="3"/>
+      <c r="CC4" s="3"/>
+      <c r="CD4" s="3"/>
+      <c r="CE4" s="3"/>
+      <c r="CF4" s="3"/>
+      <c r="CG4" s="3"/>
+      <c r="CH4" s="3"/>
+      <c r="CI4" s="3"/>
+      <c r="CJ4" s="3"/>
+      <c r="CK4" s="3"/>
+      <c r="CL4" s="10"/>
+    </row>
+    <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="11"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="14"/>
+      <c r="L5" s="14"/>
+      <c r="M5" s="14"/>
+      <c r="N5" s="14"/>
+      <c r="O5" s="14"/>
+      <c r="P5" s="14"/>
+      <c r="Q5" s="14"/>
+      <c r="R5" s="14"/>
+      <c r="S5" s="14"/>
+      <c r="T5" s="14"/>
+      <c r="U5" s="14"/>
+      <c r="V5" s="14"/>
+      <c r="W5" s="14"/>
+      <c r="X5" s="14"/>
+      <c r="Y5" s="14"/>
+      <c r="Z5" s="14"/>
+      <c r="AA5" s="14"/>
+      <c r="AB5" s="14"/>
+      <c r="AC5" s="14"/>
+      <c r="AD5" s="14"/>
+      <c r="AE5" s="14"/>
+      <c r="AF5" s="30" t="s">
         <v>112</v>
       </c>
-      <c r="AI4" s="14"/>
-      <c r="AJ4" s="14"/>
-      <c r="AK4" s="14"/>
-      <c r="AL4" s="14"/>
-      <c r="AM4" s="14"/>
-      <c r="AN4" s="14"/>
-      <c r="AO4" s="14"/>
-      <c r="AP4" s="14"/>
-      <c r="AQ4" s="14"/>
-      <c r="AR4" s="14"/>
-      <c r="AS4" s="14"/>
-      <c r="AT4" s="14"/>
-      <c r="AU4" s="14"/>
-      <c r="AV4" s="14"/>
-      <c r="AW4" s="14"/>
-      <c r="AX4" s="14"/>
-      <c r="AY4" s="14"/>
-      <c r="AZ4" s="14"/>
-      <c r="BA4" s="14"/>
-      <c r="BB4" s="14"/>
-      <c r="BC4" s="14"/>
-      <c r="BD4" s="14"/>
-      <c r="BE4" s="14"/>
-      <c r="BF4" s="14"/>
-      <c r="BG4" s="14"/>
-      <c r="BH4" s="14"/>
-      <c r="BI4" s="14"/>
-      <c r="BJ4" s="14"/>
-      <c r="BK4" s="14"/>
-      <c r="BL4" s="14"/>
-      <c r="BM4" s="14"/>
-      <c r="BN4" s="14"/>
-      <c r="BO4" s="14"/>
-      <c r="BP4" s="14"/>
-      <c r="BQ4" s="14"/>
-      <c r="BR4" s="14"/>
-      <c r="BS4" s="14"/>
-      <c r="BT4" s="14"/>
-      <c r="BU4" s="14"/>
-      <c r="BV4" s="14"/>
-      <c r="BW4" s="14"/>
-      <c r="BX4" s="14"/>
-      <c r="BY4" s="14"/>
-      <c r="BZ4" s="14"/>
-      <c r="CA4" s="14"/>
-      <c r="CB4" s="14"/>
-      <c r="CC4" s="14"/>
-      <c r="CD4" s="14"/>
-      <c r="CE4" s="14"/>
-      <c r="CF4" s="14"/>
-      <c r="CG4" s="14"/>
-      <c r="CH4" s="14"/>
-      <c r="CI4" s="14"/>
-      <c r="CJ4" s="14"/>
-      <c r="CK4" s="14"/>
-      <c r="CL4" s="15"/>
+      <c r="AG5" s="14"/>
+      <c r="AH5" s="14"/>
+      <c r="AI5" s="14"/>
+      <c r="AJ5" s="14"/>
+      <c r="AK5" s="14"/>
+      <c r="AL5" s="14"/>
+      <c r="AM5" s="14"/>
+      <c r="AN5" s="14"/>
+      <c r="AO5" s="14"/>
+      <c r="AP5" s="14"/>
+      <c r="AQ5" s="14"/>
+      <c r="AR5" s="14"/>
+      <c r="AS5" s="14"/>
+      <c r="AT5" s="14"/>
+      <c r="AU5" s="14"/>
+      <c r="AV5" s="14"/>
+      <c r="AW5" s="14"/>
+      <c r="AX5" s="14"/>
+      <c r="AY5" s="14"/>
+      <c r="AZ5" s="14"/>
+      <c r="BA5" s="14"/>
+      <c r="BB5" s="14"/>
+      <c r="BC5" s="14"/>
+      <c r="BD5" s="14"/>
+      <c r="BE5" s="14"/>
+      <c r="BF5" s="14"/>
+      <c r="BG5" s="14"/>
+      <c r="BH5" s="14"/>
+      <c r="BI5" s="14"/>
+      <c r="BJ5" s="14"/>
+      <c r="BK5" s="14"/>
+      <c r="BL5" s="14"/>
+      <c r="BM5" s="14"/>
+      <c r="BN5" s="14"/>
+      <c r="BO5" s="14"/>
+      <c r="BP5" s="14"/>
+      <c r="BQ5" s="14"/>
+      <c r="BR5" s="14"/>
+      <c r="BS5" s="14"/>
+      <c r="BT5" s="14"/>
+      <c r="BU5" s="14"/>
+      <c r="BV5" s="14"/>
+      <c r="BW5" s="14"/>
+      <c r="BX5" s="14"/>
+      <c r="BY5" s="14"/>
+      <c r="BZ5" s="14"/>
+      <c r="CA5" s="14"/>
+      <c r="CB5" s="14"/>
+      <c r="CC5" s="14"/>
+      <c r="CD5" s="14"/>
+      <c r="CE5" s="14"/>
+      <c r="CF5" s="14"/>
+      <c r="CG5" s="14"/>
+      <c r="CH5" s="14"/>
+      <c r="CI5" s="14"/>
+      <c r="CJ5" s="14"/>
+      <c r="CK5" s="14"/>
+      <c r="CL5" s="15"/>
     </row>
+    <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="8" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="9" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="10" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7D2694E-D810-4A8F-9E88-6BF6AE47836A}">
   <sheetPr codeName="Sheet69"/>
   <dimension ref="A1:CL6"/>
@@ -40943,10 +43050,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13E13F0B-BD68-436F-AC4B-0DE79A71FA29}">
-  <sheetPr codeName="Sheet70"/>
-  <dimension ref="A1:CL10"/>
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98123E36-DEC7-4BA3-914F-651666C56468}">
+  <sheetPr codeName="Sheet68"/>
+  <dimension ref="A1:CL4"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="90" width="1.75" customWidth="1"/>
@@ -41048,7 +43155,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -41164,7 +43271,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -41182,10 +43289,12 @@
       <c r="AE3" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="AF3" s="6"/>
+      <c r="AF3" s="25" t="s">
+        <v>195</v>
+      </c>
       <c r="AG3" s="6"/>
       <c r="AH3" s="25" t="s">
-        <v>80</v>
+        <v>196</v>
       </c>
       <c r="AI3" s="6"/>
       <c r="AJ3" s="6"/>
@@ -41245,511 +43354,13 @@
       <c r="CL3" s="7"/>
     </row>
     <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="8"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="U4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="3"/>
-      <c r="Y4" s="3"/>
-      <c r="Z4" s="3"/>
-      <c r="AA4" s="3"/>
-      <c r="AB4" s="3"/>
-      <c r="AC4" s="3"/>
-      <c r="AD4" s="3"/>
-      <c r="AE4" s="3"/>
-      <c r="AF4" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="AG4" s="3"/>
-      <c r="AH4" s="27" t="s">
-        <v>276</v>
-      </c>
-      <c r="AI4" s="3"/>
-      <c r="AJ4" s="3"/>
-      <c r="AK4" s="3"/>
-      <c r="AL4" s="3"/>
-      <c r="AM4" s="3"/>
-      <c r="AN4" s="3"/>
-      <c r="AO4" s="3"/>
-      <c r="AP4" s="3"/>
-      <c r="AQ4" s="3"/>
-      <c r="AR4" s="3"/>
-      <c r="AS4" s="3"/>
-      <c r="AT4" s="3"/>
-      <c r="AU4" s="3"/>
-      <c r="AV4" s="3"/>
-      <c r="AW4" s="3"/>
-      <c r="AX4" s="3"/>
-      <c r="AY4" s="3"/>
-      <c r="AZ4" s="3"/>
-      <c r="BA4" s="3"/>
-      <c r="BB4" s="3"/>
-      <c r="BC4" s="3"/>
-      <c r="BD4" s="3"/>
-      <c r="BE4" s="3"/>
-      <c r="BF4" s="3"/>
-      <c r="BG4" s="3"/>
-      <c r="BH4" s="3"/>
-      <c r="BI4" s="3"/>
-      <c r="BJ4" s="3"/>
-      <c r="BK4" s="3"/>
-      <c r="BL4" s="3"/>
-      <c r="BM4" s="3"/>
-      <c r="BN4" s="3"/>
-      <c r="BO4" s="3"/>
-      <c r="BP4" s="3"/>
-      <c r="BQ4" s="3"/>
-      <c r="BR4" s="3"/>
-      <c r="BS4" s="3"/>
-      <c r="BT4" s="3"/>
-      <c r="BU4" s="3"/>
-      <c r="BV4" s="3"/>
-      <c r="BW4" s="3"/>
-      <c r="BX4" s="3"/>
-      <c r="BY4" s="3"/>
-      <c r="BZ4" s="3"/>
-      <c r="CA4" s="3"/>
-      <c r="CB4" s="3"/>
-      <c r="CC4" s="3"/>
-      <c r="CD4" s="3"/>
-      <c r="CE4" s="3"/>
-      <c r="CF4" s="3"/>
-      <c r="CG4" s="3"/>
-      <c r="CH4" s="3"/>
-      <c r="CI4" s="3"/>
-      <c r="CJ4" s="3"/>
-      <c r="CK4" s="3"/>
-      <c r="CL4" s="10"/>
-    </row>
-    <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="11"/>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="14"/>
-      <c r="M5" s="14"/>
-      <c r="N5" s="14"/>
-      <c r="O5" s="14"/>
-      <c r="P5" s="14"/>
-      <c r="Q5" s="14"/>
-      <c r="R5" s="14"/>
-      <c r="S5" s="14"/>
-      <c r="T5" s="14"/>
-      <c r="U5" s="14"/>
-      <c r="V5" s="14"/>
-      <c r="W5" s="14"/>
-      <c r="X5" s="14"/>
-      <c r="Y5" s="14"/>
-      <c r="Z5" s="14"/>
-      <c r="AA5" s="14"/>
-      <c r="AB5" s="14"/>
-      <c r="AC5" s="14"/>
-      <c r="AD5" s="14"/>
-      <c r="AE5" s="14"/>
-      <c r="AF5" s="30" t="s">
-        <v>112</v>
-      </c>
-      <c r="AG5" s="14"/>
-      <c r="AH5" s="14"/>
-      <c r="AI5" s="14"/>
-      <c r="AJ5" s="14"/>
-      <c r="AK5" s="14"/>
-      <c r="AL5" s="14"/>
-      <c r="AM5" s="14"/>
-      <c r="AN5" s="14"/>
-      <c r="AO5" s="14"/>
-      <c r="AP5" s="14"/>
-      <c r="AQ5" s="14"/>
-      <c r="AR5" s="14"/>
-      <c r="AS5" s="14"/>
-      <c r="AT5" s="14"/>
-      <c r="AU5" s="14"/>
-      <c r="AV5" s="14"/>
-      <c r="AW5" s="14"/>
-      <c r="AX5" s="14"/>
-      <c r="AY5" s="14"/>
-      <c r="AZ5" s="14"/>
-      <c r="BA5" s="14"/>
-      <c r="BB5" s="14"/>
-      <c r="BC5" s="14"/>
-      <c r="BD5" s="14"/>
-      <c r="BE5" s="14"/>
-      <c r="BF5" s="14"/>
-      <c r="BG5" s="14"/>
-      <c r="BH5" s="14"/>
-      <c r="BI5" s="14"/>
-      <c r="BJ5" s="14"/>
-      <c r="BK5" s="14"/>
-      <c r="BL5" s="14"/>
-      <c r="BM5" s="14"/>
-      <c r="BN5" s="14"/>
-      <c r="BO5" s="14"/>
-      <c r="BP5" s="14"/>
-      <c r="BQ5" s="14"/>
-      <c r="BR5" s="14"/>
-      <c r="BS5" s="14"/>
-      <c r="BT5" s="14"/>
-      <c r="BU5" s="14"/>
-      <c r="BV5" s="14"/>
-      <c r="BW5" s="14"/>
-      <c r="BX5" s="14"/>
-      <c r="BY5" s="14"/>
-      <c r="BZ5" s="14"/>
-      <c r="CA5" s="14"/>
-      <c r="CB5" s="14"/>
-      <c r="CC5" s="14"/>
-      <c r="CD5" s="14"/>
-      <c r="CE5" s="14"/>
-      <c r="CF5" s="14"/>
-      <c r="CG5" s="14"/>
-      <c r="CH5" s="14"/>
-      <c r="CI5" s="14"/>
-      <c r="CJ5" s="14"/>
-      <c r="CK5" s="14"/>
-      <c r="CL5" s="15"/>
-    </row>
-    <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="8" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="9" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="10" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
-  </sheetData>
-  <phoneticPr fontId="2"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30AB51C2-4CAF-40D2-90C0-05BD312EBAB8}">
-  <sheetPr codeName="Sheet71"/>
-  <dimension ref="A1:CL10"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
-  <cols>
-    <col min="1" max="90" width="1.75" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
-      <c r="W1" s="1"/>
-      <c r="X1" s="1"/>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="1"/>
-      <c r="AA1" s="1"/>
-      <c r="AB1" s="1"/>
-      <c r="AC1" s="1"/>
-      <c r="AD1" s="1"/>
-      <c r="AE1" s="1"/>
-      <c r="AF1" s="1"/>
-      <c r="AG1" s="1"/>
-      <c r="AH1" s="1"/>
-      <c r="AI1" s="1"/>
-      <c r="AJ1" s="1"/>
-      <c r="AK1" s="1"/>
-      <c r="AL1" s="1"/>
-      <c r="AM1" s="1"/>
-      <c r="AN1" s="1"/>
-      <c r="AO1" s="1"/>
-      <c r="AP1" s="1"/>
-      <c r="AQ1" s="1"/>
-      <c r="AR1" s="1"/>
-      <c r="AS1" s="1"/>
-      <c r="AT1" s="1"/>
-      <c r="AU1" s="1"/>
-      <c r="AV1" s="1"/>
-      <c r="AW1" s="1"/>
-      <c r="AX1" s="1"/>
-      <c r="AY1" s="1"/>
-      <c r="AZ1" s="1"/>
-      <c r="BA1" s="1"/>
-      <c r="BB1" s="1"/>
-      <c r="BC1" s="1"/>
-      <c r="BD1" s="1"/>
-      <c r="BE1" s="1"/>
-      <c r="BF1" s="1"/>
-      <c r="BG1" s="1"/>
-      <c r="BH1" s="1"/>
-      <c r="BI1" s="1"/>
-      <c r="BJ1" s="1"/>
-      <c r="BK1" s="1"/>
-      <c r="BL1" s="1"/>
-      <c r="BM1" s="1"/>
-      <c r="BN1" s="1"/>
-      <c r="BO1" s="1"/>
-      <c r="BP1" s="1"/>
-      <c r="BQ1" s="1"/>
-      <c r="BR1" s="1"/>
-      <c r="BS1" s="1"/>
-      <c r="BT1" s="1"/>
-      <c r="BU1" s="1"/>
-      <c r="BV1" s="1"/>
-      <c r="BW1" s="1"/>
-      <c r="BX1" s="1"/>
-      <c r="BY1" s="1"/>
-      <c r="BZ1" s="1"/>
-      <c r="CA1" s="1"/>
-      <c r="CB1" s="1"/>
-      <c r="CC1" s="1"/>
-      <c r="CD1" s="1"/>
-      <c r="CE1" s="1"/>
-      <c r="CF1" s="1"/>
-      <c r="CG1" s="1"/>
-      <c r="CH1" s="1"/>
-      <c r="CI1" s="1"/>
-      <c r="CJ1" s="1"/>
-      <c r="CK1" s="1"/>
-      <c r="CL1" s="1"/>
-    </row>
-    <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
-      <c r="R2" s="1"/>
-      <c r="S2" s="1"/>
-      <c r="T2" s="1"/>
-      <c r="U2" s="1"/>
-      <c r="V2" s="1"/>
-      <c r="W2" s="1"/>
-      <c r="X2" s="1"/>
-      <c r="Y2" s="1"/>
-      <c r="Z2" s="1"/>
-      <c r="AA2" s="1"/>
-      <c r="AB2" s="1"/>
-      <c r="AC2" s="1"/>
-      <c r="AD2" s="1"/>
-      <c r="AE2" s="1"/>
-      <c r="AF2" s="1"/>
-      <c r="AG2" s="1"/>
-      <c r="AH2" s="1"/>
-      <c r="AI2" s="1"/>
-      <c r="AJ2" s="1"/>
-      <c r="AK2" s="1"/>
-      <c r="AL2" s="1"/>
-      <c r="AM2" s="1"/>
-      <c r="AN2" s="1"/>
-      <c r="AO2" s="1"/>
-      <c r="AP2" s="1"/>
-      <c r="AQ2" s="1"/>
-      <c r="AR2" s="1"/>
-      <c r="AS2" s="1"/>
-      <c r="AT2" s="1"/>
-      <c r="AU2" s="1"/>
-      <c r="AV2" s="1"/>
-      <c r="AW2" s="1"/>
-      <c r="AX2" s="1"/>
-      <c r="AY2" s="1"/>
-      <c r="AZ2" s="1"/>
-      <c r="BA2" s="1"/>
-      <c r="BB2" s="1"/>
-      <c r="BC2" s="1"/>
-      <c r="BD2" s="1"/>
-      <c r="BE2" s="1"/>
-      <c r="BF2" s="1"/>
-      <c r="BG2" s="1"/>
-      <c r="BH2" s="1"/>
-      <c r="BI2" s="1"/>
-      <c r="BJ2" s="1"/>
-      <c r="BK2" s="1"/>
-      <c r="BL2" s="1"/>
-      <c r="BM2" s="1"/>
-      <c r="BN2" s="1"/>
-      <c r="BO2" s="1"/>
-      <c r="BP2" s="1"/>
-      <c r="BQ2" s="1"/>
-      <c r="BR2" s="1"/>
-      <c r="BS2" s="1"/>
-      <c r="BT2" s="1"/>
-      <c r="BU2" s="1"/>
-      <c r="BV2" s="1"/>
-      <c r="BW2" s="1"/>
-      <c r="BX2" s="1"/>
-      <c r="BY2" s="1"/>
-      <c r="BZ2" s="1"/>
-      <c r="CA2" s="1"/>
-      <c r="CB2" s="1"/>
-      <c r="CC2" s="1"/>
-      <c r="CD2" s="1"/>
-      <c r="CE2" s="1"/>
-      <c r="CF2" s="1"/>
-      <c r="CG2" s="1"/>
-      <c r="CH2" s="1"/>
-      <c r="CI2" s="1"/>
-      <c r="CJ2" s="1"/>
-      <c r="CK2" s="1"/>
-      <c r="CL2" s="1"/>
-    </row>
-    <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="28" t="s">
-        <v>91</v>
-      </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
-      <c r="M3" s="16"/>
-      <c r="N3" s="16"/>
-      <c r="O3" s="16"/>
-      <c r="P3" s="16"/>
-      <c r="Q3" s="16"/>
-      <c r="R3" s="16"/>
-      <c r="S3" s="28" t="s">
-        <v>92</v>
-      </c>
-      <c r="T3" s="16"/>
-      <c r="U3" s="16"/>
-      <c r="V3" s="16"/>
-      <c r="W3" s="16"/>
-      <c r="X3" s="16"/>
-      <c r="Y3" s="16"/>
-      <c r="Z3" s="16"/>
-      <c r="AA3" s="16"/>
-      <c r="AB3" s="16"/>
-      <c r="AC3" s="16"/>
-      <c r="AD3" s="16"/>
-      <c r="AE3" s="16"/>
-      <c r="AF3" s="16"/>
-      <c r="AG3" s="16"/>
-      <c r="AH3" s="16"/>
-      <c r="AI3" s="16"/>
-      <c r="AJ3" s="16"/>
-      <c r="AK3" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="AL3" s="16"/>
-      <c r="AM3" s="16"/>
-      <c r="AN3" s="16"/>
-      <c r="AO3" s="16"/>
-      <c r="AP3" s="16"/>
-      <c r="AQ3" s="16"/>
-      <c r="AR3" s="16"/>
-      <c r="AS3" s="16"/>
-      <c r="AT3" s="16"/>
-      <c r="AU3" s="16"/>
-      <c r="AV3" s="16"/>
-      <c r="AW3" s="16"/>
-      <c r="AX3" s="16"/>
-      <c r="AY3" s="16"/>
-      <c r="AZ3" s="16"/>
-      <c r="BA3" s="16"/>
-      <c r="BB3" s="16"/>
-      <c r="BC3" s="16"/>
-      <c r="BD3" s="16"/>
-      <c r="BE3" s="16"/>
-      <c r="BF3" s="16"/>
-      <c r="BG3" s="16"/>
-      <c r="BH3" s="16"/>
-      <c r="BI3" s="16"/>
-      <c r="BJ3" s="16"/>
-      <c r="BK3" s="16"/>
-      <c r="BL3" s="16"/>
-      <c r="BM3" s="16"/>
-      <c r="BN3" s="16"/>
-      <c r="BO3" s="16"/>
-      <c r="BP3" s="16"/>
-      <c r="BQ3" s="16"/>
-      <c r="BR3" s="16"/>
-      <c r="BS3" s="16"/>
-      <c r="BT3" s="16"/>
-      <c r="BU3" s="16"/>
-      <c r="BV3" s="16"/>
-      <c r="BW3" s="16"/>
-      <c r="BX3" s="16"/>
-      <c r="BY3" s="16"/>
-      <c r="BZ3" s="16"/>
-      <c r="CA3" s="16"/>
-      <c r="CB3" s="16"/>
-      <c r="CC3" s="16"/>
-      <c r="CD3" s="16"/>
-      <c r="CE3" s="16"/>
-      <c r="CF3" s="16"/>
-      <c r="CG3" s="16"/>
-      <c r="CH3" s="16"/>
-      <c r="CI3" s="16"/>
-      <c r="CJ3" s="16"/>
-      <c r="CK3" s="16"/>
-      <c r="CL3" s="21"/>
-    </row>
-    <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="31" t="s">
-        <v>159</v>
-      </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
+      <c r="A4" s="11"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="13"/>
       <c r="H4" s="14"/>
       <c r="I4" s="14"/>
       <c r="J4" s="14"/>
@@ -41761,9 +43372,7 @@
       <c r="P4" s="14"/>
       <c r="Q4" s="14"/>
       <c r="R4" s="14"/>
-      <c r="S4" s="31" t="s">
-        <v>124</v>
-      </c>
+      <c r="S4" s="14"/>
       <c r="T4" s="14"/>
       <c r="U4" s="14"/>
       <c r="V4" s="14"/>
@@ -41778,609 +43387,12 @@
       <c r="AE4" s="14"/>
       <c r="AF4" s="14"/>
       <c r="AG4" s="14"/>
-      <c r="AH4" s="14"/>
-      <c r="AI4" s="30" t="s">
-        <v>7</v>
-      </c>
+      <c r="AH4" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="AI4" s="14"/>
       <c r="AJ4" s="14"/>
-      <c r="AK4" s="13"/>
-      <c r="AL4" s="14"/>
-      <c r="AM4" s="30" t="s">
-        <v>203</v>
-      </c>
-      <c r="AN4" s="14"/>
-      <c r="AO4" s="14"/>
-      <c r="AP4" s="14"/>
-      <c r="AQ4" s="14"/>
-      <c r="AR4" s="14"/>
-      <c r="AS4" s="14"/>
-      <c r="AT4" s="14"/>
-      <c r="AU4" s="14"/>
-      <c r="AV4" s="14"/>
-      <c r="AW4" s="14"/>
-      <c r="AX4" s="14"/>
-      <c r="AY4" s="14"/>
-      <c r="AZ4" s="14"/>
-      <c r="BA4" s="14"/>
-      <c r="BB4" s="14"/>
-      <c r="BC4" s="14"/>
-      <c r="BD4" s="14"/>
-      <c r="BE4" s="14"/>
-      <c r="BF4" s="14"/>
-      <c r="BG4" s="14"/>
-      <c r="BH4" s="14"/>
-      <c r="BI4" s="14"/>
-      <c r="BJ4" s="14"/>
-      <c r="BK4" s="14"/>
-      <c r="BL4" s="14"/>
-      <c r="BM4" s="14"/>
-      <c r="BN4" s="14"/>
-      <c r="BO4" s="14"/>
-      <c r="BP4" s="14"/>
-      <c r="BQ4" s="14"/>
-      <c r="BR4" s="14"/>
-      <c r="BS4" s="14"/>
-      <c r="BT4" s="14"/>
-      <c r="BU4" s="14"/>
-      <c r="BV4" s="14"/>
-      <c r="BW4" s="14"/>
-      <c r="BX4" s="14"/>
-      <c r="BY4" s="14"/>
-      <c r="BZ4" s="14"/>
-      <c r="CA4" s="14"/>
-      <c r="CB4" s="14"/>
-      <c r="CC4" s="14"/>
-      <c r="CD4" s="14"/>
-      <c r="CE4" s="14"/>
-      <c r="CF4" s="14"/>
-      <c r="CG4" s="14"/>
-      <c r="CH4" s="14"/>
-      <c r="CI4" s="14"/>
-      <c r="CJ4" s="14"/>
-      <c r="CK4" s="14"/>
-      <c r="CL4" s="15"/>
-    </row>
-    <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="17"/>
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="18"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="18"/>
-      <c r="N5" s="18"/>
-      <c r="O5" s="18"/>
-      <c r="P5" s="18"/>
-      <c r="Q5" s="18"/>
-      <c r="R5" s="18"/>
-      <c r="S5" s="17"/>
-      <c r="T5" s="18"/>
-      <c r="U5" s="18"/>
-      <c r="V5" s="18"/>
-      <c r="W5" s="18"/>
-      <c r="X5" s="18"/>
-      <c r="Y5" s="18"/>
-      <c r="Z5" s="18"/>
-      <c r="AA5" s="18"/>
-      <c r="AB5" s="18"/>
-      <c r="AC5" s="18"/>
-      <c r="AD5" s="18"/>
-      <c r="AE5" s="18"/>
-      <c r="AF5" s="18"/>
-      <c r="AG5" s="18"/>
-      <c r="AH5" s="18"/>
-      <c r="AI5" s="18"/>
-      <c r="AJ5" s="18"/>
-      <c r="AK5" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="AL5" s="18"/>
-      <c r="AM5" s="29" t="s">
-        <v>278</v>
-      </c>
-      <c r="AN5" s="18"/>
-      <c r="AO5" s="18"/>
-      <c r="AP5" s="18"/>
-      <c r="AQ5" s="18"/>
-      <c r="AR5" s="18"/>
-      <c r="AS5" s="18"/>
-      <c r="AT5" s="18"/>
-      <c r="AU5" s="18"/>
-      <c r="AV5" s="18"/>
-      <c r="AW5" s="18"/>
-      <c r="AX5" s="18"/>
-      <c r="AY5" s="18"/>
-      <c r="AZ5" s="18"/>
-      <c r="BA5" s="18"/>
-      <c r="BB5" s="18"/>
-      <c r="BC5" s="18"/>
-      <c r="BD5" s="18"/>
-      <c r="BE5" s="18"/>
-      <c r="BF5" s="18"/>
-      <c r="BG5" s="18"/>
-      <c r="BH5" s="18"/>
-      <c r="BI5" s="18"/>
-      <c r="BJ5" s="18"/>
-      <c r="BK5" s="18"/>
-      <c r="BL5" s="18"/>
-      <c r="BM5" s="18"/>
-      <c r="BN5" s="18"/>
-      <c r="BO5" s="18"/>
-      <c r="BP5" s="18"/>
-      <c r="BQ5" s="18"/>
-      <c r="BR5" s="18"/>
-      <c r="BS5" s="18"/>
-      <c r="BT5" s="18"/>
-      <c r="BU5" s="18"/>
-      <c r="BV5" s="18"/>
-      <c r="BW5" s="18"/>
-      <c r="BX5" s="18"/>
-      <c r="BY5" s="18"/>
-      <c r="BZ5" s="18"/>
-      <c r="CA5" s="18"/>
-      <c r="CB5" s="18"/>
-      <c r="CC5" s="18"/>
-      <c r="CD5" s="18"/>
-      <c r="CE5" s="18"/>
-      <c r="CF5" s="18"/>
-      <c r="CG5" s="18"/>
-      <c r="CH5" s="18"/>
-      <c r="CI5" s="18"/>
-      <c r="CJ5" s="18"/>
-      <c r="CK5" s="18"/>
-      <c r="CL5" s="19"/>
-    </row>
-    <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="17"/>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="18"/>
-      <c r="N6" s="18"/>
-      <c r="O6" s="18"/>
-      <c r="P6" s="18"/>
-      <c r="Q6" s="18"/>
-      <c r="R6" s="18"/>
-      <c r="S6" s="17"/>
-      <c r="T6" s="18"/>
-      <c r="U6" s="18"/>
-      <c r="V6" s="18"/>
-      <c r="W6" s="18"/>
-      <c r="X6" s="18"/>
-      <c r="Y6" s="18"/>
-      <c r="Z6" s="18"/>
-      <c r="AA6" s="18"/>
-      <c r="AB6" s="18"/>
-      <c r="AC6" s="18"/>
-      <c r="AD6" s="18"/>
-      <c r="AE6" s="18"/>
-      <c r="AF6" s="18"/>
-      <c r="AG6" s="18"/>
-      <c r="AH6" s="18"/>
-      <c r="AI6" s="18"/>
-      <c r="AJ6" s="18"/>
-      <c r="AK6" s="20" t="s">
-        <v>204</v>
-      </c>
-      <c r="AL6" s="18"/>
-      <c r="AM6" s="18"/>
-      <c r="AN6" s="18"/>
-      <c r="AO6" s="18"/>
-      <c r="AP6" s="18"/>
-      <c r="AQ6" s="18"/>
-      <c r="AR6" s="18"/>
-      <c r="AS6" s="18"/>
-      <c r="AT6" s="18"/>
-      <c r="AU6" s="18"/>
-      <c r="AV6" s="18"/>
-      <c r="AW6" s="18"/>
-      <c r="AX6" s="18"/>
-      <c r="AY6" s="18"/>
-      <c r="AZ6" s="18"/>
-      <c r="BA6" s="18"/>
-      <c r="BB6" s="18"/>
-      <c r="BC6" s="18"/>
-      <c r="BD6" s="18"/>
-      <c r="BE6" s="18"/>
-      <c r="BF6" s="18"/>
-      <c r="BG6" s="18"/>
-      <c r="BH6" s="18"/>
-      <c r="BI6" s="18"/>
-      <c r="BJ6" s="18"/>
-      <c r="BK6" s="18"/>
-      <c r="BL6" s="18"/>
-      <c r="BM6" s="18"/>
-      <c r="BN6" s="18"/>
-      <c r="BO6" s="18"/>
-      <c r="BP6" s="18"/>
-      <c r="BQ6" s="18"/>
-      <c r="BR6" s="18"/>
-      <c r="BS6" s="18"/>
-      <c r="BT6" s="18"/>
-      <c r="BU6" s="18"/>
-      <c r="BV6" s="18"/>
-      <c r="BW6" s="18"/>
-      <c r="BX6" s="18"/>
-      <c r="BY6" s="18"/>
-      <c r="BZ6" s="18"/>
-      <c r="CA6" s="18"/>
-      <c r="CB6" s="18"/>
-      <c r="CC6" s="18"/>
-      <c r="CD6" s="18"/>
-      <c r="CE6" s="18"/>
-      <c r="CF6" s="18"/>
-      <c r="CG6" s="18"/>
-      <c r="CH6" s="18"/>
-      <c r="CI6" s="18"/>
-      <c r="CJ6" s="18"/>
-      <c r="CK6" s="18"/>
-      <c r="CL6" s="19"/>
-    </row>
-    <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="8" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="9" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="10" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
-  </sheetData>
-  <phoneticPr fontId="2"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A2358E7-8911-407D-AA94-1AF2EC7340FC}">
-  <sheetPr codeName="Sheet72"/>
-  <dimension ref="A1:CL5"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
-  <cols>
-    <col min="1" max="90" width="1.75" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
-      <c r="W1" s="1"/>
-      <c r="X1" s="1"/>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="1"/>
-      <c r="AA1" s="1"/>
-      <c r="AB1" s="1"/>
-      <c r="AC1" s="1"/>
-      <c r="AD1" s="1"/>
-      <c r="AE1" s="1"/>
-      <c r="AF1" s="1"/>
-      <c r="AG1" s="1"/>
-      <c r="AH1" s="1"/>
-      <c r="AI1" s="1"/>
-      <c r="AJ1" s="1"/>
-      <c r="AK1" s="1"/>
-      <c r="AL1" s="1"/>
-      <c r="AM1" s="1"/>
-      <c r="AN1" s="1"/>
-      <c r="AO1" s="1"/>
-      <c r="AP1" s="1"/>
-      <c r="AQ1" s="1"/>
-      <c r="AR1" s="1"/>
-      <c r="AS1" s="1"/>
-      <c r="AT1" s="1"/>
-      <c r="AU1" s="1"/>
-      <c r="AV1" s="1"/>
-      <c r="AW1" s="1"/>
-      <c r="AX1" s="1"/>
-      <c r="AY1" s="1"/>
-      <c r="AZ1" s="1"/>
-      <c r="BA1" s="1"/>
-      <c r="BB1" s="1"/>
-      <c r="BC1" s="1"/>
-      <c r="BD1" s="1"/>
-      <c r="BE1" s="1"/>
-      <c r="BF1" s="1"/>
-      <c r="BG1" s="1"/>
-      <c r="BH1" s="1"/>
-      <c r="BI1" s="1"/>
-      <c r="BJ1" s="1"/>
-      <c r="BK1" s="1"/>
-      <c r="BL1" s="1"/>
-      <c r="BM1" s="1"/>
-      <c r="BN1" s="1"/>
-      <c r="BO1" s="1"/>
-      <c r="BP1" s="1"/>
-      <c r="BQ1" s="1"/>
-      <c r="BR1" s="1"/>
-      <c r="BS1" s="1"/>
-      <c r="BT1" s="1"/>
-      <c r="BU1" s="1"/>
-      <c r="BV1" s="1"/>
-      <c r="BW1" s="1"/>
-      <c r="BX1" s="1"/>
-      <c r="BY1" s="1"/>
-      <c r="BZ1" s="1"/>
-      <c r="CA1" s="1"/>
-      <c r="CB1" s="1"/>
-      <c r="CC1" s="1"/>
-      <c r="CD1" s="1"/>
-      <c r="CE1" s="1"/>
-      <c r="CF1" s="1"/>
-      <c r="CG1" s="1"/>
-      <c r="CH1" s="1"/>
-      <c r="CI1" s="1"/>
-      <c r="CJ1" s="1"/>
-      <c r="CK1" s="1"/>
-      <c r="CL1" s="1"/>
-    </row>
-    <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="22" t="s">
-        <v>161</v>
-      </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
-      <c r="R2" s="1"/>
-      <c r="S2" s="1"/>
-      <c r="T2" s="1"/>
-      <c r="U2" s="1"/>
-      <c r="V2" s="1"/>
-      <c r="W2" s="1"/>
-      <c r="X2" s="1"/>
-      <c r="Y2" s="1"/>
-      <c r="Z2" s="1"/>
-      <c r="AA2" s="1"/>
-      <c r="AB2" s="1"/>
-      <c r="AC2" s="1"/>
-      <c r="AD2" s="1"/>
-      <c r="AE2" s="1"/>
-      <c r="AF2" s="1"/>
-      <c r="AG2" s="1"/>
-      <c r="AH2" s="1"/>
-      <c r="AI2" s="1"/>
-      <c r="AJ2" s="1"/>
-      <c r="AK2" s="1"/>
-      <c r="AL2" s="1"/>
-      <c r="AM2" s="1"/>
-      <c r="AN2" s="1"/>
-      <c r="AO2" s="1"/>
-      <c r="AP2" s="1"/>
-      <c r="AQ2" s="1"/>
-      <c r="AR2" s="1"/>
-      <c r="AS2" s="1"/>
-      <c r="AT2" s="1"/>
-      <c r="AU2" s="1"/>
-      <c r="AV2" s="1"/>
-      <c r="AW2" s="1"/>
-      <c r="AX2" s="1"/>
-      <c r="AY2" s="1"/>
-      <c r="AZ2" s="1"/>
-      <c r="BA2" s="1"/>
-      <c r="BB2" s="1"/>
-      <c r="BC2" s="1"/>
-      <c r="BD2" s="1"/>
-      <c r="BE2" s="1"/>
-      <c r="BF2" s="1"/>
-      <c r="BG2" s="1"/>
-      <c r="BH2" s="1"/>
-      <c r="BI2" s="1"/>
-      <c r="BJ2" s="1"/>
-      <c r="BK2" s="1"/>
-      <c r="BL2" s="1"/>
-      <c r="BM2" s="1"/>
-      <c r="BN2" s="1"/>
-      <c r="BO2" s="1"/>
-      <c r="BP2" s="1"/>
-      <c r="BQ2" s="1"/>
-      <c r="BR2" s="1"/>
-      <c r="BS2" s="1"/>
-      <c r="BT2" s="1"/>
-      <c r="BU2" s="1"/>
-      <c r="BV2" s="1"/>
-      <c r="BW2" s="1"/>
-      <c r="BX2" s="1"/>
-      <c r="BY2" s="1"/>
-      <c r="BZ2" s="1"/>
-      <c r="CA2" s="1"/>
-      <c r="CB2" s="1"/>
-      <c r="CC2" s="1"/>
-      <c r="CD2" s="1"/>
-      <c r="CE2" s="1"/>
-      <c r="CF2" s="1"/>
-      <c r="CG2" s="1"/>
-      <c r="CH2" s="1"/>
-      <c r="CI2" s="1"/>
-      <c r="CJ2" s="1"/>
-      <c r="CK2" s="1"/>
-      <c r="CL2" s="1"/>
-    </row>
-    <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="28" t="s">
-        <v>91</v>
-      </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
-      <c r="M3" s="16"/>
-      <c r="N3" s="16"/>
-      <c r="O3" s="16"/>
-      <c r="P3" s="16"/>
-      <c r="Q3" s="16"/>
-      <c r="R3" s="16"/>
-      <c r="S3" s="28" t="s">
-        <v>92</v>
-      </c>
-      <c r="T3" s="16"/>
-      <c r="U3" s="16"/>
-      <c r="V3" s="16"/>
-      <c r="W3" s="16"/>
-      <c r="X3" s="16"/>
-      <c r="Y3" s="16"/>
-      <c r="Z3" s="16"/>
-      <c r="AA3" s="16"/>
-      <c r="AB3" s="16"/>
-      <c r="AC3" s="16"/>
-      <c r="AD3" s="16"/>
-      <c r="AE3" s="16"/>
-      <c r="AF3" s="16"/>
-      <c r="AG3" s="16"/>
-      <c r="AH3" s="16"/>
-      <c r="AI3" s="16"/>
-      <c r="AJ3" s="16"/>
-      <c r="AK3" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="AL3" s="16"/>
-      <c r="AM3" s="16"/>
-      <c r="AN3" s="16"/>
-      <c r="AO3" s="16"/>
-      <c r="AP3" s="16"/>
-      <c r="AQ3" s="16"/>
-      <c r="AR3" s="16"/>
-      <c r="AS3" s="16"/>
-      <c r="AT3" s="16"/>
-      <c r="AU3" s="16"/>
-      <c r="AV3" s="16"/>
-      <c r="AW3" s="16"/>
-      <c r="AX3" s="16"/>
-      <c r="AY3" s="16"/>
-      <c r="AZ3" s="16"/>
-      <c r="BA3" s="16"/>
-      <c r="BB3" s="16"/>
-      <c r="BC3" s="16"/>
-      <c r="BD3" s="16"/>
-      <c r="BE3" s="16"/>
-      <c r="BF3" s="16"/>
-      <c r="BG3" s="16"/>
-      <c r="BH3" s="16"/>
-      <c r="BI3" s="16"/>
-      <c r="BJ3" s="16"/>
-      <c r="BK3" s="16"/>
-      <c r="BL3" s="16"/>
-      <c r="BM3" s="16"/>
-      <c r="BN3" s="16"/>
-      <c r="BO3" s="16"/>
-      <c r="BP3" s="16"/>
-      <c r="BQ3" s="16"/>
-      <c r="BR3" s="16"/>
-      <c r="BS3" s="16"/>
-      <c r="BT3" s="16"/>
-      <c r="BU3" s="16"/>
-      <c r="BV3" s="16"/>
-      <c r="BW3" s="16"/>
-      <c r="BX3" s="16"/>
-      <c r="BY3" s="16"/>
-      <c r="BZ3" s="16"/>
-      <c r="CA3" s="16"/>
-      <c r="CB3" s="16"/>
-      <c r="CC3" s="16"/>
-      <c r="CD3" s="16"/>
-      <c r="CE3" s="16"/>
-      <c r="CF3" s="16"/>
-      <c r="CG3" s="16"/>
-      <c r="CH3" s="16"/>
-      <c r="CI3" s="16"/>
-      <c r="CJ3" s="16"/>
-      <c r="CK3" s="16"/>
-      <c r="CL3" s="21"/>
-    </row>
-    <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="31" t="s">
-        <v>159</v>
-      </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
-      <c r="L4" s="14"/>
-      <c r="M4" s="14"/>
-      <c r="N4" s="14"/>
-      <c r="O4" s="14"/>
-      <c r="P4" s="14"/>
-      <c r="Q4" s="14"/>
-      <c r="R4" s="14"/>
-      <c r="S4" s="31" t="s">
-        <v>124</v>
-      </c>
-      <c r="T4" s="14"/>
-      <c r="U4" s="14"/>
-      <c r="V4" s="14"/>
-      <c r="W4" s="14"/>
-      <c r="X4" s="14"/>
-      <c r="Y4" s="14"/>
-      <c r="Z4" s="14"/>
-      <c r="AA4" s="14"/>
-      <c r="AB4" s="14"/>
-      <c r="AC4" s="14"/>
-      <c r="AD4" s="14"/>
-      <c r="AE4" s="14"/>
-      <c r="AF4" s="14"/>
-      <c r="AG4" s="14"/>
-      <c r="AH4" s="14"/>
-      <c r="AI4" s="30" t="s">
-        <v>7</v>
-      </c>
-      <c r="AJ4" s="14"/>
-      <c r="AK4" s="31" t="s">
-        <v>205</v>
-      </c>
+      <c r="AK4" s="14"/>
       <c r="AL4" s="14"/>
       <c r="AM4" s="14"/>
       <c r="AN4" s="14"/>
@@ -42434,597 +43446,6 @@
       <c r="CJ4" s="14"/>
       <c r="CK4" s="14"/>
       <c r="CL4" s="15"/>
-    </row>
-    <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="17"/>
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="18"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="18"/>
-      <c r="N5" s="18"/>
-      <c r="O5" s="18"/>
-      <c r="P5" s="18"/>
-      <c r="Q5" s="18"/>
-      <c r="R5" s="18"/>
-      <c r="S5" s="17"/>
-      <c r="T5" s="18"/>
-      <c r="U5" s="18"/>
-      <c r="V5" s="18"/>
-      <c r="W5" s="18"/>
-      <c r="X5" s="18"/>
-      <c r="Y5" s="18"/>
-      <c r="Z5" s="18"/>
-      <c r="AA5" s="18"/>
-      <c r="AB5" s="18"/>
-      <c r="AC5" s="18"/>
-      <c r="AD5" s="18"/>
-      <c r="AE5" s="18"/>
-      <c r="AF5" s="18"/>
-      <c r="AG5" s="18"/>
-      <c r="AH5" s="18"/>
-      <c r="AI5" s="18"/>
-      <c r="AJ5" s="18"/>
-      <c r="AK5" s="20" t="s">
-        <v>204</v>
-      </c>
-      <c r="AL5" s="18"/>
-      <c r="AM5" s="18"/>
-      <c r="AN5" s="18"/>
-      <c r="AO5" s="18"/>
-      <c r="AP5" s="18"/>
-      <c r="AQ5" s="18"/>
-      <c r="AR5" s="18"/>
-      <c r="AS5" s="18"/>
-      <c r="AT5" s="18"/>
-      <c r="AU5" s="18"/>
-      <c r="AV5" s="18"/>
-      <c r="AW5" s="18"/>
-      <c r="AX5" s="18"/>
-      <c r="AY5" s="18"/>
-      <c r="AZ5" s="18"/>
-      <c r="BA5" s="18"/>
-      <c r="BB5" s="18"/>
-      <c r="BC5" s="18"/>
-      <c r="BD5" s="18"/>
-      <c r="BE5" s="18"/>
-      <c r="BF5" s="18"/>
-      <c r="BG5" s="18"/>
-      <c r="BH5" s="18"/>
-      <c r="BI5" s="18"/>
-      <c r="BJ5" s="18"/>
-      <c r="BK5" s="18"/>
-      <c r="BL5" s="18"/>
-      <c r="BM5" s="18"/>
-      <c r="BN5" s="18"/>
-      <c r="BO5" s="18"/>
-      <c r="BP5" s="18"/>
-      <c r="BQ5" s="18"/>
-      <c r="BR5" s="18"/>
-      <c r="BS5" s="18"/>
-      <c r="BT5" s="18"/>
-      <c r="BU5" s="18"/>
-      <c r="BV5" s="18"/>
-      <c r="BW5" s="18"/>
-      <c r="BX5" s="18"/>
-      <c r="BY5" s="18"/>
-      <c r="BZ5" s="18"/>
-      <c r="CA5" s="18"/>
-      <c r="CB5" s="18"/>
-      <c r="CC5" s="18"/>
-      <c r="CD5" s="18"/>
-      <c r="CE5" s="18"/>
-      <c r="CF5" s="18"/>
-      <c r="CG5" s="18"/>
-      <c r="CH5" s="18"/>
-      <c r="CI5" s="18"/>
-      <c r="CJ5" s="18"/>
-      <c r="CK5" s="18"/>
-      <c r="CL5" s="19"/>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="2"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{956EFD9A-0444-473E-BD83-6FED68498CDD}">
-  <sheetPr codeName="Sheet73"/>
-  <dimension ref="A1:CL5"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
-  <cols>
-    <col min="1" max="90" width="1.75" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
-      <c r="W1" s="1"/>
-      <c r="X1" s="1"/>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="1"/>
-      <c r="AA1" s="1"/>
-      <c r="AB1" s="1"/>
-      <c r="AC1" s="1"/>
-      <c r="AD1" s="1"/>
-      <c r="AE1" s="1"/>
-      <c r="AF1" s="1"/>
-      <c r="AG1" s="1"/>
-      <c r="AH1" s="1"/>
-      <c r="AI1" s="1"/>
-      <c r="AJ1" s="1"/>
-      <c r="AK1" s="1"/>
-      <c r="AL1" s="1"/>
-      <c r="AM1" s="1"/>
-      <c r="AN1" s="1"/>
-      <c r="AO1" s="1"/>
-      <c r="AP1" s="1"/>
-      <c r="AQ1" s="1"/>
-      <c r="AR1" s="1"/>
-      <c r="AS1" s="1"/>
-      <c r="AT1" s="1"/>
-      <c r="AU1" s="1"/>
-      <c r="AV1" s="1"/>
-      <c r="AW1" s="1"/>
-      <c r="AX1" s="1"/>
-      <c r="AY1" s="1"/>
-      <c r="AZ1" s="1"/>
-      <c r="BA1" s="1"/>
-      <c r="BB1" s="1"/>
-      <c r="BC1" s="1"/>
-      <c r="BD1" s="1"/>
-      <c r="BE1" s="1"/>
-      <c r="BF1" s="1"/>
-      <c r="BG1" s="1"/>
-      <c r="BH1" s="1"/>
-      <c r="BI1" s="1"/>
-      <c r="BJ1" s="1"/>
-      <c r="BK1" s="1"/>
-      <c r="BL1" s="1"/>
-      <c r="BM1" s="1"/>
-      <c r="BN1" s="1"/>
-      <c r="BO1" s="1"/>
-      <c r="BP1" s="1"/>
-      <c r="BQ1" s="1"/>
-      <c r="BR1" s="1"/>
-      <c r="BS1" s="1"/>
-      <c r="BT1" s="1"/>
-      <c r="BU1" s="1"/>
-      <c r="BV1" s="1"/>
-      <c r="BW1" s="1"/>
-      <c r="BX1" s="1"/>
-      <c r="BY1" s="1"/>
-      <c r="BZ1" s="1"/>
-      <c r="CA1" s="1"/>
-      <c r="CB1" s="1"/>
-      <c r="CC1" s="1"/>
-      <c r="CD1" s="1"/>
-      <c r="CE1" s="1"/>
-      <c r="CF1" s="1"/>
-      <c r="CG1" s="1"/>
-      <c r="CH1" s="1"/>
-      <c r="CI1" s="1"/>
-      <c r="CJ1" s="1"/>
-      <c r="CK1" s="1"/>
-      <c r="CL1" s="1"/>
-    </row>
-    <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
-      <c r="R2" s="1"/>
-      <c r="S2" s="1"/>
-      <c r="T2" s="1"/>
-      <c r="U2" s="1"/>
-      <c r="V2" s="1"/>
-      <c r="W2" s="1"/>
-      <c r="X2" s="1"/>
-      <c r="Y2" s="1"/>
-      <c r="Z2" s="1"/>
-      <c r="AA2" s="1"/>
-      <c r="AB2" s="1"/>
-      <c r="AC2" s="1"/>
-      <c r="AD2" s="1"/>
-      <c r="AE2" s="1"/>
-      <c r="AF2" s="1"/>
-      <c r="AG2" s="1"/>
-      <c r="AH2" s="1"/>
-      <c r="AI2" s="1"/>
-      <c r="AJ2" s="1"/>
-      <c r="AK2" s="1"/>
-      <c r="AL2" s="1"/>
-      <c r="AM2" s="1"/>
-      <c r="AN2" s="1"/>
-      <c r="AO2" s="1"/>
-      <c r="AP2" s="1"/>
-      <c r="AQ2" s="1"/>
-      <c r="AR2" s="1"/>
-      <c r="AS2" s="1"/>
-      <c r="AT2" s="1"/>
-      <c r="AU2" s="1"/>
-      <c r="AV2" s="1"/>
-      <c r="AW2" s="1"/>
-      <c r="AX2" s="1"/>
-      <c r="AY2" s="1"/>
-      <c r="AZ2" s="1"/>
-      <c r="BA2" s="1"/>
-      <c r="BB2" s="1"/>
-      <c r="BC2" s="1"/>
-      <c r="BD2" s="1"/>
-      <c r="BE2" s="1"/>
-      <c r="BF2" s="1"/>
-      <c r="BG2" s="1"/>
-      <c r="BH2" s="1"/>
-      <c r="BI2" s="1"/>
-      <c r="BJ2" s="1"/>
-      <c r="BK2" s="1"/>
-      <c r="BL2" s="1"/>
-      <c r="BM2" s="1"/>
-      <c r="BN2" s="1"/>
-      <c r="BO2" s="1"/>
-      <c r="BP2" s="1"/>
-      <c r="BQ2" s="1"/>
-      <c r="BR2" s="1"/>
-      <c r="BS2" s="1"/>
-      <c r="BT2" s="1"/>
-      <c r="BU2" s="1"/>
-      <c r="BV2" s="1"/>
-      <c r="BW2" s="1"/>
-      <c r="BX2" s="1"/>
-      <c r="BY2" s="1"/>
-      <c r="BZ2" s="1"/>
-      <c r="CA2" s="1"/>
-      <c r="CB2" s="1"/>
-      <c r="CC2" s="1"/>
-      <c r="CD2" s="1"/>
-      <c r="CE2" s="1"/>
-      <c r="CF2" s="1"/>
-      <c r="CG2" s="1"/>
-      <c r="CH2" s="1"/>
-      <c r="CI2" s="1"/>
-      <c r="CJ2" s="1"/>
-      <c r="CK2" s="1"/>
-      <c r="CL2" s="1"/>
-    </row>
-    <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="24" t="s">
-        <v>124</v>
-      </c>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="25" t="s">
-        <v>7</v>
-      </c>
-      <c r="P3" s="6"/>
-      <c r="Q3" s="25" t="s">
-        <v>206</v>
-      </c>
-      <c r="R3" s="6"/>
-      <c r="S3" s="6"/>
-      <c r="T3" s="6"/>
-      <c r="U3" s="6"/>
-      <c r="V3" s="6"/>
-      <c r="W3" s="6"/>
-      <c r="X3" s="6"/>
-      <c r="Y3" s="6"/>
-      <c r="Z3" s="6"/>
-      <c r="AA3" s="6"/>
-      <c r="AB3" s="6"/>
-      <c r="AC3" s="6"/>
-      <c r="AD3" s="6"/>
-      <c r="AE3" s="6"/>
-      <c r="AF3" s="6"/>
-      <c r="AG3" s="6"/>
-      <c r="AH3" s="6"/>
-      <c r="AI3" s="6"/>
-      <c r="AJ3" s="6"/>
-      <c r="AK3" s="6"/>
-      <c r="AL3" s="6"/>
-      <c r="AM3" s="6"/>
-      <c r="AN3" s="6"/>
-      <c r="AO3" s="6"/>
-      <c r="AP3" s="6"/>
-      <c r="AQ3" s="6"/>
-      <c r="AR3" s="6"/>
-      <c r="AS3" s="6"/>
-      <c r="AT3" s="6"/>
-      <c r="AU3" s="6"/>
-      <c r="AV3" s="6"/>
-      <c r="AW3" s="6"/>
-      <c r="AX3" s="6"/>
-      <c r="AY3" s="6"/>
-      <c r="AZ3" s="6"/>
-      <c r="BA3" s="6"/>
-      <c r="BB3" s="6"/>
-      <c r="BC3" s="6"/>
-      <c r="BD3" s="6"/>
-      <c r="BE3" s="6"/>
-      <c r="BF3" s="6"/>
-      <c r="BG3" s="6"/>
-      <c r="BH3" s="6"/>
-      <c r="BI3" s="6"/>
-      <c r="BJ3" s="6"/>
-      <c r="BK3" s="6"/>
-      <c r="BL3" s="6"/>
-      <c r="BM3" s="6"/>
-      <c r="BN3" s="6"/>
-      <c r="BO3" s="6"/>
-      <c r="BP3" s="6"/>
-      <c r="BQ3" s="6"/>
-      <c r="BR3" s="6"/>
-      <c r="BS3" s="6"/>
-      <c r="BT3" s="6"/>
-      <c r="BU3" s="6"/>
-      <c r="BV3" s="6"/>
-      <c r="BW3" s="6"/>
-      <c r="BX3" s="6"/>
-      <c r="BY3" s="6"/>
-      <c r="BZ3" s="6"/>
-      <c r="CA3" s="6"/>
-      <c r="CB3" s="6"/>
-      <c r="CC3" s="6"/>
-      <c r="CD3" s="6"/>
-      <c r="CE3" s="6"/>
-      <c r="CF3" s="6"/>
-      <c r="CG3" s="6"/>
-      <c r="CH3" s="6"/>
-      <c r="CI3" s="6"/>
-      <c r="CJ3" s="6"/>
-      <c r="CK3" s="6"/>
-      <c r="CL3" s="7"/>
-    </row>
-    <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="8"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="27" t="s">
-        <v>207</v>
-      </c>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="U4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="3"/>
-      <c r="Y4" s="3"/>
-      <c r="Z4" s="3"/>
-      <c r="AA4" s="3"/>
-      <c r="AB4" s="3"/>
-      <c r="AC4" s="3"/>
-      <c r="AD4" s="3"/>
-      <c r="AE4" s="3"/>
-      <c r="AF4" s="3"/>
-      <c r="AG4" s="3"/>
-      <c r="AH4" s="3"/>
-      <c r="AI4" s="3"/>
-      <c r="AJ4" s="3"/>
-      <c r="AK4" s="3"/>
-      <c r="AL4" s="3"/>
-      <c r="AM4" s="3"/>
-      <c r="AN4" s="3"/>
-      <c r="AO4" s="3"/>
-      <c r="AP4" s="3"/>
-      <c r="AQ4" s="3"/>
-      <c r="AR4" s="3"/>
-      <c r="AS4" s="3"/>
-      <c r="AT4" s="3"/>
-      <c r="AU4" s="3"/>
-      <c r="AV4" s="3"/>
-      <c r="AW4" s="3"/>
-      <c r="AX4" s="3"/>
-      <c r="AY4" s="3"/>
-      <c r="AZ4" s="3"/>
-      <c r="BA4" s="3"/>
-      <c r="BB4" s="3"/>
-      <c r="BC4" s="3"/>
-      <c r="BD4" s="3"/>
-      <c r="BE4" s="3"/>
-      <c r="BF4" s="3"/>
-      <c r="BG4" s="3"/>
-      <c r="BH4" s="3"/>
-      <c r="BI4" s="3"/>
-      <c r="BJ4" s="3"/>
-      <c r="BK4" s="3"/>
-      <c r="BL4" s="3"/>
-      <c r="BM4" s="3"/>
-      <c r="BN4" s="3"/>
-      <c r="BO4" s="3"/>
-      <c r="BP4" s="3"/>
-      <c r="BQ4" s="3"/>
-      <c r="BR4" s="3"/>
-      <c r="BS4" s="3"/>
-      <c r="BT4" s="3"/>
-      <c r="BU4" s="3"/>
-      <c r="BV4" s="3"/>
-      <c r="BW4" s="3"/>
-      <c r="BX4" s="3"/>
-      <c r="BY4" s="3"/>
-      <c r="BZ4" s="3"/>
-      <c r="CA4" s="3"/>
-      <c r="CB4" s="3"/>
-      <c r="CC4" s="3"/>
-      <c r="CD4" s="3"/>
-      <c r="CE4" s="3"/>
-      <c r="CF4" s="3"/>
-      <c r="CG4" s="3"/>
-      <c r="CH4" s="3"/>
-      <c r="CI4" s="3"/>
-      <c r="CJ4" s="3"/>
-      <c r="CK4" s="3"/>
-      <c r="CL4" s="10"/>
-    </row>
-    <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="20" t="s">
-        <v>4</v>
-      </c>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="18"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="18"/>
-      <c r="N5" s="18"/>
-      <c r="O5" s="29" t="s">
-        <v>5</v>
-      </c>
-      <c r="P5" s="18"/>
-      <c r="Q5" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="R5" s="18"/>
-      <c r="S5" s="18"/>
-      <c r="T5" s="18"/>
-      <c r="U5" s="18"/>
-      <c r="V5" s="18"/>
-      <c r="W5" s="18"/>
-      <c r="X5" s="18"/>
-      <c r="Y5" s="18"/>
-      <c r="Z5" s="18"/>
-      <c r="AA5" s="18"/>
-      <c r="AB5" s="18"/>
-      <c r="AC5" s="18"/>
-      <c r="AD5" s="18"/>
-      <c r="AE5" s="18"/>
-      <c r="AF5" s="18"/>
-      <c r="AG5" s="18"/>
-      <c r="AH5" s="18"/>
-      <c r="AI5" s="18"/>
-      <c r="AJ5" s="18"/>
-      <c r="AK5" s="18"/>
-      <c r="AL5" s="18"/>
-      <c r="AM5" s="18"/>
-      <c r="AN5" s="18"/>
-      <c r="AO5" s="18"/>
-      <c r="AP5" s="18"/>
-      <c r="AQ5" s="18"/>
-      <c r="AR5" s="18"/>
-      <c r="AS5" s="18"/>
-      <c r="AT5" s="18"/>
-      <c r="AU5" s="18"/>
-      <c r="AV5" s="18"/>
-      <c r="AW5" s="18"/>
-      <c r="AX5" s="18"/>
-      <c r="AY5" s="18"/>
-      <c r="AZ5" s="18"/>
-      <c r="BA5" s="18"/>
-      <c r="BB5" s="18"/>
-      <c r="BC5" s="18"/>
-      <c r="BD5" s="18"/>
-      <c r="BE5" s="18"/>
-      <c r="BF5" s="18"/>
-      <c r="BG5" s="18"/>
-      <c r="BH5" s="18"/>
-      <c r="BI5" s="18"/>
-      <c r="BJ5" s="18"/>
-      <c r="BK5" s="18"/>
-      <c r="BL5" s="18"/>
-      <c r="BM5" s="18"/>
-      <c r="BN5" s="18"/>
-      <c r="BO5" s="18"/>
-      <c r="BP5" s="18"/>
-      <c r="BQ5" s="18"/>
-      <c r="BR5" s="18"/>
-      <c r="BS5" s="18"/>
-      <c r="BT5" s="18"/>
-      <c r="BU5" s="18"/>
-      <c r="BV5" s="18"/>
-      <c r="BW5" s="18"/>
-      <c r="BX5" s="18"/>
-      <c r="BY5" s="18"/>
-      <c r="BZ5" s="18"/>
-      <c r="CA5" s="18"/>
-      <c r="CB5" s="18"/>
-      <c r="CC5" s="18"/>
-      <c r="CD5" s="18"/>
-      <c r="CE5" s="18"/>
-      <c r="CF5" s="18"/>
-      <c r="CG5" s="18"/>
-      <c r="CH5" s="18"/>
-      <c r="CI5" s="18"/>
-      <c r="CJ5" s="18"/>
-      <c r="CK5" s="18"/>
-      <c r="CL5" s="19"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>

</xml_diff>

<commit_message>
feat: align nested CASE and ELSE output
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Macro\SqlAnalyzerFormatter-feature\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50AB106C-FE30-4410-8F28-9CD23F9819AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B62837AA-51D3-46AA-A936-126797549C31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-8340" windowWidth="29040" windowHeight="15720" firstSheet="58" activeTab="59" xr2:uid="{41A826B0-B2A2-4DC8-9B04-8EFBE807DC37}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="58" activeTab="59" xr2:uid="{41A826B0-B2A2-4DC8-9B04-8EFBE807DC37}"/>
   </bookViews>
   <sheets>
     <sheet name="SEL-064" sheetId="66" r:id="rId1"/>
@@ -99,7 +99,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1279" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1277" uniqueCount="277">
   <si>
     <t>ソートキー2</t>
   </si>
@@ -437,31 +437,10 @@
     <t>CASE結果 = 1</t>
   </si>
   <si>
-    <t>それ以外 → 0</t>
-  </si>
-  <si>
     <t>v.ユーザーID</t>
   </si>
   <si>
     <t>v.氏名</t>
-  </si>
-  <si>
-    <t>user_category</t>
-  </si>
-  <si>
-    <t>tb1.状態 = 'ACTIVE' → CASE</t>
-  </si>
-  <si>
-    <t>tb1.ランクコード = 'VIP' → '優良'</t>
-  </si>
-  <si>
-    <t>それ以外 → '通常'</t>
-  </si>
-  <si>
-    <t>tb1.状態 = 'LOCKED' → '停止'</t>
-  </si>
-  <si>
-    <t>それ以外 → '無効'</t>
   </si>
   <si>
     <t>amount_band</t>
@@ -470,19 +449,10 @@
     <t>tb1.金額 &gt;= 10000 → 'HIGH'</t>
   </si>
   <si>
-    <t>それ以外 → 'NORMAL'</t>
-  </si>
-  <si>
     <t>CASE結果</t>
   </si>
   <si>
     <t>tb1.状態 = 'ACTIVE' → 0</t>
-  </si>
-  <si>
-    <t>tb1.状態 = 'LOCKED' → 1</t>
-  </si>
-  <si>
-    <t>それ以外 → 2</t>
   </si>
   <si>
     <t>tb1.削除日時</t>
@@ -549,9 +519,6 @@
   </si>
   <si>
     <t>COUNT(tb2.注文ID) &gt; 0 → 'STANDARD'</t>
-  </si>
-  <si>
-    <t>それ以外 → 'NONE'</t>
   </si>
   <si>
     <t>created_at</t>
@@ -698,31 +665,16 @@
     <t>tb1.状態 = 'ACTIVE' → 'ENABLED'</t>
   </si>
   <si>
-    <t>それ以外 → CASE</t>
-  </si>
-  <si>
-    <t>tb1.削除日時 IS NULL → 'PENDING'</t>
-  </si>
-  <si>
-    <t>それ以外 → 'DISABLED'</t>
-  </si>
-  <si>
     <t>eligible_flag</t>
   </si>
   <si>
     <t>tb1.削除日時 IS NULL</t>
   </si>
   <si>
-    <t>それ以外 → 'INACTIVE'</t>
-  </si>
-  <si>
     <t>@active = 1 → 'ACTIVE'</t>
   </si>
   <si>
     <t>@all_rows = 1 → 100</t>
-  </si>
-  <si>
-    <t>それ以外 → 10</t>
   </si>
   <si>
     <t>offset (CASE結果) rows fetch next 20 rows only</t>
@@ -833,12 +785,6 @@
     <t>COUNT(tb1.ユーザーID) &gt;= 10</t>
   </si>
   <si>
-    <t>status_name</t>
-  </si>
-  <si>
-    <t>tb1.状態 = 'ACTIVE' → '有効'</t>
-  </si>
-  <si>
     <t>tb1.状態 = @status</t>
   </si>
   <si>
@@ -929,20 +875,68 @@
     <t>参照テーブル: ユーザー[tb1]、注文[tb2]、SQ1</t>
   </si>
   <si>
+    <t>ELSE → 'NORMAL'</t>
+  </si>
+  <si>
+    <t>ELSE → 0</t>
+  </si>
+  <si>
+    <t>ELSE → 'NONE'</t>
+  </si>
+  <si>
+    <t>ELSE → 10</t>
+  </si>
+  <si>
+    <t>status_name</t>
+  </si>
+  <si>
+    <t>tb1.状態 = 'ACTIVE' → '有効'</t>
+  </si>
+  <si>
+    <t>ELSE → '無効'</t>
+  </si>
+  <si>
+    <t>user_category</t>
+  </si>
+  <si>
+    <t>tb1.状態 = 'ACTIVE' → tb1.ランクコード = 'VIP' → '優良'</t>
+  </si>
+  <si>
+    <t>ELSE → '通常'</t>
+  </si>
+  <si>
+    <t>tb1.状態 = 'LOCKED' → '停止'</t>
+  </si>
+  <si>
+    <t>tb1.状態 = 'LOCKED' → 1</t>
+  </si>
+  <si>
+    <t>ELSE → 2</t>
+  </si>
+  <si>
     <t>tb1.削除日時 IS NULL → 1</t>
   </si>
   <si>
     <t>tb1.作成日時 &gt;= DATEADD(day, -7, @base_date) → 1</t>
   </si>
   <si>
+    <t>ELSE → tb1.削除日時 IS NULL → 'PENDING'</t>
+  </si>
+  <si>
+    <t>ELSE → 'DISABLED'</t>
+  </si>
+  <si>
     <t>tb1.有効区分 = 1 → 'ACTIVE'</t>
+  </si>
+  <si>
+    <t>ELSE → 'INACTIVE'</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -965,21 +959,6 @@
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="游ゴシック"/>
-      <family val="3"/>
-      <charset val="128"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="游ゴシック"/>
-      <family val="3"/>
-      <charset val="128"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1001,7 +980,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -1126,22 +1105,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1247,37 +1217,7 @@
     <xf numFmtId="49" fontId="1" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1697,7 +1637,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1813,7 +1753,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -2173,7 +2113,7 @@
     </row>
     <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="22" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -2285,7 +2225,7 @@
       <c r="O8" s="18"/>
       <c r="P8" s="18"/>
       <c r="Q8" s="29" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
       <c r="R8" s="18"/>
       <c r="S8" s="18"/>
@@ -2884,7 +2824,7 @@
       </c>
       <c r="P6" s="6"/>
       <c r="Q6" s="25" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="R6" s="6"/>
       <c r="S6" s="6"/>
@@ -2903,7 +2843,7 @@
         <v>7</v>
       </c>
       <c r="AF6" s="25" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="AG6" s="6"/>
       <c r="AH6" s="6"/>
@@ -2997,7 +2937,7 @@
       <c r="AD7" s="3"/>
       <c r="AE7" s="3"/>
       <c r="AF7" s="27" t="s">
-        <v>126</v>
+        <v>269</v>
       </c>
       <c r="AG7" s="3"/>
       <c r="AH7" s="3"/>
@@ -3091,7 +3031,7 @@
       <c r="AD8" s="3"/>
       <c r="AE8" s="3"/>
       <c r="AF8" s="27" t="s">
-        <v>127</v>
+        <v>270</v>
       </c>
       <c r="AG8" s="3"/>
       <c r="AH8" s="3"/>
@@ -3477,7 +3417,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -3496,7 +3436,7 @@
         <v>7</v>
       </c>
       <c r="AF3" s="25" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="AG3" s="6"/>
       <c r="AH3" s="6"/>
@@ -3590,7 +3530,7 @@
       <c r="AD4" s="3"/>
       <c r="AE4" s="3"/>
       <c r="AF4" s="27" t="s">
-        <v>123</v>
+        <v>258</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -3777,7 +3717,7 @@
       </c>
       <c r="P6" s="6"/>
       <c r="Q6" s="25" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="R6" s="6"/>
       <c r="S6" s="6"/>
@@ -3796,7 +3736,7 @@
         <v>7</v>
       </c>
       <c r="AF6" s="25" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="AG6" s="6"/>
       <c r="AH6" s="6"/>
@@ -3890,7 +3830,7 @@
       <c r="AD7" s="14"/>
       <c r="AE7" s="14"/>
       <c r="AF7" s="30" t="s">
-        <v>123</v>
+        <v>258</v>
       </c>
       <c r="AG7" s="14"/>
       <c r="AH7" s="14"/>
@@ -3960,7 +3900,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{586B5BAC-40C5-4C4A-A485-0654F1D1B942}">
   <sheetPr codeName="Sheet12"/>
-  <dimension ref="A1:CL8"/>
+  <dimension ref="A1:CL7"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="90" width="1.75" customWidth="1"/>
@@ -4276,7 +4216,7 @@
       </c>
       <c r="P4" s="3"/>
       <c r="Q4" s="27" t="s">
-        <v>115</v>
+        <v>265</v>
       </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
@@ -4295,7 +4235,7 @@
         <v>7</v>
       </c>
       <c r="AF4" s="27" t="s">
-        <v>116</v>
+        <v>266</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -4391,7 +4331,7 @@
       <c r="AF5" s="3"/>
       <c r="AG5" s="3"/>
       <c r="AH5" s="27" t="s">
-        <v>117</v>
+        <v>267</v>
       </c>
       <c r="AI5" s="3"/>
       <c r="AJ5" s="3"/>
@@ -4482,11 +4422,11 @@
       <c r="AC6" s="3"/>
       <c r="AD6" s="3"/>
       <c r="AE6" s="3"/>
-      <c r="AF6" s="3"/>
+      <c r="AF6" s="27" t="s">
+        <v>268</v>
+      </c>
       <c r="AG6" s="3"/>
-      <c r="AH6" s="27" t="s">
-        <v>118</v>
-      </c>
+      <c r="AH6" s="3"/>
       <c r="AI6" s="3"/>
       <c r="AJ6" s="3"/>
       <c r="AK6" s="3"/>
@@ -4545,192 +4485,98 @@
       <c r="CL6" s="10"/>
     </row>
     <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="8"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3"/>
-      <c r="P7" s="3"/>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="3"/>
-      <c r="S7" s="3"/>
-      <c r="T7" s="3"/>
-      <c r="U7" s="3"/>
-      <c r="V7" s="3"/>
-      <c r="W7" s="3"/>
-      <c r="X7" s="3"/>
-      <c r="Y7" s="3"/>
-      <c r="Z7" s="3"/>
-      <c r="AA7" s="3"/>
-      <c r="AB7" s="3"/>
-      <c r="AC7" s="3"/>
-      <c r="AD7" s="3"/>
-      <c r="AE7" s="3"/>
-      <c r="AF7" s="27" t="s">
-        <v>119</v>
-      </c>
-      <c r="AG7" s="3"/>
-      <c r="AH7" s="3"/>
-      <c r="AI7" s="3"/>
-      <c r="AJ7" s="3"/>
-      <c r="AK7" s="3"/>
-      <c r="AL7" s="3"/>
-      <c r="AM7" s="3"/>
-      <c r="AN7" s="3"/>
-      <c r="AO7" s="3"/>
-      <c r="AP7" s="3"/>
-      <c r="AQ7" s="3"/>
-      <c r="AR7" s="3"/>
-      <c r="AS7" s="3"/>
-      <c r="AT7" s="3"/>
-      <c r="AU7" s="3"/>
-      <c r="AV7" s="3"/>
-      <c r="AW7" s="3"/>
-      <c r="AX7" s="3"/>
-      <c r="AY7" s="3"/>
-      <c r="AZ7" s="3"/>
-      <c r="BA7" s="3"/>
-      <c r="BB7" s="3"/>
-      <c r="BC7" s="3"/>
-      <c r="BD7" s="3"/>
-      <c r="BE7" s="3"/>
-      <c r="BF7" s="3"/>
-      <c r="BG7" s="3"/>
-      <c r="BH7" s="3"/>
-      <c r="BI7" s="3"/>
-      <c r="BJ7" s="3"/>
-      <c r="BK7" s="3"/>
-      <c r="BL7" s="3"/>
-      <c r="BM7" s="3"/>
-      <c r="BN7" s="3"/>
-      <c r="BO7" s="3"/>
-      <c r="BP7" s="3"/>
-      <c r="BQ7" s="3"/>
-      <c r="BR7" s="3"/>
-      <c r="BS7" s="3"/>
-      <c r="BT7" s="3"/>
-      <c r="BU7" s="3"/>
-      <c r="BV7" s="3"/>
-      <c r="BW7" s="3"/>
-      <c r="BX7" s="3"/>
-      <c r="BY7" s="3"/>
-      <c r="BZ7" s="3"/>
-      <c r="CA7" s="3"/>
-      <c r="CB7" s="3"/>
-      <c r="CC7" s="3"/>
-      <c r="CD7" s="3"/>
-      <c r="CE7" s="3"/>
-      <c r="CF7" s="3"/>
-      <c r="CG7" s="3"/>
-      <c r="CH7" s="3"/>
-      <c r="CI7" s="3"/>
-      <c r="CJ7" s="3"/>
-      <c r="CK7" s="3"/>
-      <c r="CL7" s="10"/>
-    </row>
-    <row r="8" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="11"/>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
-      <c r="L8" s="14"/>
-      <c r="M8" s="14"/>
-      <c r="N8" s="14"/>
-      <c r="O8" s="14"/>
-      <c r="P8" s="14"/>
-      <c r="Q8" s="14"/>
-      <c r="R8" s="14"/>
-      <c r="S8" s="14"/>
-      <c r="T8" s="14"/>
-      <c r="U8" s="14"/>
-      <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
-      <c r="X8" s="14"/>
-      <c r="Y8" s="14"/>
-      <c r="Z8" s="14"/>
-      <c r="AA8" s="14"/>
-      <c r="AB8" s="14"/>
-      <c r="AC8" s="14"/>
-      <c r="AD8" s="14"/>
-      <c r="AE8" s="14"/>
-      <c r="AF8" s="30" t="s">
-        <v>120</v>
-      </c>
-      <c r="AG8" s="14"/>
-      <c r="AH8" s="14"/>
-      <c r="AI8" s="14"/>
-      <c r="AJ8" s="14"/>
-      <c r="AK8" s="14"/>
-      <c r="AL8" s="14"/>
-      <c r="AM8" s="14"/>
-      <c r="AN8" s="14"/>
-      <c r="AO8" s="14"/>
-      <c r="AP8" s="14"/>
-      <c r="AQ8" s="14"/>
-      <c r="AR8" s="14"/>
-      <c r="AS8" s="14"/>
-      <c r="AT8" s="14"/>
-      <c r="AU8" s="14"/>
-      <c r="AV8" s="14"/>
-      <c r="AW8" s="14"/>
-      <c r="AX8" s="14"/>
-      <c r="AY8" s="14"/>
-      <c r="AZ8" s="14"/>
-      <c r="BA8" s="14"/>
-      <c r="BB8" s="14"/>
-      <c r="BC8" s="14"/>
-      <c r="BD8" s="14"/>
-      <c r="BE8" s="14"/>
-      <c r="BF8" s="14"/>
-      <c r="BG8" s="14"/>
-      <c r="BH8" s="14"/>
-      <c r="BI8" s="14"/>
-      <c r="BJ8" s="14"/>
-      <c r="BK8" s="14"/>
-      <c r="BL8" s="14"/>
-      <c r="BM8" s="14"/>
-      <c r="BN8" s="14"/>
-      <c r="BO8" s="14"/>
-      <c r="BP8" s="14"/>
-      <c r="BQ8" s="14"/>
-      <c r="BR8" s="14"/>
-      <c r="BS8" s="14"/>
-      <c r="BT8" s="14"/>
-      <c r="BU8" s="14"/>
-      <c r="BV8" s="14"/>
-      <c r="BW8" s="14"/>
-      <c r="BX8" s="14"/>
-      <c r="BY8" s="14"/>
-      <c r="BZ8" s="14"/>
-      <c r="CA8" s="14"/>
-      <c r="CB8" s="14"/>
-      <c r="CC8" s="14"/>
-      <c r="CD8" s="14"/>
-      <c r="CE8" s="14"/>
-      <c r="CF8" s="14"/>
-      <c r="CG8" s="14"/>
-      <c r="CH8" s="14"/>
-      <c r="CI8" s="14"/>
-      <c r="CJ8" s="14"/>
-      <c r="CK8" s="14"/>
-      <c r="CL8" s="15"/>
+      <c r="A7" s="11"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="14"/>
+      <c r="M7" s="14"/>
+      <c r="N7" s="14"/>
+      <c r="O7" s="14"/>
+      <c r="P7" s="14"/>
+      <c r="Q7" s="14"/>
+      <c r="R7" s="14"/>
+      <c r="S7" s="14"/>
+      <c r="T7" s="14"/>
+      <c r="U7" s="14"/>
+      <c r="V7" s="14"/>
+      <c r="W7" s="14"/>
+      <c r="X7" s="14"/>
+      <c r="Y7" s="14"/>
+      <c r="Z7" s="14"/>
+      <c r="AA7" s="14"/>
+      <c r="AB7" s="14"/>
+      <c r="AC7" s="14"/>
+      <c r="AD7" s="14"/>
+      <c r="AE7" s="14"/>
+      <c r="AF7" s="30" t="s">
+        <v>264</v>
+      </c>
+      <c r="AG7" s="14"/>
+      <c r="AH7" s="14"/>
+      <c r="AI7" s="14"/>
+      <c r="AJ7" s="14"/>
+      <c r="AK7" s="14"/>
+      <c r="AL7" s="14"/>
+      <c r="AM7" s="14"/>
+      <c r="AN7" s="14"/>
+      <c r="AO7" s="14"/>
+      <c r="AP7" s="14"/>
+      <c r="AQ7" s="14"/>
+      <c r="AR7" s="14"/>
+      <c r="AS7" s="14"/>
+      <c r="AT7" s="14"/>
+      <c r="AU7" s="14"/>
+      <c r="AV7" s="14"/>
+      <c r="AW7" s="14"/>
+      <c r="AX7" s="14"/>
+      <c r="AY7" s="14"/>
+      <c r="AZ7" s="14"/>
+      <c r="BA7" s="14"/>
+      <c r="BB7" s="14"/>
+      <c r="BC7" s="14"/>
+      <c r="BD7" s="14"/>
+      <c r="BE7" s="14"/>
+      <c r="BF7" s="14"/>
+      <c r="BG7" s="14"/>
+      <c r="BH7" s="14"/>
+      <c r="BI7" s="14"/>
+      <c r="BJ7" s="14"/>
+      <c r="BK7" s="14"/>
+      <c r="BL7" s="14"/>
+      <c r="BM7" s="14"/>
+      <c r="BN7" s="14"/>
+      <c r="BO7" s="14"/>
+      <c r="BP7" s="14"/>
+      <c r="BQ7" s="14"/>
+      <c r="BR7" s="14"/>
+      <c r="BS7" s="14"/>
+      <c r="BT7" s="14"/>
+      <c r="BU7" s="14"/>
+      <c r="BV7" s="14"/>
+      <c r="BW7" s="14"/>
+      <c r="BX7" s="14"/>
+      <c r="BY7" s="14"/>
+      <c r="BZ7" s="14"/>
+      <c r="CA7" s="14"/>
+      <c r="CB7" s="14"/>
+      <c r="CC7" s="14"/>
+      <c r="CD7" s="14"/>
+      <c r="CE7" s="14"/>
+      <c r="CF7" s="14"/>
+      <c r="CG7" s="14"/>
+      <c r="CH7" s="14"/>
+      <c r="CI7" s="14"/>
+      <c r="CJ7" s="14"/>
+      <c r="CK7" s="14"/>
+      <c r="CL7" s="15"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>
@@ -4843,7 +4689,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>262</v>
+        <v>244</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -4959,7 +4805,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -5057,7 +4903,7 @@
       </c>
       <c r="P4" s="3"/>
       <c r="Q4" s="27" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
@@ -5157,7 +5003,7 @@
       </c>
       <c r="P5" s="18"/>
       <c r="Q5" s="29" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="R5" s="18"/>
       <c r="S5" s="18"/>
@@ -5344,7 +5190,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -5536,7 +5382,7 @@
     </row>
     <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="31" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="B4" s="14"/>
       <c r="C4" s="14"/>
@@ -5632,7 +5478,7 @@
     </row>
     <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="24" t="s">
-        <v>260</v>
+        <v>242</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -5746,7 +5592,7 @@
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
       <c r="Q6" s="25" t="s">
-        <v>218</v>
+        <v>202</v>
       </c>
       <c r="R6" s="6"/>
       <c r="S6" s="6"/>
@@ -5936,7 +5782,7 @@
       <c r="O8" s="18"/>
       <c r="P8" s="18"/>
       <c r="Q8" s="29" t="s">
-        <v>261</v>
+        <v>243</v>
       </c>
       <c r="R8" s="18"/>
       <c r="S8" s="18"/>
@@ -6235,7 +6081,7 @@
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>258</v>
+        <v>240</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -6331,7 +6177,7 @@
       <c r="O4" s="14"/>
       <c r="P4" s="14"/>
       <c r="Q4" s="30" t="s">
-        <v>259</v>
+        <v>241</v>
       </c>
       <c r="R4" s="14"/>
       <c r="S4" s="14"/>
@@ -6518,7 +6364,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>254</v>
+        <v>236</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -6906,7 +6752,7 @@
     </row>
     <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="25" t="s">
-        <v>255</v>
+        <v>237</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -7022,7 +6868,7 @@
       </c>
       <c r="P7" s="6"/>
       <c r="Q7" s="25" t="s">
-        <v>256</v>
+        <v>238</v>
       </c>
       <c r="R7" s="6"/>
       <c r="S7" s="6"/>
@@ -7120,7 +6966,7 @@
       </c>
       <c r="P8" s="3"/>
       <c r="Q8" s="27" t="s">
-        <v>224</v>
+        <v>208</v>
       </c>
       <c r="R8" s="3"/>
       <c r="S8" s="3"/>
@@ -7216,7 +7062,7 @@
       <c r="O9" s="18"/>
       <c r="P9" s="18"/>
       <c r="Q9" s="29" t="s">
-        <v>257</v>
+        <v>239</v>
       </c>
       <c r="R9" s="18"/>
       <c r="S9" s="18"/>
@@ -7309,7 +7155,7 @@
   <sheetData>
     <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="22" t="s">
-        <v>250</v>
+        <v>232</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7713,7 +7559,7 @@
       <c r="O5" s="18"/>
       <c r="P5" s="18"/>
       <c r="Q5" s="29" t="s">
-        <v>246</v>
+        <v>228</v>
       </c>
       <c r="R5" s="18"/>
       <c r="S5" s="18"/>
@@ -7977,7 +7823,7 @@
     </row>
     <row r="8" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="22" t="s">
-        <v>251</v>
+        <v>233</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -8093,7 +7939,7 @@
       </c>
       <c r="P9" s="6"/>
       <c r="Q9" s="25" t="s">
-        <v>252</v>
+        <v>234</v>
       </c>
       <c r="R9" s="6"/>
       <c r="S9" s="6"/>
@@ -8191,7 +8037,7 @@
       </c>
       <c r="P10" s="14"/>
       <c r="Q10" s="30" t="s">
-        <v>253</v>
+        <v>235</v>
       </c>
       <c r="R10" s="14"/>
       <c r="S10" s="14"/>
@@ -8378,7 +8224,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -8494,7 +8340,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -8590,7 +8436,7 @@
       <c r="O4" s="18"/>
       <c r="P4" s="18"/>
       <c r="Q4" s="29" t="s">
-        <v>241</v>
+        <v>225</v>
       </c>
       <c r="R4" s="18"/>
       <c r="S4" s="18"/>
@@ -8854,7 +8700,7 @@
     </row>
     <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="22" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -9164,7 +9010,7 @@
       <c r="O10" s="18"/>
       <c r="P10" s="18"/>
       <c r="Q10" s="29" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="R10" s="18"/>
       <c r="S10" s="18"/>
@@ -9651,7 +9497,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="24" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="H5" s="6"/>
       <c r="I5" s="6"/>
@@ -9663,7 +9509,7 @@
       <c r="O5" s="6"/>
       <c r="P5" s="6"/>
       <c r="Q5" s="25" t="s">
-        <v>246</v>
+        <v>228</v>
       </c>
       <c r="R5" s="6"/>
       <c r="S5" s="6"/>
@@ -9759,7 +9605,7 @@
       </c>
       <c r="P6" s="3"/>
       <c r="Q6" s="27" t="s">
-        <v>247</v>
+        <v>229</v>
       </c>
       <c r="R6" s="3"/>
       <c r="S6" s="3"/>
@@ -9843,7 +9689,7 @@
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="26" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
@@ -9937,7 +9783,7 @@
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="26" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
@@ -9947,11 +9793,11 @@
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>
       <c r="O8" s="27" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="P8" s="3"/>
       <c r="Q8" s="27" t="s">
-        <v>248</v>
+        <v>230</v>
       </c>
       <c r="R8" s="3"/>
       <c r="S8" s="3"/>
@@ -10043,11 +9889,11 @@
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
       <c r="O9" s="27" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="P9" s="3"/>
       <c r="Q9" s="27" t="s">
-        <v>249</v>
+        <v>231</v>
       </c>
       <c r="R9" s="3"/>
       <c r="S9" s="3"/>
@@ -10131,7 +9977,7 @@
       <c r="E10" s="12"/>
       <c r="F10" s="12"/>
       <c r="G10" s="31" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="H10" s="14"/>
       <c r="I10" s="14"/>
@@ -10234,7 +10080,7 @@
   <sheetData>
     <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="22" t="s">
-        <v>171</v>
+        <v>160</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -10328,7 +10174,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>172</v>
+        <v>161</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -10444,7 +10290,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -10542,7 +10388,7 @@
       </c>
       <c r="P4" s="3"/>
       <c r="Q4" s="27" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
@@ -10561,7 +10407,7 @@
         <v>7</v>
       </c>
       <c r="AF4" s="27" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -10646,7 +10492,7 @@
       </c>
       <c r="P5" s="18"/>
       <c r="Q5" s="29" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="R5" s="18"/>
       <c r="S5" s="18"/>
@@ -10910,7 +10756,7 @@
     </row>
     <row r="8" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="22" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -11102,7 +10948,7 @@
     </row>
     <row r="10" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="26" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -11122,7 +10968,7 @@
       <c r="Q10" s="3"/>
       <c r="R10" s="3"/>
       <c r="S10" s="26" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="T10" s="3"/>
       <c r="U10" s="3"/>
@@ -11216,7 +11062,7 @@
       <c r="O11" s="6"/>
       <c r="P11" s="6"/>
       <c r="Q11" s="25" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="R11" s="6"/>
       <c r="S11" s="6"/>
@@ -11310,7 +11156,7 @@
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
       <c r="Q12" s="27" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="R12" s="3"/>
       <c r="S12" s="3"/>
@@ -11807,7 +11653,7 @@
       </c>
       <c r="P4" s="3"/>
       <c r="Q4" s="27" t="s">
-        <v>244</v>
+        <v>262</v>
       </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
@@ -11826,7 +11672,7 @@
         <v>7</v>
       </c>
       <c r="AF4" s="27" t="s">
-        <v>245</v>
+        <v>263</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -11920,7 +11766,7 @@
       <c r="AD5" s="14"/>
       <c r="AE5" s="14"/>
       <c r="AF5" s="30" t="s">
-        <v>120</v>
+        <v>264</v>
       </c>
       <c r="AG5" s="14"/>
       <c r="AH5" s="14"/>
@@ -12325,7 +12171,7 @@
         <v>7</v>
       </c>
       <c r="AF4" s="27" t="s">
-        <v>242</v>
+        <v>226</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -12506,7 +12352,7 @@
       <c r="O6" s="18"/>
       <c r="P6" s="18"/>
       <c r="Q6" s="29" t="s">
-        <v>243</v>
+        <v>227</v>
       </c>
       <c r="R6" s="18"/>
       <c r="S6" s="18"/>
@@ -12926,7 +12772,7 @@
         <v>7</v>
       </c>
       <c r="AF4" s="27" t="s">
-        <v>242</v>
+        <v>226</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -16505,7 +16351,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -16607,7 +16453,7 @@
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="24" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
@@ -16717,7 +16563,7 @@
       </c>
       <c r="P4" s="6"/>
       <c r="Q4" s="25" t="s">
-        <v>166</v>
+        <v>155</v>
       </c>
       <c r="R4" s="6"/>
       <c r="S4" s="6"/>
@@ -16913,7 +16759,7 @@
       </c>
       <c r="P6" s="18"/>
       <c r="Q6" s="29" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
       <c r="R6" s="18"/>
       <c r="S6" s="18"/>
@@ -17177,7 +17023,7 @@
     </row>
     <row r="9" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="22" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -17369,7 +17215,7 @@
     </row>
     <row r="11" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="26" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -17389,7 +17235,7 @@
       <c r="Q11" s="3"/>
       <c r="R11" s="3"/>
       <c r="S11" s="26" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="T11" s="3"/>
       <c r="U11" s="3"/>
@@ -18973,7 +18819,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -19285,7 +19131,7 @@
       </c>
       <c r="P5" s="3"/>
       <c r="Q5" s="27" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
@@ -19383,7 +19229,7 @@
       </c>
       <c r="P6" s="3"/>
       <c r="Q6" s="27" t="s">
-        <v>166</v>
+        <v>155</v>
       </c>
       <c r="R6" s="3"/>
       <c r="S6" s="3"/>
@@ -19669,7 +19515,7 @@
       <c r="O9" s="14"/>
       <c r="P9" s="14"/>
       <c r="Q9" s="30" t="s">
-        <v>241</v>
+        <v>225</v>
       </c>
       <c r="R9" s="14"/>
       <c r="S9" s="14"/>
@@ -22502,7 +22348,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -22732,7 +22578,7 @@
       <c r="AI4" s="14"/>
       <c r="AJ4" s="14"/>
       <c r="AK4" s="31" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="AL4" s="14"/>
       <c r="AM4" s="14"/>
@@ -22790,7 +22636,7 @@
     </row>
     <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="20" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="B5" s="18"/>
       <c r="C5" s="18"/>
@@ -22828,7 +22674,7 @@
       <c r="AI5" s="18"/>
       <c r="AJ5" s="18"/>
       <c r="AK5" s="20" t="s">
-        <v>163</v>
+        <v>152</v>
       </c>
       <c r="AL5" s="18"/>
       <c r="AM5" s="18"/>
@@ -22886,7 +22732,7 @@
     </row>
     <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="20" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="B6" s="18"/>
       <c r="C6" s="18"/>
@@ -22924,7 +22770,7 @@
       <c r="AI6" s="18"/>
       <c r="AJ6" s="18"/>
       <c r="AK6" s="33" t="s">
-        <v>164</v>
+        <v>153</v>
       </c>
       <c r="AL6" s="18"/>
       <c r="AM6" s="18"/>
@@ -25554,7 +25400,7 @@
         <v>7</v>
       </c>
       <c r="AF4" s="27" t="s">
-        <v>238</v>
+        <v>222</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -25637,7 +25483,7 @@
       </c>
       <c r="P5" s="14"/>
       <c r="Q5" s="30" t="s">
-        <v>239</v>
+        <v>223</v>
       </c>
       <c r="R5" s="14"/>
       <c r="S5" s="14"/>
@@ -25656,7 +25502,7 @@
         <v>7</v>
       </c>
       <c r="AF5" s="30" t="s">
-        <v>240</v>
+        <v>224</v>
       </c>
       <c r="AG5" s="14"/>
       <c r="AH5" s="14"/>
@@ -26042,7 +25888,7 @@
       </c>
       <c r="P4" s="3"/>
       <c r="Q4" s="27" t="s">
-        <v>234</v>
+        <v>218</v>
       </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
@@ -26061,7 +25907,7 @@
         <v>7</v>
       </c>
       <c r="AF4" s="27" t="s">
-        <v>235</v>
+        <v>219</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -26144,7 +25990,7 @@
       </c>
       <c r="P5" s="14"/>
       <c r="Q5" s="30" t="s">
-        <v>236</v>
+        <v>220</v>
       </c>
       <c r="R5" s="14"/>
       <c r="S5" s="14"/>
@@ -26163,7 +26009,7 @@
         <v>7</v>
       </c>
       <c r="AF5" s="30" t="s">
-        <v>237</v>
+        <v>221</v>
       </c>
       <c r="AG5" s="14"/>
       <c r="AH5" s="14"/>
@@ -26549,7 +26395,7 @@
       </c>
       <c r="P4" s="14"/>
       <c r="Q4" s="30" t="s">
-        <v>232</v>
+        <v>216</v>
       </c>
       <c r="R4" s="14"/>
       <c r="S4" s="14"/>
@@ -26568,7 +26414,7 @@
         <v>7</v>
       </c>
       <c r="AF4" s="30" t="s">
-        <v>233</v>
+        <v>217</v>
       </c>
       <c r="AG4" s="14"/>
       <c r="AH4" s="14"/>
@@ -27050,7 +26896,7 @@
       <c r="O5" s="18"/>
       <c r="P5" s="18"/>
       <c r="Q5" s="29" t="s">
-        <v>231</v>
+        <v>215</v>
       </c>
       <c r="R5" s="18"/>
       <c r="S5" s="18"/>
@@ -27353,7 +27199,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>229</v>
+        <v>213</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -27372,7 +27218,7 @@
         <v>7</v>
       </c>
       <c r="AF3" s="25" t="s">
-        <v>230</v>
+        <v>214</v>
       </c>
       <c r="AG3" s="6"/>
       <c r="AH3" s="6"/>
@@ -27758,7 +27604,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>227</v>
+        <v>211</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -27777,7 +27623,7 @@
         <v>7</v>
       </c>
       <c r="AF3" s="25" t="s">
-        <v>228</v>
+        <v>212</v>
       </c>
       <c r="AG3" s="6"/>
       <c r="AH3" s="6"/>
@@ -28141,7 +27987,7 @@
     </row>
     <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="23" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -28149,7 +27995,7 @@
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="24" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
@@ -28546,7 +28392,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>223</v>
+        <v>207</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -28858,7 +28704,7 @@
       </c>
       <c r="P5" s="3"/>
       <c r="Q5" s="27" t="s">
-        <v>224</v>
+        <v>208</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
@@ -28954,7 +28800,7 @@
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
       <c r="Q6" s="25" t="s">
-        <v>225</v>
+        <v>209</v>
       </c>
       <c r="R6" s="6"/>
       <c r="S6" s="6"/>
@@ -29048,7 +28894,7 @@
       <c r="O7" s="14"/>
       <c r="P7" s="14"/>
       <c r="Q7" s="30" t="s">
-        <v>226</v>
+        <v>210</v>
       </c>
       <c r="R7" s="14"/>
       <c r="S7" s="14"/>
@@ -29235,7 +29081,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>219</v>
+        <v>203</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -29449,7 +29295,7 @@
       </c>
       <c r="P4" s="3"/>
       <c r="Q4" s="27" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
@@ -29547,7 +29393,7 @@
       </c>
       <c r="P5" s="3"/>
       <c r="Q5" s="27" t="s">
-        <v>220</v>
+        <v>204</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
@@ -29643,7 +29489,7 @@
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
       <c r="Q6" s="25" t="s">
-        <v>218</v>
+        <v>202</v>
       </c>
       <c r="R6" s="6"/>
       <c r="S6" s="6"/>
@@ -29831,7 +29677,7 @@
       <c r="O8" s="3"/>
       <c r="P8" s="3"/>
       <c r="Q8" s="27" t="s">
-        <v>221</v>
+        <v>205</v>
       </c>
       <c r="R8" s="3"/>
       <c r="S8" s="3"/>
@@ -29925,7 +29771,7 @@
       <c r="O9" s="14"/>
       <c r="P9" s="14"/>
       <c r="Q9" s="30" t="s">
-        <v>222</v>
+        <v>206</v>
       </c>
       <c r="R9" s="14"/>
       <c r="S9" s="14"/>
@@ -30112,7 +29958,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -30424,7 +30270,7 @@
       </c>
       <c r="P5" s="3"/>
       <c r="Q5" s="27" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
@@ -30801,7 +30647,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -31113,7 +30959,7 @@
       </c>
       <c r="P5" s="3"/>
       <c r="Q5" s="27" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
@@ -31209,7 +31055,7 @@
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
       <c r="Q6" s="25" t="s">
-        <v>218</v>
+        <v>202</v>
       </c>
       <c r="R6" s="6"/>
       <c r="S6" s="6"/>
@@ -31902,7 +31748,7 @@
       </c>
       <c r="P6" s="14"/>
       <c r="Q6" s="30" t="s">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="R6" s="14"/>
       <c r="S6" s="14"/>
@@ -32403,7 +32249,7 @@
       </c>
       <c r="P5" s="18"/>
       <c r="Q5" s="29" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="R5" s="18"/>
       <c r="S5" s="18"/>
@@ -33401,7 +33247,7 @@
       <c r="O5" s="6"/>
       <c r="P5" s="6"/>
       <c r="Q5" s="25" t="s">
-        <v>214</v>
+        <v>198</v>
       </c>
       <c r="R5" s="6"/>
       <c r="S5" s="6"/>
@@ -33497,7 +33343,7 @@
       <c r="O6" s="14"/>
       <c r="P6" s="14"/>
       <c r="Q6" s="30" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="R6" s="14"/>
       <c r="S6" s="14"/>
@@ -33994,7 +33840,7 @@
       <c r="O5" s="18"/>
       <c r="P5" s="18"/>
       <c r="Q5" s="29" t="s">
-        <v>214</v>
+        <v>198</v>
       </c>
       <c r="R5" s="18"/>
       <c r="S5" s="18"/>
@@ -34582,7 +34428,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>274</v>
+        <v>256</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -35058,7 +34904,7 @@
     </row>
     <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="22" t="s">
-        <v>275</v>
+        <v>257</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -35174,7 +35020,7 @@
       </c>
       <c r="P8" s="6"/>
       <c r="Q8" s="25" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="R8" s="6"/>
       <c r="S8" s="6"/>
@@ -36127,7 +35973,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -36243,7 +36089,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -36339,7 +36185,7 @@
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
       <c r="Q4" s="25" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="R4" s="6"/>
       <c r="S4" s="6"/>
@@ -36435,7 +36281,7 @@
       <c r="O5" s="14"/>
       <c r="P5" s="14"/>
       <c r="Q5" s="30" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
       <c r="R5" s="14"/>
       <c r="S5" s="14"/>
@@ -36699,7 +36545,7 @@
     </row>
     <row r="8" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="22" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -36891,7 +36737,7 @@
     </row>
     <row r="10" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="26" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -36929,7 +36775,7 @@
       <c r="AI10" s="3"/>
       <c r="AJ10" s="3"/>
       <c r="AK10" s="34" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
       <c r="AL10" s="3"/>
       <c r="AM10" s="3"/>
@@ -37005,7 +36851,7 @@
       <c r="O11" s="18"/>
       <c r="P11" s="18"/>
       <c r="Q11" s="29" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
       <c r="R11" s="18"/>
       <c r="S11" s="18"/>
@@ -37192,7 +37038,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -37308,7 +37154,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -37327,7 +37173,7 @@
         <v>7</v>
       </c>
       <c r="AF3" s="25" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
       <c r="AG3" s="6"/>
       <c r="AH3" s="6"/>
@@ -37672,7 +37518,7 @@
     </row>
     <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="22" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -37864,7 +37710,7 @@
     </row>
     <row r="9" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="26" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -37902,7 +37748,7 @@
       <c r="AI9" s="3"/>
       <c r="AJ9" s="3"/>
       <c r="AK9" s="34" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="AL9" s="3"/>
       <c r="AM9" s="3"/>
@@ -37978,7 +37824,7 @@
       <c r="O10" s="18"/>
       <c r="P10" s="18"/>
       <c r="Q10" s="29" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="R10" s="18"/>
       <c r="S10" s="18"/>
@@ -38165,7 +38011,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -38281,7 +38127,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -38377,7 +38223,7 @@
       <c r="O4" s="18"/>
       <c r="P4" s="18"/>
       <c r="Q4" s="29" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="R4" s="18"/>
       <c r="S4" s="18"/>
@@ -38641,7 +38487,7 @@
     </row>
     <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="22" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -38833,7 +38679,7 @@
     </row>
     <row r="9" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="26" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -38871,7 +38717,7 @@
       <c r="AI9" s="3"/>
       <c r="AJ9" s="3"/>
       <c r="AK9" s="34" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="AL9" s="3"/>
       <c r="AM9" s="3"/>
@@ -38947,7 +38793,7 @@
       <c r="O10" s="18"/>
       <c r="P10" s="18"/>
       <c r="Q10" s="29" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="R10" s="18"/>
       <c r="S10" s="18"/>
@@ -39659,7 +39505,7 @@
       </c>
       <c r="AG7" s="3"/>
       <c r="AH7" s="27" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="AI7" s="3"/>
       <c r="AJ7" s="3"/>
@@ -39753,7 +39599,7 @@
       <c r="AF8" s="3"/>
       <c r="AG8" s="3"/>
       <c r="AH8" s="27" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="AI8" s="3"/>
       <c r="AJ8" s="3"/>
@@ -39849,7 +39695,7 @@
       </c>
       <c r="AG9" s="3"/>
       <c r="AH9" s="27" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="AI9" s="3"/>
       <c r="AJ9" s="3"/>
@@ -39941,7 +39787,7 @@
       <c r="AD10" s="14"/>
       <c r="AE10" s="14"/>
       <c r="AF10" s="30" t="s">
-        <v>112</v>
+        <v>259</v>
       </c>
       <c r="AG10" s="14"/>
       <c r="AH10" s="14"/>
@@ -40215,7 +40061,7 @@
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="24" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
@@ -40229,7 +40075,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -40323,7 +40169,7 @@
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="27" t="s">
-        <v>207</v>
+        <v>261</v>
       </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
@@ -40610,7 +40456,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -40802,7 +40648,7 @@
     </row>
     <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="31" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="B4" s="14"/>
       <c r="C4" s="14"/>
@@ -40822,7 +40668,7 @@
       <c r="Q4" s="14"/>
       <c r="R4" s="14"/>
       <c r="S4" s="31" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="T4" s="14"/>
       <c r="U4" s="14"/>
@@ -40844,7 +40690,7 @@
       </c>
       <c r="AJ4" s="14"/>
       <c r="AK4" s="31" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="AL4" s="14"/>
       <c r="AM4" s="14"/>
@@ -40938,7 +40784,7 @@
       <c r="AI5" s="18"/>
       <c r="AJ5" s="18"/>
       <c r="AK5" s="20" t="s">
-        <v>204</v>
+        <v>276</v>
       </c>
       <c r="AL5" s="18"/>
       <c r="AM5" s="18"/>
@@ -41003,7 +40849,7 @@
 <file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30AB51C2-4CAF-40D2-90C0-05BD312EBAB8}">
   <sheetPr codeName="Sheet71"/>
-  <dimension ref="A1:CL10"/>
+  <dimension ref="A1:CL6"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="90" width="1.75" customWidth="1"/>
@@ -41198,125 +41044,125 @@
       <c r="CL2" s="1"/>
     </row>
     <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
-      <c r="M3" s="16"/>
-      <c r="N3" s="16"/>
-      <c r="O3" s="16"/>
-      <c r="P3" s="16"/>
-      <c r="Q3" s="16"/>
-      <c r="R3" s="16"/>
-      <c r="S3" s="28" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+      <c r="S3" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="T3" s="16"/>
-      <c r="U3" s="16"/>
-      <c r="V3" s="16"/>
-      <c r="W3" s="16"/>
-      <c r="X3" s="16"/>
-      <c r="Y3" s="16"/>
-      <c r="Z3" s="16"/>
-      <c r="AA3" s="16"/>
-      <c r="AB3" s="16"/>
-      <c r="AC3" s="16"/>
-      <c r="AD3" s="16"/>
-      <c r="AE3" s="16"/>
-      <c r="AF3" s="16"/>
-      <c r="AG3" s="16"/>
-      <c r="AH3" s="16"/>
-      <c r="AI3" s="16"/>
-      <c r="AJ3" s="16"/>
-      <c r="AK3" s="28" t="s">
+      <c r="T3" s="4"/>
+      <c r="U3" s="4"/>
+      <c r="V3" s="4"/>
+      <c r="W3" s="4"/>
+      <c r="X3" s="4"/>
+      <c r="Y3" s="4"/>
+      <c r="Z3" s="4"/>
+      <c r="AA3" s="4"/>
+      <c r="AB3" s="4"/>
+      <c r="AC3" s="4"/>
+      <c r="AD3" s="4"/>
+      <c r="AE3" s="4"/>
+      <c r="AF3" s="4"/>
+      <c r="AG3" s="4"/>
+      <c r="AH3" s="4"/>
+      <c r="AI3" s="4"/>
+      <c r="AJ3" s="4"/>
+      <c r="AK3" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="AL3" s="16"/>
-      <c r="AM3" s="16"/>
-      <c r="AN3" s="16"/>
-      <c r="AO3" s="16"/>
-      <c r="AP3" s="16"/>
-      <c r="AQ3" s="16"/>
-      <c r="AR3" s="16"/>
-      <c r="AS3" s="16"/>
-      <c r="AT3" s="16"/>
-      <c r="AU3" s="16"/>
-      <c r="AV3" s="16"/>
-      <c r="AW3" s="16"/>
-      <c r="AX3" s="16"/>
-      <c r="AY3" s="16"/>
-      <c r="AZ3" s="16"/>
-      <c r="BA3" s="16"/>
-      <c r="BB3" s="16"/>
-      <c r="BC3" s="16"/>
-      <c r="BD3" s="16"/>
-      <c r="BE3" s="16"/>
-      <c r="BF3" s="16"/>
-      <c r="BG3" s="16"/>
-      <c r="BH3" s="16"/>
-      <c r="BI3" s="16"/>
-      <c r="BJ3" s="16"/>
-      <c r="BK3" s="16"/>
-      <c r="BL3" s="16"/>
-      <c r="BM3" s="16"/>
-      <c r="BN3" s="16"/>
-      <c r="BO3" s="16"/>
-      <c r="BP3" s="16"/>
-      <c r="BQ3" s="16"/>
-      <c r="BR3" s="16"/>
-      <c r="BS3" s="16"/>
-      <c r="BT3" s="16"/>
-      <c r="BU3" s="16"/>
-      <c r="BV3" s="16"/>
-      <c r="BW3" s="16"/>
-      <c r="BX3" s="16"/>
-      <c r="BY3" s="16"/>
-      <c r="BZ3" s="16"/>
-      <c r="CA3" s="16"/>
-      <c r="CB3" s="16"/>
-      <c r="CC3" s="16"/>
-      <c r="CD3" s="16"/>
-      <c r="CE3" s="16"/>
-      <c r="CF3" s="16"/>
-      <c r="CG3" s="16"/>
-      <c r="CH3" s="16"/>
-      <c r="CI3" s="16"/>
-      <c r="CJ3" s="16"/>
-      <c r="CK3" s="16"/>
-      <c r="CL3" s="21"/>
+      <c r="AL3" s="4"/>
+      <c r="AM3" s="4"/>
+      <c r="AN3" s="4"/>
+      <c r="AO3" s="4"/>
+      <c r="AP3" s="4"/>
+      <c r="AQ3" s="4"/>
+      <c r="AR3" s="4"/>
+      <c r="AS3" s="4"/>
+      <c r="AT3" s="4"/>
+      <c r="AU3" s="4"/>
+      <c r="AV3" s="4"/>
+      <c r="AW3" s="4"/>
+      <c r="AX3" s="4"/>
+      <c r="AY3" s="4"/>
+      <c r="AZ3" s="4"/>
+      <c r="BA3" s="4"/>
+      <c r="BB3" s="4"/>
+      <c r="BC3" s="4"/>
+      <c r="BD3" s="4"/>
+      <c r="BE3" s="4"/>
+      <c r="BF3" s="4"/>
+      <c r="BG3" s="4"/>
+      <c r="BH3" s="4"/>
+      <c r="BI3" s="4"/>
+      <c r="BJ3" s="4"/>
+      <c r="BK3" s="4"/>
+      <c r="BL3" s="4"/>
+      <c r="BM3" s="4"/>
+      <c r="BN3" s="4"/>
+      <c r="BO3" s="4"/>
+      <c r="BP3" s="4"/>
+      <c r="BQ3" s="4"/>
+      <c r="BR3" s="4"/>
+      <c r="BS3" s="4"/>
+      <c r="BT3" s="4"/>
+      <c r="BU3" s="4"/>
+      <c r="BV3" s="4"/>
+      <c r="BW3" s="4"/>
+      <c r="BX3" s="4"/>
+      <c r="BY3" s="4"/>
+      <c r="BZ3" s="4"/>
+      <c r="CA3" s="4"/>
+      <c r="CB3" s="4"/>
+      <c r="CC3" s="4"/>
+      <c r="CD3" s="4"/>
+      <c r="CE3" s="4"/>
+      <c r="CF3" s="4"/>
+      <c r="CG3" s="4"/>
+      <c r="CH3" s="4"/>
+      <c r="CI3" s="4"/>
+      <c r="CJ3" s="4"/>
+      <c r="CK3" s="4"/>
+      <c r="CL3" s="35"/>
     </row>
     <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="26" t="s">
-        <v>159</v>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="35"/>
+      <c r="A4" s="24" t="s">
+        <v>148</v>
+      </c>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="5"/>
       <c r="T4" s="6"/>
       <c r="U4" s="6"/>
       <c r="V4" s="6"/>
@@ -41332,68 +41178,68 @@
       <c r="AF4" s="6"/>
       <c r="AG4" s="6"/>
       <c r="AH4" s="6"/>
-      <c r="AI4" s="36"/>
-      <c r="AJ4" s="7"/>
-      <c r="AK4" s="27" t="s">
-        <v>124</v>
-      </c>
-      <c r="AL4" s="1"/>
-      <c r="AM4" s="1"/>
-      <c r="AN4" s="1"/>
-      <c r="AO4" s="1"/>
-      <c r="AP4" s="1"/>
-      <c r="AQ4" s="1"/>
-      <c r="AR4" s="1"/>
-      <c r="AS4" s="1"/>
-      <c r="AT4" s="1"/>
-      <c r="AU4" s="3"/>
-      <c r="AV4" s="3"/>
-      <c r="AW4" s="1"/>
-      <c r="AX4" s="1"/>
+      <c r="AI4" s="6"/>
+      <c r="AJ4" s="6"/>
+      <c r="AK4" s="24" t="s">
+        <v>116</v>
+      </c>
+      <c r="AL4" s="6"/>
+      <c r="AM4" s="6"/>
+      <c r="AN4" s="6"/>
+      <c r="AO4" s="6"/>
+      <c r="AP4" s="6"/>
+      <c r="AQ4" s="6"/>
+      <c r="AR4" s="6"/>
+      <c r="AS4" s="6"/>
+      <c r="AT4" s="6"/>
+      <c r="AU4" s="6"/>
+      <c r="AV4" s="6"/>
+      <c r="AW4" s="6"/>
+      <c r="AX4" s="6"/>
       <c r="AY4" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="AZ4" s="3"/>
-      <c r="BA4" s="3"/>
-      <c r="BB4" s="27" t="s">
-        <v>203</v>
-      </c>
-      <c r="BC4" s="3"/>
-      <c r="BD4" s="3"/>
-      <c r="BE4" s="3"/>
-      <c r="BF4" s="3"/>
-      <c r="BG4" s="3"/>
-      <c r="BH4" s="3"/>
-      <c r="BI4" s="3"/>
-      <c r="BJ4" s="3"/>
-      <c r="BK4" s="3"/>
-      <c r="BL4" s="3"/>
-      <c r="BM4" s="3"/>
-      <c r="BN4" s="3"/>
-      <c r="BO4" s="3"/>
-      <c r="BP4" s="3"/>
-      <c r="BQ4" s="3"/>
-      <c r="BR4" s="3"/>
-      <c r="BS4" s="1"/>
-      <c r="BT4" s="1"/>
-      <c r="BU4" s="1"/>
-      <c r="BV4" s="1"/>
-      <c r="BW4" s="1"/>
-      <c r="BX4" s="1"/>
-      <c r="BY4" s="1"/>
-      <c r="BZ4" s="1"/>
-      <c r="CA4" s="1"/>
-      <c r="CB4" s="3"/>
-      <c r="CC4" s="3"/>
-      <c r="CD4" s="3"/>
-      <c r="CE4" s="3"/>
-      <c r="CF4" s="3"/>
-      <c r="CG4" s="3"/>
-      <c r="CH4" s="3"/>
-      <c r="CI4" s="3"/>
-      <c r="CJ4" s="3"/>
-      <c r="CK4" s="3"/>
-      <c r="CL4" s="10"/>
+      <c r="AZ4" s="6"/>
+      <c r="BA4" s="6"/>
+      <c r="BB4" s="25" t="s">
+        <v>189</v>
+      </c>
+      <c r="BC4" s="6"/>
+      <c r="BD4" s="6"/>
+      <c r="BE4" s="6"/>
+      <c r="BF4" s="6"/>
+      <c r="BG4" s="6"/>
+      <c r="BH4" s="6"/>
+      <c r="BI4" s="6"/>
+      <c r="BJ4" s="6"/>
+      <c r="BK4" s="6"/>
+      <c r="BL4" s="6"/>
+      <c r="BM4" s="6"/>
+      <c r="BN4" s="6"/>
+      <c r="BO4" s="6"/>
+      <c r="BP4" s="6"/>
+      <c r="BQ4" s="6"/>
+      <c r="BR4" s="6"/>
+      <c r="BS4" s="6"/>
+      <c r="BT4" s="6"/>
+      <c r="BU4" s="6"/>
+      <c r="BV4" s="6"/>
+      <c r="BW4" s="6"/>
+      <c r="BX4" s="6"/>
+      <c r="BY4" s="6"/>
+      <c r="BZ4" s="6"/>
+      <c r="CA4" s="6"/>
+      <c r="CB4" s="6"/>
+      <c r="CC4" s="6"/>
+      <c r="CD4" s="6"/>
+      <c r="CE4" s="6"/>
+      <c r="CF4" s="6"/>
+      <c r="CG4" s="6"/>
+      <c r="CH4" s="6"/>
+      <c r="CI4" s="6"/>
+      <c r="CJ4" s="6"/>
+      <c r="CK4" s="6"/>
+      <c r="CL4" s="7"/>
     </row>
     <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="9"/>
@@ -41431,28 +41277,28 @@
       <c r="AG5" s="3"/>
       <c r="AH5" s="3"/>
       <c r="AI5" s="3"/>
-      <c r="AJ5" s="10"/>
-      <c r="AK5" s="37"/>
-      <c r="AL5" s="1"/>
-      <c r="AM5" s="1"/>
-      <c r="AN5" s="1"/>
-      <c r="AO5" s="1"/>
-      <c r="AP5" s="1"/>
-      <c r="AQ5" s="1"/>
-      <c r="AR5" s="1"/>
-      <c r="AS5" s="1"/>
-      <c r="AT5" s="1"/>
+      <c r="AJ5" s="3"/>
+      <c r="AK5" s="9"/>
+      <c r="AL5" s="3"/>
+      <c r="AM5" s="3"/>
+      <c r="AN5" s="3"/>
+      <c r="AO5" s="3"/>
+      <c r="AP5" s="3"/>
+      <c r="AQ5" s="3"/>
+      <c r="AR5" s="3"/>
+      <c r="AS5" s="3"/>
+      <c r="AT5" s="3"/>
       <c r="AU5" s="3"/>
       <c r="AV5" s="3"/>
-      <c r="AW5" s="1"/>
-      <c r="AX5" s="1"/>
+      <c r="AW5" s="3"/>
+      <c r="AX5" s="3"/>
       <c r="AY5" s="3"/>
       <c r="AZ5" s="27" t="s">
         <v>86</v>
       </c>
       <c r="BA5" s="3"/>
       <c r="BB5" s="27" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="BC5" s="3"/>
       <c r="BD5" s="3"/>
@@ -41470,15 +41316,15 @@
       <c r="BP5" s="3"/>
       <c r="BQ5" s="3"/>
       <c r="BR5" s="3"/>
-      <c r="BS5" s="1"/>
-      <c r="BT5" s="1"/>
-      <c r="BU5" s="1"/>
-      <c r="BV5" s="1"/>
-      <c r="BW5" s="1"/>
-      <c r="BX5" s="1"/>
-      <c r="BY5" s="1"/>
-      <c r="BZ5" s="1"/>
-      <c r="CA5" s="1"/>
+      <c r="BS5" s="3"/>
+      <c r="BT5" s="3"/>
+      <c r="BU5" s="3"/>
+      <c r="BV5" s="3"/>
+      <c r="BW5" s="3"/>
+      <c r="BX5" s="3"/>
+      <c r="BY5" s="3"/>
+      <c r="BZ5" s="3"/>
+      <c r="CA5" s="3"/>
       <c r="CB5" s="3"/>
       <c r="CC5" s="3"/>
       <c r="CD5" s="3"/>
@@ -41527,27 +41373,27 @@
       <c r="AG6" s="14"/>
       <c r="AH6" s="14"/>
       <c r="AI6" s="14"/>
-      <c r="AJ6" s="15"/>
-      <c r="AK6" s="38"/>
-      <c r="AL6" s="39"/>
-      <c r="AM6" s="39"/>
-      <c r="AN6" s="39"/>
-      <c r="AO6" s="39"/>
-      <c r="AP6" s="39"/>
-      <c r="AQ6" s="39"/>
-      <c r="AR6" s="39"/>
-      <c r="AS6" s="39"/>
-      <c r="AT6" s="39"/>
-      <c r="AU6" s="40"/>
-      <c r="AV6" s="40"/>
-      <c r="AW6" s="41"/>
-      <c r="AX6" s="41"/>
-      <c r="AY6" s="40"/>
-      <c r="AZ6" s="42" t="s">
-        <v>204</v>
-      </c>
-      <c r="BA6" s="40"/>
-      <c r="BB6" s="40"/>
+      <c r="AJ6" s="14"/>
+      <c r="AK6" s="13"/>
+      <c r="AL6" s="14"/>
+      <c r="AM6" s="14"/>
+      <c r="AN6" s="14"/>
+      <c r="AO6" s="14"/>
+      <c r="AP6" s="14"/>
+      <c r="AQ6" s="14"/>
+      <c r="AR6" s="14"/>
+      <c r="AS6" s="14"/>
+      <c r="AT6" s="14"/>
+      <c r="AU6" s="14"/>
+      <c r="AV6" s="14"/>
+      <c r="AW6" s="14"/>
+      <c r="AX6" s="14"/>
+      <c r="AY6" s="14"/>
+      <c r="AZ6" s="30" t="s">
+        <v>276</v>
+      </c>
+      <c r="BA6" s="14"/>
+      <c r="BB6" s="14"/>
       <c r="BC6" s="14"/>
       <c r="BD6" s="14"/>
       <c r="BE6" s="14"/>
@@ -41564,17 +41410,17 @@
       <c r="BP6" s="14"/>
       <c r="BQ6" s="14"/>
       <c r="BR6" s="14"/>
-      <c r="BS6" s="41"/>
-      <c r="BT6" s="41"/>
-      <c r="BU6" s="41"/>
-      <c r="BV6" s="41"/>
-      <c r="BW6" s="41"/>
-      <c r="BX6" s="41"/>
-      <c r="BY6" s="41"/>
-      <c r="BZ6" s="41"/>
-      <c r="CA6" s="41"/>
-      <c r="CB6" s="40"/>
-      <c r="CC6" s="40"/>
+      <c r="BS6" s="14"/>
+      <c r="BT6" s="14"/>
+      <c r="BU6" s="14"/>
+      <c r="BV6" s="14"/>
+      <c r="BW6" s="14"/>
+      <c r="BX6" s="14"/>
+      <c r="BY6" s="14"/>
+      <c r="BZ6" s="14"/>
+      <c r="CA6" s="14"/>
+      <c r="CB6" s="14"/>
+      <c r="CC6" s="14"/>
       <c r="CD6" s="14"/>
       <c r="CE6" s="14"/>
       <c r="CF6" s="14"/>
@@ -41585,374 +41431,6 @@
       <c r="CK6" s="14"/>
       <c r="CL6" s="15"/>
     </row>
-    <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="43"/>
-      <c r="B7" s="43"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="43"/>
-      <c r="F7" s="43"/>
-      <c r="G7" s="43"/>
-      <c r="H7" s="43"/>
-      <c r="I7" s="43"/>
-      <c r="J7" s="43"/>
-      <c r="K7" s="43"/>
-      <c r="L7" s="43"/>
-      <c r="M7" s="43"/>
-      <c r="N7" s="43"/>
-      <c r="O7" s="43"/>
-      <c r="P7" s="43"/>
-      <c r="Q7" s="43"/>
-      <c r="R7" s="43"/>
-      <c r="S7" s="43"/>
-      <c r="T7" s="43"/>
-      <c r="U7" s="43"/>
-      <c r="V7" s="43"/>
-      <c r="W7" s="43"/>
-      <c r="X7" s="43"/>
-      <c r="Y7" s="43"/>
-      <c r="Z7" s="43"/>
-      <c r="AA7" s="43"/>
-      <c r="AB7" s="43"/>
-      <c r="AC7" s="43"/>
-      <c r="AD7" s="43"/>
-      <c r="AE7" s="43"/>
-      <c r="AF7" s="43"/>
-      <c r="AG7" s="43"/>
-      <c r="AH7" s="43"/>
-      <c r="AI7" s="43"/>
-      <c r="AJ7" s="43"/>
-      <c r="AK7" s="44"/>
-      <c r="AL7" s="45"/>
-      <c r="AM7" s="45"/>
-      <c r="AN7" s="45"/>
-      <c r="AO7" s="45"/>
-      <c r="AP7" s="45"/>
-      <c r="AQ7" s="45"/>
-      <c r="AR7" s="45"/>
-      <c r="AS7" s="45"/>
-      <c r="AT7" s="45"/>
-      <c r="AU7" s="45"/>
-      <c r="AV7" s="45"/>
-      <c r="AW7" s="45"/>
-      <c r="AX7" s="45"/>
-      <c r="AY7" s="44"/>
-      <c r="AZ7" s="44"/>
-      <c r="BA7" s="45"/>
-      <c r="BB7" s="43"/>
-      <c r="BC7" s="43"/>
-      <c r="BD7" s="43"/>
-      <c r="BE7" s="43"/>
-      <c r="BF7" s="43"/>
-      <c r="BG7" s="43"/>
-      <c r="BH7" s="43"/>
-      <c r="BI7" s="43"/>
-      <c r="BJ7" s="43"/>
-      <c r="BK7" s="43"/>
-      <c r="BL7" s="43"/>
-      <c r="BM7" s="43"/>
-      <c r="BN7" s="43"/>
-      <c r="BO7" s="43"/>
-      <c r="BP7" s="43"/>
-      <c r="BQ7" s="43"/>
-      <c r="BR7" s="43"/>
-      <c r="BS7" s="43"/>
-      <c r="BT7" s="43"/>
-      <c r="BU7" s="43"/>
-      <c r="BV7" s="43"/>
-      <c r="BW7" s="43"/>
-      <c r="BX7" s="43"/>
-      <c r="BY7" s="43"/>
-      <c r="BZ7" s="43"/>
-      <c r="CA7" s="43"/>
-      <c r="CB7" s="43"/>
-      <c r="CC7" s="43"/>
-      <c r="CD7" s="43"/>
-      <c r="CE7" s="43"/>
-      <c r="CF7" s="43"/>
-      <c r="CG7" s="43"/>
-      <c r="CH7" s="43"/>
-      <c r="CI7" s="43"/>
-      <c r="CJ7" s="43"/>
-      <c r="CK7" s="43"/>
-      <c r="CL7" s="43"/>
-    </row>
-    <row r="8" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="43"/>
-      <c r="B8" s="43"/>
-      <c r="C8" s="43"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="43"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="43"/>
-      <c r="H8" s="43"/>
-      <c r="I8" s="43"/>
-      <c r="J8" s="43"/>
-      <c r="K8" s="43"/>
-      <c r="L8" s="43"/>
-      <c r="M8" s="43"/>
-      <c r="N8" s="43"/>
-      <c r="O8" s="43"/>
-      <c r="P8" s="43"/>
-      <c r="Q8" s="43"/>
-      <c r="R8" s="43"/>
-      <c r="S8" s="43"/>
-      <c r="T8" s="43"/>
-      <c r="U8" s="43"/>
-      <c r="V8" s="43"/>
-      <c r="W8" s="43"/>
-      <c r="X8" s="43"/>
-      <c r="Y8" s="43"/>
-      <c r="Z8" s="43"/>
-      <c r="AA8" s="43"/>
-      <c r="AB8" s="43"/>
-      <c r="AC8" s="43"/>
-      <c r="AD8" s="43"/>
-      <c r="AE8" s="43"/>
-      <c r="AF8" s="43"/>
-      <c r="AG8" s="43"/>
-      <c r="AH8" s="43"/>
-      <c r="AI8" s="43"/>
-      <c r="AJ8" s="43"/>
-      <c r="AK8" s="43"/>
-      <c r="AL8" s="43"/>
-      <c r="AM8" s="43"/>
-      <c r="AN8" s="43"/>
-      <c r="AO8" s="43"/>
-      <c r="AP8" s="43"/>
-      <c r="AQ8" s="43"/>
-      <c r="AR8" s="43"/>
-      <c r="AS8" s="43"/>
-      <c r="AT8" s="43"/>
-      <c r="AU8" s="43"/>
-      <c r="AV8" s="43"/>
-      <c r="AW8" s="43"/>
-      <c r="AX8" s="43"/>
-      <c r="AY8" s="43"/>
-      <c r="AZ8" s="43"/>
-      <c r="BA8" s="43"/>
-      <c r="BB8" s="43"/>
-      <c r="BC8" s="43"/>
-      <c r="BD8" s="43"/>
-      <c r="BE8" s="43"/>
-      <c r="BF8" s="43"/>
-      <c r="BG8" s="43"/>
-      <c r="BH8" s="43"/>
-      <c r="BI8" s="43"/>
-      <c r="BJ8" s="43"/>
-      <c r="BK8" s="43"/>
-      <c r="BL8" s="43"/>
-      <c r="BM8" s="43"/>
-      <c r="BN8" s="43"/>
-      <c r="BO8" s="43"/>
-      <c r="BP8" s="43"/>
-      <c r="BQ8" s="43"/>
-      <c r="BR8" s="43"/>
-      <c r="BS8" s="43"/>
-      <c r="BT8" s="43"/>
-      <c r="BU8" s="43"/>
-      <c r="BV8" s="43"/>
-      <c r="BW8" s="43"/>
-      <c r="BX8" s="43"/>
-      <c r="BY8" s="43"/>
-      <c r="BZ8" s="43"/>
-      <c r="CA8" s="43"/>
-      <c r="CB8" s="43"/>
-      <c r="CC8" s="43"/>
-      <c r="CD8" s="43"/>
-      <c r="CE8" s="43"/>
-      <c r="CF8" s="43"/>
-      <c r="CG8" s="43"/>
-      <c r="CH8" s="43"/>
-      <c r="CI8" s="43"/>
-      <c r="CJ8" s="43"/>
-      <c r="CK8" s="43"/>
-      <c r="CL8" s="43"/>
-    </row>
-    <row r="9" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="43"/>
-      <c r="B9" s="43"/>
-      <c r="C9" s="43"/>
-      <c r="D9" s="43"/>
-      <c r="E9" s="43"/>
-      <c r="F9" s="43"/>
-      <c r="G9" s="43"/>
-      <c r="H9" s="43"/>
-      <c r="I9" s="43"/>
-      <c r="J9" s="43"/>
-      <c r="K9" s="43"/>
-      <c r="L9" s="43"/>
-      <c r="M9" s="43"/>
-      <c r="N9" s="43"/>
-      <c r="O9" s="43"/>
-      <c r="P9" s="43"/>
-      <c r="Q9" s="43"/>
-      <c r="R9" s="43"/>
-      <c r="S9" s="43"/>
-      <c r="T9" s="43"/>
-      <c r="U9" s="43"/>
-      <c r="V9" s="43"/>
-      <c r="W9" s="43"/>
-      <c r="X9" s="43"/>
-      <c r="Y9" s="43"/>
-      <c r="Z9" s="43"/>
-      <c r="AA9" s="43"/>
-      <c r="AB9" s="43"/>
-      <c r="AC9" s="43"/>
-      <c r="AD9" s="43"/>
-      <c r="AE9" s="43"/>
-      <c r="AF9" s="43"/>
-      <c r="AG9" s="43"/>
-      <c r="AH9" s="43"/>
-      <c r="AI9" s="43"/>
-      <c r="AJ9" s="43"/>
-      <c r="AK9" s="43"/>
-      <c r="AL9" s="43"/>
-      <c r="AM9" s="43"/>
-      <c r="AN9" s="43"/>
-      <c r="AO9" s="43"/>
-      <c r="AP9" s="43"/>
-      <c r="AQ9" s="43"/>
-      <c r="AR9" s="43"/>
-      <c r="AS9" s="43"/>
-      <c r="AT9" s="43"/>
-      <c r="AU9" s="43"/>
-      <c r="AV9" s="43"/>
-      <c r="AW9" s="43"/>
-      <c r="AX9" s="43"/>
-      <c r="AY9" s="43"/>
-      <c r="AZ9" s="43"/>
-      <c r="BA9" s="43"/>
-      <c r="BB9" s="43"/>
-      <c r="BC9" s="43"/>
-      <c r="BD9" s="43"/>
-      <c r="BE9" s="43"/>
-      <c r="BF9" s="43"/>
-      <c r="BG9" s="43"/>
-      <c r="BH9" s="43"/>
-      <c r="BI9" s="43"/>
-      <c r="BJ9" s="43"/>
-      <c r="BK9" s="43"/>
-      <c r="BL9" s="43"/>
-      <c r="BM9" s="43"/>
-      <c r="BN9" s="43"/>
-      <c r="BO9" s="43"/>
-      <c r="BP9" s="43"/>
-      <c r="BQ9" s="43"/>
-      <c r="BR9" s="43"/>
-      <c r="BS9" s="43"/>
-      <c r="BT9" s="43"/>
-      <c r="BU9" s="43"/>
-      <c r="BV9" s="43"/>
-      <c r="BW9" s="43"/>
-      <c r="BX9" s="43"/>
-      <c r="BY9" s="43"/>
-      <c r="BZ9" s="43"/>
-      <c r="CA9" s="43"/>
-      <c r="CB9" s="43"/>
-      <c r="CC9" s="43"/>
-      <c r="CD9" s="43"/>
-      <c r="CE9" s="43"/>
-      <c r="CF9" s="43"/>
-      <c r="CG9" s="43"/>
-      <c r="CH9" s="43"/>
-      <c r="CI9" s="43"/>
-      <c r="CJ9" s="43"/>
-      <c r="CK9" s="43"/>
-      <c r="CL9" s="43"/>
-    </row>
-    <row r="10" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="43"/>
-      <c r="B10" s="43"/>
-      <c r="C10" s="43"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="43"/>
-      <c r="F10" s="43"/>
-      <c r="G10" s="43"/>
-      <c r="H10" s="43"/>
-      <c r="I10" s="43"/>
-      <c r="J10" s="43"/>
-      <c r="K10" s="43"/>
-      <c r="L10" s="43"/>
-      <c r="M10" s="43"/>
-      <c r="N10" s="43"/>
-      <c r="O10" s="43"/>
-      <c r="P10" s="43"/>
-      <c r="Q10" s="43"/>
-      <c r="R10" s="43"/>
-      <c r="S10" s="43"/>
-      <c r="T10" s="43"/>
-      <c r="U10" s="43"/>
-      <c r="V10" s="43"/>
-      <c r="W10" s="43"/>
-      <c r="X10" s="43"/>
-      <c r="Y10" s="43"/>
-      <c r="Z10" s="43"/>
-      <c r="AA10" s="43"/>
-      <c r="AB10" s="43"/>
-      <c r="AC10" s="43"/>
-      <c r="AD10" s="43"/>
-      <c r="AE10" s="43"/>
-      <c r="AF10" s="43"/>
-      <c r="AG10" s="43"/>
-      <c r="AH10" s="43"/>
-      <c r="AI10" s="43"/>
-      <c r="AJ10" s="43"/>
-      <c r="AK10" s="43"/>
-      <c r="AL10" s="43"/>
-      <c r="AM10" s="43"/>
-      <c r="AN10" s="43"/>
-      <c r="AO10" s="43"/>
-      <c r="AP10" s="43"/>
-      <c r="AQ10" s="43"/>
-      <c r="AR10" s="43"/>
-      <c r="AS10" s="43"/>
-      <c r="AT10" s="43"/>
-      <c r="AU10" s="43"/>
-      <c r="AV10" s="43"/>
-      <c r="AW10" s="43"/>
-      <c r="AX10" s="43"/>
-      <c r="AY10" s="43"/>
-      <c r="AZ10" s="43"/>
-      <c r="BA10" s="43"/>
-      <c r="BB10" s="43"/>
-      <c r="BC10" s="43"/>
-      <c r="BD10" s="43"/>
-      <c r="BE10" s="43"/>
-      <c r="BF10" s="43"/>
-      <c r="BG10" s="43"/>
-      <c r="BH10" s="43"/>
-      <c r="BI10" s="43"/>
-      <c r="BJ10" s="43"/>
-      <c r="BK10" s="43"/>
-      <c r="BL10" s="43"/>
-      <c r="BM10" s="43"/>
-      <c r="BN10" s="43"/>
-      <c r="BO10" s="43"/>
-      <c r="BP10" s="43"/>
-      <c r="BQ10" s="43"/>
-      <c r="BR10" s="43"/>
-      <c r="BS10" s="43"/>
-      <c r="BT10" s="43"/>
-      <c r="BU10" s="43"/>
-      <c r="BV10" s="43"/>
-      <c r="BW10" s="43"/>
-      <c r="BX10" s="43"/>
-      <c r="BY10" s="43"/>
-      <c r="BZ10" s="43"/>
-      <c r="CA10" s="43"/>
-      <c r="CB10" s="43"/>
-      <c r="CC10" s="43"/>
-      <c r="CD10" s="43"/>
-      <c r="CE10" s="43"/>
-      <c r="CF10" s="43"/>
-      <c r="CG10" s="43"/>
-      <c r="CH10" s="43"/>
-      <c r="CI10" s="43"/>
-      <c r="CJ10" s="43"/>
-      <c r="CK10" s="43"/>
-      <c r="CL10" s="43"/>
-    </row>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -41962,7 +41440,7 @@
 <file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13E13F0B-BD68-436F-AC4B-0DE79A71FA29}">
   <sheetPr codeName="Sheet70"/>
-  <dimension ref="A1:CL10"/>
+  <dimension ref="A1:CL5"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="90" width="1.75" customWidth="1"/>
@@ -42180,7 +41658,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -42297,7 +41775,7 @@
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="27" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="AI4" s="3"/>
       <c r="AJ4" s="3"/>
@@ -42389,7 +41867,7 @@
       <c r="AD5" s="14"/>
       <c r="AE5" s="14"/>
       <c r="AF5" s="30" t="s">
-        <v>112</v>
+        <v>259</v>
       </c>
       <c r="AG5" s="14"/>
       <c r="AH5" s="14"/>
@@ -42450,11 +41928,6 @@
       <c r="CK5" s="14"/>
       <c r="CL5" s="15"/>
     </row>
-    <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="8" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="9" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="10" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -42464,7 +41937,7 @@
 <file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7D2694E-D810-4A8F-9E88-6BF6AE47836A}">
   <sheetPr codeName="Sheet69"/>
-  <dimension ref="A1:CL6"/>
+  <dimension ref="A1:CL5"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="90" width="1.75" customWidth="1"/>
@@ -42682,7 +42155,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -42701,7 +42174,7 @@
         <v>7</v>
       </c>
       <c r="AF3" s="25" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="AG3" s="6"/>
       <c r="AH3" s="6"/>
@@ -42795,7 +42268,7 @@
       <c r="AD4" s="3"/>
       <c r="AE4" s="3"/>
       <c r="AF4" s="27" t="s">
-        <v>199</v>
+        <v>273</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -42857,192 +42330,98 @@
       <c r="CL4" s="10"/>
     </row>
     <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="8"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="3"/>
-      <c r="O5" s="3"/>
-      <c r="P5" s="3"/>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="3"/>
-      <c r="S5" s="3"/>
-      <c r="T5" s="3"/>
-      <c r="U5" s="3"/>
-      <c r="V5" s="3"/>
-      <c r="W5" s="3"/>
-      <c r="X5" s="3"/>
-      <c r="Y5" s="3"/>
-      <c r="Z5" s="3"/>
-      <c r="AA5" s="3"/>
-      <c r="AB5" s="3"/>
-      <c r="AC5" s="3"/>
-      <c r="AD5" s="3"/>
-      <c r="AE5" s="3"/>
-      <c r="AF5" s="3"/>
-      <c r="AG5" s="3"/>
-      <c r="AH5" s="27" t="s">
-        <v>200</v>
-      </c>
-      <c r="AI5" s="3"/>
-      <c r="AJ5" s="3"/>
-      <c r="AK5" s="3"/>
-      <c r="AL5" s="3"/>
-      <c r="AM5" s="3"/>
-      <c r="AN5" s="3"/>
-      <c r="AO5" s="3"/>
-      <c r="AP5" s="3"/>
-      <c r="AQ5" s="3"/>
-      <c r="AR5" s="3"/>
-      <c r="AS5" s="3"/>
-      <c r="AT5" s="3"/>
-      <c r="AU5" s="3"/>
-      <c r="AV5" s="3"/>
-      <c r="AW5" s="3"/>
-      <c r="AX5" s="3"/>
-      <c r="AY5" s="3"/>
-      <c r="AZ5" s="3"/>
-      <c r="BA5" s="3"/>
-      <c r="BB5" s="3"/>
-      <c r="BC5" s="3"/>
-      <c r="BD5" s="3"/>
-      <c r="BE5" s="3"/>
-      <c r="BF5" s="3"/>
-      <c r="BG5" s="3"/>
-      <c r="BH5" s="3"/>
-      <c r="BI5" s="3"/>
-      <c r="BJ5" s="3"/>
-      <c r="BK5" s="3"/>
-      <c r="BL5" s="3"/>
-      <c r="BM5" s="3"/>
-      <c r="BN5" s="3"/>
-      <c r="BO5" s="3"/>
-      <c r="BP5" s="3"/>
-      <c r="BQ5" s="3"/>
-      <c r="BR5" s="3"/>
-      <c r="BS5" s="3"/>
-      <c r="BT5" s="3"/>
-      <c r="BU5" s="3"/>
-      <c r="BV5" s="3"/>
-      <c r="BW5" s="3"/>
-      <c r="BX5" s="3"/>
-      <c r="BY5" s="3"/>
-      <c r="BZ5" s="3"/>
-      <c r="CA5" s="3"/>
-      <c r="CB5" s="3"/>
-      <c r="CC5" s="3"/>
-      <c r="CD5" s="3"/>
-      <c r="CE5" s="3"/>
-      <c r="CF5" s="3"/>
-      <c r="CG5" s="3"/>
-      <c r="CH5" s="3"/>
-      <c r="CI5" s="3"/>
-      <c r="CJ5" s="3"/>
-      <c r="CK5" s="3"/>
-      <c r="CL5" s="10"/>
-    </row>
-    <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="11"/>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="14"/>
-      <c r="L6" s="14"/>
-      <c r="M6" s="14"/>
-      <c r="N6" s="14"/>
-      <c r="O6" s="14"/>
-      <c r="P6" s="14"/>
-      <c r="Q6" s="14"/>
-      <c r="R6" s="14"/>
-      <c r="S6" s="14"/>
-      <c r="T6" s="14"/>
-      <c r="U6" s="14"/>
-      <c r="V6" s="14"/>
-      <c r="W6" s="14"/>
-      <c r="X6" s="14"/>
-      <c r="Y6" s="14"/>
-      <c r="Z6" s="14"/>
-      <c r="AA6" s="14"/>
-      <c r="AB6" s="14"/>
-      <c r="AC6" s="14"/>
-      <c r="AD6" s="14"/>
-      <c r="AE6" s="14"/>
-      <c r="AF6" s="14"/>
-      <c r="AG6" s="14"/>
-      <c r="AH6" s="30" t="s">
-        <v>201</v>
-      </c>
-      <c r="AI6" s="14"/>
-      <c r="AJ6" s="14"/>
-      <c r="AK6" s="14"/>
-      <c r="AL6" s="14"/>
-      <c r="AM6" s="14"/>
-      <c r="AN6" s="14"/>
-      <c r="AO6" s="14"/>
-      <c r="AP6" s="14"/>
-      <c r="AQ6" s="14"/>
-      <c r="AR6" s="14"/>
-      <c r="AS6" s="14"/>
-      <c r="AT6" s="14"/>
-      <c r="AU6" s="14"/>
-      <c r="AV6" s="14"/>
-      <c r="AW6" s="14"/>
-      <c r="AX6" s="14"/>
-      <c r="AY6" s="14"/>
-      <c r="AZ6" s="14"/>
-      <c r="BA6" s="14"/>
-      <c r="BB6" s="14"/>
-      <c r="BC6" s="14"/>
-      <c r="BD6" s="14"/>
-      <c r="BE6" s="14"/>
-      <c r="BF6" s="14"/>
-      <c r="BG6" s="14"/>
-      <c r="BH6" s="14"/>
-      <c r="BI6" s="14"/>
-      <c r="BJ6" s="14"/>
-      <c r="BK6" s="14"/>
-      <c r="BL6" s="14"/>
-      <c r="BM6" s="14"/>
-      <c r="BN6" s="14"/>
-      <c r="BO6" s="14"/>
-      <c r="BP6" s="14"/>
-      <c r="BQ6" s="14"/>
-      <c r="BR6" s="14"/>
-      <c r="BS6" s="14"/>
-      <c r="BT6" s="14"/>
-      <c r="BU6" s="14"/>
-      <c r="BV6" s="14"/>
-      <c r="BW6" s="14"/>
-      <c r="BX6" s="14"/>
-      <c r="BY6" s="14"/>
-      <c r="BZ6" s="14"/>
-      <c r="CA6" s="14"/>
-      <c r="CB6" s="14"/>
-      <c r="CC6" s="14"/>
-      <c r="CD6" s="14"/>
-      <c r="CE6" s="14"/>
-      <c r="CF6" s="14"/>
-      <c r="CG6" s="14"/>
-      <c r="CH6" s="14"/>
-      <c r="CI6" s="14"/>
-      <c r="CJ6" s="14"/>
-      <c r="CK6" s="14"/>
-      <c r="CL6" s="15"/>
+      <c r="A5" s="11"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="14"/>
+      <c r="L5" s="14"/>
+      <c r="M5" s="14"/>
+      <c r="N5" s="14"/>
+      <c r="O5" s="14"/>
+      <c r="P5" s="14"/>
+      <c r="Q5" s="14"/>
+      <c r="R5" s="14"/>
+      <c r="S5" s="14"/>
+      <c r="T5" s="14"/>
+      <c r="U5" s="14"/>
+      <c r="V5" s="14"/>
+      <c r="W5" s="14"/>
+      <c r="X5" s="14"/>
+      <c r="Y5" s="14"/>
+      <c r="Z5" s="14"/>
+      <c r="AA5" s="14"/>
+      <c r="AB5" s="14"/>
+      <c r="AC5" s="14"/>
+      <c r="AD5" s="14"/>
+      <c r="AE5" s="14"/>
+      <c r="AF5" s="14"/>
+      <c r="AG5" s="14"/>
+      <c r="AH5" s="30" t="s">
+        <v>274</v>
+      </c>
+      <c r="AI5" s="14"/>
+      <c r="AJ5" s="14"/>
+      <c r="AK5" s="14"/>
+      <c r="AL5" s="14"/>
+      <c r="AM5" s="14"/>
+      <c r="AN5" s="14"/>
+      <c r="AO5" s="14"/>
+      <c r="AP5" s="14"/>
+      <c r="AQ5" s="14"/>
+      <c r="AR5" s="14"/>
+      <c r="AS5" s="14"/>
+      <c r="AT5" s="14"/>
+      <c r="AU5" s="14"/>
+      <c r="AV5" s="14"/>
+      <c r="AW5" s="14"/>
+      <c r="AX5" s="14"/>
+      <c r="AY5" s="14"/>
+      <c r="AZ5" s="14"/>
+      <c r="BA5" s="14"/>
+      <c r="BB5" s="14"/>
+      <c r="BC5" s="14"/>
+      <c r="BD5" s="14"/>
+      <c r="BE5" s="14"/>
+      <c r="BF5" s="14"/>
+      <c r="BG5" s="14"/>
+      <c r="BH5" s="14"/>
+      <c r="BI5" s="14"/>
+      <c r="BJ5" s="14"/>
+      <c r="BK5" s="14"/>
+      <c r="BL5" s="14"/>
+      <c r="BM5" s="14"/>
+      <c r="BN5" s="14"/>
+      <c r="BO5" s="14"/>
+      <c r="BP5" s="14"/>
+      <c r="BQ5" s="14"/>
+      <c r="BR5" s="14"/>
+      <c r="BS5" s="14"/>
+      <c r="BT5" s="14"/>
+      <c r="BU5" s="14"/>
+      <c r="BV5" s="14"/>
+      <c r="BW5" s="14"/>
+      <c r="BX5" s="14"/>
+      <c r="BY5" s="14"/>
+      <c r="BZ5" s="14"/>
+      <c r="CA5" s="14"/>
+      <c r="CB5" s="14"/>
+      <c r="CC5" s="14"/>
+      <c r="CD5" s="14"/>
+      <c r="CE5" s="14"/>
+      <c r="CF5" s="14"/>
+      <c r="CG5" s="14"/>
+      <c r="CH5" s="14"/>
+      <c r="CI5" s="14"/>
+      <c r="CJ5" s="14"/>
+      <c r="CK5" s="14"/>
+      <c r="CL5" s="15"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>
@@ -43271,7 +42650,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -43290,11 +42669,11 @@
         <v>7</v>
       </c>
       <c r="AF3" s="25" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="AG3" s="6"/>
       <c r="AH3" s="25" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="AI3" s="6"/>
       <c r="AJ3" s="6"/>
@@ -43388,7 +42767,7 @@
       <c r="AF4" s="14"/>
       <c r="AG4" s="14"/>
       <c r="AH4" s="30" t="s">
-        <v>112</v>
+        <v>259</v>
       </c>
       <c r="AI4" s="14"/>
       <c r="AJ4" s="14"/>
@@ -43464,7 +42843,7 @@
   <sheetData>
     <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="22" t="s">
-        <v>171</v>
+        <v>160</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -43558,7 +42937,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -43674,7 +43053,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -43791,7 +43170,7 @@
         <v>7</v>
       </c>
       <c r="AF4" s="27" t="s">
-        <v>265</v>
+        <v>247</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -43874,7 +43253,7 @@
       </c>
       <c r="P5" s="3"/>
       <c r="Q5" s="27" t="s">
-        <v>266</v>
+        <v>248</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
@@ -43893,7 +43272,7 @@
         <v>7</v>
       </c>
       <c r="AF5" s="27" t="s">
-        <v>267</v>
+        <v>249</v>
       </c>
       <c r="AG5" s="3"/>
       <c r="AH5" s="3"/>
@@ -43974,7 +43353,7 @@
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
       <c r="Q6" s="25" t="s">
-        <v>268</v>
+        <v>250</v>
       </c>
       <c r="R6" s="6"/>
       <c r="S6" s="6"/>
@@ -44074,7 +43453,7 @@
       </c>
       <c r="P7" s="6"/>
       <c r="Q7" s="25" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="R7" s="6"/>
       <c r="S7" s="6"/>
@@ -44170,7 +43549,7 @@
       <c r="O8" s="18"/>
       <c r="P8" s="18"/>
       <c r="Q8" s="29" t="s">
-        <v>269</v>
+        <v>251</v>
       </c>
       <c r="R8" s="18"/>
       <c r="S8" s="18"/>
@@ -44434,7 +43813,7 @@
     </row>
     <row r="11" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="22" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -44746,7 +44125,7 @@
       </c>
       <c r="P14" s="3"/>
       <c r="Q14" s="27" t="s">
-        <v>270</v>
+        <v>252</v>
       </c>
       <c r="R14" s="3"/>
       <c r="S14" s="3"/>
@@ -44844,7 +44223,7 @@
       </c>
       <c r="P15" s="3"/>
       <c r="Q15" s="27" t="s">
-        <v>271</v>
+        <v>253</v>
       </c>
       <c r="R15" s="3"/>
       <c r="S15" s="3"/>
@@ -44940,7 +44319,7 @@
       <c r="O16" s="6"/>
       <c r="P16" s="6"/>
       <c r="Q16" s="25" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="R16" s="6"/>
       <c r="S16" s="6"/>
@@ -45034,7 +44413,7 @@
       <c r="O17" s="3"/>
       <c r="P17" s="3"/>
       <c r="Q17" s="27" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="R17" s="3"/>
       <c r="S17" s="3"/>
@@ -45130,7 +44509,7 @@
       <c r="O18" s="3"/>
       <c r="P18" s="3"/>
       <c r="Q18" s="27" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R18" s="3"/>
       <c r="S18" s="3"/>
@@ -45326,7 +44705,7 @@
       </c>
       <c r="P20" s="18"/>
       <c r="Q20" s="29" t="s">
-        <v>273</v>
+        <v>255</v>
       </c>
       <c r="R20" s="18"/>
       <c r="S20" s="18"/>
@@ -45513,7 +44892,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -45727,7 +45106,7 @@
       </c>
       <c r="P4" s="3"/>
       <c r="Q4" s="27" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
@@ -45746,7 +45125,7 @@
         <v>7</v>
       </c>
       <c r="AF4" s="27" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -45848,7 +45227,7 @@
         <v>7</v>
       </c>
       <c r="AF5" s="27" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="AG5" s="3"/>
       <c r="AH5" s="3"/>
@@ -45931,7 +45310,7 @@
       </c>
       <c r="P6" s="3"/>
       <c r="Q6" s="27" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="R6" s="3"/>
       <c r="S6" s="3"/>
@@ -45950,7 +45329,7 @@
         <v>7</v>
       </c>
       <c r="AF6" s="27" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="AG6" s="3"/>
       <c r="AH6" s="3"/>
@@ -46044,7 +45423,7 @@
       <c r="AD7" s="3"/>
       <c r="AE7" s="3"/>
       <c r="AF7" s="27" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="AG7" s="3"/>
       <c r="AH7" s="3"/>
@@ -46138,7 +45517,7 @@
       <c r="AD8" s="3"/>
       <c r="AE8" s="3"/>
       <c r="AF8" s="27" t="s">
-        <v>150</v>
+        <v>260</v>
       </c>
       <c r="AG8" s="3"/>
       <c r="AH8" s="3"/>
@@ -46221,7 +45600,7 @@
       </c>
       <c r="P9" s="3"/>
       <c r="Q9" s="27" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="R9" s="3"/>
       <c r="S9" s="3"/>
@@ -46240,7 +45619,7 @@
         <v>7</v>
       </c>
       <c r="AF9" s="27" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="AG9" s="3"/>
       <c r="AH9" s="3"/>
@@ -46309,7 +45688,7 @@
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="26" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
@@ -46323,7 +45702,7 @@
       </c>
       <c r="P10" s="3"/>
       <c r="Q10" s="27" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="R10" s="3"/>
       <c r="S10" s="3"/>
@@ -46342,7 +45721,7 @@
         <v>7</v>
       </c>
       <c r="AF10" s="32" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="AG10" s="3"/>
       <c r="AH10" s="3"/>
@@ -47365,7 +46744,7 @@
     </row>
     <row r="21" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A21" s="22" t="s">
-        <v>212</v>
+        <v>196</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -47673,7 +47052,7 @@
       <c r="Q24" s="18"/>
       <c r="R24" s="18"/>
       <c r="S24" s="20" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="T24" s="18"/>
       <c r="U24" s="18"/>
@@ -47769,7 +47148,7 @@
       <c r="Q25" s="18"/>
       <c r="R25" s="18"/>
       <c r="S25" s="20" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="T25" s="18"/>
       <c r="U25" s="18"/>
@@ -47845,7 +47224,7 @@
     </row>
     <row r="26" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="20" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="B26" s="18"/>
       <c r="C26" s="18"/>
@@ -47865,7 +47244,7 @@
       <c r="Q26" s="18"/>
       <c r="R26" s="18"/>
       <c r="S26" s="20" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="T26" s="18"/>
       <c r="U26" s="18"/>
@@ -47887,7 +47266,7 @@
       </c>
       <c r="AJ26" s="18"/>
       <c r="AK26" s="20" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="AL26" s="18"/>
       <c r="AM26" s="18"/>
@@ -47981,7 +47360,7 @@
       <c r="AI27" s="18"/>
       <c r="AJ27" s="18"/>
       <c r="AK27" s="20" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="AL27" s="18"/>
       <c r="AM27" s="18"/>
@@ -48075,7 +47454,7 @@
       <c r="AI28" s="18"/>
       <c r="AJ28" s="18"/>
       <c r="AK28" s="20" t="s">
-        <v>150</v>
+        <v>260</v>
       </c>
       <c r="AL28" s="18"/>
       <c r="AM28" s="18"/>
@@ -48171,7 +47550,7 @@
       <c r="AI29" s="18"/>
       <c r="AJ29" s="18"/>
       <c r="AK29" s="20" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="AL29" s="18"/>
       <c r="AM29" s="18"/>
@@ -48267,7 +47646,7 @@
       <c r="AI30" s="18"/>
       <c r="AJ30" s="18"/>
       <c r="AK30" s="33" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="AL30" s="18"/>
       <c r="AM30" s="18"/>
@@ -48912,7 +48291,7 @@
     </row>
     <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="22" t="s">
-        <v>213</v>
+        <v>197</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -49200,7 +48579,7 @@
     </row>
     <row r="10" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="20" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="B10" s="18"/>
       <c r="C10" s="18"/>
@@ -49405,7 +48784,7 @@
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -49619,7 +48998,7 @@
       </c>
       <c r="P4" s="3"/>
       <c r="Q4" s="27" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
@@ -49638,7 +49017,7 @@
         <v>7</v>
       </c>
       <c r="AF4" s="27" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -49740,7 +49119,7 @@
         <v>7</v>
       </c>
       <c r="AF5" s="27" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="AG5" s="3"/>
       <c r="AH5" s="3"/>
@@ -49823,7 +49202,7 @@
       </c>
       <c r="P6" s="3"/>
       <c r="Q6" s="27" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="R6" s="3"/>
       <c r="S6" s="3"/>
@@ -49921,7 +49300,7 @@
       </c>
       <c r="P7" s="3"/>
       <c r="Q7" s="32" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="R7" s="3"/>
       <c r="S7" s="3"/>
@@ -50959,7 +50338,7 @@
     </row>
     <row r="18" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="22" t="s">
-        <v>212</v>
+        <v>196</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -51267,7 +50646,7 @@
       <c r="Q21" s="18"/>
       <c r="R21" s="18"/>
       <c r="S21" s="20" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="T21" s="18"/>
       <c r="U21" s="18"/>
@@ -51363,7 +50742,7 @@
       <c r="Q22" s="18"/>
       <c r="R22" s="18"/>
       <c r="S22" s="20" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="T22" s="18"/>
       <c r="U22" s="18"/>
@@ -51477,7 +50856,7 @@
       <c r="AI23" s="18"/>
       <c r="AJ23" s="18"/>
       <c r="AK23" s="20" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="AL23" s="18"/>
       <c r="AM23" s="18"/>
@@ -51573,7 +50952,7 @@
       <c r="AI24" s="18"/>
       <c r="AJ24" s="18"/>
       <c r="AK24" s="33" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="AL24" s="18"/>
       <c r="AM24" s="18"/>
@@ -52148,7 +51527,7 @@
       <c r="O6" s="18"/>
       <c r="P6" s="18"/>
       <c r="Q6" s="29" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="R6" s="18"/>
       <c r="S6" s="18"/>
@@ -52412,7 +51791,7 @@
     </row>
     <row r="9" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="22" t="s">
-        <v>211</v>
+        <v>195</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -52700,7 +52079,7 @@
     </row>
     <row r="12" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="20" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="B12" s="18"/>
       <c r="C12" s="18"/>
@@ -52796,7 +52175,7 @@
     </row>
     <row r="13" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="20" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="B13" s="18"/>
       <c r="C13" s="18"/>
@@ -53117,7 +52496,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -53136,7 +52515,7 @@
         <v>7</v>
       </c>
       <c r="AF3" s="25" t="s">
-        <v>210</v>
+        <v>194</v>
       </c>
       <c r="AG3" s="6"/>
       <c r="AH3" s="6"/>
@@ -53230,7 +52609,7 @@
       <c r="AD4" s="14"/>
       <c r="AE4" s="14"/>
       <c r="AF4" s="30" t="s">
-        <v>112</v>
+        <v>259</v>
       </c>
       <c r="AG4" s="14"/>
       <c r="AH4" s="14"/>
@@ -53504,7 +52883,7 @@
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="24" t="s">
-        <v>208</v>
+        <v>192</v>
       </c>
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
@@ -53518,7 +52897,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>209</v>
+        <v>193</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -53612,7 +52991,7 @@
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="27" t="s">
-        <v>112</v>
+        <v>259</v>
       </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
@@ -54299,7 +53678,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="24" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="H5" s="6"/>
       <c r="I5" s="6"/>
@@ -54309,11 +53688,11 @@
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
       <c r="O5" s="25" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="P5" s="6"/>
       <c r="Q5" s="25" t="s">
-        <v>263</v>
+        <v>245</v>
       </c>
       <c r="R5" s="6"/>
       <c r="S5" s="6"/>
@@ -54411,7 +53790,7 @@
       </c>
       <c r="R6" s="3"/>
       <c r="S6" s="27" t="s">
-        <v>264</v>
+        <v>246</v>
       </c>
       <c r="T6" s="3"/>
       <c r="U6" s="3"/>
@@ -54501,7 +53880,7 @@
       <c r="M7" s="3"/>
       <c r="N7" s="3"/>
       <c r="O7" s="27" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="P7" s="3"/>
       <c r="Q7" s="3"/>
@@ -54595,15 +53974,15 @@
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>
       <c r="O8" s="27" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="P8" s="3"/>
       <c r="Q8" s="27" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="R8" s="3"/>
       <c r="S8" s="27" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="T8" s="3"/>
       <c r="U8" s="3"/>
@@ -54701,7 +54080,7 @@
       </c>
       <c r="T9" s="3"/>
       <c r="U9" s="27" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="V9" s="3"/>
       <c r="W9" s="3"/>
@@ -54789,7 +54168,7 @@
       <c r="M10" s="3"/>
       <c r="N10" s="3"/>
       <c r="O10" s="27" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="P10" s="3"/>
       <c r="Q10" s="3"/>
@@ -54875,7 +54254,7 @@
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
       <c r="G11" s="26" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
@@ -54979,11 +54358,11 @@
       <c r="M12" s="3"/>
       <c r="N12" s="3"/>
       <c r="O12" s="27" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="P12" s="3"/>
       <c r="Q12" s="27" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="R12" s="3"/>
       <c r="S12" s="3"/>
@@ -55075,15 +54454,15 @@
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
       <c r="O13" s="27" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="P13" s="3"/>
       <c r="Q13" s="27" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="R13" s="3"/>
       <c r="S13" s="27" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="T13" s="3"/>
       <c r="U13" s="3"/>
@@ -55181,7 +54560,7 @@
       </c>
       <c r="T14" s="3"/>
       <c r="U14" s="27" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="V14" s="3"/>
       <c r="W14" s="3"/>
@@ -55269,7 +54648,7 @@
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
       <c r="O15" s="27" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="P15" s="3"/>
       <c r="Q15" s="3"/>
@@ -55355,7 +54734,7 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
       <c r="G16" s="26" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
@@ -55449,7 +54828,7 @@
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="26" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
@@ -55459,11 +54838,11 @@
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
       <c r="O17" s="27" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="P17" s="3"/>
       <c r="Q17" s="27" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="R17" s="3"/>
       <c r="S17" s="3"/>
@@ -55555,11 +54934,11 @@
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
       <c r="O18" s="27" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="P18" s="3"/>
       <c r="Q18" s="27" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="R18" s="3"/>
       <c r="S18" s="3"/>
@@ -55643,7 +55022,7 @@
       <c r="E19" s="12"/>
       <c r="F19" s="12"/>
       <c r="G19" s="31" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="H19" s="14"/>
       <c r="I19" s="14"/>
@@ -56152,7 +55531,7 @@
       </c>
       <c r="P5" s="3"/>
       <c r="Q5" s="27" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
@@ -56252,7 +55631,7 @@
       </c>
       <c r="P6" s="6"/>
       <c r="Q6" s="25" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="R6" s="6"/>
       <c r="S6" s="6"/>
@@ -56350,7 +55729,7 @@
       </c>
       <c r="P7" s="14"/>
       <c r="Q7" s="30" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="R7" s="14"/>
       <c r="S7" s="14"/>

</xml_diff>

<commit_message>
feat: align INSERT VALUES CASE transfer layout
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Macro\SqlAnalyzerFormatter-feature\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B62837AA-51D3-46AA-A936-126797549C31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B46EF11B-238F-498A-A46B-AA684FB4725F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="58" activeTab="59" xr2:uid="{41A826B0-B2A2-4DC8-9B04-8EFBE807DC37}"/>
   </bookViews>
@@ -40549,296 +40549,296 @@
       <c r="CL2" s="1"/>
     </row>
     <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
-      <c r="M3" s="16"/>
-      <c r="N3" s="16"/>
-      <c r="O3" s="16"/>
-      <c r="P3" s="16"/>
-      <c r="Q3" s="16"/>
-      <c r="R3" s="16"/>
-      <c r="S3" s="28" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+      <c r="S3" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="T3" s="16"/>
-      <c r="U3" s="16"/>
-      <c r="V3" s="16"/>
-      <c r="W3" s="16"/>
-      <c r="X3" s="16"/>
-      <c r="Y3" s="16"/>
-      <c r="Z3" s="16"/>
-      <c r="AA3" s="16"/>
-      <c r="AB3" s="16"/>
-      <c r="AC3" s="16"/>
-      <c r="AD3" s="16"/>
-      <c r="AE3" s="16"/>
-      <c r="AF3" s="16"/>
-      <c r="AG3" s="16"/>
-      <c r="AH3" s="16"/>
-      <c r="AI3" s="16"/>
-      <c r="AJ3" s="16"/>
-      <c r="AK3" s="28" t="s">
+      <c r="T3" s="4"/>
+      <c r="U3" s="4"/>
+      <c r="V3" s="4"/>
+      <c r="W3" s="4"/>
+      <c r="X3" s="4"/>
+      <c r="Y3" s="4"/>
+      <c r="Z3" s="4"/>
+      <c r="AA3" s="4"/>
+      <c r="AB3" s="4"/>
+      <c r="AC3" s="4"/>
+      <c r="AD3" s="4"/>
+      <c r="AE3" s="4"/>
+      <c r="AF3" s="4"/>
+      <c r="AG3" s="4"/>
+      <c r="AH3" s="4"/>
+      <c r="AI3" s="4"/>
+      <c r="AJ3" s="4"/>
+      <c r="AK3" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="AL3" s="16"/>
-      <c r="AM3" s="16"/>
-      <c r="AN3" s="16"/>
-      <c r="AO3" s="16"/>
-      <c r="AP3" s="16"/>
-      <c r="AQ3" s="16"/>
-      <c r="AR3" s="16"/>
-      <c r="AS3" s="16"/>
-      <c r="AT3" s="16"/>
-      <c r="AU3" s="16"/>
-      <c r="AV3" s="16"/>
-      <c r="AW3" s="16"/>
-      <c r="AX3" s="16"/>
-      <c r="AY3" s="16"/>
-      <c r="AZ3" s="16"/>
-      <c r="BA3" s="16"/>
-      <c r="BB3" s="16"/>
-      <c r="BC3" s="16"/>
-      <c r="BD3" s="16"/>
-      <c r="BE3" s="16"/>
-      <c r="BF3" s="16"/>
-      <c r="BG3" s="16"/>
-      <c r="BH3" s="16"/>
-      <c r="BI3" s="16"/>
-      <c r="BJ3" s="16"/>
-      <c r="BK3" s="16"/>
-      <c r="BL3" s="16"/>
-      <c r="BM3" s="16"/>
-      <c r="BN3" s="16"/>
-      <c r="BO3" s="16"/>
-      <c r="BP3" s="16"/>
-      <c r="BQ3" s="16"/>
-      <c r="BR3" s="16"/>
-      <c r="BS3" s="16"/>
-      <c r="BT3" s="16"/>
-      <c r="BU3" s="16"/>
-      <c r="BV3" s="16"/>
-      <c r="BW3" s="16"/>
-      <c r="BX3" s="16"/>
-      <c r="BY3" s="16"/>
-      <c r="BZ3" s="16"/>
-      <c r="CA3" s="16"/>
-      <c r="CB3" s="16"/>
-      <c r="CC3" s="16"/>
-      <c r="CD3" s="16"/>
-      <c r="CE3" s="16"/>
-      <c r="CF3" s="16"/>
-      <c r="CG3" s="16"/>
-      <c r="CH3" s="16"/>
-      <c r="CI3" s="16"/>
-      <c r="CJ3" s="16"/>
-      <c r="CK3" s="16"/>
-      <c r="CL3" s="21"/>
+      <c r="AL3" s="4"/>
+      <c r="AM3" s="4"/>
+      <c r="AN3" s="4"/>
+      <c r="AO3" s="4"/>
+      <c r="AP3" s="4"/>
+      <c r="AQ3" s="4"/>
+      <c r="AR3" s="4"/>
+      <c r="AS3" s="4"/>
+      <c r="AT3" s="4"/>
+      <c r="AU3" s="4"/>
+      <c r="AV3" s="4"/>
+      <c r="AW3" s="4"/>
+      <c r="AX3" s="4"/>
+      <c r="AY3" s="4"/>
+      <c r="AZ3" s="4"/>
+      <c r="BA3" s="4"/>
+      <c r="BB3" s="4"/>
+      <c r="BC3" s="4"/>
+      <c r="BD3" s="4"/>
+      <c r="BE3" s="4"/>
+      <c r="BF3" s="4"/>
+      <c r="BG3" s="4"/>
+      <c r="BH3" s="4"/>
+      <c r="BI3" s="4"/>
+      <c r="BJ3" s="4"/>
+      <c r="BK3" s="4"/>
+      <c r="BL3" s="4"/>
+      <c r="BM3" s="4"/>
+      <c r="BN3" s="4"/>
+      <c r="BO3" s="4"/>
+      <c r="BP3" s="4"/>
+      <c r="BQ3" s="4"/>
+      <c r="BR3" s="4"/>
+      <c r="BS3" s="4"/>
+      <c r="BT3" s="4"/>
+      <c r="BU3" s="4"/>
+      <c r="BV3" s="4"/>
+      <c r="BW3" s="4"/>
+      <c r="BX3" s="4"/>
+      <c r="BY3" s="4"/>
+      <c r="BZ3" s="4"/>
+      <c r="CA3" s="4"/>
+      <c r="CB3" s="4"/>
+      <c r="CC3" s="4"/>
+      <c r="CD3" s="4"/>
+      <c r="CE3" s="4"/>
+      <c r="CF3" s="4"/>
+      <c r="CG3" s="4"/>
+      <c r="CH3" s="4"/>
+      <c r="CI3" s="4"/>
+      <c r="CJ3" s="4"/>
+      <c r="CK3" s="4"/>
+      <c r="CL3" s="35"/>
     </row>
     <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="31" t="s">
+      <c r="A4" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
-      <c r="L4" s="14"/>
-      <c r="M4" s="14"/>
-      <c r="N4" s="14"/>
-      <c r="O4" s="14"/>
-      <c r="P4" s="14"/>
-      <c r="Q4" s="14"/>
-      <c r="R4" s="14"/>
-      <c r="S4" s="31" t="s">
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="5"/>
+      <c r="T4" s="6"/>
+      <c r="U4" s="6"/>
+      <c r="V4" s="6"/>
+      <c r="W4" s="6"/>
+      <c r="X4" s="6"/>
+      <c r="Y4" s="6"/>
+      <c r="Z4" s="6"/>
+      <c r="AA4" s="6"/>
+      <c r="AB4" s="6"/>
+      <c r="AC4" s="6"/>
+      <c r="AD4" s="6"/>
+      <c r="AE4" s="6"/>
+      <c r="AF4" s="6"/>
+      <c r="AG4" s="6"/>
+      <c r="AH4" s="6"/>
+      <c r="AI4" s="6"/>
+      <c r="AJ4" s="6"/>
+      <c r="AK4" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="T4" s="14"/>
-      <c r="U4" s="14"/>
-      <c r="V4" s="14"/>
-      <c r="W4" s="14"/>
-      <c r="X4" s="14"/>
-      <c r="Y4" s="14"/>
-      <c r="Z4" s="14"/>
-      <c r="AA4" s="14"/>
-      <c r="AB4" s="14"/>
-      <c r="AC4" s="14"/>
-      <c r="AD4" s="14"/>
-      <c r="AE4" s="14"/>
-      <c r="AF4" s="14"/>
-      <c r="AG4" s="14"/>
-      <c r="AH4" s="14"/>
-      <c r="AI4" s="30" t="s">
+      <c r="AL4" s="6"/>
+      <c r="AM4" s="6"/>
+      <c r="AN4" s="6"/>
+      <c r="AO4" s="6"/>
+      <c r="AP4" s="6"/>
+      <c r="AQ4" s="6"/>
+      <c r="AR4" s="6"/>
+      <c r="AS4" s="6"/>
+      <c r="AT4" s="6"/>
+      <c r="AU4" s="6"/>
+      <c r="AV4" s="6"/>
+      <c r="AW4" s="6"/>
+      <c r="AX4" s="6"/>
+      <c r="AY4" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="AJ4" s="14"/>
-      <c r="AK4" s="31" t="s">
+      <c r="AZ4" s="25" t="s">
         <v>190</v>
       </c>
-      <c r="AL4" s="14"/>
-      <c r="AM4" s="14"/>
-      <c r="AN4" s="14"/>
-      <c r="AO4" s="14"/>
-      <c r="AP4" s="14"/>
-      <c r="AQ4" s="14"/>
-      <c r="AR4" s="14"/>
-      <c r="AS4" s="14"/>
-      <c r="AT4" s="14"/>
-      <c r="AU4" s="14"/>
-      <c r="AV4" s="14"/>
-      <c r="AW4" s="14"/>
-      <c r="AX4" s="14"/>
-      <c r="AY4" s="14"/>
-      <c r="AZ4" s="14"/>
-      <c r="BA4" s="14"/>
-      <c r="BB4" s="14"/>
-      <c r="BC4" s="14"/>
-      <c r="BD4" s="14"/>
-      <c r="BE4" s="14"/>
-      <c r="BF4" s="14"/>
-      <c r="BG4" s="14"/>
-      <c r="BH4" s="14"/>
-      <c r="BI4" s="14"/>
-      <c r="BJ4" s="14"/>
-      <c r="BK4" s="14"/>
-      <c r="BL4" s="14"/>
-      <c r="BM4" s="14"/>
-      <c r="BN4" s="14"/>
-      <c r="BO4" s="14"/>
-      <c r="BP4" s="14"/>
-      <c r="BQ4" s="14"/>
-      <c r="BR4" s="14"/>
-      <c r="BS4" s="14"/>
-      <c r="BT4" s="14"/>
-      <c r="BU4" s="14"/>
-      <c r="BV4" s="14"/>
-      <c r="BW4" s="14"/>
-      <c r="BX4" s="14"/>
-      <c r="BY4" s="14"/>
-      <c r="BZ4" s="14"/>
-      <c r="CA4" s="14"/>
-      <c r="CB4" s="14"/>
-      <c r="CC4" s="14"/>
-      <c r="CD4" s="14"/>
-      <c r="CE4" s="14"/>
-      <c r="CF4" s="14"/>
-      <c r="CG4" s="14"/>
-      <c r="CH4" s="14"/>
-      <c r="CI4" s="14"/>
-      <c r="CJ4" s="14"/>
-      <c r="CK4" s="14"/>
-      <c r="CL4" s="15"/>
+      <c r="BA4" s="6"/>
+      <c r="BB4" s="6"/>
+      <c r="BC4" s="6"/>
+      <c r="BD4" s="6"/>
+      <c r="BE4" s="6"/>
+      <c r="BF4" s="6"/>
+      <c r="BG4" s="6"/>
+      <c r="BH4" s="6"/>
+      <c r="BI4" s="6"/>
+      <c r="BJ4" s="6"/>
+      <c r="BK4" s="6"/>
+      <c r="BL4" s="6"/>
+      <c r="BM4" s="6"/>
+      <c r="BN4" s="6"/>
+      <c r="BO4" s="6"/>
+      <c r="BP4" s="6"/>
+      <c r="BQ4" s="6"/>
+      <c r="BR4" s="6"/>
+      <c r="BS4" s="6"/>
+      <c r="BT4" s="6"/>
+      <c r="BU4" s="6"/>
+      <c r="BV4" s="6"/>
+      <c r="BW4" s="6"/>
+      <c r="BX4" s="6"/>
+      <c r="BY4" s="6"/>
+      <c r="BZ4" s="6"/>
+      <c r="CA4" s="6"/>
+      <c r="CB4" s="6"/>
+      <c r="CC4" s="6"/>
+      <c r="CD4" s="6"/>
+      <c r="CE4" s="6"/>
+      <c r="CF4" s="6"/>
+      <c r="CG4" s="6"/>
+      <c r="CH4" s="6"/>
+      <c r="CI4" s="6"/>
+      <c r="CJ4" s="6"/>
+      <c r="CK4" s="6"/>
+      <c r="CL4" s="7"/>
     </row>
     <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="17"/>
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="18"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="18"/>
-      <c r="N5" s="18"/>
-      <c r="O5" s="18"/>
-      <c r="P5" s="18"/>
-      <c r="Q5" s="18"/>
-      <c r="R5" s="18"/>
-      <c r="S5" s="17"/>
-      <c r="T5" s="18"/>
-      <c r="U5" s="18"/>
-      <c r="V5" s="18"/>
-      <c r="W5" s="18"/>
-      <c r="X5" s="18"/>
-      <c r="Y5" s="18"/>
-      <c r="Z5" s="18"/>
-      <c r="AA5" s="18"/>
-      <c r="AB5" s="18"/>
-      <c r="AC5" s="18"/>
-      <c r="AD5" s="18"/>
-      <c r="AE5" s="18"/>
-      <c r="AF5" s="18"/>
-      <c r="AG5" s="18"/>
-      <c r="AH5" s="18"/>
-      <c r="AI5" s="18"/>
-      <c r="AJ5" s="18"/>
-      <c r="AK5" s="20" t="s">
+      <c r="A5" s="13"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="14"/>
+      <c r="L5" s="14"/>
+      <c r="M5" s="14"/>
+      <c r="N5" s="14"/>
+      <c r="O5" s="14"/>
+      <c r="P5" s="14"/>
+      <c r="Q5" s="14"/>
+      <c r="R5" s="14"/>
+      <c r="S5" s="13"/>
+      <c r="T5" s="14"/>
+      <c r="U5" s="14"/>
+      <c r="V5" s="14"/>
+      <c r="W5" s="14"/>
+      <c r="X5" s="14"/>
+      <c r="Y5" s="14"/>
+      <c r="Z5" s="14"/>
+      <c r="AA5" s="14"/>
+      <c r="AB5" s="14"/>
+      <c r="AC5" s="14"/>
+      <c r="AD5" s="14"/>
+      <c r="AE5" s="14"/>
+      <c r="AF5" s="14"/>
+      <c r="AG5" s="14"/>
+      <c r="AH5" s="14"/>
+      <c r="AI5" s="14"/>
+      <c r="AJ5" s="14"/>
+      <c r="AK5" s="13"/>
+      <c r="AL5" s="14"/>
+      <c r="AM5" s="14"/>
+      <c r="AN5" s="14"/>
+      <c r="AO5" s="14"/>
+      <c r="AP5" s="14"/>
+      <c r="AQ5" s="14"/>
+      <c r="AR5" s="14"/>
+      <c r="AS5" s="14"/>
+      <c r="AT5" s="14"/>
+      <c r="AU5" s="14"/>
+      <c r="AV5" s="14"/>
+      <c r="AW5" s="14"/>
+      <c r="AX5" s="14"/>
+      <c r="AY5" s="14"/>
+      <c r="AZ5" s="30" t="s">
         <v>276</v>
       </c>
-      <c r="AL5" s="18"/>
-      <c r="AM5" s="18"/>
-      <c r="AN5" s="18"/>
-      <c r="AO5" s="18"/>
-      <c r="AP5" s="18"/>
-      <c r="AQ5" s="18"/>
-      <c r="AR5" s="18"/>
-      <c r="AS5" s="18"/>
-      <c r="AT5" s="18"/>
-      <c r="AU5" s="18"/>
-      <c r="AV5" s="18"/>
-      <c r="AW5" s="18"/>
-      <c r="AX5" s="18"/>
-      <c r="AY5" s="18"/>
-      <c r="AZ5" s="18"/>
-      <c r="BA5" s="18"/>
-      <c r="BB5" s="18"/>
-      <c r="BC5" s="18"/>
-      <c r="BD5" s="18"/>
-      <c r="BE5" s="18"/>
-      <c r="BF5" s="18"/>
-      <c r="BG5" s="18"/>
-      <c r="BH5" s="18"/>
-      <c r="BI5" s="18"/>
-      <c r="BJ5" s="18"/>
-      <c r="BK5" s="18"/>
-      <c r="BL5" s="18"/>
-      <c r="BM5" s="18"/>
-      <c r="BN5" s="18"/>
-      <c r="BO5" s="18"/>
-      <c r="BP5" s="18"/>
-      <c r="BQ5" s="18"/>
-      <c r="BR5" s="18"/>
-      <c r="BS5" s="18"/>
-      <c r="BT5" s="18"/>
-      <c r="BU5" s="18"/>
-      <c r="BV5" s="18"/>
-      <c r="BW5" s="18"/>
-      <c r="BX5" s="18"/>
-      <c r="BY5" s="18"/>
-      <c r="BZ5" s="18"/>
-      <c r="CA5" s="18"/>
-      <c r="CB5" s="18"/>
-      <c r="CC5" s="18"/>
-      <c r="CD5" s="18"/>
-      <c r="CE5" s="18"/>
-      <c r="CF5" s="18"/>
-      <c r="CG5" s="18"/>
-      <c r="CH5" s="18"/>
-      <c r="CI5" s="18"/>
-      <c r="CJ5" s="18"/>
-      <c r="CK5" s="18"/>
-      <c r="CL5" s="19"/>
+      <c r="BA5" s="14"/>
+      <c r="BB5" s="14"/>
+      <c r="BC5" s="14"/>
+      <c r="BD5" s="14"/>
+      <c r="BE5" s="14"/>
+      <c r="BF5" s="14"/>
+      <c r="BG5" s="14"/>
+      <c r="BH5" s="14"/>
+      <c r="BI5" s="14"/>
+      <c r="BJ5" s="14"/>
+      <c r="BK5" s="14"/>
+      <c r="BL5" s="14"/>
+      <c r="BM5" s="14"/>
+      <c r="BN5" s="14"/>
+      <c r="BO5" s="14"/>
+      <c r="BP5" s="14"/>
+      <c r="BQ5" s="14"/>
+      <c r="BR5" s="14"/>
+      <c r="BS5" s="14"/>
+      <c r="BT5" s="14"/>
+      <c r="BU5" s="14"/>
+      <c r="BV5" s="14"/>
+      <c r="BW5" s="14"/>
+      <c r="BX5" s="14"/>
+      <c r="BY5" s="14"/>
+      <c r="BZ5" s="14"/>
+      <c r="CA5" s="14"/>
+      <c r="CB5" s="14"/>
+      <c r="CC5" s="14"/>
+      <c r="CD5" s="14"/>
+      <c r="CE5" s="14"/>
+      <c r="CF5" s="14"/>
+      <c r="CG5" s="14"/>
+      <c r="CH5" s="14"/>
+      <c r="CI5" s="14"/>
+      <c r="CJ5" s="14"/>
+      <c r="CK5" s="14"/>
+      <c r="CL5" s="15"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>

</xml_diff>

<commit_message>
docs: confirm SEL-060 output review
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -10,84 +10,84 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B46EF11B-238F-498A-A46B-AA684FB4725F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="58" activeTab="59" xr2:uid="{41A826B0-B2A2-4DC8-9B04-8EFBE807DC37}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="0" activeTab="64" xr2:uid="{41A826B0-B2A2-4DC8-9B04-8EFBE807DC37}"/>
   </bookViews>
   <sheets>
+    <sheet name="SEL-001" sheetId="1" r:id="rId59"/>
+    <sheet name="SEL-002" sheetId="2" r:id="rId58"/>
+    <sheet name="SEL-003" sheetId="3" r:id="rId57"/>
+    <sheet name="SEL-004" sheetId="4" r:id="rId56"/>
+    <sheet name="SEL-005" sheetId="5" r:id="rId55"/>
+    <sheet name="SEL-006" sheetId="6" r:id="rId54"/>
+    <sheet name="SEL-007" sheetId="7" r:id="rId53"/>
+    <sheet name="SEL-008" sheetId="8" r:id="rId52"/>
+    <sheet name="SEL-009" sheetId="9" r:id="rId51"/>
+    <sheet name="SEL-010" sheetId="10" r:id="rId50"/>
+    <sheet name="SEL-011" sheetId="11" r:id="rId49"/>
+    <sheet name="SEL-012" sheetId="12" r:id="rId48"/>
+    <sheet name="SEL-013" sheetId="13" r:id="rId47"/>
+    <sheet name="SEL-014" sheetId="14" r:id="rId46"/>
+    <sheet name="SEL-015" sheetId="15" r:id="rId45"/>
+    <sheet name="SEL-016" sheetId="16" r:id="rId44"/>
+    <sheet name="SEL-017" sheetId="17" r:id="rId43"/>
+    <sheet name="SEL-018" sheetId="18" r:id="rId42"/>
+    <sheet name="SEL-019" sheetId="19" r:id="rId41"/>
+    <sheet name="SEL-020" sheetId="20" r:id="rId40"/>
+    <sheet name="SEL-021" sheetId="21" r:id="rId39"/>
+    <sheet name="SEL-022" sheetId="22" r:id="rId38"/>
+    <sheet name="SEL-023" sheetId="23" r:id="rId37"/>
+    <sheet name="SEL-024" sheetId="24" r:id="rId36"/>
+    <sheet name="SEL-025" sheetId="25" r:id="rId35"/>
+    <sheet name="SEL-026" sheetId="26" r:id="rId34"/>
+    <sheet name="SEL-027" sheetId="37" r:id="rId33"/>
+    <sheet name="SEL-028" sheetId="27" r:id="rId32"/>
+    <sheet name="SEL-029" sheetId="28" r:id="rId31"/>
+    <sheet name="SEL-030" sheetId="29" r:id="rId30"/>
+    <sheet name="SEL-031" sheetId="30" r:id="rId29"/>
+    <sheet name="SEL-032" sheetId="31" r:id="rId28"/>
+    <sheet name="SEL-033" sheetId="32" r:id="rId27"/>
+    <sheet name="SEL-034" sheetId="33" r:id="rId26"/>
+    <sheet name="SEL-035" sheetId="34" r:id="rId25"/>
+    <sheet name="SEL-036" sheetId="35" r:id="rId24"/>
+    <sheet name="SEL-037" sheetId="36" r:id="rId23"/>
+    <sheet name="SEL-038" sheetId="38" r:id="rId22"/>
+    <sheet name="SEL-039" sheetId="39" r:id="rId21"/>
+    <sheet name="SEL-040" sheetId="40" r:id="rId20"/>
+    <sheet name="SEL-041" sheetId="41" r:id="rId19"/>
+    <sheet name="SEL-042" sheetId="42" r:id="rId18"/>
+    <sheet name="SEL-043" sheetId="43" r:id="rId17"/>
+    <sheet name="SEL-044" sheetId="44" r:id="rId16"/>
+    <sheet name="SEL-045" sheetId="79" r:id="rId73"/>
+    <sheet name="SEL-046" sheetId="46" r:id="rId15"/>
+    <sheet name="SEL-047" sheetId="47" r:id="rId14"/>
+    <sheet name="SEL-048" sheetId="52" r:id="rId13"/>
+    <sheet name="SEL-049" sheetId="53" r:id="rId12"/>
+    <sheet name="SEL-050" sheetId="54" r:id="rId11"/>
+    <sheet name="SEL-051" sheetId="55" r:id="rId10"/>
+    <sheet name="SEL-052" sheetId="56" r:id="rId9"/>
+    <sheet name="SEL-053" sheetId="57" r:id="rId8"/>
+    <sheet name="SEL-054" sheetId="48" r:id="rId7"/>
+    <sheet name="SEL-055" sheetId="49" r:id="rId6"/>
+    <sheet name="SEL-056" sheetId="80" r:id="rId72"/>
+    <sheet name="SEL-057" sheetId="70" r:id="rId63"/>
+    <sheet name="SEL-058" sheetId="58" r:id="rId5"/>
+    <sheet name="SEL-059" sheetId="81" r:id="rId71"/>
+    <sheet name="SEL-060" sheetId="63" r:id="rId4"/>
+    <sheet name="SEL-061" sheetId="82" r:id="rId70"/>
+    <sheet name="SEL-062" sheetId="64" r:id="rId3"/>
+    <sheet name="SEL-063" sheetId="65" r:id="rId2"/>
     <sheet name="SEL-064" sheetId="66" r:id="rId1"/>
-    <sheet name="SEL-063" sheetId="65" r:id="rId2"/>
-    <sheet name="SEL-062" sheetId="64" r:id="rId3"/>
-    <sheet name="SEL-060" sheetId="63" r:id="rId4"/>
-    <sheet name="SEL-058" sheetId="58" r:id="rId5"/>
-    <sheet name="SEL-055" sheetId="49" r:id="rId6"/>
-    <sheet name="SEL-054" sheetId="48" r:id="rId7"/>
-    <sheet name="SEL-053" sheetId="57" r:id="rId8"/>
-    <sheet name="SEL-052" sheetId="56" r:id="rId9"/>
-    <sheet name="SEL-051" sheetId="55" r:id="rId10"/>
-    <sheet name="SEL-050" sheetId="54" r:id="rId11"/>
-    <sheet name="SEL-049" sheetId="53" r:id="rId12"/>
-    <sheet name="SEL-048" sheetId="52" r:id="rId13"/>
-    <sheet name="SEL-047" sheetId="47" r:id="rId14"/>
-    <sheet name="SEL-046" sheetId="46" r:id="rId15"/>
-    <sheet name="SEL-044" sheetId="44" r:id="rId16"/>
-    <sheet name="SEL-043" sheetId="43" r:id="rId17"/>
-    <sheet name="SEL-042" sheetId="42" r:id="rId18"/>
-    <sheet name="SEL-041" sheetId="41" r:id="rId19"/>
-    <sheet name="SEL-040" sheetId="40" r:id="rId20"/>
-    <sheet name="SEL-039" sheetId="39" r:id="rId21"/>
-    <sheet name="SEL-038" sheetId="38" r:id="rId22"/>
-    <sheet name="SEL-037" sheetId="36" r:id="rId23"/>
-    <sheet name="SEL-036" sheetId="35" r:id="rId24"/>
-    <sheet name="SEL-035" sheetId="34" r:id="rId25"/>
-    <sheet name="SEL-034" sheetId="33" r:id="rId26"/>
-    <sheet name="SEL-033" sheetId="32" r:id="rId27"/>
-    <sheet name="SEL-032" sheetId="31" r:id="rId28"/>
-    <sheet name="SEL-031" sheetId="30" r:id="rId29"/>
-    <sheet name="SEL-030" sheetId="29" r:id="rId30"/>
-    <sheet name="SEL-029" sheetId="28" r:id="rId31"/>
-    <sheet name="SEL-028" sheetId="27" r:id="rId32"/>
-    <sheet name="SEL-027" sheetId="37" r:id="rId33"/>
-    <sheet name="SEL-026" sheetId="26" r:id="rId34"/>
-    <sheet name="SEL-025" sheetId="25" r:id="rId35"/>
-    <sheet name="SEL-024" sheetId="24" r:id="rId36"/>
-    <sheet name="SEL-023" sheetId="23" r:id="rId37"/>
-    <sheet name="SEL-022" sheetId="22" r:id="rId38"/>
-    <sheet name="SEL-021" sheetId="21" r:id="rId39"/>
-    <sheet name="SEL-020" sheetId="20" r:id="rId40"/>
-    <sheet name="SEL-019" sheetId="19" r:id="rId41"/>
-    <sheet name="SEL-018" sheetId="18" r:id="rId42"/>
-    <sheet name="SEL-017" sheetId="17" r:id="rId43"/>
-    <sheet name="SEL-016" sheetId="16" r:id="rId44"/>
-    <sheet name="SEL-015" sheetId="15" r:id="rId45"/>
-    <sheet name="SEL-014" sheetId="14" r:id="rId46"/>
-    <sheet name="SEL-013" sheetId="13" r:id="rId47"/>
-    <sheet name="SEL-012" sheetId="12" r:id="rId48"/>
-    <sheet name="SEL-011" sheetId="11" r:id="rId49"/>
-    <sheet name="SEL-010" sheetId="10" r:id="rId50"/>
-    <sheet name="SEL-009" sheetId="9" r:id="rId51"/>
-    <sheet name="SEL-008" sheetId="8" r:id="rId52"/>
-    <sheet name="SEL-007" sheetId="7" r:id="rId53"/>
-    <sheet name="SEL-006" sheetId="6" r:id="rId54"/>
-    <sheet name="SEL-005" sheetId="5" r:id="rId55"/>
-    <sheet name="SEL-004" sheetId="4" r:id="rId56"/>
-    <sheet name="SEL-003" sheetId="3" r:id="rId57"/>
-    <sheet name="SEL-002" sheetId="2" r:id="rId58"/>
-    <sheet name="SEL-001" sheetId="1" r:id="rId59"/>
     <sheet name="SEL-065" sheetId="67" r:id="rId60"/>
     <sheet name="SEL-066" sheetId="68" r:id="rId61"/>
     <sheet name="SEL-067" sheetId="69" r:id="rId62"/>
-    <sheet name="SEL-057" sheetId="70" r:id="rId63"/>
+    <sheet name="SEL-068" sheetId="71" r:id="rId69"/>
+    <sheet name="SEL-069" sheetId="72" r:id="rId68"/>
+    <sheet name="SEL-070" sheetId="73" r:id="rId67"/>
+    <sheet name="SEL-071" sheetId="74" r:id="rId66"/>
+    <sheet name="SEL-072" sheetId="75" r:id="rId65"/>
     <sheet name="SEL-073" sheetId="76" r:id="rId64"/>
-    <sheet name="SEL-072" sheetId="75" r:id="rId65"/>
-    <sheet name="SEL-071" sheetId="74" r:id="rId66"/>
-    <sheet name="SEL-070" sheetId="73" r:id="rId67"/>
-    <sheet name="SEL-069" sheetId="72" r:id="rId68"/>
-    <sheet name="SEL-068" sheetId="71" r:id="rId69"/>
-    <sheet name="SEL-061" sheetId="82" r:id="rId70"/>
-    <sheet name="SEL-059" sheetId="81" r:id="rId71"/>
-    <sheet name="SEL-056" sheetId="80" r:id="rId72"/>
-    <sheet name="SEL-045" sheetId="79" r:id="rId73"/>
+    <sheet name="SEL-074" sheetId="77" r:id="rId75"/>
     <sheet name="SEL-075" sheetId="78" r:id="rId74"/>
-    <sheet name="SEL-074" sheetId="77" r:id="rId75"/>
   </sheets>
   <calcPr calcId="191029" calcMode="manual"/>
   <extLst>

</xml_diff>

<commit_message>
fix: preserve CASE condition parentheses
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -2,81 +2,81 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-001" sheetId="1" r:id="R84e3a2b02c874987"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-002" sheetId="2" r:id="Rb168c7d266ef4d2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-003" sheetId="3" r:id="R9a8d83c0c4e341a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-004" sheetId="4" r:id="Rf7ac52a93e0d4664"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-005" sheetId="5" r:id="R55402f88192941c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-006" sheetId="6" r:id="Rf9e5ff74fffa4a72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-007" sheetId="7" r:id="R151451a861a84d63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-008" sheetId="8" r:id="R66fb20fab42f4228"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-009" sheetId="9" r:id="Rdd16a0fbdd3f4f3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-010" sheetId="10" r:id="Rfcf39e46c10049c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-011" sheetId="11" r:id="R2cadca3846eb4841"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-012" sheetId="12" r:id="R84807aab0db443cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-013" sheetId="13" r:id="R62e0542802c44a3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-014" sheetId="14" r:id="Rd8c383ce130d4deb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-015" sheetId="15" r:id="Rd1ee8bf15dcf4375"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-016" sheetId="16" r:id="Rc7ee2b3265944ef6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-017" sheetId="17" r:id="Rd904e89a2a1741ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-018" sheetId="18" r:id="Rc4c69e8570e942b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-019" sheetId="19" r:id="R6d1f49a2eb7d4a75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-020" sheetId="20" r:id="Rb3cbed9abf0a4513"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-021" sheetId="21" r:id="R5d4f371594524d25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-022" sheetId="22" r:id="R98e703ae3bae45b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-023" sheetId="23" r:id="R7bf45741d5a241fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-024" sheetId="24" r:id="R193a1b44f4014d96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-025" sheetId="25" r:id="Rbbb9117d1c6243bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-026" sheetId="26" r:id="R9a37f756fc8d42fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-027" sheetId="37" r:id="Re282aba8ca644b99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-028" sheetId="27" r:id="R9d9e73683e95496f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-029" sheetId="28" r:id="R05e03d32105f433d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-030" sheetId="29" r:id="R7eb46526703143fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-031" sheetId="30" r:id="Rcc252693adf54c45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-032" sheetId="31" r:id="R20e70cc1412d4787"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-033" sheetId="32" r:id="R6d3b4b0c8149485c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-034" sheetId="33" r:id="R44601dc335604ab4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-035" sheetId="34" r:id="Rd528688e724f45ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-036" sheetId="35" r:id="R4d81549be4c54144"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-037" sheetId="36" r:id="R977d32247c364453"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-038" sheetId="38" r:id="R76b75c981ce24dc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-039" sheetId="39" r:id="R2b47635be48b4477"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-040" sheetId="40" r:id="R5d8aabde5f2d4056"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-041" sheetId="41" r:id="R4dc32c77df074104"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-042" sheetId="42" r:id="R5e3a2d21d3d746e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-043" sheetId="43" r:id="Rea9dd5ffc102464f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-044" sheetId="44" r:id="R51920e1237404b38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-045" sheetId="79" r:id="R9c860c362e45499f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-046" sheetId="46" r:id="Reb0d42318d43408a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-047" sheetId="47" r:id="R362d4bd60da34ce4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-048" sheetId="52" r:id="Rfe7b4b013ace4e13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-049" sheetId="53" r:id="R868555eb020945fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-050" sheetId="54" r:id="R430dab95cc4b47e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-051" sheetId="55" r:id="R941afe461e75455f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-052" sheetId="56" r:id="R4976adf0154143bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-053" sheetId="57" r:id="Re92e680aa37144e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-054" sheetId="48" r:id="Rde5e96c1f49e452f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-055" sheetId="49" r:id="R81798ed6dd8943bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-056" sheetId="80" r:id="R982578f4b43e46e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-057" sheetId="70" r:id="Rcc34540ab4964de9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-058" sheetId="58" r:id="R77995a0e675147ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-059" sheetId="81" r:id="R29ddd604093b4ee3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-060" sheetId="63" r:id="R6bb36c82237c4461"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-061" sheetId="82" r:id="R64b80036184a4407"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-062" sheetId="64" r:id="Reea00d8c9dc448ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-063" sheetId="65" r:id="Rf098a3f9c7824e27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-064" sheetId="66" r:id="R73dbc3af6e3a400b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-065" sheetId="67" r:id="Rb8f2edba092b4faf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-066" sheetId="68" r:id="R86c985c29d484b23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-067" sheetId="69" r:id="Re170bd135c34421a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-068" sheetId="71" r:id="Rd396d1bfd14843c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-069" sheetId="72" r:id="R7e01bca22ffd4aa0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-070" sheetId="73" r:id="R9cf6d19e368749bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-071" sheetId="74" r:id="R69ec39ea8c96444f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-072" sheetId="75" r:id="R9f7a8052f8d94ca9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-073" sheetId="76" r:id="Rb0d8a45a4ad0479e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-074" sheetId="77" r:id="Rf514bcea3f094e86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-075" sheetId="78" r:id="Reae4e171eccf40f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-001" sheetId="1" r:id="Re3d60d232002441c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-002" sheetId="2" r:id="Reaff004d4fb54bad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-003" sheetId="3" r:id="R8838b10aed8a4616"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-004" sheetId="4" r:id="R31dceb04a79b41d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-005" sheetId="5" r:id="R45a8515e4def4173"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-006" sheetId="6" r:id="R6de82e3aa9e74108"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-007" sheetId="7" r:id="R45efd9e865d14a0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-008" sheetId="8" r:id="Rc51e5a0284ce4359"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-009" sheetId="9" r:id="Rca106a0fa9f04f82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-010" sheetId="10" r:id="R2ef531694d804715"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-011" sheetId="11" r:id="Rd376e3bc62464cdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-012" sheetId="12" r:id="R11e36c15d7c24576"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-013" sheetId="13" r:id="Rc0840a5829504498"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-014" sheetId="14" r:id="R92491fb6435f4e14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-015" sheetId="15" r:id="R507f6ad758c54f3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-016" sheetId="16" r:id="R3a7422a324b0465a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-017" sheetId="17" r:id="Rbc4b27f61b0c4a63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-018" sheetId="18" r:id="R5b5a4242ebfe46a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-019" sheetId="19" r:id="Rdf26e27e817647df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-020" sheetId="20" r:id="Rf0bf0f6b94ba4768"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-021" sheetId="21" r:id="Radc2a298fb244a93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-022" sheetId="22" r:id="Ra9b02ae62bf94948"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-023" sheetId="23" r:id="R16f20d6d462b45c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-024" sheetId="24" r:id="Rbb003898dba74f8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-025" sheetId="25" r:id="R1a92c8ba899a4a81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-026" sheetId="26" r:id="Ra814fa2a3f8b4b0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-027" sheetId="37" r:id="Reb05a109f9834fb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-028" sheetId="27" r:id="R6b104ccc23564c78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-029" sheetId="28" r:id="R97afb3f8d90c4c41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-030" sheetId="29" r:id="Rf1ab75245c8c4110"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-031" sheetId="30" r:id="R80e2754764a54786"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-032" sheetId="31" r:id="Re4899ecf53d04210"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-033" sheetId="32" r:id="R2d90060736284376"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-034" sheetId="33" r:id="R0c4ebd46480247bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-035" sheetId="34" r:id="R91fc92cb87c74b65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-036" sheetId="35" r:id="R74df7aedc09c4dd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-037" sheetId="36" r:id="Ra0c5f2e3f9d74b6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-038" sheetId="38" r:id="R214c4806c4804a64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-039" sheetId="39" r:id="Raea840452a2a4e95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-040" sheetId="40" r:id="R505193ec7b414332"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-041" sheetId="41" r:id="R976252189c7641a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-042" sheetId="42" r:id="R8cc3e6f82a2e43b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-043" sheetId="43" r:id="Re32586e690aa45e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-044" sheetId="44" r:id="Rda52f2d3a38441ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-045" sheetId="79" r:id="R1f27c28613974eb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-046" sheetId="46" r:id="Rc3ad41954f084760"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-047" sheetId="47" r:id="R2cf387e2f06d46b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-048" sheetId="52" r:id="R5d432b69f0df476e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-049" sheetId="53" r:id="R2ce1a1c77a3b4206"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-050" sheetId="54" r:id="Re3e536489c3e4549"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-051" sheetId="55" r:id="Rb502b55cdcf64086"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-052" sheetId="56" r:id="R11fd0812c4cd45ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-053" sheetId="57" r:id="R18acae09662e4b65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-054" sheetId="48" r:id="R088b5890b4f34bd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-055" sheetId="49" r:id="Rd7d20d56caa74cff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-056" sheetId="80" r:id="R7eeabb56c43b4b61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-057" sheetId="70" r:id="R07d2e82871dc4335"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-058" sheetId="58" r:id="R1aef3219c29347a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-059" sheetId="81" r:id="Ra2ad9d2e80f24ee2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-060" sheetId="63" r:id="R9295ca66ffc94eb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-061" sheetId="82" r:id="R251969822bfa464a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-062" sheetId="64" r:id="R1d7753a6c8594db0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-063" sheetId="65" r:id="R5dff84819d864e32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-064" sheetId="66" r:id="Rafc64599ef564a3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-065" sheetId="67" r:id="R914316d04df241c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-066" sheetId="68" r:id="R091c0dd69f6a44fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-067" sheetId="69" r:id="R0c1829c8420f493c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-068" sheetId="71" r:id="R622a1dab730948c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-069" sheetId="72" r:id="Rbd1bc953bf6a4a23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-070" sheetId="73" r:id="Rebf606570b6f4575"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-071" sheetId="74" r:id="Rf42a2c2145da41ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-072" sheetId="75" r:id="R1fa9348c73dc40dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-073" sheetId="76" r:id="R672cd6701c8d4dcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-074" sheetId="77" r:id="Rc0f2959263c64354"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-075" sheetId="78" r:id="R6fa511d7a3e44119"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -51161,8 +51161,8 @@
       </x:c>
       <x:c r="AF3" s="6"/>
       <x:c r="AG3" s="6"/>
-      <x:c r="AH3" s="25" t="s">
-        <x:v>140</x:v>
+      <x:c r="AH3" s="25" t="str">
+        <x:v>(tb1.状態 = 'ACTIVE'</x:v>
       </x:c>
       <x:c r="AI3" s="6"/>
       <x:c r="AJ3" s="6"/>
@@ -51257,8 +51257,8 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="AG4" s="3"/>
-      <x:c r="AH4" s="27" t="s">
-        <x:v>223</x:v>
+      <x:c r="AH4" s="27" t="str">
+        <x:v>tb1.削除日時 IS NULL) → 1</x:v>
       </x:c>
       <x:c r="AI4" s="3"/>
       <x:c r="AJ4" s="3"/>

</xml_diff>

<commit_message>
test: add provisional multi-row insert expectations
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -2,81 +2,83 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-001" sheetId="1" r:id="Rf686810751fe4d68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-002" sheetId="2" r:id="Ra8011ad2fb864d89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-003" sheetId="3" r:id="Rffd839c4de9649fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-004" sheetId="4" r:id="Rf1d4ae1f86774a6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-005" sheetId="5" r:id="R67a879a598374ee1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-006" sheetId="6" r:id="R856a947654fd47fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-007" sheetId="7" r:id="Rbbe8367cb8e9404e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-008" sheetId="8" r:id="R6a2463e8b88649bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-009" sheetId="9" r:id="Rd6d10fca3cc2413f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-010" sheetId="10" r:id="Rc9577af229544780"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-011" sheetId="11" r:id="R1bad759e45764704"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-012" sheetId="12" r:id="R798648c165074af0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-013" sheetId="13" r:id="R72ed89b42d4d4e9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-014" sheetId="14" r:id="R659aed7c8a65441b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-015" sheetId="15" r:id="R2ffdf17dddf944f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-016" sheetId="16" r:id="R7ce821e416dc45e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-017" sheetId="17" r:id="R316bce1dee824e74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-018" sheetId="18" r:id="R591a234213f64c37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-019" sheetId="19" r:id="R57a9330b0c0f4289"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-020" sheetId="20" r:id="R3991a239326d4630"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-021" sheetId="21" r:id="Rce57e1f3bb4c497e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-022" sheetId="22" r:id="R33b74155f2924354"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-023" sheetId="23" r:id="Ra10fd05be90442ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-024" sheetId="24" r:id="Re4dbdfb9dbd14ec4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-025" sheetId="25" r:id="R043a8422f1794809"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-026" sheetId="26" r:id="R3d6ffc678d4a486b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-027" sheetId="37" r:id="R7a6cd80f98a84f7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-028" sheetId="27" r:id="Rffd96d3bbf7649a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-029" sheetId="28" r:id="Raf1e07e377084a8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-030" sheetId="29" r:id="R7d46c0ee8a414c76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-031" sheetId="30" r:id="Rc8738514743f4a90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-032" sheetId="31" r:id="R8708216bc321499d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-033" sheetId="32" r:id="Rab7130daa005447c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-034" sheetId="33" r:id="R4f1d196ec7a44b7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-035" sheetId="34" r:id="Re99af788f1354b3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-036" sheetId="35" r:id="R406ab449c7c74922"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-037" sheetId="36" r:id="Rcd3f99b5ee4c4565"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-038" sheetId="38" r:id="R410e33190db4407e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-039" sheetId="39" r:id="R4e49618187424b0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-040" sheetId="40" r:id="R76d7dac6ecab4608"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-041" sheetId="41" r:id="Rc3b8501ac0e2472c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-042" sheetId="42" r:id="Rc741462d1047443a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-043" sheetId="43" r:id="R9fad8dd7ed7943b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-044" sheetId="44" r:id="Rd5d531fd49754f94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-045" sheetId="79" r:id="Rc016684d579649dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-046" sheetId="46" r:id="R3add21420b2d4e29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-047" sheetId="47" r:id="Rba84b9c179ad4340"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-048" sheetId="52" r:id="R503eebaf238e482a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-049" sheetId="53" r:id="R509e172818f14cd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-050" sheetId="54" r:id="Raf7f88a22fa446a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-051" sheetId="55" r:id="Rcff2e1bc2fc1472e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-052" sheetId="56" r:id="R4d0c73cb80fd4846"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-053" sheetId="57" r:id="R2a13f7f5e6694a1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-054" sheetId="48" r:id="Rbee5a001ef9e4a7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-055" sheetId="49" r:id="R502f0d51c28941fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-056" sheetId="80" r:id="R54bfd7f31c2445d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-057" sheetId="70" r:id="Rd9440d6dffbd46f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-058" sheetId="58" r:id="R5c7a13eb95194e54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-059" sheetId="81" r:id="R8151e5f210a8495f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-060" sheetId="63" r:id="R84f48c47f8404f35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-061" sheetId="82" r:id="R60f6b69d9f7a495b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-062" sheetId="64" r:id="Rde9348b969dd489b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-063" sheetId="65" r:id="R7610585d4d184198"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-064" sheetId="66" r:id="Re7cfa79e9c4b47c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-065" sheetId="67" r:id="Ra03a08e139fa4f86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-066" sheetId="68" r:id="Rd2d3e69b40c24dd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-067" sheetId="69" r:id="R58200b61814343f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-068" sheetId="71" r:id="R1a81ccfd03df44d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-069" sheetId="72" r:id="Rc8b19ed7e3e54756"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-070" sheetId="73" r:id="R04b675fe77974344"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-071" sheetId="74" r:id="Rce21db7d5f6b47a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-072" sheetId="75" r:id="R98594971f23f4c22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-073" sheetId="76" r:id="Raeee1dbf3f35424b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-074" sheetId="77" r:id="R79dde9fdad034be4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-075" sheetId="78" r:id="R4107ca8b06d94454"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-001" sheetId="1" r:id="R90522b0d9b3046f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-002" sheetId="2" r:id="R2f580149777549a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-003" sheetId="3" r:id="R5a9596d56a294bed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-004" sheetId="4" r:id="R63c32d0dbda2420b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-005" sheetId="5" r:id="R821d4f9bd2fb4104"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-006" sheetId="6" r:id="Reb793db6563f4eb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-007" sheetId="7" r:id="R2f5485cee91f4f92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-008" sheetId="8" r:id="R7ea4b9c4ac8c432a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-009" sheetId="9" r:id="R443b55cf0b0c4891"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-010" sheetId="10" r:id="R1f4b9bbc1c404629"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-011" sheetId="11" r:id="R4487c9fa764847b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-012" sheetId="12" r:id="Rd2e39118cbbc4242"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-013" sheetId="13" r:id="Rbebbc9167cfb4b7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-014" sheetId="14" r:id="R49b03ec6231944ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-015" sheetId="15" r:id="Rbe22d6b94766448d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-016" sheetId="16" r:id="R99b325f2c6614f89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-017" sheetId="17" r:id="R8180eda84f6543d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-018" sheetId="18" r:id="R8c84f33331e74cfd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-019" sheetId="19" r:id="R222bd4dce1114a58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-020" sheetId="20" r:id="R6e8a38f666804bbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-021" sheetId="21" r:id="R914cab2b3baa4132"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-022" sheetId="22" r:id="Readea579412b4f7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-023" sheetId="23" r:id="R5a32e5cb303340eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-024" sheetId="24" r:id="R72ea034dc2e64263"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-025" sheetId="25" r:id="R55d542803e4f407c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-026" sheetId="26" r:id="Rec4f8650793849e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-027" sheetId="37" r:id="R2715f25b66f54378"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-028" sheetId="27" r:id="R55f117de58fc4d6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-029" sheetId="28" r:id="Re99d349348644416"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-030" sheetId="29" r:id="Rb58c9ca6a8ef4027"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-031" sheetId="30" r:id="R555408f05bbe4b6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-032" sheetId="31" r:id="Rd425e53b8eae45a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-033" sheetId="32" r:id="Rba529a6d16c44931"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-034" sheetId="33" r:id="Rb79284f1fdae446a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-035" sheetId="34" r:id="Rf581733061e244c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-036" sheetId="35" r:id="Rfec22ff4c41f41ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-037" sheetId="36" r:id="R26c80b031f4a420e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-038" sheetId="38" r:id="R4d4d050bd3154297"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-039" sheetId="39" r:id="Rde2eb570d97e4c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-040" sheetId="40" r:id="R220f963822fc48df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-041" sheetId="41" r:id="R345fb4f00558481c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-042" sheetId="42" r:id="R93d2f1c78f9a4cff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-043" sheetId="43" r:id="Rd23883b40c024de0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-044" sheetId="44" r:id="Rd4cd261b865d4679"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-045" sheetId="79" r:id="Rb9e92253910743da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-046" sheetId="46" r:id="R1142a2e82f5e4b55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-047" sheetId="47" r:id="R90a5c7b8d0d94907"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-048" sheetId="52" r:id="Ra8b511cc1a404e38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-049" sheetId="53" r:id="R00ba6cfcc1d34c5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-050" sheetId="54" r:id="R31dc0a7e09f949ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-051" sheetId="55" r:id="R3250861511a6418f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-052" sheetId="56" r:id="R80676cbeaa104554"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-053" sheetId="57" r:id="R4c02ad32ecf14484"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-054" sheetId="48" r:id="R1c51b935f07b41ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-055" sheetId="49" r:id="Re7031591db684831"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-056" sheetId="80" r:id="Rdecaea7f738a4e66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-057" sheetId="70" r:id="R590b917de9544387"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-058" sheetId="58" r:id="Rad350a3fc5184c33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-059" sheetId="81" r:id="Rd84c5d71bdb74870"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-060" sheetId="63" r:id="Re87660ded3524994"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-061" sheetId="82" r:id="Rf2369ef8ba394fe6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-062" sheetId="64" r:id="R3a62405d1ae34adf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-063" sheetId="65" r:id="Rc0bb938c60f04754"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-064" sheetId="66" r:id="R6031ae8f15fa451f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-065" sheetId="67" r:id="R6fb8f183be9b4ad7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-066" sheetId="68" r:id="Rce181c168a984261"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-067" sheetId="69" r:id="R27963fd5d85143e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-068" sheetId="71" r:id="Rf85843c9c9714948"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-069" sheetId="72" r:id="Rdde18e46e328408f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-070" sheetId="73" r:id="R795178ccde074e86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-071" sheetId="74" r:id="R4fcb7d917aa64fba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-072" sheetId="75" r:id="Rac00426f96a64e3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-073" sheetId="76" r:id="R61faed93ae344ca0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-074" sheetId="77" r:id="R1e1a2bbf2a6b4b36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-075" sheetId="78" r:id="R97c4463a2ec841c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-076" sheetId="83" r:id="R29df998fd1e64d00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-077" sheetId="84" r:id="Rfa60a475ad564d36"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -935,7 +937,7 @@
       <x:name val="游ゴシック"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -950,6 +952,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2CEEF"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -1109,7 +1121,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="60">
+  <x:cellXfs count="85">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -1288,6 +1300,81 @@
       <x:alignment vertical="center" wrapText="0"/>
     </x:xf>
     <x:xf numFmtId="49" fontId="1" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
@@ -53990,6 +54077,3468 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="33" max="33" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="35" max="35" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="36" max="36" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="37" max="37" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="38" max="38" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="39" max="39" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="40" max="40" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="41" max="41" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="42" max="42" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="43" max="43" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="44" max="44" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="45" max="45" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="46" max="46" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="47" max="47" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="48" max="48" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="49" max="49" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="50" max="50" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="51" max="51" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="52" max="52" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="53" max="53" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="54" max="54" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="55" max="55" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="56" max="56" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="57" max="57" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="58" max="58" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="59" max="59" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="60" max="60" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="61" max="61" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="62" max="62" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="63" max="63" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="64" max="64" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="65" max="65" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="66" max="66" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="67" max="67" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="68" max="68" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="69" max="69" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="70" max="70" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="71" max="71" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="72" max="72" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="73" max="73" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="74" max="74" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="75" max="75" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="76" max="76" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="77" max="77" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="78" max="78" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="79" max="79" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="80" max="80" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="81" max="81" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="82" max="82" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="83" max="83" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="84" max="84" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="85" max="85" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="86" max="86" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="87" max="87" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="88" max="88" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="89" max="89" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="90" max="90" width="1.1399999856948853" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="13.5" customHeight="1">
+      <x:c r="A1" s="61" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="B1" s="61"/>
+      <x:c r="C1" s="61"/>
+      <x:c r="D1" s="61"/>
+      <x:c r="E1" s="61"/>
+      <x:c r="F1" s="61"/>
+      <x:c r="G1" s="61"/>
+      <x:c r="H1" s="61"/>
+      <x:c r="I1" s="61"/>
+      <x:c r="J1" s="61"/>
+      <x:c r="K1" s="61"/>
+      <x:c r="L1" s="61"/>
+      <x:c r="M1" s="61"/>
+      <x:c r="N1" s="61"/>
+      <x:c r="O1" s="61"/>
+      <x:c r="P1" s="61"/>
+      <x:c r="Q1" s="61"/>
+      <x:c r="R1" s="61"/>
+      <x:c r="S1" s="61"/>
+      <x:c r="T1" s="61"/>
+      <x:c r="U1" s="61"/>
+      <x:c r="V1" s="61"/>
+      <x:c r="W1" s="61"/>
+      <x:c r="X1" s="61"/>
+      <x:c r="Y1" s="61"/>
+      <x:c r="Z1" s="61"/>
+      <x:c r="AA1" s="61"/>
+      <x:c r="AB1" s="61"/>
+      <x:c r="AC1" s="61"/>
+      <x:c r="AD1" s="61"/>
+      <x:c r="AE1" s="61"/>
+      <x:c r="AF1" s="61"/>
+      <x:c r="AG1" s="61"/>
+      <x:c r="AH1" s="61"/>
+      <x:c r="AI1" s="61"/>
+      <x:c r="AJ1" s="61"/>
+      <x:c r="AK1" s="61"/>
+      <x:c r="AL1" s="61"/>
+      <x:c r="AM1" s="61"/>
+      <x:c r="AN1" s="61"/>
+      <x:c r="AO1" s="61"/>
+      <x:c r="AP1" s="61"/>
+      <x:c r="AQ1" s="61"/>
+      <x:c r="AR1" s="61"/>
+      <x:c r="AS1" s="61"/>
+      <x:c r="AT1" s="61"/>
+      <x:c r="AU1" s="61"/>
+      <x:c r="AV1" s="61"/>
+      <x:c r="AW1" s="61"/>
+      <x:c r="AX1" s="61"/>
+      <x:c r="AY1" s="61"/>
+      <x:c r="AZ1" s="61"/>
+      <x:c r="BA1" s="61"/>
+      <x:c r="BB1" s="61"/>
+      <x:c r="BC1" s="61"/>
+      <x:c r="BD1" s="61"/>
+      <x:c r="BE1" s="61"/>
+      <x:c r="BF1" s="61"/>
+      <x:c r="BG1" s="61"/>
+      <x:c r="BH1" s="61"/>
+      <x:c r="BI1" s="61"/>
+      <x:c r="BJ1" s="61"/>
+      <x:c r="BK1" s="61"/>
+      <x:c r="BL1" s="61"/>
+      <x:c r="BM1" s="61"/>
+      <x:c r="BN1" s="61"/>
+      <x:c r="BO1" s="61"/>
+      <x:c r="BP1" s="61"/>
+      <x:c r="BQ1" s="61"/>
+      <x:c r="BR1" s="61"/>
+      <x:c r="BS1" s="61"/>
+      <x:c r="BT1" s="61"/>
+      <x:c r="BU1" s="61"/>
+      <x:c r="BV1" s="61"/>
+      <x:c r="BW1" s="61"/>
+      <x:c r="BX1" s="61"/>
+      <x:c r="BY1" s="61"/>
+      <x:c r="BZ1" s="61"/>
+      <x:c r="CA1" s="61"/>
+      <x:c r="CB1" s="61"/>
+      <x:c r="CC1" s="61"/>
+      <x:c r="CD1" s="61"/>
+      <x:c r="CE1" s="61"/>
+      <x:c r="CF1" s="61"/>
+      <x:c r="CG1" s="61"/>
+      <x:c r="CH1" s="61"/>
+      <x:c r="CI1" s="61"/>
+      <x:c r="CJ1" s="61"/>
+      <x:c r="CK1" s="61"/>
+      <x:c r="CL1" s="61"/>
+    </x:row>
+    <x:row r="2" ht="13.5" customHeight="1">
+      <x:c r="A2" s="61" t="s">
+        <x:v>230</x:v>
+      </x:c>
+      <x:c r="B2" s="61"/>
+      <x:c r="C2" s="61"/>
+      <x:c r="D2" s="61"/>
+      <x:c r="E2" s="61"/>
+      <x:c r="F2" s="61"/>
+      <x:c r="G2" s="61"/>
+      <x:c r="H2" s="61"/>
+      <x:c r="I2" s="61"/>
+      <x:c r="J2" s="61"/>
+      <x:c r="K2" s="61"/>
+      <x:c r="L2" s="61"/>
+      <x:c r="M2" s="61"/>
+      <x:c r="N2" s="61"/>
+      <x:c r="O2" s="61"/>
+      <x:c r="P2" s="61"/>
+      <x:c r="Q2" s="61"/>
+      <x:c r="R2" s="61"/>
+      <x:c r="S2" s="61"/>
+      <x:c r="T2" s="61"/>
+      <x:c r="U2" s="61"/>
+      <x:c r="V2" s="61"/>
+      <x:c r="W2" s="61"/>
+      <x:c r="X2" s="61"/>
+      <x:c r="Y2" s="61"/>
+      <x:c r="Z2" s="61"/>
+      <x:c r="AA2" s="61"/>
+      <x:c r="AB2" s="61"/>
+      <x:c r="AC2" s="61"/>
+      <x:c r="AD2" s="61"/>
+      <x:c r="AE2" s="61"/>
+      <x:c r="AF2" s="61"/>
+      <x:c r="AG2" s="61"/>
+      <x:c r="AH2" s="61"/>
+      <x:c r="AI2" s="61"/>
+      <x:c r="AJ2" s="61"/>
+      <x:c r="AK2" s="61"/>
+      <x:c r="AL2" s="61"/>
+      <x:c r="AM2" s="61"/>
+      <x:c r="AN2" s="61"/>
+      <x:c r="AO2" s="61"/>
+      <x:c r="AP2" s="61"/>
+      <x:c r="AQ2" s="61"/>
+      <x:c r="AR2" s="61"/>
+      <x:c r="AS2" s="61"/>
+      <x:c r="AT2" s="61"/>
+      <x:c r="AU2" s="61"/>
+      <x:c r="AV2" s="61"/>
+      <x:c r="AW2" s="61"/>
+      <x:c r="AX2" s="61"/>
+      <x:c r="AY2" s="61"/>
+      <x:c r="AZ2" s="61"/>
+      <x:c r="BA2" s="61"/>
+      <x:c r="BB2" s="61"/>
+      <x:c r="BC2" s="61"/>
+      <x:c r="BD2" s="61"/>
+      <x:c r="BE2" s="61"/>
+      <x:c r="BF2" s="61"/>
+      <x:c r="BG2" s="61"/>
+      <x:c r="BH2" s="61"/>
+      <x:c r="BI2" s="61"/>
+      <x:c r="BJ2" s="61"/>
+      <x:c r="BK2" s="61"/>
+      <x:c r="BL2" s="61"/>
+      <x:c r="BM2" s="61"/>
+      <x:c r="BN2" s="61"/>
+      <x:c r="BO2" s="61"/>
+      <x:c r="BP2" s="61"/>
+      <x:c r="BQ2" s="61"/>
+      <x:c r="BR2" s="61"/>
+      <x:c r="BS2" s="61"/>
+      <x:c r="BT2" s="61"/>
+      <x:c r="BU2" s="61"/>
+      <x:c r="BV2" s="61"/>
+      <x:c r="BW2" s="61"/>
+      <x:c r="BX2" s="61"/>
+      <x:c r="BY2" s="61"/>
+      <x:c r="BZ2" s="61"/>
+      <x:c r="CA2" s="61"/>
+      <x:c r="CB2" s="61"/>
+      <x:c r="CC2" s="61"/>
+      <x:c r="CD2" s="61"/>
+      <x:c r="CE2" s="61"/>
+      <x:c r="CF2" s="61"/>
+      <x:c r="CG2" s="61"/>
+      <x:c r="CH2" s="61"/>
+      <x:c r="CI2" s="61"/>
+      <x:c r="CJ2" s="61"/>
+      <x:c r="CK2" s="61"/>
+      <x:c r="CL2" s="61"/>
+    </x:row>
+    <x:row r="3" ht="13.5" customHeight="1">
+      <x:c r="A3" s="63" t="str">
+        <x:v>＜VALUES 1行目＞</x:v>
+      </x:c>
+      <x:c r="B3" s="63"/>
+      <x:c r="C3" s="63"/>
+      <x:c r="D3" s="63"/>
+      <x:c r="E3" s="63"/>
+      <x:c r="F3" s="63"/>
+      <x:c r="G3" s="63"/>
+      <x:c r="H3" s="63"/>
+      <x:c r="I3" s="63"/>
+      <x:c r="J3" s="63"/>
+      <x:c r="K3" s="63"/>
+      <x:c r="L3" s="63"/>
+      <x:c r="M3" s="63"/>
+      <x:c r="N3" s="63"/>
+      <x:c r="O3" s="63"/>
+      <x:c r="P3" s="63"/>
+      <x:c r="Q3" s="63"/>
+      <x:c r="R3" s="63"/>
+      <x:c r="S3" s="63"/>
+      <x:c r="T3" s="63"/>
+      <x:c r="U3" s="63"/>
+      <x:c r="V3" s="63"/>
+      <x:c r="W3" s="63"/>
+      <x:c r="X3" s="63"/>
+      <x:c r="Y3" s="63"/>
+      <x:c r="Z3" s="63"/>
+      <x:c r="AA3" s="63"/>
+      <x:c r="AB3" s="63"/>
+      <x:c r="AC3" s="63"/>
+      <x:c r="AD3" s="63"/>
+      <x:c r="AE3" s="63"/>
+      <x:c r="AF3" s="63"/>
+      <x:c r="AG3" s="63"/>
+      <x:c r="AH3" s="63"/>
+      <x:c r="AI3" s="63"/>
+      <x:c r="AJ3" s="63"/>
+      <x:c r="AK3" s="63"/>
+      <x:c r="AL3" s="63"/>
+      <x:c r="AM3" s="63"/>
+      <x:c r="AN3" s="63"/>
+      <x:c r="AO3" s="63"/>
+      <x:c r="AP3" s="63"/>
+      <x:c r="AQ3" s="63"/>
+      <x:c r="AR3" s="63"/>
+      <x:c r="AS3" s="63"/>
+      <x:c r="AT3" s="63"/>
+      <x:c r="AU3" s="63"/>
+      <x:c r="AV3" s="63"/>
+      <x:c r="AW3" s="63"/>
+      <x:c r="AX3" s="63"/>
+      <x:c r="AY3" s="63"/>
+      <x:c r="AZ3" s="63"/>
+      <x:c r="BA3" s="63"/>
+      <x:c r="BB3" s="63"/>
+      <x:c r="BC3" s="63"/>
+      <x:c r="BD3" s="63"/>
+      <x:c r="BE3" s="63"/>
+      <x:c r="BF3" s="63"/>
+      <x:c r="BG3" s="63"/>
+      <x:c r="BH3" s="63"/>
+      <x:c r="BI3" s="63"/>
+      <x:c r="BJ3" s="63"/>
+      <x:c r="BK3" s="63"/>
+      <x:c r="BL3" s="63"/>
+      <x:c r="BM3" s="63"/>
+      <x:c r="BN3" s="63"/>
+      <x:c r="BO3" s="63"/>
+      <x:c r="BP3" s="63"/>
+      <x:c r="BQ3" s="63"/>
+      <x:c r="BR3" s="63"/>
+      <x:c r="BS3" s="63"/>
+      <x:c r="BT3" s="63"/>
+      <x:c r="BU3" s="63"/>
+      <x:c r="BV3" s="63"/>
+      <x:c r="BW3" s="63"/>
+      <x:c r="BX3" s="63"/>
+      <x:c r="BY3" s="63"/>
+      <x:c r="BZ3" s="63"/>
+      <x:c r="CA3" s="63"/>
+      <x:c r="CB3" s="63"/>
+      <x:c r="CC3" s="63"/>
+      <x:c r="CD3" s="63"/>
+      <x:c r="CE3" s="63"/>
+      <x:c r="CF3" s="63"/>
+      <x:c r="CG3" s="63"/>
+      <x:c r="CH3" s="63"/>
+      <x:c r="CI3" s="63"/>
+      <x:c r="CJ3" s="63"/>
+      <x:c r="CK3" s="63"/>
+      <x:c r="CL3" s="63"/>
+    </x:row>
+    <x:row r="4" ht="13.5" customHeight="1">
+      <x:c r="A4" s="67" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="B4" s="68"/>
+      <x:c r="C4" s="68"/>
+      <x:c r="D4" s="68"/>
+      <x:c r="E4" s="68"/>
+      <x:c r="F4" s="68"/>
+      <x:c r="G4" s="68"/>
+      <x:c r="H4" s="68"/>
+      <x:c r="I4" s="68"/>
+      <x:c r="J4" s="68"/>
+      <x:c r="K4" s="68"/>
+      <x:c r="L4" s="68"/>
+      <x:c r="M4" s="68"/>
+      <x:c r="N4" s="68"/>
+      <x:c r="O4" s="68"/>
+      <x:c r="P4" s="68"/>
+      <x:c r="Q4" s="68"/>
+      <x:c r="R4" s="68"/>
+      <x:c r="S4" s="67" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="T4" s="68"/>
+      <x:c r="U4" s="68"/>
+      <x:c r="V4" s="68"/>
+      <x:c r="W4" s="68"/>
+      <x:c r="X4" s="68"/>
+      <x:c r="Y4" s="68"/>
+      <x:c r="Z4" s="68"/>
+      <x:c r="AA4" s="68"/>
+      <x:c r="AB4" s="68"/>
+      <x:c r="AC4" s="68"/>
+      <x:c r="AD4" s="68"/>
+      <x:c r="AE4" s="68"/>
+      <x:c r="AF4" s="68"/>
+      <x:c r="AG4" s="68"/>
+      <x:c r="AH4" s="68"/>
+      <x:c r="AI4" s="68"/>
+      <x:c r="AJ4" s="68"/>
+      <x:c r="AK4" s="67" t="str">
+        <x:v>移送方法ほか</x:v>
+      </x:c>
+      <x:c r="AL4" s="68"/>
+      <x:c r="AM4" s="68"/>
+      <x:c r="AN4" s="68"/>
+      <x:c r="AO4" s="68"/>
+      <x:c r="AP4" s="68"/>
+      <x:c r="AQ4" s="68"/>
+      <x:c r="AR4" s="68"/>
+      <x:c r="AS4" s="68"/>
+      <x:c r="AT4" s="68"/>
+      <x:c r="AU4" s="68"/>
+      <x:c r="AV4" s="68"/>
+      <x:c r="AW4" s="68"/>
+      <x:c r="AX4" s="68"/>
+      <x:c r="AY4" s="68"/>
+      <x:c r="AZ4" s="68"/>
+      <x:c r="BA4" s="68"/>
+      <x:c r="BB4" s="68"/>
+      <x:c r="BC4" s="68"/>
+      <x:c r="BD4" s="68"/>
+      <x:c r="BE4" s="68"/>
+      <x:c r="BF4" s="68"/>
+      <x:c r="BG4" s="68"/>
+      <x:c r="BH4" s="68"/>
+      <x:c r="BI4" s="68"/>
+      <x:c r="BJ4" s="68"/>
+      <x:c r="BK4" s="68"/>
+      <x:c r="BL4" s="68"/>
+      <x:c r="BM4" s="68"/>
+      <x:c r="BN4" s="68"/>
+      <x:c r="BO4" s="68"/>
+      <x:c r="BP4" s="68"/>
+      <x:c r="BQ4" s="68"/>
+      <x:c r="BR4" s="68"/>
+      <x:c r="BS4" s="68"/>
+      <x:c r="BT4" s="68"/>
+      <x:c r="BU4" s="68"/>
+      <x:c r="BV4" s="68"/>
+      <x:c r="BW4" s="68"/>
+      <x:c r="BX4" s="68"/>
+      <x:c r="BY4" s="68"/>
+      <x:c r="BZ4" s="68"/>
+      <x:c r="CA4" s="68"/>
+      <x:c r="CB4" s="68"/>
+      <x:c r="CC4" s="68"/>
+      <x:c r="CD4" s="68"/>
+      <x:c r="CE4" s="68"/>
+      <x:c r="CF4" s="68"/>
+      <x:c r="CG4" s="68"/>
+      <x:c r="CH4" s="68"/>
+      <x:c r="CI4" s="68"/>
+      <x:c r="CJ4" s="68"/>
+      <x:c r="CK4" s="68"/>
+      <x:c r="CL4" s="69"/>
+    </x:row>
+    <x:row r="5" ht="13.5" customHeight="1">
+      <x:c r="A5" s="64" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="B5" s="65"/>
+      <x:c r="C5" s="65"/>
+      <x:c r="D5" s="65"/>
+      <x:c r="E5" s="65"/>
+      <x:c r="F5" s="65"/>
+      <x:c r="G5" s="65"/>
+      <x:c r="H5" s="65"/>
+      <x:c r="I5" s="65"/>
+      <x:c r="J5" s="65"/>
+      <x:c r="K5" s="65"/>
+      <x:c r="L5" s="65"/>
+      <x:c r="M5" s="65"/>
+      <x:c r="N5" s="65"/>
+      <x:c r="O5" s="65"/>
+      <x:c r="P5" s="65"/>
+      <x:c r="Q5" s="65"/>
+      <x:c r="R5" s="65"/>
+      <x:c r="S5" s="64"/>
+      <x:c r="T5" s="65"/>
+      <x:c r="U5" s="65"/>
+      <x:c r="V5" s="65"/>
+      <x:c r="W5" s="65"/>
+      <x:c r="X5" s="65"/>
+      <x:c r="Y5" s="65"/>
+      <x:c r="Z5" s="65"/>
+      <x:c r="AA5" s="65"/>
+      <x:c r="AB5" s="65"/>
+      <x:c r="AC5" s="65"/>
+      <x:c r="AD5" s="65"/>
+      <x:c r="AE5" s="65"/>
+      <x:c r="AF5" s="65"/>
+      <x:c r="AG5" s="65"/>
+      <x:c r="AH5" s="65"/>
+      <x:c r="AI5" s="65"/>
+      <x:c r="AJ5" s="65"/>
+      <x:c r="AK5" s="64" t="str">
+        <x:v>@user_id_1</x:v>
+      </x:c>
+      <x:c r="AL5" s="65"/>
+      <x:c r="AM5" s="65"/>
+      <x:c r="AN5" s="65"/>
+      <x:c r="AO5" s="65"/>
+      <x:c r="AP5" s="65"/>
+      <x:c r="AQ5" s="65"/>
+      <x:c r="AR5" s="65"/>
+      <x:c r="AS5" s="65"/>
+      <x:c r="AT5" s="65"/>
+      <x:c r="AU5" s="65"/>
+      <x:c r="AV5" s="65"/>
+      <x:c r="AW5" s="65"/>
+      <x:c r="AX5" s="65"/>
+      <x:c r="AY5" s="65"/>
+      <x:c r="AZ5" s="65"/>
+      <x:c r="BA5" s="65"/>
+      <x:c r="BB5" s="65"/>
+      <x:c r="BC5" s="65"/>
+      <x:c r="BD5" s="65"/>
+      <x:c r="BE5" s="65"/>
+      <x:c r="BF5" s="65"/>
+      <x:c r="BG5" s="65"/>
+      <x:c r="BH5" s="65"/>
+      <x:c r="BI5" s="65"/>
+      <x:c r="BJ5" s="65"/>
+      <x:c r="BK5" s="65"/>
+      <x:c r="BL5" s="65"/>
+      <x:c r="BM5" s="65"/>
+      <x:c r="BN5" s="65"/>
+      <x:c r="BO5" s="65"/>
+      <x:c r="BP5" s="65"/>
+      <x:c r="BQ5" s="65"/>
+      <x:c r="BR5" s="65"/>
+      <x:c r="BS5" s="65"/>
+      <x:c r="BT5" s="65"/>
+      <x:c r="BU5" s="65"/>
+      <x:c r="BV5" s="65"/>
+      <x:c r="BW5" s="65"/>
+      <x:c r="BX5" s="65"/>
+      <x:c r="BY5" s="65"/>
+      <x:c r="BZ5" s="65"/>
+      <x:c r="CA5" s="65"/>
+      <x:c r="CB5" s="65"/>
+      <x:c r="CC5" s="65"/>
+      <x:c r="CD5" s="65"/>
+      <x:c r="CE5" s="65"/>
+      <x:c r="CF5" s="65"/>
+      <x:c r="CG5" s="65"/>
+      <x:c r="CH5" s="65"/>
+      <x:c r="CI5" s="65"/>
+      <x:c r="CJ5" s="65"/>
+      <x:c r="CK5" s="65"/>
+      <x:c r="CL5" s="66"/>
+    </x:row>
+    <x:row r="6" ht="13.5" customHeight="1">
+      <x:c r="A6" s="64" t="s">
+        <x:v>151</x:v>
+      </x:c>
+      <x:c r="B6" s="65"/>
+      <x:c r="C6" s="65"/>
+      <x:c r="D6" s="65"/>
+      <x:c r="E6" s="65"/>
+      <x:c r="F6" s="65"/>
+      <x:c r="G6" s="65"/>
+      <x:c r="H6" s="65"/>
+      <x:c r="I6" s="65"/>
+      <x:c r="J6" s="65"/>
+      <x:c r="K6" s="65"/>
+      <x:c r="L6" s="65"/>
+      <x:c r="M6" s="65"/>
+      <x:c r="N6" s="65"/>
+      <x:c r="O6" s="65"/>
+      <x:c r="P6" s="65"/>
+      <x:c r="Q6" s="65"/>
+      <x:c r="R6" s="65"/>
+      <x:c r="S6" s="64"/>
+      <x:c r="T6" s="65"/>
+      <x:c r="U6" s="65"/>
+      <x:c r="V6" s="65"/>
+      <x:c r="W6" s="65"/>
+      <x:c r="X6" s="65"/>
+      <x:c r="Y6" s="65"/>
+      <x:c r="Z6" s="65"/>
+      <x:c r="AA6" s="65"/>
+      <x:c r="AB6" s="65"/>
+      <x:c r="AC6" s="65"/>
+      <x:c r="AD6" s="65"/>
+      <x:c r="AE6" s="65"/>
+      <x:c r="AF6" s="65"/>
+      <x:c r="AG6" s="65"/>
+      <x:c r="AH6" s="65"/>
+      <x:c r="AI6" s="65"/>
+      <x:c r="AJ6" s="65"/>
+      <x:c r="AK6" s="64" t="str">
+        <x:v>@name_1</x:v>
+      </x:c>
+      <x:c r="AL6" s="65"/>
+      <x:c r="AM6" s="65"/>
+      <x:c r="AN6" s="65"/>
+      <x:c r="AO6" s="65"/>
+      <x:c r="AP6" s="65"/>
+      <x:c r="AQ6" s="65"/>
+      <x:c r="AR6" s="65"/>
+      <x:c r="AS6" s="65"/>
+      <x:c r="AT6" s="65"/>
+      <x:c r="AU6" s="65"/>
+      <x:c r="AV6" s="65"/>
+      <x:c r="AW6" s="65"/>
+      <x:c r="AX6" s="65"/>
+      <x:c r="AY6" s="65"/>
+      <x:c r="AZ6" s="65"/>
+      <x:c r="BA6" s="65"/>
+      <x:c r="BB6" s="65"/>
+      <x:c r="BC6" s="65"/>
+      <x:c r="BD6" s="65"/>
+      <x:c r="BE6" s="65"/>
+      <x:c r="BF6" s="65"/>
+      <x:c r="BG6" s="65"/>
+      <x:c r="BH6" s="65"/>
+      <x:c r="BI6" s="65"/>
+      <x:c r="BJ6" s="65"/>
+      <x:c r="BK6" s="65"/>
+      <x:c r="BL6" s="65"/>
+      <x:c r="BM6" s="65"/>
+      <x:c r="BN6" s="65"/>
+      <x:c r="BO6" s="65"/>
+      <x:c r="BP6" s="65"/>
+      <x:c r="BQ6" s="65"/>
+      <x:c r="BR6" s="65"/>
+      <x:c r="BS6" s="65"/>
+      <x:c r="BT6" s="65"/>
+      <x:c r="BU6" s="65"/>
+      <x:c r="BV6" s="65"/>
+      <x:c r="BW6" s="65"/>
+      <x:c r="BX6" s="65"/>
+      <x:c r="BY6" s="65"/>
+      <x:c r="BZ6" s="65"/>
+      <x:c r="CA6" s="65"/>
+      <x:c r="CB6" s="65"/>
+      <x:c r="CC6" s="65"/>
+      <x:c r="CD6" s="65"/>
+      <x:c r="CE6" s="65"/>
+      <x:c r="CF6" s="65"/>
+      <x:c r="CG6" s="65"/>
+      <x:c r="CH6" s="65"/>
+      <x:c r="CI6" s="65"/>
+      <x:c r="CJ6" s="65"/>
+      <x:c r="CK6" s="65"/>
+      <x:c r="CL6" s="66"/>
+    </x:row>
+    <x:row r="7" ht="13.5" customHeight="1">
+      <x:c r="A7" s="64" t="s">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="B7" s="65"/>
+      <x:c r="C7" s="65"/>
+      <x:c r="D7" s="65"/>
+      <x:c r="E7" s="65"/>
+      <x:c r="F7" s="65"/>
+      <x:c r="G7" s="65"/>
+      <x:c r="H7" s="65"/>
+      <x:c r="I7" s="65"/>
+      <x:c r="J7" s="65"/>
+      <x:c r="K7" s="65"/>
+      <x:c r="L7" s="65"/>
+      <x:c r="M7" s="65"/>
+      <x:c r="N7" s="65"/>
+      <x:c r="O7" s="65"/>
+      <x:c r="P7" s="65"/>
+      <x:c r="Q7" s="65"/>
+      <x:c r="R7" s="65"/>
+      <x:c r="S7" s="64"/>
+      <x:c r="T7" s="65"/>
+      <x:c r="U7" s="65"/>
+      <x:c r="V7" s="65"/>
+      <x:c r="W7" s="65"/>
+      <x:c r="X7" s="65"/>
+      <x:c r="Y7" s="65"/>
+      <x:c r="Z7" s="65"/>
+      <x:c r="AA7" s="65"/>
+      <x:c r="AB7" s="65"/>
+      <x:c r="AC7" s="65"/>
+      <x:c r="AD7" s="65"/>
+      <x:c r="AE7" s="65"/>
+      <x:c r="AF7" s="65"/>
+      <x:c r="AG7" s="65"/>
+      <x:c r="AH7" s="65"/>
+      <x:c r="AI7" s="65"/>
+      <x:c r="AJ7" s="65"/>
+      <x:c r="AK7" s="64" t="str">
+        <x:v>'ACTIVE'</x:v>
+      </x:c>
+      <x:c r="AL7" s="65"/>
+      <x:c r="AM7" s="65"/>
+      <x:c r="AN7" s="65"/>
+      <x:c r="AO7" s="65"/>
+      <x:c r="AP7" s="65"/>
+      <x:c r="AQ7" s="65"/>
+      <x:c r="AR7" s="65"/>
+      <x:c r="AS7" s="65"/>
+      <x:c r="AT7" s="65"/>
+      <x:c r="AU7" s="65"/>
+      <x:c r="AV7" s="65"/>
+      <x:c r="AW7" s="65"/>
+      <x:c r="AX7" s="65"/>
+      <x:c r="AY7" s="65"/>
+      <x:c r="AZ7" s="65"/>
+      <x:c r="BA7" s="65"/>
+      <x:c r="BB7" s="65"/>
+      <x:c r="BC7" s="65"/>
+      <x:c r="BD7" s="65"/>
+      <x:c r="BE7" s="65"/>
+      <x:c r="BF7" s="65"/>
+      <x:c r="BG7" s="65"/>
+      <x:c r="BH7" s="65"/>
+      <x:c r="BI7" s="65"/>
+      <x:c r="BJ7" s="65"/>
+      <x:c r="BK7" s="65"/>
+      <x:c r="BL7" s="65"/>
+      <x:c r="BM7" s="65"/>
+      <x:c r="BN7" s="65"/>
+      <x:c r="BO7" s="65"/>
+      <x:c r="BP7" s="65"/>
+      <x:c r="BQ7" s="65"/>
+      <x:c r="BR7" s="65"/>
+      <x:c r="BS7" s="65"/>
+      <x:c r="BT7" s="65"/>
+      <x:c r="BU7" s="65"/>
+      <x:c r="BV7" s="65"/>
+      <x:c r="BW7" s="65"/>
+      <x:c r="BX7" s="65"/>
+      <x:c r="BY7" s="65"/>
+      <x:c r="BZ7" s="65"/>
+      <x:c r="CA7" s="65"/>
+      <x:c r="CB7" s="65"/>
+      <x:c r="CC7" s="65"/>
+      <x:c r="CD7" s="65"/>
+      <x:c r="CE7" s="65"/>
+      <x:c r="CF7" s="65"/>
+      <x:c r="CG7" s="65"/>
+      <x:c r="CH7" s="65"/>
+      <x:c r="CI7" s="65"/>
+      <x:c r="CJ7" s="65"/>
+      <x:c r="CK7" s="65"/>
+      <x:c r="CL7" s="66"/>
+    </x:row>
+    <x:row r="8" ht="13.5" customHeight="1">
+      <x:c r="A8" s="64" t="s">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="B8" s="65"/>
+      <x:c r="C8" s="65"/>
+      <x:c r="D8" s="65"/>
+      <x:c r="E8" s="65"/>
+      <x:c r="F8" s="65"/>
+      <x:c r="G8" s="65"/>
+      <x:c r="H8" s="65"/>
+      <x:c r="I8" s="65"/>
+      <x:c r="J8" s="65"/>
+      <x:c r="K8" s="65"/>
+      <x:c r="L8" s="65"/>
+      <x:c r="M8" s="65"/>
+      <x:c r="N8" s="65"/>
+      <x:c r="O8" s="65"/>
+      <x:c r="P8" s="65"/>
+      <x:c r="Q8" s="65"/>
+      <x:c r="R8" s="65"/>
+      <x:c r="S8" s="64"/>
+      <x:c r="T8" s="65"/>
+      <x:c r="U8" s="65"/>
+      <x:c r="V8" s="65"/>
+      <x:c r="W8" s="65"/>
+      <x:c r="X8" s="65"/>
+      <x:c r="Y8" s="65"/>
+      <x:c r="Z8" s="65"/>
+      <x:c r="AA8" s="65"/>
+      <x:c r="AB8" s="65"/>
+      <x:c r="AC8" s="65"/>
+      <x:c r="AD8" s="65"/>
+      <x:c r="AE8" s="65"/>
+      <x:c r="AF8" s="65"/>
+      <x:c r="AG8" s="65"/>
+      <x:c r="AH8" s="65"/>
+      <x:c r="AI8" s="65"/>
+      <x:c r="AJ8" s="65"/>
+      <x:c r="AK8" s="64" t="str">
+        <x:v>SYSDATETIME()</x:v>
+      </x:c>
+      <x:c r="AL8" s="65"/>
+      <x:c r="AM8" s="65"/>
+      <x:c r="AN8" s="65"/>
+      <x:c r="AO8" s="65"/>
+      <x:c r="AP8" s="65"/>
+      <x:c r="AQ8" s="65"/>
+      <x:c r="AR8" s="65"/>
+      <x:c r="AS8" s="65"/>
+      <x:c r="AT8" s="65"/>
+      <x:c r="AU8" s="65"/>
+      <x:c r="AV8" s="65"/>
+      <x:c r="AW8" s="65"/>
+      <x:c r="AX8" s="65"/>
+      <x:c r="AY8" s="65"/>
+      <x:c r="AZ8" s="65"/>
+      <x:c r="BA8" s="65"/>
+      <x:c r="BB8" s="65"/>
+      <x:c r="BC8" s="65"/>
+      <x:c r="BD8" s="65"/>
+      <x:c r="BE8" s="65"/>
+      <x:c r="BF8" s="65"/>
+      <x:c r="BG8" s="65"/>
+      <x:c r="BH8" s="65"/>
+      <x:c r="BI8" s="65"/>
+      <x:c r="BJ8" s="65"/>
+      <x:c r="BK8" s="65"/>
+      <x:c r="BL8" s="65"/>
+      <x:c r="BM8" s="65"/>
+      <x:c r="BN8" s="65"/>
+      <x:c r="BO8" s="65"/>
+      <x:c r="BP8" s="65"/>
+      <x:c r="BQ8" s="65"/>
+      <x:c r="BR8" s="65"/>
+      <x:c r="BS8" s="65"/>
+      <x:c r="BT8" s="65"/>
+      <x:c r="BU8" s="65"/>
+      <x:c r="BV8" s="65"/>
+      <x:c r="BW8" s="65"/>
+      <x:c r="BX8" s="65"/>
+      <x:c r="BY8" s="65"/>
+      <x:c r="BZ8" s="65"/>
+      <x:c r="CA8" s="65"/>
+      <x:c r="CB8" s="65"/>
+      <x:c r="CC8" s="65"/>
+      <x:c r="CD8" s="65"/>
+      <x:c r="CE8" s="65"/>
+      <x:c r="CF8" s="65"/>
+      <x:c r="CG8" s="65"/>
+      <x:c r="CH8" s="65"/>
+      <x:c r="CI8" s="65"/>
+      <x:c r="CJ8" s="65"/>
+      <x:c r="CK8" s="65"/>
+      <x:c r="CL8" s="66"/>
+    </x:row>
+    <x:row r="9" ht="13.5" customHeight="1">
+      <x:c r="A9" s="63" t="str">
+        <x:v>＜VALUES 2行目＞</x:v>
+      </x:c>
+      <x:c r="B9" s="63"/>
+      <x:c r="C9" s="63"/>
+      <x:c r="D9" s="63"/>
+      <x:c r="E9" s="63"/>
+      <x:c r="F9" s="63"/>
+      <x:c r="G9" s="63"/>
+      <x:c r="H9" s="63"/>
+      <x:c r="I9" s="63"/>
+      <x:c r="J9" s="63"/>
+      <x:c r="K9" s="63"/>
+      <x:c r="L9" s="63"/>
+      <x:c r="M9" s="63"/>
+      <x:c r="N9" s="63"/>
+      <x:c r="O9" s="63"/>
+      <x:c r="P9" s="63"/>
+      <x:c r="Q9" s="63"/>
+      <x:c r="R9" s="63"/>
+      <x:c r="S9" s="63"/>
+      <x:c r="T9" s="63"/>
+      <x:c r="U9" s="63"/>
+      <x:c r="V9" s="63"/>
+      <x:c r="W9" s="63"/>
+      <x:c r="X9" s="63"/>
+      <x:c r="Y9" s="63"/>
+      <x:c r="Z9" s="63"/>
+      <x:c r="AA9" s="63"/>
+      <x:c r="AB9" s="63"/>
+      <x:c r="AC9" s="63"/>
+      <x:c r="AD9" s="63"/>
+      <x:c r="AE9" s="63"/>
+      <x:c r="AF9" s="63"/>
+      <x:c r="AG9" s="63"/>
+      <x:c r="AH9" s="63"/>
+      <x:c r="AI9" s="63"/>
+      <x:c r="AJ9" s="63"/>
+      <x:c r="AK9" s="63"/>
+      <x:c r="AL9" s="63"/>
+      <x:c r="AM9" s="63"/>
+      <x:c r="AN9" s="63"/>
+      <x:c r="AO9" s="63"/>
+      <x:c r="AP9" s="63"/>
+      <x:c r="AQ9" s="63"/>
+      <x:c r="AR9" s="63"/>
+      <x:c r="AS9" s="63"/>
+      <x:c r="AT9" s="63"/>
+      <x:c r="AU9" s="63"/>
+      <x:c r="AV9" s="63"/>
+      <x:c r="AW9" s="63"/>
+      <x:c r="AX9" s="63"/>
+      <x:c r="AY9" s="63"/>
+      <x:c r="AZ9" s="63"/>
+      <x:c r="BA9" s="63"/>
+      <x:c r="BB9" s="63"/>
+      <x:c r="BC9" s="63"/>
+      <x:c r="BD9" s="63"/>
+      <x:c r="BE9" s="63"/>
+      <x:c r="BF9" s="63"/>
+      <x:c r="BG9" s="63"/>
+      <x:c r="BH9" s="63"/>
+      <x:c r="BI9" s="63"/>
+      <x:c r="BJ9" s="63"/>
+      <x:c r="BK9" s="63"/>
+      <x:c r="BL9" s="63"/>
+      <x:c r="BM9" s="63"/>
+      <x:c r="BN9" s="63"/>
+      <x:c r="BO9" s="63"/>
+      <x:c r="BP9" s="63"/>
+      <x:c r="BQ9" s="63"/>
+      <x:c r="BR9" s="63"/>
+      <x:c r="BS9" s="63"/>
+      <x:c r="BT9" s="63"/>
+      <x:c r="BU9" s="63"/>
+      <x:c r="BV9" s="63"/>
+      <x:c r="BW9" s="63"/>
+      <x:c r="BX9" s="63"/>
+      <x:c r="BY9" s="63"/>
+      <x:c r="BZ9" s="63"/>
+      <x:c r="CA9" s="63"/>
+      <x:c r="CB9" s="63"/>
+      <x:c r="CC9" s="63"/>
+      <x:c r="CD9" s="63"/>
+      <x:c r="CE9" s="63"/>
+      <x:c r="CF9" s="63"/>
+      <x:c r="CG9" s="63"/>
+      <x:c r="CH9" s="63"/>
+      <x:c r="CI9" s="63"/>
+      <x:c r="CJ9" s="63"/>
+      <x:c r="CK9" s="63"/>
+      <x:c r="CL9" s="63"/>
+    </x:row>
+    <x:row r="10" ht="13.5" customHeight="1">
+      <x:c r="A10" s="67" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="B10" s="68"/>
+      <x:c r="C10" s="68"/>
+      <x:c r="D10" s="68"/>
+      <x:c r="E10" s="68"/>
+      <x:c r="F10" s="68"/>
+      <x:c r="G10" s="68"/>
+      <x:c r="H10" s="68"/>
+      <x:c r="I10" s="68"/>
+      <x:c r="J10" s="68"/>
+      <x:c r="K10" s="68"/>
+      <x:c r="L10" s="68"/>
+      <x:c r="M10" s="68"/>
+      <x:c r="N10" s="68"/>
+      <x:c r="O10" s="68"/>
+      <x:c r="P10" s="68"/>
+      <x:c r="Q10" s="68"/>
+      <x:c r="R10" s="68"/>
+      <x:c r="S10" s="67" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="T10" s="68"/>
+      <x:c r="U10" s="68"/>
+      <x:c r="V10" s="68"/>
+      <x:c r="W10" s="68"/>
+      <x:c r="X10" s="68"/>
+      <x:c r="Y10" s="68"/>
+      <x:c r="Z10" s="68"/>
+      <x:c r="AA10" s="68"/>
+      <x:c r="AB10" s="68"/>
+      <x:c r="AC10" s="68"/>
+      <x:c r="AD10" s="68"/>
+      <x:c r="AE10" s="68"/>
+      <x:c r="AF10" s="68"/>
+      <x:c r="AG10" s="68"/>
+      <x:c r="AH10" s="68"/>
+      <x:c r="AI10" s="68"/>
+      <x:c r="AJ10" s="68"/>
+      <x:c r="AK10" s="67" t="str">
+        <x:v>移送方法ほか</x:v>
+      </x:c>
+      <x:c r="AL10" s="68"/>
+      <x:c r="AM10" s="68"/>
+      <x:c r="AN10" s="68"/>
+      <x:c r="AO10" s="68"/>
+      <x:c r="AP10" s="68"/>
+      <x:c r="AQ10" s="68"/>
+      <x:c r="AR10" s="68"/>
+      <x:c r="AS10" s="68"/>
+      <x:c r="AT10" s="68"/>
+      <x:c r="AU10" s="68"/>
+      <x:c r="AV10" s="68"/>
+      <x:c r="AW10" s="68"/>
+      <x:c r="AX10" s="68"/>
+      <x:c r="AY10" s="68"/>
+      <x:c r="AZ10" s="68"/>
+      <x:c r="BA10" s="68"/>
+      <x:c r="BB10" s="68"/>
+      <x:c r="BC10" s="68"/>
+      <x:c r="BD10" s="68"/>
+      <x:c r="BE10" s="68"/>
+      <x:c r="BF10" s="68"/>
+      <x:c r="BG10" s="68"/>
+      <x:c r="BH10" s="68"/>
+      <x:c r="BI10" s="68"/>
+      <x:c r="BJ10" s="68"/>
+      <x:c r="BK10" s="68"/>
+      <x:c r="BL10" s="68"/>
+      <x:c r="BM10" s="68"/>
+      <x:c r="BN10" s="68"/>
+      <x:c r="BO10" s="68"/>
+      <x:c r="BP10" s="68"/>
+      <x:c r="BQ10" s="68"/>
+      <x:c r="BR10" s="68"/>
+      <x:c r="BS10" s="68"/>
+      <x:c r="BT10" s="68"/>
+      <x:c r="BU10" s="68"/>
+      <x:c r="BV10" s="68"/>
+      <x:c r="BW10" s="68"/>
+      <x:c r="BX10" s="68"/>
+      <x:c r="BY10" s="68"/>
+      <x:c r="BZ10" s="68"/>
+      <x:c r="CA10" s="68"/>
+      <x:c r="CB10" s="68"/>
+      <x:c r="CC10" s="68"/>
+      <x:c r="CD10" s="68"/>
+      <x:c r="CE10" s="68"/>
+      <x:c r="CF10" s="68"/>
+      <x:c r="CG10" s="68"/>
+      <x:c r="CH10" s="68"/>
+      <x:c r="CI10" s="68"/>
+      <x:c r="CJ10" s="68"/>
+      <x:c r="CK10" s="68"/>
+      <x:c r="CL10" s="69"/>
+    </x:row>
+    <x:row r="11" ht="13.5" customHeight="1">
+      <x:c r="A11" s="64" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="B11" s="65"/>
+      <x:c r="C11" s="65"/>
+      <x:c r="D11" s="65"/>
+      <x:c r="E11" s="65"/>
+      <x:c r="F11" s="65"/>
+      <x:c r="G11" s="65"/>
+      <x:c r="H11" s="65"/>
+      <x:c r="I11" s="65"/>
+      <x:c r="J11" s="65"/>
+      <x:c r="K11" s="65"/>
+      <x:c r="L11" s="65"/>
+      <x:c r="M11" s="65"/>
+      <x:c r="N11" s="65"/>
+      <x:c r="O11" s="65"/>
+      <x:c r="P11" s="65"/>
+      <x:c r="Q11" s="65"/>
+      <x:c r="R11" s="65"/>
+      <x:c r="S11" s="64"/>
+      <x:c r="T11" s="65"/>
+      <x:c r="U11" s="65"/>
+      <x:c r="V11" s="65"/>
+      <x:c r="W11" s="65"/>
+      <x:c r="X11" s="65"/>
+      <x:c r="Y11" s="65"/>
+      <x:c r="Z11" s="65"/>
+      <x:c r="AA11" s="65"/>
+      <x:c r="AB11" s="65"/>
+      <x:c r="AC11" s="65"/>
+      <x:c r="AD11" s="65"/>
+      <x:c r="AE11" s="65"/>
+      <x:c r="AF11" s="65"/>
+      <x:c r="AG11" s="65"/>
+      <x:c r="AH11" s="65"/>
+      <x:c r="AI11" s="65"/>
+      <x:c r="AJ11" s="65"/>
+      <x:c r="AK11" s="64" t="str">
+        <x:v>@user_id_2</x:v>
+      </x:c>
+      <x:c r="AL11" s="65"/>
+      <x:c r="AM11" s="65"/>
+      <x:c r="AN11" s="65"/>
+      <x:c r="AO11" s="65"/>
+      <x:c r="AP11" s="65"/>
+      <x:c r="AQ11" s="65"/>
+      <x:c r="AR11" s="65"/>
+      <x:c r="AS11" s="65"/>
+      <x:c r="AT11" s="65"/>
+      <x:c r="AU11" s="65"/>
+      <x:c r="AV11" s="65"/>
+      <x:c r="AW11" s="65"/>
+      <x:c r="AX11" s="65"/>
+      <x:c r="AY11" s="65"/>
+      <x:c r="AZ11" s="65"/>
+      <x:c r="BA11" s="65"/>
+      <x:c r="BB11" s="65"/>
+      <x:c r="BC11" s="65"/>
+      <x:c r="BD11" s="65"/>
+      <x:c r="BE11" s="65"/>
+      <x:c r="BF11" s="65"/>
+      <x:c r="BG11" s="65"/>
+      <x:c r="BH11" s="65"/>
+      <x:c r="BI11" s="65"/>
+      <x:c r="BJ11" s="65"/>
+      <x:c r="BK11" s="65"/>
+      <x:c r="BL11" s="65"/>
+      <x:c r="BM11" s="65"/>
+      <x:c r="BN11" s="65"/>
+      <x:c r="BO11" s="65"/>
+      <x:c r="BP11" s="65"/>
+      <x:c r="BQ11" s="65"/>
+      <x:c r="BR11" s="65"/>
+      <x:c r="BS11" s="65"/>
+      <x:c r="BT11" s="65"/>
+      <x:c r="BU11" s="65"/>
+      <x:c r="BV11" s="65"/>
+      <x:c r="BW11" s="65"/>
+      <x:c r="BX11" s="65"/>
+      <x:c r="BY11" s="65"/>
+      <x:c r="BZ11" s="65"/>
+      <x:c r="CA11" s="65"/>
+      <x:c r="CB11" s="65"/>
+      <x:c r="CC11" s="65"/>
+      <x:c r="CD11" s="65"/>
+      <x:c r="CE11" s="65"/>
+      <x:c r="CF11" s="65"/>
+      <x:c r="CG11" s="65"/>
+      <x:c r="CH11" s="65"/>
+      <x:c r="CI11" s="65"/>
+      <x:c r="CJ11" s="65"/>
+      <x:c r="CK11" s="65"/>
+      <x:c r="CL11" s="66"/>
+    </x:row>
+    <x:row r="12" ht="13.5" customHeight="1">
+      <x:c r="A12" s="64" t="s">
+        <x:v>151</x:v>
+      </x:c>
+      <x:c r="B12" s="65"/>
+      <x:c r="C12" s="65"/>
+      <x:c r="D12" s="65"/>
+      <x:c r="E12" s="65"/>
+      <x:c r="F12" s="65"/>
+      <x:c r="G12" s="65"/>
+      <x:c r="H12" s="65"/>
+      <x:c r="I12" s="65"/>
+      <x:c r="J12" s="65"/>
+      <x:c r="K12" s="65"/>
+      <x:c r="L12" s="65"/>
+      <x:c r="M12" s="65"/>
+      <x:c r="N12" s="65"/>
+      <x:c r="O12" s="65"/>
+      <x:c r="P12" s="65"/>
+      <x:c r="Q12" s="65"/>
+      <x:c r="R12" s="65"/>
+      <x:c r="S12" s="64"/>
+      <x:c r="T12" s="65"/>
+      <x:c r="U12" s="65"/>
+      <x:c r="V12" s="65"/>
+      <x:c r="W12" s="65"/>
+      <x:c r="X12" s="65"/>
+      <x:c r="Y12" s="65"/>
+      <x:c r="Z12" s="65"/>
+      <x:c r="AA12" s="65"/>
+      <x:c r="AB12" s="65"/>
+      <x:c r="AC12" s="65"/>
+      <x:c r="AD12" s="65"/>
+      <x:c r="AE12" s="65"/>
+      <x:c r="AF12" s="65"/>
+      <x:c r="AG12" s="65"/>
+      <x:c r="AH12" s="65"/>
+      <x:c r="AI12" s="65"/>
+      <x:c r="AJ12" s="65"/>
+      <x:c r="AK12" s="64" t="str">
+        <x:v>@name_2</x:v>
+      </x:c>
+      <x:c r="AL12" s="65"/>
+      <x:c r="AM12" s="65"/>
+      <x:c r="AN12" s="65"/>
+      <x:c r="AO12" s="65"/>
+      <x:c r="AP12" s="65"/>
+      <x:c r="AQ12" s="65"/>
+      <x:c r="AR12" s="65"/>
+      <x:c r="AS12" s="65"/>
+      <x:c r="AT12" s="65"/>
+      <x:c r="AU12" s="65"/>
+      <x:c r="AV12" s="65"/>
+      <x:c r="AW12" s="65"/>
+      <x:c r="AX12" s="65"/>
+      <x:c r="AY12" s="65"/>
+      <x:c r="AZ12" s="65"/>
+      <x:c r="BA12" s="65"/>
+      <x:c r="BB12" s="65"/>
+      <x:c r="BC12" s="65"/>
+      <x:c r="BD12" s="65"/>
+      <x:c r="BE12" s="65"/>
+      <x:c r="BF12" s="65"/>
+      <x:c r="BG12" s="65"/>
+      <x:c r="BH12" s="65"/>
+      <x:c r="BI12" s="65"/>
+      <x:c r="BJ12" s="65"/>
+      <x:c r="BK12" s="65"/>
+      <x:c r="BL12" s="65"/>
+      <x:c r="BM12" s="65"/>
+      <x:c r="BN12" s="65"/>
+      <x:c r="BO12" s="65"/>
+      <x:c r="BP12" s="65"/>
+      <x:c r="BQ12" s="65"/>
+      <x:c r="BR12" s="65"/>
+      <x:c r="BS12" s="65"/>
+      <x:c r="BT12" s="65"/>
+      <x:c r="BU12" s="65"/>
+      <x:c r="BV12" s="65"/>
+      <x:c r="BW12" s="65"/>
+      <x:c r="BX12" s="65"/>
+      <x:c r="BY12" s="65"/>
+      <x:c r="BZ12" s="65"/>
+      <x:c r="CA12" s="65"/>
+      <x:c r="CB12" s="65"/>
+      <x:c r="CC12" s="65"/>
+      <x:c r="CD12" s="65"/>
+      <x:c r="CE12" s="65"/>
+      <x:c r="CF12" s="65"/>
+      <x:c r="CG12" s="65"/>
+      <x:c r="CH12" s="65"/>
+      <x:c r="CI12" s="65"/>
+      <x:c r="CJ12" s="65"/>
+      <x:c r="CK12" s="65"/>
+      <x:c r="CL12" s="66"/>
+    </x:row>
+    <x:row r="13" ht="13.5" customHeight="1">
+      <x:c r="A13" s="64" t="s">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="B13" s="65"/>
+      <x:c r="C13" s="65"/>
+      <x:c r="D13" s="65"/>
+      <x:c r="E13" s="65"/>
+      <x:c r="F13" s="65"/>
+      <x:c r="G13" s="65"/>
+      <x:c r="H13" s="65"/>
+      <x:c r="I13" s="65"/>
+      <x:c r="J13" s="65"/>
+      <x:c r="K13" s="65"/>
+      <x:c r="L13" s="65"/>
+      <x:c r="M13" s="65"/>
+      <x:c r="N13" s="65"/>
+      <x:c r="O13" s="65"/>
+      <x:c r="P13" s="65"/>
+      <x:c r="Q13" s="65"/>
+      <x:c r="R13" s="65"/>
+      <x:c r="S13" s="64"/>
+      <x:c r="T13" s="65"/>
+      <x:c r="U13" s="65"/>
+      <x:c r="V13" s="65"/>
+      <x:c r="W13" s="65"/>
+      <x:c r="X13" s="65"/>
+      <x:c r="Y13" s="65"/>
+      <x:c r="Z13" s="65"/>
+      <x:c r="AA13" s="65"/>
+      <x:c r="AB13" s="65"/>
+      <x:c r="AC13" s="65"/>
+      <x:c r="AD13" s="65"/>
+      <x:c r="AE13" s="65"/>
+      <x:c r="AF13" s="65"/>
+      <x:c r="AG13" s="65"/>
+      <x:c r="AH13" s="65"/>
+      <x:c r="AI13" s="65"/>
+      <x:c r="AJ13" s="65"/>
+      <x:c r="AK13" s="64" t="str">
+        <x:v>'PENDING'</x:v>
+      </x:c>
+      <x:c r="AL13" s="65"/>
+      <x:c r="AM13" s="65"/>
+      <x:c r="AN13" s="65"/>
+      <x:c r="AO13" s="65"/>
+      <x:c r="AP13" s="65"/>
+      <x:c r="AQ13" s="65"/>
+      <x:c r="AR13" s="65"/>
+      <x:c r="AS13" s="65"/>
+      <x:c r="AT13" s="65"/>
+      <x:c r="AU13" s="65"/>
+      <x:c r="AV13" s="65"/>
+      <x:c r="AW13" s="65"/>
+      <x:c r="AX13" s="65"/>
+      <x:c r="AY13" s="65"/>
+      <x:c r="AZ13" s="65"/>
+      <x:c r="BA13" s="65"/>
+      <x:c r="BB13" s="65"/>
+      <x:c r="BC13" s="65"/>
+      <x:c r="BD13" s="65"/>
+      <x:c r="BE13" s="65"/>
+      <x:c r="BF13" s="65"/>
+      <x:c r="BG13" s="65"/>
+      <x:c r="BH13" s="65"/>
+      <x:c r="BI13" s="65"/>
+      <x:c r="BJ13" s="65"/>
+      <x:c r="BK13" s="65"/>
+      <x:c r="BL13" s="65"/>
+      <x:c r="BM13" s="65"/>
+      <x:c r="BN13" s="65"/>
+      <x:c r="BO13" s="65"/>
+      <x:c r="BP13" s="65"/>
+      <x:c r="BQ13" s="65"/>
+      <x:c r="BR13" s="65"/>
+      <x:c r="BS13" s="65"/>
+      <x:c r="BT13" s="65"/>
+      <x:c r="BU13" s="65"/>
+      <x:c r="BV13" s="65"/>
+      <x:c r="BW13" s="65"/>
+      <x:c r="BX13" s="65"/>
+      <x:c r="BY13" s="65"/>
+      <x:c r="BZ13" s="65"/>
+      <x:c r="CA13" s="65"/>
+      <x:c r="CB13" s="65"/>
+      <x:c r="CC13" s="65"/>
+      <x:c r="CD13" s="65"/>
+      <x:c r="CE13" s="65"/>
+      <x:c r="CF13" s="65"/>
+      <x:c r="CG13" s="65"/>
+      <x:c r="CH13" s="65"/>
+      <x:c r="CI13" s="65"/>
+      <x:c r="CJ13" s="65"/>
+      <x:c r="CK13" s="65"/>
+      <x:c r="CL13" s="66"/>
+    </x:row>
+    <x:row r="14" ht="13.5" customHeight="1">
+      <x:c r="A14" s="64" t="s">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="B14" s="65"/>
+      <x:c r="C14" s="65"/>
+      <x:c r="D14" s="65"/>
+      <x:c r="E14" s="65"/>
+      <x:c r="F14" s="65"/>
+      <x:c r="G14" s="65"/>
+      <x:c r="H14" s="65"/>
+      <x:c r="I14" s="65"/>
+      <x:c r="J14" s="65"/>
+      <x:c r="K14" s="65"/>
+      <x:c r="L14" s="65"/>
+      <x:c r="M14" s="65"/>
+      <x:c r="N14" s="65"/>
+      <x:c r="O14" s="65"/>
+      <x:c r="P14" s="65"/>
+      <x:c r="Q14" s="65"/>
+      <x:c r="R14" s="65"/>
+      <x:c r="S14" s="64"/>
+      <x:c r="T14" s="65"/>
+      <x:c r="U14" s="65"/>
+      <x:c r="V14" s="65"/>
+      <x:c r="W14" s="65"/>
+      <x:c r="X14" s="65"/>
+      <x:c r="Y14" s="65"/>
+      <x:c r="Z14" s="65"/>
+      <x:c r="AA14" s="65"/>
+      <x:c r="AB14" s="65"/>
+      <x:c r="AC14" s="65"/>
+      <x:c r="AD14" s="65"/>
+      <x:c r="AE14" s="65"/>
+      <x:c r="AF14" s="65"/>
+      <x:c r="AG14" s="65"/>
+      <x:c r="AH14" s="65"/>
+      <x:c r="AI14" s="65"/>
+      <x:c r="AJ14" s="65"/>
+      <x:c r="AK14" s="64" t="str">
+        <x:v>SYSDATETIME()</x:v>
+      </x:c>
+      <x:c r="AL14" s="65"/>
+      <x:c r="AM14" s="65"/>
+      <x:c r="AN14" s="65"/>
+      <x:c r="AO14" s="65"/>
+      <x:c r="AP14" s="65"/>
+      <x:c r="AQ14" s="65"/>
+      <x:c r="AR14" s="65"/>
+      <x:c r="AS14" s="65"/>
+      <x:c r="AT14" s="65"/>
+      <x:c r="AU14" s="65"/>
+      <x:c r="AV14" s="65"/>
+      <x:c r="AW14" s="65"/>
+      <x:c r="AX14" s="65"/>
+      <x:c r="AY14" s="65"/>
+      <x:c r="AZ14" s="65"/>
+      <x:c r="BA14" s="65"/>
+      <x:c r="BB14" s="65"/>
+      <x:c r="BC14" s="65"/>
+      <x:c r="BD14" s="65"/>
+      <x:c r="BE14" s="65"/>
+      <x:c r="BF14" s="65"/>
+      <x:c r="BG14" s="65"/>
+      <x:c r="BH14" s="65"/>
+      <x:c r="BI14" s="65"/>
+      <x:c r="BJ14" s="65"/>
+      <x:c r="BK14" s="65"/>
+      <x:c r="BL14" s="65"/>
+      <x:c r="BM14" s="65"/>
+      <x:c r="BN14" s="65"/>
+      <x:c r="BO14" s="65"/>
+      <x:c r="BP14" s="65"/>
+      <x:c r="BQ14" s="65"/>
+      <x:c r="BR14" s="65"/>
+      <x:c r="BS14" s="65"/>
+      <x:c r="BT14" s="65"/>
+      <x:c r="BU14" s="65"/>
+      <x:c r="BV14" s="65"/>
+      <x:c r="BW14" s="65"/>
+      <x:c r="BX14" s="65"/>
+      <x:c r="BY14" s="65"/>
+      <x:c r="BZ14" s="65"/>
+      <x:c r="CA14" s="65"/>
+      <x:c r="CB14" s="65"/>
+      <x:c r="CC14" s="65"/>
+      <x:c r="CD14" s="65"/>
+      <x:c r="CE14" s="65"/>
+      <x:c r="CF14" s="65"/>
+      <x:c r="CG14" s="65"/>
+      <x:c r="CH14" s="65"/>
+      <x:c r="CI14" s="65"/>
+      <x:c r="CJ14" s="65"/>
+      <x:c r="CK14" s="65"/>
+      <x:c r="CL14" s="66"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="33" max="33" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="35" max="35" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="36" max="36" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="37" max="37" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="38" max="38" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="39" max="39" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="40" max="40" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="41" max="41" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="42" max="42" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="43" max="43" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="44" max="44" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="45" max="45" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="46" max="46" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="47" max="47" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="48" max="48" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="49" max="49" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="50" max="50" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="51" max="51" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="52" max="52" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="53" max="53" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="54" max="54" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="55" max="55" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="56" max="56" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="57" max="57" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="58" max="58" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="59" max="59" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="60" max="60" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="61" max="61" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="62" max="62" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="63" max="63" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="64" max="64" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="65" max="65" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="66" max="66" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="67" max="67" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="68" max="68" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="69" max="69" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="70" max="70" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="71" max="71" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="72" max="72" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="73" max="73" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="74" max="74" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="75" max="75" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="76" max="76" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="77" max="77" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="78" max="78" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="79" max="79" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="80" max="80" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="81" max="81" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="82" max="82" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="83" max="83" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="84" max="84" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="85" max="85" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="86" max="86" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="87" max="87" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="88" max="88" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="89" max="89" width="1.1399999856948853" hidden="0" customWidth="1"/>
+    <x:col min="90" max="90" width="1.1399999856948853" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="13.5" customHeight="1">
+      <x:c r="A1" s="61" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B1" s="61"/>
+      <x:c r="C1" s="61"/>
+      <x:c r="D1" s="61"/>
+      <x:c r="E1" s="61"/>
+      <x:c r="F1" s="61"/>
+      <x:c r="G1" s="61"/>
+      <x:c r="H1" s="61"/>
+      <x:c r="I1" s="61"/>
+      <x:c r="J1" s="61"/>
+      <x:c r="K1" s="61"/>
+      <x:c r="L1" s="61"/>
+      <x:c r="M1" s="61"/>
+      <x:c r="N1" s="61"/>
+      <x:c r="O1" s="61"/>
+      <x:c r="P1" s="61"/>
+      <x:c r="Q1" s="61"/>
+      <x:c r="R1" s="61"/>
+      <x:c r="S1" s="61"/>
+      <x:c r="T1" s="61"/>
+      <x:c r="U1" s="61"/>
+      <x:c r="V1" s="61"/>
+      <x:c r="W1" s="61"/>
+      <x:c r="X1" s="61"/>
+      <x:c r="Y1" s="61"/>
+      <x:c r="Z1" s="61"/>
+      <x:c r="AA1" s="61"/>
+      <x:c r="AB1" s="61"/>
+      <x:c r="AC1" s="61"/>
+      <x:c r="AD1" s="61"/>
+      <x:c r="AE1" s="61"/>
+      <x:c r="AF1" s="61"/>
+      <x:c r="AG1" s="61"/>
+      <x:c r="AH1" s="61"/>
+      <x:c r="AI1" s="61"/>
+      <x:c r="AJ1" s="61"/>
+      <x:c r="AK1" s="61"/>
+      <x:c r="AL1" s="61"/>
+      <x:c r="AM1" s="61"/>
+      <x:c r="AN1" s="61"/>
+      <x:c r="AO1" s="61"/>
+      <x:c r="AP1" s="61"/>
+      <x:c r="AQ1" s="61"/>
+      <x:c r="AR1" s="61"/>
+      <x:c r="AS1" s="61"/>
+      <x:c r="AT1" s="61"/>
+      <x:c r="AU1" s="61"/>
+      <x:c r="AV1" s="61"/>
+      <x:c r="AW1" s="61"/>
+      <x:c r="AX1" s="61"/>
+      <x:c r="AY1" s="61"/>
+      <x:c r="AZ1" s="61"/>
+      <x:c r="BA1" s="61"/>
+      <x:c r="BB1" s="61"/>
+      <x:c r="BC1" s="61"/>
+      <x:c r="BD1" s="61"/>
+      <x:c r="BE1" s="61"/>
+      <x:c r="BF1" s="61"/>
+      <x:c r="BG1" s="61"/>
+      <x:c r="BH1" s="61"/>
+      <x:c r="BI1" s="61"/>
+      <x:c r="BJ1" s="61"/>
+      <x:c r="BK1" s="61"/>
+      <x:c r="BL1" s="61"/>
+      <x:c r="BM1" s="61"/>
+      <x:c r="BN1" s="61"/>
+      <x:c r="BO1" s="61"/>
+      <x:c r="BP1" s="61"/>
+      <x:c r="BQ1" s="61"/>
+      <x:c r="BR1" s="61"/>
+      <x:c r="BS1" s="61"/>
+      <x:c r="BT1" s="61"/>
+      <x:c r="BU1" s="61"/>
+      <x:c r="BV1" s="61"/>
+      <x:c r="BW1" s="61"/>
+      <x:c r="BX1" s="61"/>
+      <x:c r="BY1" s="61"/>
+      <x:c r="BZ1" s="61"/>
+      <x:c r="CA1" s="61"/>
+      <x:c r="CB1" s="61"/>
+      <x:c r="CC1" s="61"/>
+      <x:c r="CD1" s="61"/>
+      <x:c r="CE1" s="61"/>
+      <x:c r="CF1" s="61"/>
+      <x:c r="CG1" s="61"/>
+      <x:c r="CH1" s="61"/>
+      <x:c r="CI1" s="61"/>
+      <x:c r="CJ1" s="61"/>
+      <x:c r="CK1" s="61"/>
+      <x:c r="CL1" s="61"/>
+    </x:row>
+    <x:row r="2" ht="13.5" customHeight="1">
+      <x:c r="A2" s="61" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="B2" s="61"/>
+      <x:c r="C2" s="61"/>
+      <x:c r="D2" s="61"/>
+      <x:c r="E2" s="61"/>
+      <x:c r="F2" s="61"/>
+      <x:c r="G2" s="61"/>
+      <x:c r="H2" s="61"/>
+      <x:c r="I2" s="61"/>
+      <x:c r="J2" s="61"/>
+      <x:c r="K2" s="61"/>
+      <x:c r="L2" s="61"/>
+      <x:c r="M2" s="61"/>
+      <x:c r="N2" s="61"/>
+      <x:c r="O2" s="61"/>
+      <x:c r="P2" s="61"/>
+      <x:c r="Q2" s="61"/>
+      <x:c r="R2" s="61"/>
+      <x:c r="S2" s="61"/>
+      <x:c r="T2" s="61"/>
+      <x:c r="U2" s="61"/>
+      <x:c r="V2" s="61"/>
+      <x:c r="W2" s="61"/>
+      <x:c r="X2" s="61"/>
+      <x:c r="Y2" s="61"/>
+      <x:c r="Z2" s="61"/>
+      <x:c r="AA2" s="61"/>
+      <x:c r="AB2" s="61"/>
+      <x:c r="AC2" s="61"/>
+      <x:c r="AD2" s="61"/>
+      <x:c r="AE2" s="61"/>
+      <x:c r="AF2" s="61"/>
+      <x:c r="AG2" s="61"/>
+      <x:c r="AH2" s="61"/>
+      <x:c r="AI2" s="61"/>
+      <x:c r="AJ2" s="61"/>
+      <x:c r="AK2" s="61"/>
+      <x:c r="AL2" s="61"/>
+      <x:c r="AM2" s="61"/>
+      <x:c r="AN2" s="61"/>
+      <x:c r="AO2" s="61"/>
+      <x:c r="AP2" s="61"/>
+      <x:c r="AQ2" s="61"/>
+      <x:c r="AR2" s="61"/>
+      <x:c r="AS2" s="61"/>
+      <x:c r="AT2" s="61"/>
+      <x:c r="AU2" s="61"/>
+      <x:c r="AV2" s="61"/>
+      <x:c r="AW2" s="61"/>
+      <x:c r="AX2" s="61"/>
+      <x:c r="AY2" s="61"/>
+      <x:c r="AZ2" s="61"/>
+      <x:c r="BA2" s="61"/>
+      <x:c r="BB2" s="61"/>
+      <x:c r="BC2" s="61"/>
+      <x:c r="BD2" s="61"/>
+      <x:c r="BE2" s="61"/>
+      <x:c r="BF2" s="61"/>
+      <x:c r="BG2" s="61"/>
+      <x:c r="BH2" s="61"/>
+      <x:c r="BI2" s="61"/>
+      <x:c r="BJ2" s="61"/>
+      <x:c r="BK2" s="61"/>
+      <x:c r="BL2" s="61"/>
+      <x:c r="BM2" s="61"/>
+      <x:c r="BN2" s="61"/>
+      <x:c r="BO2" s="61"/>
+      <x:c r="BP2" s="61"/>
+      <x:c r="BQ2" s="61"/>
+      <x:c r="BR2" s="61"/>
+      <x:c r="BS2" s="61"/>
+      <x:c r="BT2" s="61"/>
+      <x:c r="BU2" s="61"/>
+      <x:c r="BV2" s="61"/>
+      <x:c r="BW2" s="61"/>
+      <x:c r="BX2" s="61"/>
+      <x:c r="BY2" s="61"/>
+      <x:c r="BZ2" s="61"/>
+      <x:c r="CA2" s="61"/>
+      <x:c r="CB2" s="61"/>
+      <x:c r="CC2" s="61"/>
+      <x:c r="CD2" s="61"/>
+      <x:c r="CE2" s="61"/>
+      <x:c r="CF2" s="61"/>
+      <x:c r="CG2" s="61"/>
+      <x:c r="CH2" s="61"/>
+      <x:c r="CI2" s="61"/>
+      <x:c r="CJ2" s="61"/>
+      <x:c r="CK2" s="61"/>
+      <x:c r="CL2" s="61"/>
+    </x:row>
+    <x:row r="3" ht="13.5" customHeight="1">
+      <x:c r="A3" s="71" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="72"/>
+      <x:c r="C3" s="72"/>
+      <x:c r="D3" s="72"/>
+      <x:c r="E3" s="72"/>
+      <x:c r="F3" s="72"/>
+      <x:c r="G3" s="77" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H3" s="63"/>
+      <x:c r="I3" s="63"/>
+      <x:c r="J3" s="63"/>
+      <x:c r="K3" s="63"/>
+      <x:c r="L3" s="63"/>
+      <x:c r="M3" s="63"/>
+      <x:c r="N3" s="63"/>
+      <x:c r="O3" s="63" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="P3" s="63"/>
+      <x:c r="Q3" s="63" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="R3" s="63"/>
+      <x:c r="S3" s="63"/>
+      <x:c r="T3" s="63"/>
+      <x:c r="U3" s="63"/>
+      <x:c r="V3" s="63"/>
+      <x:c r="W3" s="63"/>
+      <x:c r="X3" s="63"/>
+      <x:c r="Y3" s="63"/>
+      <x:c r="Z3" s="63"/>
+      <x:c r="AA3" s="63"/>
+      <x:c r="AB3" s="63"/>
+      <x:c r="AC3" s="63"/>
+      <x:c r="AD3" s="63"/>
+      <x:c r="AE3" s="63"/>
+      <x:c r="AF3" s="63"/>
+      <x:c r="AG3" s="63"/>
+      <x:c r="AH3" s="63"/>
+      <x:c r="AI3" s="63"/>
+      <x:c r="AJ3" s="63"/>
+      <x:c r="AK3" s="63"/>
+      <x:c r="AL3" s="63"/>
+      <x:c r="AM3" s="63"/>
+      <x:c r="AN3" s="63"/>
+      <x:c r="AO3" s="63"/>
+      <x:c r="AP3" s="63"/>
+      <x:c r="AQ3" s="63"/>
+      <x:c r="AR3" s="63"/>
+      <x:c r="AS3" s="63"/>
+      <x:c r="AT3" s="63"/>
+      <x:c r="AU3" s="63"/>
+      <x:c r="AV3" s="63"/>
+      <x:c r="AW3" s="63"/>
+      <x:c r="AX3" s="63"/>
+      <x:c r="AY3" s="63"/>
+      <x:c r="AZ3" s="63"/>
+      <x:c r="BA3" s="63"/>
+      <x:c r="BB3" s="63"/>
+      <x:c r="BC3" s="63"/>
+      <x:c r="BD3" s="63"/>
+      <x:c r="BE3" s="63"/>
+      <x:c r="BF3" s="63"/>
+      <x:c r="BG3" s="63"/>
+      <x:c r="BH3" s="63"/>
+      <x:c r="BI3" s="63"/>
+      <x:c r="BJ3" s="63"/>
+      <x:c r="BK3" s="63"/>
+      <x:c r="BL3" s="63"/>
+      <x:c r="BM3" s="63"/>
+      <x:c r="BN3" s="63"/>
+      <x:c r="BO3" s="63"/>
+      <x:c r="BP3" s="63"/>
+      <x:c r="BQ3" s="63"/>
+      <x:c r="BR3" s="63"/>
+      <x:c r="BS3" s="63"/>
+      <x:c r="BT3" s="63"/>
+      <x:c r="BU3" s="63"/>
+      <x:c r="BV3" s="63"/>
+      <x:c r="BW3" s="63"/>
+      <x:c r="BX3" s="63"/>
+      <x:c r="BY3" s="63"/>
+      <x:c r="BZ3" s="63"/>
+      <x:c r="CA3" s="63"/>
+      <x:c r="CB3" s="63"/>
+      <x:c r="CC3" s="63"/>
+      <x:c r="CD3" s="63"/>
+      <x:c r="CE3" s="63"/>
+      <x:c r="CF3" s="63"/>
+      <x:c r="CG3" s="63"/>
+      <x:c r="CH3" s="63"/>
+      <x:c r="CI3" s="63"/>
+      <x:c r="CJ3" s="63"/>
+      <x:c r="CK3" s="63"/>
+      <x:c r="CL3" s="78"/>
+    </x:row>
+    <x:row r="4" ht="13.5" customHeight="1">
+      <x:c r="A4" s="73"/>
+      <x:c r="B4" s="74"/>
+      <x:c r="C4" s="74"/>
+      <x:c r="D4" s="74"/>
+      <x:c r="E4" s="74"/>
+      <x:c r="F4" s="74"/>
+      <x:c r="G4" s="79" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H4" s="80"/>
+      <x:c r="I4" s="80"/>
+      <x:c r="J4" s="80"/>
+      <x:c r="K4" s="80"/>
+      <x:c r="L4" s="80"/>
+      <x:c r="M4" s="80"/>
+      <x:c r="N4" s="80"/>
+      <x:c r="O4" s="80" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="P4" s="80"/>
+      <x:c r="Q4" s="80" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="R4" s="80"/>
+      <x:c r="S4" s="80"/>
+      <x:c r="T4" s="80"/>
+      <x:c r="U4" s="80"/>
+      <x:c r="V4" s="80"/>
+      <x:c r="W4" s="80"/>
+      <x:c r="X4" s="80"/>
+      <x:c r="Y4" s="80"/>
+      <x:c r="Z4" s="80"/>
+      <x:c r="AA4" s="80"/>
+      <x:c r="AB4" s="80"/>
+      <x:c r="AC4" s="80"/>
+      <x:c r="AD4" s="80"/>
+      <x:c r="AE4" s="80"/>
+      <x:c r="AF4" s="80"/>
+      <x:c r="AG4" s="80"/>
+      <x:c r="AH4" s="80"/>
+      <x:c r="AI4" s="80"/>
+      <x:c r="AJ4" s="80"/>
+      <x:c r="AK4" s="80"/>
+      <x:c r="AL4" s="80"/>
+      <x:c r="AM4" s="80"/>
+      <x:c r="AN4" s="80"/>
+      <x:c r="AO4" s="80"/>
+      <x:c r="AP4" s="80"/>
+      <x:c r="AQ4" s="80"/>
+      <x:c r="AR4" s="80"/>
+      <x:c r="AS4" s="80"/>
+      <x:c r="AT4" s="80"/>
+      <x:c r="AU4" s="80"/>
+      <x:c r="AV4" s="80"/>
+      <x:c r="AW4" s="80"/>
+      <x:c r="AX4" s="80"/>
+      <x:c r="AY4" s="80"/>
+      <x:c r="AZ4" s="80"/>
+      <x:c r="BA4" s="80"/>
+      <x:c r="BB4" s="80"/>
+      <x:c r="BC4" s="80"/>
+      <x:c r="BD4" s="80"/>
+      <x:c r="BE4" s="80"/>
+      <x:c r="BF4" s="80"/>
+      <x:c r="BG4" s="80"/>
+      <x:c r="BH4" s="80"/>
+      <x:c r="BI4" s="80"/>
+      <x:c r="BJ4" s="80"/>
+      <x:c r="BK4" s="80"/>
+      <x:c r="BL4" s="80"/>
+      <x:c r="BM4" s="80"/>
+      <x:c r="BN4" s="80"/>
+      <x:c r="BO4" s="80"/>
+      <x:c r="BP4" s="80"/>
+      <x:c r="BQ4" s="80"/>
+      <x:c r="BR4" s="80"/>
+      <x:c r="BS4" s="80"/>
+      <x:c r="BT4" s="80"/>
+      <x:c r="BU4" s="80"/>
+      <x:c r="BV4" s="80"/>
+      <x:c r="BW4" s="80"/>
+      <x:c r="BX4" s="80"/>
+      <x:c r="BY4" s="80"/>
+      <x:c r="BZ4" s="80"/>
+      <x:c r="CA4" s="80"/>
+      <x:c r="CB4" s="80"/>
+      <x:c r="CC4" s="80"/>
+      <x:c r="CD4" s="80"/>
+      <x:c r="CE4" s="80"/>
+      <x:c r="CF4" s="80"/>
+      <x:c r="CG4" s="80"/>
+      <x:c r="CH4" s="80"/>
+      <x:c r="CI4" s="80"/>
+      <x:c r="CJ4" s="80"/>
+      <x:c r="CK4" s="80"/>
+      <x:c r="CL4" s="81"/>
+    </x:row>
+    <x:row r="5" ht="13.5" customHeight="1">
+      <x:c r="A5" s="67" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B5" s="68"/>
+      <x:c r="C5" s="68"/>
+      <x:c r="D5" s="68"/>
+      <x:c r="E5" s="68"/>
+      <x:c r="F5" s="68"/>
+      <x:c r="G5" s="64"/>
+      <x:c r="H5" s="65"/>
+      <x:c r="I5" s="65"/>
+      <x:c r="J5" s="65"/>
+      <x:c r="K5" s="65"/>
+      <x:c r="L5" s="65"/>
+      <x:c r="M5" s="65"/>
+      <x:c r="N5" s="65"/>
+      <x:c r="O5" s="65"/>
+      <x:c r="P5" s="65"/>
+      <x:c r="Q5" s="65" t="s">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="R5" s="65"/>
+      <x:c r="S5" s="65"/>
+      <x:c r="T5" s="65"/>
+      <x:c r="U5" s="65"/>
+      <x:c r="V5" s="65"/>
+      <x:c r="W5" s="65"/>
+      <x:c r="X5" s="65"/>
+      <x:c r="Y5" s="65"/>
+      <x:c r="Z5" s="65"/>
+      <x:c r="AA5" s="65"/>
+      <x:c r="AB5" s="65"/>
+      <x:c r="AC5" s="65"/>
+      <x:c r="AD5" s="65"/>
+      <x:c r="AE5" s="65"/>
+      <x:c r="AF5" s="65"/>
+      <x:c r="AG5" s="65"/>
+      <x:c r="AH5" s="65"/>
+      <x:c r="AI5" s="65"/>
+      <x:c r="AJ5" s="65"/>
+      <x:c r="AK5" s="65"/>
+      <x:c r="AL5" s="65"/>
+      <x:c r="AM5" s="65"/>
+      <x:c r="AN5" s="65"/>
+      <x:c r="AO5" s="65"/>
+      <x:c r="AP5" s="65"/>
+      <x:c r="AQ5" s="65"/>
+      <x:c r="AR5" s="65"/>
+      <x:c r="AS5" s="65"/>
+      <x:c r="AT5" s="65"/>
+      <x:c r="AU5" s="65"/>
+      <x:c r="AV5" s="65"/>
+      <x:c r="AW5" s="65"/>
+      <x:c r="AX5" s="65"/>
+      <x:c r="AY5" s="65"/>
+      <x:c r="AZ5" s="65"/>
+      <x:c r="BA5" s="65"/>
+      <x:c r="BB5" s="65"/>
+      <x:c r="BC5" s="65"/>
+      <x:c r="BD5" s="65"/>
+      <x:c r="BE5" s="65"/>
+      <x:c r="BF5" s="65"/>
+      <x:c r="BG5" s="65"/>
+      <x:c r="BH5" s="65"/>
+      <x:c r="BI5" s="65"/>
+      <x:c r="BJ5" s="65"/>
+      <x:c r="BK5" s="65"/>
+      <x:c r="BL5" s="65"/>
+      <x:c r="BM5" s="65"/>
+      <x:c r="BN5" s="65"/>
+      <x:c r="BO5" s="65"/>
+      <x:c r="BP5" s="65"/>
+      <x:c r="BQ5" s="65"/>
+      <x:c r="BR5" s="65"/>
+      <x:c r="BS5" s="65"/>
+      <x:c r="BT5" s="65"/>
+      <x:c r="BU5" s="65"/>
+      <x:c r="BV5" s="65"/>
+      <x:c r="BW5" s="65"/>
+      <x:c r="BX5" s="65"/>
+      <x:c r="BY5" s="65"/>
+      <x:c r="BZ5" s="65"/>
+      <x:c r="CA5" s="65"/>
+      <x:c r="CB5" s="65"/>
+      <x:c r="CC5" s="65"/>
+      <x:c r="CD5" s="65"/>
+      <x:c r="CE5" s="65"/>
+      <x:c r="CF5" s="65"/>
+      <x:c r="CG5" s="65"/>
+      <x:c r="CH5" s="65"/>
+      <x:c r="CI5" s="65"/>
+      <x:c r="CJ5" s="65"/>
+      <x:c r="CK5" s="65"/>
+      <x:c r="CL5" s="66"/>
+    </x:row>
+    <x:row r="6" ht="13.5" customHeight="1">
+      <x:c r="A6" s="63" t="str">
+        <x:v>＜UNION ALL＞</x:v>
+      </x:c>
+      <x:c r="B6" s="63"/>
+      <x:c r="C6" s="63"/>
+      <x:c r="D6" s="63"/>
+      <x:c r="E6" s="63"/>
+      <x:c r="F6" s="63"/>
+      <x:c r="G6" s="63"/>
+      <x:c r="H6" s="63"/>
+      <x:c r="I6" s="63"/>
+      <x:c r="J6" s="63"/>
+      <x:c r="K6" s="63"/>
+      <x:c r="L6" s="63"/>
+      <x:c r="M6" s="63"/>
+      <x:c r="N6" s="63"/>
+      <x:c r="O6" s="63"/>
+      <x:c r="P6" s="63"/>
+      <x:c r="Q6" s="63"/>
+      <x:c r="R6" s="63"/>
+      <x:c r="S6" s="63"/>
+      <x:c r="T6" s="63"/>
+      <x:c r="U6" s="63"/>
+      <x:c r="V6" s="63"/>
+      <x:c r="W6" s="63"/>
+      <x:c r="X6" s="63"/>
+      <x:c r="Y6" s="63"/>
+      <x:c r="Z6" s="63"/>
+      <x:c r="AA6" s="63"/>
+      <x:c r="AB6" s="63"/>
+      <x:c r="AC6" s="63"/>
+      <x:c r="AD6" s="63"/>
+      <x:c r="AE6" s="63"/>
+      <x:c r="AF6" s="63"/>
+      <x:c r="AG6" s="63"/>
+      <x:c r="AH6" s="63"/>
+      <x:c r="AI6" s="63"/>
+      <x:c r="AJ6" s="63"/>
+      <x:c r="AK6" s="63"/>
+      <x:c r="AL6" s="63"/>
+      <x:c r="AM6" s="63"/>
+      <x:c r="AN6" s="63"/>
+      <x:c r="AO6" s="63"/>
+      <x:c r="AP6" s="63"/>
+      <x:c r="AQ6" s="63"/>
+      <x:c r="AR6" s="63"/>
+      <x:c r="AS6" s="63"/>
+      <x:c r="AT6" s="63"/>
+      <x:c r="AU6" s="63"/>
+      <x:c r="AV6" s="63"/>
+      <x:c r="AW6" s="63"/>
+      <x:c r="AX6" s="63"/>
+      <x:c r="AY6" s="63"/>
+      <x:c r="AZ6" s="63"/>
+      <x:c r="BA6" s="63"/>
+      <x:c r="BB6" s="63"/>
+      <x:c r="BC6" s="63"/>
+      <x:c r="BD6" s="63"/>
+      <x:c r="BE6" s="63"/>
+      <x:c r="BF6" s="63"/>
+      <x:c r="BG6" s="63"/>
+      <x:c r="BH6" s="63"/>
+      <x:c r="BI6" s="63"/>
+      <x:c r="BJ6" s="63"/>
+      <x:c r="BK6" s="63"/>
+      <x:c r="BL6" s="63"/>
+      <x:c r="BM6" s="63"/>
+      <x:c r="BN6" s="63"/>
+      <x:c r="BO6" s="63"/>
+      <x:c r="BP6" s="63"/>
+      <x:c r="BQ6" s="63"/>
+      <x:c r="BR6" s="63"/>
+      <x:c r="BS6" s="63"/>
+      <x:c r="BT6" s="63"/>
+      <x:c r="BU6" s="63"/>
+      <x:c r="BV6" s="63"/>
+      <x:c r="BW6" s="63"/>
+      <x:c r="BX6" s="63"/>
+      <x:c r="BY6" s="63"/>
+      <x:c r="BZ6" s="63"/>
+      <x:c r="CA6" s="63"/>
+      <x:c r="CB6" s="63"/>
+      <x:c r="CC6" s="63"/>
+      <x:c r="CD6" s="63"/>
+      <x:c r="CE6" s="63"/>
+      <x:c r="CF6" s="63"/>
+      <x:c r="CG6" s="63"/>
+      <x:c r="CH6" s="63"/>
+      <x:c r="CI6" s="63"/>
+      <x:c r="CJ6" s="63"/>
+      <x:c r="CK6" s="63"/>
+      <x:c r="CL6" s="63"/>
+    </x:row>
+    <x:row r="7" ht="13.5" customHeight="1">
+      <x:c r="A7" s="71" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B7" s="72"/>
+      <x:c r="C7" s="72"/>
+      <x:c r="D7" s="72"/>
+      <x:c r="E7" s="72"/>
+      <x:c r="F7" s="72"/>
+      <x:c r="G7" s="77" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H7" s="63"/>
+      <x:c r="I7" s="63"/>
+      <x:c r="J7" s="63"/>
+      <x:c r="K7" s="63"/>
+      <x:c r="L7" s="63"/>
+      <x:c r="M7" s="63"/>
+      <x:c r="N7" s="63"/>
+      <x:c r="O7" s="63" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="P7" s="63"/>
+      <x:c r="Q7" s="63" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="R7" s="63"/>
+      <x:c r="S7" s="63"/>
+      <x:c r="T7" s="63"/>
+      <x:c r="U7" s="63"/>
+      <x:c r="V7" s="63"/>
+      <x:c r="W7" s="63"/>
+      <x:c r="X7" s="63"/>
+      <x:c r="Y7" s="63"/>
+      <x:c r="Z7" s="63"/>
+      <x:c r="AA7" s="63"/>
+      <x:c r="AB7" s="63"/>
+      <x:c r="AC7" s="63"/>
+      <x:c r="AD7" s="63"/>
+      <x:c r="AE7" s="63"/>
+      <x:c r="AF7" s="63"/>
+      <x:c r="AG7" s="63"/>
+      <x:c r="AH7" s="63"/>
+      <x:c r="AI7" s="63"/>
+      <x:c r="AJ7" s="63"/>
+      <x:c r="AK7" s="63"/>
+      <x:c r="AL7" s="63"/>
+      <x:c r="AM7" s="63"/>
+      <x:c r="AN7" s="63"/>
+      <x:c r="AO7" s="63"/>
+      <x:c r="AP7" s="63"/>
+      <x:c r="AQ7" s="63"/>
+      <x:c r="AR7" s="63"/>
+      <x:c r="AS7" s="63"/>
+      <x:c r="AT7" s="63"/>
+      <x:c r="AU7" s="63"/>
+      <x:c r="AV7" s="63"/>
+      <x:c r="AW7" s="63"/>
+      <x:c r="AX7" s="63"/>
+      <x:c r="AY7" s="63"/>
+      <x:c r="AZ7" s="63"/>
+      <x:c r="BA7" s="63"/>
+      <x:c r="BB7" s="63"/>
+      <x:c r="BC7" s="63"/>
+      <x:c r="BD7" s="63"/>
+      <x:c r="BE7" s="63"/>
+      <x:c r="BF7" s="63"/>
+      <x:c r="BG7" s="63"/>
+      <x:c r="BH7" s="63"/>
+      <x:c r="BI7" s="63"/>
+      <x:c r="BJ7" s="63"/>
+      <x:c r="BK7" s="63"/>
+      <x:c r="BL7" s="63"/>
+      <x:c r="BM7" s="63"/>
+      <x:c r="BN7" s="63"/>
+      <x:c r="BO7" s="63"/>
+      <x:c r="BP7" s="63"/>
+      <x:c r="BQ7" s="63"/>
+      <x:c r="BR7" s="63"/>
+      <x:c r="BS7" s="63"/>
+      <x:c r="BT7" s="63"/>
+      <x:c r="BU7" s="63"/>
+      <x:c r="BV7" s="63"/>
+      <x:c r="BW7" s="63"/>
+      <x:c r="BX7" s="63"/>
+      <x:c r="BY7" s="63"/>
+      <x:c r="BZ7" s="63"/>
+      <x:c r="CA7" s="63"/>
+      <x:c r="CB7" s="63"/>
+      <x:c r="CC7" s="63"/>
+      <x:c r="CD7" s="63"/>
+      <x:c r="CE7" s="63"/>
+      <x:c r="CF7" s="63"/>
+      <x:c r="CG7" s="63"/>
+      <x:c r="CH7" s="63"/>
+      <x:c r="CI7" s="63"/>
+      <x:c r="CJ7" s="63"/>
+      <x:c r="CK7" s="63"/>
+      <x:c r="CL7" s="78"/>
+    </x:row>
+    <x:row r="8" ht="13.5" customHeight="1">
+      <x:c r="A8" s="73"/>
+      <x:c r="B8" s="74"/>
+      <x:c r="C8" s="74"/>
+      <x:c r="D8" s="74"/>
+      <x:c r="E8" s="74"/>
+      <x:c r="F8" s="74"/>
+      <x:c r="G8" s="79" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H8" s="80"/>
+      <x:c r="I8" s="80"/>
+      <x:c r="J8" s="80"/>
+      <x:c r="K8" s="80"/>
+      <x:c r="L8" s="80"/>
+      <x:c r="M8" s="80"/>
+      <x:c r="N8" s="80"/>
+      <x:c r="O8" s="80" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="P8" s="80"/>
+      <x:c r="Q8" s="80" t="str">
+        <x:v>TRIM(tb2.氏名)</x:v>
+      </x:c>
+      <x:c r="R8" s="80"/>
+      <x:c r="S8" s="80"/>
+      <x:c r="T8" s="80"/>
+      <x:c r="U8" s="80"/>
+      <x:c r="V8" s="80"/>
+      <x:c r="W8" s="80"/>
+      <x:c r="X8" s="80"/>
+      <x:c r="Y8" s="80"/>
+      <x:c r="Z8" s="80"/>
+      <x:c r="AA8" s="80"/>
+      <x:c r="AB8" s="80"/>
+      <x:c r="AC8" s="80"/>
+      <x:c r="AD8" s="80"/>
+      <x:c r="AE8" s="80"/>
+      <x:c r="AF8" s="80"/>
+      <x:c r="AG8" s="80"/>
+      <x:c r="AH8" s="80"/>
+      <x:c r="AI8" s="80"/>
+      <x:c r="AJ8" s="80"/>
+      <x:c r="AK8" s="80"/>
+      <x:c r="AL8" s="80"/>
+      <x:c r="AM8" s="80"/>
+      <x:c r="AN8" s="80"/>
+      <x:c r="AO8" s="80"/>
+      <x:c r="AP8" s="80"/>
+      <x:c r="AQ8" s="80"/>
+      <x:c r="AR8" s="80"/>
+      <x:c r="AS8" s="80"/>
+      <x:c r="AT8" s="80"/>
+      <x:c r="AU8" s="80"/>
+      <x:c r="AV8" s="80"/>
+      <x:c r="AW8" s="80"/>
+      <x:c r="AX8" s="80"/>
+      <x:c r="AY8" s="80"/>
+      <x:c r="AZ8" s="80"/>
+      <x:c r="BA8" s="80"/>
+      <x:c r="BB8" s="80"/>
+      <x:c r="BC8" s="80"/>
+      <x:c r="BD8" s="80"/>
+      <x:c r="BE8" s="80"/>
+      <x:c r="BF8" s="80"/>
+      <x:c r="BG8" s="80"/>
+      <x:c r="BH8" s="80"/>
+      <x:c r="BI8" s="80"/>
+      <x:c r="BJ8" s="80"/>
+      <x:c r="BK8" s="80"/>
+      <x:c r="BL8" s="80"/>
+      <x:c r="BM8" s="80"/>
+      <x:c r="BN8" s="80"/>
+      <x:c r="BO8" s="80"/>
+      <x:c r="BP8" s="80"/>
+      <x:c r="BQ8" s="80"/>
+      <x:c r="BR8" s="80"/>
+      <x:c r="BS8" s="80"/>
+      <x:c r="BT8" s="80"/>
+      <x:c r="BU8" s="80"/>
+      <x:c r="BV8" s="80"/>
+      <x:c r="BW8" s="80"/>
+      <x:c r="BX8" s="80"/>
+      <x:c r="BY8" s="80"/>
+      <x:c r="BZ8" s="80"/>
+      <x:c r="CA8" s="80"/>
+      <x:c r="CB8" s="80"/>
+      <x:c r="CC8" s="80"/>
+      <x:c r="CD8" s="80"/>
+      <x:c r="CE8" s="80"/>
+      <x:c r="CF8" s="80"/>
+      <x:c r="CG8" s="80"/>
+      <x:c r="CH8" s="80"/>
+      <x:c r="CI8" s="80"/>
+      <x:c r="CJ8" s="80"/>
+      <x:c r="CK8" s="80"/>
+      <x:c r="CL8" s="81"/>
+    </x:row>
+    <x:row r="9" ht="13.5" customHeight="1">
+      <x:c r="A9" s="67" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B9" s="68"/>
+      <x:c r="C9" s="68"/>
+      <x:c r="D9" s="68"/>
+      <x:c r="E9" s="68"/>
+      <x:c r="F9" s="68"/>
+      <x:c r="G9" s="64"/>
+      <x:c r="H9" s="65"/>
+      <x:c r="I9" s="65"/>
+      <x:c r="J9" s="65"/>
+      <x:c r="K9" s="65"/>
+      <x:c r="L9" s="65"/>
+      <x:c r="M9" s="65"/>
+      <x:c r="N9" s="65"/>
+      <x:c r="O9" s="65"/>
+      <x:c r="P9" s="65"/>
+      <x:c r="Q9" s="65" t="str">
+        <x:v>tb2.状態 = 'INACTIVE'</x:v>
+      </x:c>
+      <x:c r="R9" s="65"/>
+      <x:c r="S9" s="65"/>
+      <x:c r="T9" s="65"/>
+      <x:c r="U9" s="65"/>
+      <x:c r="V9" s="65"/>
+      <x:c r="W9" s="65"/>
+      <x:c r="X9" s="65"/>
+      <x:c r="Y9" s="65"/>
+      <x:c r="Z9" s="65"/>
+      <x:c r="AA9" s="65"/>
+      <x:c r="AB9" s="65"/>
+      <x:c r="AC9" s="65"/>
+      <x:c r="AD9" s="65"/>
+      <x:c r="AE9" s="65"/>
+      <x:c r="AF9" s="65"/>
+      <x:c r="AG9" s="65"/>
+      <x:c r="AH9" s="65"/>
+      <x:c r="AI9" s="65"/>
+      <x:c r="AJ9" s="65"/>
+      <x:c r="AK9" s="65"/>
+      <x:c r="AL9" s="65"/>
+      <x:c r="AM9" s="65"/>
+      <x:c r="AN9" s="65"/>
+      <x:c r="AO9" s="65"/>
+      <x:c r="AP9" s="65"/>
+      <x:c r="AQ9" s="65"/>
+      <x:c r="AR9" s="65"/>
+      <x:c r="AS9" s="65"/>
+      <x:c r="AT9" s="65"/>
+      <x:c r="AU9" s="65"/>
+      <x:c r="AV9" s="65"/>
+      <x:c r="AW9" s="65"/>
+      <x:c r="AX9" s="65"/>
+      <x:c r="AY9" s="65"/>
+      <x:c r="AZ9" s="65"/>
+      <x:c r="BA9" s="65"/>
+      <x:c r="BB9" s="65"/>
+      <x:c r="BC9" s="65"/>
+      <x:c r="BD9" s="65"/>
+      <x:c r="BE9" s="65"/>
+      <x:c r="BF9" s="65"/>
+      <x:c r="BG9" s="65"/>
+      <x:c r="BH9" s="65"/>
+      <x:c r="BI9" s="65"/>
+      <x:c r="BJ9" s="65"/>
+      <x:c r="BK9" s="65"/>
+      <x:c r="BL9" s="65"/>
+      <x:c r="BM9" s="65"/>
+      <x:c r="BN9" s="65"/>
+      <x:c r="BO9" s="65"/>
+      <x:c r="BP9" s="65"/>
+      <x:c r="BQ9" s="65"/>
+      <x:c r="BR9" s="65"/>
+      <x:c r="BS9" s="65"/>
+      <x:c r="BT9" s="65"/>
+      <x:c r="BU9" s="65"/>
+      <x:c r="BV9" s="65"/>
+      <x:c r="BW9" s="65"/>
+      <x:c r="BX9" s="65"/>
+      <x:c r="BY9" s="65"/>
+      <x:c r="BZ9" s="65"/>
+      <x:c r="CA9" s="65"/>
+      <x:c r="CB9" s="65"/>
+      <x:c r="CC9" s="65"/>
+      <x:c r="CD9" s="65"/>
+      <x:c r="CE9" s="65"/>
+      <x:c r="CF9" s="65"/>
+      <x:c r="CG9" s="65"/>
+      <x:c r="CH9" s="65"/>
+      <x:c r="CI9" s="65"/>
+      <x:c r="CJ9" s="65"/>
+      <x:c r="CK9" s="65"/>
+      <x:c r="CL9" s="66"/>
+    </x:row>
+    <x:row r="10" ht="13.5" customHeight="1">
+      <x:c r="A10" s="61"/>
+      <x:c r="B10" s="61"/>
+      <x:c r="C10" s="61"/>
+      <x:c r="D10" s="61"/>
+      <x:c r="E10" s="61"/>
+      <x:c r="F10" s="61"/>
+      <x:c r="G10" s="61"/>
+      <x:c r="H10" s="61"/>
+      <x:c r="I10" s="61"/>
+      <x:c r="J10" s="61"/>
+      <x:c r="K10" s="61"/>
+      <x:c r="L10" s="61"/>
+      <x:c r="M10" s="61"/>
+      <x:c r="N10" s="61"/>
+      <x:c r="O10" s="61"/>
+      <x:c r="P10" s="61"/>
+      <x:c r="Q10" s="61"/>
+      <x:c r="R10" s="61"/>
+      <x:c r="S10" s="61"/>
+      <x:c r="T10" s="61"/>
+      <x:c r="U10" s="61"/>
+      <x:c r="V10" s="61"/>
+      <x:c r="W10" s="61"/>
+      <x:c r="X10" s="61"/>
+      <x:c r="Y10" s="61"/>
+      <x:c r="Z10" s="61"/>
+      <x:c r="AA10" s="61"/>
+      <x:c r="AB10" s="61"/>
+      <x:c r="AC10" s="61"/>
+      <x:c r="AD10" s="61"/>
+      <x:c r="AE10" s="61"/>
+      <x:c r="AF10" s="61"/>
+      <x:c r="AG10" s="61"/>
+      <x:c r="AH10" s="61"/>
+      <x:c r="AI10" s="61"/>
+      <x:c r="AJ10" s="61"/>
+      <x:c r="AK10" s="61"/>
+      <x:c r="AL10" s="61"/>
+      <x:c r="AM10" s="61"/>
+      <x:c r="AN10" s="61"/>
+      <x:c r="AO10" s="61"/>
+      <x:c r="AP10" s="61"/>
+      <x:c r="AQ10" s="61"/>
+      <x:c r="AR10" s="61"/>
+      <x:c r="AS10" s="61"/>
+      <x:c r="AT10" s="61"/>
+      <x:c r="AU10" s="61"/>
+      <x:c r="AV10" s="61"/>
+      <x:c r="AW10" s="61"/>
+      <x:c r="AX10" s="61"/>
+      <x:c r="AY10" s="61"/>
+      <x:c r="AZ10" s="61"/>
+      <x:c r="BA10" s="61"/>
+      <x:c r="BB10" s="61"/>
+      <x:c r="BC10" s="61"/>
+      <x:c r="BD10" s="61"/>
+      <x:c r="BE10" s="61"/>
+      <x:c r="BF10" s="61"/>
+      <x:c r="BG10" s="61"/>
+      <x:c r="BH10" s="61"/>
+      <x:c r="BI10" s="61"/>
+      <x:c r="BJ10" s="61"/>
+      <x:c r="BK10" s="61"/>
+      <x:c r="BL10" s="61"/>
+      <x:c r="BM10" s="61"/>
+      <x:c r="BN10" s="61"/>
+      <x:c r="BO10" s="61"/>
+      <x:c r="BP10" s="61"/>
+      <x:c r="BQ10" s="61"/>
+      <x:c r="BR10" s="61"/>
+      <x:c r="BS10" s="61"/>
+      <x:c r="BT10" s="61"/>
+      <x:c r="BU10" s="61"/>
+      <x:c r="BV10" s="61"/>
+      <x:c r="BW10" s="61"/>
+      <x:c r="BX10" s="61"/>
+      <x:c r="BY10" s="61"/>
+      <x:c r="BZ10" s="61"/>
+      <x:c r="CA10" s="61"/>
+      <x:c r="CB10" s="61"/>
+      <x:c r="CC10" s="61"/>
+      <x:c r="CD10" s="61"/>
+      <x:c r="CE10" s="61"/>
+      <x:c r="CF10" s="61"/>
+      <x:c r="CG10" s="61"/>
+      <x:c r="CH10" s="61"/>
+      <x:c r="CI10" s="61"/>
+      <x:c r="CJ10" s="61"/>
+      <x:c r="CK10" s="61"/>
+      <x:c r="CL10" s="61"/>
+    </x:row>
+    <x:row r="11" ht="13.5" customHeight="1">
+      <x:c r="A11" s="61" t="str">
+        <x:v>＜データ移送表＞</x:v>
+      </x:c>
+      <x:c r="B11" s="61"/>
+      <x:c r="C11" s="61"/>
+      <x:c r="D11" s="61"/>
+      <x:c r="E11" s="61"/>
+      <x:c r="F11" s="61"/>
+      <x:c r="G11" s="61"/>
+      <x:c r="H11" s="61"/>
+      <x:c r="I11" s="61"/>
+      <x:c r="J11" s="61"/>
+      <x:c r="K11" s="61"/>
+      <x:c r="L11" s="61"/>
+      <x:c r="M11" s="61"/>
+      <x:c r="N11" s="61"/>
+      <x:c r="O11" s="61"/>
+      <x:c r="P11" s="61"/>
+      <x:c r="Q11" s="61"/>
+      <x:c r="R11" s="61"/>
+      <x:c r="S11" s="61"/>
+      <x:c r="T11" s="61"/>
+      <x:c r="U11" s="61"/>
+      <x:c r="V11" s="61"/>
+      <x:c r="W11" s="61"/>
+      <x:c r="X11" s="61"/>
+      <x:c r="Y11" s="61"/>
+      <x:c r="Z11" s="61"/>
+      <x:c r="AA11" s="61"/>
+      <x:c r="AB11" s="61"/>
+      <x:c r="AC11" s="61"/>
+      <x:c r="AD11" s="61"/>
+      <x:c r="AE11" s="61"/>
+      <x:c r="AF11" s="61"/>
+      <x:c r="AG11" s="61"/>
+      <x:c r="AH11" s="61"/>
+      <x:c r="AI11" s="61"/>
+      <x:c r="AJ11" s="61"/>
+      <x:c r="AK11" s="61"/>
+      <x:c r="AL11" s="61"/>
+      <x:c r="AM11" s="61"/>
+      <x:c r="AN11" s="61"/>
+      <x:c r="AO11" s="61"/>
+      <x:c r="AP11" s="61"/>
+      <x:c r="AQ11" s="61"/>
+      <x:c r="AR11" s="61"/>
+      <x:c r="AS11" s="61"/>
+      <x:c r="AT11" s="61"/>
+      <x:c r="AU11" s="61"/>
+      <x:c r="AV11" s="61"/>
+      <x:c r="AW11" s="61"/>
+      <x:c r="AX11" s="61"/>
+      <x:c r="AY11" s="61"/>
+      <x:c r="AZ11" s="61"/>
+      <x:c r="BA11" s="61"/>
+      <x:c r="BB11" s="61"/>
+      <x:c r="BC11" s="61"/>
+      <x:c r="BD11" s="61"/>
+      <x:c r="BE11" s="61"/>
+      <x:c r="BF11" s="61"/>
+      <x:c r="BG11" s="61"/>
+      <x:c r="BH11" s="61"/>
+      <x:c r="BI11" s="61"/>
+      <x:c r="BJ11" s="61"/>
+      <x:c r="BK11" s="61"/>
+      <x:c r="BL11" s="61"/>
+      <x:c r="BM11" s="61"/>
+      <x:c r="BN11" s="61"/>
+      <x:c r="BO11" s="61"/>
+      <x:c r="BP11" s="61"/>
+      <x:c r="BQ11" s="61"/>
+      <x:c r="BR11" s="61"/>
+      <x:c r="BS11" s="61"/>
+      <x:c r="BT11" s="61"/>
+      <x:c r="BU11" s="61"/>
+      <x:c r="BV11" s="61"/>
+      <x:c r="BW11" s="61"/>
+      <x:c r="BX11" s="61"/>
+      <x:c r="BY11" s="61"/>
+      <x:c r="BZ11" s="61"/>
+      <x:c r="CA11" s="61"/>
+      <x:c r="CB11" s="61"/>
+      <x:c r="CC11" s="61"/>
+      <x:c r="CD11" s="61"/>
+      <x:c r="CE11" s="61"/>
+      <x:c r="CF11" s="61"/>
+      <x:c r="CG11" s="61"/>
+      <x:c r="CH11" s="61"/>
+      <x:c r="CI11" s="61"/>
+      <x:c r="CJ11" s="61"/>
+      <x:c r="CK11" s="61"/>
+      <x:c r="CL11" s="61"/>
+    </x:row>
+    <x:row r="12" ht="13.5" customHeight="1">
+      <x:c r="A12" s="61" t="str">
+        <x:v>参照テーブル: ユーザーアーカイブ</x:v>
+      </x:c>
+      <x:c r="B12" s="61"/>
+      <x:c r="C12" s="61"/>
+      <x:c r="D12" s="61"/>
+      <x:c r="E12" s="61"/>
+      <x:c r="F12" s="61"/>
+      <x:c r="G12" s="61"/>
+      <x:c r="H12" s="61"/>
+      <x:c r="I12" s="61"/>
+      <x:c r="J12" s="61"/>
+      <x:c r="K12" s="61"/>
+      <x:c r="L12" s="61"/>
+      <x:c r="M12" s="61"/>
+      <x:c r="N12" s="61"/>
+      <x:c r="O12" s="61"/>
+      <x:c r="P12" s="61"/>
+      <x:c r="Q12" s="61"/>
+      <x:c r="R12" s="61"/>
+      <x:c r="S12" s="61"/>
+      <x:c r="T12" s="61"/>
+      <x:c r="U12" s="61"/>
+      <x:c r="V12" s="61"/>
+      <x:c r="W12" s="61"/>
+      <x:c r="X12" s="61"/>
+      <x:c r="Y12" s="61"/>
+      <x:c r="Z12" s="61"/>
+      <x:c r="AA12" s="61"/>
+      <x:c r="AB12" s="61"/>
+      <x:c r="AC12" s="61"/>
+      <x:c r="AD12" s="61"/>
+      <x:c r="AE12" s="61"/>
+      <x:c r="AF12" s="61"/>
+      <x:c r="AG12" s="61"/>
+      <x:c r="AH12" s="61"/>
+      <x:c r="AI12" s="61"/>
+      <x:c r="AJ12" s="61"/>
+      <x:c r="AK12" s="61"/>
+      <x:c r="AL12" s="61"/>
+      <x:c r="AM12" s="61"/>
+      <x:c r="AN12" s="61"/>
+      <x:c r="AO12" s="61"/>
+      <x:c r="AP12" s="61"/>
+      <x:c r="AQ12" s="61"/>
+      <x:c r="AR12" s="61"/>
+      <x:c r="AS12" s="61"/>
+      <x:c r="AT12" s="61"/>
+      <x:c r="AU12" s="61"/>
+      <x:c r="AV12" s="61"/>
+      <x:c r="AW12" s="61"/>
+      <x:c r="AX12" s="61"/>
+      <x:c r="AY12" s="61"/>
+      <x:c r="AZ12" s="61"/>
+      <x:c r="BA12" s="61"/>
+      <x:c r="BB12" s="61"/>
+      <x:c r="BC12" s="61"/>
+      <x:c r="BD12" s="61"/>
+      <x:c r="BE12" s="61"/>
+      <x:c r="BF12" s="61"/>
+      <x:c r="BG12" s="61"/>
+      <x:c r="BH12" s="61"/>
+      <x:c r="BI12" s="61"/>
+      <x:c r="BJ12" s="61"/>
+      <x:c r="BK12" s="61"/>
+      <x:c r="BL12" s="61"/>
+      <x:c r="BM12" s="61"/>
+      <x:c r="BN12" s="61"/>
+      <x:c r="BO12" s="61"/>
+      <x:c r="BP12" s="61"/>
+      <x:c r="BQ12" s="61"/>
+      <x:c r="BR12" s="61"/>
+      <x:c r="BS12" s="61"/>
+      <x:c r="BT12" s="61"/>
+      <x:c r="BU12" s="61"/>
+      <x:c r="BV12" s="61"/>
+      <x:c r="BW12" s="61"/>
+      <x:c r="BX12" s="61"/>
+      <x:c r="BY12" s="61"/>
+      <x:c r="BZ12" s="61"/>
+      <x:c r="CA12" s="61"/>
+      <x:c r="CB12" s="61"/>
+      <x:c r="CC12" s="61"/>
+      <x:c r="CD12" s="61"/>
+      <x:c r="CE12" s="61"/>
+      <x:c r="CF12" s="61"/>
+      <x:c r="CG12" s="61"/>
+      <x:c r="CH12" s="61"/>
+      <x:c r="CI12" s="61"/>
+      <x:c r="CJ12" s="61"/>
+      <x:c r="CK12" s="61"/>
+      <x:c r="CL12" s="61"/>
+    </x:row>
+    <x:row r="13" ht="13.5" customHeight="1">
+      <x:c r="A13" s="63" t="str">
+        <x:v>＜移送パターン1＞</x:v>
+      </x:c>
+      <x:c r="B13" s="63"/>
+      <x:c r="C13" s="63"/>
+      <x:c r="D13" s="63"/>
+      <x:c r="E13" s="63"/>
+      <x:c r="F13" s="63"/>
+      <x:c r="G13" s="63"/>
+      <x:c r="H13" s="63"/>
+      <x:c r="I13" s="63"/>
+      <x:c r="J13" s="63"/>
+      <x:c r="K13" s="63"/>
+      <x:c r="L13" s="63"/>
+      <x:c r="M13" s="63"/>
+      <x:c r="N13" s="63"/>
+      <x:c r="O13" s="63"/>
+      <x:c r="P13" s="63"/>
+      <x:c r="Q13" s="63"/>
+      <x:c r="R13" s="63"/>
+      <x:c r="S13" s="63"/>
+      <x:c r="T13" s="63"/>
+      <x:c r="U13" s="63"/>
+      <x:c r="V13" s="63"/>
+      <x:c r="W13" s="63"/>
+      <x:c r="X13" s="63"/>
+      <x:c r="Y13" s="63"/>
+      <x:c r="Z13" s="63"/>
+      <x:c r="AA13" s="63"/>
+      <x:c r="AB13" s="63"/>
+      <x:c r="AC13" s="63"/>
+      <x:c r="AD13" s="63"/>
+      <x:c r="AE13" s="63"/>
+      <x:c r="AF13" s="63"/>
+      <x:c r="AG13" s="63"/>
+      <x:c r="AH13" s="63"/>
+      <x:c r="AI13" s="63"/>
+      <x:c r="AJ13" s="63"/>
+      <x:c r="AK13" s="63"/>
+      <x:c r="AL13" s="63"/>
+      <x:c r="AM13" s="63"/>
+      <x:c r="AN13" s="63"/>
+      <x:c r="AO13" s="63"/>
+      <x:c r="AP13" s="63"/>
+      <x:c r="AQ13" s="63"/>
+      <x:c r="AR13" s="63"/>
+      <x:c r="AS13" s="63"/>
+      <x:c r="AT13" s="63"/>
+      <x:c r="AU13" s="63"/>
+      <x:c r="AV13" s="63"/>
+      <x:c r="AW13" s="63"/>
+      <x:c r="AX13" s="63"/>
+      <x:c r="AY13" s="63"/>
+      <x:c r="AZ13" s="63"/>
+      <x:c r="BA13" s="63"/>
+      <x:c r="BB13" s="63"/>
+      <x:c r="BC13" s="63"/>
+      <x:c r="BD13" s="63"/>
+      <x:c r="BE13" s="63"/>
+      <x:c r="BF13" s="63"/>
+      <x:c r="BG13" s="63"/>
+      <x:c r="BH13" s="63"/>
+      <x:c r="BI13" s="63"/>
+      <x:c r="BJ13" s="63"/>
+      <x:c r="BK13" s="63"/>
+      <x:c r="BL13" s="63"/>
+      <x:c r="BM13" s="63"/>
+      <x:c r="BN13" s="63"/>
+      <x:c r="BO13" s="63"/>
+      <x:c r="BP13" s="63"/>
+      <x:c r="BQ13" s="63"/>
+      <x:c r="BR13" s="63"/>
+      <x:c r="BS13" s="63"/>
+      <x:c r="BT13" s="63"/>
+      <x:c r="BU13" s="63"/>
+      <x:c r="BV13" s="63"/>
+      <x:c r="BW13" s="63"/>
+      <x:c r="BX13" s="63"/>
+      <x:c r="BY13" s="63"/>
+      <x:c r="BZ13" s="63"/>
+      <x:c r="CA13" s="63"/>
+      <x:c r="CB13" s="63"/>
+      <x:c r="CC13" s="63"/>
+      <x:c r="CD13" s="63"/>
+      <x:c r="CE13" s="63"/>
+      <x:c r="CF13" s="63"/>
+      <x:c r="CG13" s="63"/>
+      <x:c r="CH13" s="63"/>
+      <x:c r="CI13" s="63"/>
+      <x:c r="CJ13" s="63"/>
+      <x:c r="CK13" s="63"/>
+      <x:c r="CL13" s="63"/>
+    </x:row>
+    <x:row r="14" ht="13.5" customHeight="1">
+      <x:c r="A14" s="67" t="str">
+        <x:v>項目</x:v>
+      </x:c>
+      <x:c r="B14" s="68"/>
+      <x:c r="C14" s="68"/>
+      <x:c r="D14" s="68"/>
+      <x:c r="E14" s="68"/>
+      <x:c r="F14" s="68"/>
+      <x:c r="G14" s="68"/>
+      <x:c r="H14" s="68"/>
+      <x:c r="I14" s="68"/>
+      <x:c r="J14" s="68"/>
+      <x:c r="K14" s="68"/>
+      <x:c r="L14" s="68"/>
+      <x:c r="M14" s="68"/>
+      <x:c r="N14" s="68"/>
+      <x:c r="O14" s="68"/>
+      <x:c r="P14" s="68"/>
+      <x:c r="Q14" s="68"/>
+      <x:c r="R14" s="68"/>
+      <x:c r="S14" s="67" t="str">
+        <x:v>移送元</x:v>
+      </x:c>
+      <x:c r="T14" s="68"/>
+      <x:c r="U14" s="68"/>
+      <x:c r="V14" s="68"/>
+      <x:c r="W14" s="68"/>
+      <x:c r="X14" s="68"/>
+      <x:c r="Y14" s="68"/>
+      <x:c r="Z14" s="68"/>
+      <x:c r="AA14" s="68"/>
+      <x:c r="AB14" s="68"/>
+      <x:c r="AC14" s="68"/>
+      <x:c r="AD14" s="68"/>
+      <x:c r="AE14" s="68"/>
+      <x:c r="AF14" s="68"/>
+      <x:c r="AG14" s="68"/>
+      <x:c r="AH14" s="68"/>
+      <x:c r="AI14" s="68"/>
+      <x:c r="AJ14" s="68"/>
+      <x:c r="AK14" s="67" t="str">
+        <x:v>移送方法ほか</x:v>
+      </x:c>
+      <x:c r="AL14" s="68"/>
+      <x:c r="AM14" s="68"/>
+      <x:c r="AN14" s="68"/>
+      <x:c r="AO14" s="68"/>
+      <x:c r="AP14" s="68"/>
+      <x:c r="AQ14" s="68"/>
+      <x:c r="AR14" s="68"/>
+      <x:c r="AS14" s="68"/>
+      <x:c r="AT14" s="68"/>
+      <x:c r="AU14" s="68"/>
+      <x:c r="AV14" s="68"/>
+      <x:c r="AW14" s="68"/>
+      <x:c r="AX14" s="68"/>
+      <x:c r="AY14" s="68"/>
+      <x:c r="AZ14" s="68"/>
+      <x:c r="BA14" s="68"/>
+      <x:c r="BB14" s="68"/>
+      <x:c r="BC14" s="68"/>
+      <x:c r="BD14" s="68"/>
+      <x:c r="BE14" s="68"/>
+      <x:c r="BF14" s="68"/>
+      <x:c r="BG14" s="68"/>
+      <x:c r="BH14" s="68"/>
+      <x:c r="BI14" s="68"/>
+      <x:c r="BJ14" s="68"/>
+      <x:c r="BK14" s="68"/>
+      <x:c r="BL14" s="68"/>
+      <x:c r="BM14" s="68"/>
+      <x:c r="BN14" s="68"/>
+      <x:c r="BO14" s="68"/>
+      <x:c r="BP14" s="68"/>
+      <x:c r="BQ14" s="68"/>
+      <x:c r="BR14" s="68"/>
+      <x:c r="BS14" s="68"/>
+      <x:c r="BT14" s="68"/>
+      <x:c r="BU14" s="68"/>
+      <x:c r="BV14" s="68"/>
+      <x:c r="BW14" s="68"/>
+      <x:c r="BX14" s="68"/>
+      <x:c r="BY14" s="68"/>
+      <x:c r="BZ14" s="68"/>
+      <x:c r="CA14" s="68"/>
+      <x:c r="CB14" s="68"/>
+      <x:c r="CC14" s="68"/>
+      <x:c r="CD14" s="68"/>
+      <x:c r="CE14" s="68"/>
+      <x:c r="CF14" s="68"/>
+      <x:c r="CG14" s="68"/>
+      <x:c r="CH14" s="68"/>
+      <x:c r="CI14" s="68"/>
+      <x:c r="CJ14" s="68"/>
+      <x:c r="CK14" s="68"/>
+      <x:c r="CL14" s="69"/>
+    </x:row>
+    <x:row r="15" ht="13.5" customHeight="1">
+      <x:c r="A15" s="64" t="str">
+        <x:v>ユーザーID</x:v>
+      </x:c>
+      <x:c r="B15" s="65"/>
+      <x:c r="C15" s="65"/>
+      <x:c r="D15" s="65"/>
+      <x:c r="E15" s="65"/>
+      <x:c r="F15" s="65"/>
+      <x:c r="G15" s="65"/>
+      <x:c r="H15" s="65"/>
+      <x:c r="I15" s="65"/>
+      <x:c r="J15" s="65"/>
+      <x:c r="K15" s="65"/>
+      <x:c r="L15" s="65"/>
+      <x:c r="M15" s="65"/>
+      <x:c r="N15" s="65"/>
+      <x:c r="O15" s="65"/>
+      <x:c r="P15" s="65"/>
+      <x:c r="Q15" s="65"/>
+      <x:c r="R15" s="65"/>
+      <x:c r="S15" s="64" t="str">
+        <x:v>tb1.ユーザーID</x:v>
+      </x:c>
+      <x:c r="T15" s="65"/>
+      <x:c r="U15" s="65"/>
+      <x:c r="V15" s="65"/>
+      <x:c r="W15" s="65"/>
+      <x:c r="X15" s="65"/>
+      <x:c r="Y15" s="65"/>
+      <x:c r="Z15" s="65"/>
+      <x:c r="AA15" s="65"/>
+      <x:c r="AB15" s="65"/>
+      <x:c r="AC15" s="65"/>
+      <x:c r="AD15" s="65"/>
+      <x:c r="AE15" s="65"/>
+      <x:c r="AF15" s="65"/>
+      <x:c r="AG15" s="65"/>
+      <x:c r="AH15" s="65"/>
+      <x:c r="AI15" s="65"/>
+      <x:c r="AJ15" s="65"/>
+      <x:c r="AK15" s="64"/>
+      <x:c r="AL15" s="65"/>
+      <x:c r="AM15" s="65"/>
+      <x:c r="AN15" s="65"/>
+      <x:c r="AO15" s="65"/>
+      <x:c r="AP15" s="65"/>
+      <x:c r="AQ15" s="65"/>
+      <x:c r="AR15" s="65"/>
+      <x:c r="AS15" s="65"/>
+      <x:c r="AT15" s="65"/>
+      <x:c r="AU15" s="65"/>
+      <x:c r="AV15" s="65"/>
+      <x:c r="AW15" s="65"/>
+      <x:c r="AX15" s="65"/>
+      <x:c r="AY15" s="65"/>
+      <x:c r="AZ15" s="65"/>
+      <x:c r="BA15" s="65"/>
+      <x:c r="BB15" s="65"/>
+      <x:c r="BC15" s="65"/>
+      <x:c r="BD15" s="65"/>
+      <x:c r="BE15" s="65"/>
+      <x:c r="BF15" s="65"/>
+      <x:c r="BG15" s="65"/>
+      <x:c r="BH15" s="65"/>
+      <x:c r="BI15" s="65"/>
+      <x:c r="BJ15" s="65"/>
+      <x:c r="BK15" s="65"/>
+      <x:c r="BL15" s="65"/>
+      <x:c r="BM15" s="65"/>
+      <x:c r="BN15" s="65"/>
+      <x:c r="BO15" s="65"/>
+      <x:c r="BP15" s="65"/>
+      <x:c r="BQ15" s="65"/>
+      <x:c r="BR15" s="65"/>
+      <x:c r="BS15" s="65"/>
+      <x:c r="BT15" s="65"/>
+      <x:c r="BU15" s="65"/>
+      <x:c r="BV15" s="65"/>
+      <x:c r="BW15" s="65"/>
+      <x:c r="BX15" s="65"/>
+      <x:c r="BY15" s="65"/>
+      <x:c r="BZ15" s="65"/>
+      <x:c r="CA15" s="65"/>
+      <x:c r="CB15" s="65"/>
+      <x:c r="CC15" s="65"/>
+      <x:c r="CD15" s="65"/>
+      <x:c r="CE15" s="65"/>
+      <x:c r="CF15" s="65"/>
+      <x:c r="CG15" s="65"/>
+      <x:c r="CH15" s="65"/>
+      <x:c r="CI15" s="65"/>
+      <x:c r="CJ15" s="65"/>
+      <x:c r="CK15" s="65"/>
+      <x:c r="CL15" s="66"/>
+    </x:row>
+    <x:row r="16" ht="13.5" customHeight="1">
+      <x:c r="A16" s="64" t="str">
+        <x:v>氏名</x:v>
+      </x:c>
+      <x:c r="B16" s="65"/>
+      <x:c r="C16" s="65"/>
+      <x:c r="D16" s="65"/>
+      <x:c r="E16" s="65"/>
+      <x:c r="F16" s="65"/>
+      <x:c r="G16" s="65"/>
+      <x:c r="H16" s="65"/>
+      <x:c r="I16" s="65"/>
+      <x:c r="J16" s="65"/>
+      <x:c r="K16" s="65"/>
+      <x:c r="L16" s="65"/>
+      <x:c r="M16" s="65"/>
+      <x:c r="N16" s="65"/>
+      <x:c r="O16" s="65"/>
+      <x:c r="P16" s="65"/>
+      <x:c r="Q16" s="65"/>
+      <x:c r="R16" s="65"/>
+      <x:c r="S16" s="64" t="str">
+        <x:v>tb1.氏名</x:v>
+      </x:c>
+      <x:c r="T16" s="65"/>
+      <x:c r="U16" s="65"/>
+      <x:c r="V16" s="65"/>
+      <x:c r="W16" s="65"/>
+      <x:c r="X16" s="65"/>
+      <x:c r="Y16" s="65"/>
+      <x:c r="Z16" s="65"/>
+      <x:c r="AA16" s="65"/>
+      <x:c r="AB16" s="65"/>
+      <x:c r="AC16" s="65"/>
+      <x:c r="AD16" s="65"/>
+      <x:c r="AE16" s="65"/>
+      <x:c r="AF16" s="65"/>
+      <x:c r="AG16" s="65"/>
+      <x:c r="AH16" s="65"/>
+      <x:c r="AI16" s="65"/>
+      <x:c r="AJ16" s="65"/>
+      <x:c r="AK16" s="64"/>
+      <x:c r="AL16" s="65"/>
+      <x:c r="AM16" s="65"/>
+      <x:c r="AN16" s="65"/>
+      <x:c r="AO16" s="65"/>
+      <x:c r="AP16" s="65"/>
+      <x:c r="AQ16" s="65"/>
+      <x:c r="AR16" s="65"/>
+      <x:c r="AS16" s="65"/>
+      <x:c r="AT16" s="65"/>
+      <x:c r="AU16" s="65"/>
+      <x:c r="AV16" s="65"/>
+      <x:c r="AW16" s="65"/>
+      <x:c r="AX16" s="65"/>
+      <x:c r="AY16" s="65"/>
+      <x:c r="AZ16" s="65"/>
+      <x:c r="BA16" s="65"/>
+      <x:c r="BB16" s="65"/>
+      <x:c r="BC16" s="65"/>
+      <x:c r="BD16" s="65"/>
+      <x:c r="BE16" s="65"/>
+      <x:c r="BF16" s="65"/>
+      <x:c r="BG16" s="65"/>
+      <x:c r="BH16" s="65"/>
+      <x:c r="BI16" s="65"/>
+      <x:c r="BJ16" s="65"/>
+      <x:c r="BK16" s="65"/>
+      <x:c r="BL16" s="65"/>
+      <x:c r="BM16" s="65"/>
+      <x:c r="BN16" s="65"/>
+      <x:c r="BO16" s="65"/>
+      <x:c r="BP16" s="65"/>
+      <x:c r="BQ16" s="65"/>
+      <x:c r="BR16" s="65"/>
+      <x:c r="BS16" s="65"/>
+      <x:c r="BT16" s="65"/>
+      <x:c r="BU16" s="65"/>
+      <x:c r="BV16" s="65"/>
+      <x:c r="BW16" s="65"/>
+      <x:c r="BX16" s="65"/>
+      <x:c r="BY16" s="65"/>
+      <x:c r="BZ16" s="65"/>
+      <x:c r="CA16" s="65"/>
+      <x:c r="CB16" s="65"/>
+      <x:c r="CC16" s="65"/>
+      <x:c r="CD16" s="65"/>
+      <x:c r="CE16" s="65"/>
+      <x:c r="CF16" s="65"/>
+      <x:c r="CG16" s="65"/>
+      <x:c r="CH16" s="65"/>
+      <x:c r="CI16" s="65"/>
+      <x:c r="CJ16" s="65"/>
+      <x:c r="CK16" s="65"/>
+      <x:c r="CL16" s="66"/>
+    </x:row>
+    <x:row r="17" ht="13.5" customHeight="1">
+      <x:c r="A17" s="63" t="str">
+        <x:v>＜移送パターン2＞</x:v>
+      </x:c>
+      <x:c r="B17" s="63"/>
+      <x:c r="C17" s="63"/>
+      <x:c r="D17" s="63"/>
+      <x:c r="E17" s="63"/>
+      <x:c r="F17" s="63"/>
+      <x:c r="G17" s="63"/>
+      <x:c r="H17" s="63"/>
+      <x:c r="I17" s="63"/>
+      <x:c r="J17" s="63"/>
+      <x:c r="K17" s="63"/>
+      <x:c r="L17" s="63"/>
+      <x:c r="M17" s="63"/>
+      <x:c r="N17" s="63"/>
+      <x:c r="O17" s="63"/>
+      <x:c r="P17" s="63"/>
+      <x:c r="Q17" s="63"/>
+      <x:c r="R17" s="63"/>
+      <x:c r="S17" s="63"/>
+      <x:c r="T17" s="63"/>
+      <x:c r="U17" s="63"/>
+      <x:c r="V17" s="63"/>
+      <x:c r="W17" s="63"/>
+      <x:c r="X17" s="63"/>
+      <x:c r="Y17" s="63"/>
+      <x:c r="Z17" s="63"/>
+      <x:c r="AA17" s="63"/>
+      <x:c r="AB17" s="63"/>
+      <x:c r="AC17" s="63"/>
+      <x:c r="AD17" s="63"/>
+      <x:c r="AE17" s="63"/>
+      <x:c r="AF17" s="63"/>
+      <x:c r="AG17" s="63"/>
+      <x:c r="AH17" s="63"/>
+      <x:c r="AI17" s="63"/>
+      <x:c r="AJ17" s="63"/>
+      <x:c r="AK17" s="63"/>
+      <x:c r="AL17" s="63"/>
+      <x:c r="AM17" s="63"/>
+      <x:c r="AN17" s="63"/>
+      <x:c r="AO17" s="63"/>
+      <x:c r="AP17" s="63"/>
+      <x:c r="AQ17" s="63"/>
+      <x:c r="AR17" s="63"/>
+      <x:c r="AS17" s="63"/>
+      <x:c r="AT17" s="63"/>
+      <x:c r="AU17" s="63"/>
+      <x:c r="AV17" s="63"/>
+      <x:c r="AW17" s="63"/>
+      <x:c r="AX17" s="63"/>
+      <x:c r="AY17" s="63"/>
+      <x:c r="AZ17" s="63"/>
+      <x:c r="BA17" s="63"/>
+      <x:c r="BB17" s="63"/>
+      <x:c r="BC17" s="63"/>
+      <x:c r="BD17" s="63"/>
+      <x:c r="BE17" s="63"/>
+      <x:c r="BF17" s="63"/>
+      <x:c r="BG17" s="63"/>
+      <x:c r="BH17" s="63"/>
+      <x:c r="BI17" s="63"/>
+      <x:c r="BJ17" s="63"/>
+      <x:c r="BK17" s="63"/>
+      <x:c r="BL17" s="63"/>
+      <x:c r="BM17" s="63"/>
+      <x:c r="BN17" s="63"/>
+      <x:c r="BO17" s="63"/>
+      <x:c r="BP17" s="63"/>
+      <x:c r="BQ17" s="63"/>
+      <x:c r="BR17" s="63"/>
+      <x:c r="BS17" s="63"/>
+      <x:c r="BT17" s="63"/>
+      <x:c r="BU17" s="63"/>
+      <x:c r="BV17" s="63"/>
+      <x:c r="BW17" s="63"/>
+      <x:c r="BX17" s="63"/>
+      <x:c r="BY17" s="63"/>
+      <x:c r="BZ17" s="63"/>
+      <x:c r="CA17" s="63"/>
+      <x:c r="CB17" s="63"/>
+      <x:c r="CC17" s="63"/>
+      <x:c r="CD17" s="63"/>
+      <x:c r="CE17" s="63"/>
+      <x:c r="CF17" s="63"/>
+      <x:c r="CG17" s="63"/>
+      <x:c r="CH17" s="63"/>
+      <x:c r="CI17" s="63"/>
+      <x:c r="CJ17" s="63"/>
+      <x:c r="CK17" s="63"/>
+      <x:c r="CL17" s="63"/>
+    </x:row>
+    <x:row r="18" ht="13.5" customHeight="1">
+      <x:c r="A18" s="67" t="str">
+        <x:v>項目</x:v>
+      </x:c>
+      <x:c r="B18" s="68"/>
+      <x:c r="C18" s="68"/>
+      <x:c r="D18" s="68"/>
+      <x:c r="E18" s="68"/>
+      <x:c r="F18" s="68"/>
+      <x:c r="G18" s="68"/>
+      <x:c r="H18" s="68"/>
+      <x:c r="I18" s="68"/>
+      <x:c r="J18" s="68"/>
+      <x:c r="K18" s="68"/>
+      <x:c r="L18" s="68"/>
+      <x:c r="M18" s="68"/>
+      <x:c r="N18" s="68"/>
+      <x:c r="O18" s="68"/>
+      <x:c r="P18" s="68"/>
+      <x:c r="Q18" s="68"/>
+      <x:c r="R18" s="68"/>
+      <x:c r="S18" s="67" t="str">
+        <x:v>移送元</x:v>
+      </x:c>
+      <x:c r="T18" s="68"/>
+      <x:c r="U18" s="68"/>
+      <x:c r="V18" s="68"/>
+      <x:c r="W18" s="68"/>
+      <x:c r="X18" s="68"/>
+      <x:c r="Y18" s="68"/>
+      <x:c r="Z18" s="68"/>
+      <x:c r="AA18" s="68"/>
+      <x:c r="AB18" s="68"/>
+      <x:c r="AC18" s="68"/>
+      <x:c r="AD18" s="68"/>
+      <x:c r="AE18" s="68"/>
+      <x:c r="AF18" s="68"/>
+      <x:c r="AG18" s="68"/>
+      <x:c r="AH18" s="68"/>
+      <x:c r="AI18" s="68"/>
+      <x:c r="AJ18" s="68"/>
+      <x:c r="AK18" s="67" t="str">
+        <x:v>移送方法ほか</x:v>
+      </x:c>
+      <x:c r="AL18" s="68"/>
+      <x:c r="AM18" s="68"/>
+      <x:c r="AN18" s="68"/>
+      <x:c r="AO18" s="68"/>
+      <x:c r="AP18" s="68"/>
+      <x:c r="AQ18" s="68"/>
+      <x:c r="AR18" s="68"/>
+      <x:c r="AS18" s="68"/>
+      <x:c r="AT18" s="68"/>
+      <x:c r="AU18" s="68"/>
+      <x:c r="AV18" s="68"/>
+      <x:c r="AW18" s="68"/>
+      <x:c r="AX18" s="68"/>
+      <x:c r="AY18" s="68"/>
+      <x:c r="AZ18" s="68"/>
+      <x:c r="BA18" s="68"/>
+      <x:c r="BB18" s="68"/>
+      <x:c r="BC18" s="68"/>
+      <x:c r="BD18" s="68"/>
+      <x:c r="BE18" s="68"/>
+      <x:c r="BF18" s="68"/>
+      <x:c r="BG18" s="68"/>
+      <x:c r="BH18" s="68"/>
+      <x:c r="BI18" s="68"/>
+      <x:c r="BJ18" s="68"/>
+      <x:c r="BK18" s="68"/>
+      <x:c r="BL18" s="68"/>
+      <x:c r="BM18" s="68"/>
+      <x:c r="BN18" s="68"/>
+      <x:c r="BO18" s="68"/>
+      <x:c r="BP18" s="68"/>
+      <x:c r="BQ18" s="68"/>
+      <x:c r="BR18" s="68"/>
+      <x:c r="BS18" s="68"/>
+      <x:c r="BT18" s="68"/>
+      <x:c r="BU18" s="68"/>
+      <x:c r="BV18" s="68"/>
+      <x:c r="BW18" s="68"/>
+      <x:c r="BX18" s="68"/>
+      <x:c r="BY18" s="68"/>
+      <x:c r="BZ18" s="68"/>
+      <x:c r="CA18" s="68"/>
+      <x:c r="CB18" s="68"/>
+      <x:c r="CC18" s="68"/>
+      <x:c r="CD18" s="68"/>
+      <x:c r="CE18" s="68"/>
+      <x:c r="CF18" s="68"/>
+      <x:c r="CG18" s="68"/>
+      <x:c r="CH18" s="68"/>
+      <x:c r="CI18" s="68"/>
+      <x:c r="CJ18" s="68"/>
+      <x:c r="CK18" s="68"/>
+      <x:c r="CL18" s="69"/>
+    </x:row>
+    <x:row r="19" ht="13.5" customHeight="1">
+      <x:c r="A19" s="64" t="str">
+        <x:v>ユーザーID</x:v>
+      </x:c>
+      <x:c r="B19" s="65"/>
+      <x:c r="C19" s="65"/>
+      <x:c r="D19" s="65"/>
+      <x:c r="E19" s="65"/>
+      <x:c r="F19" s="65"/>
+      <x:c r="G19" s="65"/>
+      <x:c r="H19" s="65"/>
+      <x:c r="I19" s="65"/>
+      <x:c r="J19" s="65"/>
+      <x:c r="K19" s="65"/>
+      <x:c r="L19" s="65"/>
+      <x:c r="M19" s="65"/>
+      <x:c r="N19" s="65"/>
+      <x:c r="O19" s="65"/>
+      <x:c r="P19" s="65"/>
+      <x:c r="Q19" s="65"/>
+      <x:c r="R19" s="65"/>
+      <x:c r="S19" s="64" t="str">
+        <x:v>tb2.ユーザーID</x:v>
+      </x:c>
+      <x:c r="T19" s="65"/>
+      <x:c r="U19" s="65"/>
+      <x:c r="V19" s="65"/>
+      <x:c r="W19" s="65"/>
+      <x:c r="X19" s="65"/>
+      <x:c r="Y19" s="65"/>
+      <x:c r="Z19" s="65"/>
+      <x:c r="AA19" s="65"/>
+      <x:c r="AB19" s="65"/>
+      <x:c r="AC19" s="65"/>
+      <x:c r="AD19" s="65"/>
+      <x:c r="AE19" s="65"/>
+      <x:c r="AF19" s="65"/>
+      <x:c r="AG19" s="65"/>
+      <x:c r="AH19" s="65"/>
+      <x:c r="AI19" s="65"/>
+      <x:c r="AJ19" s="65"/>
+      <x:c r="AK19" s="64"/>
+      <x:c r="AL19" s="65"/>
+      <x:c r="AM19" s="65"/>
+      <x:c r="AN19" s="65"/>
+      <x:c r="AO19" s="65"/>
+      <x:c r="AP19" s="65"/>
+      <x:c r="AQ19" s="65"/>
+      <x:c r="AR19" s="65"/>
+      <x:c r="AS19" s="65"/>
+      <x:c r="AT19" s="65"/>
+      <x:c r="AU19" s="65"/>
+      <x:c r="AV19" s="65"/>
+      <x:c r="AW19" s="65"/>
+      <x:c r="AX19" s="65"/>
+      <x:c r="AY19" s="65"/>
+      <x:c r="AZ19" s="65"/>
+      <x:c r="BA19" s="65"/>
+      <x:c r="BB19" s="65"/>
+      <x:c r="BC19" s="65"/>
+      <x:c r="BD19" s="65"/>
+      <x:c r="BE19" s="65"/>
+      <x:c r="BF19" s="65"/>
+      <x:c r="BG19" s="65"/>
+      <x:c r="BH19" s="65"/>
+      <x:c r="BI19" s="65"/>
+      <x:c r="BJ19" s="65"/>
+      <x:c r="BK19" s="65"/>
+      <x:c r="BL19" s="65"/>
+      <x:c r="BM19" s="65"/>
+      <x:c r="BN19" s="65"/>
+      <x:c r="BO19" s="65"/>
+      <x:c r="BP19" s="65"/>
+      <x:c r="BQ19" s="65"/>
+      <x:c r="BR19" s="65"/>
+      <x:c r="BS19" s="65"/>
+      <x:c r="BT19" s="65"/>
+      <x:c r="BU19" s="65"/>
+      <x:c r="BV19" s="65"/>
+      <x:c r="BW19" s="65"/>
+      <x:c r="BX19" s="65"/>
+      <x:c r="BY19" s="65"/>
+      <x:c r="BZ19" s="65"/>
+      <x:c r="CA19" s="65"/>
+      <x:c r="CB19" s="65"/>
+      <x:c r="CC19" s="65"/>
+      <x:c r="CD19" s="65"/>
+      <x:c r="CE19" s="65"/>
+      <x:c r="CF19" s="65"/>
+      <x:c r="CG19" s="65"/>
+      <x:c r="CH19" s="65"/>
+      <x:c r="CI19" s="65"/>
+      <x:c r="CJ19" s="65"/>
+      <x:c r="CK19" s="65"/>
+      <x:c r="CL19" s="66"/>
+    </x:row>
+    <x:row r="20" ht="13.5" customHeight="1">
+      <x:c r="A20" s="64" t="str">
+        <x:v>氏名</x:v>
+      </x:c>
+      <x:c r="B20" s="65"/>
+      <x:c r="C20" s="65"/>
+      <x:c r="D20" s="65"/>
+      <x:c r="E20" s="65"/>
+      <x:c r="F20" s="65"/>
+      <x:c r="G20" s="65"/>
+      <x:c r="H20" s="65"/>
+      <x:c r="I20" s="65"/>
+      <x:c r="J20" s="65"/>
+      <x:c r="K20" s="65"/>
+      <x:c r="L20" s="65"/>
+      <x:c r="M20" s="65"/>
+      <x:c r="N20" s="65"/>
+      <x:c r="O20" s="65"/>
+      <x:c r="P20" s="65"/>
+      <x:c r="Q20" s="65"/>
+      <x:c r="R20" s="65"/>
+      <x:c r="S20" s="64" t="str">
+        <x:v>tb2.氏名</x:v>
+      </x:c>
+      <x:c r="T20" s="65"/>
+      <x:c r="U20" s="65"/>
+      <x:c r="V20" s="65"/>
+      <x:c r="W20" s="65"/>
+      <x:c r="X20" s="65"/>
+      <x:c r="Y20" s="65"/>
+      <x:c r="Z20" s="65"/>
+      <x:c r="AA20" s="65"/>
+      <x:c r="AB20" s="65"/>
+      <x:c r="AC20" s="65"/>
+      <x:c r="AD20" s="65"/>
+      <x:c r="AE20" s="65"/>
+      <x:c r="AF20" s="65"/>
+      <x:c r="AG20" s="65"/>
+      <x:c r="AH20" s="65"/>
+      <x:c r="AI20" s="65"/>
+      <x:c r="AJ20" s="65"/>
+      <x:c r="AK20" s="64" t="str">
+        <x:v>TRIM(tb2.氏名)</x:v>
+      </x:c>
+      <x:c r="AL20" s="65"/>
+      <x:c r="AM20" s="65"/>
+      <x:c r="AN20" s="65"/>
+      <x:c r="AO20" s="65"/>
+      <x:c r="AP20" s="65"/>
+      <x:c r="AQ20" s="65"/>
+      <x:c r="AR20" s="65"/>
+      <x:c r="AS20" s="65"/>
+      <x:c r="AT20" s="65"/>
+      <x:c r="AU20" s="65"/>
+      <x:c r="AV20" s="65"/>
+      <x:c r="AW20" s="65"/>
+      <x:c r="AX20" s="65"/>
+      <x:c r="AY20" s="65"/>
+      <x:c r="AZ20" s="65"/>
+      <x:c r="BA20" s="65"/>
+      <x:c r="BB20" s="65"/>
+      <x:c r="BC20" s="65"/>
+      <x:c r="BD20" s="65"/>
+      <x:c r="BE20" s="65"/>
+      <x:c r="BF20" s="65"/>
+      <x:c r="BG20" s="65"/>
+      <x:c r="BH20" s="65"/>
+      <x:c r="BI20" s="65"/>
+      <x:c r="BJ20" s="65"/>
+      <x:c r="BK20" s="65"/>
+      <x:c r="BL20" s="65"/>
+      <x:c r="BM20" s="65"/>
+      <x:c r="BN20" s="65"/>
+      <x:c r="BO20" s="65"/>
+      <x:c r="BP20" s="65"/>
+      <x:c r="BQ20" s="65"/>
+      <x:c r="BR20" s="65"/>
+      <x:c r="BS20" s="65"/>
+      <x:c r="BT20" s="65"/>
+      <x:c r="BU20" s="65"/>
+      <x:c r="BV20" s="65"/>
+      <x:c r="BW20" s="65"/>
+      <x:c r="BX20" s="65"/>
+      <x:c r="BY20" s="65"/>
+      <x:c r="BZ20" s="65"/>
+      <x:c r="CA20" s="65"/>
+      <x:c r="CB20" s="65"/>
+      <x:c r="CC20" s="65"/>
+      <x:c r="CD20" s="65"/>
+      <x:c r="CE20" s="65"/>
+      <x:c r="CF20" s="65"/>
+      <x:c r="CG20" s="65"/>
+      <x:c r="CH20" s="65"/>
+      <x:c r="CI20" s="65"/>
+      <x:c r="CJ20" s="65"/>
+      <x:c r="CK20" s="65"/>
+      <x:c r="CL20" s="66"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="18.75"/>

</xml_diff>

<commit_message>
test: prepare multi-row values review
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -2,83 +2,83 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-001" sheetId="1" r:id="Re8cc6367cadb468a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-002" sheetId="2" r:id="Ra6aa173c11874eb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-003" sheetId="3" r:id="R23e05e832a2a438a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-004" sheetId="4" r:id="R2616ba582a6e4841"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-005" sheetId="5" r:id="Rbc92f1e6e7644664"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-006" sheetId="6" r:id="R2e631fa6f52d423e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-007" sheetId="7" r:id="R986d4677c6e44f6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-008" sheetId="8" r:id="R472bb021b2db4cba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-009" sheetId="9" r:id="Refe46be8114d43b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-010" sheetId="10" r:id="Rcaf93847564a4387"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-011" sheetId="11" r:id="Rdad09afbbbc74623"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-012" sheetId="12" r:id="R0304d5b240a54f42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-013" sheetId="13" r:id="R8c54992a7ea441c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-014" sheetId="14" r:id="Rc4b33685c09f475d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-015" sheetId="15" r:id="R5f39288d505646ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-016" sheetId="16" r:id="R11262d4b28be4b40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-017" sheetId="17" r:id="R5a01a5f9243d494b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-018" sheetId="18" r:id="R0a60f39ac92a4a56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-019" sheetId="19" r:id="R8fa0ac62ef564e7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-020" sheetId="20" r:id="Rb377f18f40fe4b2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-021" sheetId="21" r:id="Ra11c8e652aa14b58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-022" sheetId="22" r:id="R4a0d1453be10482a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-023" sheetId="23" r:id="Rb057381b703b43c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-024" sheetId="24" r:id="Rfe321699ea5844eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-025" sheetId="25" r:id="Rca2d57cdcbe54574"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-026" sheetId="26" r:id="Rc9db76e7a35643e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-027" sheetId="37" r:id="R035cc205f3d14b73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-028" sheetId="27" r:id="R55076a7ba6cb4055"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-029" sheetId="28" r:id="R33a4b540b75c46b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-030" sheetId="29" r:id="R6a503962d13d4275"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-031" sheetId="30" r:id="Reaac6f884c6e42df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-032" sheetId="31" r:id="Re69a66039c2e409c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-033" sheetId="32" r:id="R99c7c9f75a944263"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-034" sheetId="33" r:id="R59364af4d96043f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-035" sheetId="34" r:id="R53cadddf077e46ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-036" sheetId="35" r:id="Rde5bb3591ddd455a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-037" sheetId="36" r:id="R35a2919a124a4a13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-038" sheetId="38" r:id="Rbff6ad4955fb4c59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-039" sheetId="39" r:id="Rdb69d605facf420e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-040" sheetId="40" r:id="R3302bffc83144cf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-041" sheetId="41" r:id="R5f5c6ccb29ea49f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-042" sheetId="42" r:id="Rc3d9b4703ed94668"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-043" sheetId="43" r:id="R9183cb0150a946e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-044" sheetId="44" r:id="R89b1dc9cd22e4aef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-045" sheetId="79" r:id="Rc9cf75528e484873"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-046" sheetId="46" r:id="R77785c467db64945"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-047" sheetId="47" r:id="Re39a1a30735346c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-048" sheetId="52" r:id="R65e9133444df44de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-049" sheetId="53" r:id="Rdd1766288b1f4dcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-050" sheetId="54" r:id="Rf42d273e22ff490a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-051" sheetId="55" r:id="Rb33a6bd3d0f04069"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-052" sheetId="56" r:id="R36b5b8ad13724277"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-053" sheetId="57" r:id="R9979a20fe4e149fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-054" sheetId="48" r:id="Rd1e6d4cbb9664e76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-055" sheetId="49" r:id="R821e284697674be1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-056" sheetId="80" r:id="R87ce4183a7484df8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-057" sheetId="70" r:id="Rbe03d408ec744837"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-058" sheetId="58" r:id="R256e5caa22b84021"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-059" sheetId="81" r:id="R85dc8864325c4b24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-060" sheetId="63" r:id="R89f12f6e5d6e44d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-061" sheetId="82" r:id="Rd6b55f3f1eee4d81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-062" sheetId="64" r:id="R9cd29edbb17a4ce3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-063" sheetId="65" r:id="R475e57af146b417e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-064" sheetId="66" r:id="Re22d909f1fb44e71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-065" sheetId="67" r:id="R40c8922c57504637"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-066" sheetId="68" r:id="Rab29bdc5e7b34de0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-067" sheetId="69" r:id="R999e183a7e854126"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-068" sheetId="71" r:id="R1761ed956e204f4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-069" sheetId="72" r:id="R0a366b6f4fa44d9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-070" sheetId="73" r:id="R356224734e154655"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-071" sheetId="74" r:id="R3229cd251ebe4521"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-072" sheetId="75" r:id="Rc58a887196df43bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-073" sheetId="76" r:id="R2d45fe446db34f18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-074" sheetId="77" r:id="R004f3ea88c1244eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-075" sheetId="78" r:id="Ra18cfac5e9e04c59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-076" sheetId="83" r:id="R2e377d9fd4ae46f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-077" sheetId="84" r:id="R263556a746c14d4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-001" sheetId="1" r:id="R9a3c72fe510349f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-002" sheetId="2" r:id="Rbd68a8ddf9cf4d43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-003" sheetId="3" r:id="R26131e583edf4edc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-004" sheetId="4" r:id="R01e64dd6897e434f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-005" sheetId="5" r:id="Rb8a15a2d31934d77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-006" sheetId="6" r:id="R2fc714ff7b9e4d4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-007" sheetId="7" r:id="Rc3dc5580ecd747ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-008" sheetId="8" r:id="Rb14ac55f6e754f0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-009" sheetId="9" r:id="Rd0d8870214a5467d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-010" sheetId="10" r:id="R405a7df310da4d7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-011" sheetId="11" r:id="R3cfd31e430994335"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-012" sheetId="12" r:id="R13d80575052e4aae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-013" sheetId="13" r:id="Rb4b2b16023db4a69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-014" sheetId="14" r:id="Rc7a6a14d9cd4400c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-015" sheetId="15" r:id="R74fadf2888be4ad4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-016" sheetId="16" r:id="Rc4da3ba197da4216"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-017" sheetId="17" r:id="Rab36d4c42e1c4479"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-018" sheetId="18" r:id="R98c0fe2c070b47e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-019" sheetId="19" r:id="R326c7f2a74cc4a48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-020" sheetId="20" r:id="R6553ea0916e44aa2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-021" sheetId="21" r:id="R2a28a074ad2b47f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-022" sheetId="22" r:id="R7410f15be64140d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-023" sheetId="23" r:id="R6d5236d039f143af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-024" sheetId="24" r:id="Ra58b974b87cf4012"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-025" sheetId="25" r:id="R07ead86467814665"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-026" sheetId="26" r:id="Re273ef39273b4f90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-027" sheetId="37" r:id="R55b8380377394dfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-028" sheetId="27" r:id="R4d16118ff8894869"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-029" sheetId="28" r:id="Rfebc73d61db04b78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-030" sheetId="29" r:id="R2d061f03386742a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-031" sheetId="30" r:id="R42691e9a79c845d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-032" sheetId="31" r:id="R23a67d319c7c41a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-033" sheetId="32" r:id="Rfaed17a08e424eef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-034" sheetId="33" r:id="R555039ebc0544e16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-035" sheetId="34" r:id="R9cb86b7f67b548d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-036" sheetId="35" r:id="Rb6c1c078c60b4637"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-037" sheetId="36" r:id="R26679a23f39140e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-038" sheetId="38" r:id="Rd0405493324d4c63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-039" sheetId="39" r:id="R0c51a96f2a3e49d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-040" sheetId="40" r:id="R1809880b2c7c4ce3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-041" sheetId="41" r:id="R12adccc5e7a94d0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-042" sheetId="42" r:id="R2c98cc8831c943b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-043" sheetId="43" r:id="Rb5d01d69898447c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-044" sheetId="44" r:id="R4c654ea08fbe4467"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-045" sheetId="79" r:id="R252455d78b114f76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-046" sheetId="46" r:id="Reb4230c3f19a4678"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-047" sheetId="47" r:id="R3ae0589fd14f4135"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-048" sheetId="52" r:id="R774b8312d51c47ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-049" sheetId="53" r:id="R60defacbc4544a10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-050" sheetId="54" r:id="R6945e4dee5b14414"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-051" sheetId="55" r:id="Ra4ceb2e1e3994350"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-052" sheetId="56" r:id="R5e6a10b91cf740ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-053" sheetId="57" r:id="R534d206a58864c39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-054" sheetId="48" r:id="R45d525b9b26941dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-055" sheetId="49" r:id="R07627f2add4d4060"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-056" sheetId="80" r:id="R2e1f630281764883"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-057" sheetId="70" r:id="Rc4bca0c438aa4558"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-058" sheetId="58" r:id="R6f6cad21c916484e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-059" sheetId="81" r:id="Rc3419242a77d4864"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-060" sheetId="63" r:id="Reaf0de7e274c4f0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-061" sheetId="82" r:id="R7c35bd5968ab4fea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-062" sheetId="64" r:id="R3db1aeb5f97b4cc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-063" sheetId="65" r:id="R1155d01d80c54f6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-064" sheetId="66" r:id="Rda0c59118f7f4b03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-065" sheetId="67" r:id="Rddcd7a65e24e4db4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-066" sheetId="68" r:id="Rd0db0ce5e71d41e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-067" sheetId="69" r:id="R8c9d32dfa9854d03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-068" sheetId="71" r:id="Reef7aefee0ff41d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-069" sheetId="72" r:id="R2e9c3ef4949f497b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-070" sheetId="73" r:id="Rb1aca84580b04767"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-071" sheetId="74" r:id="Rb40fcb718f904a89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-072" sheetId="75" r:id="R0f2c00cb8aa74f07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-073" sheetId="76" r:id="R349c03244cc4462b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-074" sheetId="77" r:id="R703ba4934d674b24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-075" sheetId="78" r:id="Rf3afd4b4d6f04b52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-076" sheetId="83" r:id="R5d62a0f718ef40f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-077" sheetId="84" r:id="R1a710b1dcaa24b50"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -54048,6 +54048,96 @@
   <x:sheetFormatPr defaultRowHeight="18.75"/>
   <x:cols>
     <x:col min="1" max="90" width="1.125" customWidth="1"/>
+    <x:col min="1" max="1" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="33" max="33" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="35" max="35" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="36" max="36" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="37" max="37" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="38" max="38" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="39" max="39" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="40" max="40" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="41" max="41" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="42" max="42" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="43" max="43" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="44" max="44" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="45" max="45" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="46" max="46" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="47" max="47" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="48" max="48" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="49" max="49" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="50" max="50" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="51" max="51" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="52" max="52" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="53" max="53" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="54" max="54" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="55" max="55" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="56" max="56" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="57" max="57" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="58" max="58" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="59" max="59" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="60" max="60" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="61" max="61" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="62" max="62" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="63" max="63" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="64" max="64" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="65" max="65" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="66" max="66" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="67" max="67" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="68" max="68" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="69" max="69" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="70" max="70" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="71" max="71" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="72" max="72" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="73" max="73" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="74" max="74" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="75" max="75" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="76" max="76" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="77" max="77" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="78" max="78" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="79" max="79" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="80" max="80" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="81" max="81" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="82" max="82" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="83" max="83" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="84" max="84" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="85" max="85" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="86" max="86" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="87" max="87" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="88" max="88" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="89" max="89" width="1.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="90" max="90" width="1.7799999713897705" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="13.5" customHeight="1">
@@ -54757,8 +54847,8 @@
       <x:c r="AH8" s="48"/>
       <x:c r="AI8" s="48"/>
       <x:c r="AJ8" s="48"/>
-      <x:c r="AK8" s="47" t="s">
-        <x:v>210</x:v>
+      <x:c r="AK8" s="47" t="str">
+        <x:v>sysdatetime()</x:v>
       </x:c>
       <x:c r="AL8" s="48"/>
       <x:c r="AM8" s="48"/>
@@ -55333,8 +55423,8 @@
       <x:c r="AH14" s="48"/>
       <x:c r="AI14" s="48"/>
       <x:c r="AJ14" s="48"/>
-      <x:c r="AK14" s="47" t="s">
-        <x:v>210</x:v>
+      <x:c r="AK14" s="47" t="str">
+        <x:v>sysdatetime()</x:v>
       </x:c>
       <x:c r="AL14" s="48"/>
       <x:c r="AM14" s="48"/>

</xml_diff>

<commit_message>
feat: indent wrapped CASE branches
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -2,83 +2,83 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-001" sheetId="1" r:id="R9a3c72fe510349f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-002" sheetId="2" r:id="Rbd68a8ddf9cf4d43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-003" sheetId="3" r:id="R26131e583edf4edc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-004" sheetId="4" r:id="R01e64dd6897e434f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-005" sheetId="5" r:id="Rb8a15a2d31934d77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-006" sheetId="6" r:id="R2fc714ff7b9e4d4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-007" sheetId="7" r:id="Rc3dc5580ecd747ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-008" sheetId="8" r:id="Rb14ac55f6e754f0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-009" sheetId="9" r:id="Rd0d8870214a5467d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-010" sheetId="10" r:id="R405a7df310da4d7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-011" sheetId="11" r:id="R3cfd31e430994335"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-012" sheetId="12" r:id="R13d80575052e4aae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-013" sheetId="13" r:id="Rb4b2b16023db4a69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-014" sheetId="14" r:id="Rc7a6a14d9cd4400c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-015" sheetId="15" r:id="R74fadf2888be4ad4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-016" sheetId="16" r:id="Rc4da3ba197da4216"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-017" sheetId="17" r:id="Rab36d4c42e1c4479"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-018" sheetId="18" r:id="R98c0fe2c070b47e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-019" sheetId="19" r:id="R326c7f2a74cc4a48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-020" sheetId="20" r:id="R6553ea0916e44aa2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-021" sheetId="21" r:id="R2a28a074ad2b47f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-022" sheetId="22" r:id="R7410f15be64140d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-023" sheetId="23" r:id="R6d5236d039f143af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-024" sheetId="24" r:id="Ra58b974b87cf4012"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-025" sheetId="25" r:id="R07ead86467814665"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-026" sheetId="26" r:id="Re273ef39273b4f90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-027" sheetId="37" r:id="R55b8380377394dfa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-028" sheetId="27" r:id="R4d16118ff8894869"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-029" sheetId="28" r:id="Rfebc73d61db04b78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-030" sheetId="29" r:id="R2d061f03386742a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-031" sheetId="30" r:id="R42691e9a79c845d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-032" sheetId="31" r:id="R23a67d319c7c41a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-033" sheetId="32" r:id="Rfaed17a08e424eef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-034" sheetId="33" r:id="R555039ebc0544e16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-035" sheetId="34" r:id="R9cb86b7f67b548d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-036" sheetId="35" r:id="Rb6c1c078c60b4637"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-037" sheetId="36" r:id="R26679a23f39140e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-038" sheetId="38" r:id="Rd0405493324d4c63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-039" sheetId="39" r:id="R0c51a96f2a3e49d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-040" sheetId="40" r:id="R1809880b2c7c4ce3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-041" sheetId="41" r:id="R12adccc5e7a94d0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-042" sheetId="42" r:id="R2c98cc8831c943b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-043" sheetId="43" r:id="Rb5d01d69898447c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-044" sheetId="44" r:id="R4c654ea08fbe4467"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-045" sheetId="79" r:id="R252455d78b114f76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-046" sheetId="46" r:id="Reb4230c3f19a4678"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-047" sheetId="47" r:id="R3ae0589fd14f4135"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-048" sheetId="52" r:id="R774b8312d51c47ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-049" sheetId="53" r:id="R60defacbc4544a10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-050" sheetId="54" r:id="R6945e4dee5b14414"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-051" sheetId="55" r:id="Ra4ceb2e1e3994350"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-052" sheetId="56" r:id="R5e6a10b91cf740ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-053" sheetId="57" r:id="R534d206a58864c39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-054" sheetId="48" r:id="R45d525b9b26941dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-055" sheetId="49" r:id="R07627f2add4d4060"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-056" sheetId="80" r:id="R2e1f630281764883"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-057" sheetId="70" r:id="Rc4bca0c438aa4558"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-058" sheetId="58" r:id="R6f6cad21c916484e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-059" sheetId="81" r:id="Rc3419242a77d4864"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-060" sheetId="63" r:id="Reaf0de7e274c4f0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-061" sheetId="82" r:id="R7c35bd5968ab4fea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-062" sheetId="64" r:id="R3db1aeb5f97b4cc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-063" sheetId="65" r:id="R1155d01d80c54f6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-064" sheetId="66" r:id="Rda0c59118f7f4b03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-065" sheetId="67" r:id="Rddcd7a65e24e4db4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-066" sheetId="68" r:id="Rd0db0ce5e71d41e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-067" sheetId="69" r:id="R8c9d32dfa9854d03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-068" sheetId="71" r:id="Reef7aefee0ff41d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-069" sheetId="72" r:id="R2e9c3ef4949f497b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-070" sheetId="73" r:id="Rb1aca84580b04767"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-071" sheetId="74" r:id="Rb40fcb718f904a89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-072" sheetId="75" r:id="R0f2c00cb8aa74f07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-073" sheetId="76" r:id="R349c03244cc4462b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-074" sheetId="77" r:id="R703ba4934d674b24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-075" sheetId="78" r:id="Rf3afd4b4d6f04b52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-076" sheetId="83" r:id="R5d62a0f718ef40f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-077" sheetId="84" r:id="R1a710b1dcaa24b50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-001" sheetId="1" r:id="R5ac6ee9dea4049a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-002" sheetId="2" r:id="R1570402777444de0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-003" sheetId="3" r:id="R41c9174116374ae6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-004" sheetId="4" r:id="Re7287cbde13b40b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-005" sheetId="5" r:id="Rf1d15fb3e8604b37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-006" sheetId="6" r:id="R53829ea2763241e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-007" sheetId="7" r:id="Ra8188803b0a44d1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-008" sheetId="8" r:id="Rb963d823aa354895"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-009" sheetId="9" r:id="Rdb89ab54a7774087"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-010" sheetId="10" r:id="R445af00ae8304936"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-011" sheetId="11" r:id="R6b448e30b24a4bd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-012" sheetId="12" r:id="R51e637c660874e9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-013" sheetId="13" r:id="R2a3cfa0e081d4b79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-014" sheetId="14" r:id="R20c554476c364641"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-015" sheetId="15" r:id="R22eaf1ad707548dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-016" sheetId="16" r:id="Ra173fe00f43745f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-017" sheetId="17" r:id="R75a7a3d7d46d4d08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-018" sheetId="18" r:id="R4a1856fc6f124863"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-019" sheetId="19" r:id="R68b9571a41b54d8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-020" sheetId="20" r:id="Rf5e0170efa764c83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-021" sheetId="21" r:id="Rb78723b2dfb14f42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-022" sheetId="22" r:id="Rcdf4396827bf402e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-023" sheetId="23" r:id="R1985ea16733d48be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-024" sheetId="24" r:id="Rbe9565a8dd9f4da4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-025" sheetId="25" r:id="R0622895cac8a448f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-026" sheetId="26" r:id="Re2e2c9e3ba964b1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-027" sheetId="37" r:id="Rb4b79c5caa8545ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-028" sheetId="27" r:id="R26427d819c69409f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-029" sheetId="28" r:id="R946df934b5734d1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-030" sheetId="29" r:id="Re6840d35190b4581"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-031" sheetId="30" r:id="R8a1d0bae797a4f0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-032" sheetId="31" r:id="R0ae673cff2784bff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-033" sheetId="32" r:id="Rd2fde10bc981447d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-034" sheetId="33" r:id="R7cf0f838e7d8458e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-035" sheetId="34" r:id="Rff8da4f088fc4b21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-036" sheetId="35" r:id="Rd2346e8a9bda42a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-037" sheetId="36" r:id="R4119695518324c26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-038" sheetId="38" r:id="R15f23eed87dd4a9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-039" sheetId="39" r:id="Rd7c684e238494d37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-040" sheetId="40" r:id="R4fa22b298173441c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-041" sheetId="41" r:id="R497f172770664164"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-042" sheetId="42" r:id="R45b2bb06bacc445e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-043" sheetId="43" r:id="Rc258212773204660"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-044" sheetId="44" r:id="R16fcf4f6c7a74c5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-045" sheetId="79" r:id="Rebbe24f0c8354383"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-046" sheetId="46" r:id="R6c550a786252408c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-047" sheetId="47" r:id="Rfa0c0d21c6174f64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-048" sheetId="52" r:id="Rb33e43c82a7842fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-049" sheetId="53" r:id="Rdb470caf969a4761"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-050" sheetId="54" r:id="R99ff1006973e4e0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-051" sheetId="55" r:id="R7a6f71da426440a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-052" sheetId="56" r:id="Reec2f3c2fb1b4aac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-053" sheetId="57" r:id="Rc3a3573a31db4970"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-054" sheetId="48" r:id="R37a1f027f70342f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-055" sheetId="49" r:id="R371c2f56127242a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-056" sheetId="80" r:id="Rd1ec9a1c9549407c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-057" sheetId="70" r:id="Rcdca889dae1e411b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-058" sheetId="58" r:id="R3a7c7b0416d349e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-059" sheetId="81" r:id="R032af493c823445c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-060" sheetId="63" r:id="R6a44e30dba4e4cca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-061" sheetId="82" r:id="Rd6485057f8884a04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-062" sheetId="64" r:id="Rf465cab306aa4a96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-063" sheetId="65" r:id="R0598d3543bea4523"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-064" sheetId="66" r:id="R1cca7fc0449f45f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-065" sheetId="67" r:id="Red26f875eb0d4efa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-066" sheetId="68" r:id="R98ee0211990740a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-067" sheetId="69" r:id="R3c868d21562044a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-068" sheetId="71" r:id="R2b96090d5a654060"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-069" sheetId="72" r:id="Rdc7655904dc54913"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-070" sheetId="73" r:id="R3d2ea641fd964486"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-071" sheetId="74" r:id="R40f0fc95c4324002"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-072" sheetId="75" r:id="R24d7a228e14048b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-073" sheetId="76" r:id="R04691cf5f7544434"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-074" sheetId="77" r:id="Rff6493560e374680"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-075" sheetId="78" r:id="Reaf9d7e0f9144044"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-076" sheetId="83" r:id="R343e8efca9c9441e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-077" sheetId="84" r:id="R26a1267f0ff24047"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -878,9 +878,6 @@
     <x:t xml:space="preserve">SUM(CASE結果)</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">tb1.状態 = 'PAID' → tb1.金額</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">user_status</x:t>
   </x:si>
   <x:si>
@@ -49646,15 +49643,15 @@
         <x:v>263</x:v>
       </x:c>
       <x:c r="AG3" s="6"/>
-      <x:c r="AH3" s="25" t="s">
-        <x:v>264</x:v>
-      </x:c>
+      <x:c r="AH3" s="25"/>
       <x:c r="AI3" s="6"/>
       <x:c r="AJ3" s="6"/>
       <x:c r="AK3" s="6"/>
       <x:c r="AL3" s="6"/>
       <x:c r="AM3" s="6"/>
-      <x:c r="AN3" s="6"/>
+      <x:c r="AN3" s="6" t="str">
+        <x:v>tb1.状態 = 'PAID' → tb1.金額</x:v>
+      </x:c>
       <x:c r="AO3" s="6"/>
       <x:c r="AP3" s="6"/>
       <x:c r="AQ3" s="6"/>
@@ -49740,15 +49737,15 @@
       <x:c r="AE4" s="14"/>
       <x:c r="AF4" s="14"/>
       <x:c r="AG4" s="14"/>
-      <x:c r="AH4" s="30" t="s">
-        <x:v>226</x:v>
-      </x:c>
+      <x:c r="AH4" s="30"/>
       <x:c r="AI4" s="14"/>
       <x:c r="AJ4" s="14"/>
       <x:c r="AK4" s="14"/>
       <x:c r="AL4" s="14"/>
       <x:c r="AM4" s="14"/>
-      <x:c r="AN4" s="14"/>
+      <x:c r="AN4" s="14" t="str">
+        <x:v>ELSE → 0</x:v>
+      </x:c>
       <x:c r="AO4" s="14"/>
       <x:c r="AP4" s="14"/>
       <x:c r="AQ4" s="14"/>
@@ -50024,7 +50021,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>265</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -50043,7 +50040,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF3" s="25" t="s">
-        <x:v>266</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="AG3" s="6"/>
       <x:c r="AH3" s="6"/>
@@ -50137,7 +50134,7 @@
       <x:c r="AD4" s="3"/>
       <x:c r="AE4" s="3"/>
       <x:c r="AF4" s="27" t="s">
-        <x:v>267</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="AG4" s="3"/>
       <x:c r="AH4" s="3"/>
@@ -50233,7 +50230,7 @@
       <x:c r="AF5" s="14"/>
       <x:c r="AG5" s="14"/>
       <x:c r="AH5" s="30" t="s">
-        <x:v>268</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="AI5" s="14"/>
       <x:c r="AJ5" s="14"/>
@@ -51202,7 +51199,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>269</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -51223,7 +51220,7 @@
       <x:c r="AF3" s="6"/>
       <x:c r="AG3" s="6"/>
       <x:c r="AH3" s="25" t="s">
-        <x:v>270</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="AI3" s="6"/>
       <x:c r="AJ3" s="6"/>
@@ -51319,7 +51316,7 @@
       </x:c>
       <x:c r="AG4" s="3"/>
       <x:c r="AH4" s="27" t="s">
-        <x:v>271</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="AI4" s="3"/>
       <x:c r="AJ4" s="3"/>
@@ -51927,7 +51924,7 @@
       </x:c>
       <x:c r="BA5" s="3"/>
       <x:c r="BB5" s="27" t="s">
-        <x:v>272</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="BC5" s="3"/>
       <x:c r="BD5" s="3"/>
@@ -52019,7 +52016,7 @@
       <x:c r="AX6" s="14"/>
       <x:c r="AY6" s="14"/>
       <x:c r="AZ6" s="30" t="s">
-        <x:v>273</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="BA6" s="14"/>
       <x:c r="BB6" s="14"/>
@@ -52417,7 +52414,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AZ4" s="25" t="s">
-        <x:v>274</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="BA4" s="6"/>
       <x:c r="BB4" s="6"/>
@@ -52511,7 +52508,7 @@
       <x:c r="AX5" s="14"/>
       <x:c r="AY5" s="14"/>
       <x:c r="AZ5" s="30" t="s">
-        <x:v>273</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="BA5" s="14"/>
       <x:c r="BB5" s="14"/>
@@ -52776,7 +52773,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>275</x:v>
+        <x:v>274</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -52870,7 +52867,7 @@
       <x:c r="O4" s="3"/>
       <x:c r="P4" s="3"/>
       <x:c r="Q4" s="27" t="s">
-        <x:v>276</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="R4" s="3"/>
       <x:c r="S4" s="3"/>
@@ -53256,7 +53253,7 @@
       <x:c r="E3" s="4"/>
       <x:c r="F3" s="4"/>
       <x:c r="G3" s="24" t="s">
-        <x:v>277</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="H3" s="6"/>
       <x:c r="I3" s="6"/>
@@ -53270,7 +53267,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>278</x:v>
+        <x:v>277</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -53883,7 +53880,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF3" s="25" t="s">
-        <x:v>279</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="AG3" s="6"/>
       <x:c r="AH3" s="6"/>
@@ -54330,7 +54327,7 @@
     </x:row>
     <x:row r="3" ht="13.5" customHeight="1">
       <x:c r="A3" s="61" t="s">
-        <x:v>280</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="B3" s="61"/>
       <x:c r="C3" s="61"/>
@@ -54560,7 +54557,7 @@
       <x:c r="AI5" s="48"/>
       <x:c r="AJ5" s="48"/>
       <x:c r="AK5" s="47" t="s">
-        <x:v>281</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="AL5" s="48"/>
       <x:c r="AM5" s="48"/>
@@ -54656,7 +54653,7 @@
       <x:c r="AI6" s="48"/>
       <x:c r="AJ6" s="48"/>
       <x:c r="AK6" s="47" t="s">
-        <x:v>282</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="AL6" s="48"/>
       <x:c r="AM6" s="48"/>
@@ -54906,7 +54903,7 @@
     </x:row>
     <x:row r="9" ht="13.5" customHeight="1">
       <x:c r="A9" s="46" t="s">
-        <x:v>283</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="B9" s="46"/>
       <x:c r="C9" s="46"/>
@@ -55136,7 +55133,7 @@
       <x:c r="AI11" s="48"/>
       <x:c r="AJ11" s="48"/>
       <x:c r="AK11" s="47" t="s">
-        <x:v>284</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="AL11" s="48"/>
       <x:c r="AM11" s="48"/>
@@ -55232,7 +55229,7 @@
       <x:c r="AI12" s="48"/>
       <x:c r="AJ12" s="48"/>
       <x:c r="AK12" s="47" t="s">
-        <x:v>285</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="AL12" s="48"/>
       <x:c r="AM12" s="48"/>
@@ -55328,7 +55325,7 @@
       <x:c r="AI13" s="48"/>
       <x:c r="AJ13" s="48"/>
       <x:c r="AK13" s="47" t="s">
-        <x:v>286</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="AL13" s="48"/>
       <x:c r="AM13" s="48"/>
@@ -56066,7 +56063,7 @@
     </x:row>
     <x:row r="6" ht="13.5" customHeight="1">
       <x:c r="A6" s="46" t="s">
-        <x:v>287</x:v>
+        <x:v>286</x:v>
       </x:c>
       <x:c r="B6" s="46"/>
       <x:c r="C6" s="46"/>
@@ -56280,7 +56277,7 @@
       </x:c>
       <x:c r="P8" s="45"/>
       <x:c r="Q8" s="45" t="s">
-        <x:v>288</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="R8" s="45"/>
       <x:c r="S8" s="45"/>
@@ -56376,7 +56373,7 @@
       <x:c r="O9" s="48"/>
       <x:c r="P9" s="48"/>
       <x:c r="Q9" s="48" t="s">
-        <x:v>289</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="R9" s="48"/>
       <x:c r="S9" s="48"/>
@@ -56734,7 +56731,7 @@
     </x:row>
     <x:row r="13" ht="13.5" customHeight="1">
       <x:c r="A13" s="62" t="s">
-        <x:v>290</x:v>
+        <x:v>289</x:v>
       </x:c>
       <x:c r="B13" s="61"/>
       <x:c r="C13" s="61"/>
@@ -57118,7 +57115,7 @@
     </x:row>
     <x:row r="17" ht="13.5" customHeight="1">
       <x:c r="A17" s="46" t="s">
-        <x:v>291</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="B17" s="48"/>
       <x:c r="C17" s="48"/>
@@ -57446,7 +57443,7 @@
       <x:c r="AI20" s="48"/>
       <x:c r="AJ20" s="48"/>
       <x:c r="AK20" s="47" t="s">
-        <x:v>288</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="AL20" s="48"/>
       <x:c r="AM20" s="48"/>

</xml_diff>

<commit_message>
test: add aliased aggregate CASE review case
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Macro\SqlAnalyzerFormatter-feature\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AAF14E3-8ECA-4AB8-BCEB-D4608EDA8EAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7EBA3E4-76E4-4AF4-8B8D-C58F33777A57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -91,13 +91,14 @@
     <sheet name="SEL-076" sheetId="83" r:id="rId76"/>
     <sheet name="SEL-077" sheetId="84" r:id="rId77"/>
     <sheet name="SEL-078" sheetId="85" r:id="rId78"/>
+    <sheet name="SEL-079" sheetId="86" r:id="rId79"/>
   </sheets>
   <calcPr calcId="0" calcMode="manual"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1361" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1376" uniqueCount="298">
   <si>
     <t>＜DB入出力項目定義＞</t>
   </si>
@@ -891,6 +892,9 @@
     <t>SUM(CASE結果)</t>
   </si>
   <si>
+    <t>tb1.状態 = 'PAID' → tb1.金額</t>
+  </si>
+  <si>
     <t>user_status</t>
   </si>
   <si>
@@ -972,9 +976,6 @@
     <t>＜移送パターン2＞</t>
   </si>
   <si>
-    <t>tb1.状態 = 'PAID' → tb1.金額</t>
-  </si>
-  <si>
     <t>net_amount</t>
   </si>
   <si>
@@ -988,6 +989,9 @@
   </si>
   <si>
     <t>tb1.状態 = 'REFUND' → tb1.金額</t>
+  </si>
+  <si>
+    <t>refund_amount</t>
   </si>
 </sst>
 </file>
@@ -1014,7 +1018,7 @@
       <charset val="128"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1039,6 +1043,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2CEEF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2CEEF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -1272,7 +1286,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1510,6 +1524,51 @@
     <xf numFmtId="49" fontId="1" fillId="7" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="8" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="8" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="8" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="9" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -50026,7 +50085,7 @@
       <c r="AL3" s="6"/>
       <c r="AM3" s="6"/>
       <c r="AN3" s="6" t="s">
-        <v>291</v>
+        <v>264</v>
       </c>
       <c r="AO3" s="6"/>
       <c r="AP3" s="6"/>
@@ -50400,7 +50459,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -50419,7 +50478,7 @@
         <v>33</v>
       </c>
       <c r="AF3" s="25" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="AG3" s="6"/>
       <c r="AH3" s="6"/>
@@ -50513,7 +50572,7 @@
       <c r="AD4" s="3"/>
       <c r="AE4" s="3"/>
       <c r="AF4" s="27" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
@@ -50609,7 +50668,7 @@
       <c r="AF5" s="14"/>
       <c r="AG5" s="14"/>
       <c r="AH5" s="30" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="AI5" s="14"/>
       <c r="AJ5" s="14"/>
@@ -51584,7 +51643,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -51605,7 +51664,7 @@
       <c r="AF3" s="6"/>
       <c r="AG3" s="6"/>
       <c r="AH3" s="25" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="AI3" s="6"/>
       <c r="AJ3" s="6"/>
@@ -51701,7 +51760,7 @@
       </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="27" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="AI4" s="3"/>
       <c r="AJ4" s="3"/>
@@ -52312,7 +52371,7 @@
       </c>
       <c r="BA5" s="3"/>
       <c r="BB5" s="27" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="BC5" s="3"/>
       <c r="BD5" s="3"/>
@@ -52404,7 +52463,7 @@
       <c r="AX6" s="14"/>
       <c r="AY6" s="14"/>
       <c r="AZ6" s="30" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="BA6" s="14"/>
       <c r="BB6" s="14"/>
@@ -52805,7 +52864,7 @@
         <v>33</v>
       </c>
       <c r="AZ4" s="25" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="BA4" s="6"/>
       <c r="BB4" s="6"/>
@@ -52899,7 +52958,7 @@
       <c r="AX5" s="14"/>
       <c r="AY5" s="14"/>
       <c r="AZ5" s="30" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="BA5" s="14"/>
       <c r="BB5" s="14"/>
@@ -53167,7 +53226,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -53261,7 +53320,7 @@
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="27" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
@@ -53650,7 +53709,7 @@
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="24" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
@@ -53664,7 +53723,7 @@
       </c>
       <c r="P3" s="6"/>
       <c r="Q3" s="25" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -54280,7 +54339,7 @@
         <v>33</v>
       </c>
       <c r="AF3" s="25" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="AG3" s="6"/>
       <c r="AH3" s="6"/>
@@ -54640,7 +54699,7 @@
     </row>
     <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="61" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B3" s="61"/>
       <c r="C3" s="61"/>
@@ -54870,7 +54929,7 @@
       <c r="AI5" s="48"/>
       <c r="AJ5" s="48"/>
       <c r="AK5" s="47" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="AL5" s="48"/>
       <c r="AM5" s="48"/>
@@ -54966,7 +55025,7 @@
       <c r="AI6" s="48"/>
       <c r="AJ6" s="48"/>
       <c r="AK6" s="47" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="AL6" s="48"/>
       <c r="AM6" s="48"/>
@@ -55216,7 +55275,7 @@
     </row>
     <row r="9" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="46" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B9" s="46"/>
       <c r="C9" s="46"/>
@@ -55446,7 +55505,7 @@
       <c r="AI11" s="48"/>
       <c r="AJ11" s="48"/>
       <c r="AK11" s="47" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="AL11" s="48"/>
       <c r="AM11" s="48"/>
@@ -55542,7 +55601,7 @@
       <c r="AI12" s="48"/>
       <c r="AJ12" s="48"/>
       <c r="AK12" s="47" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="AL12" s="48"/>
       <c r="AM12" s="48"/>
@@ -55638,7 +55697,7 @@
       <c r="AI13" s="48"/>
       <c r="AJ13" s="48"/>
       <c r="AK13" s="47" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="AL13" s="48"/>
       <c r="AM13" s="48"/>
@@ -56289,7 +56348,7 @@
     </row>
     <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="46" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B6" s="46"/>
       <c r="C6" s="46"/>
@@ -56503,7 +56562,7 @@
       </c>
       <c r="P8" s="45"/>
       <c r="Q8" s="45" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="R8" s="45"/>
       <c r="S8" s="45"/>
@@ -56599,7 +56658,7 @@
       <c r="O9" s="48"/>
       <c r="P9" s="48"/>
       <c r="Q9" s="48" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="R9" s="48"/>
       <c r="S9" s="48"/>
@@ -56957,7 +57016,7 @@
     </row>
     <row r="13" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="62" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -57341,7 +57400,7 @@
     </row>
     <row r="17" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="46" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B17" s="48"/>
       <c r="C17" s="48"/>
@@ -57669,7 +57728,7 @@
       <c r="AI20" s="48"/>
       <c r="AJ20" s="48"/>
       <c r="AK20" s="47" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="AL20" s="48"/>
       <c r="AM20" s="48"/>
@@ -57995,7 +58054,7 @@
       <c r="AX3" s="67"/>
       <c r="AY3" s="67"/>
       <c r="AZ3" s="67" t="s">
-        <v>291</v>
+        <v>264</v>
       </c>
       <c r="BA3" s="67"/>
       <c r="BB3" s="67"/>
@@ -58326,6 +58385,603 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-4E00-000000000000}">
+  <sheetPr codeName="Sheet79"/>
+  <dimension ref="A1:CL6"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="90" width="1.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="22" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
+      <c r="Q1" s="22"/>
+      <c r="R1" s="22"/>
+      <c r="S1" s="22"/>
+      <c r="T1" s="22"/>
+      <c r="U1" s="22"/>
+      <c r="V1" s="22"/>
+      <c r="W1" s="22"/>
+      <c r="X1" s="22"/>
+      <c r="Y1" s="22"/>
+      <c r="Z1" s="22"/>
+      <c r="AA1" s="22"/>
+      <c r="AB1" s="22"/>
+      <c r="AC1" s="22"/>
+      <c r="AD1" s="22"/>
+      <c r="AE1" s="22"/>
+      <c r="AF1" s="22"/>
+      <c r="AG1" s="22"/>
+      <c r="AH1" s="22"/>
+      <c r="AI1" s="22"/>
+      <c r="AJ1" s="22"/>
+      <c r="AK1" s="22"/>
+      <c r="AL1" s="22"/>
+      <c r="AM1" s="22"/>
+      <c r="AN1" s="22"/>
+      <c r="AO1" s="22"/>
+      <c r="AP1" s="22"/>
+      <c r="AQ1" s="22"/>
+      <c r="AR1" s="22"/>
+      <c r="AS1" s="22"/>
+      <c r="AT1" s="22"/>
+      <c r="AU1" s="22"/>
+      <c r="AV1" s="22"/>
+      <c r="AW1" s="22"/>
+      <c r="AX1" s="22"/>
+      <c r="AY1" s="22"/>
+      <c r="AZ1" s="22"/>
+      <c r="BA1" s="22"/>
+      <c r="BB1" s="22"/>
+      <c r="BC1" s="22"/>
+      <c r="BD1" s="22"/>
+      <c r="BE1" s="22"/>
+      <c r="BF1" s="22"/>
+      <c r="BG1" s="22"/>
+      <c r="BH1" s="22"/>
+      <c r="BI1" s="22"/>
+      <c r="BJ1" s="22"/>
+      <c r="BK1" s="22"/>
+      <c r="BL1" s="22"/>
+      <c r="BM1" s="22"/>
+      <c r="BN1" s="22"/>
+      <c r="BO1" s="22"/>
+      <c r="BP1" s="22"/>
+      <c r="BQ1" s="22"/>
+      <c r="BR1" s="22"/>
+      <c r="BS1" s="22"/>
+      <c r="BT1" s="22"/>
+      <c r="BU1" s="22"/>
+      <c r="BV1" s="22"/>
+      <c r="BW1" s="22"/>
+      <c r="BX1" s="22"/>
+      <c r="BY1" s="22"/>
+      <c r="BZ1" s="22"/>
+      <c r="CA1" s="22"/>
+      <c r="CB1" s="22"/>
+      <c r="CC1" s="22"/>
+      <c r="CD1" s="22"/>
+      <c r="CE1" s="22"/>
+      <c r="CF1" s="22"/>
+      <c r="CG1" s="22"/>
+      <c r="CH1" s="22"/>
+      <c r="CI1" s="22"/>
+      <c r="CJ1" s="22"/>
+      <c r="CK1" s="22"/>
+      <c r="CL1" s="22"/>
+    </row>
+    <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="63" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
+      <c r="K2" s="63"/>
+      <c r="L2" s="63"/>
+      <c r="M2" s="63"/>
+      <c r="N2" s="63"/>
+      <c r="O2" s="63"/>
+      <c r="P2" s="63"/>
+      <c r="Q2" s="63"/>
+      <c r="R2" s="63"/>
+      <c r="S2" s="63"/>
+      <c r="T2" s="63"/>
+      <c r="U2" s="63"/>
+      <c r="V2" s="63"/>
+      <c r="W2" s="63"/>
+      <c r="X2" s="63"/>
+      <c r="Y2" s="63"/>
+      <c r="Z2" s="63"/>
+      <c r="AA2" s="63"/>
+      <c r="AB2" s="63"/>
+      <c r="AC2" s="63"/>
+      <c r="AD2" s="63"/>
+      <c r="AE2" s="63"/>
+      <c r="AF2" s="63"/>
+      <c r="AG2" s="63"/>
+      <c r="AH2" s="63"/>
+      <c r="AI2" s="63"/>
+      <c r="AJ2" s="63"/>
+      <c r="AK2" s="63"/>
+      <c r="AL2" s="63"/>
+      <c r="AM2" s="63"/>
+      <c r="AN2" s="63"/>
+      <c r="AO2" s="63"/>
+      <c r="AP2" s="63"/>
+      <c r="AQ2" s="63"/>
+      <c r="AR2" s="63"/>
+      <c r="AS2" s="63"/>
+      <c r="AT2" s="63"/>
+      <c r="AU2" s="63"/>
+      <c r="AV2" s="63"/>
+      <c r="AW2" s="63"/>
+      <c r="AX2" s="63"/>
+      <c r="AY2" s="63"/>
+      <c r="AZ2" s="63"/>
+      <c r="BA2" s="63"/>
+      <c r="BB2" s="63"/>
+      <c r="BC2" s="63"/>
+      <c r="BD2" s="63"/>
+      <c r="BE2" s="63"/>
+      <c r="BF2" s="63"/>
+      <c r="BG2" s="63"/>
+      <c r="BH2" s="63"/>
+      <c r="BI2" s="63"/>
+      <c r="BJ2" s="63"/>
+      <c r="BK2" s="63"/>
+      <c r="BL2" s="63"/>
+      <c r="BM2" s="63"/>
+      <c r="BN2" s="63"/>
+      <c r="BO2" s="63"/>
+      <c r="BP2" s="63"/>
+      <c r="BQ2" s="63"/>
+      <c r="BR2" s="63"/>
+      <c r="BS2" s="63"/>
+      <c r="BT2" s="63"/>
+      <c r="BU2" s="63"/>
+      <c r="BV2" s="63"/>
+      <c r="BW2" s="63"/>
+      <c r="BX2" s="63"/>
+      <c r="BY2" s="63"/>
+      <c r="BZ2" s="63"/>
+      <c r="CA2" s="63"/>
+      <c r="CB2" s="63"/>
+      <c r="CC2" s="63"/>
+      <c r="CD2" s="63"/>
+      <c r="CE2" s="63"/>
+      <c r="CF2" s="63"/>
+      <c r="CG2" s="63"/>
+      <c r="CH2" s="63"/>
+      <c r="CI2" s="63"/>
+      <c r="CJ2" s="63"/>
+      <c r="CK2" s="63"/>
+      <c r="CL2" s="63"/>
+    </row>
+    <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="79" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="80"/>
+      <c r="C3" s="80"/>
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="81" t="s">
+        <v>3</v>
+      </c>
+      <c r="H3" s="82"/>
+      <c r="I3" s="82"/>
+      <c r="J3" s="82"/>
+      <c r="K3" s="82"/>
+      <c r="L3" s="82"/>
+      <c r="M3" s="82"/>
+      <c r="N3" s="82"/>
+      <c r="O3" s="82" t="s">
+        <v>4</v>
+      </c>
+      <c r="P3" s="82"/>
+      <c r="Q3" s="82" t="s">
+        <v>262</v>
+      </c>
+      <c r="R3" s="82"/>
+      <c r="S3" s="82"/>
+      <c r="T3" s="82"/>
+      <c r="U3" s="82"/>
+      <c r="V3" s="82"/>
+      <c r="W3" s="82"/>
+      <c r="X3" s="82"/>
+      <c r="Y3" s="82"/>
+      <c r="Z3" s="82"/>
+      <c r="AA3" s="82"/>
+      <c r="AB3" s="82"/>
+      <c r="AC3" s="82"/>
+      <c r="AD3" s="82"/>
+      <c r="AE3" s="82" t="s">
+        <v>33</v>
+      </c>
+      <c r="AF3" s="82" t="s">
+        <v>264</v>
+      </c>
+      <c r="AG3" s="82"/>
+      <c r="AH3" s="82"/>
+      <c r="AI3" s="82"/>
+      <c r="AJ3" s="82"/>
+      <c r="AK3" s="82"/>
+      <c r="AL3" s="82"/>
+      <c r="AM3" s="82"/>
+      <c r="AN3" s="82"/>
+      <c r="AO3" s="82"/>
+      <c r="AP3" s="82"/>
+      <c r="AQ3" s="82"/>
+      <c r="AR3" s="82"/>
+      <c r="AS3" s="82"/>
+      <c r="AT3" s="82"/>
+      <c r="AU3" s="82"/>
+      <c r="AV3" s="82"/>
+      <c r="AW3" s="82"/>
+      <c r="AX3" s="82"/>
+      <c r="AY3" s="82"/>
+      <c r="AZ3" s="82"/>
+      <c r="BA3" s="82"/>
+      <c r="BB3" s="82"/>
+      <c r="BC3" s="82"/>
+      <c r="BD3" s="82"/>
+      <c r="BE3" s="82"/>
+      <c r="BF3" s="82"/>
+      <c r="BG3" s="82"/>
+      <c r="BH3" s="82"/>
+      <c r="BI3" s="82"/>
+      <c r="BJ3" s="82"/>
+      <c r="BK3" s="82"/>
+      <c r="BL3" s="82"/>
+      <c r="BM3" s="82"/>
+      <c r="BN3" s="82"/>
+      <c r="BO3" s="82"/>
+      <c r="BP3" s="82"/>
+      <c r="BQ3" s="82"/>
+      <c r="BR3" s="82"/>
+      <c r="BS3" s="82"/>
+      <c r="BT3" s="82"/>
+      <c r="BU3" s="82"/>
+      <c r="BV3" s="82"/>
+      <c r="BW3" s="82"/>
+      <c r="BX3" s="82"/>
+      <c r="BY3" s="82"/>
+      <c r="BZ3" s="82"/>
+      <c r="CA3" s="82"/>
+      <c r="CB3" s="82"/>
+      <c r="CC3" s="82"/>
+      <c r="CD3" s="82"/>
+      <c r="CE3" s="82"/>
+      <c r="CF3" s="82"/>
+      <c r="CG3" s="82"/>
+      <c r="CH3" s="82"/>
+      <c r="CI3" s="82"/>
+      <c r="CJ3" s="82"/>
+      <c r="CK3" s="82"/>
+      <c r="CL3" s="83"/>
+    </row>
+    <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="84"/>
+      <c r="B4" s="85"/>
+      <c r="C4" s="85"/>
+      <c r="D4" s="85"/>
+      <c r="E4" s="85"/>
+      <c r="F4" s="85"/>
+      <c r="G4" s="86"/>
+      <c r="H4" s="87"/>
+      <c r="I4" s="87"/>
+      <c r="J4" s="87"/>
+      <c r="K4" s="87"/>
+      <c r="L4" s="87"/>
+      <c r="M4" s="87"/>
+      <c r="N4" s="87"/>
+      <c r="O4" s="87"/>
+      <c r="P4" s="87"/>
+      <c r="Q4" s="87"/>
+      <c r="R4" s="87"/>
+      <c r="S4" s="87"/>
+      <c r="T4" s="87"/>
+      <c r="U4" s="87"/>
+      <c r="V4" s="87"/>
+      <c r="W4" s="87"/>
+      <c r="X4" s="87"/>
+      <c r="Y4" s="87"/>
+      <c r="Z4" s="87"/>
+      <c r="AA4" s="87"/>
+      <c r="AB4" s="87"/>
+      <c r="AC4" s="87"/>
+      <c r="AD4" s="87"/>
+      <c r="AE4" s="87"/>
+      <c r="AF4" s="87" t="s">
+        <v>226</v>
+      </c>
+      <c r="AG4" s="87"/>
+      <c r="AH4" s="87"/>
+      <c r="AI4" s="87"/>
+      <c r="AJ4" s="87"/>
+      <c r="AK4" s="87"/>
+      <c r="AL4" s="87"/>
+      <c r="AM4" s="87"/>
+      <c r="AN4" s="87"/>
+      <c r="AO4" s="87"/>
+      <c r="AP4" s="87"/>
+      <c r="AQ4" s="87"/>
+      <c r="AR4" s="87"/>
+      <c r="AS4" s="87"/>
+      <c r="AT4" s="87"/>
+      <c r="AU4" s="87"/>
+      <c r="AV4" s="87"/>
+      <c r="AW4" s="87"/>
+      <c r="AX4" s="87"/>
+      <c r="AY4" s="87"/>
+      <c r="AZ4" s="87"/>
+      <c r="BA4" s="87"/>
+      <c r="BB4" s="87"/>
+      <c r="BC4" s="87"/>
+      <c r="BD4" s="87"/>
+      <c r="BE4" s="87"/>
+      <c r="BF4" s="87"/>
+      <c r="BG4" s="87"/>
+      <c r="BH4" s="87"/>
+      <c r="BI4" s="87"/>
+      <c r="BJ4" s="87"/>
+      <c r="BK4" s="87"/>
+      <c r="BL4" s="87"/>
+      <c r="BM4" s="87"/>
+      <c r="BN4" s="87"/>
+      <c r="BO4" s="87"/>
+      <c r="BP4" s="87"/>
+      <c r="BQ4" s="87"/>
+      <c r="BR4" s="87"/>
+      <c r="BS4" s="87"/>
+      <c r="BT4" s="87"/>
+      <c r="BU4" s="87"/>
+      <c r="BV4" s="87"/>
+      <c r="BW4" s="87"/>
+      <c r="BX4" s="87"/>
+      <c r="BY4" s="87"/>
+      <c r="BZ4" s="87"/>
+      <c r="CA4" s="87"/>
+      <c r="CB4" s="87"/>
+      <c r="CC4" s="87"/>
+      <c r="CD4" s="87"/>
+      <c r="CE4" s="87"/>
+      <c r="CF4" s="87"/>
+      <c r="CG4" s="87"/>
+      <c r="CH4" s="87"/>
+      <c r="CI4" s="87"/>
+      <c r="CJ4" s="87"/>
+      <c r="CK4" s="87"/>
+      <c r="CL4" s="88"/>
+    </row>
+    <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="84"/>
+      <c r="B5" s="85"/>
+      <c r="C5" s="85"/>
+      <c r="D5" s="85"/>
+      <c r="E5" s="85"/>
+      <c r="F5" s="85"/>
+      <c r="G5" s="86" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5" s="87"/>
+      <c r="I5" s="87"/>
+      <c r="J5" s="87"/>
+      <c r="K5" s="87"/>
+      <c r="L5" s="87"/>
+      <c r="M5" s="87"/>
+      <c r="N5" s="87"/>
+      <c r="O5" s="87" t="s">
+        <v>4</v>
+      </c>
+      <c r="P5" s="87"/>
+      <c r="Q5" s="87" t="s">
+        <v>297</v>
+      </c>
+      <c r="R5" s="87"/>
+      <c r="S5" s="87"/>
+      <c r="T5" s="87"/>
+      <c r="U5" s="87"/>
+      <c r="V5" s="87"/>
+      <c r="W5" s="87"/>
+      <c r="X5" s="87"/>
+      <c r="Y5" s="87"/>
+      <c r="Z5" s="87"/>
+      <c r="AA5" s="87"/>
+      <c r="AB5" s="87"/>
+      <c r="AC5" s="87"/>
+      <c r="AD5" s="87"/>
+      <c r="AE5" s="87" t="s">
+        <v>33</v>
+      </c>
+      <c r="AF5" s="87" t="s">
+        <v>296</v>
+      </c>
+      <c r="AG5" s="87"/>
+      <c r="AH5" s="87"/>
+      <c r="AI5" s="87"/>
+      <c r="AJ5" s="87"/>
+      <c r="AK5" s="87"/>
+      <c r="AL5" s="87"/>
+      <c r="AM5" s="87"/>
+      <c r="AN5" s="87"/>
+      <c r="AO5" s="87"/>
+      <c r="AP5" s="87"/>
+      <c r="AQ5" s="87"/>
+      <c r="AR5" s="87"/>
+      <c r="AS5" s="87"/>
+      <c r="AT5" s="87"/>
+      <c r="AU5" s="87"/>
+      <c r="AV5" s="87"/>
+      <c r="AW5" s="87"/>
+      <c r="AX5" s="87"/>
+      <c r="AY5" s="87"/>
+      <c r="AZ5" s="87"/>
+      <c r="BA5" s="87"/>
+      <c r="BB5" s="87"/>
+      <c r="BC5" s="87"/>
+      <c r="BD5" s="87"/>
+      <c r="BE5" s="87"/>
+      <c r="BF5" s="87"/>
+      <c r="BG5" s="87"/>
+      <c r="BH5" s="87"/>
+      <c r="BI5" s="87"/>
+      <c r="BJ5" s="87"/>
+      <c r="BK5" s="87"/>
+      <c r="BL5" s="87"/>
+      <c r="BM5" s="87"/>
+      <c r="BN5" s="87"/>
+      <c r="BO5" s="87"/>
+      <c r="BP5" s="87"/>
+      <c r="BQ5" s="87"/>
+      <c r="BR5" s="87"/>
+      <c r="BS5" s="87"/>
+      <c r="BT5" s="87"/>
+      <c r="BU5" s="87"/>
+      <c r="BV5" s="87"/>
+      <c r="BW5" s="87"/>
+      <c r="BX5" s="87"/>
+      <c r="BY5" s="87"/>
+      <c r="BZ5" s="87"/>
+      <c r="CA5" s="87"/>
+      <c r="CB5" s="87"/>
+      <c r="CC5" s="87"/>
+      <c r="CD5" s="87"/>
+      <c r="CE5" s="87"/>
+      <c r="CF5" s="87"/>
+      <c r="CG5" s="87"/>
+      <c r="CH5" s="87"/>
+      <c r="CI5" s="87"/>
+      <c r="CJ5" s="87"/>
+      <c r="CK5" s="87"/>
+      <c r="CL5" s="88"/>
+    </row>
+    <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="89"/>
+      <c r="B6" s="90"/>
+      <c r="C6" s="90"/>
+      <c r="D6" s="90"/>
+      <c r="E6" s="90"/>
+      <c r="F6" s="90"/>
+      <c r="G6" s="91"/>
+      <c r="H6" s="92"/>
+      <c r="I6" s="92"/>
+      <c r="J6" s="92"/>
+      <c r="K6" s="92"/>
+      <c r="L6" s="92"/>
+      <c r="M6" s="92"/>
+      <c r="N6" s="92"/>
+      <c r="O6" s="92"/>
+      <c r="P6" s="92"/>
+      <c r="Q6" s="92"/>
+      <c r="R6" s="92"/>
+      <c r="S6" s="92"/>
+      <c r="T6" s="92"/>
+      <c r="U6" s="92"/>
+      <c r="V6" s="92"/>
+      <c r="W6" s="92"/>
+      <c r="X6" s="92"/>
+      <c r="Y6" s="92"/>
+      <c r="Z6" s="92"/>
+      <c r="AA6" s="92"/>
+      <c r="AB6" s="92"/>
+      <c r="AC6" s="92"/>
+      <c r="AD6" s="92"/>
+      <c r="AE6" s="92"/>
+      <c r="AF6" s="92" t="s">
+        <v>226</v>
+      </c>
+      <c r="AG6" s="92"/>
+      <c r="AH6" s="92"/>
+      <c r="AI6" s="92"/>
+      <c r="AJ6" s="92"/>
+      <c r="AK6" s="92"/>
+      <c r="AL6" s="92"/>
+      <c r="AM6" s="92"/>
+      <c r="AN6" s="92"/>
+      <c r="AO6" s="92"/>
+      <c r="AP6" s="92"/>
+      <c r="AQ6" s="92"/>
+      <c r="AR6" s="92"/>
+      <c r="AS6" s="92"/>
+      <c r="AT6" s="92"/>
+      <c r="AU6" s="92"/>
+      <c r="AV6" s="92"/>
+      <c r="AW6" s="92"/>
+      <c r="AX6" s="92"/>
+      <c r="AY6" s="92"/>
+      <c r="AZ6" s="92"/>
+      <c r="BA6" s="92"/>
+      <c r="BB6" s="92"/>
+      <c r="BC6" s="92"/>
+      <c r="BD6" s="92"/>
+      <c r="BE6" s="92"/>
+      <c r="BF6" s="92"/>
+      <c r="BG6" s="92"/>
+      <c r="BH6" s="92"/>
+      <c r="BI6" s="92"/>
+      <c r="BJ6" s="92"/>
+      <c r="BK6" s="92"/>
+      <c r="BL6" s="92"/>
+      <c r="BM6" s="92"/>
+      <c r="BN6" s="92"/>
+      <c r="BO6" s="92"/>
+      <c r="BP6" s="92"/>
+      <c r="BQ6" s="92"/>
+      <c r="BR6" s="92"/>
+      <c r="BS6" s="92"/>
+      <c r="BT6" s="92"/>
+      <c r="BU6" s="92"/>
+      <c r="BV6" s="92"/>
+      <c r="BW6" s="92"/>
+      <c r="BX6" s="92"/>
+      <c r="BY6" s="92"/>
+      <c r="BZ6" s="92"/>
+      <c r="CA6" s="92"/>
+      <c r="CB6" s="92"/>
+      <c r="CC6" s="92"/>
+      <c r="CD6" s="92"/>
+      <c r="CE6" s="92"/>
+      <c r="CF6" s="92"/>
+      <c r="CG6" s="92"/>
+      <c r="CH6" s="92"/>
+      <c r="CI6" s="92"/>
+      <c r="CJ6" s="92"/>
+      <c r="CK6" s="92"/>
+      <c r="CL6" s="93"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr codeName="Sheet8"/>

</xml_diff>

<commit_message>
test: finalize SEL-080 review case
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Macro\SqlAnalyzerFormatter-feature\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7EBA3E4-76E4-4AF4-8B8D-C58F33777A57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F815FA5B-F9A2-4C34-8683-58BEB56CC43B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -92,13 +92,14 @@
     <sheet name="SEL-077" sheetId="84" r:id="rId77"/>
     <sheet name="SEL-078" sheetId="85" r:id="rId78"/>
     <sheet name="SEL-079" sheetId="86" r:id="rId79"/>
+    <sheet name="SEL-080" sheetId="87" r:id="rId80"/>
   </sheets>
   <calcPr calcId="0" calcMode="manual"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1376" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1393" uniqueCount="298">
   <si>
     <t>＜DB入出力項目定義＞</t>
   </si>
@@ -1018,7 +1019,7 @@
       <charset val="128"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1043,6 +1044,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2CEEF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2CEEF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -1286,7 +1297,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1569,6 +1580,51 @@
     <xf numFmtId="49" fontId="1" fillId="9" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="10" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="10" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="11" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="11" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="11" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="10" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="10" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="11" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="11" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="11" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="10" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="11" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="11" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="11" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -59671,6 +59727,607 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet80.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-4F00-000000000000}">
+  <sheetPr codeName="Sheet80"/>
+  <dimension ref="A1:CL6"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="90" width="1.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="22" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
+      <c r="Q1" s="22"/>
+      <c r="R1" s="22"/>
+      <c r="S1" s="22"/>
+      <c r="T1" s="22"/>
+      <c r="U1" s="22"/>
+      <c r="V1" s="22"/>
+      <c r="W1" s="22"/>
+      <c r="X1" s="22"/>
+      <c r="Y1" s="22"/>
+      <c r="Z1" s="22"/>
+      <c r="AA1" s="22"/>
+      <c r="AB1" s="22"/>
+      <c r="AC1" s="22"/>
+      <c r="AD1" s="22"/>
+      <c r="AE1" s="22"/>
+      <c r="AF1" s="22"/>
+      <c r="AG1" s="22"/>
+      <c r="AH1" s="22"/>
+      <c r="AI1" s="22"/>
+      <c r="AJ1" s="22"/>
+      <c r="AK1" s="22"/>
+      <c r="AL1" s="22"/>
+      <c r="AM1" s="22"/>
+      <c r="AN1" s="22"/>
+      <c r="AO1" s="22"/>
+      <c r="AP1" s="22"/>
+      <c r="AQ1" s="22"/>
+      <c r="AR1" s="22"/>
+      <c r="AS1" s="22"/>
+      <c r="AT1" s="22"/>
+      <c r="AU1" s="22"/>
+      <c r="AV1" s="22"/>
+      <c r="AW1" s="22"/>
+      <c r="AX1" s="22"/>
+      <c r="AY1" s="22"/>
+      <c r="AZ1" s="22"/>
+      <c r="BA1" s="22"/>
+      <c r="BB1" s="22"/>
+      <c r="BC1" s="22"/>
+      <c r="BD1" s="22"/>
+      <c r="BE1" s="22"/>
+      <c r="BF1" s="22"/>
+      <c r="BG1" s="22"/>
+      <c r="BH1" s="22"/>
+      <c r="BI1" s="22"/>
+      <c r="BJ1" s="22"/>
+      <c r="BK1" s="22"/>
+      <c r="BL1" s="22"/>
+      <c r="BM1" s="22"/>
+      <c r="BN1" s="22"/>
+      <c r="BO1" s="22"/>
+      <c r="BP1" s="22"/>
+      <c r="BQ1" s="22"/>
+      <c r="BR1" s="22"/>
+      <c r="BS1" s="22"/>
+      <c r="BT1" s="22"/>
+      <c r="BU1" s="22"/>
+      <c r="BV1" s="22"/>
+      <c r="BW1" s="22"/>
+      <c r="BX1" s="22"/>
+      <c r="BY1" s="22"/>
+      <c r="BZ1" s="22"/>
+      <c r="CA1" s="22"/>
+      <c r="CB1" s="22"/>
+      <c r="CC1" s="22"/>
+      <c r="CD1" s="22"/>
+      <c r="CE1" s="22"/>
+      <c r="CF1" s="22"/>
+      <c r="CG1" s="22"/>
+      <c r="CH1" s="22"/>
+      <c r="CI1" s="22"/>
+      <c r="CJ1" s="22"/>
+      <c r="CK1" s="22"/>
+      <c r="CL1" s="22"/>
+    </row>
+    <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="63" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
+      <c r="K2" s="63"/>
+      <c r="L2" s="63"/>
+      <c r="M2" s="63"/>
+      <c r="N2" s="63"/>
+      <c r="O2" s="63"/>
+      <c r="P2" s="63"/>
+      <c r="Q2" s="63"/>
+      <c r="R2" s="63"/>
+      <c r="S2" s="63"/>
+      <c r="T2" s="63"/>
+      <c r="U2" s="63"/>
+      <c r="V2" s="63"/>
+      <c r="W2" s="63"/>
+      <c r="X2" s="63"/>
+      <c r="Y2" s="63"/>
+      <c r="Z2" s="63"/>
+      <c r="AA2" s="63"/>
+      <c r="AB2" s="63"/>
+      <c r="AC2" s="63"/>
+      <c r="AD2" s="63"/>
+      <c r="AE2" s="63"/>
+      <c r="AF2" s="63"/>
+      <c r="AG2" s="63"/>
+      <c r="AH2" s="63"/>
+      <c r="AI2" s="63"/>
+      <c r="AJ2" s="63"/>
+      <c r="AK2" s="63"/>
+      <c r="AL2" s="63"/>
+      <c r="AM2" s="63"/>
+      <c r="AN2" s="63"/>
+      <c r="AO2" s="63"/>
+      <c r="AP2" s="63"/>
+      <c r="AQ2" s="63"/>
+      <c r="AR2" s="63"/>
+      <c r="AS2" s="63"/>
+      <c r="AT2" s="63"/>
+      <c r="AU2" s="63"/>
+      <c r="AV2" s="63"/>
+      <c r="AW2" s="63"/>
+      <c r="AX2" s="63"/>
+      <c r="AY2" s="63"/>
+      <c r="AZ2" s="63"/>
+      <c r="BA2" s="63"/>
+      <c r="BB2" s="63"/>
+      <c r="BC2" s="63"/>
+      <c r="BD2" s="63"/>
+      <c r="BE2" s="63"/>
+      <c r="BF2" s="63"/>
+      <c r="BG2" s="63"/>
+      <c r="BH2" s="63"/>
+      <c r="BI2" s="63"/>
+      <c r="BJ2" s="63"/>
+      <c r="BK2" s="63"/>
+      <c r="BL2" s="63"/>
+      <c r="BM2" s="63"/>
+      <c r="BN2" s="63"/>
+      <c r="BO2" s="63"/>
+      <c r="BP2" s="63"/>
+      <c r="BQ2" s="63"/>
+      <c r="BR2" s="63"/>
+      <c r="BS2" s="63"/>
+      <c r="BT2" s="63"/>
+      <c r="BU2" s="63"/>
+      <c r="BV2" s="63"/>
+      <c r="BW2" s="63"/>
+      <c r="BX2" s="63"/>
+      <c r="BY2" s="63"/>
+      <c r="BZ2" s="63"/>
+      <c r="CA2" s="63"/>
+      <c r="CB2" s="63"/>
+      <c r="CC2" s="63"/>
+      <c r="CD2" s="63"/>
+      <c r="CE2" s="63"/>
+      <c r="CF2" s="63"/>
+      <c r="CG2" s="63"/>
+      <c r="CH2" s="63"/>
+      <c r="CI2" s="63"/>
+      <c r="CJ2" s="63"/>
+      <c r="CK2" s="63"/>
+      <c r="CL2" s="63"/>
+    </row>
+    <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="94" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="95"/>
+      <c r="C3" s="95"/>
+      <c r="D3" s="95"/>
+      <c r="E3" s="95"/>
+      <c r="F3" s="95"/>
+      <c r="G3" s="96" t="s">
+        <v>3</v>
+      </c>
+      <c r="H3" s="97"/>
+      <c r="I3" s="97"/>
+      <c r="J3" s="97"/>
+      <c r="K3" s="97"/>
+      <c r="L3" s="97"/>
+      <c r="M3" s="97"/>
+      <c r="N3" s="97"/>
+      <c r="O3" s="97" t="s">
+        <v>4</v>
+      </c>
+      <c r="P3" s="97"/>
+      <c r="Q3" s="97" t="s">
+        <v>262</v>
+      </c>
+      <c r="R3" s="97"/>
+      <c r="S3" s="97"/>
+      <c r="T3" s="97"/>
+      <c r="U3" s="97"/>
+      <c r="V3" s="97"/>
+      <c r="W3" s="97"/>
+      <c r="X3" s="97"/>
+      <c r="Y3" s="97"/>
+      <c r="Z3" s="97"/>
+      <c r="AA3" s="97"/>
+      <c r="AB3" s="97"/>
+      <c r="AC3" s="97"/>
+      <c r="AD3" s="97"/>
+      <c r="AE3" s="97" t="s">
+        <v>33</v>
+      </c>
+      <c r="AF3" s="97" t="s">
+        <v>263</v>
+      </c>
+      <c r="AG3" s="97"/>
+      <c r="AH3" s="97"/>
+      <c r="AI3" s="97"/>
+      <c r="AJ3" s="97"/>
+      <c r="AK3" s="97"/>
+      <c r="AL3" s="97"/>
+      <c r="AM3" s="97"/>
+      <c r="AN3" s="97" t="s">
+        <v>264</v>
+      </c>
+      <c r="AO3" s="97"/>
+      <c r="AP3" s="97"/>
+      <c r="AQ3" s="97"/>
+      <c r="AR3" s="97"/>
+      <c r="AS3" s="97"/>
+      <c r="AT3" s="97"/>
+      <c r="AU3" s="97"/>
+      <c r="AV3" s="97"/>
+      <c r="AW3" s="97"/>
+      <c r="AX3" s="97"/>
+      <c r="AY3" s="97"/>
+      <c r="AZ3" s="97"/>
+      <c r="BA3" s="97"/>
+      <c r="BB3" s="97"/>
+      <c r="BC3" s="97"/>
+      <c r="BD3" s="97"/>
+      <c r="BE3" s="97"/>
+      <c r="BF3" s="97"/>
+      <c r="BG3" s="97"/>
+      <c r="BH3" s="97"/>
+      <c r="BI3" s="97"/>
+      <c r="BJ3" s="97"/>
+      <c r="BK3" s="97"/>
+      <c r="BL3" s="97"/>
+      <c r="BM3" s="97"/>
+      <c r="BN3" s="97"/>
+      <c r="BO3" s="97"/>
+      <c r="BP3" s="97"/>
+      <c r="BQ3" s="97"/>
+      <c r="BR3" s="97"/>
+      <c r="BS3" s="97"/>
+      <c r="BT3" s="97"/>
+      <c r="BU3" s="97"/>
+      <c r="BV3" s="97"/>
+      <c r="BW3" s="97"/>
+      <c r="BX3" s="97"/>
+      <c r="BY3" s="97"/>
+      <c r="BZ3" s="97"/>
+      <c r="CA3" s="97"/>
+      <c r="CB3" s="97"/>
+      <c r="CC3" s="97"/>
+      <c r="CD3" s="97"/>
+      <c r="CE3" s="97"/>
+      <c r="CF3" s="97"/>
+      <c r="CG3" s="97"/>
+      <c r="CH3" s="97"/>
+      <c r="CI3" s="97"/>
+      <c r="CJ3" s="97"/>
+      <c r="CK3" s="97"/>
+      <c r="CL3" s="98"/>
+    </row>
+    <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="99"/>
+      <c r="B4" s="100"/>
+      <c r="C4" s="100"/>
+      <c r="D4" s="100"/>
+      <c r="E4" s="100"/>
+      <c r="F4" s="100"/>
+      <c r="G4" s="101"/>
+      <c r="H4" s="102"/>
+      <c r="I4" s="102"/>
+      <c r="J4" s="102"/>
+      <c r="K4" s="102"/>
+      <c r="L4" s="102"/>
+      <c r="M4" s="102"/>
+      <c r="N4" s="102"/>
+      <c r="O4" s="102"/>
+      <c r="P4" s="102"/>
+      <c r="Q4" s="102"/>
+      <c r="R4" s="102"/>
+      <c r="S4" s="102"/>
+      <c r="T4" s="102"/>
+      <c r="U4" s="102"/>
+      <c r="V4" s="102"/>
+      <c r="W4" s="102"/>
+      <c r="X4" s="102"/>
+      <c r="Y4" s="102"/>
+      <c r="Z4" s="102"/>
+      <c r="AA4" s="102"/>
+      <c r="AB4" s="102"/>
+      <c r="AC4" s="102"/>
+      <c r="AD4" s="102"/>
+      <c r="AE4" s="102"/>
+      <c r="AF4" s="102"/>
+      <c r="AG4" s="102"/>
+      <c r="AH4" s="102"/>
+      <c r="AI4" s="102"/>
+      <c r="AJ4" s="102"/>
+      <c r="AK4" s="102"/>
+      <c r="AL4" s="102"/>
+      <c r="AM4" s="102"/>
+      <c r="AN4" s="102" t="s">
+        <v>226</v>
+      </c>
+      <c r="AO4" s="102"/>
+      <c r="AP4" s="102"/>
+      <c r="AQ4" s="102"/>
+      <c r="AR4" s="102"/>
+      <c r="AS4" s="102"/>
+      <c r="AT4" s="102"/>
+      <c r="AU4" s="102"/>
+      <c r="AV4" s="102"/>
+      <c r="AW4" s="102"/>
+      <c r="AX4" s="102"/>
+      <c r="AY4" s="102"/>
+      <c r="AZ4" s="102"/>
+      <c r="BA4" s="102"/>
+      <c r="BB4" s="102"/>
+      <c r="BC4" s="102"/>
+      <c r="BD4" s="102"/>
+      <c r="BE4" s="102"/>
+      <c r="BF4" s="102"/>
+      <c r="BG4" s="102"/>
+      <c r="BH4" s="102"/>
+      <c r="BI4" s="102"/>
+      <c r="BJ4" s="102"/>
+      <c r="BK4" s="102"/>
+      <c r="BL4" s="102"/>
+      <c r="BM4" s="102"/>
+      <c r="BN4" s="102"/>
+      <c r="BO4" s="102"/>
+      <c r="BP4" s="102"/>
+      <c r="BQ4" s="102"/>
+      <c r="BR4" s="102"/>
+      <c r="BS4" s="102"/>
+      <c r="BT4" s="102"/>
+      <c r="BU4" s="102"/>
+      <c r="BV4" s="102"/>
+      <c r="BW4" s="102"/>
+      <c r="BX4" s="102"/>
+      <c r="BY4" s="102"/>
+      <c r="BZ4" s="102"/>
+      <c r="CA4" s="102"/>
+      <c r="CB4" s="102"/>
+      <c r="CC4" s="102"/>
+      <c r="CD4" s="102"/>
+      <c r="CE4" s="102"/>
+      <c r="CF4" s="102"/>
+      <c r="CG4" s="102"/>
+      <c r="CH4" s="102"/>
+      <c r="CI4" s="102"/>
+      <c r="CJ4" s="102"/>
+      <c r="CK4" s="102"/>
+      <c r="CL4" s="103"/>
+    </row>
+    <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="99"/>
+      <c r="B5" s="100"/>
+      <c r="C5" s="100"/>
+      <c r="D5" s="100"/>
+      <c r="E5" s="100"/>
+      <c r="F5" s="100"/>
+      <c r="G5" s="101" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5" s="102"/>
+      <c r="I5" s="102"/>
+      <c r="J5" s="102"/>
+      <c r="K5" s="102"/>
+      <c r="L5" s="102"/>
+      <c r="M5" s="102"/>
+      <c r="N5" s="102"/>
+      <c r="O5" s="102" t="s">
+        <v>4</v>
+      </c>
+      <c r="P5" s="102"/>
+      <c r="Q5" s="102" t="s">
+        <v>297</v>
+      </c>
+      <c r="R5" s="102"/>
+      <c r="S5" s="102"/>
+      <c r="T5" s="102"/>
+      <c r="U5" s="102"/>
+      <c r="V5" s="102"/>
+      <c r="W5" s="102"/>
+      <c r="X5" s="102"/>
+      <c r="Y5" s="102"/>
+      <c r="Z5" s="102"/>
+      <c r="AA5" s="102"/>
+      <c r="AB5" s="102"/>
+      <c r="AC5" s="102"/>
+      <c r="AD5" s="102"/>
+      <c r="AE5" s="102" t="s">
+        <v>33</v>
+      </c>
+      <c r="AF5" s="102" t="s">
+        <v>263</v>
+      </c>
+      <c r="AG5" s="102"/>
+      <c r="AH5" s="102"/>
+      <c r="AI5" s="102"/>
+      <c r="AJ5" s="102"/>
+      <c r="AK5" s="102"/>
+      <c r="AL5" s="102"/>
+      <c r="AM5" s="102"/>
+      <c r="AN5" s="102" t="s">
+        <v>296</v>
+      </c>
+      <c r="AO5" s="102"/>
+      <c r="AP5" s="102"/>
+      <c r="AQ5" s="102"/>
+      <c r="AR5" s="102"/>
+      <c r="AS5" s="102"/>
+      <c r="AT5" s="102"/>
+      <c r="AU5" s="102"/>
+      <c r="AV5" s="102"/>
+      <c r="AW5" s="102"/>
+      <c r="AX5" s="102"/>
+      <c r="AY5" s="102"/>
+      <c r="AZ5" s="102"/>
+      <c r="BA5" s="102"/>
+      <c r="BB5" s="102"/>
+      <c r="BC5" s="102"/>
+      <c r="BD5" s="102"/>
+      <c r="BE5" s="102"/>
+      <c r="BF5" s="102"/>
+      <c r="BG5" s="102"/>
+      <c r="BH5" s="102"/>
+      <c r="BI5" s="102"/>
+      <c r="BJ5" s="102"/>
+      <c r="BK5" s="102"/>
+      <c r="BL5" s="102"/>
+      <c r="BM5" s="102"/>
+      <c r="BN5" s="102"/>
+      <c r="BO5" s="102"/>
+      <c r="BP5" s="102"/>
+      <c r="BQ5" s="102"/>
+      <c r="BR5" s="102"/>
+      <c r="BS5" s="102"/>
+      <c r="BT5" s="102"/>
+      <c r="BU5" s="102"/>
+      <c r="BV5" s="102"/>
+      <c r="BW5" s="102"/>
+      <c r="BX5" s="102"/>
+      <c r="BY5" s="102"/>
+      <c r="BZ5" s="102"/>
+      <c r="CA5" s="102"/>
+      <c r="CB5" s="102"/>
+      <c r="CC5" s="102"/>
+      <c r="CD5" s="102"/>
+      <c r="CE5" s="102"/>
+      <c r="CF5" s="102"/>
+      <c r="CG5" s="102"/>
+      <c r="CH5" s="102"/>
+      <c r="CI5" s="102"/>
+      <c r="CJ5" s="102"/>
+      <c r="CK5" s="102"/>
+      <c r="CL5" s="103"/>
+    </row>
+    <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="104"/>
+      <c r="B6" s="105"/>
+      <c r="C6" s="105"/>
+      <c r="D6" s="105"/>
+      <c r="E6" s="105"/>
+      <c r="F6" s="105"/>
+      <c r="G6" s="106"/>
+      <c r="H6" s="107"/>
+      <c r="I6" s="107"/>
+      <c r="J6" s="107"/>
+      <c r="K6" s="107"/>
+      <c r="L6" s="107"/>
+      <c r="M6" s="107"/>
+      <c r="N6" s="107"/>
+      <c r="O6" s="107"/>
+      <c r="P6" s="107"/>
+      <c r="Q6" s="107"/>
+      <c r="R6" s="107"/>
+      <c r="S6" s="107"/>
+      <c r="T6" s="107"/>
+      <c r="U6" s="107"/>
+      <c r="V6" s="107"/>
+      <c r="W6" s="107"/>
+      <c r="X6" s="107"/>
+      <c r="Y6" s="107"/>
+      <c r="Z6" s="107"/>
+      <c r="AA6" s="107"/>
+      <c r="AB6" s="107"/>
+      <c r="AC6" s="107"/>
+      <c r="AD6" s="107"/>
+      <c r="AE6" s="107"/>
+      <c r="AF6" s="107"/>
+      <c r="AG6" s="107"/>
+      <c r="AH6" s="107"/>
+      <c r="AI6" s="107"/>
+      <c r="AJ6" s="107"/>
+      <c r="AK6" s="107"/>
+      <c r="AL6" s="107"/>
+      <c r="AM6" s="107"/>
+      <c r="AN6" s="107" t="s">
+        <v>226</v>
+      </c>
+      <c r="AO6" s="107"/>
+      <c r="AP6" s="107"/>
+      <c r="AQ6" s="107"/>
+      <c r="AR6" s="107"/>
+      <c r="AS6" s="107"/>
+      <c r="AT6" s="107"/>
+      <c r="AU6" s="107"/>
+      <c r="AV6" s="107"/>
+      <c r="AW6" s="107"/>
+      <c r="AX6" s="107"/>
+      <c r="AY6" s="107"/>
+      <c r="AZ6" s="107"/>
+      <c r="BA6" s="107"/>
+      <c r="BB6" s="107"/>
+      <c r="BC6" s="107"/>
+      <c r="BD6" s="107"/>
+      <c r="BE6" s="107"/>
+      <c r="BF6" s="107"/>
+      <c r="BG6" s="107"/>
+      <c r="BH6" s="107"/>
+      <c r="BI6" s="107"/>
+      <c r="BJ6" s="107"/>
+      <c r="BK6" s="107"/>
+      <c r="BL6" s="107"/>
+      <c r="BM6" s="107"/>
+      <c r="BN6" s="107"/>
+      <c r="BO6" s="107"/>
+      <c r="BP6" s="107"/>
+      <c r="BQ6" s="107"/>
+      <c r="BR6" s="107"/>
+      <c r="BS6" s="107"/>
+      <c r="BT6" s="107"/>
+      <c r="BU6" s="107"/>
+      <c r="BV6" s="107"/>
+      <c r="BW6" s="107"/>
+      <c r="BX6" s="107"/>
+      <c r="BY6" s="107"/>
+      <c r="BZ6" s="107"/>
+      <c r="CA6" s="107"/>
+      <c r="CB6" s="107"/>
+      <c r="CC6" s="107"/>
+      <c r="CD6" s="107"/>
+      <c r="CE6" s="107"/>
+      <c r="CF6" s="107"/>
+      <c r="CG6" s="107"/>
+      <c r="CH6" s="107"/>
+      <c r="CI6" s="107"/>
+      <c r="CJ6" s="107"/>
+      <c r="CK6" s="107"/>
+      <c r="CL6" s="108"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <sheetPr codeName="Sheet9"/>

</xml_diff>

<commit_message>
feat: include SELECT INTO source table references
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -2,86 +2,86 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-001" sheetId="1" r:id="R57e90812016d4849"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-002" sheetId="2" r:id="R468416bbf8ca4b9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-003" sheetId="3" r:id="R4c49027cac26488f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-004" sheetId="4" r:id="R7aa9544bf0b146b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-005" sheetId="5" r:id="R8240ce4373df46a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-006" sheetId="6" r:id="R9f8d3453949141ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-007" sheetId="7" r:id="Rf07db026df874616"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-008" sheetId="8" r:id="R07f2a8d762bd4e8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-009" sheetId="9" r:id="Rc66dd20a99834942"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-010" sheetId="10" r:id="Ra27c02d9c73540cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-011" sheetId="11" r:id="R9afafa34d5e44245"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-012" sheetId="12" r:id="R8e0c34ffe6af4b74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-013" sheetId="13" r:id="Rb1a8c94547a6474c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-014" sheetId="14" r:id="R99bc5658655a49ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-015" sheetId="15" r:id="R260fcba2f6774ae8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-016" sheetId="16" r:id="R8c4671d5d2b04f0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-017" sheetId="17" r:id="R4402f98d62ba4946"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-018" sheetId="18" r:id="R2d121c5e67c74386"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-019" sheetId="19" r:id="R33b33de9fb0b4e4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-020" sheetId="20" r:id="R6f32b689c9164969"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-021" sheetId="21" r:id="Rf771e2a410da45c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-022" sheetId="22" r:id="R48145269c86b4a4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-023" sheetId="23" r:id="R8a2b3d00b73c46af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-024" sheetId="24" r:id="Rae2542a6168247e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-025" sheetId="25" r:id="R5ff665cbf8844ef0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-026" sheetId="26" r:id="R5d74e13aa5ff4839"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-027" sheetId="37" r:id="Rccd15bbdc5cf4587"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-028" sheetId="27" r:id="R729c60db8022410e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-029" sheetId="28" r:id="R33dd48b0b3994ce2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-030" sheetId="29" r:id="R127af271e4b940d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-031" sheetId="30" r:id="R7ec293e77aaa4427"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-032" sheetId="31" r:id="R8f512ea090054815"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-033" sheetId="32" r:id="R7924ba6f322a4f4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-034" sheetId="33" r:id="Rbfe5b2b347064f97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-035" sheetId="34" r:id="R3c73d0ce1b7b40e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-036" sheetId="35" r:id="R7a2b206b5d8f4586"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-037" sheetId="36" r:id="R46cf352be5344184"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-038" sheetId="38" r:id="R14b961970df94597"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-039" sheetId="39" r:id="R66ac2c7449b64685"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-040" sheetId="40" r:id="Rdb30986ea12b4058"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-041" sheetId="41" r:id="R8a5549d004924a20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-042" sheetId="42" r:id="R486f2d2bb7c94638"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-043" sheetId="43" r:id="R5649e3c96b51433d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-044" sheetId="44" r:id="Rd149e16e5d304986"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-045" sheetId="79" r:id="Rdcf2f8b6c50d408a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-046" sheetId="46" r:id="Rcbf7d6ead213498e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-047" sheetId="47" r:id="R3c235a4471154ac1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-048" sheetId="52" r:id="R5aad0afa14ee492d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-049" sheetId="53" r:id="R03aa65603df34b94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-050" sheetId="54" r:id="R6c35c1625bde40ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-051" sheetId="55" r:id="Rdd3f45f3570b46b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-052" sheetId="56" r:id="R607280765c7b488d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-053" sheetId="57" r:id="R5a667e03a6364402"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-054" sheetId="48" r:id="R13041d95d8f04bb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-055" sheetId="49" r:id="Rcb7ff3042f13424b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-056" sheetId="80" r:id="R154241ac13ce48dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-057" sheetId="70" r:id="R592ea53cab094688"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-058" sheetId="58" r:id="R3763277dfff54e38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-059" sheetId="81" r:id="R960c1ca601c44c9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-060" sheetId="63" r:id="R9239fc9f859a4d39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-061" sheetId="82" r:id="R8d2c64509cb54f9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-062" sheetId="64" r:id="R8794190a2753454e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-063" sheetId="65" r:id="Ra8f64a881dcc4bf6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-064" sheetId="66" r:id="Reab259fbc4014389"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-065" sheetId="67" r:id="Re11735ce961e4149"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-066" sheetId="68" r:id="R41e58df1e34548e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-067" sheetId="69" r:id="R17fe45a7bb97438f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-068" sheetId="71" r:id="Ra8156319acda4ea5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-069" sheetId="72" r:id="R79dce2b470694c2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-070" sheetId="73" r:id="Ra35d2911476c43cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-071" sheetId="74" r:id="R4b41093530354258"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-072" sheetId="75" r:id="R7441574bd67b4900"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-073" sheetId="76" r:id="R4b1b693f6e304d87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-074" sheetId="77" r:id="Rdff688a57d344e2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-075" sheetId="78" r:id="R816f162f7f30433b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-076" sheetId="83" r:id="R37e7c525a20e4efe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-077" sheetId="84" r:id="Rbdf3fa356c2d4459"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-078" sheetId="85" r:id="R649ce15d0e314945"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-079" sheetId="86" r:id="R57de3139b25640ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-080" sheetId="87" r:id="R26802778220644fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-001" sheetId="1" r:id="Rc0612a8968594661"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-002" sheetId="2" r:id="Ra5a1b7a9b66a4e11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-003" sheetId="3" r:id="R9ebeb60332b94d62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-004" sheetId="4" r:id="R3799c49c988c45c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-005" sheetId="5" r:id="Rd05a83d196bd4454"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-006" sheetId="6" r:id="Rc7b4b80efb624239"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-007" sheetId="7" r:id="Rec8e4c803e3c4b66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-008" sheetId="8" r:id="Rd155b29bbf7d43c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-009" sheetId="9" r:id="R42fd3a0352f941f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-010" sheetId="10" r:id="Rad883de173e64846"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-011" sheetId="11" r:id="R4c8d678fc0754cc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-012" sheetId="12" r:id="Rf8da778c898145b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-013" sheetId="13" r:id="R5e8a29546edc404e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-014" sheetId="14" r:id="Re0ffee208d7349c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-015" sheetId="15" r:id="Rf68ffdb761604cd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-016" sheetId="16" r:id="R0a7aa4625a2f41ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-017" sheetId="17" r:id="R84f8156a44a8441d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-018" sheetId="18" r:id="R4ba0ce5569904740"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-019" sheetId="19" r:id="R4ae34701f6ad4fc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-020" sheetId="20" r:id="Rc7589f78dd0c4078"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-021" sheetId="21" r:id="R4cc35331cb184c8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-022" sheetId="22" r:id="R8fe983ce42c14a5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-023" sheetId="23" r:id="Rdbbddcc69bb943db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-024" sheetId="24" r:id="Rd995b4370e1a4b05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-025" sheetId="25" r:id="R7fde30ebed6643a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-026" sheetId="26" r:id="R8166b871bbf44d20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-027" sheetId="37" r:id="R1f440cc2a3e04a71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-028" sheetId="27" r:id="R5b482c226e254dd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-029" sheetId="28" r:id="Ra693e282006d403f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-030" sheetId="29" r:id="R04bcfed2cbcd4451"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-031" sheetId="30" r:id="Rb24a93d71e0d43d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-032" sheetId="31" r:id="Rf785eddeb55e48e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-033" sheetId="32" r:id="Ra501c836b1eb4a36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-034" sheetId="33" r:id="Rac30f464e9934cab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-035" sheetId="34" r:id="R8cd98465131e4af6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-036" sheetId="35" r:id="R51490e69880a4bc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-037" sheetId="36" r:id="R3545ae70acb44816"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-038" sheetId="38" r:id="Rd18f1ce79576471e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-039" sheetId="39" r:id="R572c48ed8f354934"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-040" sheetId="40" r:id="R0fed2d2d0b16463f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-041" sheetId="41" r:id="R90b84b5d12dc4b94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-042" sheetId="42" r:id="Red2ccc56dc784c8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-043" sheetId="43" r:id="R91160fc3c7694124"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-044" sheetId="44" r:id="R865301f7abad4c32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-045" sheetId="79" r:id="Rbd255ba8243d4521"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-046" sheetId="46" r:id="Ra83c1693a9a34641"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-047" sheetId="47" r:id="Rb6703a2350b64117"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-048" sheetId="52" r:id="Re3837960d5084b05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-049" sheetId="53" r:id="Rb6a83f0d3c1f49cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-050" sheetId="54" r:id="R8e48b3eab23c42b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-051" sheetId="55" r:id="R564e0e49bb454e3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-052" sheetId="56" r:id="R94e6ea7712fc4c30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-053" sheetId="57" r:id="Rfebe87de49074efb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-054" sheetId="48" r:id="R976ef0670d3348de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-055" sheetId="49" r:id="Rd03c3c985ad74011"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-056" sheetId="80" r:id="R9616d2e5f646484f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-057" sheetId="70" r:id="R6aaafc0f690c4e2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-058" sheetId="58" r:id="R1ada62b658e443a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-059" sheetId="81" r:id="Rf38934427a2d444f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-060" sheetId="63" r:id="R04bb3fdfd7404583"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-061" sheetId="82" r:id="R2c4a6e23f9844f65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-062" sheetId="64" r:id="R6cef9f05232848c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-063" sheetId="65" r:id="R10f40d5be88d4c90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-064" sheetId="66" r:id="Rddc83d2d273b4d47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-065" sheetId="67" r:id="R598a6ac6be104bfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-066" sheetId="68" r:id="Rd951338cca5b4c9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-067" sheetId="69" r:id="R0c7703367c6c4df1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-068" sheetId="71" r:id="R2dbed6506ce0496c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-069" sheetId="72" r:id="Rb034aab3771e4816"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-070" sheetId="73" r:id="R7dde09cfbf4c4a69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-071" sheetId="74" r:id="R07233d937b7f4744"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-072" sheetId="75" r:id="Rdf0b140830584694"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-073" sheetId="76" r:id="Rba6e11c04d53438f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-074" sheetId="77" r:id="R3271ee50a68e4122"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-075" sheetId="78" r:id="R26c519f13c3e45dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-076" sheetId="83" r:id="R3d6c7b323d034df3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-077" sheetId="84" r:id="R41155df28d8f4875"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-078" sheetId="85" r:id="R8606797c47234dfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-079" sheetId="86" r:id="R7a4dcadf2be1498b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-080" sheetId="87" r:id="Ra5faf82c51794913"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -774,9 +774,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">DISTINCT</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">参照テーブル: ユーザー出力</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">メール</x:t>
@@ -38806,8 +38803,8 @@
       <x:c r="CL6" s="1"/>
     </x:row>
     <x:row r="7" ht="13.5" customHeight="1">
-      <x:c r="A7" s="22" t="s">
-        <x:v>229</x:v>
+      <x:c r="A7" s="22" t="str">
+        <x:v>参照テーブル: ユーザー出力、ユーザー[tb1]</x:v>
       </x:c>
       <x:c r="B7" s="1"/>
       <x:c r="C7" s="1"/>
@@ -39095,7 +39092,7 @@
     </x:row>
     <x:row r="10" ht="13.5" customHeight="1">
       <x:c r="A10" s="20" t="s">
-        <x:v>230</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="B10" s="18"/>
       <x:c r="C10" s="18"/>
@@ -39893,7 +39890,7 @@
     </x:row>
     <x:row r="2" ht="13.5" customHeight="1">
       <x:c r="A2" s="22" t="s">
-        <x:v>231</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -40123,7 +40120,7 @@
       <x:c r="AI4" s="14"/>
       <x:c r="AJ4" s="14"/>
       <x:c r="AK4" s="31" t="s">
-        <x:v>232</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="AL4" s="14"/>
       <x:c r="AM4" s="14"/>
@@ -40219,7 +40216,7 @@
       <x:c r="AI5" s="18"/>
       <x:c r="AJ5" s="18"/>
       <x:c r="AK5" s="20" t="s">
-        <x:v>233</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="AL5" s="18"/>
       <x:c r="AM5" s="18"/>
@@ -40315,7 +40312,7 @@
       <x:c r="AI6" s="18"/>
       <x:c r="AJ6" s="18"/>
       <x:c r="AK6" s="20" t="s">
-        <x:v>234</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="AL6" s="18"/>
       <x:c r="AM6" s="18"/>
@@ -40993,7 +40990,7 @@
       </x:c>
       <x:c r="P6" s="3"/>
       <x:c r="Q6" s="27" t="s">
-        <x:v>235</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="R6" s="3"/>
       <x:c r="S6" s="3"/>
@@ -41012,7 +41009,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF6" s="27" t="s">
-        <x:v>236</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="AG6" s="3"/>
       <x:c r="AH6" s="3"/>
@@ -41106,7 +41103,7 @@
       <x:c r="AD7" s="3"/>
       <x:c r="AE7" s="3"/>
       <x:c r="AF7" s="27" t="s">
-        <x:v>237</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="AG7" s="3"/>
       <x:c r="AH7" s="3"/>
@@ -41200,7 +41197,7 @@
       <x:c r="AD8" s="3"/>
       <x:c r="AE8" s="3"/>
       <x:c r="AF8" s="27" t="s">
-        <x:v>238</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="AG8" s="3"/>
       <x:c r="AH8" s="3"/>
@@ -41283,7 +41280,7 @@
       </x:c>
       <x:c r="P9" s="3"/>
       <x:c r="Q9" s="27" t="s">
-        <x:v>239</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="R9" s="3"/>
       <x:c r="S9" s="3"/>
@@ -41371,7 +41368,7 @@
       <x:c r="E10" s="2"/>
       <x:c r="F10" s="2"/>
       <x:c r="G10" s="26" t="s">
-        <x:v>240</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="H10" s="3"/>
       <x:c r="I10" s="3"/>
@@ -41385,7 +41382,7 @@
       </x:c>
       <x:c r="P10" s="3"/>
       <x:c r="Q10" s="27" t="s">
-        <x:v>241</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="R10" s="3"/>
       <x:c r="S10" s="3"/>
@@ -42426,8 +42423,8 @@
       <x:c r="CL20" s="1"/>
     </x:row>
     <x:row r="21" ht="13.5" customHeight="1">
-      <x:c r="A21" s="22" t="s">
-        <x:v>217</x:v>
+      <x:c r="A21" s="22" t="str">
+        <x:v>参照テーブル: ユーザー集計、ユーザー[tb1]、注文[tb2]</x:v>
       </x:c>
       <x:c r="B21" s="1"/>
       <x:c r="C21" s="1"/>
@@ -42911,7 +42908,7 @@
     </x:row>
     <x:row r="26" ht="13.5" customHeight="1">
       <x:c r="A26" s="33" t="s">
-        <x:v>242</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="B26" s="34"/>
       <x:c r="C26" s="34"/>
@@ -42968,7 +42965,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AZ26" s="34" t="s">
-        <x:v>236</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="BA26" s="34"/>
       <x:c r="BB26" s="34"/>
@@ -43062,7 +43059,7 @@
       <x:c r="AX27" s="37"/>
       <x:c r="AY27" s="37"/>
       <x:c r="AZ27" s="37" t="s">
-        <x:v>237</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="BA27" s="37"/>
       <x:c r="BB27" s="37"/>
@@ -43156,7 +43153,7 @@
       <x:c r="AX28" s="40"/>
       <x:c r="AY28" s="40"/>
       <x:c r="AZ28" s="40" t="s">
-        <x:v>238</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="BA28" s="40"/>
       <x:c r="BB28" s="40"/>
@@ -43905,7 +43902,7 @@
       </x:c>
       <x:c r="P6" s="18"/>
       <x:c r="Q6" s="29" t="s">
-        <x:v>243</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="R6" s="18"/>
       <x:c r="S6" s="18"/>
@@ -44361,7 +44358,7 @@
     </x:row>
     <x:row r="11" ht="13.5" customHeight="1">
       <x:c r="A11" s="26" t="s">
-        <x:v>244</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="B11" s="3"/>
       <x:c r="C11" s="3"/>
@@ -44381,7 +44378,7 @@
       <x:c r="Q11" s="3"/>
       <x:c r="R11" s="3"/>
       <x:c r="S11" s="26" t="s">
-        <x:v>245</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="T11" s="3"/>
       <x:c r="U11" s="3"/>
@@ -44659,7 +44656,7 @@
     </x:row>
     <x:row r="2" ht="13.5" customHeight="1">
       <x:c r="A2" s="22" t="s">
-        <x:v>246</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -44873,7 +44870,7 @@
       </x:c>
       <x:c r="P4" s="3"/>
       <x:c r="Q4" s="27" t="s">
-        <x:v>247</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="R4" s="3"/>
       <x:c r="S4" s="3"/>
@@ -44892,7 +44889,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF4" s="27" t="s">
-        <x:v>248</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="AG4" s="3"/>
       <x:c r="AH4" s="3"/>
@@ -45453,7 +45450,7 @@
       <x:c r="Q10" s="3"/>
       <x:c r="R10" s="3"/>
       <x:c r="S10" s="26" t="s">
-        <x:v>249</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="T10" s="3"/>
       <x:c r="U10" s="3"/>
@@ -46509,7 +46506,7 @@
       <x:c r="O8" s="18"/>
       <x:c r="P8" s="18"/>
       <x:c r="Q8" s="29" t="s">
-        <x:v>250</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="R8" s="18"/>
       <x:c r="S8" s="18"/>
@@ -46693,7 +46690,7 @@
     </x:row>
     <x:row r="2" ht="13.5" customHeight="1">
       <x:c r="A2" s="22" t="s">
-        <x:v>251</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -46905,7 +46902,7 @@
       <x:c r="O4" s="6"/>
       <x:c r="P4" s="6"/>
       <x:c r="Q4" s="25" t="s">
-        <x:v>252</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="R4" s="6"/>
       <x:c r="S4" s="6"/>
@@ -47001,7 +46998,7 @@
       <x:c r="O5" s="14"/>
       <x:c r="P5" s="14"/>
       <x:c r="Q5" s="30" t="s">
-        <x:v>253</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="R5" s="14"/>
       <x:c r="S5" s="14"/>
@@ -47265,7 +47262,7 @@
     </x:row>
     <x:row r="8" ht="13.5" customHeight="1">
       <x:c r="A8" s="22" t="s">
-        <x:v>254</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="B8" s="1"/>
       <x:c r="C8" s="1"/>
@@ -47495,7 +47492,7 @@
       <x:c r="AI10" s="3"/>
       <x:c r="AJ10" s="3"/>
       <x:c r="AK10" s="26" t="s">
-        <x:v>255</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="AL10" s="3"/>
       <x:c r="AM10" s="3"/>
@@ -47571,7 +47568,7 @@
       <x:c r="O11" s="18"/>
       <x:c r="P11" s="18"/>
       <x:c r="Q11" s="29" t="s">
-        <x:v>250</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="R11" s="18"/>
       <x:c r="S11" s="18"/>
@@ -47871,7 +47868,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>256</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -47890,7 +47887,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF3" s="25" t="s">
-        <x:v>257</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="AG3" s="6"/>
       <x:c r="AH3" s="6"/>
@@ -48465,7 +48462,7 @@
       <x:c r="AI9" s="3"/>
       <x:c r="AJ9" s="3"/>
       <x:c r="AK9" s="26" t="s">
-        <x:v>258</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="AL9" s="3"/>
       <x:c r="AM9" s="3"/>
@@ -48541,7 +48538,7 @@
       <x:c r="O10" s="18"/>
       <x:c r="P10" s="18"/>
       <x:c r="Q10" s="29" t="s">
-        <x:v>259</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="R10" s="18"/>
       <x:c r="S10" s="18"/>
@@ -48937,7 +48934,7 @@
       <x:c r="O4" s="18"/>
       <x:c r="P4" s="18"/>
       <x:c r="Q4" s="29" t="s">
-        <x:v>260</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="R4" s="18"/>
       <x:c r="S4" s="18"/>
@@ -49431,7 +49428,7 @@
       <x:c r="AI9" s="3"/>
       <x:c r="AJ9" s="3"/>
       <x:c r="AK9" s="26" t="s">
-        <x:v>261</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="AL9" s="3"/>
       <x:c r="AM9" s="3"/>
@@ -49807,7 +49804,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>262</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -49826,7 +49823,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF3" s="25" t="s">
-        <x:v>263</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="AG3" s="6"/>
       <x:c r="AH3" s="25"/>
@@ -49836,7 +49833,7 @@
       <x:c r="AL3" s="6"/>
       <x:c r="AM3" s="6"/>
       <x:c r="AN3" s="6" t="s">
-        <x:v>264</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="AO3" s="6"/>
       <x:c r="AP3" s="6"/>
@@ -50207,7 +50204,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>265</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -50226,7 +50223,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF3" s="25" t="s">
-        <x:v>266</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="AG3" s="6"/>
       <x:c r="AH3" s="6"/>
@@ -50320,7 +50317,7 @@
       <x:c r="AD4" s="3"/>
       <x:c r="AE4" s="3"/>
       <x:c r="AF4" s="27" t="s">
-        <x:v>267</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="AG4" s="3"/>
       <x:c r="AH4" s="3"/>
@@ -50416,7 +50413,7 @@
       <x:c r="AF5" s="14"/>
       <x:c r="AG5" s="14"/>
       <x:c r="AH5" s="30" t="s">
-        <x:v>268</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="AI5" s="14"/>
       <x:c r="AJ5" s="14"/>
@@ -51385,7 +51382,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>269</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -51406,7 +51403,7 @@
       <x:c r="AF3" s="6"/>
       <x:c r="AG3" s="6"/>
       <x:c r="AH3" s="25" t="s">
-        <x:v>270</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="AI3" s="6"/>
       <x:c r="AJ3" s="6"/>
@@ -51502,7 +51499,7 @@
       </x:c>
       <x:c r="AG4" s="3"/>
       <x:c r="AH4" s="27" t="s">
-        <x:v>271</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="AI4" s="3"/>
       <x:c r="AJ4" s="3"/>
@@ -52110,7 +52107,7 @@
       </x:c>
       <x:c r="BA5" s="3"/>
       <x:c r="BB5" s="27" t="s">
-        <x:v>272</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="BC5" s="3"/>
       <x:c r="BD5" s="3"/>
@@ -52202,7 +52199,7 @@
       <x:c r="AX6" s="14"/>
       <x:c r="AY6" s="14"/>
       <x:c r="AZ6" s="30" t="s">
-        <x:v>273</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="BA6" s="14"/>
       <x:c r="BB6" s="14"/>
@@ -52351,7 +52348,7 @@
     </x:row>
     <x:row r="2" ht="13.5" customHeight="1">
       <x:c r="A2" s="22" t="s">
-        <x:v>231</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -52600,7 +52597,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AZ4" s="25" t="s">
-        <x:v>274</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="BA4" s="6"/>
       <x:c r="BB4" s="6"/>
@@ -52694,7 +52691,7 @@
       <x:c r="AX5" s="14"/>
       <x:c r="AY5" s="14"/>
       <x:c r="AZ5" s="30" t="s">
-        <x:v>273</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="BA5" s="14"/>
       <x:c r="BB5" s="14"/>
@@ -52959,7 +52956,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>275</x:v>
+        <x:v>274</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -53053,7 +53050,7 @@
       <x:c r="O4" s="3"/>
       <x:c r="P4" s="3"/>
       <x:c r="Q4" s="27" t="s">
-        <x:v>276</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="R4" s="3"/>
       <x:c r="S4" s="3"/>
@@ -54434,7 +54431,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF3" s="25" t="s">
-        <x:v>277</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="AG3" s="6"/>
       <x:c r="AH3" s="6"/>
@@ -54697,7 +54694,7 @@
     </x:row>
     <x:row r="2" ht="13.5" customHeight="1">
       <x:c r="A2" s="1" t="s">
-        <x:v>231</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -54791,7 +54788,7 @@
     </x:row>
     <x:row r="3" ht="13.5" customHeight="1">
       <x:c r="A3" s="61" t="s">
-        <x:v>278</x:v>
+        <x:v>277</x:v>
       </x:c>
       <x:c r="B3" s="61"/>
       <x:c r="C3" s="61"/>
@@ -55021,7 +55018,7 @@
       <x:c r="AI5" s="48"/>
       <x:c r="AJ5" s="48"/>
       <x:c r="AK5" s="47" t="s">
-        <x:v>279</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="AL5" s="48"/>
       <x:c r="AM5" s="48"/>
@@ -55117,7 +55114,7 @@
       <x:c r="AI6" s="48"/>
       <x:c r="AJ6" s="48"/>
       <x:c r="AK6" s="47" t="s">
-        <x:v>280</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="AL6" s="48"/>
       <x:c r="AM6" s="48"/>
@@ -55213,7 +55210,7 @@
       <x:c r="AI7" s="48"/>
       <x:c r="AJ7" s="48"/>
       <x:c r="AK7" s="47" t="s">
-        <x:v>234</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="AL7" s="48"/>
       <x:c r="AM7" s="48"/>
@@ -55367,7 +55364,7 @@
     </x:row>
     <x:row r="9" ht="13.5" customHeight="1">
       <x:c r="A9" s="46" t="s">
-        <x:v>281</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="B9" s="46"/>
       <x:c r="C9" s="46"/>
@@ -55597,7 +55594,7 @@
       <x:c r="AI11" s="48"/>
       <x:c r="AJ11" s="48"/>
       <x:c r="AK11" s="47" t="s">
-        <x:v>282</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="AL11" s="48"/>
       <x:c r="AM11" s="48"/>
@@ -55693,7 +55690,7 @@
       <x:c r="AI12" s="48"/>
       <x:c r="AJ12" s="48"/>
       <x:c r="AK12" s="47" t="s">
-        <x:v>283</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="AL12" s="48"/>
       <x:c r="AM12" s="48"/>
@@ -55789,7 +55786,7 @@
       <x:c r="AI13" s="48"/>
       <x:c r="AJ13" s="48"/>
       <x:c r="AK13" s="47" t="s">
-        <x:v>284</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="AL13" s="48"/>
       <x:c r="AM13" s="48"/>
@@ -56437,7 +56434,7 @@
     </x:row>
     <x:row r="6" ht="13.5" customHeight="1">
       <x:c r="A6" s="46" t="s">
-        <x:v>285</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="B6" s="46"/>
       <x:c r="C6" s="46"/>
@@ -56651,7 +56648,7 @@
       </x:c>
       <x:c r="P8" s="45"/>
       <x:c r="Q8" s="45" t="s">
-        <x:v>286</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="R8" s="45"/>
       <x:c r="S8" s="45"/>
@@ -56747,7 +56744,7 @@
       <x:c r="O9" s="48"/>
       <x:c r="P9" s="48"/>
       <x:c r="Q9" s="48" t="s">
-        <x:v>287</x:v>
+        <x:v>286</x:v>
       </x:c>
       <x:c r="R9" s="48"/>
       <x:c r="S9" s="48"/>
@@ -57105,7 +57102,7 @@
     </x:row>
     <x:row r="13" ht="13.5" customHeight="1">
       <x:c r="A13" s="62" t="s">
-        <x:v>288</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="B13" s="61"/>
       <x:c r="C13" s="61"/>
@@ -57489,7 +57486,7 @@
     </x:row>
     <x:row r="17" ht="13.5" customHeight="1">
       <x:c r="A17" s="46" t="s">
-        <x:v>289</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="B17" s="48"/>
       <x:c r="C17" s="48"/>
@@ -57817,7 +57814,7 @@
       <x:c r="AI20" s="48"/>
       <x:c r="AJ20" s="48"/>
       <x:c r="AK20" s="47" t="s">
-        <x:v>286</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="AL20" s="48"/>
       <x:c r="AM20" s="48"/>
@@ -58097,7 +58094,7 @@
       </x:c>
       <x:c r="P3" s="67"/>
       <x:c r="Q3" s="67" t="s">
-        <x:v>290</x:v>
+        <x:v>289</x:v>
       </x:c>
       <x:c r="R3" s="67"/>
       <x:c r="S3" s="67"/>
@@ -58116,7 +58113,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF3" s="67" t="s">
-        <x:v>291</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="AG3" s="67"/>
       <x:c r="AH3" s="67"/>
@@ -58132,7 +58129,7 @@
       <x:c r="AR3" s="67"/>
       <x:c r="AS3" s="67"/>
       <x:c r="AT3" s="67" t="s">
-        <x:v>292</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="AU3" s="67"/>
       <x:c r="AV3" s="67"/>
@@ -58140,7 +58137,7 @@
       <x:c r="AX3" s="67"/>
       <x:c r="AY3" s="67"/>
       <x:c r="AZ3" s="67" t="s">
-        <x:v>264</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="BA3" s="67"/>
       <x:c r="BB3" s="67"/>
@@ -58322,7 +58319,7 @@
       <x:c r="AR5" s="72"/>
       <x:c r="AS5" s="72"/>
       <x:c r="AT5" s="72" t="s">
-        <x:v>293</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="AU5" s="72"/>
       <x:c r="AV5" s="72"/>
@@ -58330,7 +58327,7 @@
       <x:c r="AX5" s="72"/>
       <x:c r="AY5" s="72"/>
       <x:c r="AZ5" s="72" t="s">
-        <x:v>294</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="BA5" s="72"/>
       <x:c r="BB5" s="72"/>
@@ -58689,7 +58686,7 @@
       </x:c>
       <x:c r="P3" s="82"/>
       <x:c r="Q3" s="82" t="s">
-        <x:v>262</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="R3" s="82"/>
       <x:c r="S3" s="82"/>
@@ -58708,7 +58705,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF3" s="82" t="s">
-        <x:v>264</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="AG3" s="82"/>
       <x:c r="AH3" s="82"/>
@@ -58885,7 +58882,7 @@
       </x:c>
       <x:c r="P5" s="87"/>
       <x:c r="Q5" s="87" t="s">
-        <x:v>295</x:v>
+        <x:v>294</x:v>
       </x:c>
       <x:c r="R5" s="87"/>
       <x:c r="S5" s="87"/>
@@ -58904,7 +58901,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF5" s="87" t="s">
-        <x:v>294</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="AG5" s="87"/>
       <x:c r="AH5" s="87"/>
@@ -59969,7 +59966,7 @@
       </x:c>
       <x:c r="P3" s="97"/>
       <x:c r="Q3" s="97" t="s">
-        <x:v>262</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="R3" s="97"/>
       <x:c r="S3" s="97"/>
@@ -59988,7 +59985,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF3" s="97" t="s">
-        <x:v>263</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="AG3" s="97"/>
       <x:c r="AH3" s="97"/>
@@ -59998,7 +59995,7 @@
       <x:c r="AL3" s="97"/>
       <x:c r="AM3" s="97"/>
       <x:c r="AN3" s="97" t="s">
-        <x:v>264</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="AO3" s="97"/>
       <x:c r="AP3" s="97"/>
@@ -60167,7 +60164,7 @@
       </x:c>
       <x:c r="P5" s="102"/>
       <x:c r="Q5" s="102" t="s">
-        <x:v>295</x:v>
+        <x:v>294</x:v>
       </x:c>
       <x:c r="R5" s="102"/>
       <x:c r="S5" s="102"/>
@@ -60186,7 +60183,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF5" s="102" t="s">
-        <x:v>263</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="AG5" s="102"/>
       <x:c r="AH5" s="102"/>
@@ -60196,7 +60193,7 @@
       <x:c r="AL5" s="102"/>
       <x:c r="AM5" s="102"/>
       <x:c r="AN5" s="102" t="s">
-        <x:v>294</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="AO5" s="102"/>
       <x:c r="AP5" s="102"/>

</xml_diff>

<commit_message>
feat: include DML source table references
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -2,86 +2,86 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-001" sheetId="1" r:id="Rc0612a8968594661"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-002" sheetId="2" r:id="Ra5a1b7a9b66a4e11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-003" sheetId="3" r:id="R9ebeb60332b94d62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-004" sheetId="4" r:id="R3799c49c988c45c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-005" sheetId="5" r:id="Rd05a83d196bd4454"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-006" sheetId="6" r:id="Rc7b4b80efb624239"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-007" sheetId="7" r:id="Rec8e4c803e3c4b66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-008" sheetId="8" r:id="Rd155b29bbf7d43c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-009" sheetId="9" r:id="R42fd3a0352f941f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-010" sheetId="10" r:id="Rad883de173e64846"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-011" sheetId="11" r:id="R4c8d678fc0754cc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-012" sheetId="12" r:id="Rf8da778c898145b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-013" sheetId="13" r:id="R5e8a29546edc404e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-014" sheetId="14" r:id="Re0ffee208d7349c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-015" sheetId="15" r:id="Rf68ffdb761604cd5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-016" sheetId="16" r:id="R0a7aa4625a2f41ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-017" sheetId="17" r:id="R84f8156a44a8441d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-018" sheetId="18" r:id="R4ba0ce5569904740"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-019" sheetId="19" r:id="R4ae34701f6ad4fc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-020" sheetId="20" r:id="Rc7589f78dd0c4078"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-021" sheetId="21" r:id="R4cc35331cb184c8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-022" sheetId="22" r:id="R8fe983ce42c14a5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-023" sheetId="23" r:id="Rdbbddcc69bb943db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-024" sheetId="24" r:id="Rd995b4370e1a4b05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-025" sheetId="25" r:id="R7fde30ebed6643a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-026" sheetId="26" r:id="R8166b871bbf44d20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-027" sheetId="37" r:id="R1f440cc2a3e04a71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-028" sheetId="27" r:id="R5b482c226e254dd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-029" sheetId="28" r:id="Ra693e282006d403f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-030" sheetId="29" r:id="R04bcfed2cbcd4451"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-031" sheetId="30" r:id="Rb24a93d71e0d43d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-032" sheetId="31" r:id="Rf785eddeb55e48e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-033" sheetId="32" r:id="Ra501c836b1eb4a36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-034" sheetId="33" r:id="Rac30f464e9934cab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-035" sheetId="34" r:id="R8cd98465131e4af6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-036" sheetId="35" r:id="R51490e69880a4bc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-037" sheetId="36" r:id="R3545ae70acb44816"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-038" sheetId="38" r:id="Rd18f1ce79576471e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-039" sheetId="39" r:id="R572c48ed8f354934"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-040" sheetId="40" r:id="R0fed2d2d0b16463f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-041" sheetId="41" r:id="R90b84b5d12dc4b94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-042" sheetId="42" r:id="Red2ccc56dc784c8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-043" sheetId="43" r:id="R91160fc3c7694124"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-044" sheetId="44" r:id="R865301f7abad4c32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-045" sheetId="79" r:id="Rbd255ba8243d4521"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-046" sheetId="46" r:id="Ra83c1693a9a34641"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-047" sheetId="47" r:id="Rb6703a2350b64117"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-048" sheetId="52" r:id="Re3837960d5084b05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-049" sheetId="53" r:id="Rb6a83f0d3c1f49cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-050" sheetId="54" r:id="R8e48b3eab23c42b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-051" sheetId="55" r:id="R564e0e49bb454e3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-052" sheetId="56" r:id="R94e6ea7712fc4c30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-053" sheetId="57" r:id="Rfebe87de49074efb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-054" sheetId="48" r:id="R976ef0670d3348de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-055" sheetId="49" r:id="Rd03c3c985ad74011"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-056" sheetId="80" r:id="R9616d2e5f646484f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-057" sheetId="70" r:id="R6aaafc0f690c4e2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-058" sheetId="58" r:id="R1ada62b658e443a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-059" sheetId="81" r:id="Rf38934427a2d444f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-060" sheetId="63" r:id="R04bb3fdfd7404583"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-061" sheetId="82" r:id="R2c4a6e23f9844f65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-062" sheetId="64" r:id="R6cef9f05232848c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-063" sheetId="65" r:id="R10f40d5be88d4c90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-064" sheetId="66" r:id="Rddc83d2d273b4d47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-065" sheetId="67" r:id="R598a6ac6be104bfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-066" sheetId="68" r:id="Rd951338cca5b4c9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-067" sheetId="69" r:id="R0c7703367c6c4df1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-068" sheetId="71" r:id="R2dbed6506ce0496c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-069" sheetId="72" r:id="Rb034aab3771e4816"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-070" sheetId="73" r:id="R7dde09cfbf4c4a69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-071" sheetId="74" r:id="R07233d937b7f4744"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-072" sheetId="75" r:id="Rdf0b140830584694"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-073" sheetId="76" r:id="Rba6e11c04d53438f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-074" sheetId="77" r:id="R3271ee50a68e4122"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-075" sheetId="78" r:id="R26c519f13c3e45dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-076" sheetId="83" r:id="R3d6c7b323d034df3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-077" sheetId="84" r:id="R41155df28d8f4875"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-078" sheetId="85" r:id="R8606797c47234dfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-079" sheetId="86" r:id="R7a4dcadf2be1498b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-080" sheetId="87" r:id="Ra5faf82c51794913"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-001" sheetId="1" r:id="R9e31f1c082624221"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-002" sheetId="2" r:id="R6c5c85d85cea4fa9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-003" sheetId="3" r:id="R8acca56f2b07416b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-004" sheetId="4" r:id="Rf3b3f66b4f084183"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-005" sheetId="5" r:id="R05532699aaf54c0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-006" sheetId="6" r:id="R5cf1ee78b67841c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-007" sheetId="7" r:id="Rcce4cc803f81442a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-008" sheetId="8" r:id="R1dd50293bfff4c82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-009" sheetId="9" r:id="R5835f5c051124d1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-010" sheetId="10" r:id="Rab222cbf57a448b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-011" sheetId="11" r:id="R7e6eb7c54c754539"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-012" sheetId="12" r:id="Rba61485383494a2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-013" sheetId="13" r:id="R4276550ffba1479e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-014" sheetId="14" r:id="Re273ff204576418c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-015" sheetId="15" r:id="R5ac138d403c441cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-016" sheetId="16" r:id="R8ae01eb4953a46c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-017" sheetId="17" r:id="Rae204ab5bcaf477b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-018" sheetId="18" r:id="R674033c3dedd436f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-019" sheetId="19" r:id="Red1a481e6148418c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-020" sheetId="20" r:id="R88cad74a06b04453"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-021" sheetId="21" r:id="Rea8b681bcc784b4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-022" sheetId="22" r:id="R181d9202e11a4231"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-023" sheetId="23" r:id="Rcdb6f863abe841bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-024" sheetId="24" r:id="R5643fd17304b497e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-025" sheetId="25" r:id="R70a863fddd7d4db7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-026" sheetId="26" r:id="Rc39f2fc41d9f48a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-027" sheetId="37" r:id="Re7586820766544e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-028" sheetId="27" r:id="R5bf8bcc45a2a4f3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-029" sheetId="28" r:id="Rdc3bb458df894670"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-030" sheetId="29" r:id="Rd10ea07adec04708"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-031" sheetId="30" r:id="Re990fb46612a4704"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-032" sheetId="31" r:id="R12a3454afc6948fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-033" sheetId="32" r:id="R5255db377b384df5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-034" sheetId="33" r:id="R89a6ba40a4484654"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-035" sheetId="34" r:id="R0dddfdea25974994"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-036" sheetId="35" r:id="R441819a150104a58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-037" sheetId="36" r:id="Rdcfd95da92764aee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-038" sheetId="38" r:id="R36e9708c3b9e4c6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-039" sheetId="39" r:id="R154eb474776749f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-040" sheetId="40" r:id="Re123610114c34055"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-041" sheetId="41" r:id="R2fd9939f192a41d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-042" sheetId="42" r:id="R0acd6e3d85334ee9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-043" sheetId="43" r:id="Rfbb54c3982d7479d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-044" sheetId="44" r:id="R547b8b76fa3940f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-045" sheetId="79" r:id="R42f9e57fc7b347ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-046" sheetId="46" r:id="R304b2d44c52a4868"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-047" sheetId="47" r:id="R64eced95184d40a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-048" sheetId="52" r:id="Rc7c41b133d324065"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-049" sheetId="53" r:id="R1fa49aeb0d3648b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-050" sheetId="54" r:id="R802a5119050d433c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-051" sheetId="55" r:id="Ra98e022d51c34175"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-052" sheetId="56" r:id="R09c04080641f484a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-053" sheetId="57" r:id="R27d49c0f403a47f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-054" sheetId="48" r:id="R61e6dc505893436e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-055" sheetId="49" r:id="Rcf8a9f3c17b747a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-056" sheetId="80" r:id="R3d7236a5f7ce4670"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-057" sheetId="70" r:id="Rcc1ea59be06a4ad8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-058" sheetId="58" r:id="Rb767d73e7f984b65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-059" sheetId="81" r:id="R70547f5766eb4349"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-060" sheetId="63" r:id="R99359405dcb34695"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-061" sheetId="82" r:id="R746fdba3cc354477"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-062" sheetId="64" r:id="R4888b8f99c4b484b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-063" sheetId="65" r:id="Raada8c4b4bb54cdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-064" sheetId="66" r:id="R85e2ceacdb4944b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-065" sheetId="67" r:id="R5d3b6c216b9045b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-066" sheetId="68" r:id="Rae0df96d86224b62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-067" sheetId="69" r:id="Rfdd6fe93b32c49cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-068" sheetId="71" r:id="R9fb1d91d9c194afb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-069" sheetId="72" r:id="R1b95bd1d58104482"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-070" sheetId="73" r:id="R1d72890d93694eb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-071" sheetId="74" r:id="Rbdb399e23b034d70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-072" sheetId="75" r:id="R57d5303f8bf64bda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-073" sheetId="76" r:id="Rf69e88da60ad4c37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-074" sheetId="77" r:id="R7b1566c3a1de4493"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-075" sheetId="78" r:id="R2eb699157c644fb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-076" sheetId="83" r:id="Rf2a9626065e240d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-077" sheetId="84" r:id="R4c380fea39874dfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-078" sheetId="85" r:id="Rd28fb0f54a4b488f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-079" sheetId="86" r:id="Rfa14d46e4a5c4b48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEL-080" sheetId="87" r:id="Rcde8e1de36944864"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -527,9 +527,6 @@
     <x:t xml:space="preserve">＜データ移送表＞</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">参照テーブル: ユーザーアーカイブ</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">項目</x:t>
   </x:si>
   <x:si>
@@ -738,9 +735,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">COUNT(tb2.注文ID) &gt;= @min_order_count</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">参照テーブル: ユーザー集計</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">表示名</x:t>
@@ -23473,8 +23467,8 @@
       <x:c r="CL8" s="1"/>
     </x:row>
     <x:row r="9" ht="13.5" customHeight="1">
-      <x:c r="A9" s="22" t="s">
-        <x:v>146</x:v>
+      <x:c r="A9" s="22" t="str">
+        <x:v>参照テーブル: ユーザーアーカイブ、ユーザー[tb1]</x:v>
       </x:c>
       <x:c r="B9" s="1"/>
       <x:c r="C9" s="1"/>
@@ -23568,7 +23562,7 @@
     </x:row>
     <x:row r="10" ht="13.5" customHeight="1">
       <x:c r="A10" s="28" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B10" s="16"/>
       <x:c r="C10" s="16"/>
@@ -23588,7 +23582,7 @@
       <x:c r="Q10" s="16"/>
       <x:c r="R10" s="16"/>
       <x:c r="S10" s="28" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="T10" s="16"/>
       <x:c r="U10" s="16"/>
@@ -23608,7 +23602,7 @@
       <x:c r="AI10" s="16"/>
       <x:c r="AJ10" s="16"/>
       <x:c r="AK10" s="28" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="AL10" s="16"/>
       <x:c r="AM10" s="16"/>
@@ -23666,7 +23660,7 @@
     </x:row>
     <x:row r="11" ht="13.5" customHeight="1">
       <x:c r="A11" s="31" t="s">
-        <x:v>150</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="B11" s="14"/>
       <x:c r="C11" s="14"/>
@@ -23762,7 +23756,7 @@
     </x:row>
     <x:row r="12" ht="13.5" customHeight="1">
       <x:c r="A12" s="20" t="s">
-        <x:v>151</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="B12" s="18"/>
       <x:c r="C12" s="18"/>
@@ -23858,7 +23852,7 @@
     </x:row>
     <x:row r="13" ht="13.5" customHeight="1">
       <x:c r="A13" s="20" t="s">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B13" s="18"/>
       <x:c r="C13" s="18"/>
@@ -24172,7 +24166,7 @@
       <x:c r="O3" s="6"/>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>153</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -24268,7 +24262,7 @@
       <x:c r="O4" s="14"/>
       <x:c r="P4" s="14"/>
       <x:c r="Q4" s="30" t="s">
-        <x:v>154</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="R4" s="14"/>
       <x:c r="S4" s="14"/>
@@ -24546,7 +24540,7 @@
     </x:row>
     <x:row r="3" ht="13.5" customHeight="1">
       <x:c r="A3" s="28" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B3" s="16"/>
       <x:c r="C3" s="16"/>
@@ -24566,7 +24560,7 @@
       <x:c r="Q3" s="16"/>
       <x:c r="R3" s="16"/>
       <x:c r="S3" s="28" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="T3" s="16"/>
       <x:c r="U3" s="16"/>
@@ -24586,7 +24580,7 @@
       <x:c r="AI3" s="16"/>
       <x:c r="AJ3" s="16"/>
       <x:c r="AK3" s="28" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="AL3" s="16"/>
       <x:c r="AM3" s="16"/>
@@ -24644,7 +24638,7 @@
     </x:row>
     <x:row r="4" ht="13.5" customHeight="1">
       <x:c r="A4" s="31" t="s">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B4" s="14"/>
       <x:c r="C4" s="14"/>
@@ -24682,7 +24676,7 @@
       <x:c r="AI4" s="14"/>
       <x:c r="AJ4" s="14"/>
       <x:c r="AK4" s="31" t="s">
-        <x:v>155</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="AL4" s="14"/>
       <x:c r="AM4" s="14"/>
@@ -24740,7 +24734,7 @@
     </x:row>
     <x:row r="5" ht="13.5" customHeight="1">
       <x:c r="A5" s="24" t="s">
-        <x:v>156</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="B5" s="6"/>
       <x:c r="C5" s="6"/>
@@ -24778,7 +24772,7 @@
       <x:c r="AI5" s="6"/>
       <x:c r="AJ5" s="6"/>
       <x:c r="AK5" s="24" t="s">
-        <x:v>157</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="AL5" s="6"/>
       <x:c r="AM5" s="6"/>
@@ -25044,7 +25038,7 @@
       <x:c r="O8" s="18"/>
       <x:c r="P8" s="18"/>
       <x:c r="Q8" s="29" t="s">
-        <x:v>158</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="R8" s="18"/>
       <x:c r="S8" s="18"/>
@@ -25228,7 +25222,7 @@
     </x:row>
     <x:row r="2" ht="13.5" customHeight="1">
       <x:c r="A2" s="22" t="s">
-        <x:v>159</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -25344,7 +25338,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>160</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -25442,7 +25436,7 @@
       </x:c>
       <x:c r="P4" s="3"/>
       <x:c r="Q4" s="27" t="s">
-        <x:v>161</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="R4" s="3"/>
       <x:c r="S4" s="3"/>
@@ -25542,7 +25536,7 @@
       </x:c>
       <x:c r="P5" s="18"/>
       <x:c r="Q5" s="29" t="s">
-        <x:v>160</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="R5" s="18"/>
       <x:c r="S5" s="18"/>
@@ -25940,7 +25934,7 @@
       </x:c>
       <x:c r="P4" s="3"/>
       <x:c r="Q4" s="27" t="s">
-        <x:v>162</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="R4" s="3"/>
       <x:c r="S4" s="3"/>
@@ -25959,7 +25953,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF4" s="27" t="s">
-        <x:v>163</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="AG4" s="3"/>
       <x:c r="AH4" s="3"/>
@@ -26055,7 +26049,7 @@
       <x:c r="AF5" s="3"/>
       <x:c r="AG5" s="3"/>
       <x:c r="AH5" s="27" t="s">
-        <x:v>164</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="AI5" s="3"/>
       <x:c r="AJ5" s="3"/>
@@ -26147,7 +26141,7 @@
       <x:c r="AD6" s="3"/>
       <x:c r="AE6" s="3"/>
       <x:c r="AF6" s="27" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="AG6" s="3"/>
       <x:c r="AH6" s="3"/>
@@ -27024,7 +27018,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>166</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -27043,7 +27037,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF3" s="25" t="s">
-        <x:v>167</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="AG3" s="6"/>
       <x:c r="AH3" s="6"/>
@@ -27137,7 +27131,7 @@
       <x:c r="AD4" s="3"/>
       <x:c r="AE4" s="3"/>
       <x:c r="AF4" s="27" t="s">
-        <x:v>168</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="AG4" s="3"/>
       <x:c r="AH4" s="3"/>
@@ -27324,7 +27318,7 @@
       </x:c>
       <x:c r="P6" s="6"/>
       <x:c r="Q6" s="25" t="s">
-        <x:v>166</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="R6" s="6"/>
       <x:c r="S6" s="6"/>
@@ -27343,7 +27337,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF6" s="25" t="s">
-        <x:v>167</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="AG6" s="6"/>
       <x:c r="AH6" s="6"/>
@@ -27437,7 +27431,7 @@
       <x:c r="AD7" s="14"/>
       <x:c r="AE7" s="14"/>
       <x:c r="AF7" s="30" t="s">
-        <x:v>168</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="AG7" s="14"/>
       <x:c r="AH7" s="14"/>
@@ -28018,7 +28012,7 @@
       </x:c>
       <x:c r="P6" s="6"/>
       <x:c r="Q6" s="25" t="s">
-        <x:v>169</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="R6" s="6"/>
       <x:c r="S6" s="6"/>
@@ -28037,7 +28031,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF6" s="25" t="s">
-        <x:v>170</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="AG6" s="6"/>
       <x:c r="AH6" s="6"/>
@@ -28131,7 +28125,7 @@
       <x:c r="AD7" s="3"/>
       <x:c r="AE7" s="3"/>
       <x:c r="AF7" s="27" t="s">
-        <x:v>171</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="AG7" s="3"/>
       <x:c r="AH7" s="3"/>
@@ -28225,7 +28219,7 @@
       <x:c r="AD8" s="3"/>
       <x:c r="AE8" s="3"/>
       <x:c r="AF8" s="27" t="s">
-        <x:v>172</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="AG8" s="3"/>
       <x:c r="AH8" s="3"/>
@@ -28804,7 +28798,7 @@
       </x:c>
       <x:c r="P5" s="3"/>
       <x:c r="Q5" s="27" t="s">
-        <x:v>173</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="R5" s="3"/>
       <x:c r="S5" s="3"/>
@@ -28904,7 +28898,7 @@
       </x:c>
       <x:c r="P6" s="6"/>
       <x:c r="Q6" s="25" t="s">
-        <x:v>174</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="R6" s="6"/>
       <x:c r="S6" s="6"/>
@@ -29500,7 +29494,7 @@
       </x:c>
       <x:c r="P5" s="6"/>
       <x:c r="Q5" s="25" t="s">
-        <x:v>175</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="R5" s="6"/>
       <x:c r="S5" s="6"/>
@@ -29598,7 +29592,7 @@
       </x:c>
       <x:c r="R6" s="3"/>
       <x:c r="S6" s="27" t="s">
-        <x:v>176</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="T6" s="3"/>
       <x:c r="U6" s="3"/>
@@ -29790,7 +29784,7 @@
       </x:c>
       <x:c r="R8" s="3"/>
       <x:c r="S8" s="27" t="s">
-        <x:v>177</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="T8" s="3"/>
       <x:c r="U8" s="3"/>
@@ -29888,7 +29882,7 @@
       </x:c>
       <x:c r="T9" s="3"/>
       <x:c r="U9" s="27" t="s">
-        <x:v>178</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="V9" s="3"/>
       <x:c r="W9" s="3"/>
@@ -30170,7 +30164,7 @@
       </x:c>
       <x:c r="P12" s="3"/>
       <x:c r="Q12" s="27" t="s">
-        <x:v>179</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="R12" s="3"/>
       <x:c r="S12" s="3"/>
@@ -30270,7 +30264,7 @@
       </x:c>
       <x:c r="R13" s="3"/>
       <x:c r="S13" s="27" t="s">
-        <x:v>180</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="T13" s="3"/>
       <x:c r="U13" s="3"/>
@@ -30368,7 +30362,7 @@
       </x:c>
       <x:c r="T14" s="3"/>
       <x:c r="U14" s="27" t="s">
-        <x:v>181</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="V14" s="3"/>
       <x:c r="W14" s="3"/>
@@ -30650,7 +30644,7 @@
       </x:c>
       <x:c r="P17" s="3"/>
       <x:c r="Q17" s="27" t="s">
-        <x:v>182</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="R17" s="3"/>
       <x:c r="S17" s="3"/>
@@ -30746,7 +30740,7 @@
       </x:c>
       <x:c r="P18" s="3"/>
       <x:c r="Q18" s="27" t="s">
-        <x:v>183</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="R18" s="3"/>
       <x:c r="S18" s="3"/>
@@ -30930,7 +30924,7 @@
   <x:sheetData>
     <x:row r="1" ht="13.5" customHeight="1">
       <x:c r="A1" s="22" t="s">
-        <x:v>184</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1"/>
@@ -31257,7 +31251,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF4" s="27" t="s">
-        <x:v>185</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="AG4" s="3"/>
       <x:c r="AH4" s="3"/>
@@ -31340,7 +31334,7 @@
       </x:c>
       <x:c r="P5" s="3"/>
       <x:c r="Q5" s="27" t="s">
-        <x:v>186</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="R5" s="3"/>
       <x:c r="S5" s="3"/>
@@ -31359,7 +31353,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF5" s="27" t="s">
-        <x:v>187</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="AG5" s="3"/>
       <x:c r="AH5" s="3"/>
@@ -31440,7 +31434,7 @@
       <x:c r="O6" s="6"/>
       <x:c r="P6" s="6"/>
       <x:c r="Q6" s="25" t="s">
-        <x:v>188</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="R6" s="6"/>
       <x:c r="S6" s="6"/>
@@ -31636,7 +31630,7 @@
       <x:c r="O8" s="18"/>
       <x:c r="P8" s="18"/>
       <x:c r="Q8" s="29" t="s">
-        <x:v>189</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="R8" s="18"/>
       <x:c r="S8" s="18"/>
@@ -31900,7 +31894,7 @@
     </x:row>
     <x:row r="11" ht="13.5" customHeight="1">
       <x:c r="A11" s="22" t="s">
-        <x:v>190</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="B11" s="1"/>
       <x:c r="C11" s="1"/>
@@ -32212,7 +32206,7 @@
       </x:c>
       <x:c r="P14" s="3"/>
       <x:c r="Q14" s="27" t="s">
-        <x:v>191</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="R14" s="3"/>
       <x:c r="S14" s="3"/>
@@ -32310,7 +32304,7 @@
       </x:c>
       <x:c r="P15" s="3"/>
       <x:c r="Q15" s="27" t="s">
-        <x:v>192</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="R15" s="3"/>
       <x:c r="S15" s="3"/>
@@ -32406,7 +32400,7 @@
       <x:c r="O16" s="6"/>
       <x:c r="P16" s="6"/>
       <x:c r="Q16" s="25" t="s">
-        <x:v>193</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="R16" s="6"/>
       <x:c r="S16" s="6"/>
@@ -32500,7 +32494,7 @@
       <x:c r="O17" s="3"/>
       <x:c r="P17" s="3"/>
       <x:c r="Q17" s="27" t="s">
-        <x:v>194</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="R17" s="3"/>
       <x:c r="S17" s="3"/>
@@ -32596,7 +32590,7 @@
       <x:c r="O18" s="3"/>
       <x:c r="P18" s="3"/>
       <x:c r="Q18" s="27" t="s">
-        <x:v>195</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="R18" s="3"/>
       <x:c r="S18" s="3"/>
@@ -32792,7 +32786,7 @@
       </x:c>
       <x:c r="P20" s="18"/>
       <x:c r="Q20" s="29" t="s">
-        <x:v>196</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="R20" s="18"/>
       <x:c r="S20" s="18"/>
@@ -32976,7 +32970,7 @@
     </x:row>
     <x:row r="2" ht="13.5" customHeight="1">
       <x:c r="A2" s="22" t="s">
-        <x:v>197</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -33092,7 +33086,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>198</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -33188,7 +33182,7 @@
       <x:c r="O4" s="18"/>
       <x:c r="P4" s="18"/>
       <x:c r="Q4" s="29" t="s">
-        <x:v>199</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="R4" s="18"/>
       <x:c r="S4" s="18"/>
@@ -33358,7 +33352,7 @@
     </x:row>
     <x:row r="6" ht="13.5" customHeight="1">
       <x:c r="A6" s="22" t="s">
-        <x:v>200</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="B6" s="1"/>
       <x:c r="C6" s="1"/>
@@ -33452,7 +33446,7 @@
     </x:row>
     <x:row r="7" ht="13.5" customHeight="1">
       <x:c r="A7" s="22" t="s">
-        <x:v>201</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="B7" s="1"/>
       <x:c r="C7" s="1"/>
@@ -33568,7 +33562,7 @@
       </x:c>
       <x:c r="P8" s="6"/>
       <x:c r="Q8" s="25" t="s">
-        <x:v>202</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="R8" s="6"/>
       <x:c r="S8" s="6"/>
@@ -33664,7 +33658,7 @@
       <x:c r="O9" s="6"/>
       <x:c r="P9" s="6"/>
       <x:c r="Q9" s="25" t="s">
-        <x:v>203</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="R9" s="6"/>
       <x:c r="S9" s="6"/>
@@ -33760,7 +33754,7 @@
       <x:c r="O10" s="14"/>
       <x:c r="P10" s="14"/>
       <x:c r="Q10" s="30" t="s">
-        <x:v>204</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="R10" s="14"/>
       <x:c r="S10" s="14"/>
@@ -34024,7 +34018,7 @@
     </x:row>
     <x:row r="13" ht="13.5" customHeight="1">
       <x:c r="A13" s="22" t="s">
-        <x:v>205</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="B13" s="1"/>
       <x:c r="C13" s="1"/>
@@ -34334,7 +34328,7 @@
       <x:c r="O16" s="18"/>
       <x:c r="P16" s="18"/>
       <x:c r="Q16" s="29" t="s">
-        <x:v>206</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="R16" s="18"/>
       <x:c r="S16" s="18"/>
@@ -34732,7 +34726,7 @@
       </x:c>
       <x:c r="P4" s="3"/>
       <x:c r="Q4" s="27" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="R4" s="3"/>
       <x:c r="S4" s="3"/>
@@ -34751,7 +34745,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF4" s="27" t="s">
-        <x:v>208</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="AG4" s="3"/>
       <x:c r="AH4" s="3"/>
@@ -34853,7 +34847,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF5" s="27" t="s">
-        <x:v>209</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="AG5" s="3"/>
       <x:c r="AH5" s="3"/>
@@ -34936,7 +34930,7 @@
       </x:c>
       <x:c r="P6" s="3"/>
       <x:c r="Q6" s="27" t="s">
-        <x:v>210</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="R6" s="3"/>
       <x:c r="S6" s="3"/>
@@ -35034,7 +35028,7 @@
       </x:c>
       <x:c r="P7" s="3"/>
       <x:c r="Q7" s="27" t="s">
-        <x:v>211</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="R7" s="3"/>
       <x:c r="S7" s="3"/>
@@ -35320,7 +35314,7 @@
       <x:c r="O10" s="3"/>
       <x:c r="P10" s="3"/>
       <x:c r="Q10" s="27" t="s">
-        <x:v>212</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="R10" s="3"/>
       <x:c r="S10" s="3"/>
@@ -35600,7 +35594,7 @@
       <x:c r="E13" s="2"/>
       <x:c r="F13" s="2"/>
       <x:c r="G13" s="26" t="s">
-        <x:v>213</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="H13" s="3"/>
       <x:c r="I13" s="3"/>
@@ -35698,7 +35692,7 @@
       <x:c r="E14" s="2"/>
       <x:c r="F14" s="2"/>
       <x:c r="G14" s="26" t="s">
-        <x:v>214</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="H14" s="3"/>
       <x:c r="I14" s="3"/>
@@ -35712,7 +35706,7 @@
       </x:c>
       <x:c r="P14" s="3"/>
       <x:c r="Q14" s="27" t="s">
-        <x:v>215</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="R14" s="3"/>
       <x:c r="S14" s="3"/>
@@ -35808,7 +35802,7 @@
       <x:c r="O15" s="18"/>
       <x:c r="P15" s="18"/>
       <x:c r="Q15" s="29" t="s">
-        <x:v>216</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="R15" s="18"/>
       <x:c r="S15" s="18"/>
@@ -36071,8 +36065,8 @@
       <x:c r="CL17" s="1"/>
     </x:row>
     <x:row r="18" ht="13.5" customHeight="1">
-      <x:c r="A18" s="22" t="s">
-        <x:v>217</x:v>
+      <x:c r="A18" s="22" t="str">
+        <x:v>参照テーブル: ユーザー集計、ユーザー[tb1]、注文[tb2]</x:v>
       </x:c>
       <x:c r="B18" s="1"/>
       <x:c r="C18" s="1"/>
@@ -36166,7 +36160,7 @@
     </x:row>
     <x:row r="19" ht="13.5" customHeight="1">
       <x:c r="A19" s="28" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B19" s="16"/>
       <x:c r="C19" s="16"/>
@@ -36186,7 +36180,7 @@
       <x:c r="Q19" s="16"/>
       <x:c r="R19" s="16"/>
       <x:c r="S19" s="28" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="T19" s="16"/>
       <x:c r="U19" s="16"/>
@@ -36206,7 +36200,7 @@
       <x:c r="AI19" s="16"/>
       <x:c r="AJ19" s="16"/>
       <x:c r="AK19" s="28" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="AL19" s="16"/>
       <x:c r="AM19" s="16"/>
@@ -36264,7 +36258,7 @@
     </x:row>
     <x:row r="20" ht="13.5" customHeight="1">
       <x:c r="A20" s="31" t="s">
-        <x:v>150</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="B20" s="14"/>
       <x:c r="C20" s="14"/>
@@ -36360,7 +36354,7 @@
     </x:row>
     <x:row r="21" ht="13.5" customHeight="1">
       <x:c r="A21" s="20" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="B21" s="18"/>
       <x:c r="C21" s="18"/>
@@ -36380,7 +36374,7 @@
       <x:c r="Q21" s="18"/>
       <x:c r="R21" s="18"/>
       <x:c r="S21" s="20" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="T21" s="18"/>
       <x:c r="U21" s="18"/>
@@ -36400,7 +36394,7 @@
       <x:c r="AI21" s="18"/>
       <x:c r="AJ21" s="18"/>
       <x:c r="AK21" s="17" t="s">
-        <x:v>208</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="AL21" s="18"/>
       <x:c r="AM21" s="18"/>
@@ -36458,7 +36452,7 @@
     </x:row>
     <x:row r="22" ht="13.5" customHeight="1">
       <x:c r="A22" s="20" t="s">
-        <x:v>220</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="B22" s="18"/>
       <x:c r="C22" s="18"/>
@@ -36498,7 +36492,7 @@
       <x:c r="AI22" s="18"/>
       <x:c r="AJ22" s="18"/>
       <x:c r="AK22" s="17" t="s">
-        <x:v>209</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="AL22" s="18"/>
       <x:c r="AM22" s="18"/>
@@ -36556,7 +36550,7 @@
     </x:row>
     <x:row r="23" ht="13.5" customHeight="1">
       <x:c r="A23" s="20" t="s">
-        <x:v>221</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="B23" s="18"/>
       <x:c r="C23" s="18"/>
@@ -36594,7 +36588,7 @@
       <x:c r="AI23" s="18"/>
       <x:c r="AJ23" s="18"/>
       <x:c r="AK23" s="20" t="s">
-        <x:v>210</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="AL23" s="18"/>
       <x:c r="AM23" s="18"/>
@@ -36652,7 +36646,7 @@
     </x:row>
     <x:row r="24" ht="13.5" customHeight="1">
       <x:c r="A24" s="20" t="s">
-        <x:v>222</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="B24" s="18"/>
       <x:c r="C24" s="18"/>
@@ -36690,7 +36684,7 @@
       <x:c r="AI24" s="18"/>
       <x:c r="AJ24" s="18"/>
       <x:c r="AK24" s="20" t="s">
-        <x:v>211</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="AL24" s="18"/>
       <x:c r="AM24" s="18"/>
@@ -37262,7 +37256,7 @@
       <x:c r="O6" s="6"/>
       <x:c r="P6" s="6"/>
       <x:c r="Q6" s="25" t="s">
-        <x:v>223</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="R6" s="6"/>
       <x:c r="S6" s="6"/>
@@ -37379,7 +37373,7 @@
       </x:c>
       <x:c r="AG7" s="3"/>
       <x:c r="AH7" s="27" t="s">
-        <x:v>224</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="AI7" s="3"/>
       <x:c r="AJ7" s="3"/>
@@ -37473,7 +37467,7 @@
       <x:c r="AF8" s="3"/>
       <x:c r="AG8" s="3"/>
       <x:c r="AH8" s="27" t="s">
-        <x:v>177</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="AI8" s="3"/>
       <x:c r="AJ8" s="3"/>
@@ -37569,7 +37563,7 @@
       </x:c>
       <x:c r="AG9" s="3"/>
       <x:c r="AH9" s="27" t="s">
-        <x:v>225</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="AI9" s="3"/>
       <x:c r="AJ9" s="3"/>
@@ -37661,7 +37655,7 @@
       <x:c r="AD10" s="14"/>
       <x:c r="AE10" s="14"/>
       <x:c r="AF10" s="30" t="s">
-        <x:v>226</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="AG10" s="14"/>
       <x:c r="AH10" s="14"/>
@@ -37924,7 +37918,7 @@
     </x:row>
     <x:row r="3" ht="13.5" customHeight="1">
       <x:c r="A3" s="23" t="s">
-        <x:v>227</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="B3" s="4"/>
       <x:c r="C3" s="4"/>
@@ -37932,7 +37926,7 @@
       <x:c r="E3" s="4"/>
       <x:c r="F3" s="4"/>
       <x:c r="G3" s="24" t="s">
-        <x:v>228</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="H3" s="6"/>
       <x:c r="I3" s="6"/>
@@ -38540,7 +38534,7 @@
       </x:c>
       <x:c r="P4" s="14"/>
       <x:c r="Q4" s="30" t="s">
-        <x:v>215</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="R4" s="14"/>
       <x:c r="S4" s="14"/>
@@ -38898,7 +38892,7 @@
     </x:row>
     <x:row r="8" ht="13.5" customHeight="1">
       <x:c r="A8" s="28" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B8" s="16"/>
       <x:c r="C8" s="16"/>
@@ -38918,7 +38912,7 @@
       <x:c r="Q8" s="16"/>
       <x:c r="R8" s="16"/>
       <x:c r="S8" s="28" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="T8" s="16"/>
       <x:c r="U8" s="16"/>
@@ -38938,7 +38932,7 @@
       <x:c r="AI8" s="16"/>
       <x:c r="AJ8" s="16"/>
       <x:c r="AK8" s="28" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="AL8" s="16"/>
       <x:c r="AM8" s="16"/>
@@ -38996,7 +38990,7 @@
     </x:row>
     <x:row r="9" ht="13.5" customHeight="1">
       <x:c r="A9" s="31" t="s">
-        <x:v>150</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="B9" s="14"/>
       <x:c r="C9" s="14"/>
@@ -39092,7 +39086,7 @@
     </x:row>
     <x:row r="10" ht="13.5" customHeight="1">
       <x:c r="A10" s="20" t="s">
-        <x:v>229</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="B10" s="18"/>
       <x:c r="C10" s="18"/>
@@ -39112,7 +39106,7 @@
       <x:c r="Q10" s="18"/>
       <x:c r="R10" s="18"/>
       <x:c r="S10" s="20" t="s">
-        <x:v>215</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="T10" s="18"/>
       <x:c r="U10" s="18"/>
@@ -39890,7 +39884,7 @@
     </x:row>
     <x:row r="2" ht="13.5" customHeight="1">
       <x:c r="A2" s="22" t="s">
-        <x:v>230</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -39984,7 +39978,7 @@
     </x:row>
     <x:row r="3" ht="13.5" customHeight="1">
       <x:c r="A3" s="28" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B3" s="16"/>
       <x:c r="C3" s="16"/>
@@ -40004,7 +39998,7 @@
       <x:c r="Q3" s="16"/>
       <x:c r="R3" s="16"/>
       <x:c r="S3" s="28" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="T3" s="16"/>
       <x:c r="U3" s="16"/>
@@ -40024,7 +40018,7 @@
       <x:c r="AI3" s="16"/>
       <x:c r="AJ3" s="16"/>
       <x:c r="AK3" s="28" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="AL3" s="16"/>
       <x:c r="AM3" s="16"/>
@@ -40082,7 +40076,7 @@
     </x:row>
     <x:row r="4" ht="13.5" customHeight="1">
       <x:c r="A4" s="31" t="s">
-        <x:v>150</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="B4" s="14"/>
       <x:c r="C4" s="14"/>
@@ -40120,7 +40114,7 @@
       <x:c r="AI4" s="14"/>
       <x:c r="AJ4" s="14"/>
       <x:c r="AK4" s="31" t="s">
-        <x:v>231</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="AL4" s="14"/>
       <x:c r="AM4" s="14"/>
@@ -40178,7 +40172,7 @@
     </x:row>
     <x:row r="5" ht="13.5" customHeight="1">
       <x:c r="A5" s="20" t="s">
-        <x:v>151</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="B5" s="18"/>
       <x:c r="C5" s="18"/>
@@ -40216,7 +40210,7 @@
       <x:c r="AI5" s="18"/>
       <x:c r="AJ5" s="18"/>
       <x:c r="AK5" s="20" t="s">
-        <x:v>232</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="AL5" s="18"/>
       <x:c r="AM5" s="18"/>
@@ -40274,7 +40268,7 @@
     </x:row>
     <x:row r="6" ht="13.5" customHeight="1">
       <x:c r="A6" s="20" t="s">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B6" s="18"/>
       <x:c r="C6" s="18"/>
@@ -40312,7 +40306,7 @@
       <x:c r="AI6" s="18"/>
       <x:c r="AJ6" s="18"/>
       <x:c r="AK6" s="20" t="s">
-        <x:v>233</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="AL6" s="18"/>
       <x:c r="AM6" s="18"/>
@@ -40370,7 +40364,7 @@
     </x:row>
     <x:row r="7" ht="13.5" customHeight="1">
       <x:c r="A7" s="20" t="s">
-        <x:v>221</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="B7" s="18"/>
       <x:c r="C7" s="18"/>
@@ -40408,7 +40402,7 @@
       <x:c r="AI7" s="18"/>
       <x:c r="AJ7" s="18"/>
       <x:c r="AK7" s="20" t="s">
-        <x:v>157</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="AL7" s="18"/>
       <x:c r="AM7" s="18"/>
@@ -40786,7 +40780,7 @@
       </x:c>
       <x:c r="P4" s="3"/>
       <x:c r="Q4" s="27" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="R4" s="3"/>
       <x:c r="S4" s="3"/>
@@ -40805,7 +40799,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF4" s="27" t="s">
-        <x:v>208</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="AG4" s="3"/>
       <x:c r="AH4" s="3"/>
@@ -40907,7 +40901,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF5" s="27" t="s">
-        <x:v>209</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="AG5" s="3"/>
       <x:c r="AH5" s="3"/>
@@ -40990,7 +40984,7 @@
       </x:c>
       <x:c r="P6" s="3"/>
       <x:c r="Q6" s="27" t="s">
-        <x:v>234</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="R6" s="3"/>
       <x:c r="S6" s="3"/>
@@ -41009,7 +41003,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF6" s="27" t="s">
-        <x:v>235</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="AG6" s="3"/>
       <x:c r="AH6" s="3"/>
@@ -41103,7 +41097,7 @@
       <x:c r="AD7" s="3"/>
       <x:c r="AE7" s="3"/>
       <x:c r="AF7" s="27" t="s">
-        <x:v>236</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="AG7" s="3"/>
       <x:c r="AH7" s="3"/>
@@ -41197,7 +41191,7 @@
       <x:c r="AD8" s="3"/>
       <x:c r="AE8" s="3"/>
       <x:c r="AF8" s="27" t="s">
-        <x:v>237</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="AG8" s="3"/>
       <x:c r="AH8" s="3"/>
@@ -41280,7 +41274,7 @@
       </x:c>
       <x:c r="P9" s="3"/>
       <x:c r="Q9" s="27" t="s">
-        <x:v>238</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="R9" s="3"/>
       <x:c r="S9" s="3"/>
@@ -41299,7 +41293,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF9" s="27" t="s">
-        <x:v>210</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="AG9" s="3"/>
       <x:c r="AH9" s="3"/>
@@ -41368,7 +41362,7 @@
       <x:c r="E10" s="2"/>
       <x:c r="F10" s="2"/>
       <x:c r="G10" s="26" t="s">
-        <x:v>239</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="H10" s="3"/>
       <x:c r="I10" s="3"/>
@@ -41382,7 +41376,7 @@
       </x:c>
       <x:c r="P10" s="3"/>
       <x:c r="Q10" s="27" t="s">
-        <x:v>240</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="R10" s="3"/>
       <x:c r="S10" s="3"/>
@@ -41401,7 +41395,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF10" s="27" t="s">
-        <x:v>211</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="AG10" s="3"/>
       <x:c r="AH10" s="3"/>
@@ -41672,7 +41666,7 @@
       <x:c r="O13" s="3"/>
       <x:c r="P13" s="3"/>
       <x:c r="Q13" s="27" t="s">
-        <x:v>212</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="R13" s="3"/>
       <x:c r="S13" s="3"/>
@@ -41952,7 +41946,7 @@
       <x:c r="E16" s="2"/>
       <x:c r="F16" s="2"/>
       <x:c r="G16" s="26" t="s">
-        <x:v>213</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="H16" s="3"/>
       <x:c r="I16" s="3"/>
@@ -42050,7 +42044,7 @@
       <x:c r="E17" s="2"/>
       <x:c r="F17" s="2"/>
       <x:c r="G17" s="26" t="s">
-        <x:v>214</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="H17" s="3"/>
       <x:c r="I17" s="3"/>
@@ -42064,7 +42058,7 @@
       </x:c>
       <x:c r="P17" s="3"/>
       <x:c r="Q17" s="27" t="s">
-        <x:v>215</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="R17" s="3"/>
       <x:c r="S17" s="3"/>
@@ -42160,7 +42154,7 @@
       <x:c r="O18" s="18"/>
       <x:c r="P18" s="18"/>
       <x:c r="Q18" s="29" t="s">
-        <x:v>216</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="R18" s="18"/>
       <x:c r="S18" s="18"/>
@@ -42518,7 +42512,7 @@
     </x:row>
     <x:row r="22" ht="13.5" customHeight="1">
       <x:c r="A22" s="28" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B22" s="16"/>
       <x:c r="C22" s="16"/>
@@ -42538,7 +42532,7 @@
       <x:c r="Q22" s="16"/>
       <x:c r="R22" s="16"/>
       <x:c r="S22" s="28" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="T22" s="16"/>
       <x:c r="U22" s="16"/>
@@ -42558,7 +42552,7 @@
       <x:c r="AI22" s="16"/>
       <x:c r="AJ22" s="16"/>
       <x:c r="AK22" s="28" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="AL22" s="16"/>
       <x:c r="AM22" s="16"/>
@@ -42616,7 +42610,7 @@
     </x:row>
     <x:row r="23" ht="13.5" customHeight="1">
       <x:c r="A23" s="31" t="s">
-        <x:v>150</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="B23" s="14"/>
       <x:c r="C23" s="14"/>
@@ -42712,7 +42706,7 @@
     </x:row>
     <x:row r="24" ht="13.5" customHeight="1">
       <x:c r="A24" s="20" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="B24" s="18"/>
       <x:c r="C24" s="18"/>
@@ -42732,7 +42726,7 @@
       <x:c r="Q24" s="18"/>
       <x:c r="R24" s="18"/>
       <x:c r="S24" s="20" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="T24" s="18"/>
       <x:c r="U24" s="18"/>
@@ -42752,7 +42746,7 @@
       <x:c r="AI24" s="18"/>
       <x:c r="AJ24" s="18"/>
       <x:c r="AK24" s="17" t="s">
-        <x:v>208</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="AL24" s="18"/>
       <x:c r="AM24" s="18"/>
@@ -42810,7 +42804,7 @@
     </x:row>
     <x:row r="25" ht="13.5" customHeight="1">
       <x:c r="A25" s="20" t="s">
-        <x:v>220</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="B25" s="18"/>
       <x:c r="C25" s="18"/>
@@ -42850,7 +42844,7 @@
       <x:c r="AI25" s="18"/>
       <x:c r="AJ25" s="18"/>
       <x:c r="AK25" s="17" t="s">
-        <x:v>209</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="AL25" s="18"/>
       <x:c r="AM25" s="18"/>
@@ -42908,7 +42902,7 @@
     </x:row>
     <x:row r="26" ht="13.5" customHeight="1">
       <x:c r="A26" s="33" t="s">
-        <x:v>241</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="B26" s="34"/>
       <x:c r="C26" s="34"/>
@@ -42946,7 +42940,7 @@
       <x:c r="AI26" s="42"/>
       <x:c r="AJ26" s="35"/>
       <x:c r="AK26" s="33" t="s">
-        <x:v>169</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="AL26" s="34"/>
       <x:c r="AM26" s="34"/>
@@ -42965,7 +42959,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AZ26" s="34" t="s">
-        <x:v>235</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="BA26" s="34"/>
       <x:c r="BB26" s="34"/>
@@ -43059,7 +43053,7 @@
       <x:c r="AX27" s="37"/>
       <x:c r="AY27" s="37"/>
       <x:c r="AZ27" s="37" t="s">
-        <x:v>236</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="BA27" s="37"/>
       <x:c r="BB27" s="37"/>
@@ -43153,7 +43147,7 @@
       <x:c r="AX28" s="40"/>
       <x:c r="AY28" s="40"/>
       <x:c r="AZ28" s="40" t="s">
-        <x:v>237</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="BA28" s="40"/>
       <x:c r="BB28" s="40"/>
@@ -43196,7 +43190,7 @@
     </x:row>
     <x:row r="29" ht="13.5" customHeight="1">
       <x:c r="A29" s="20" t="s">
-        <x:v>221</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="B29" s="18"/>
       <x:c r="C29" s="18"/>
@@ -43234,7 +43228,7 @@
       <x:c r="AI29" s="18"/>
       <x:c r="AJ29" s="18"/>
       <x:c r="AK29" s="20" t="s">
-        <x:v>210</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="AL29" s="18"/>
       <x:c r="AM29" s="18"/>
@@ -43292,7 +43286,7 @@
     </x:row>
     <x:row r="30" ht="13.5" customHeight="1">
       <x:c r="A30" s="20" t="s">
-        <x:v>222</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="B30" s="18"/>
       <x:c r="C30" s="18"/>
@@ -43330,7 +43324,7 @@
       <x:c r="AI30" s="18"/>
       <x:c r="AJ30" s="18"/>
       <x:c r="AK30" s="20" t="s">
-        <x:v>211</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="AL30" s="18"/>
       <x:c r="AM30" s="18"/>
@@ -43596,7 +43590,7 @@
       <x:c r="E3" s="4"/>
       <x:c r="F3" s="4"/>
       <x:c r="G3" s="24" t="s">
-        <x:v>202</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="H3" s="6"/>
       <x:c r="I3" s="6"/>
@@ -43802,7 +43796,7 @@
       <x:c r="O5" s="6"/>
       <x:c r="P5" s="6"/>
       <x:c r="Q5" s="25" t="s">
-        <x:v>203</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="R5" s="6"/>
       <x:c r="S5" s="6"/>
@@ -43902,7 +43896,7 @@
       </x:c>
       <x:c r="P6" s="18"/>
       <x:c r="Q6" s="29" t="s">
-        <x:v>242</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="R6" s="18"/>
       <x:c r="S6" s="18"/>
@@ -44260,7 +44254,7 @@
     </x:row>
     <x:row r="10" ht="13.5" customHeight="1">
       <x:c r="A10" s="28" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B10" s="16"/>
       <x:c r="C10" s="16"/>
@@ -44280,7 +44274,7 @@
       <x:c r="Q10" s="16"/>
       <x:c r="R10" s="16"/>
       <x:c r="S10" s="28" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="T10" s="16"/>
       <x:c r="U10" s="16"/>
@@ -44300,7 +44294,7 @@
       <x:c r="AI10" s="16"/>
       <x:c r="AJ10" s="16"/>
       <x:c r="AK10" s="28" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="AL10" s="16"/>
       <x:c r="AM10" s="16"/>
@@ -44358,7 +44352,7 @@
     </x:row>
     <x:row r="11" ht="13.5" customHeight="1">
       <x:c r="A11" s="26" t="s">
-        <x:v>243</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="B11" s="3"/>
       <x:c r="C11" s="3"/>
@@ -44378,7 +44372,7 @@
       <x:c r="Q11" s="3"/>
       <x:c r="R11" s="3"/>
       <x:c r="S11" s="26" t="s">
-        <x:v>244</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="T11" s="3"/>
       <x:c r="U11" s="3"/>
@@ -44562,7 +44556,7 @@
   <x:sheetData>
     <x:row r="1" ht="13.5" customHeight="1">
       <x:c r="A1" s="22" t="s">
-        <x:v>184</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1"/>
@@ -44656,7 +44650,7 @@
     </x:row>
     <x:row r="2" ht="13.5" customHeight="1">
       <x:c r="A2" s="22" t="s">
-        <x:v>245</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -44870,7 +44864,7 @@
       </x:c>
       <x:c r="P4" s="3"/>
       <x:c r="Q4" s="27" t="s">
-        <x:v>246</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="R4" s="3"/>
       <x:c r="S4" s="3"/>
@@ -44889,7 +44883,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF4" s="27" t="s">
-        <x:v>247</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="AG4" s="3"/>
       <x:c r="AH4" s="3"/>
@@ -45238,7 +45232,7 @@
     </x:row>
     <x:row r="8" ht="13.5" customHeight="1">
       <x:c r="A8" s="22" t="s">
-        <x:v>190</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="B8" s="1"/>
       <x:c r="C8" s="1"/>
@@ -45332,7 +45326,7 @@
     </x:row>
     <x:row r="9" ht="13.5" customHeight="1">
       <x:c r="A9" s="28" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B9" s="16"/>
       <x:c r="C9" s="16"/>
@@ -45352,7 +45346,7 @@
       <x:c r="Q9" s="16"/>
       <x:c r="R9" s="16"/>
       <x:c r="S9" s="28" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="T9" s="16"/>
       <x:c r="U9" s="16"/>
@@ -45372,7 +45366,7 @@
       <x:c r="AI9" s="16"/>
       <x:c r="AJ9" s="16"/>
       <x:c r="AK9" s="28" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="AL9" s="16"/>
       <x:c r="AM9" s="16"/>
@@ -45430,7 +45424,7 @@
     </x:row>
     <x:row r="10" ht="13.5" customHeight="1">
       <x:c r="A10" s="26" t="s">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B10" s="3"/>
       <x:c r="C10" s="3"/>
@@ -45450,7 +45444,7 @@
       <x:c r="Q10" s="3"/>
       <x:c r="R10" s="3"/>
       <x:c r="S10" s="26" t="s">
-        <x:v>248</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="T10" s="3"/>
       <x:c r="U10" s="3"/>
@@ -45544,7 +45538,7 @@
       <x:c r="O11" s="6"/>
       <x:c r="P11" s="6"/>
       <x:c r="Q11" s="25" t="s">
-        <x:v>193</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="R11" s="6"/>
       <x:c r="S11" s="6"/>
@@ -45638,7 +45632,7 @@
       <x:c r="O12" s="3"/>
       <x:c r="P12" s="3"/>
       <x:c r="Q12" s="27" t="s">
-        <x:v>194</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="R12" s="3"/>
       <x:c r="S12" s="3"/>
@@ -46034,7 +46028,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>202</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -46130,7 +46124,7 @@
       <x:c r="O4" s="18"/>
       <x:c r="P4" s="18"/>
       <x:c r="Q4" s="29" t="s">
-        <x:v>203</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="R4" s="18"/>
       <x:c r="S4" s="18"/>
@@ -46506,7 +46500,7 @@
       <x:c r="O8" s="18"/>
       <x:c r="P8" s="18"/>
       <x:c r="Q8" s="29" t="s">
-        <x:v>249</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="R8" s="18"/>
       <x:c r="S8" s="18"/>
@@ -46690,7 +46684,7 @@
     </x:row>
     <x:row r="2" ht="13.5" customHeight="1">
       <x:c r="A2" s="22" t="s">
-        <x:v>250</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -46806,7 +46800,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>202</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -46902,7 +46896,7 @@
       <x:c r="O4" s="6"/>
       <x:c r="P4" s="6"/>
       <x:c r="Q4" s="25" t="s">
-        <x:v>251</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="R4" s="6"/>
       <x:c r="S4" s="6"/>
@@ -46998,7 +46992,7 @@
       <x:c r="O5" s="14"/>
       <x:c r="P5" s="14"/>
       <x:c r="Q5" s="30" t="s">
-        <x:v>252</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="R5" s="14"/>
       <x:c r="S5" s="14"/>
@@ -47262,7 +47256,7 @@
     </x:row>
     <x:row r="8" ht="13.5" customHeight="1">
       <x:c r="A8" s="22" t="s">
-        <x:v>253</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="B8" s="1"/>
       <x:c r="C8" s="1"/>
@@ -47356,7 +47350,7 @@
     </x:row>
     <x:row r="9" ht="13.5" customHeight="1">
       <x:c r="A9" s="28" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B9" s="16"/>
       <x:c r="C9" s="16"/>
@@ -47376,7 +47370,7 @@
       <x:c r="Q9" s="16"/>
       <x:c r="R9" s="16"/>
       <x:c r="S9" s="28" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="T9" s="16"/>
       <x:c r="U9" s="16"/>
@@ -47396,7 +47390,7 @@
       <x:c r="AI9" s="16"/>
       <x:c r="AJ9" s="16"/>
       <x:c r="AK9" s="28" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="AL9" s="16"/>
       <x:c r="AM9" s="16"/>
@@ -47454,7 +47448,7 @@
     </x:row>
     <x:row r="10" ht="13.5" customHeight="1">
       <x:c r="A10" s="26" t="s">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B10" s="3"/>
       <x:c r="C10" s="3"/>
@@ -47492,7 +47486,7 @@
       <x:c r="AI10" s="3"/>
       <x:c r="AJ10" s="3"/>
       <x:c r="AK10" s="26" t="s">
-        <x:v>254</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="AL10" s="3"/>
       <x:c r="AM10" s="3"/>
@@ -47568,7 +47562,7 @@
       <x:c r="O11" s="18"/>
       <x:c r="P11" s="18"/>
       <x:c r="Q11" s="29" t="s">
-        <x:v>249</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="R11" s="18"/>
       <x:c r="S11" s="18"/>
@@ -47868,7 +47862,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>255</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -47887,7 +47881,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF3" s="25" t="s">
-        <x:v>256</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="AG3" s="6"/>
       <x:c r="AH3" s="6"/>
@@ -47968,7 +47962,7 @@
       <x:c r="O4" s="18"/>
       <x:c r="P4" s="18"/>
       <x:c r="Q4" s="29" t="s">
-        <x:v>203</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="R4" s="18"/>
       <x:c r="S4" s="18"/>
@@ -48326,7 +48320,7 @@
     </x:row>
     <x:row r="8" ht="13.5" customHeight="1">
       <x:c r="A8" s="28" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B8" s="16"/>
       <x:c r="C8" s="16"/>
@@ -48346,7 +48340,7 @@
       <x:c r="Q8" s="16"/>
       <x:c r="R8" s="16"/>
       <x:c r="S8" s="28" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="T8" s="16"/>
       <x:c r="U8" s="16"/>
@@ -48366,7 +48360,7 @@
       <x:c r="AI8" s="16"/>
       <x:c r="AJ8" s="16"/>
       <x:c r="AK8" s="28" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="AL8" s="16"/>
       <x:c r="AM8" s="16"/>
@@ -48424,7 +48418,7 @@
     </x:row>
     <x:row r="9" ht="13.5" customHeight="1">
       <x:c r="A9" s="26" t="s">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B9" s="3"/>
       <x:c r="C9" s="3"/>
@@ -48462,7 +48456,7 @@
       <x:c r="AI9" s="3"/>
       <x:c r="AJ9" s="3"/>
       <x:c r="AK9" s="26" t="s">
-        <x:v>257</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="AL9" s="3"/>
       <x:c r="AM9" s="3"/>
@@ -48538,7 +48532,7 @@
       <x:c r="O10" s="18"/>
       <x:c r="P10" s="18"/>
       <x:c r="Q10" s="29" t="s">
-        <x:v>258</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="R10" s="18"/>
       <x:c r="S10" s="18"/>
@@ -48934,7 +48928,7 @@
       <x:c r="O4" s="18"/>
       <x:c r="P4" s="18"/>
       <x:c r="Q4" s="29" t="s">
-        <x:v>259</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="R4" s="18"/>
       <x:c r="S4" s="18"/>
@@ -49292,7 +49286,7 @@
     </x:row>
     <x:row r="8" ht="13.5" customHeight="1">
       <x:c r="A8" s="28" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B8" s="16"/>
       <x:c r="C8" s="16"/>
@@ -49312,7 +49306,7 @@
       <x:c r="Q8" s="16"/>
       <x:c r="R8" s="16"/>
       <x:c r="S8" s="28" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="T8" s="16"/>
       <x:c r="U8" s="16"/>
@@ -49332,7 +49326,7 @@
       <x:c r="AI8" s="16"/>
       <x:c r="AJ8" s="16"/>
       <x:c r="AK8" s="28" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="AL8" s="16"/>
       <x:c r="AM8" s="16"/>
@@ -49390,7 +49384,7 @@
     </x:row>
     <x:row r="9" ht="13.5" customHeight="1">
       <x:c r="A9" s="26" t="s">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B9" s="3"/>
       <x:c r="C9" s="3"/>
@@ -49428,7 +49422,7 @@
       <x:c r="AI9" s="3"/>
       <x:c r="AJ9" s="3"/>
       <x:c r="AK9" s="26" t="s">
-        <x:v>260</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="AL9" s="3"/>
       <x:c r="AM9" s="3"/>
@@ -49804,7 +49798,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>261</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -49823,7 +49817,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF3" s="25" t="s">
-        <x:v>262</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="AG3" s="6"/>
       <x:c r="AH3" s="25"/>
@@ -49833,7 +49827,7 @@
       <x:c r="AL3" s="6"/>
       <x:c r="AM3" s="6"/>
       <x:c r="AN3" s="6" t="s">
-        <x:v>263</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="AO3" s="6"/>
       <x:c r="AP3" s="6"/>
@@ -49927,7 +49921,7 @@
       <x:c r="AL4" s="14"/>
       <x:c r="AM4" s="14"/>
       <x:c r="AN4" s="14" t="s">
-        <x:v>226</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="AO4" s="14"/>
       <x:c r="AP4" s="14"/>
@@ -50204,7 +50198,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>264</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -50223,7 +50217,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF3" s="25" t="s">
-        <x:v>265</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="AG3" s="6"/>
       <x:c r="AH3" s="6"/>
@@ -50317,7 +50311,7 @@
       <x:c r="AD4" s="3"/>
       <x:c r="AE4" s="3"/>
       <x:c r="AF4" s="27" t="s">
-        <x:v>266</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="AG4" s="3"/>
       <x:c r="AH4" s="3"/>
@@ -50413,7 +50407,7 @@
       <x:c r="AF5" s="14"/>
       <x:c r="AG5" s="14"/>
       <x:c r="AH5" s="30" t="s">
-        <x:v>267</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="AI5" s="14"/>
       <x:c r="AJ5" s="14"/>
@@ -51382,7 +51376,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>268</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -51403,7 +51397,7 @@
       <x:c r="AF3" s="6"/>
       <x:c r="AG3" s="6"/>
       <x:c r="AH3" s="25" t="s">
-        <x:v>269</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="AI3" s="6"/>
       <x:c r="AJ3" s="6"/>
@@ -51499,7 +51493,7 @@
       </x:c>
       <x:c r="AG4" s="3"/>
       <x:c r="AH4" s="27" t="s">
-        <x:v>270</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="AI4" s="3"/>
       <x:c r="AJ4" s="3"/>
@@ -51591,7 +51585,7 @@
       <x:c r="AD5" s="14"/>
       <x:c r="AE5" s="14"/>
       <x:c r="AF5" s="30" t="s">
-        <x:v>226</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="AG5" s="14"/>
       <x:c r="AH5" s="14"/>
@@ -51854,7 +51848,7 @@
     </x:row>
     <x:row r="3" ht="13.5" customHeight="1">
       <x:c r="A3" s="23" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B3" s="4"/>
       <x:c r="C3" s="4"/>
@@ -51874,7 +51868,7 @@
       <x:c r="Q3" s="4"/>
       <x:c r="R3" s="4"/>
       <x:c r="S3" s="23" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="T3" s="4"/>
       <x:c r="U3" s="4"/>
@@ -51894,7 +51888,7 @@
       <x:c r="AI3" s="4"/>
       <x:c r="AJ3" s="4"/>
       <x:c r="AK3" s="23" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="AL3" s="4"/>
       <x:c r="AM3" s="4"/>
@@ -51952,7 +51946,7 @@
     </x:row>
     <x:row r="4" ht="13.5" customHeight="1">
       <x:c r="A4" s="24" t="s">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B4" s="6"/>
       <x:c r="C4" s="6"/>
@@ -51990,7 +51984,7 @@
       <x:c r="AI4" s="6"/>
       <x:c r="AJ4" s="6"/>
       <x:c r="AK4" s="24" t="s">
-        <x:v>169</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="AL4" s="6"/>
       <x:c r="AM4" s="6"/>
@@ -52011,7 +52005,7 @@
       <x:c r="AZ4" s="6"/>
       <x:c r="BA4" s="6"/>
       <x:c r="BB4" s="25" t="s">
-        <x:v>178</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="BC4" s="6"/>
       <x:c r="BD4" s="6"/>
@@ -52107,7 +52101,7 @@
       </x:c>
       <x:c r="BA5" s="3"/>
       <x:c r="BB5" s="27" t="s">
-        <x:v>271</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="BC5" s="3"/>
       <x:c r="BD5" s="3"/>
@@ -52199,7 +52193,7 @@
       <x:c r="AX6" s="14"/>
       <x:c r="AY6" s="14"/>
       <x:c r="AZ6" s="30" t="s">
-        <x:v>272</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="BA6" s="14"/>
       <x:c r="BB6" s="14"/>
@@ -52348,7 +52342,7 @@
     </x:row>
     <x:row r="2" ht="13.5" customHeight="1">
       <x:c r="A2" s="22" t="s">
-        <x:v>230</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -52442,7 +52436,7 @@
     </x:row>
     <x:row r="3" ht="13.5" customHeight="1">
       <x:c r="A3" s="23" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B3" s="4"/>
       <x:c r="C3" s="4"/>
@@ -52462,7 +52456,7 @@
       <x:c r="Q3" s="4"/>
       <x:c r="R3" s="4"/>
       <x:c r="S3" s="23" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="T3" s="4"/>
       <x:c r="U3" s="4"/>
@@ -52482,7 +52476,7 @@
       <x:c r="AI3" s="4"/>
       <x:c r="AJ3" s="4"/>
       <x:c r="AK3" s="23" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="AL3" s="4"/>
       <x:c r="AM3" s="4"/>
@@ -52540,7 +52534,7 @@
     </x:row>
     <x:row r="4" ht="13.5" customHeight="1">
       <x:c r="A4" s="24" t="s">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B4" s="6"/>
       <x:c r="C4" s="6"/>
@@ -52578,7 +52572,7 @@
       <x:c r="AI4" s="6"/>
       <x:c r="AJ4" s="6"/>
       <x:c r="AK4" s="24" t="s">
-        <x:v>169</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="AL4" s="6"/>
       <x:c r="AM4" s="6"/>
@@ -52597,7 +52591,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AZ4" s="25" t="s">
-        <x:v>273</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="BA4" s="6"/>
       <x:c r="BB4" s="6"/>
@@ -52691,7 +52685,7 @@
       <x:c r="AX5" s="14"/>
       <x:c r="AY5" s="14"/>
       <x:c r="AZ5" s="30" t="s">
-        <x:v>272</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="BA5" s="14"/>
       <x:c r="BB5" s="14"/>
@@ -52942,7 +52936,7 @@
       <x:c r="E3" s="4"/>
       <x:c r="F3" s="4"/>
       <x:c r="G3" s="24" t="s">
-        <x:v>169</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="H3" s="6"/>
       <x:c r="I3" s="6"/>
@@ -52956,7 +52950,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>274</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -53050,7 +53044,7 @@
       <x:c r="O4" s="3"/>
       <x:c r="P4" s="3"/>
       <x:c r="Q4" s="27" t="s">
-        <x:v>275</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="R4" s="3"/>
       <x:c r="S4" s="3"/>
@@ -54412,7 +54406,7 @@
       </x:c>
       <x:c r="P3" s="6"/>
       <x:c r="Q3" s="25" t="s">
-        <x:v>169</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="R3" s="6"/>
       <x:c r="S3" s="6"/>
@@ -54431,7 +54425,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF3" s="25" t="s">
-        <x:v>276</x:v>
+        <x:v>274</x:v>
       </x:c>
       <x:c r="AG3" s="6"/>
       <x:c r="AH3" s="6"/>
@@ -54525,7 +54519,7 @@
       <x:c r="AD4" s="14"/>
       <x:c r="AE4" s="14"/>
       <x:c r="AF4" s="30" t="s">
-        <x:v>226</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="AG4" s="14"/>
       <x:c r="AH4" s="14"/>
@@ -54694,7 +54688,7 @@
     </x:row>
     <x:row r="2" ht="13.5" customHeight="1">
       <x:c r="A2" s="1" t="s">
-        <x:v>230</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -54788,7 +54782,7 @@
     </x:row>
     <x:row r="3" ht="13.5" customHeight="1">
       <x:c r="A3" s="61" t="s">
-        <x:v>277</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="B3" s="61"/>
       <x:c r="C3" s="61"/>
@@ -54882,7 +54876,7 @@
     </x:row>
     <x:row r="4" ht="13.5" customHeight="1">
       <x:c r="A4" s="50" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B4" s="51"/>
       <x:c r="C4" s="51"/>
@@ -54902,7 +54896,7 @@
       <x:c r="Q4" s="51"/>
       <x:c r="R4" s="51"/>
       <x:c r="S4" s="50" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="T4" s="51"/>
       <x:c r="U4" s="51"/>
@@ -54922,7 +54916,7 @@
       <x:c r="AI4" s="51"/>
       <x:c r="AJ4" s="51"/>
       <x:c r="AK4" s="50" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="AL4" s="51"/>
       <x:c r="AM4" s="51"/>
@@ -54980,7 +54974,7 @@
     </x:row>
     <x:row r="5" ht="13.5" customHeight="1">
       <x:c r="A5" s="47" t="s">
-        <x:v>150</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="B5" s="48"/>
       <x:c r="C5" s="48"/>
@@ -55018,7 +55012,7 @@
       <x:c r="AI5" s="48"/>
       <x:c r="AJ5" s="48"/>
       <x:c r="AK5" s="47" t="s">
-        <x:v>278</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="AL5" s="48"/>
       <x:c r="AM5" s="48"/>
@@ -55076,7 +55070,7 @@
     </x:row>
     <x:row r="6" ht="13.5" customHeight="1">
       <x:c r="A6" s="47" t="s">
-        <x:v>151</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="B6" s="48"/>
       <x:c r="C6" s="48"/>
@@ -55114,7 +55108,7 @@
       <x:c r="AI6" s="48"/>
       <x:c r="AJ6" s="48"/>
       <x:c r="AK6" s="47" t="s">
-        <x:v>279</x:v>
+        <x:v>277</x:v>
       </x:c>
       <x:c r="AL6" s="48"/>
       <x:c r="AM6" s="48"/>
@@ -55172,7 +55166,7 @@
     </x:row>
     <x:row r="7" ht="13.5" customHeight="1">
       <x:c r="A7" s="47" t="s">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B7" s="48"/>
       <x:c r="C7" s="48"/>
@@ -55210,7 +55204,7 @@
       <x:c r="AI7" s="48"/>
       <x:c r="AJ7" s="48"/>
       <x:c r="AK7" s="47" t="s">
-        <x:v>233</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="AL7" s="48"/>
       <x:c r="AM7" s="48"/>
@@ -55268,7 +55262,7 @@
     </x:row>
     <x:row r="8" ht="13.5" customHeight="1">
       <x:c r="A8" s="47" t="s">
-        <x:v>221</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="B8" s="48"/>
       <x:c r="C8" s="48"/>
@@ -55306,7 +55300,7 @@
       <x:c r="AI8" s="48"/>
       <x:c r="AJ8" s="48"/>
       <x:c r="AK8" s="47" t="s">
-        <x:v>157</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="AL8" s="48"/>
       <x:c r="AM8" s="48"/>
@@ -55364,7 +55358,7 @@
     </x:row>
     <x:row r="9" ht="13.5" customHeight="1">
       <x:c r="A9" s="46" t="s">
-        <x:v>280</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="B9" s="46"/>
       <x:c r="C9" s="46"/>
@@ -55458,7 +55452,7 @@
     </x:row>
     <x:row r="10" ht="13.5" customHeight="1">
       <x:c r="A10" s="50" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B10" s="51"/>
       <x:c r="C10" s="51"/>
@@ -55478,7 +55472,7 @@
       <x:c r="Q10" s="51"/>
       <x:c r="R10" s="51"/>
       <x:c r="S10" s="50" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="T10" s="51"/>
       <x:c r="U10" s="51"/>
@@ -55498,7 +55492,7 @@
       <x:c r="AI10" s="51"/>
       <x:c r="AJ10" s="51"/>
       <x:c r="AK10" s="50" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="AL10" s="51"/>
       <x:c r="AM10" s="51"/>
@@ -55556,7 +55550,7 @@
     </x:row>
     <x:row r="11" ht="13.5" customHeight="1">
       <x:c r="A11" s="47" t="s">
-        <x:v>150</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="B11" s="48"/>
       <x:c r="C11" s="48"/>
@@ -55594,7 +55588,7 @@
       <x:c r="AI11" s="48"/>
       <x:c r="AJ11" s="48"/>
       <x:c r="AK11" s="47" t="s">
-        <x:v>281</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="AL11" s="48"/>
       <x:c r="AM11" s="48"/>
@@ -55652,7 +55646,7 @@
     </x:row>
     <x:row r="12" ht="13.5" customHeight="1">
       <x:c r="A12" s="47" t="s">
-        <x:v>151</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="B12" s="48"/>
       <x:c r="C12" s="48"/>
@@ -55690,7 +55684,7 @@
       <x:c r="AI12" s="48"/>
       <x:c r="AJ12" s="48"/>
       <x:c r="AK12" s="47" t="s">
-        <x:v>282</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="AL12" s="48"/>
       <x:c r="AM12" s="48"/>
@@ -55748,7 +55742,7 @@
     </x:row>
     <x:row r="13" ht="13.5" customHeight="1">
       <x:c r="A13" s="47" t="s">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B13" s="48"/>
       <x:c r="C13" s="48"/>
@@ -55786,7 +55780,7 @@
       <x:c r="AI13" s="48"/>
       <x:c r="AJ13" s="48"/>
       <x:c r="AK13" s="47" t="s">
-        <x:v>283</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="AL13" s="48"/>
       <x:c r="AM13" s="48"/>
@@ -55844,7 +55838,7 @@
     </x:row>
     <x:row r="14" ht="13.5" customHeight="1">
       <x:c r="A14" s="47" t="s">
-        <x:v>221</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="B14" s="48"/>
       <x:c r="C14" s="48"/>
@@ -55882,7 +55876,7 @@
       <x:c r="AI14" s="48"/>
       <x:c r="AJ14" s="48"/>
       <x:c r="AK14" s="47" t="s">
-        <x:v>157</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="AL14" s="48"/>
       <x:c r="AM14" s="48"/>
@@ -56434,7 +56428,7 @@
     </x:row>
     <x:row r="6" ht="13.5" customHeight="1">
       <x:c r="A6" s="46" t="s">
-        <x:v>284</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="B6" s="46"/>
       <x:c r="C6" s="46"/>
@@ -56648,7 +56642,7 @@
       </x:c>
       <x:c r="P8" s="45"/>
       <x:c r="Q8" s="45" t="s">
-        <x:v>285</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="R8" s="45"/>
       <x:c r="S8" s="45"/>
@@ -56744,7 +56738,7 @@
       <x:c r="O9" s="48"/>
       <x:c r="P9" s="48"/>
       <x:c r="Q9" s="48" t="s">
-        <x:v>286</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="R9" s="48"/>
       <x:c r="S9" s="48"/>
@@ -57007,8 +57001,8 @@
       <x:c r="CL11" s="1"/>
     </x:row>
     <x:row r="12" ht="13.5" customHeight="1">
-      <x:c r="A12" s="1" t="s">
-        <x:v>146</x:v>
+      <x:c r="A12" s="1" t="str">
+        <x:v>参照テーブル: ユーザーアーカイブ、ユーザー[tb1]、退会ユーザー[tb2]</x:v>
       </x:c>
       <x:c r="B12" s="1"/>
       <x:c r="C12" s="1"/>
@@ -57102,7 +57096,7 @@
     </x:row>
     <x:row r="13" ht="13.5" customHeight="1">
       <x:c r="A13" s="62" t="s">
-        <x:v>287</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="B13" s="61"/>
       <x:c r="C13" s="61"/>
@@ -57196,7 +57190,7 @@
     </x:row>
     <x:row r="14" ht="13.5" customHeight="1">
       <x:c r="A14" s="50" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B14" s="51"/>
       <x:c r="C14" s="51"/>
@@ -57216,7 +57210,7 @@
       <x:c r="Q14" s="51"/>
       <x:c r="R14" s="51"/>
       <x:c r="S14" s="50" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="T14" s="51"/>
       <x:c r="U14" s="51"/>
@@ -57236,7 +57230,7 @@
       <x:c r="AI14" s="51"/>
       <x:c r="AJ14" s="51"/>
       <x:c r="AK14" s="50" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="AL14" s="51"/>
       <x:c r="AM14" s="51"/>
@@ -57294,7 +57288,7 @@
     </x:row>
     <x:row r="15" ht="13.5" customHeight="1">
       <x:c r="A15" s="47" t="s">
-        <x:v>150</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="B15" s="48"/>
       <x:c r="C15" s="48"/>
@@ -57390,7 +57384,7 @@
     </x:row>
     <x:row r="16" ht="13.5" customHeight="1">
       <x:c r="A16" s="47" t="s">
-        <x:v>151</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="B16" s="48"/>
       <x:c r="C16" s="48"/>
@@ -57486,7 +57480,7 @@
     </x:row>
     <x:row r="17" ht="13.5" customHeight="1">
       <x:c r="A17" s="46" t="s">
-        <x:v>288</x:v>
+        <x:v>286</x:v>
       </x:c>
       <x:c r="B17" s="48"/>
       <x:c r="C17" s="48"/>
@@ -57580,7 +57574,7 @@
     </x:row>
     <x:row r="18" ht="13.5" customHeight="1">
       <x:c r="A18" s="50" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B18" s="51"/>
       <x:c r="C18" s="51"/>
@@ -57600,7 +57594,7 @@
       <x:c r="Q18" s="51"/>
       <x:c r="R18" s="51"/>
       <x:c r="S18" s="50" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="T18" s="51"/>
       <x:c r="U18" s="51"/>
@@ -57620,7 +57614,7 @@
       <x:c r="AI18" s="51"/>
       <x:c r="AJ18" s="51"/>
       <x:c r="AK18" s="50" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="AL18" s="51"/>
       <x:c r="AM18" s="51"/>
@@ -57678,7 +57672,7 @@
     </x:row>
     <x:row r="19" ht="13.5" customHeight="1">
       <x:c r="A19" s="47" t="s">
-        <x:v>150</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="B19" s="48"/>
       <x:c r="C19" s="48"/>
@@ -57774,7 +57768,7 @@
     </x:row>
     <x:row r="20" ht="13.5" customHeight="1">
       <x:c r="A20" s="47" t="s">
-        <x:v>151</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="B20" s="48"/>
       <x:c r="C20" s="48"/>
@@ -57814,7 +57808,7 @@
       <x:c r="AI20" s="48"/>
       <x:c r="AJ20" s="48"/>
       <x:c r="AK20" s="47" t="s">
-        <x:v>285</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="AL20" s="48"/>
       <x:c r="AM20" s="48"/>
@@ -58094,7 +58088,7 @@
       </x:c>
       <x:c r="P3" s="67"/>
       <x:c r="Q3" s="67" t="s">
-        <x:v>289</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="R3" s="67"/>
       <x:c r="S3" s="67"/>
@@ -58113,7 +58107,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF3" s="67" t="s">
-        <x:v>290</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="AG3" s="67"/>
       <x:c r="AH3" s="67"/>
@@ -58129,7 +58123,7 @@
       <x:c r="AR3" s="67"/>
       <x:c r="AS3" s="67"/>
       <x:c r="AT3" s="67" t="s">
-        <x:v>291</x:v>
+        <x:v>289</x:v>
       </x:c>
       <x:c r="AU3" s="67"/>
       <x:c r="AV3" s="67"/>
@@ -58137,7 +58131,7 @@
       <x:c r="AX3" s="67"/>
       <x:c r="AY3" s="67"/>
       <x:c r="AZ3" s="67" t="s">
-        <x:v>263</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="BA3" s="67"/>
       <x:c r="BB3" s="67"/>
@@ -58231,7 +58225,7 @@
       <x:c r="AX4" s="72"/>
       <x:c r="AY4" s="72"/>
       <x:c r="AZ4" s="72" t="s">
-        <x:v>226</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="BA4" s="72"/>
       <x:c r="BB4" s="72"/>
@@ -58319,7 +58313,7 @@
       <x:c r="AR5" s="72"/>
       <x:c r="AS5" s="72"/>
       <x:c r="AT5" s="72" t="s">
-        <x:v>292</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="AU5" s="72"/>
       <x:c r="AV5" s="72"/>
@@ -58327,7 +58321,7 @@
       <x:c r="AX5" s="72"/>
       <x:c r="AY5" s="72"/>
       <x:c r="AZ5" s="72" t="s">
-        <x:v>293</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="BA5" s="72"/>
       <x:c r="BB5" s="72"/>
@@ -58421,7 +58415,7 @@
       <x:c r="AX6" s="77"/>
       <x:c r="AY6" s="77"/>
       <x:c r="AZ6" s="77" t="s">
-        <x:v>226</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="BA6" s="77"/>
       <x:c r="BB6" s="77"/>
@@ -58686,7 +58680,7 @@
       </x:c>
       <x:c r="P3" s="82"/>
       <x:c r="Q3" s="82" t="s">
-        <x:v>261</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="R3" s="82"/>
       <x:c r="S3" s="82"/>
@@ -58705,7 +58699,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF3" s="82" t="s">
-        <x:v>263</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="AG3" s="82"/>
       <x:c r="AH3" s="82"/>
@@ -58799,7 +58793,7 @@
       <x:c r="AD4" s="87"/>
       <x:c r="AE4" s="87"/>
       <x:c r="AF4" s="87" t="s">
-        <x:v>226</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="AG4" s="87"/>
       <x:c r="AH4" s="87"/>
@@ -58882,7 +58876,7 @@
       </x:c>
       <x:c r="P5" s="87"/>
       <x:c r="Q5" s="87" t="s">
-        <x:v>294</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="R5" s="87"/>
       <x:c r="S5" s="87"/>
@@ -58901,7 +58895,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF5" s="87" t="s">
-        <x:v>293</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="AG5" s="87"/>
       <x:c r="AH5" s="87"/>
@@ -58995,7 +58989,7 @@
       <x:c r="AD6" s="92"/>
       <x:c r="AE6" s="92"/>
       <x:c r="AF6" s="92" t="s">
-        <x:v>226</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="AG6" s="92"/>
       <x:c r="AH6" s="92"/>
@@ -59966,7 +59960,7 @@
       </x:c>
       <x:c r="P3" s="97"/>
       <x:c r="Q3" s="97" t="s">
-        <x:v>261</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="R3" s="97"/>
       <x:c r="S3" s="97"/>
@@ -59985,7 +59979,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF3" s="97" t="s">
-        <x:v>262</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="AG3" s="97"/>
       <x:c r="AH3" s="97"/>
@@ -59995,7 +59989,7 @@
       <x:c r="AL3" s="97"/>
       <x:c r="AM3" s="97"/>
       <x:c r="AN3" s="97" t="s">
-        <x:v>263</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="AO3" s="97"/>
       <x:c r="AP3" s="97"/>
@@ -60089,7 +60083,7 @@
       <x:c r="AL4" s="102"/>
       <x:c r="AM4" s="102"/>
       <x:c r="AN4" s="102" t="s">
-        <x:v>226</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="AO4" s="102"/>
       <x:c r="AP4" s="102"/>
@@ -60164,7 +60158,7 @@
       </x:c>
       <x:c r="P5" s="102"/>
       <x:c r="Q5" s="102" t="s">
-        <x:v>294</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="R5" s="102"/>
       <x:c r="S5" s="102"/>
@@ -60183,7 +60177,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AF5" s="102" t="s">
-        <x:v>262</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="AG5" s="102"/>
       <x:c r="AH5" s="102"/>
@@ -60193,7 +60187,7 @@
       <x:c r="AL5" s="102"/>
       <x:c r="AM5" s="102"/>
       <x:c r="AN5" s="102" t="s">
-        <x:v>293</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="AO5" s="102"/>
       <x:c r="AP5" s="102"/>
@@ -60287,7 +60281,7 @@
       <x:c r="AL6" s="107"/>
       <x:c r="AM6" s="107"/>
       <x:c r="AN6" s="107" t="s">
-        <x:v>226</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="AO6" s="107"/>
       <x:c r="AP6" s="107"/>

</xml_diff>

<commit_message>
test: simplify compound nested CASE review case
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Macro\SqlAnalyzerFormatter\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73952CE2-F25D-4AA0-94FE-39566921612C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{446614F3-D109-470D-9E37-CC1D8EBE18FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-8340" windowWidth="29040" windowHeight="15720" firstSheet="71" activeTab="81" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -101,7 +101,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1465" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1431" uniqueCount="316">
   <si>
     <t>＜DB入出力項目定義＞</t>
   </si>
@@ -1027,40 +1027,16 @@
     <t>tb1.状態 = 'PENDING')</t>
   </si>
   <si>
-    <t>(tb1.削除日時 IS NULL</t>
-  </si>
-  <si>
-    <t>tb1.更新日時 &gt;= @base_date)) → ((tb1.ランクコード = 'VIP'</t>
-  </si>
-  <si>
-    <t>tb1.ランクコード = 'GOLD')</t>
+    <t>tb1.削除日時 IS NULL) → (tb1.ランクコード = 'VIP'</t>
   </si>
   <si>
     <t>(tb1.評価点 &gt;= 90</t>
   </si>
   <si>
-    <t>tb1.優先フラグ = 1)) → ((tb1.地域コード = 'JP'</t>
+    <t>tb1.優先フラグ = 1)) → 'ACTIVE_PRIORITY'</t>
   </si>
   <si>
-    <t>tb1.地域コード = 'US')</t>
-  </si>
-  <si>
-    <t>(tb1.年齢 &gt;= 20</t>
-  </si>
-  <si>
-    <t>tb1.確認済みフラグ = 1)) → 'ACTIVE_VIP_HIGH'</t>
-  </si>
-  <si>
-    <t>ELSE → ((tb1.ログイン回数 &gt; 0</t>
-  </si>
-  <si>
-    <t>tb1.最終ログイン日時 IS NOT NULL)</t>
-  </si>
-  <si>
-    <t>(tb1.作成日時 &gt;= @recent_date</t>
-  </si>
-  <si>
-    <t>tb1.確認済みフラグ = 1)) → 'ACTIVE_GENERAL_HIGH'</t>
+    <t>ELSE → 'ACTIVE_STANDARD'</t>
   </si>
   <si>
     <t>ELSE → ((tb1.状態 = 'LOCKED'</t>
@@ -1069,28 +1045,10 @@
     <t>tb1.状態 = 'INACTIVE')</t>
   </si>
   <si>
-    <t>tb1.停止日時 IS NOT NULL)) → ((tb1.再試行回数 &lt; 3</t>
+    <t>tb1.削除日時 IS NOT NULL) → 'INACTIVE_DELETED'</t>
   </si>
   <si>
-    <t>tb1.エラー件数 = 0)</t>
-  </si>
-  <si>
-    <t>(tb1.上長ID IS NOT NULL</t>
-  </si>
-  <si>
-    <t>tb1.承認日時 IS NOT NULL)) → 'PENDING'</t>
-  </si>
-  <si>
-    <t>ELSE → ((tb1.削除日時 IS NOT NULL</t>
-  </si>
-  <si>
-    <t>tb1.削除対象フラグ = 0)</t>
-  </si>
-  <si>
-    <t>(tb1.アーカイブフラグ = 1</t>
-  </si>
-  <si>
-    <t>tb1.アーカイブ日時 IS NOT NULL)) → 'LOCKED_DELETED'</t>
+    <t>ELSE → 'OTHER'</t>
   </si>
 </sst>
 </file>
@@ -1420,7 +1378,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="147">
+  <cellXfs count="149">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1808,59 +1766,65 @@
     <xf numFmtId="0" fontId="3" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -61452,2977 +61416,1161 @@
 
 <file path=xl/worksheets/sheet82.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-5100-000000000000}">
-  <dimension ref="A1:CL31"/>
+  <dimension ref="A1:CL12"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="90" width="1.75" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="109" t="s">
+      <c r="A1" s="129" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="109"/>
-      <c r="C1" s="109"/>
-      <c r="D1" s="109"/>
-      <c r="E1" s="109"/>
-      <c r="F1" s="109"/>
-      <c r="G1" s="109"/>
-      <c r="H1" s="109"/>
-      <c r="I1" s="109"/>
-      <c r="J1" s="109"/>
-      <c r="K1" s="109"/>
-      <c r="L1" s="109"/>
-      <c r="M1" s="109"/>
-      <c r="N1" s="109"/>
-      <c r="O1" s="109"/>
-      <c r="P1" s="109"/>
-      <c r="Q1" s="109"/>
-      <c r="R1" s="109"/>
-      <c r="S1" s="109"/>
-      <c r="T1" s="109"/>
-      <c r="U1" s="109"/>
-      <c r="V1" s="109"/>
-      <c r="W1" s="109"/>
-      <c r="X1" s="109"/>
-      <c r="Y1" s="109"/>
-      <c r="Z1" s="109"/>
-      <c r="AA1" s="109"/>
-      <c r="AB1" s="109"/>
-      <c r="AC1" s="109"/>
-      <c r="AD1" s="109"/>
-      <c r="AE1" s="109"/>
-      <c r="AF1" s="109"/>
-      <c r="AG1" s="109"/>
-      <c r="AH1" s="109"/>
-      <c r="AI1" s="109"/>
-      <c r="AJ1" s="109"/>
-      <c r="AK1" s="109"/>
-      <c r="AL1" s="109"/>
-      <c r="AM1" s="109"/>
-      <c r="AN1" s="109"/>
-      <c r="AO1" s="109"/>
-      <c r="AP1" s="109"/>
-      <c r="AQ1" s="109"/>
-      <c r="AR1" s="109"/>
-      <c r="AS1" s="109"/>
-      <c r="AT1" s="109"/>
-      <c r="AU1" s="109"/>
-      <c r="AV1" s="109"/>
-      <c r="AW1" s="109"/>
-      <c r="AX1" s="109"/>
-      <c r="AY1" s="109"/>
-      <c r="AZ1" s="109"/>
-      <c r="BA1" s="109"/>
-      <c r="BB1" s="109"/>
-      <c r="BC1" s="109"/>
-      <c r="BD1" s="109"/>
-      <c r="BE1" s="109"/>
-      <c r="BF1" s="109"/>
-      <c r="BG1" s="109"/>
-      <c r="BH1" s="109"/>
-      <c r="BI1" s="109"/>
-      <c r="BJ1" s="109"/>
-      <c r="BK1" s="109"/>
-      <c r="BL1" s="109"/>
-      <c r="BM1" s="109"/>
-      <c r="BN1" s="109"/>
-      <c r="BO1" s="109"/>
-      <c r="BP1" s="109"/>
-      <c r="BQ1" s="109"/>
-      <c r="BR1" s="109"/>
-      <c r="BS1" s="109"/>
-      <c r="BT1" s="109"/>
-      <c r="BU1" s="109"/>
-      <c r="BV1" s="109"/>
-      <c r="BW1" s="109"/>
-      <c r="BX1" s="109"/>
-      <c r="BY1" s="109"/>
-      <c r="BZ1" s="109"/>
-      <c r="CA1" s="109"/>
-      <c r="CB1" s="109"/>
-      <c r="CC1" s="109"/>
-      <c r="CD1" s="109"/>
-      <c r="CE1" s="109"/>
-      <c r="CF1" s="109"/>
-      <c r="CG1" s="109"/>
-      <c r="CH1" s="109"/>
-      <c r="CI1" s="109"/>
-      <c r="CJ1" s="109"/>
-      <c r="CK1" s="109"/>
-      <c r="CL1" s="109"/>
+      <c r="B1" s="129"/>
+      <c r="C1" s="129"/>
+      <c r="D1" s="129"/>
+      <c r="E1" s="129"/>
+      <c r="F1" s="129"/>
+      <c r="G1" s="129"/>
+      <c r="H1" s="129"/>
+      <c r="I1" s="129"/>
+      <c r="J1" s="129"/>
+      <c r="K1" s="129"/>
+      <c r="L1" s="129"/>
+      <c r="M1" s="129"/>
+      <c r="N1" s="129"/>
+      <c r="O1" s="129"/>
+      <c r="P1" s="129"/>
+      <c r="Q1" s="129"/>
+      <c r="R1" s="129"/>
+      <c r="S1" s="129"/>
+      <c r="T1" s="129"/>
+      <c r="U1" s="129"/>
+      <c r="V1" s="129"/>
+      <c r="W1" s="129"/>
+      <c r="X1" s="129"/>
+      <c r="Y1" s="129"/>
+      <c r="Z1" s="129"/>
+      <c r="AA1" s="129"/>
+      <c r="AB1" s="129"/>
+      <c r="AC1" s="129"/>
+      <c r="AD1" s="129"/>
+      <c r="AE1" s="129"/>
+      <c r="AF1" s="129"/>
+      <c r="AG1" s="129"/>
+      <c r="AH1" s="129"/>
+      <c r="AI1" s="129"/>
+      <c r="AJ1" s="129"/>
+      <c r="AK1" s="129"/>
+      <c r="AL1" s="129"/>
+      <c r="AM1" s="129"/>
+      <c r="AN1" s="129"/>
+      <c r="AO1" s="129"/>
+      <c r="AP1" s="129"/>
+      <c r="AQ1" s="129"/>
+      <c r="AR1" s="129"/>
+      <c r="AS1" s="129"/>
+      <c r="AT1" s="129"/>
+      <c r="AU1" s="129"/>
+      <c r="AV1" s="129"/>
+      <c r="AW1" s="129"/>
+      <c r="AX1" s="129"/>
+      <c r="AY1" s="129"/>
+      <c r="AZ1" s="129"/>
+      <c r="BA1" s="129"/>
+      <c r="BB1" s="129"/>
+      <c r="BC1" s="129"/>
+      <c r="BD1" s="129"/>
+      <c r="BE1" s="129"/>
+      <c r="BF1" s="129"/>
+      <c r="BG1" s="129"/>
+      <c r="BH1" s="129"/>
+      <c r="BI1" s="129"/>
+      <c r="BJ1" s="129"/>
+      <c r="BK1" s="129"/>
+      <c r="BL1" s="129"/>
+      <c r="BM1" s="129"/>
+      <c r="BN1" s="129"/>
+      <c r="BO1" s="129"/>
+      <c r="BP1" s="129"/>
+      <c r="BQ1" s="129"/>
+      <c r="BR1" s="129"/>
+      <c r="BS1" s="129"/>
+      <c r="BT1" s="129"/>
+      <c r="BU1" s="129"/>
+      <c r="BV1" s="129"/>
+      <c r="BW1" s="129"/>
+      <c r="BX1" s="129"/>
+      <c r="BY1" s="129"/>
+      <c r="BZ1" s="129"/>
+      <c r="CA1" s="129"/>
+      <c r="CB1" s="129"/>
+      <c r="CC1" s="129"/>
+      <c r="CD1" s="129"/>
+      <c r="CE1" s="129"/>
+      <c r="CF1" s="129"/>
+      <c r="CG1" s="129"/>
+      <c r="CH1" s="129"/>
+      <c r="CI1" s="129"/>
+      <c r="CJ1" s="129"/>
+      <c r="CK1" s="129"/>
+      <c r="CL1" s="129"/>
     </row>
     <row r="2" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="110" t="s">
+      <c r="A2" s="130" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="110"/>
-      <c r="C2" s="110"/>
-      <c r="D2" s="110"/>
-      <c r="E2" s="110"/>
-      <c r="F2" s="110"/>
-      <c r="G2" s="110"/>
-      <c r="H2" s="110"/>
-      <c r="I2" s="110"/>
-      <c r="J2" s="110"/>
-      <c r="K2" s="110"/>
-      <c r="L2" s="110"/>
-      <c r="M2" s="110"/>
-      <c r="N2" s="110"/>
-      <c r="O2" s="110"/>
-      <c r="P2" s="110"/>
-      <c r="Q2" s="110"/>
-      <c r="R2" s="110"/>
-      <c r="S2" s="110"/>
-      <c r="T2" s="110"/>
-      <c r="U2" s="110"/>
-      <c r="V2" s="110"/>
-      <c r="W2" s="110"/>
-      <c r="X2" s="110"/>
-      <c r="Y2" s="110"/>
-      <c r="Z2" s="110"/>
-      <c r="AA2" s="110"/>
-      <c r="AB2" s="110"/>
-      <c r="AC2" s="110"/>
-      <c r="AD2" s="110"/>
-      <c r="AE2" s="110"/>
-      <c r="AF2" s="110"/>
-      <c r="AG2" s="110"/>
-      <c r="AH2" s="110"/>
-      <c r="AI2" s="110"/>
-      <c r="AJ2" s="110"/>
-      <c r="AK2" s="110"/>
-      <c r="AL2" s="110"/>
-      <c r="AM2" s="110"/>
-      <c r="AN2" s="110"/>
-      <c r="AO2" s="110"/>
-      <c r="AP2" s="110"/>
-      <c r="AQ2" s="110"/>
-      <c r="AR2" s="110"/>
-      <c r="AS2" s="110"/>
-      <c r="AT2" s="110"/>
-      <c r="AU2" s="110"/>
-      <c r="AV2" s="110"/>
-      <c r="AW2" s="110"/>
-      <c r="AX2" s="110"/>
-      <c r="AY2" s="110"/>
-      <c r="AZ2" s="110"/>
-      <c r="BA2" s="110"/>
-      <c r="BB2" s="110"/>
-      <c r="BC2" s="110"/>
-      <c r="BD2" s="110"/>
-      <c r="BE2" s="110"/>
-      <c r="BF2" s="110"/>
-      <c r="BG2" s="110"/>
-      <c r="BH2" s="110"/>
-      <c r="BI2" s="110"/>
-      <c r="BJ2" s="110"/>
-      <c r="BK2" s="110"/>
-      <c r="BL2" s="110"/>
-      <c r="BM2" s="110"/>
-      <c r="BN2" s="110"/>
-      <c r="BO2" s="110"/>
-      <c r="BP2" s="110"/>
-      <c r="BQ2" s="110"/>
-      <c r="BR2" s="110"/>
-      <c r="BS2" s="110"/>
-      <c r="BT2" s="110"/>
-      <c r="BU2" s="110"/>
-      <c r="BV2" s="110"/>
-      <c r="BW2" s="110"/>
-      <c r="BX2" s="110"/>
-      <c r="BY2" s="110"/>
-      <c r="BZ2" s="110"/>
-      <c r="CA2" s="110"/>
-      <c r="CB2" s="110"/>
-      <c r="CC2" s="110"/>
-      <c r="CD2" s="110"/>
-      <c r="CE2" s="110"/>
-      <c r="CF2" s="110"/>
-      <c r="CG2" s="110"/>
-      <c r="CH2" s="110"/>
-      <c r="CI2" s="110"/>
-      <c r="CJ2" s="110"/>
-      <c r="CK2" s="110"/>
-      <c r="CL2" s="110"/>
+      <c r="B2" s="130"/>
+      <c r="C2" s="130"/>
+      <c r="D2" s="130"/>
+      <c r="E2" s="130"/>
+      <c r="F2" s="130"/>
+      <c r="G2" s="130"/>
+      <c r="H2" s="130"/>
+      <c r="I2" s="130"/>
+      <c r="J2" s="130"/>
+      <c r="K2" s="130"/>
+      <c r="L2" s="130"/>
+      <c r="M2" s="130"/>
+      <c r="N2" s="130"/>
+      <c r="O2" s="130"/>
+      <c r="P2" s="130"/>
+      <c r="Q2" s="130"/>
+      <c r="R2" s="130"/>
+      <c r="S2" s="130"/>
+      <c r="T2" s="130"/>
+      <c r="U2" s="130"/>
+      <c r="V2" s="130"/>
+      <c r="W2" s="130"/>
+      <c r="X2" s="130"/>
+      <c r="Y2" s="130"/>
+      <c r="Z2" s="130"/>
+      <c r="AA2" s="130"/>
+      <c r="AB2" s="130"/>
+      <c r="AC2" s="130"/>
+      <c r="AD2" s="130"/>
+      <c r="AE2" s="130"/>
+      <c r="AF2" s="130"/>
+      <c r="AG2" s="130"/>
+      <c r="AH2" s="130"/>
+      <c r="AI2" s="130"/>
+      <c r="AJ2" s="130"/>
+      <c r="AK2" s="130"/>
+      <c r="AL2" s="130"/>
+      <c r="AM2" s="130"/>
+      <c r="AN2" s="130"/>
+      <c r="AO2" s="130"/>
+      <c r="AP2" s="130"/>
+      <c r="AQ2" s="130"/>
+      <c r="AR2" s="130"/>
+      <c r="AS2" s="130"/>
+      <c r="AT2" s="130"/>
+      <c r="AU2" s="130"/>
+      <c r="AV2" s="130"/>
+      <c r="AW2" s="130"/>
+      <c r="AX2" s="130"/>
+      <c r="AY2" s="130"/>
+      <c r="AZ2" s="130"/>
+      <c r="BA2" s="130"/>
+      <c r="BB2" s="130"/>
+      <c r="BC2" s="130"/>
+      <c r="BD2" s="130"/>
+      <c r="BE2" s="130"/>
+      <c r="BF2" s="130"/>
+      <c r="BG2" s="130"/>
+      <c r="BH2" s="130"/>
+      <c r="BI2" s="130"/>
+      <c r="BJ2" s="130"/>
+      <c r="BK2" s="130"/>
+      <c r="BL2" s="130"/>
+      <c r="BM2" s="130"/>
+      <c r="BN2" s="130"/>
+      <c r="BO2" s="130"/>
+      <c r="BP2" s="130"/>
+      <c r="BQ2" s="130"/>
+      <c r="BR2" s="130"/>
+      <c r="BS2" s="130"/>
+      <c r="BT2" s="130"/>
+      <c r="BU2" s="130"/>
+      <c r="BV2" s="130"/>
+      <c r="BW2" s="130"/>
+      <c r="BX2" s="130"/>
+      <c r="BY2" s="130"/>
+      <c r="BZ2" s="130"/>
+      <c r="CA2" s="130"/>
+      <c r="CB2" s="130"/>
+      <c r="CC2" s="130"/>
+      <c r="CD2" s="130"/>
+      <c r="CE2" s="130"/>
+      <c r="CF2" s="130"/>
+      <c r="CG2" s="130"/>
+      <c r="CH2" s="130"/>
+      <c r="CI2" s="130"/>
+      <c r="CJ2" s="130"/>
+      <c r="CK2" s="130"/>
+      <c r="CL2" s="130"/>
     </row>
     <row r="3" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="130" t="s">
+      <c r="A3" s="132" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="131"/>
-      <c r="C3" s="131"/>
-      <c r="D3" s="131"/>
-      <c r="E3" s="131"/>
-      <c r="F3" s="132"/>
-      <c r="G3" s="139" t="s">
+      <c r="B3" s="133"/>
+      <c r="C3" s="133"/>
+      <c r="D3" s="133"/>
+      <c r="E3" s="133"/>
+      <c r="F3" s="134"/>
+      <c r="G3" s="141" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="140"/>
-      <c r="I3" s="140"/>
-      <c r="J3" s="140"/>
-      <c r="K3" s="140"/>
-      <c r="L3" s="140"/>
-      <c r="M3" s="140"/>
-      <c r="N3" s="140"/>
-      <c r="O3" s="140" t="s">
+      <c r="H3" s="142"/>
+      <c r="I3" s="142"/>
+      <c r="J3" s="142"/>
+      <c r="K3" s="142"/>
+      <c r="L3" s="142"/>
+      <c r="M3" s="142"/>
+      <c r="N3" s="142"/>
+      <c r="O3" s="142" t="s">
         <v>4</v>
       </c>
-      <c r="P3" s="140"/>
-      <c r="Q3" s="140" t="s">
+      <c r="P3" s="142"/>
+      <c r="Q3" s="142" t="s">
         <v>162</v>
       </c>
-      <c r="R3" s="140"/>
-      <c r="S3" s="140"/>
-      <c r="T3" s="140"/>
-      <c r="U3" s="140"/>
-      <c r="V3" s="140"/>
-      <c r="W3" s="140"/>
-      <c r="X3" s="140"/>
-      <c r="Y3" s="140"/>
-      <c r="Z3" s="140"/>
-      <c r="AA3" s="140"/>
-      <c r="AB3" s="140"/>
-      <c r="AC3" s="140"/>
-      <c r="AD3" s="140"/>
-      <c r="AE3" s="140" t="s">
+      <c r="R3" s="142"/>
+      <c r="S3" s="142"/>
+      <c r="T3" s="142"/>
+      <c r="U3" s="142"/>
+      <c r="V3" s="142"/>
+      <c r="W3" s="142"/>
+      <c r="X3" s="142"/>
+      <c r="Y3" s="142"/>
+      <c r="Z3" s="142"/>
+      <c r="AA3" s="142"/>
+      <c r="AB3" s="142"/>
+      <c r="AC3" s="142"/>
+      <c r="AD3" s="142"/>
+      <c r="AE3" s="142" t="s">
         <v>33</v>
       </c>
-      <c r="AF3" s="140"/>
-      <c r="AG3" s="140"/>
-      <c r="AH3" s="140"/>
-      <c r="AI3" s="140"/>
-      <c r="AJ3" s="140" t="s">
+      <c r="AF3" s="142"/>
+      <c r="AG3" s="142"/>
+      <c r="AH3" s="142"/>
+      <c r="AI3" s="142"/>
+      <c r="AJ3" s="142" t="s">
         <v>306</v>
       </c>
-      <c r="AK3" s="140"/>
-      <c r="AL3" s="140"/>
-      <c r="AM3" s="140"/>
-      <c r="AN3" s="140"/>
-      <c r="AO3" s="140"/>
-      <c r="AP3" s="140"/>
-      <c r="AQ3" s="140"/>
-      <c r="AR3" s="140"/>
-      <c r="AS3" s="140"/>
-      <c r="AT3" s="140"/>
-      <c r="AU3" s="140"/>
-      <c r="AV3" s="140"/>
-      <c r="AW3" s="140"/>
-      <c r="AX3" s="140"/>
-      <c r="AY3" s="140"/>
-      <c r="AZ3" s="140"/>
-      <c r="BA3" s="140"/>
-      <c r="BB3" s="140"/>
-      <c r="BC3" s="140"/>
-      <c r="BD3" s="140"/>
-      <c r="BE3" s="140"/>
-      <c r="BF3" s="140"/>
-      <c r="BG3" s="140"/>
-      <c r="BH3" s="140"/>
-      <c r="BI3" s="140"/>
-      <c r="BJ3" s="140"/>
-      <c r="BK3" s="140"/>
-      <c r="BL3" s="140"/>
-      <c r="BM3" s="140"/>
-      <c r="BN3" s="140"/>
-      <c r="BO3" s="140"/>
-      <c r="BP3" s="140"/>
-      <c r="BQ3" s="140"/>
-      <c r="BR3" s="140"/>
-      <c r="BS3" s="140"/>
-      <c r="BT3" s="140"/>
-      <c r="BU3" s="140"/>
-      <c r="BV3" s="140"/>
-      <c r="BW3" s="140"/>
-      <c r="BX3" s="140"/>
-      <c r="BY3" s="140"/>
-      <c r="BZ3" s="140"/>
-      <c r="CA3" s="140"/>
-      <c r="CB3" s="140"/>
-      <c r="CC3" s="140"/>
-      <c r="CD3" s="140"/>
-      <c r="CE3" s="140"/>
-      <c r="CF3" s="140"/>
-      <c r="CG3" s="140"/>
-      <c r="CH3" s="140"/>
-      <c r="CI3" s="140"/>
-      <c r="CJ3" s="140"/>
-      <c r="CK3" s="140"/>
-      <c r="CL3" s="141"/>
+      <c r="AK3" s="142"/>
+      <c r="AL3" s="142"/>
+      <c r="AM3" s="142"/>
+      <c r="AN3" s="142"/>
+      <c r="AO3" s="142"/>
+      <c r="AP3" s="142"/>
+      <c r="AQ3" s="142"/>
+      <c r="AR3" s="142"/>
+      <c r="AS3" s="142"/>
+      <c r="AT3" s="142"/>
+      <c r="AU3" s="142"/>
+      <c r="AV3" s="142"/>
+      <c r="AW3" s="142"/>
+      <c r="AX3" s="142"/>
+      <c r="AY3" s="142"/>
+      <c r="AZ3" s="142"/>
+      <c r="BA3" s="142"/>
+      <c r="BB3" s="142"/>
+      <c r="BC3" s="142"/>
+      <c r="BD3" s="142"/>
+      <c r="BE3" s="142"/>
+      <c r="BF3" s="142"/>
+      <c r="BG3" s="142"/>
+      <c r="BH3" s="142"/>
+      <c r="BI3" s="142"/>
+      <c r="BJ3" s="142"/>
+      <c r="BK3" s="142"/>
+      <c r="BL3" s="142"/>
+      <c r="BM3" s="142"/>
+      <c r="BN3" s="142"/>
+      <c r="BO3" s="142"/>
+      <c r="BP3" s="142"/>
+      <c r="BQ3" s="142"/>
+      <c r="BR3" s="142"/>
+      <c r="BS3" s="142"/>
+      <c r="BT3" s="142"/>
+      <c r="BU3" s="142"/>
+      <c r="BV3" s="142"/>
+      <c r="BW3" s="142"/>
+      <c r="BX3" s="142"/>
+      <c r="BY3" s="142"/>
+      <c r="BZ3" s="142"/>
+      <c r="CA3" s="142"/>
+      <c r="CB3" s="142"/>
+      <c r="CC3" s="142"/>
+      <c r="CD3" s="142"/>
+      <c r="CE3" s="142"/>
+      <c r="CF3" s="142"/>
+      <c r="CG3" s="142"/>
+      <c r="CH3" s="142"/>
+      <c r="CI3" s="142"/>
+      <c r="CJ3" s="142"/>
+      <c r="CK3" s="142"/>
+      <c r="CL3" s="143"/>
     </row>
     <row r="4" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="133"/>
-      <c r="B4" s="129"/>
-      <c r="C4" s="129"/>
-      <c r="D4" s="129"/>
-      <c r="E4" s="129"/>
-      <c r="F4" s="134"/>
-      <c r="G4" s="142"/>
-      <c r="H4" s="138"/>
-      <c r="I4" s="138"/>
-      <c r="J4" s="138"/>
-      <c r="K4" s="138"/>
-      <c r="L4" s="138"/>
-      <c r="M4" s="138"/>
-      <c r="N4" s="138"/>
-      <c r="O4" s="138"/>
-      <c r="P4" s="138"/>
-      <c r="Q4" s="138"/>
-      <c r="R4" s="138"/>
-      <c r="S4" s="138"/>
-      <c r="T4" s="138"/>
-      <c r="U4" s="138"/>
-      <c r="V4" s="138"/>
-      <c r="W4" s="138"/>
-      <c r="X4" s="138"/>
-      <c r="Y4" s="138"/>
-      <c r="Z4" s="138"/>
-      <c r="AA4" s="138"/>
-      <c r="AB4" s="138"/>
-      <c r="AC4" s="138"/>
-      <c r="AD4" s="138"/>
-      <c r="AE4" s="138"/>
-      <c r="AF4" s="138"/>
-      <c r="AG4" s="138"/>
-      <c r="AH4" s="138" t="s">
+      <c r="A4" s="135"/>
+      <c r="B4" s="131"/>
+      <c r="C4" s="131"/>
+      <c r="D4" s="131"/>
+      <c r="E4" s="131"/>
+      <c r="F4" s="136"/>
+      <c r="G4" s="144"/>
+      <c r="H4" s="140"/>
+      <c r="I4" s="140"/>
+      <c r="J4" s="140"/>
+      <c r="K4" s="140"/>
+      <c r="L4" s="140"/>
+      <c r="M4" s="140"/>
+      <c r="N4" s="140"/>
+      <c r="O4" s="140"/>
+      <c r="P4" s="140"/>
+      <c r="Q4" s="140"/>
+      <c r="R4" s="140"/>
+      <c r="S4" s="140"/>
+      <c r="T4" s="140"/>
+      <c r="U4" s="140"/>
+      <c r="V4" s="140"/>
+      <c r="W4" s="140"/>
+      <c r="X4" s="140"/>
+      <c r="Y4" s="140"/>
+      <c r="Z4" s="140"/>
+      <c r="AA4" s="140"/>
+      <c r="AB4" s="140"/>
+      <c r="AC4" s="140"/>
+      <c r="AD4" s="140"/>
+      <c r="AE4" s="140"/>
+      <c r="AF4" s="140"/>
+      <c r="AG4" s="140"/>
+      <c r="AH4" s="140" t="s">
         <v>128</v>
       </c>
-      <c r="AI4" s="138"/>
-      <c r="AJ4" s="138" t="s">
+      <c r="AI4" s="140"/>
+      <c r="AJ4" s="140" t="s">
         <v>307</v>
       </c>
-      <c r="AK4" s="138"/>
-      <c r="AL4" s="138"/>
-      <c r="AM4" s="138"/>
-      <c r="AN4" s="138"/>
-      <c r="AO4" s="138"/>
-      <c r="AP4" s="138"/>
-      <c r="AQ4" s="138"/>
-      <c r="AR4" s="138"/>
-      <c r="AS4" s="138"/>
-      <c r="AT4" s="138"/>
-      <c r="AU4" s="138"/>
-      <c r="AV4" s="138"/>
-      <c r="AW4" s="138"/>
-      <c r="AX4" s="138"/>
-      <c r="AY4" s="138"/>
-      <c r="AZ4" s="138"/>
-      <c r="BA4" s="138"/>
-      <c r="BB4" s="138"/>
-      <c r="BC4" s="138"/>
-      <c r="BD4" s="138"/>
-      <c r="BE4" s="138"/>
-      <c r="BF4" s="138"/>
-      <c r="BG4" s="138"/>
-      <c r="BH4" s="138"/>
-      <c r="BI4" s="138"/>
-      <c r="BJ4" s="138"/>
-      <c r="BK4" s="138"/>
-      <c r="BL4" s="138"/>
-      <c r="BM4" s="138"/>
-      <c r="BN4" s="138"/>
-      <c r="BO4" s="138"/>
-      <c r="BP4" s="138"/>
-      <c r="BQ4" s="138"/>
-      <c r="BR4" s="138"/>
-      <c r="BS4" s="138"/>
-      <c r="BT4" s="138"/>
-      <c r="BU4" s="138"/>
-      <c r="BV4" s="138"/>
-      <c r="BW4" s="138"/>
-      <c r="BX4" s="138"/>
-      <c r="BY4" s="138"/>
-      <c r="BZ4" s="138"/>
-      <c r="CA4" s="138"/>
-      <c r="CB4" s="138"/>
-      <c r="CC4" s="138"/>
-      <c r="CD4" s="138"/>
-      <c r="CE4" s="138"/>
-      <c r="CF4" s="138"/>
-      <c r="CG4" s="138"/>
-      <c r="CH4" s="138"/>
-      <c r="CI4" s="138"/>
-      <c r="CJ4" s="138"/>
-      <c r="CK4" s="138"/>
-      <c r="CL4" s="143"/>
+      <c r="AK4" s="140"/>
+      <c r="AL4" s="140"/>
+      <c r="AM4" s="140"/>
+      <c r="AN4" s="140"/>
+      <c r="AO4" s="140"/>
+      <c r="AP4" s="140"/>
+      <c r="AQ4" s="140"/>
+      <c r="AR4" s="140"/>
+      <c r="AS4" s="140"/>
+      <c r="AT4" s="140"/>
+      <c r="AU4" s="140"/>
+      <c r="AV4" s="140"/>
+      <c r="AW4" s="140"/>
+      <c r="AX4" s="140"/>
+      <c r="AY4" s="140"/>
+      <c r="AZ4" s="140"/>
+      <c r="BA4" s="140"/>
+      <c r="BB4" s="140"/>
+      <c r="BC4" s="140"/>
+      <c r="BD4" s="140"/>
+      <c r="BE4" s="140"/>
+      <c r="BF4" s="140"/>
+      <c r="BG4" s="140"/>
+      <c r="BH4" s="140"/>
+      <c r="BI4" s="140"/>
+      <c r="BJ4" s="140"/>
+      <c r="BK4" s="140"/>
+      <c r="BL4" s="140"/>
+      <c r="BM4" s="140"/>
+      <c r="BN4" s="140"/>
+      <c r="BO4" s="140"/>
+      <c r="BP4" s="140"/>
+      <c r="BQ4" s="140"/>
+      <c r="BR4" s="140"/>
+      <c r="BS4" s="140"/>
+      <c r="BT4" s="140"/>
+      <c r="BU4" s="140"/>
+      <c r="BV4" s="140"/>
+      <c r="BW4" s="140"/>
+      <c r="BX4" s="140"/>
+      <c r="BY4" s="140"/>
+      <c r="BZ4" s="140"/>
+      <c r="CA4" s="140"/>
+      <c r="CB4" s="140"/>
+      <c r="CC4" s="140"/>
+      <c r="CD4" s="140"/>
+      <c r="CE4" s="140"/>
+      <c r="CF4" s="140"/>
+      <c r="CG4" s="140"/>
+      <c r="CH4" s="140"/>
+      <c r="CI4" s="140"/>
+      <c r="CJ4" s="140"/>
+      <c r="CK4" s="140"/>
+      <c r="CL4" s="145"/>
     </row>
     <row r="5" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="133"/>
-      <c r="B5" s="129"/>
-      <c r="C5" s="129"/>
-      <c r="D5" s="129"/>
-      <c r="E5" s="129"/>
-      <c r="F5" s="134"/>
-      <c r="G5" s="142"/>
-      <c r="H5" s="138"/>
-      <c r="I5" s="138"/>
-      <c r="J5" s="138"/>
-      <c r="K5" s="138"/>
-      <c r="L5" s="138"/>
-      <c r="M5" s="138"/>
-      <c r="N5" s="138"/>
-      <c r="O5" s="138"/>
-      <c r="P5" s="138"/>
-      <c r="Q5" s="138"/>
-      <c r="R5" s="138"/>
-      <c r="S5" s="138"/>
-      <c r="T5" s="138"/>
-      <c r="U5" s="138"/>
-      <c r="V5" s="138"/>
-      <c r="W5" s="138"/>
-      <c r="X5" s="138"/>
-      <c r="Y5" s="138"/>
-      <c r="Z5" s="138"/>
-      <c r="AA5" s="138"/>
-      <c r="AB5" s="138"/>
-      <c r="AC5" s="138"/>
-      <c r="AD5" s="138"/>
-      <c r="AE5" s="138"/>
-      <c r="AF5" s="138" t="s">
+      <c r="A5" s="135"/>
+      <c r="B5" s="131"/>
+      <c r="C5" s="131"/>
+      <c r="D5" s="131"/>
+      <c r="E5" s="131"/>
+      <c r="F5" s="136"/>
+      <c r="G5" s="144"/>
+      <c r="H5" s="140"/>
+      <c r="I5" s="140"/>
+      <c r="J5" s="140"/>
+      <c r="K5" s="140"/>
+      <c r="L5" s="140"/>
+      <c r="M5" s="140"/>
+      <c r="N5" s="140"/>
+      <c r="O5" s="140"/>
+      <c r="P5" s="140"/>
+      <c r="Q5" s="140"/>
+      <c r="R5" s="140"/>
+      <c r="S5" s="140"/>
+      <c r="T5" s="140"/>
+      <c r="U5" s="140"/>
+      <c r="V5" s="140"/>
+      <c r="W5" s="140"/>
+      <c r="X5" s="140"/>
+      <c r="Y5" s="140"/>
+      <c r="Z5" s="140"/>
+      <c r="AA5" s="140"/>
+      <c r="AB5" s="140"/>
+      <c r="AC5" s="140"/>
+      <c r="AD5" s="140"/>
+      <c r="AE5" s="140"/>
+      <c r="AF5" s="140" t="s">
         <v>10</v>
       </c>
-      <c r="AG5" s="138"/>
-      <c r="AH5" s="138"/>
-      <c r="AI5" s="138"/>
-      <c r="AJ5" s="138" t="s">
+      <c r="AG5" s="140"/>
+      <c r="AH5" s="140" t="s">
         <v>308</v>
       </c>
-      <c r="AK5" s="138"/>
-      <c r="AL5" s="138"/>
-      <c r="AM5" s="138"/>
-      <c r="AN5" s="138"/>
-      <c r="AO5" s="138"/>
-      <c r="AP5" s="138"/>
-      <c r="AQ5" s="138"/>
-      <c r="AR5" s="138"/>
-      <c r="AS5" s="138"/>
-      <c r="AT5" s="138"/>
-      <c r="AU5" s="138"/>
-      <c r="AV5" s="138"/>
-      <c r="AW5" s="138"/>
-      <c r="AX5" s="138"/>
-      <c r="AY5" s="138"/>
-      <c r="AZ5" s="138"/>
-      <c r="BA5" s="138"/>
-      <c r="BB5" s="138"/>
-      <c r="BC5" s="138"/>
-      <c r="BD5" s="138"/>
-      <c r="BE5" s="138"/>
-      <c r="BF5" s="138"/>
-      <c r="BG5" s="138"/>
-      <c r="BH5" s="138"/>
-      <c r="BI5" s="138"/>
-      <c r="BJ5" s="138"/>
-      <c r="BK5" s="138"/>
-      <c r="BL5" s="138"/>
-      <c r="BM5" s="138"/>
-      <c r="BN5" s="138"/>
-      <c r="BO5" s="138"/>
-      <c r="BP5" s="138"/>
-      <c r="BQ5" s="138"/>
-      <c r="BR5" s="138"/>
-      <c r="BS5" s="138"/>
-      <c r="BT5" s="138"/>
-      <c r="BU5" s="138"/>
-      <c r="BV5" s="138"/>
-      <c r="BW5" s="138"/>
-      <c r="BX5" s="138"/>
-      <c r="BY5" s="138"/>
-      <c r="BZ5" s="138"/>
-      <c r="CA5" s="138"/>
-      <c r="CB5" s="138"/>
-      <c r="CC5" s="138"/>
-      <c r="CD5" s="138"/>
-      <c r="CE5" s="138"/>
-      <c r="CF5" s="138"/>
-      <c r="CG5" s="138"/>
-      <c r="CH5" s="138"/>
-      <c r="CI5" s="138"/>
-      <c r="CJ5" s="138"/>
-      <c r="CK5" s="138"/>
-      <c r="CL5" s="143"/>
+      <c r="AI5" s="140"/>
+      <c r="AJ5" s="140"/>
+      <c r="AK5" s="140"/>
+      <c r="AL5" s="140"/>
+      <c r="AM5" s="140"/>
+      <c r="AN5" s="140"/>
+      <c r="AO5" s="140"/>
+      <c r="AP5" s="140"/>
+      <c r="AQ5" s="140"/>
+      <c r="AR5" s="140"/>
+      <c r="AS5" s="140"/>
+      <c r="AT5" s="140"/>
+      <c r="AU5" s="140"/>
+      <c r="AV5" s="140"/>
+      <c r="AW5" s="140"/>
+      <c r="AX5" s="140"/>
+      <c r="AY5" s="140"/>
+      <c r="AZ5" s="140"/>
+      <c r="BA5" s="140"/>
+      <c r="BB5" s="140"/>
+      <c r="BC5" s="140"/>
+      <c r="BD5" s="140"/>
+      <c r="BE5" s="140"/>
+      <c r="BF5" s="140"/>
+      <c r="BG5" s="140"/>
+      <c r="BH5" s="140"/>
+      <c r="BI5" s="140"/>
+      <c r="BJ5" s="140"/>
+      <c r="BK5" s="140"/>
+      <c r="BL5" s="140"/>
+      <c r="BM5" s="140"/>
+      <c r="BN5" s="140"/>
+      <c r="BO5" s="140"/>
+      <c r="BP5" s="140"/>
+      <c r="BQ5" s="140"/>
+      <c r="BR5" s="140"/>
+      <c r="BS5" s="140"/>
+      <c r="BT5" s="140"/>
+      <c r="BU5" s="140"/>
+      <c r="BV5" s="140"/>
+      <c r="BW5" s="140"/>
+      <c r="BX5" s="140"/>
+      <c r="BY5" s="140"/>
+      <c r="BZ5" s="140"/>
+      <c r="CA5" s="140"/>
+      <c r="CB5" s="140"/>
+      <c r="CC5" s="140"/>
+      <c r="CD5" s="140"/>
+      <c r="CE5" s="140"/>
+      <c r="CF5" s="140"/>
+      <c r="CG5" s="140"/>
+      <c r="CH5" s="140"/>
+      <c r="CI5" s="140"/>
+      <c r="CJ5" s="140"/>
+      <c r="CK5" s="140"/>
+      <c r="CL5" s="145"/>
     </row>
     <row r="6" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="133"/>
-      <c r="B6" s="129"/>
-      <c r="C6" s="129"/>
-      <c r="D6" s="129"/>
-      <c r="E6" s="129"/>
-      <c r="F6" s="134"/>
-      <c r="G6" s="142"/>
-      <c r="H6" s="138"/>
-      <c r="I6" s="138"/>
-      <c r="J6" s="138"/>
-      <c r="K6" s="138"/>
-      <c r="L6" s="138"/>
-      <c r="M6" s="138"/>
-      <c r="N6" s="138"/>
-      <c r="O6" s="138"/>
-      <c r="P6" s="138"/>
-      <c r="Q6" s="138"/>
-      <c r="R6" s="138"/>
-      <c r="S6" s="138"/>
-      <c r="T6" s="138"/>
-      <c r="U6" s="138"/>
-      <c r="V6" s="138"/>
-      <c r="W6" s="138"/>
-      <c r="X6" s="138"/>
-      <c r="Y6" s="138"/>
-      <c r="Z6" s="138"/>
-      <c r="AA6" s="138"/>
-      <c r="AB6" s="138"/>
-      <c r="AC6" s="138"/>
-      <c r="AD6" s="138"/>
-      <c r="AE6" s="138"/>
-      <c r="AF6" s="138"/>
-      <c r="AG6" s="138"/>
-      <c r="AH6" s="138" t="s">
-        <v>128</v>
-      </c>
-      <c r="AI6" s="138"/>
-      <c r="AJ6" s="138" t="s">
+      <c r="A6" s="135"/>
+      <c r="B6" s="131"/>
+      <c r="C6" s="131"/>
+      <c r="D6" s="131"/>
+      <c r="E6" s="131"/>
+      <c r="F6" s="136"/>
+      <c r="G6" s="144"/>
+      <c r="H6" s="140"/>
+      <c r="I6" s="140"/>
+      <c r="J6" s="140"/>
+      <c r="K6" s="140"/>
+      <c r="L6" s="140"/>
+      <c r="M6" s="140"/>
+      <c r="N6" s="140"/>
+      <c r="O6" s="140"/>
+      <c r="P6" s="140"/>
+      <c r="Q6" s="140"/>
+      <c r="R6" s="140"/>
+      <c r="S6" s="140"/>
+      <c r="T6" s="140"/>
+      <c r="U6" s="140"/>
+      <c r="V6" s="140"/>
+      <c r="W6" s="140"/>
+      <c r="X6" s="140"/>
+      <c r="Y6" s="140"/>
+      <c r="Z6" s="140"/>
+      <c r="AA6" s="140"/>
+      <c r="AB6" s="140"/>
+      <c r="AC6" s="140"/>
+      <c r="AD6" s="140"/>
+      <c r="AE6" s="140"/>
+      <c r="AF6" s="140"/>
+      <c r="AG6" s="140"/>
+      <c r="AH6" s="140"/>
+      <c r="AI6" s="140"/>
+      <c r="AJ6" s="140" t="s">
+        <v>10</v>
+      </c>
+      <c r="AK6" s="140"/>
+      <c r="AL6" s="140"/>
+      <c r="AM6" s="140"/>
+      <c r="AN6" s="140" t="s">
         <v>309</v>
       </c>
-      <c r="AK6" s="138"/>
-      <c r="AL6" s="138"/>
-      <c r="AM6" s="138"/>
-      <c r="AN6" s="138"/>
-      <c r="AO6" s="138"/>
-      <c r="AP6" s="138"/>
-      <c r="AQ6" s="138"/>
-      <c r="AR6" s="138"/>
-      <c r="AS6" s="138"/>
-      <c r="AT6" s="138"/>
-      <c r="AU6" s="138"/>
-      <c r="AV6" s="138"/>
-      <c r="AW6" s="138"/>
-      <c r="AX6" s="138"/>
-      <c r="AY6" s="138"/>
-      <c r="AZ6" s="138"/>
-      <c r="BA6" s="138"/>
-      <c r="BB6" s="138"/>
-      <c r="BC6" s="138"/>
-      <c r="BD6" s="138"/>
-      <c r="BE6" s="138"/>
-      <c r="BF6" s="138"/>
-      <c r="BG6" s="138"/>
-      <c r="BH6" s="138"/>
-      <c r="BI6" s="138"/>
-      <c r="BJ6" s="138"/>
-      <c r="BK6" s="138"/>
-      <c r="BL6" s="138"/>
-      <c r="BM6" s="138"/>
-      <c r="BN6" s="138"/>
-      <c r="BO6" s="138"/>
-      <c r="BP6" s="138"/>
-      <c r="BQ6" s="138"/>
-      <c r="BR6" s="138"/>
-      <c r="BS6" s="138"/>
-      <c r="BT6" s="138"/>
-      <c r="BU6" s="138"/>
-      <c r="BV6" s="138"/>
-      <c r="BW6" s="138"/>
-      <c r="BX6" s="138"/>
-      <c r="BY6" s="138"/>
-      <c r="BZ6" s="138"/>
-      <c r="CA6" s="138"/>
-      <c r="CB6" s="138"/>
-      <c r="CC6" s="138"/>
-      <c r="CD6" s="138"/>
-      <c r="CE6" s="138"/>
-      <c r="CF6" s="138"/>
-      <c r="CG6" s="138"/>
-      <c r="CH6" s="138"/>
-      <c r="CI6" s="138"/>
-      <c r="CJ6" s="138"/>
-      <c r="CK6" s="138"/>
-      <c r="CL6" s="143"/>
+      <c r="AO6" s="140"/>
+      <c r="AP6" s="140"/>
+      <c r="AQ6" s="140"/>
+      <c r="AR6" s="140"/>
+      <c r="AS6" s="140"/>
+      <c r="AT6" s="140"/>
+      <c r="AU6" s="140"/>
+      <c r="AV6" s="140"/>
+      <c r="AW6" s="140"/>
+      <c r="AX6" s="140"/>
+      <c r="AY6" s="140"/>
+      <c r="AZ6" s="140"/>
+      <c r="BA6" s="140"/>
+      <c r="BB6" s="140"/>
+      <c r="BC6" s="140"/>
+      <c r="BD6" s="140"/>
+      <c r="BE6" s="140"/>
+      <c r="BF6" s="140"/>
+      <c r="BG6" s="140"/>
+      <c r="BH6" s="140"/>
+      <c r="BI6" s="140"/>
+      <c r="BJ6" s="140"/>
+      <c r="BK6" s="140"/>
+      <c r="BL6" s="140"/>
+      <c r="BM6" s="140"/>
+      <c r="BN6" s="140"/>
+      <c r="BO6" s="140"/>
+      <c r="BP6" s="140"/>
+      <c r="BQ6" s="140"/>
+      <c r="BR6" s="140"/>
+      <c r="BS6" s="140"/>
+      <c r="BT6" s="140"/>
+      <c r="BU6" s="140"/>
+      <c r="BV6" s="140"/>
+      <c r="BW6" s="140"/>
+      <c r="BX6" s="140"/>
+      <c r="BY6" s="140"/>
+      <c r="BZ6" s="140"/>
+      <c r="CA6" s="140"/>
+      <c r="CB6" s="140"/>
+      <c r="CC6" s="140"/>
+      <c r="CD6" s="140"/>
+      <c r="CE6" s="140"/>
+      <c r="CF6" s="140"/>
+      <c r="CG6" s="140"/>
+      <c r="CH6" s="140"/>
+      <c r="CI6" s="140"/>
+      <c r="CJ6" s="140"/>
+      <c r="CK6" s="140"/>
+      <c r="CL6" s="145"/>
     </row>
     <row r="7" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="133"/>
-      <c r="B7" s="129"/>
-      <c r="C7" s="129"/>
-      <c r="D7" s="129"/>
-      <c r="E7" s="129"/>
-      <c r="F7" s="134"/>
-      <c r="G7" s="142"/>
-      <c r="H7" s="138"/>
-      <c r="I7" s="138"/>
-      <c r="J7" s="138"/>
-      <c r="K7" s="138"/>
-      <c r="L7" s="138"/>
-      <c r="M7" s="138"/>
-      <c r="N7" s="138"/>
-      <c r="O7" s="138"/>
-      <c r="P7" s="138"/>
-      <c r="Q7" s="138"/>
-      <c r="R7" s="138"/>
-      <c r="S7" s="138"/>
-      <c r="T7" s="138"/>
-      <c r="U7" s="138"/>
-      <c r="V7" s="138"/>
-      <c r="W7" s="138"/>
-      <c r="X7" s="138"/>
-      <c r="Y7" s="138"/>
-      <c r="Z7" s="138"/>
-      <c r="AA7" s="138"/>
-      <c r="AB7" s="138"/>
-      <c r="AC7" s="138"/>
-      <c r="AD7" s="138"/>
-      <c r="AE7" s="138"/>
-      <c r="AF7" s="138"/>
-      <c r="AG7" s="138"/>
-      <c r="AH7" s="138"/>
-      <c r="AI7" s="138"/>
-      <c r="AJ7" s="138"/>
-      <c r="AK7" s="138"/>
-      <c r="AL7" s="138"/>
-      <c r="AM7" s="138"/>
-      <c r="AN7" s="138" t="s">
+      <c r="A7" s="135"/>
+      <c r="B7" s="131"/>
+      <c r="C7" s="131"/>
+      <c r="D7" s="131"/>
+      <c r="E7" s="131"/>
+      <c r="F7" s="136"/>
+      <c r="G7" s="144"/>
+      <c r="H7" s="140"/>
+      <c r="I7" s="140"/>
+      <c r="J7" s="140"/>
+      <c r="K7" s="140"/>
+      <c r="L7" s="140"/>
+      <c r="M7" s="140"/>
+      <c r="N7" s="140"/>
+      <c r="O7" s="140"/>
+      <c r="P7" s="140"/>
+      <c r="Q7" s="140"/>
+      <c r="R7" s="140"/>
+      <c r="S7" s="140"/>
+      <c r="T7" s="140"/>
+      <c r="U7" s="140"/>
+      <c r="V7" s="140"/>
+      <c r="W7" s="140"/>
+      <c r="X7" s="140"/>
+      <c r="Y7" s="140"/>
+      <c r="Z7" s="140"/>
+      <c r="AA7" s="140"/>
+      <c r="AB7" s="140"/>
+      <c r="AC7" s="140"/>
+      <c r="AD7" s="140"/>
+      <c r="AE7" s="140"/>
+      <c r="AF7" s="140"/>
+      <c r="AG7" s="140"/>
+      <c r="AH7" s="140"/>
+      <c r="AI7" s="140"/>
+      <c r="AJ7" s="140"/>
+      <c r="AK7" s="140"/>
+      <c r="AL7" s="140" t="s">
         <v>128</v>
       </c>
-      <c r="AO7" s="138"/>
-      <c r="AP7" s="138" t="s">
+      <c r="AM7" s="140"/>
+      <c r="AN7" s="140" t="s">
         <v>310</v>
       </c>
-      <c r="AQ7" s="138"/>
-      <c r="AR7" s="138"/>
-      <c r="AS7" s="138"/>
-      <c r="AT7" s="138"/>
-      <c r="AU7" s="138"/>
-      <c r="AV7" s="138"/>
-      <c r="AW7" s="138"/>
-      <c r="AX7" s="138"/>
-      <c r="AY7" s="138"/>
-      <c r="AZ7" s="138"/>
-      <c r="BA7" s="138"/>
-      <c r="BB7" s="138"/>
-      <c r="BC7" s="138"/>
-      <c r="BD7" s="138"/>
-      <c r="BE7" s="138"/>
-      <c r="BF7" s="138"/>
-      <c r="BG7" s="138"/>
-      <c r="BH7" s="138"/>
-      <c r="BI7" s="138"/>
-      <c r="BJ7" s="138"/>
-      <c r="BK7" s="138"/>
-      <c r="BL7" s="138"/>
-      <c r="BM7" s="138"/>
-      <c r="BN7" s="138"/>
-      <c r="BO7" s="138"/>
-      <c r="BP7" s="138"/>
-      <c r="BQ7" s="138"/>
-      <c r="BR7" s="138"/>
-      <c r="BS7" s="138"/>
-      <c r="BT7" s="138"/>
-      <c r="BU7" s="138"/>
-      <c r="BV7" s="138"/>
-      <c r="BW7" s="138"/>
-      <c r="BX7" s="138"/>
-      <c r="BY7" s="138"/>
-      <c r="BZ7" s="138"/>
-      <c r="CA7" s="138"/>
-      <c r="CB7" s="138"/>
-      <c r="CC7" s="138"/>
-      <c r="CD7" s="138"/>
-      <c r="CE7" s="138"/>
-      <c r="CF7" s="138"/>
-      <c r="CG7" s="138"/>
-      <c r="CH7" s="138"/>
-      <c r="CI7" s="138"/>
-      <c r="CJ7" s="138"/>
-      <c r="CK7" s="138"/>
-      <c r="CL7" s="143"/>
+      <c r="AO7" s="140"/>
+      <c r="AP7" s="140"/>
+      <c r="AQ7" s="140"/>
+      <c r="AR7" s="140"/>
+      <c r="AS7" s="140"/>
+      <c r="AT7" s="140"/>
+      <c r="AU7" s="140"/>
+      <c r="AV7" s="140"/>
+      <c r="AW7" s="140"/>
+      <c r="AX7" s="140"/>
+      <c r="AY7" s="140"/>
+      <c r="AZ7" s="140"/>
+      <c r="BA7" s="140"/>
+      <c r="BB7" s="140"/>
+      <c r="BC7" s="140"/>
+      <c r="BD7" s="140"/>
+      <c r="BE7" s="140"/>
+      <c r="BF7" s="140"/>
+      <c r="BG7" s="140"/>
+      <c r="BH7" s="140"/>
+      <c r="BI7" s="140"/>
+      <c r="BJ7" s="140"/>
+      <c r="BK7" s="140"/>
+      <c r="BL7" s="140"/>
+      <c r="BM7" s="140"/>
+      <c r="BN7" s="140"/>
+      <c r="BO7" s="140"/>
+      <c r="BP7" s="140"/>
+      <c r="BQ7" s="140"/>
+      <c r="BR7" s="140"/>
+      <c r="BS7" s="140"/>
+      <c r="BT7" s="140"/>
+      <c r="BU7" s="140"/>
+      <c r="BV7" s="140"/>
+      <c r="BW7" s="140"/>
+      <c r="BX7" s="140"/>
+      <c r="BY7" s="140"/>
+      <c r="BZ7" s="140"/>
+      <c r="CA7" s="140"/>
+      <c r="CB7" s="140"/>
+      <c r="CC7" s="140"/>
+      <c r="CD7" s="140"/>
+      <c r="CE7" s="140"/>
+      <c r="CF7" s="140"/>
+      <c r="CG7" s="140"/>
+      <c r="CH7" s="140"/>
+      <c r="CI7" s="140"/>
+      <c r="CJ7" s="140"/>
+      <c r="CK7" s="140"/>
+      <c r="CL7" s="145"/>
     </row>
     <row r="8" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="133"/>
-      <c r="B8" s="129"/>
-      <c r="C8" s="129"/>
-      <c r="D8" s="129"/>
-      <c r="E8" s="129"/>
-      <c r="F8" s="134"/>
-      <c r="G8" s="142"/>
-      <c r="H8" s="138"/>
-      <c r="I8" s="138"/>
-      <c r="J8" s="138"/>
-      <c r="K8" s="138"/>
-      <c r="L8" s="138"/>
-      <c r="M8" s="138"/>
-      <c r="N8" s="138"/>
-      <c r="O8" s="138"/>
-      <c r="P8" s="138"/>
-      <c r="Q8" s="138"/>
-      <c r="R8" s="138"/>
-      <c r="S8" s="138"/>
-      <c r="T8" s="138"/>
-      <c r="U8" s="138"/>
-      <c r="V8" s="138"/>
-      <c r="W8" s="138"/>
-      <c r="X8" s="138"/>
-      <c r="Y8" s="138"/>
-      <c r="Z8" s="138"/>
-      <c r="AA8" s="138"/>
-      <c r="AB8" s="138"/>
-      <c r="AC8" s="138"/>
-      <c r="AD8" s="138"/>
-      <c r="AE8" s="138"/>
-      <c r="AF8" s="138"/>
-      <c r="AG8" s="138"/>
-      <c r="AH8" s="138"/>
-      <c r="AI8" s="138"/>
-      <c r="AJ8" s="138"/>
-      <c r="AK8" s="138"/>
-      <c r="AL8" s="138" t="s">
-        <v>10</v>
-      </c>
-      <c r="AM8" s="138"/>
-      <c r="AN8" s="138"/>
-      <c r="AO8" s="138"/>
-      <c r="AP8" s="138" t="s">
+      <c r="A8" s="135"/>
+      <c r="B8" s="131"/>
+      <c r="C8" s="131"/>
+      <c r="D8" s="131"/>
+      <c r="E8" s="131"/>
+      <c r="F8" s="136"/>
+      <c r="G8" s="144"/>
+      <c r="H8" s="140"/>
+      <c r="I8" s="140"/>
+      <c r="J8" s="140"/>
+      <c r="K8" s="140"/>
+      <c r="L8" s="140"/>
+      <c r="M8" s="140"/>
+      <c r="N8" s="140"/>
+      <c r="O8" s="140"/>
+      <c r="P8" s="140"/>
+      <c r="Q8" s="140"/>
+      <c r="R8" s="140"/>
+      <c r="S8" s="140"/>
+      <c r="T8" s="140"/>
+      <c r="U8" s="140"/>
+      <c r="V8" s="140"/>
+      <c r="W8" s="140"/>
+      <c r="X8" s="140"/>
+      <c r="Y8" s="140"/>
+      <c r="Z8" s="140"/>
+      <c r="AA8" s="140"/>
+      <c r="AB8" s="140"/>
+      <c r="AC8" s="140"/>
+      <c r="AD8" s="140"/>
+      <c r="AE8" s="140"/>
+      <c r="AF8" s="140"/>
+      <c r="AG8" s="140"/>
+      <c r="AH8" s="140"/>
+      <c r="AI8" s="140"/>
+      <c r="AJ8" s="140" t="s">
         <v>311</v>
       </c>
-      <c r="AQ8" s="138"/>
-      <c r="AR8" s="138"/>
-      <c r="AS8" s="138"/>
-      <c r="AT8" s="138"/>
-      <c r="AU8" s="138"/>
-      <c r="AV8" s="138"/>
-      <c r="AW8" s="138"/>
-      <c r="AX8" s="138"/>
-      <c r="AY8" s="138"/>
-      <c r="AZ8" s="138"/>
-      <c r="BA8" s="138"/>
-      <c r="BB8" s="138"/>
-      <c r="BC8" s="138"/>
-      <c r="BD8" s="138"/>
-      <c r="BE8" s="138"/>
-      <c r="BF8" s="138"/>
-      <c r="BG8" s="138"/>
-      <c r="BH8" s="138"/>
-      <c r="BI8" s="138"/>
-      <c r="BJ8" s="138"/>
-      <c r="BK8" s="138"/>
-      <c r="BL8" s="138"/>
-      <c r="BM8" s="138"/>
-      <c r="BN8" s="138"/>
-      <c r="BO8" s="138"/>
-      <c r="BP8" s="138"/>
-      <c r="BQ8" s="138"/>
-      <c r="BR8" s="138"/>
-      <c r="BS8" s="138"/>
-      <c r="BT8" s="138"/>
-      <c r="BU8" s="138"/>
-      <c r="BV8" s="138"/>
-      <c r="BW8" s="138"/>
-      <c r="BX8" s="138"/>
-      <c r="BY8" s="138"/>
-      <c r="BZ8" s="138"/>
-      <c r="CA8" s="138"/>
-      <c r="CB8" s="138"/>
-      <c r="CC8" s="138"/>
-      <c r="CD8" s="138"/>
-      <c r="CE8" s="138"/>
-      <c r="CF8" s="138"/>
-      <c r="CG8" s="138"/>
-      <c r="CH8" s="138"/>
-      <c r="CI8" s="138"/>
-      <c r="CJ8" s="138"/>
-      <c r="CK8" s="138"/>
-      <c r="CL8" s="143"/>
+      <c r="AK8" s="140"/>
+      <c r="AL8" s="140"/>
+      <c r="AM8" s="140"/>
+      <c r="AN8" s="140"/>
+      <c r="AO8" s="140"/>
+      <c r="AP8" s="140"/>
+      <c r="AQ8" s="140"/>
+      <c r="AR8" s="140"/>
+      <c r="AS8" s="140"/>
+      <c r="AT8" s="140"/>
+      <c r="AU8" s="140"/>
+      <c r="AV8" s="140"/>
+      <c r="AW8" s="140"/>
+      <c r="AX8" s="140"/>
+      <c r="AY8" s="140"/>
+      <c r="AZ8" s="140"/>
+      <c r="BA8" s="140"/>
+      <c r="BB8" s="140"/>
+      <c r="BC8" s="140"/>
+      <c r="BD8" s="140"/>
+      <c r="BE8" s="140"/>
+      <c r="BF8" s="140"/>
+      <c r="BG8" s="140"/>
+      <c r="BH8" s="140"/>
+      <c r="BI8" s="140"/>
+      <c r="BJ8" s="140"/>
+      <c r="BK8" s="140"/>
+      <c r="BL8" s="140"/>
+      <c r="BM8" s="140"/>
+      <c r="BN8" s="140"/>
+      <c r="BO8" s="140"/>
+      <c r="BP8" s="140"/>
+      <c r="BQ8" s="140"/>
+      <c r="BR8" s="140"/>
+      <c r="BS8" s="140"/>
+      <c r="BT8" s="140"/>
+      <c r="BU8" s="140"/>
+      <c r="BV8" s="140"/>
+      <c r="BW8" s="140"/>
+      <c r="BX8" s="140"/>
+      <c r="BY8" s="140"/>
+      <c r="BZ8" s="140"/>
+      <c r="CA8" s="140"/>
+      <c r="CB8" s="140"/>
+      <c r="CC8" s="140"/>
+      <c r="CD8" s="140"/>
+      <c r="CE8" s="140"/>
+      <c r="CF8" s="140"/>
+      <c r="CG8" s="140"/>
+      <c r="CH8" s="140"/>
+      <c r="CI8" s="140"/>
+      <c r="CJ8" s="140"/>
+      <c r="CK8" s="140"/>
+      <c r="CL8" s="145"/>
     </row>
     <row r="9" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="133"/>
-      <c r="B9" s="129"/>
-      <c r="C9" s="129"/>
-      <c r="D9" s="129"/>
-      <c r="E9" s="129"/>
-      <c r="F9" s="134"/>
-      <c r="G9" s="142"/>
-      <c r="H9" s="138"/>
-      <c r="I9" s="138"/>
-      <c r="J9" s="138"/>
-      <c r="K9" s="138"/>
-      <c r="L9" s="138"/>
-      <c r="M9" s="138"/>
-      <c r="N9" s="138"/>
-      <c r="O9" s="138"/>
-      <c r="P9" s="138"/>
-      <c r="Q9" s="138"/>
-      <c r="R9" s="138"/>
-      <c r="S9" s="138"/>
-      <c r="T9" s="138"/>
-      <c r="U9" s="138"/>
-      <c r="V9" s="138"/>
-      <c r="W9" s="138"/>
-      <c r="X9" s="138"/>
-      <c r="Y9" s="138"/>
-      <c r="Z9" s="138"/>
-      <c r="AA9" s="138"/>
-      <c r="AB9" s="138"/>
-      <c r="AC9" s="138"/>
-      <c r="AD9" s="138"/>
-      <c r="AE9" s="138"/>
-      <c r="AF9" s="138"/>
-      <c r="AG9" s="138"/>
-      <c r="AH9" s="138"/>
-      <c r="AI9" s="138"/>
-      <c r="AJ9" s="138"/>
-      <c r="AK9" s="138"/>
-      <c r="AL9" s="138"/>
-      <c r="AM9" s="138"/>
-      <c r="AN9" s="138" t="s">
-        <v>128</v>
-      </c>
-      <c r="AO9" s="138"/>
-      <c r="AP9" s="138" t="s">
+      <c r="A9" s="135"/>
+      <c r="B9" s="131"/>
+      <c r="C9" s="131"/>
+      <c r="D9" s="131"/>
+      <c r="E9" s="131"/>
+      <c r="F9" s="136"/>
+      <c r="G9" s="144"/>
+      <c r="H9" s="140"/>
+      <c r="I9" s="140"/>
+      <c r="J9" s="140"/>
+      <c r="K9" s="140"/>
+      <c r="L9" s="140"/>
+      <c r="M9" s="140"/>
+      <c r="N9" s="140"/>
+      <c r="O9" s="140"/>
+      <c r="P9" s="140"/>
+      <c r="Q9" s="140"/>
+      <c r="R9" s="140"/>
+      <c r="S9" s="140"/>
+      <c r="T9" s="140"/>
+      <c r="U9" s="140"/>
+      <c r="V9" s="140"/>
+      <c r="W9" s="140"/>
+      <c r="X9" s="140"/>
+      <c r="Y9" s="140"/>
+      <c r="Z9" s="140"/>
+      <c r="AA9" s="140"/>
+      <c r="AB9" s="140"/>
+      <c r="AC9" s="140"/>
+      <c r="AD9" s="140"/>
+      <c r="AE9" s="140"/>
+      <c r="AF9" s="140" t="s">
         <v>312</v>
       </c>
-      <c r="AQ9" s="138"/>
-      <c r="AR9" s="138"/>
-      <c r="AS9" s="138"/>
-      <c r="AT9" s="138"/>
-      <c r="AU9" s="138"/>
-      <c r="AV9" s="138"/>
-      <c r="AW9" s="138"/>
-      <c r="AX9" s="138"/>
-      <c r="AY9" s="138"/>
-      <c r="AZ9" s="138"/>
-      <c r="BA9" s="138"/>
-      <c r="BB9" s="138"/>
-      <c r="BC9" s="138"/>
-      <c r="BD9" s="138"/>
-      <c r="BE9" s="138"/>
-      <c r="BF9" s="138"/>
-      <c r="BG9" s="138"/>
-      <c r="BH9" s="138"/>
-      <c r="BI9" s="138"/>
-      <c r="BJ9" s="138"/>
-      <c r="BK9" s="138"/>
-      <c r="BL9" s="138"/>
-      <c r="BM9" s="138"/>
-      <c r="BN9" s="138"/>
-      <c r="BO9" s="138"/>
-      <c r="BP9" s="138"/>
-      <c r="BQ9" s="138"/>
-      <c r="BR9" s="138"/>
-      <c r="BS9" s="138"/>
-      <c r="BT9" s="138"/>
-      <c r="BU9" s="138"/>
-      <c r="BV9" s="138"/>
-      <c r="BW9" s="138"/>
-      <c r="BX9" s="138"/>
-      <c r="BY9" s="138"/>
-      <c r="BZ9" s="138"/>
-      <c r="CA9" s="138"/>
-      <c r="CB9" s="138"/>
-      <c r="CC9" s="138"/>
-      <c r="CD9" s="138"/>
-      <c r="CE9" s="138"/>
-      <c r="CF9" s="138"/>
-      <c r="CG9" s="138"/>
-      <c r="CH9" s="138"/>
-      <c r="CI9" s="138"/>
-      <c r="CJ9" s="138"/>
-      <c r="CK9" s="138"/>
-      <c r="CL9" s="143"/>
+      <c r="AG9" s="140"/>
+      <c r="AH9" s="140"/>
+      <c r="AI9" s="140"/>
+      <c r="AJ9" s="140"/>
+      <c r="AK9" s="140"/>
+      <c r="AL9" s="140"/>
+      <c r="AM9" s="140"/>
+      <c r="AN9" s="140"/>
+      <c r="AO9" s="140"/>
+      <c r="AP9" s="140"/>
+      <c r="AQ9" s="140"/>
+      <c r="AR9" s="140"/>
+      <c r="AS9" s="140"/>
+      <c r="AT9" s="140"/>
+      <c r="AU9" s="140"/>
+      <c r="AV9" s="140"/>
+      <c r="AW9" s="140"/>
+      <c r="AX9" s="140"/>
+      <c r="AY9" s="140"/>
+      <c r="AZ9" s="140"/>
+      <c r="BA9" s="140"/>
+      <c r="BB9" s="140"/>
+      <c r="BC9" s="140"/>
+      <c r="BD9" s="140"/>
+      <c r="BE9" s="140"/>
+      <c r="BF9" s="140"/>
+      <c r="BG9" s="140"/>
+      <c r="BH9" s="140"/>
+      <c r="BI9" s="140"/>
+      <c r="BJ9" s="140"/>
+      <c r="BK9" s="140"/>
+      <c r="BL9" s="140"/>
+      <c r="BM9" s="140"/>
+      <c r="BN9" s="140"/>
+      <c r="BO9" s="140"/>
+      <c r="BP9" s="140"/>
+      <c r="BQ9" s="140"/>
+      <c r="BR9" s="140"/>
+      <c r="BS9" s="140"/>
+      <c r="BT9" s="140"/>
+      <c r="BU9" s="140"/>
+      <c r="BV9" s="140"/>
+      <c r="BW9" s="140"/>
+      <c r="BX9" s="140"/>
+      <c r="BY9" s="140"/>
+      <c r="BZ9" s="140"/>
+      <c r="CA9" s="140"/>
+      <c r="CB9" s="140"/>
+      <c r="CC9" s="140"/>
+      <c r="CD9" s="140"/>
+      <c r="CE9" s="140"/>
+      <c r="CF9" s="140"/>
+      <c r="CG9" s="140"/>
+      <c r="CH9" s="140"/>
+      <c r="CI9" s="140"/>
+      <c r="CJ9" s="140"/>
+      <c r="CK9" s="140"/>
+      <c r="CL9" s="145"/>
     </row>
     <row r="10" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="133"/>
-      <c r="B10" s="129"/>
-      <c r="C10" s="129"/>
-      <c r="D10" s="129"/>
-      <c r="E10" s="129"/>
-      <c r="F10" s="134"/>
-      <c r="G10" s="142"/>
-      <c r="H10" s="138"/>
-      <c r="I10" s="138"/>
-      <c r="J10" s="138"/>
-      <c r="K10" s="138"/>
-      <c r="L10" s="138"/>
-      <c r="M10" s="138"/>
-      <c r="N10" s="138"/>
-      <c r="O10" s="138"/>
-      <c r="P10" s="138"/>
-      <c r="Q10" s="138"/>
-      <c r="R10" s="138"/>
-      <c r="S10" s="138"/>
-      <c r="T10" s="138"/>
-      <c r="U10" s="138"/>
-      <c r="V10" s="138"/>
-      <c r="W10" s="138"/>
-      <c r="X10" s="138"/>
-      <c r="Y10" s="138"/>
-      <c r="Z10" s="138"/>
-      <c r="AA10" s="138"/>
-      <c r="AB10" s="138"/>
-      <c r="AC10" s="138"/>
-      <c r="AD10" s="138"/>
-      <c r="AE10" s="138"/>
-      <c r="AF10" s="138"/>
-      <c r="AG10" s="138"/>
-      <c r="AH10" s="138"/>
-      <c r="AI10" s="138"/>
-      <c r="AJ10" s="138"/>
-      <c r="AK10" s="138"/>
-      <c r="AL10" s="138"/>
-      <c r="AM10" s="138"/>
-      <c r="AN10" s="138"/>
-      <c r="AO10" s="138"/>
-      <c r="AP10" s="138"/>
-      <c r="AQ10" s="138"/>
-      <c r="AR10" s="138"/>
-      <c r="AS10" s="138"/>
-      <c r="AT10" s="138" t="s">
+      <c r="A10" s="135"/>
+      <c r="B10" s="131"/>
+      <c r="C10" s="131"/>
+      <c r="D10" s="131"/>
+      <c r="E10" s="131"/>
+      <c r="F10" s="136"/>
+      <c r="G10" s="144"/>
+      <c r="H10" s="140"/>
+      <c r="I10" s="140"/>
+      <c r="J10" s="140"/>
+      <c r="K10" s="140"/>
+      <c r="L10" s="140"/>
+      <c r="M10" s="140"/>
+      <c r="N10" s="140"/>
+      <c r="O10" s="140"/>
+      <c r="P10" s="140"/>
+      <c r="Q10" s="140"/>
+      <c r="R10" s="140"/>
+      <c r="S10" s="140"/>
+      <c r="T10" s="140"/>
+      <c r="U10" s="140"/>
+      <c r="V10" s="140"/>
+      <c r="W10" s="140"/>
+      <c r="X10" s="140"/>
+      <c r="Y10" s="140"/>
+      <c r="Z10" s="140"/>
+      <c r="AA10" s="140"/>
+      <c r="AB10" s="140"/>
+      <c r="AC10" s="140"/>
+      <c r="AD10" s="140"/>
+      <c r="AE10" s="140"/>
+      <c r="AF10" s="140"/>
+      <c r="AG10" s="140"/>
+      <c r="AH10" s="140"/>
+      <c r="AI10" s="140"/>
+      <c r="AJ10" s="140" t="s">
         <v>128</v>
       </c>
-      <c r="AU10" s="138"/>
-      <c r="AV10" s="138" t="s">
+      <c r="AK10" s="140"/>
+      <c r="AL10" s="140" t="s">
         <v>313</v>
       </c>
-      <c r="AW10" s="138"/>
-      <c r="AX10" s="138"/>
-      <c r="AY10" s="138"/>
-      <c r="AZ10" s="138"/>
-      <c r="BA10" s="138"/>
-      <c r="BB10" s="138"/>
-      <c r="BC10" s="138"/>
-      <c r="BD10" s="138"/>
-      <c r="BE10" s="138"/>
-      <c r="BF10" s="138"/>
-      <c r="BG10" s="138"/>
-      <c r="BH10" s="138"/>
-      <c r="BI10" s="138"/>
-      <c r="BJ10" s="138"/>
-      <c r="BK10" s="138"/>
-      <c r="BL10" s="138"/>
-      <c r="BM10" s="138"/>
-      <c r="BN10" s="138"/>
-      <c r="BO10" s="138"/>
-      <c r="BP10" s="138"/>
-      <c r="BQ10" s="138"/>
-      <c r="BR10" s="138"/>
-      <c r="BS10" s="138"/>
-      <c r="BT10" s="138"/>
-      <c r="BU10" s="138"/>
-      <c r="BV10" s="138"/>
-      <c r="BW10" s="138"/>
-      <c r="BX10" s="138"/>
-      <c r="BY10" s="138"/>
-      <c r="BZ10" s="138"/>
-      <c r="CA10" s="138"/>
-      <c r="CB10" s="138"/>
-      <c r="CC10" s="138"/>
-      <c r="CD10" s="138"/>
-      <c r="CE10" s="138"/>
-      <c r="CF10" s="138"/>
-      <c r="CG10" s="138"/>
-      <c r="CH10" s="138"/>
-      <c r="CI10" s="138"/>
-      <c r="CJ10" s="138"/>
-      <c r="CK10" s="138"/>
-      <c r="CL10" s="143"/>
+      <c r="AM10" s="140"/>
+      <c r="AN10" s="140"/>
+      <c r="AO10" s="140"/>
+      <c r="AP10" s="140"/>
+      <c r="AQ10" s="140"/>
+      <c r="AR10" s="140"/>
+      <c r="AS10" s="140"/>
+      <c r="AT10" s="140"/>
+      <c r="AU10" s="140"/>
+      <c r="AV10" s="140"/>
+      <c r="AW10" s="140"/>
+      <c r="AX10" s="140"/>
+      <c r="AY10" s="140"/>
+      <c r="AZ10" s="140"/>
+      <c r="BA10" s="140"/>
+      <c r="BB10" s="140"/>
+      <c r="BC10" s="140"/>
+      <c r="BD10" s="140"/>
+      <c r="BE10" s="140"/>
+      <c r="BF10" s="140"/>
+      <c r="BG10" s="140"/>
+      <c r="BH10" s="140"/>
+      <c r="BI10" s="140"/>
+      <c r="BJ10" s="140"/>
+      <c r="BK10" s="140"/>
+      <c r="BL10" s="140"/>
+      <c r="BM10" s="140"/>
+      <c r="BN10" s="140"/>
+      <c r="BO10" s="140"/>
+      <c r="BP10" s="140"/>
+      <c r="BQ10" s="140"/>
+      <c r="BR10" s="140"/>
+      <c r="BS10" s="140"/>
+      <c r="BT10" s="140"/>
+      <c r="BU10" s="140"/>
+      <c r="BV10" s="140"/>
+      <c r="BW10" s="140"/>
+      <c r="BX10" s="140"/>
+      <c r="BY10" s="140"/>
+      <c r="BZ10" s="140"/>
+      <c r="CA10" s="140"/>
+      <c r="CB10" s="140"/>
+      <c r="CC10" s="140"/>
+      <c r="CD10" s="140"/>
+      <c r="CE10" s="140"/>
+      <c r="CF10" s="140"/>
+      <c r="CG10" s="140"/>
+      <c r="CH10" s="140"/>
+      <c r="CI10" s="140"/>
+      <c r="CJ10" s="140"/>
+      <c r="CK10" s="140"/>
+      <c r="CL10" s="145"/>
     </row>
     <row r="11" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="133"/>
-      <c r="B11" s="129"/>
-      <c r="C11" s="129"/>
-      <c r="D11" s="129"/>
-      <c r="E11" s="129"/>
-      <c r="F11" s="134"/>
-      <c r="G11" s="142"/>
-      <c r="H11" s="138"/>
-      <c r="I11" s="138"/>
-      <c r="J11" s="138"/>
-      <c r="K11" s="138"/>
-      <c r="L11" s="138"/>
-      <c r="M11" s="138"/>
-      <c r="N11" s="138"/>
-      <c r="O11" s="138"/>
-      <c r="P11" s="138"/>
-      <c r="Q11" s="138"/>
-      <c r="R11" s="138"/>
-      <c r="S11" s="138"/>
-      <c r="T11" s="138"/>
-      <c r="U11" s="138"/>
-      <c r="V11" s="138"/>
-      <c r="W11" s="138"/>
-      <c r="X11" s="138"/>
-      <c r="Y11" s="138"/>
-      <c r="Z11" s="138"/>
-      <c r="AA11" s="138"/>
-      <c r="AB11" s="138"/>
-      <c r="AC11" s="138"/>
-      <c r="AD11" s="138"/>
-      <c r="AE11" s="138"/>
-      <c r="AF11" s="138"/>
-      <c r="AG11" s="138"/>
-      <c r="AH11" s="138"/>
-      <c r="AI11" s="138"/>
-      <c r="AJ11" s="138"/>
-      <c r="AK11" s="138"/>
-      <c r="AL11" s="138"/>
-      <c r="AM11" s="138"/>
-      <c r="AN11" s="138"/>
-      <c r="AO11" s="138"/>
-      <c r="AP11" s="138"/>
-      <c r="AQ11" s="138"/>
-      <c r="AR11" s="138" t="s">
+      <c r="A11" s="135"/>
+      <c r="B11" s="131"/>
+      <c r="C11" s="131"/>
+      <c r="D11" s="131"/>
+      <c r="E11" s="131"/>
+      <c r="F11" s="136"/>
+      <c r="G11" s="144"/>
+      <c r="H11" s="140"/>
+      <c r="I11" s="140"/>
+      <c r="J11" s="140"/>
+      <c r="K11" s="140"/>
+      <c r="L11" s="140"/>
+      <c r="M11" s="140"/>
+      <c r="N11" s="140"/>
+      <c r="O11" s="140"/>
+      <c r="P11" s="140"/>
+      <c r="Q11" s="140"/>
+      <c r="R11" s="140"/>
+      <c r="S11" s="140"/>
+      <c r="T11" s="140"/>
+      <c r="U11" s="140"/>
+      <c r="V11" s="140"/>
+      <c r="W11" s="140"/>
+      <c r="X11" s="140"/>
+      <c r="Y11" s="140"/>
+      <c r="Z11" s="140"/>
+      <c r="AA11" s="140"/>
+      <c r="AB11" s="140"/>
+      <c r="AC11" s="140"/>
+      <c r="AD11" s="140"/>
+      <c r="AE11" s="140"/>
+      <c r="AF11" s="140"/>
+      <c r="AG11" s="140"/>
+      <c r="AH11" s="140" t="s">
         <v>10</v>
       </c>
-      <c r="AS11" s="138"/>
-      <c r="AT11" s="138"/>
-      <c r="AU11" s="138"/>
-      <c r="AV11" s="138" t="s">
+      <c r="AI11" s="140"/>
+      <c r="AJ11" s="140" t="s">
         <v>314</v>
       </c>
-      <c r="AW11" s="138"/>
-      <c r="AX11" s="138"/>
-      <c r="AY11" s="138"/>
-      <c r="AZ11" s="138"/>
-      <c r="BA11" s="138"/>
-      <c r="BB11" s="138"/>
-      <c r="BC11" s="138"/>
-      <c r="BD11" s="138"/>
-      <c r="BE11" s="138"/>
-      <c r="BF11" s="138"/>
-      <c r="BG11" s="138"/>
-      <c r="BH11" s="138"/>
-      <c r="BI11" s="138"/>
-      <c r="BJ11" s="138"/>
-      <c r="BK11" s="138"/>
-      <c r="BL11" s="138"/>
-      <c r="BM11" s="138"/>
-      <c r="BN11" s="138"/>
-      <c r="BO11" s="138"/>
-      <c r="BP11" s="138"/>
-      <c r="BQ11" s="138"/>
-      <c r="BR11" s="138"/>
-      <c r="BS11" s="138"/>
-      <c r="BT11" s="138"/>
-      <c r="BU11" s="138"/>
-      <c r="BV11" s="138"/>
-      <c r="BW11" s="138"/>
-      <c r="BX11" s="138"/>
-      <c r="BY11" s="138"/>
-      <c r="BZ11" s="138"/>
-      <c r="CA11" s="138"/>
-      <c r="CB11" s="138"/>
-      <c r="CC11" s="138"/>
-      <c r="CD11" s="138"/>
-      <c r="CE11" s="138"/>
-      <c r="CF11" s="138"/>
-      <c r="CG11" s="138"/>
-      <c r="CH11" s="138"/>
-      <c r="CI11" s="138"/>
-      <c r="CJ11" s="138"/>
-      <c r="CK11" s="138"/>
-      <c r="CL11" s="143"/>
+      <c r="AK11" s="140"/>
+      <c r="AL11" s="140"/>
+      <c r="AM11" s="140"/>
+      <c r="AN11" s="140"/>
+      <c r="AO11" s="140"/>
+      <c r="AP11" s="140"/>
+      <c r="AQ11" s="140"/>
+      <c r="AR11" s="140"/>
+      <c r="AS11" s="140"/>
+      <c r="AT11" s="140"/>
+      <c r="AU11" s="140"/>
+      <c r="AV11" s="140"/>
+      <c r="AW11" s="140"/>
+      <c r="AX11" s="140"/>
+      <c r="AY11" s="140"/>
+      <c r="AZ11" s="140"/>
+      <c r="BA11" s="140"/>
+      <c r="BB11" s="140"/>
+      <c r="BC11" s="140"/>
+      <c r="BD11" s="140"/>
+      <c r="BE11" s="140"/>
+      <c r="BF11" s="140"/>
+      <c r="BG11" s="140"/>
+      <c r="BH11" s="140"/>
+      <c r="BI11" s="140"/>
+      <c r="BJ11" s="140"/>
+      <c r="BK11" s="140"/>
+      <c r="BL11" s="140"/>
+      <c r="BM11" s="140"/>
+      <c r="BN11" s="140"/>
+      <c r="BO11" s="140"/>
+      <c r="BP11" s="140"/>
+      <c r="BQ11" s="140"/>
+      <c r="BR11" s="140"/>
+      <c r="BS11" s="140"/>
+      <c r="BT11" s="140"/>
+      <c r="BU11" s="140"/>
+      <c r="BV11" s="140"/>
+      <c r="BW11" s="140"/>
+      <c r="BX11" s="140"/>
+      <c r="BY11" s="140"/>
+      <c r="BZ11" s="140"/>
+      <c r="CA11" s="140"/>
+      <c r="CB11" s="140"/>
+      <c r="CC11" s="140"/>
+      <c r="CD11" s="140"/>
+      <c r="CE11" s="140"/>
+      <c r="CF11" s="140"/>
+      <c r="CG11" s="140"/>
+      <c r="CH11" s="140"/>
+      <c r="CI11" s="140"/>
+      <c r="CJ11" s="140"/>
+      <c r="CK11" s="140"/>
+      <c r="CL11" s="145"/>
     </row>
     <row r="12" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="133"/>
-      <c r="B12" s="129"/>
-      <c r="C12" s="129"/>
-      <c r="D12" s="129"/>
-      <c r="E12" s="129"/>
-      <c r="F12" s="134"/>
-      <c r="G12" s="142"/>
-      <c r="H12" s="138"/>
-      <c r="I12" s="138"/>
-      <c r="J12" s="138"/>
-      <c r="K12" s="138"/>
-      <c r="L12" s="138"/>
-      <c r="M12" s="138"/>
-      <c r="N12" s="138"/>
-      <c r="O12" s="138"/>
-      <c r="P12" s="138"/>
-      <c r="Q12" s="138"/>
-      <c r="R12" s="138"/>
-      <c r="S12" s="138"/>
-      <c r="T12" s="138"/>
-      <c r="U12" s="138"/>
-      <c r="V12" s="138"/>
-      <c r="W12" s="138"/>
-      <c r="X12" s="138"/>
-      <c r="Y12" s="138"/>
-      <c r="Z12" s="138"/>
-      <c r="AA12" s="138"/>
-      <c r="AB12" s="138"/>
-      <c r="AC12" s="138"/>
-      <c r="AD12" s="138"/>
-      <c r="AE12" s="138"/>
-      <c r="AF12" s="138"/>
-      <c r="AG12" s="138"/>
-      <c r="AH12" s="138"/>
-      <c r="AI12" s="138"/>
-      <c r="AJ12" s="138"/>
-      <c r="AK12" s="138"/>
-      <c r="AL12" s="138"/>
-      <c r="AM12" s="138"/>
-      <c r="AN12" s="138"/>
-      <c r="AO12" s="138"/>
-      <c r="AP12" s="138"/>
-      <c r="AQ12" s="138"/>
-      <c r="AR12" s="138"/>
-      <c r="AS12" s="138"/>
-      <c r="AT12" s="138" t="s">
-        <v>128</v>
-      </c>
-      <c r="AU12" s="138"/>
-      <c r="AV12" s="138" t="s">
+      <c r="A12" s="137"/>
+      <c r="B12" s="138"/>
+      <c r="C12" s="138"/>
+      <c r="D12" s="138"/>
+      <c r="E12" s="138"/>
+      <c r="F12" s="139"/>
+      <c r="G12" s="146"/>
+      <c r="H12" s="147"/>
+      <c r="I12" s="147"/>
+      <c r="J12" s="147"/>
+      <c r="K12" s="147"/>
+      <c r="L12" s="147"/>
+      <c r="M12" s="147"/>
+      <c r="N12" s="147"/>
+      <c r="O12" s="147"/>
+      <c r="P12" s="147"/>
+      <c r="Q12" s="147"/>
+      <c r="R12" s="147"/>
+      <c r="S12" s="147"/>
+      <c r="T12" s="147"/>
+      <c r="U12" s="147"/>
+      <c r="V12" s="147"/>
+      <c r="W12" s="147"/>
+      <c r="X12" s="147"/>
+      <c r="Y12" s="147"/>
+      <c r="Z12" s="147"/>
+      <c r="AA12" s="147"/>
+      <c r="AB12" s="147"/>
+      <c r="AC12" s="147"/>
+      <c r="AD12" s="147"/>
+      <c r="AE12" s="147"/>
+      <c r="AF12" s="147"/>
+      <c r="AG12" s="147"/>
+      <c r="AH12" s="147" t="s">
         <v>315</v>
       </c>
-      <c r="AW12" s="138"/>
-      <c r="AX12" s="138"/>
-      <c r="AY12" s="138"/>
-      <c r="AZ12" s="138"/>
-      <c r="BA12" s="138"/>
-      <c r="BB12" s="138"/>
-      <c r="BC12" s="138"/>
-      <c r="BD12" s="138"/>
-      <c r="BE12" s="138"/>
-      <c r="BF12" s="138"/>
-      <c r="BG12" s="138"/>
-      <c r="BH12" s="138"/>
-      <c r="BI12" s="138"/>
-      <c r="BJ12" s="138"/>
-      <c r="BK12" s="138"/>
-      <c r="BL12" s="138"/>
-      <c r="BM12" s="138"/>
-      <c r="BN12" s="138"/>
-      <c r="BO12" s="138"/>
-      <c r="BP12" s="138"/>
-      <c r="BQ12" s="138"/>
-      <c r="BR12" s="138"/>
-      <c r="BS12" s="138"/>
-      <c r="BT12" s="138"/>
-      <c r="BU12" s="138"/>
-      <c r="BV12" s="138"/>
-      <c r="BW12" s="138"/>
-      <c r="BX12" s="138"/>
-      <c r="BY12" s="138"/>
-      <c r="BZ12" s="138"/>
-      <c r="CA12" s="138"/>
-      <c r="CB12" s="138"/>
-      <c r="CC12" s="138"/>
-      <c r="CD12" s="138"/>
-      <c r="CE12" s="138"/>
-      <c r="CF12" s="138"/>
-      <c r="CG12" s="138"/>
-      <c r="CH12" s="138"/>
-      <c r="CI12" s="138"/>
-      <c r="CJ12" s="138"/>
-      <c r="CK12" s="138"/>
-      <c r="CL12" s="143"/>
-    </row>
-    <row r="13" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="133"/>
-      <c r="B13" s="129"/>
-      <c r="C13" s="129"/>
-      <c r="D13" s="129"/>
-      <c r="E13" s="129"/>
-      <c r="F13" s="134"/>
-      <c r="G13" s="142"/>
-      <c r="H13" s="138"/>
-      <c r="I13" s="138"/>
-      <c r="J13" s="138"/>
-      <c r="K13" s="138"/>
-      <c r="L13" s="138"/>
-      <c r="M13" s="138"/>
-      <c r="N13" s="138"/>
-      <c r="O13" s="138"/>
-      <c r="P13" s="138"/>
-      <c r="Q13" s="138"/>
-      <c r="R13" s="138"/>
-      <c r="S13" s="138"/>
-      <c r="T13" s="138"/>
-      <c r="U13" s="138"/>
-      <c r="V13" s="138"/>
-      <c r="W13" s="138"/>
-      <c r="X13" s="138"/>
-      <c r="Y13" s="138"/>
-      <c r="Z13" s="138"/>
-      <c r="AA13" s="138"/>
-      <c r="AB13" s="138"/>
-      <c r="AC13" s="138"/>
-      <c r="AD13" s="138"/>
-      <c r="AE13" s="138"/>
-      <c r="AF13" s="138"/>
-      <c r="AG13" s="138"/>
-      <c r="AH13" s="138"/>
-      <c r="AI13" s="138"/>
-      <c r="AJ13" s="138"/>
-      <c r="AK13" s="138"/>
-      <c r="AL13" s="138"/>
-      <c r="AM13" s="138"/>
-      <c r="AN13" s="138"/>
-      <c r="AO13" s="138"/>
-      <c r="AP13" s="138"/>
-      <c r="AQ13" s="138"/>
-      <c r="AR13" s="138" t="s">
-        <v>300</v>
-      </c>
-      <c r="AS13" s="138"/>
-      <c r="AT13" s="138"/>
-      <c r="AU13" s="138"/>
-      <c r="AV13" s="138"/>
-      <c r="AW13" s="138"/>
-      <c r="AX13" s="138"/>
-      <c r="AY13" s="138"/>
-      <c r="AZ13" s="138"/>
-      <c r="BA13" s="138"/>
-      <c r="BB13" s="138"/>
-      <c r="BC13" s="138"/>
-      <c r="BD13" s="138"/>
-      <c r="BE13" s="138"/>
-      <c r="BF13" s="138"/>
-      <c r="BG13" s="138"/>
-      <c r="BH13" s="138"/>
-      <c r="BI13" s="138"/>
-      <c r="BJ13" s="138"/>
-      <c r="BK13" s="138"/>
-      <c r="BL13" s="138"/>
-      <c r="BM13" s="138"/>
-      <c r="BN13" s="138"/>
-      <c r="BO13" s="138"/>
-      <c r="BP13" s="138"/>
-      <c r="BQ13" s="138"/>
-      <c r="BR13" s="138"/>
-      <c r="BS13" s="138"/>
-      <c r="BT13" s="138"/>
-      <c r="BU13" s="138"/>
-      <c r="BV13" s="138"/>
-      <c r="BW13" s="138"/>
-      <c r="BX13" s="138"/>
-      <c r="BY13" s="138"/>
-      <c r="BZ13" s="138"/>
-      <c r="CA13" s="138"/>
-      <c r="CB13" s="138"/>
-      <c r="CC13" s="138"/>
-      <c r="CD13" s="138"/>
-      <c r="CE13" s="138"/>
-      <c r="CF13" s="138"/>
-      <c r="CG13" s="138"/>
-      <c r="CH13" s="138"/>
-      <c r="CI13" s="138"/>
-      <c r="CJ13" s="138"/>
-      <c r="CK13" s="138"/>
-      <c r="CL13" s="143"/>
-    </row>
-    <row r="14" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="133"/>
-      <c r="B14" s="129"/>
-      <c r="C14" s="129"/>
-      <c r="D14" s="129"/>
-      <c r="E14" s="129"/>
-      <c r="F14" s="134"/>
-      <c r="G14" s="142"/>
-      <c r="H14" s="138"/>
-      <c r="I14" s="138"/>
-      <c r="J14" s="138"/>
-      <c r="K14" s="138"/>
-      <c r="L14" s="138"/>
-      <c r="M14" s="138"/>
-      <c r="N14" s="138"/>
-      <c r="O14" s="138"/>
-      <c r="P14" s="138"/>
-      <c r="Q14" s="138"/>
-      <c r="R14" s="138"/>
-      <c r="S14" s="138"/>
-      <c r="T14" s="138"/>
-      <c r="U14" s="138"/>
-      <c r="V14" s="138"/>
-      <c r="W14" s="138"/>
-      <c r="X14" s="138"/>
-      <c r="Y14" s="138"/>
-      <c r="Z14" s="138"/>
-      <c r="AA14" s="138"/>
-      <c r="AB14" s="138"/>
-      <c r="AC14" s="138"/>
-      <c r="AD14" s="138"/>
-      <c r="AE14" s="138"/>
-      <c r="AF14" s="138"/>
-      <c r="AG14" s="138"/>
-      <c r="AH14" s="138"/>
-      <c r="AI14" s="138"/>
-      <c r="AJ14" s="138"/>
-      <c r="AK14" s="138"/>
-      <c r="AL14" s="138" t="s">
-        <v>316</v>
-      </c>
-      <c r="AM14" s="138"/>
-      <c r="AN14" s="138"/>
-      <c r="AO14" s="138"/>
-      <c r="AP14" s="138"/>
-      <c r="AQ14" s="138"/>
-      <c r="AR14" s="138"/>
-      <c r="AS14" s="138"/>
-      <c r="AT14" s="138"/>
-      <c r="AU14" s="138"/>
-      <c r="AV14" s="138"/>
-      <c r="AW14" s="138"/>
-      <c r="AX14" s="138"/>
-      <c r="AY14" s="138"/>
-      <c r="AZ14" s="138"/>
-      <c r="BA14" s="138"/>
-      <c r="BB14" s="138"/>
-      <c r="BC14" s="138"/>
-      <c r="BD14" s="138"/>
-      <c r="BE14" s="138"/>
-      <c r="BF14" s="138"/>
-      <c r="BG14" s="138"/>
-      <c r="BH14" s="138"/>
-      <c r="BI14" s="138"/>
-      <c r="BJ14" s="138"/>
-      <c r="BK14" s="138"/>
-      <c r="BL14" s="138"/>
-      <c r="BM14" s="138"/>
-      <c r="BN14" s="138"/>
-      <c r="BO14" s="138"/>
-      <c r="BP14" s="138"/>
-      <c r="BQ14" s="138"/>
-      <c r="BR14" s="138"/>
-      <c r="BS14" s="138"/>
-      <c r="BT14" s="138"/>
-      <c r="BU14" s="138"/>
-      <c r="BV14" s="138"/>
-      <c r="BW14" s="138"/>
-      <c r="BX14" s="138"/>
-      <c r="BY14" s="138"/>
-      <c r="BZ14" s="138"/>
-      <c r="CA14" s="138"/>
-      <c r="CB14" s="138"/>
-      <c r="CC14" s="138"/>
-      <c r="CD14" s="138"/>
-      <c r="CE14" s="138"/>
-      <c r="CF14" s="138"/>
-      <c r="CG14" s="138"/>
-      <c r="CH14" s="138"/>
-      <c r="CI14" s="138"/>
-      <c r="CJ14" s="138"/>
-      <c r="CK14" s="138"/>
-      <c r="CL14" s="143"/>
-    </row>
-    <row r="15" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="133"/>
-      <c r="B15" s="129"/>
-      <c r="C15" s="129"/>
-      <c r="D15" s="129"/>
-      <c r="E15" s="129"/>
-      <c r="F15" s="134"/>
-      <c r="G15" s="142"/>
-      <c r="H15" s="138"/>
-      <c r="I15" s="138"/>
-      <c r="J15" s="138"/>
-      <c r="K15" s="138"/>
-      <c r="L15" s="138"/>
-      <c r="M15" s="138"/>
-      <c r="N15" s="138"/>
-      <c r="O15" s="138"/>
-      <c r="P15" s="138"/>
-      <c r="Q15" s="138"/>
-      <c r="R15" s="138"/>
-      <c r="S15" s="138"/>
-      <c r="T15" s="138"/>
-      <c r="U15" s="138"/>
-      <c r="V15" s="138"/>
-      <c r="W15" s="138"/>
-      <c r="X15" s="138"/>
-      <c r="Y15" s="138"/>
-      <c r="Z15" s="138"/>
-      <c r="AA15" s="138"/>
-      <c r="AB15" s="138"/>
-      <c r="AC15" s="138"/>
-      <c r="AD15" s="138"/>
-      <c r="AE15" s="138"/>
-      <c r="AF15" s="138"/>
-      <c r="AG15" s="138"/>
-      <c r="AH15" s="138"/>
-      <c r="AI15" s="138"/>
-      <c r="AJ15" s="138"/>
-      <c r="AK15" s="138"/>
-      <c r="AL15" s="138"/>
-      <c r="AM15" s="138"/>
-      <c r="AN15" s="138"/>
-      <c r="AO15" s="138"/>
-      <c r="AP15" s="138" t="s">
-        <v>128</v>
-      </c>
-      <c r="AQ15" s="138"/>
-      <c r="AR15" s="138" t="s">
-        <v>317</v>
-      </c>
-      <c r="AS15" s="138"/>
-      <c r="AT15" s="138"/>
-      <c r="AU15" s="138"/>
-      <c r="AV15" s="138"/>
-      <c r="AW15" s="138"/>
-      <c r="AX15" s="138"/>
-      <c r="AY15" s="138"/>
-      <c r="AZ15" s="138"/>
-      <c r="BA15" s="138"/>
-      <c r="BB15" s="138"/>
-      <c r="BC15" s="138"/>
-      <c r="BD15" s="138"/>
-      <c r="BE15" s="138"/>
-      <c r="BF15" s="138"/>
-      <c r="BG15" s="138"/>
-      <c r="BH15" s="138"/>
-      <c r="BI15" s="138"/>
-      <c r="BJ15" s="138"/>
-      <c r="BK15" s="138"/>
-      <c r="BL15" s="138"/>
-      <c r="BM15" s="138"/>
-      <c r="BN15" s="138"/>
-      <c r="BO15" s="138"/>
-      <c r="BP15" s="138"/>
-      <c r="BQ15" s="138"/>
-      <c r="BR15" s="138"/>
-      <c r="BS15" s="138"/>
-      <c r="BT15" s="138"/>
-      <c r="BU15" s="138"/>
-      <c r="BV15" s="138"/>
-      <c r="BW15" s="138"/>
-      <c r="BX15" s="138"/>
-      <c r="BY15" s="138"/>
-      <c r="BZ15" s="138"/>
-      <c r="CA15" s="138"/>
-      <c r="CB15" s="138"/>
-      <c r="CC15" s="138"/>
-      <c r="CD15" s="138"/>
-      <c r="CE15" s="138"/>
-      <c r="CF15" s="138"/>
-      <c r="CG15" s="138"/>
-      <c r="CH15" s="138"/>
-      <c r="CI15" s="138"/>
-      <c r="CJ15" s="138"/>
-      <c r="CK15" s="138"/>
-      <c r="CL15" s="143"/>
-    </row>
-    <row r="16" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="133"/>
-      <c r="B16" s="129"/>
-      <c r="C16" s="129"/>
-      <c r="D16" s="129"/>
-      <c r="E16" s="129"/>
-      <c r="F16" s="134"/>
-      <c r="G16" s="142"/>
-      <c r="H16" s="138"/>
-      <c r="I16" s="138"/>
-      <c r="J16" s="138"/>
-      <c r="K16" s="138"/>
-      <c r="L16" s="138"/>
-      <c r="M16" s="138"/>
-      <c r="N16" s="138"/>
-      <c r="O16" s="138"/>
-      <c r="P16" s="138"/>
-      <c r="Q16" s="138"/>
-      <c r="R16" s="138"/>
-      <c r="S16" s="138"/>
-      <c r="T16" s="138"/>
-      <c r="U16" s="138"/>
-      <c r="V16" s="138"/>
-      <c r="W16" s="138"/>
-      <c r="X16" s="138"/>
-      <c r="Y16" s="138"/>
-      <c r="Z16" s="138"/>
-      <c r="AA16" s="138"/>
-      <c r="AB16" s="138"/>
-      <c r="AC16" s="138"/>
-      <c r="AD16" s="138"/>
-      <c r="AE16" s="138"/>
-      <c r="AF16" s="138"/>
-      <c r="AG16" s="138"/>
-      <c r="AH16" s="138"/>
-      <c r="AI16" s="138"/>
-      <c r="AJ16" s="138"/>
-      <c r="AK16" s="138"/>
-      <c r="AL16" s="138"/>
-      <c r="AM16" s="138"/>
-      <c r="AN16" s="138" t="s">
-        <v>10</v>
-      </c>
-      <c r="AO16" s="138"/>
-      <c r="AP16" s="138"/>
-      <c r="AQ16" s="138"/>
-      <c r="AR16" s="138" t="s">
-        <v>318</v>
-      </c>
-      <c r="AS16" s="138"/>
-      <c r="AT16" s="138"/>
-      <c r="AU16" s="138"/>
-      <c r="AV16" s="138"/>
-      <c r="AW16" s="138"/>
-      <c r="AX16" s="138"/>
-      <c r="AY16" s="138"/>
-      <c r="AZ16" s="138"/>
-      <c r="BA16" s="138"/>
-      <c r="BB16" s="138"/>
-      <c r="BC16" s="138"/>
-      <c r="BD16" s="138"/>
-      <c r="BE16" s="138"/>
-      <c r="BF16" s="138"/>
-      <c r="BG16" s="138"/>
-      <c r="BH16" s="138"/>
-      <c r="BI16" s="138"/>
-      <c r="BJ16" s="138"/>
-      <c r="BK16" s="138"/>
-      <c r="BL16" s="138"/>
-      <c r="BM16" s="138"/>
-      <c r="BN16" s="138"/>
-      <c r="BO16" s="138"/>
-      <c r="BP16" s="138"/>
-      <c r="BQ16" s="138"/>
-      <c r="BR16" s="138"/>
-      <c r="BS16" s="138"/>
-      <c r="BT16" s="138"/>
-      <c r="BU16" s="138"/>
-      <c r="BV16" s="138"/>
-      <c r="BW16" s="138"/>
-      <c r="BX16" s="138"/>
-      <c r="BY16" s="138"/>
-      <c r="BZ16" s="138"/>
-      <c r="CA16" s="138"/>
-      <c r="CB16" s="138"/>
-      <c r="CC16" s="138"/>
-      <c r="CD16" s="138"/>
-      <c r="CE16" s="138"/>
-      <c r="CF16" s="138"/>
-      <c r="CG16" s="138"/>
-      <c r="CH16" s="138"/>
-      <c r="CI16" s="138"/>
-      <c r="CJ16" s="138"/>
-      <c r="CK16" s="138"/>
-      <c r="CL16" s="143"/>
-    </row>
-    <row r="17" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="133"/>
-      <c r="B17" s="129"/>
-      <c r="C17" s="129"/>
-      <c r="D17" s="129"/>
-      <c r="E17" s="129"/>
-      <c r="F17" s="134"/>
-      <c r="G17" s="142"/>
-      <c r="H17" s="138"/>
-      <c r="I17" s="138"/>
-      <c r="J17" s="138"/>
-      <c r="K17" s="138"/>
-      <c r="L17" s="138"/>
-      <c r="M17" s="138"/>
-      <c r="N17" s="138"/>
-      <c r="O17" s="138"/>
-      <c r="P17" s="138"/>
-      <c r="Q17" s="138"/>
-      <c r="R17" s="138"/>
-      <c r="S17" s="138"/>
-      <c r="T17" s="138"/>
-      <c r="U17" s="138"/>
-      <c r="V17" s="138"/>
-      <c r="W17" s="138"/>
-      <c r="X17" s="138"/>
-      <c r="Y17" s="138"/>
-      <c r="Z17" s="138"/>
-      <c r="AA17" s="138"/>
-      <c r="AB17" s="138"/>
-      <c r="AC17" s="138"/>
-      <c r="AD17" s="138"/>
-      <c r="AE17" s="138"/>
-      <c r="AF17" s="138"/>
-      <c r="AG17" s="138"/>
-      <c r="AH17" s="138"/>
-      <c r="AI17" s="138"/>
-      <c r="AJ17" s="138"/>
-      <c r="AK17" s="138"/>
-      <c r="AL17" s="138"/>
-      <c r="AM17" s="138"/>
-      <c r="AN17" s="138"/>
-      <c r="AO17" s="138"/>
-      <c r="AP17" s="138" t="s">
-        <v>128</v>
-      </c>
-      <c r="AQ17" s="138"/>
-      <c r="AR17" s="138" t="s">
-        <v>319</v>
-      </c>
-      <c r="AS17" s="138"/>
-      <c r="AT17" s="138"/>
-      <c r="AU17" s="138"/>
-      <c r="AV17" s="138"/>
-      <c r="AW17" s="138"/>
-      <c r="AX17" s="138"/>
-      <c r="AY17" s="138"/>
-      <c r="AZ17" s="138"/>
-      <c r="BA17" s="138"/>
-      <c r="BB17" s="138"/>
-      <c r="BC17" s="138"/>
-      <c r="BD17" s="138"/>
-      <c r="BE17" s="138"/>
-      <c r="BF17" s="138"/>
-      <c r="BG17" s="138"/>
-      <c r="BH17" s="138"/>
-      <c r="BI17" s="138"/>
-      <c r="BJ17" s="138"/>
-      <c r="BK17" s="138"/>
-      <c r="BL17" s="138"/>
-      <c r="BM17" s="138"/>
-      <c r="BN17" s="138"/>
-      <c r="BO17" s="138"/>
-      <c r="BP17" s="138"/>
-      <c r="BQ17" s="138"/>
-      <c r="BR17" s="138"/>
-      <c r="BS17" s="138"/>
-      <c r="BT17" s="138"/>
-      <c r="BU17" s="138"/>
-      <c r="BV17" s="138"/>
-      <c r="BW17" s="138"/>
-      <c r="BX17" s="138"/>
-      <c r="BY17" s="138"/>
-      <c r="BZ17" s="138"/>
-      <c r="CA17" s="138"/>
-      <c r="CB17" s="138"/>
-      <c r="CC17" s="138"/>
-      <c r="CD17" s="138"/>
-      <c r="CE17" s="138"/>
-      <c r="CF17" s="138"/>
-      <c r="CG17" s="138"/>
-      <c r="CH17" s="138"/>
-      <c r="CI17" s="138"/>
-      <c r="CJ17" s="138"/>
-      <c r="CK17" s="138"/>
-      <c r="CL17" s="143"/>
-    </row>
-    <row r="18" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="133"/>
-      <c r="B18" s="129"/>
-      <c r="C18" s="129"/>
-      <c r="D18" s="129"/>
-      <c r="E18" s="129"/>
-      <c r="F18" s="134"/>
-      <c r="G18" s="142"/>
-      <c r="H18" s="138"/>
-      <c r="I18" s="138"/>
-      <c r="J18" s="138"/>
-      <c r="K18" s="138"/>
-      <c r="L18" s="138"/>
-      <c r="M18" s="138"/>
-      <c r="N18" s="138"/>
-      <c r="O18" s="138"/>
-      <c r="P18" s="138"/>
-      <c r="Q18" s="138"/>
-      <c r="R18" s="138"/>
-      <c r="S18" s="138"/>
-      <c r="T18" s="138"/>
-      <c r="U18" s="138"/>
-      <c r="V18" s="138"/>
-      <c r="W18" s="138"/>
-      <c r="X18" s="138"/>
-      <c r="Y18" s="138"/>
-      <c r="Z18" s="138"/>
-      <c r="AA18" s="138"/>
-      <c r="AB18" s="138"/>
-      <c r="AC18" s="138"/>
-      <c r="AD18" s="138"/>
-      <c r="AE18" s="138"/>
-      <c r="AF18" s="138"/>
-      <c r="AG18" s="138"/>
-      <c r="AH18" s="138"/>
-      <c r="AI18" s="138"/>
-      <c r="AJ18" s="138"/>
-      <c r="AK18" s="138"/>
-      <c r="AL18" s="138"/>
-      <c r="AM18" s="138"/>
-      <c r="AN18" s="138" t="s">
-        <v>302</v>
-      </c>
-      <c r="AO18" s="138"/>
-      <c r="AP18" s="138"/>
-      <c r="AQ18" s="138"/>
-      <c r="AR18" s="138"/>
-      <c r="AS18" s="138"/>
-      <c r="AT18" s="138"/>
-      <c r="AU18" s="138"/>
-      <c r="AV18" s="138"/>
-      <c r="AW18" s="138"/>
-      <c r="AX18" s="138"/>
-      <c r="AY18" s="138"/>
-      <c r="AZ18" s="138"/>
-      <c r="BA18" s="138"/>
-      <c r="BB18" s="138"/>
-      <c r="BC18" s="138"/>
-      <c r="BD18" s="138"/>
-      <c r="BE18" s="138"/>
-      <c r="BF18" s="138"/>
-      <c r="BG18" s="138"/>
-      <c r="BH18" s="138"/>
-      <c r="BI18" s="138"/>
-      <c r="BJ18" s="138"/>
-      <c r="BK18" s="138"/>
-      <c r="BL18" s="138"/>
-      <c r="BM18" s="138"/>
-      <c r="BN18" s="138"/>
-      <c r="BO18" s="138"/>
-      <c r="BP18" s="138"/>
-      <c r="BQ18" s="138"/>
-      <c r="BR18" s="138"/>
-      <c r="BS18" s="138"/>
-      <c r="BT18" s="138"/>
-      <c r="BU18" s="138"/>
-      <c r="BV18" s="138"/>
-      <c r="BW18" s="138"/>
-      <c r="BX18" s="138"/>
-      <c r="BY18" s="138"/>
-      <c r="BZ18" s="138"/>
-      <c r="CA18" s="138"/>
-      <c r="CB18" s="138"/>
-      <c r="CC18" s="138"/>
-      <c r="CD18" s="138"/>
-      <c r="CE18" s="138"/>
-      <c r="CF18" s="138"/>
-      <c r="CG18" s="138"/>
-      <c r="CH18" s="138"/>
-      <c r="CI18" s="138"/>
-      <c r="CJ18" s="138"/>
-      <c r="CK18" s="138"/>
-      <c r="CL18" s="143"/>
-    </row>
-    <row r="19" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="133"/>
-      <c r="B19" s="129"/>
-      <c r="C19" s="129"/>
-      <c r="D19" s="129"/>
-      <c r="E19" s="129"/>
-      <c r="F19" s="134"/>
-      <c r="G19" s="142"/>
-      <c r="H19" s="138"/>
-      <c r="I19" s="138"/>
-      <c r="J19" s="138"/>
-      <c r="K19" s="138"/>
-      <c r="L19" s="138"/>
-      <c r="M19" s="138"/>
-      <c r="N19" s="138"/>
-      <c r="O19" s="138"/>
-      <c r="P19" s="138"/>
-      <c r="Q19" s="138"/>
-      <c r="R19" s="138"/>
-      <c r="S19" s="138"/>
-      <c r="T19" s="138"/>
-      <c r="U19" s="138"/>
-      <c r="V19" s="138"/>
-      <c r="W19" s="138"/>
-      <c r="X19" s="138"/>
-      <c r="Y19" s="138"/>
-      <c r="Z19" s="138"/>
-      <c r="AA19" s="138"/>
-      <c r="AB19" s="138"/>
-      <c r="AC19" s="138"/>
-      <c r="AD19" s="138"/>
-      <c r="AE19" s="138"/>
-      <c r="AF19" s="138" t="s">
-        <v>320</v>
-      </c>
-      <c r="AG19" s="138"/>
-      <c r="AH19" s="138"/>
-      <c r="AI19" s="138"/>
-      <c r="AJ19" s="138"/>
-      <c r="AK19" s="138"/>
-      <c r="AL19" s="138"/>
-      <c r="AM19" s="138"/>
-      <c r="AN19" s="138"/>
-      <c r="AO19" s="138"/>
-      <c r="AP19" s="138"/>
-      <c r="AQ19" s="138"/>
-      <c r="AR19" s="138"/>
-      <c r="AS19" s="138"/>
-      <c r="AT19" s="138"/>
-      <c r="AU19" s="138"/>
-      <c r="AV19" s="138"/>
-      <c r="AW19" s="138"/>
-      <c r="AX19" s="138"/>
-      <c r="AY19" s="138"/>
-      <c r="AZ19" s="138"/>
-      <c r="BA19" s="138"/>
-      <c r="BB19" s="138"/>
-      <c r="BC19" s="138"/>
-      <c r="BD19" s="138"/>
-      <c r="BE19" s="138"/>
-      <c r="BF19" s="138"/>
-      <c r="BG19" s="138"/>
-      <c r="BH19" s="138"/>
-      <c r="BI19" s="138"/>
-      <c r="BJ19" s="138"/>
-      <c r="BK19" s="138"/>
-      <c r="BL19" s="138"/>
-      <c r="BM19" s="138"/>
-      <c r="BN19" s="138"/>
-      <c r="BO19" s="138"/>
-      <c r="BP19" s="138"/>
-      <c r="BQ19" s="138"/>
-      <c r="BR19" s="138"/>
-      <c r="BS19" s="138"/>
-      <c r="BT19" s="138"/>
-      <c r="BU19" s="138"/>
-      <c r="BV19" s="138"/>
-      <c r="BW19" s="138"/>
-      <c r="BX19" s="138"/>
-      <c r="BY19" s="138"/>
-      <c r="BZ19" s="138"/>
-      <c r="CA19" s="138"/>
-      <c r="CB19" s="138"/>
-      <c r="CC19" s="138"/>
-      <c r="CD19" s="138"/>
-      <c r="CE19" s="138"/>
-      <c r="CF19" s="138"/>
-      <c r="CG19" s="138"/>
-      <c r="CH19" s="138"/>
-      <c r="CI19" s="138"/>
-      <c r="CJ19" s="138"/>
-      <c r="CK19" s="138"/>
-      <c r="CL19" s="143"/>
-    </row>
-    <row r="20" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="133"/>
-      <c r="B20" s="129"/>
-      <c r="C20" s="129"/>
-      <c r="D20" s="129"/>
-      <c r="E20" s="129"/>
-      <c r="F20" s="134"/>
-      <c r="G20" s="142"/>
-      <c r="H20" s="138"/>
-      <c r="I20" s="138"/>
-      <c r="J20" s="138"/>
-      <c r="K20" s="138"/>
-      <c r="L20" s="138"/>
-      <c r="M20" s="138"/>
-      <c r="N20" s="138"/>
-      <c r="O20" s="138"/>
-      <c r="P20" s="138"/>
-      <c r="Q20" s="138"/>
-      <c r="R20" s="138"/>
-      <c r="S20" s="138"/>
-      <c r="T20" s="138"/>
-      <c r="U20" s="138"/>
-      <c r="V20" s="138"/>
-      <c r="W20" s="138"/>
-      <c r="X20" s="138"/>
-      <c r="Y20" s="138"/>
-      <c r="Z20" s="138"/>
-      <c r="AA20" s="138"/>
-      <c r="AB20" s="138"/>
-      <c r="AC20" s="138"/>
-      <c r="AD20" s="138"/>
-      <c r="AE20" s="138"/>
-      <c r="AF20" s="138"/>
-      <c r="AG20" s="138"/>
-      <c r="AH20" s="138"/>
-      <c r="AI20" s="138"/>
-      <c r="AJ20" s="138" t="s">
-        <v>128</v>
-      </c>
-      <c r="AK20" s="138"/>
-      <c r="AL20" s="138" t="s">
-        <v>321</v>
-      </c>
-      <c r="AM20" s="138"/>
-      <c r="AN20" s="138"/>
-      <c r="AO20" s="138"/>
-      <c r="AP20" s="138"/>
-      <c r="AQ20" s="138"/>
-      <c r="AR20" s="138"/>
-      <c r="AS20" s="138"/>
-      <c r="AT20" s="138"/>
-      <c r="AU20" s="138"/>
-      <c r="AV20" s="138"/>
-      <c r="AW20" s="138"/>
-      <c r="AX20" s="138"/>
-      <c r="AY20" s="138"/>
-      <c r="AZ20" s="138"/>
-      <c r="BA20" s="138"/>
-      <c r="BB20" s="138"/>
-      <c r="BC20" s="138"/>
-      <c r="BD20" s="138"/>
-      <c r="BE20" s="138"/>
-      <c r="BF20" s="138"/>
-      <c r="BG20" s="138"/>
-      <c r="BH20" s="138"/>
-      <c r="BI20" s="138"/>
-      <c r="BJ20" s="138"/>
-      <c r="BK20" s="138"/>
-      <c r="BL20" s="138"/>
-      <c r="BM20" s="138"/>
-      <c r="BN20" s="138"/>
-      <c r="BO20" s="138"/>
-      <c r="BP20" s="138"/>
-      <c r="BQ20" s="138"/>
-      <c r="BR20" s="138"/>
-      <c r="BS20" s="138"/>
-      <c r="BT20" s="138"/>
-      <c r="BU20" s="138"/>
-      <c r="BV20" s="138"/>
-      <c r="BW20" s="138"/>
-      <c r="BX20" s="138"/>
-      <c r="BY20" s="138"/>
-      <c r="BZ20" s="138"/>
-      <c r="CA20" s="138"/>
-      <c r="CB20" s="138"/>
-      <c r="CC20" s="138"/>
-      <c r="CD20" s="138"/>
-      <c r="CE20" s="138"/>
-      <c r="CF20" s="138"/>
-      <c r="CG20" s="138"/>
-      <c r="CH20" s="138"/>
-      <c r="CI20" s="138"/>
-      <c r="CJ20" s="138"/>
-      <c r="CK20" s="138"/>
-      <c r="CL20" s="143"/>
-    </row>
-    <row r="21" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="133"/>
-      <c r="B21" s="129"/>
-      <c r="C21" s="129"/>
-      <c r="D21" s="129"/>
-      <c r="E21" s="129"/>
-      <c r="F21" s="134"/>
-      <c r="G21" s="142"/>
-      <c r="H21" s="138"/>
-      <c r="I21" s="138"/>
-      <c r="J21" s="138"/>
-      <c r="K21" s="138"/>
-      <c r="L21" s="138"/>
-      <c r="M21" s="138"/>
-      <c r="N21" s="138"/>
-      <c r="O21" s="138"/>
-      <c r="P21" s="138"/>
-      <c r="Q21" s="138"/>
-      <c r="R21" s="138"/>
-      <c r="S21" s="138"/>
-      <c r="T21" s="138"/>
-      <c r="U21" s="138"/>
-      <c r="V21" s="138"/>
-      <c r="W21" s="138"/>
-      <c r="X21" s="138"/>
-      <c r="Y21" s="138"/>
-      <c r="Z21" s="138"/>
-      <c r="AA21" s="138"/>
-      <c r="AB21" s="138"/>
-      <c r="AC21" s="138"/>
-      <c r="AD21" s="138"/>
-      <c r="AE21" s="138"/>
-      <c r="AF21" s="138"/>
-      <c r="AG21" s="138"/>
-      <c r="AH21" s="138" t="s">
-        <v>10</v>
-      </c>
-      <c r="AI21" s="138"/>
-      <c r="AJ21" s="138"/>
-      <c r="AK21" s="138"/>
-      <c r="AL21" s="138" t="s">
-        <v>308</v>
-      </c>
-      <c r="AM21" s="138"/>
-      <c r="AN21" s="138"/>
-      <c r="AO21" s="138"/>
-      <c r="AP21" s="138"/>
-      <c r="AQ21" s="138"/>
-      <c r="AR21" s="138"/>
-      <c r="AS21" s="138"/>
-      <c r="AT21" s="138"/>
-      <c r="AU21" s="138"/>
-      <c r="AV21" s="138"/>
-      <c r="AW21" s="138"/>
-      <c r="AX21" s="138"/>
-      <c r="AY21" s="138"/>
-      <c r="AZ21" s="138"/>
-      <c r="BA21" s="138"/>
-      <c r="BB21" s="138"/>
-      <c r="BC21" s="138"/>
-      <c r="BD21" s="138"/>
-      <c r="BE21" s="138"/>
-      <c r="BF21" s="138"/>
-      <c r="BG21" s="138"/>
-      <c r="BH21" s="138"/>
-      <c r="BI21" s="138"/>
-      <c r="BJ21" s="138"/>
-      <c r="BK21" s="138"/>
-      <c r="BL21" s="138"/>
-      <c r="BM21" s="138"/>
-      <c r="BN21" s="138"/>
-      <c r="BO21" s="138"/>
-      <c r="BP21" s="138"/>
-      <c r="BQ21" s="138"/>
-      <c r="BR21" s="138"/>
-      <c r="BS21" s="138"/>
-      <c r="BT21" s="138"/>
-      <c r="BU21" s="138"/>
-      <c r="BV21" s="138"/>
-      <c r="BW21" s="138"/>
-      <c r="BX21" s="138"/>
-      <c r="BY21" s="138"/>
-      <c r="BZ21" s="138"/>
-      <c r="CA21" s="138"/>
-      <c r="CB21" s="138"/>
-      <c r="CC21" s="138"/>
-      <c r="CD21" s="138"/>
-      <c r="CE21" s="138"/>
-      <c r="CF21" s="138"/>
-      <c r="CG21" s="138"/>
-      <c r="CH21" s="138"/>
-      <c r="CI21" s="138"/>
-      <c r="CJ21" s="138"/>
-      <c r="CK21" s="138"/>
-      <c r="CL21" s="143"/>
-    </row>
-    <row r="22" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="133"/>
-      <c r="B22" s="129"/>
-      <c r="C22" s="129"/>
-      <c r="D22" s="129"/>
-      <c r="E22" s="129"/>
-      <c r="F22" s="134"/>
-      <c r="G22" s="142"/>
-      <c r="H22" s="138"/>
-      <c r="I22" s="138"/>
-      <c r="J22" s="138"/>
-      <c r="K22" s="138"/>
-      <c r="L22" s="138"/>
-      <c r="M22" s="138"/>
-      <c r="N22" s="138"/>
-      <c r="O22" s="138"/>
-      <c r="P22" s="138"/>
-      <c r="Q22" s="138"/>
-      <c r="R22" s="138"/>
-      <c r="S22" s="138"/>
-      <c r="T22" s="138"/>
-      <c r="U22" s="138"/>
-      <c r="V22" s="138"/>
-      <c r="W22" s="138"/>
-      <c r="X22" s="138"/>
-      <c r="Y22" s="138"/>
-      <c r="Z22" s="138"/>
-      <c r="AA22" s="138"/>
-      <c r="AB22" s="138"/>
-      <c r="AC22" s="138"/>
-      <c r="AD22" s="138"/>
-      <c r="AE22" s="138"/>
-      <c r="AF22" s="138"/>
-      <c r="AG22" s="138"/>
-      <c r="AH22" s="138"/>
-      <c r="AI22" s="138"/>
-      <c r="AJ22" s="138" t="s">
-        <v>128</v>
-      </c>
-      <c r="AK22" s="138"/>
-      <c r="AL22" s="138" t="s">
-        <v>322</v>
-      </c>
-      <c r="AM22" s="138"/>
-      <c r="AN22" s="138"/>
-      <c r="AO22" s="138"/>
-      <c r="AP22" s="138"/>
-      <c r="AQ22" s="138"/>
-      <c r="AR22" s="138"/>
-      <c r="AS22" s="138"/>
-      <c r="AT22" s="138"/>
-      <c r="AU22" s="138"/>
-      <c r="AV22" s="138"/>
-      <c r="AW22" s="138"/>
-      <c r="AX22" s="138"/>
-      <c r="AY22" s="138"/>
-      <c r="AZ22" s="138"/>
-      <c r="BA22" s="138"/>
-      <c r="BB22" s="138"/>
-      <c r="BC22" s="138"/>
-      <c r="BD22" s="138"/>
-      <c r="BE22" s="138"/>
-      <c r="BF22" s="138"/>
-      <c r="BG22" s="138"/>
-      <c r="BH22" s="138"/>
-      <c r="BI22" s="138"/>
-      <c r="BJ22" s="138"/>
-      <c r="BK22" s="138"/>
-      <c r="BL22" s="138"/>
-      <c r="BM22" s="138"/>
-      <c r="BN22" s="138"/>
-      <c r="BO22" s="138"/>
-      <c r="BP22" s="138"/>
-      <c r="BQ22" s="138"/>
-      <c r="BR22" s="138"/>
-      <c r="BS22" s="138"/>
-      <c r="BT22" s="138"/>
-      <c r="BU22" s="138"/>
-      <c r="BV22" s="138"/>
-      <c r="BW22" s="138"/>
-      <c r="BX22" s="138"/>
-      <c r="BY22" s="138"/>
-      <c r="BZ22" s="138"/>
-      <c r="CA22" s="138"/>
-      <c r="CB22" s="138"/>
-      <c r="CC22" s="138"/>
-      <c r="CD22" s="138"/>
-      <c r="CE22" s="138"/>
-      <c r="CF22" s="138"/>
-      <c r="CG22" s="138"/>
-      <c r="CH22" s="138"/>
-      <c r="CI22" s="138"/>
-      <c r="CJ22" s="138"/>
-      <c r="CK22" s="138"/>
-      <c r="CL22" s="143"/>
-    </row>
-    <row r="23" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="133"/>
-      <c r="B23" s="129"/>
-      <c r="C23" s="129"/>
-      <c r="D23" s="129"/>
-      <c r="E23" s="129"/>
-      <c r="F23" s="134"/>
-      <c r="G23" s="142"/>
-      <c r="H23" s="138"/>
-      <c r="I23" s="138"/>
-      <c r="J23" s="138"/>
-      <c r="K23" s="138"/>
-      <c r="L23" s="138"/>
-      <c r="M23" s="138"/>
-      <c r="N23" s="138"/>
-      <c r="O23" s="138"/>
-      <c r="P23" s="138"/>
-      <c r="Q23" s="138"/>
-      <c r="R23" s="138"/>
-      <c r="S23" s="138"/>
-      <c r="T23" s="138"/>
-      <c r="U23" s="138"/>
-      <c r="V23" s="138"/>
-      <c r="W23" s="138"/>
-      <c r="X23" s="138"/>
-      <c r="Y23" s="138"/>
-      <c r="Z23" s="138"/>
-      <c r="AA23" s="138"/>
-      <c r="AB23" s="138"/>
-      <c r="AC23" s="138"/>
-      <c r="AD23" s="138"/>
-      <c r="AE23" s="138"/>
-      <c r="AF23" s="138"/>
-      <c r="AG23" s="138"/>
-      <c r="AH23" s="138"/>
-      <c r="AI23" s="138"/>
-      <c r="AJ23" s="138"/>
-      <c r="AK23" s="138"/>
-      <c r="AL23" s="138"/>
-      <c r="AM23" s="138"/>
-      <c r="AN23" s="138"/>
-      <c r="AO23" s="138"/>
-      <c r="AP23" s="138" t="s">
-        <v>128</v>
-      </c>
-      <c r="AQ23" s="138"/>
-      <c r="AR23" s="138" t="s">
-        <v>323</v>
-      </c>
-      <c r="AS23" s="138"/>
-      <c r="AT23" s="138"/>
-      <c r="AU23" s="138"/>
-      <c r="AV23" s="138"/>
-      <c r="AW23" s="138"/>
-      <c r="AX23" s="138"/>
-      <c r="AY23" s="138"/>
-      <c r="AZ23" s="138"/>
-      <c r="BA23" s="138"/>
-      <c r="BB23" s="138"/>
-      <c r="BC23" s="138"/>
-      <c r="BD23" s="138"/>
-      <c r="BE23" s="138"/>
-      <c r="BF23" s="138"/>
-      <c r="BG23" s="138"/>
-      <c r="BH23" s="138"/>
-      <c r="BI23" s="138"/>
-      <c r="BJ23" s="138"/>
-      <c r="BK23" s="138"/>
-      <c r="BL23" s="138"/>
-      <c r="BM23" s="138"/>
-      <c r="BN23" s="138"/>
-      <c r="BO23" s="138"/>
-      <c r="BP23" s="138"/>
-      <c r="BQ23" s="138"/>
-      <c r="BR23" s="138"/>
-      <c r="BS23" s="138"/>
-      <c r="BT23" s="138"/>
-      <c r="BU23" s="138"/>
-      <c r="BV23" s="138"/>
-      <c r="BW23" s="138"/>
-      <c r="BX23" s="138"/>
-      <c r="BY23" s="138"/>
-      <c r="BZ23" s="138"/>
-      <c r="CA23" s="138"/>
-      <c r="CB23" s="138"/>
-      <c r="CC23" s="138"/>
-      <c r="CD23" s="138"/>
-      <c r="CE23" s="138"/>
-      <c r="CF23" s="138"/>
-      <c r="CG23" s="138"/>
-      <c r="CH23" s="138"/>
-      <c r="CI23" s="138"/>
-      <c r="CJ23" s="138"/>
-      <c r="CK23" s="138"/>
-      <c r="CL23" s="143"/>
-    </row>
-    <row r="24" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="133"/>
-      <c r="B24" s="129"/>
-      <c r="C24" s="129"/>
-      <c r="D24" s="129"/>
-      <c r="E24" s="129"/>
-      <c r="F24" s="134"/>
-      <c r="G24" s="142"/>
-      <c r="H24" s="138"/>
-      <c r="I24" s="138"/>
-      <c r="J24" s="138"/>
-      <c r="K24" s="138"/>
-      <c r="L24" s="138"/>
-      <c r="M24" s="138"/>
-      <c r="N24" s="138"/>
-      <c r="O24" s="138"/>
-      <c r="P24" s="138"/>
-      <c r="Q24" s="138"/>
-      <c r="R24" s="138"/>
-      <c r="S24" s="138"/>
-      <c r="T24" s="138"/>
-      <c r="U24" s="138"/>
-      <c r="V24" s="138"/>
-      <c r="W24" s="138"/>
-      <c r="X24" s="138"/>
-      <c r="Y24" s="138"/>
-      <c r="Z24" s="138"/>
-      <c r="AA24" s="138"/>
-      <c r="AB24" s="138"/>
-      <c r="AC24" s="138"/>
-      <c r="AD24" s="138"/>
-      <c r="AE24" s="138"/>
-      <c r="AF24" s="138"/>
-      <c r="AG24" s="138"/>
-      <c r="AH24" s="138"/>
-      <c r="AI24" s="138"/>
-      <c r="AJ24" s="138"/>
-      <c r="AK24" s="138"/>
-      <c r="AL24" s="138"/>
-      <c r="AM24" s="138"/>
-      <c r="AN24" s="138" t="s">
-        <v>10</v>
-      </c>
-      <c r="AO24" s="138"/>
-      <c r="AP24" s="138"/>
-      <c r="AQ24" s="138"/>
-      <c r="AR24" s="138" t="s">
-        <v>324</v>
-      </c>
-      <c r="AS24" s="138"/>
-      <c r="AT24" s="138"/>
-      <c r="AU24" s="138"/>
-      <c r="AV24" s="138"/>
-      <c r="AW24" s="138"/>
-      <c r="AX24" s="138"/>
-      <c r="AY24" s="138"/>
-      <c r="AZ24" s="138"/>
-      <c r="BA24" s="138"/>
-      <c r="BB24" s="138"/>
-      <c r="BC24" s="138"/>
-      <c r="BD24" s="138"/>
-      <c r="BE24" s="138"/>
-      <c r="BF24" s="138"/>
-      <c r="BG24" s="138"/>
-      <c r="BH24" s="138"/>
-      <c r="BI24" s="138"/>
-      <c r="BJ24" s="138"/>
-      <c r="BK24" s="138"/>
-      <c r="BL24" s="138"/>
-      <c r="BM24" s="138"/>
-      <c r="BN24" s="138"/>
-      <c r="BO24" s="138"/>
-      <c r="BP24" s="138"/>
-      <c r="BQ24" s="138"/>
-      <c r="BR24" s="138"/>
-      <c r="BS24" s="138"/>
-      <c r="BT24" s="138"/>
-      <c r="BU24" s="138"/>
-      <c r="BV24" s="138"/>
-      <c r="BW24" s="138"/>
-      <c r="BX24" s="138"/>
-      <c r="BY24" s="138"/>
-      <c r="BZ24" s="138"/>
-      <c r="CA24" s="138"/>
-      <c r="CB24" s="138"/>
-      <c r="CC24" s="138"/>
-      <c r="CD24" s="138"/>
-      <c r="CE24" s="138"/>
-      <c r="CF24" s="138"/>
-      <c r="CG24" s="138"/>
-      <c r="CH24" s="138"/>
-      <c r="CI24" s="138"/>
-      <c r="CJ24" s="138"/>
-      <c r="CK24" s="138"/>
-      <c r="CL24" s="143"/>
-    </row>
-    <row r="25" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="133"/>
-      <c r="B25" s="129"/>
-      <c r="C25" s="129"/>
-      <c r="D25" s="129"/>
-      <c r="E25" s="129"/>
-      <c r="F25" s="134"/>
-      <c r="G25" s="142"/>
-      <c r="H25" s="138"/>
-      <c r="I25" s="138"/>
-      <c r="J25" s="138"/>
-      <c r="K25" s="138"/>
-      <c r="L25" s="138"/>
-      <c r="M25" s="138"/>
-      <c r="N25" s="138"/>
-      <c r="O25" s="138"/>
-      <c r="P25" s="138"/>
-      <c r="Q25" s="138"/>
-      <c r="R25" s="138"/>
-      <c r="S25" s="138"/>
-      <c r="T25" s="138"/>
-      <c r="U25" s="138"/>
-      <c r="V25" s="138"/>
-      <c r="W25" s="138"/>
-      <c r="X25" s="138"/>
-      <c r="Y25" s="138"/>
-      <c r="Z25" s="138"/>
-      <c r="AA25" s="138"/>
-      <c r="AB25" s="138"/>
-      <c r="AC25" s="138"/>
-      <c r="AD25" s="138"/>
-      <c r="AE25" s="138"/>
-      <c r="AF25" s="138"/>
-      <c r="AG25" s="138"/>
-      <c r="AH25" s="138"/>
-      <c r="AI25" s="138"/>
-      <c r="AJ25" s="138"/>
-      <c r="AK25" s="138"/>
-      <c r="AL25" s="138"/>
-      <c r="AM25" s="138"/>
-      <c r="AN25" s="138"/>
-      <c r="AO25" s="138"/>
-      <c r="AP25" s="138" t="s">
-        <v>128</v>
-      </c>
-      <c r="AQ25" s="138"/>
-      <c r="AR25" s="138" t="s">
-        <v>325</v>
-      </c>
-      <c r="AS25" s="138"/>
-      <c r="AT25" s="138"/>
-      <c r="AU25" s="138"/>
-      <c r="AV25" s="138"/>
-      <c r="AW25" s="138"/>
-      <c r="AX25" s="138"/>
-      <c r="AY25" s="138"/>
-      <c r="AZ25" s="138"/>
-      <c r="BA25" s="138"/>
-      <c r="BB25" s="138"/>
-      <c r="BC25" s="138"/>
-      <c r="BD25" s="138"/>
-      <c r="BE25" s="138"/>
-      <c r="BF25" s="138"/>
-      <c r="BG25" s="138"/>
-      <c r="BH25" s="138"/>
-      <c r="BI25" s="138"/>
-      <c r="BJ25" s="138"/>
-      <c r="BK25" s="138"/>
-      <c r="BL25" s="138"/>
-      <c r="BM25" s="138"/>
-      <c r="BN25" s="138"/>
-      <c r="BO25" s="138"/>
-      <c r="BP25" s="138"/>
-      <c r="BQ25" s="138"/>
-      <c r="BR25" s="138"/>
-      <c r="BS25" s="138"/>
-      <c r="BT25" s="138"/>
-      <c r="BU25" s="138"/>
-      <c r="BV25" s="138"/>
-      <c r="BW25" s="138"/>
-      <c r="BX25" s="138"/>
-      <c r="BY25" s="138"/>
-      <c r="BZ25" s="138"/>
-      <c r="CA25" s="138"/>
-      <c r="CB25" s="138"/>
-      <c r="CC25" s="138"/>
-      <c r="CD25" s="138"/>
-      <c r="CE25" s="138"/>
-      <c r="CF25" s="138"/>
-      <c r="CG25" s="138"/>
-      <c r="CH25" s="138"/>
-      <c r="CI25" s="138"/>
-      <c r="CJ25" s="138"/>
-      <c r="CK25" s="138"/>
-      <c r="CL25" s="143"/>
-    </row>
-    <row r="26" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="133"/>
-      <c r="B26" s="129"/>
-      <c r="C26" s="129"/>
-      <c r="D26" s="129"/>
-      <c r="E26" s="129"/>
-      <c r="F26" s="134"/>
-      <c r="G26" s="142"/>
-      <c r="H26" s="138"/>
-      <c r="I26" s="138"/>
-      <c r="J26" s="138"/>
-      <c r="K26" s="138"/>
-      <c r="L26" s="138"/>
-      <c r="M26" s="138"/>
-      <c r="N26" s="138"/>
-      <c r="O26" s="138"/>
-      <c r="P26" s="138"/>
-      <c r="Q26" s="138"/>
-      <c r="R26" s="138"/>
-      <c r="S26" s="138"/>
-      <c r="T26" s="138"/>
-      <c r="U26" s="138"/>
-      <c r="V26" s="138"/>
-      <c r="W26" s="138"/>
-      <c r="X26" s="138"/>
-      <c r="Y26" s="138"/>
-      <c r="Z26" s="138"/>
-      <c r="AA26" s="138"/>
-      <c r="AB26" s="138"/>
-      <c r="AC26" s="138"/>
-      <c r="AD26" s="138"/>
-      <c r="AE26" s="138"/>
-      <c r="AF26" s="138"/>
-      <c r="AG26" s="138"/>
-      <c r="AH26" s="138"/>
-      <c r="AI26" s="138"/>
-      <c r="AJ26" s="138"/>
-      <c r="AK26" s="138"/>
-      <c r="AL26" s="138"/>
-      <c r="AM26" s="138"/>
-      <c r="AN26" s="138" t="s">
-        <v>273</v>
-      </c>
-      <c r="AO26" s="138"/>
-      <c r="AP26" s="138"/>
-      <c r="AQ26" s="138"/>
-      <c r="AR26" s="138"/>
-      <c r="AS26" s="138"/>
-      <c r="AT26" s="138"/>
-      <c r="AU26" s="138"/>
-      <c r="AV26" s="138"/>
-      <c r="AW26" s="138"/>
-      <c r="AX26" s="138"/>
-      <c r="AY26" s="138"/>
-      <c r="AZ26" s="138"/>
-      <c r="BA26" s="138"/>
-      <c r="BB26" s="138"/>
-      <c r="BC26" s="138"/>
-      <c r="BD26" s="138"/>
-      <c r="BE26" s="138"/>
-      <c r="BF26" s="138"/>
-      <c r="BG26" s="138"/>
-      <c r="BH26" s="138"/>
-      <c r="BI26" s="138"/>
-      <c r="BJ26" s="138"/>
-      <c r="BK26" s="138"/>
-      <c r="BL26" s="138"/>
-      <c r="BM26" s="138"/>
-      <c r="BN26" s="138"/>
-      <c r="BO26" s="138"/>
-      <c r="BP26" s="138"/>
-      <c r="BQ26" s="138"/>
-      <c r="BR26" s="138"/>
-      <c r="BS26" s="138"/>
-      <c r="BT26" s="138"/>
-      <c r="BU26" s="138"/>
-      <c r="BV26" s="138"/>
-      <c r="BW26" s="138"/>
-      <c r="BX26" s="138"/>
-      <c r="BY26" s="138"/>
-      <c r="BZ26" s="138"/>
-      <c r="CA26" s="138"/>
-      <c r="CB26" s="138"/>
-      <c r="CC26" s="138"/>
-      <c r="CD26" s="138"/>
-      <c r="CE26" s="138"/>
-      <c r="CF26" s="138"/>
-      <c r="CG26" s="138"/>
-      <c r="CH26" s="138"/>
-      <c r="CI26" s="138"/>
-      <c r="CJ26" s="138"/>
-      <c r="CK26" s="138"/>
-      <c r="CL26" s="143"/>
-    </row>
-    <row r="27" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="133"/>
-      <c r="B27" s="129"/>
-      <c r="C27" s="129"/>
-      <c r="D27" s="129"/>
-      <c r="E27" s="129"/>
-      <c r="F27" s="134"/>
-      <c r="G27" s="142"/>
-      <c r="H27" s="138"/>
-      <c r="I27" s="138"/>
-      <c r="J27" s="138"/>
-      <c r="K27" s="138"/>
-      <c r="L27" s="138"/>
-      <c r="M27" s="138"/>
-      <c r="N27" s="138"/>
-      <c r="O27" s="138"/>
-      <c r="P27" s="138"/>
-      <c r="Q27" s="138"/>
-      <c r="R27" s="138"/>
-      <c r="S27" s="138"/>
-      <c r="T27" s="138"/>
-      <c r="U27" s="138"/>
-      <c r="V27" s="138"/>
-      <c r="W27" s="138"/>
-      <c r="X27" s="138"/>
-      <c r="Y27" s="138"/>
-      <c r="Z27" s="138"/>
-      <c r="AA27" s="138"/>
-      <c r="AB27" s="138"/>
-      <c r="AC27" s="138"/>
-      <c r="AD27" s="138"/>
-      <c r="AE27" s="138"/>
-      <c r="AF27" s="138"/>
-      <c r="AG27" s="138"/>
-      <c r="AH27" s="138" t="s">
-        <v>326</v>
-      </c>
-      <c r="AI27" s="138"/>
-      <c r="AJ27" s="138"/>
-      <c r="AK27" s="138"/>
-      <c r="AL27" s="138"/>
-      <c r="AM27" s="138"/>
-      <c r="AN27" s="138"/>
-      <c r="AO27" s="138"/>
-      <c r="AP27" s="138"/>
-      <c r="AQ27" s="138"/>
-      <c r="AR27" s="138"/>
-      <c r="AS27" s="138"/>
-      <c r="AT27" s="138"/>
-      <c r="AU27" s="138"/>
-      <c r="AV27" s="138"/>
-      <c r="AW27" s="138"/>
-      <c r="AX27" s="138"/>
-      <c r="AY27" s="138"/>
-      <c r="AZ27" s="138"/>
-      <c r="BA27" s="138"/>
-      <c r="BB27" s="138"/>
-      <c r="BC27" s="138"/>
-      <c r="BD27" s="138"/>
-      <c r="BE27" s="138"/>
-      <c r="BF27" s="138"/>
-      <c r="BG27" s="138"/>
-      <c r="BH27" s="138"/>
-      <c r="BI27" s="138"/>
-      <c r="BJ27" s="138"/>
-      <c r="BK27" s="138"/>
-      <c r="BL27" s="138"/>
-      <c r="BM27" s="138"/>
-      <c r="BN27" s="138"/>
-      <c r="BO27" s="138"/>
-      <c r="BP27" s="138"/>
-      <c r="BQ27" s="138"/>
-      <c r="BR27" s="138"/>
-      <c r="BS27" s="138"/>
-      <c r="BT27" s="138"/>
-      <c r="BU27" s="138"/>
-      <c r="BV27" s="138"/>
-      <c r="BW27" s="138"/>
-      <c r="BX27" s="138"/>
-      <c r="BY27" s="138"/>
-      <c r="BZ27" s="138"/>
-      <c r="CA27" s="138"/>
-      <c r="CB27" s="138"/>
-      <c r="CC27" s="138"/>
-      <c r="CD27" s="138"/>
-      <c r="CE27" s="138"/>
-      <c r="CF27" s="138"/>
-      <c r="CG27" s="138"/>
-      <c r="CH27" s="138"/>
-      <c r="CI27" s="138"/>
-      <c r="CJ27" s="138"/>
-      <c r="CK27" s="138"/>
-      <c r="CL27" s="143"/>
-    </row>
-    <row r="28" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="133"/>
-      <c r="B28" s="129"/>
-      <c r="C28" s="129"/>
-      <c r="D28" s="129"/>
-      <c r="E28" s="129"/>
-      <c r="F28" s="134"/>
-      <c r="G28" s="142"/>
-      <c r="H28" s="138"/>
-      <c r="I28" s="138"/>
-      <c r="J28" s="138"/>
-      <c r="K28" s="138"/>
-      <c r="L28" s="138"/>
-      <c r="M28" s="138"/>
-      <c r="N28" s="138"/>
-      <c r="O28" s="138"/>
-      <c r="P28" s="138"/>
-      <c r="Q28" s="138"/>
-      <c r="R28" s="138"/>
-      <c r="S28" s="138"/>
-      <c r="T28" s="138"/>
-      <c r="U28" s="138"/>
-      <c r="V28" s="138"/>
-      <c r="W28" s="138"/>
-      <c r="X28" s="138"/>
-      <c r="Y28" s="138"/>
-      <c r="Z28" s="138"/>
-      <c r="AA28" s="138"/>
-      <c r="AB28" s="138"/>
-      <c r="AC28" s="138"/>
-      <c r="AD28" s="138"/>
-      <c r="AE28" s="138"/>
-      <c r="AF28" s="138"/>
-      <c r="AG28" s="138"/>
-      <c r="AH28" s="138"/>
-      <c r="AI28" s="138"/>
-      <c r="AJ28" s="138"/>
-      <c r="AK28" s="138"/>
-      <c r="AL28" s="138" t="s">
-        <v>128</v>
-      </c>
-      <c r="AM28" s="138"/>
-      <c r="AN28" s="138" t="s">
-        <v>327</v>
-      </c>
-      <c r="AO28" s="138"/>
-      <c r="AP28" s="138"/>
-      <c r="AQ28" s="138"/>
-      <c r="AR28" s="138"/>
-      <c r="AS28" s="138"/>
-      <c r="AT28" s="138"/>
-      <c r="AU28" s="138"/>
-      <c r="AV28" s="138"/>
-      <c r="AW28" s="138"/>
-      <c r="AX28" s="138"/>
-      <c r="AY28" s="138"/>
-      <c r="AZ28" s="138"/>
-      <c r="BA28" s="138"/>
-      <c r="BB28" s="138"/>
-      <c r="BC28" s="138"/>
-      <c r="BD28" s="138"/>
-      <c r="BE28" s="138"/>
-      <c r="BF28" s="138"/>
-      <c r="BG28" s="138"/>
-      <c r="BH28" s="138"/>
-      <c r="BI28" s="138"/>
-      <c r="BJ28" s="138"/>
-      <c r="BK28" s="138"/>
-      <c r="BL28" s="138"/>
-      <c r="BM28" s="138"/>
-      <c r="BN28" s="138"/>
-      <c r="BO28" s="138"/>
-      <c r="BP28" s="138"/>
-      <c r="BQ28" s="138"/>
-      <c r="BR28" s="138"/>
-      <c r="BS28" s="138"/>
-      <c r="BT28" s="138"/>
-      <c r="BU28" s="138"/>
-      <c r="BV28" s="138"/>
-      <c r="BW28" s="138"/>
-      <c r="BX28" s="138"/>
-      <c r="BY28" s="138"/>
-      <c r="BZ28" s="138"/>
-      <c r="CA28" s="138"/>
-      <c r="CB28" s="138"/>
-      <c r="CC28" s="138"/>
-      <c r="CD28" s="138"/>
-      <c r="CE28" s="138"/>
-      <c r="CF28" s="138"/>
-      <c r="CG28" s="138"/>
-      <c r="CH28" s="138"/>
-      <c r="CI28" s="138"/>
-      <c r="CJ28" s="138"/>
-      <c r="CK28" s="138"/>
-      <c r="CL28" s="143"/>
-    </row>
-    <row r="29" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="133"/>
-      <c r="B29" s="129"/>
-      <c r="C29" s="129"/>
-      <c r="D29" s="129"/>
-      <c r="E29" s="129"/>
-      <c r="F29" s="134"/>
-      <c r="G29" s="142"/>
-      <c r="H29" s="138"/>
-      <c r="I29" s="138"/>
-      <c r="J29" s="138"/>
-      <c r="K29" s="138"/>
-      <c r="L29" s="138"/>
-      <c r="M29" s="138"/>
-      <c r="N29" s="138"/>
-      <c r="O29" s="138"/>
-      <c r="P29" s="138"/>
-      <c r="Q29" s="138"/>
-      <c r="R29" s="138"/>
-      <c r="S29" s="138"/>
-      <c r="T29" s="138"/>
-      <c r="U29" s="138"/>
-      <c r="V29" s="138"/>
-      <c r="W29" s="138"/>
-      <c r="X29" s="138"/>
-      <c r="Y29" s="138"/>
-      <c r="Z29" s="138"/>
-      <c r="AA29" s="138"/>
-      <c r="AB29" s="138"/>
-      <c r="AC29" s="138"/>
-      <c r="AD29" s="138"/>
-      <c r="AE29" s="138"/>
-      <c r="AF29" s="138"/>
-      <c r="AG29" s="138"/>
-      <c r="AH29" s="138"/>
-      <c r="AI29" s="138"/>
-      <c r="AJ29" s="138" t="s">
-        <v>10</v>
-      </c>
-      <c r="AK29" s="138"/>
-      <c r="AL29" s="138"/>
-      <c r="AM29" s="138"/>
-      <c r="AN29" s="138" t="s">
-        <v>328</v>
-      </c>
-      <c r="AO29" s="138"/>
-      <c r="AP29" s="138"/>
-      <c r="AQ29" s="138"/>
-      <c r="AR29" s="138"/>
-      <c r="AS29" s="138"/>
-      <c r="AT29" s="138"/>
-      <c r="AU29" s="138"/>
-      <c r="AV29" s="138"/>
-      <c r="AW29" s="138"/>
-      <c r="AX29" s="138"/>
-      <c r="AY29" s="138"/>
-      <c r="AZ29" s="138"/>
-      <c r="BA29" s="138"/>
-      <c r="BB29" s="138"/>
-      <c r="BC29" s="138"/>
-      <c r="BD29" s="138"/>
-      <c r="BE29" s="138"/>
-      <c r="BF29" s="138"/>
-      <c r="BG29" s="138"/>
-      <c r="BH29" s="138"/>
-      <c r="BI29" s="138"/>
-      <c r="BJ29" s="138"/>
-      <c r="BK29" s="138"/>
-      <c r="BL29" s="138"/>
-      <c r="BM29" s="138"/>
-      <c r="BN29" s="138"/>
-      <c r="BO29" s="138"/>
-      <c r="BP29" s="138"/>
-      <c r="BQ29" s="138"/>
-      <c r="BR29" s="138"/>
-      <c r="BS29" s="138"/>
-      <c r="BT29" s="138"/>
-      <c r="BU29" s="138"/>
-      <c r="BV29" s="138"/>
-      <c r="BW29" s="138"/>
-      <c r="BX29" s="138"/>
-      <c r="BY29" s="138"/>
-      <c r="BZ29" s="138"/>
-      <c r="CA29" s="138"/>
-      <c r="CB29" s="138"/>
-      <c r="CC29" s="138"/>
-      <c r="CD29" s="138"/>
-      <c r="CE29" s="138"/>
-      <c r="CF29" s="138"/>
-      <c r="CG29" s="138"/>
-      <c r="CH29" s="138"/>
-      <c r="CI29" s="138"/>
-      <c r="CJ29" s="138"/>
-      <c r="CK29" s="138"/>
-      <c r="CL29" s="143"/>
-    </row>
-    <row r="30" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="133"/>
-      <c r="B30" s="129"/>
-      <c r="C30" s="129"/>
-      <c r="D30" s="129"/>
-      <c r="E30" s="129"/>
-      <c r="F30" s="134"/>
-      <c r="G30" s="142"/>
-      <c r="H30" s="138"/>
-      <c r="I30" s="138"/>
-      <c r="J30" s="138"/>
-      <c r="K30" s="138"/>
-      <c r="L30" s="138"/>
-      <c r="M30" s="138"/>
-      <c r="N30" s="138"/>
-      <c r="O30" s="138"/>
-      <c r="P30" s="138"/>
-      <c r="Q30" s="138"/>
-      <c r="R30" s="138"/>
-      <c r="S30" s="138"/>
-      <c r="T30" s="138"/>
-      <c r="U30" s="138"/>
-      <c r="V30" s="138"/>
-      <c r="W30" s="138"/>
-      <c r="X30" s="138"/>
-      <c r="Y30" s="138"/>
-      <c r="Z30" s="138"/>
-      <c r="AA30" s="138"/>
-      <c r="AB30" s="138"/>
-      <c r="AC30" s="138"/>
-      <c r="AD30" s="138"/>
-      <c r="AE30" s="138"/>
-      <c r="AF30" s="138"/>
-      <c r="AG30" s="138"/>
-      <c r="AH30" s="138"/>
-      <c r="AI30" s="138"/>
-      <c r="AJ30" s="138"/>
-      <c r="AK30" s="138"/>
-      <c r="AL30" s="138" t="s">
-        <v>128</v>
-      </c>
-      <c r="AM30" s="138"/>
-      <c r="AN30" s="138" t="s">
-        <v>329</v>
-      </c>
-      <c r="AO30" s="138"/>
-      <c r="AP30" s="138"/>
-      <c r="AQ30" s="138"/>
-      <c r="AR30" s="138"/>
-      <c r="AS30" s="138"/>
-      <c r="AT30" s="138"/>
-      <c r="AU30" s="138"/>
-      <c r="AV30" s="138"/>
-      <c r="AW30" s="138"/>
-      <c r="AX30" s="138"/>
-      <c r="AY30" s="138"/>
-      <c r="AZ30" s="138"/>
-      <c r="BA30" s="138"/>
-      <c r="BB30" s="138"/>
-      <c r="BC30" s="138"/>
-      <c r="BD30" s="138"/>
-      <c r="BE30" s="138"/>
-      <c r="BF30" s="138"/>
-      <c r="BG30" s="138"/>
-      <c r="BH30" s="138"/>
-      <c r="BI30" s="138"/>
-      <c r="BJ30" s="138"/>
-      <c r="BK30" s="138"/>
-      <c r="BL30" s="138"/>
-      <c r="BM30" s="138"/>
-      <c r="BN30" s="138"/>
-      <c r="BO30" s="138"/>
-      <c r="BP30" s="138"/>
-      <c r="BQ30" s="138"/>
-      <c r="BR30" s="138"/>
-      <c r="BS30" s="138"/>
-      <c r="BT30" s="138"/>
-      <c r="BU30" s="138"/>
-      <c r="BV30" s="138"/>
-      <c r="BW30" s="138"/>
-      <c r="BX30" s="138"/>
-      <c r="BY30" s="138"/>
-      <c r="BZ30" s="138"/>
-      <c r="CA30" s="138"/>
-      <c r="CB30" s="138"/>
-      <c r="CC30" s="138"/>
-      <c r="CD30" s="138"/>
-      <c r="CE30" s="138"/>
-      <c r="CF30" s="138"/>
-      <c r="CG30" s="138"/>
-      <c r="CH30" s="138"/>
-      <c r="CI30" s="138"/>
-      <c r="CJ30" s="138"/>
-      <c r="CK30" s="138"/>
-      <c r="CL30" s="143"/>
-    </row>
-    <row r="31" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A31" s="135"/>
-      <c r="B31" s="136"/>
-      <c r="C31" s="136"/>
-      <c r="D31" s="136"/>
-      <c r="E31" s="136"/>
-      <c r="F31" s="137"/>
-      <c r="G31" s="144"/>
-      <c r="H31" s="145"/>
-      <c r="I31" s="145"/>
-      <c r="J31" s="145"/>
-      <c r="K31" s="145"/>
-      <c r="L31" s="145"/>
-      <c r="M31" s="145"/>
-      <c r="N31" s="145"/>
-      <c r="O31" s="145"/>
-      <c r="P31" s="145"/>
-      <c r="Q31" s="145"/>
-      <c r="R31" s="145"/>
-      <c r="S31" s="145"/>
-      <c r="T31" s="145"/>
-      <c r="U31" s="145"/>
-      <c r="V31" s="145"/>
-      <c r="W31" s="145"/>
-      <c r="X31" s="145"/>
-      <c r="Y31" s="145"/>
-      <c r="Z31" s="145"/>
-      <c r="AA31" s="145"/>
-      <c r="AB31" s="145"/>
-      <c r="AC31" s="145"/>
-      <c r="AD31" s="145"/>
-      <c r="AE31" s="145"/>
-      <c r="AF31" s="145"/>
-      <c r="AG31" s="145"/>
-      <c r="AH31" s="145"/>
-      <c r="AI31" s="145"/>
-      <c r="AJ31" s="145" t="s">
-        <v>305</v>
-      </c>
-      <c r="AK31" s="145"/>
-      <c r="AL31" s="145"/>
-      <c r="AM31" s="145"/>
-      <c r="AN31" s="145"/>
-      <c r="AO31" s="145"/>
-      <c r="AP31" s="145"/>
-      <c r="AQ31" s="145"/>
-      <c r="AR31" s="145"/>
-      <c r="AS31" s="145"/>
-      <c r="AT31" s="145"/>
-      <c r="AU31" s="145"/>
-      <c r="AV31" s="145"/>
-      <c r="AW31" s="145"/>
-      <c r="AX31" s="145"/>
-      <c r="AY31" s="145"/>
-      <c r="AZ31" s="145"/>
-      <c r="BA31" s="145"/>
-      <c r="BB31" s="145"/>
-      <c r="BC31" s="145"/>
-      <c r="BD31" s="145"/>
-      <c r="BE31" s="145"/>
-      <c r="BF31" s="145"/>
-      <c r="BG31" s="145"/>
-      <c r="BH31" s="145"/>
-      <c r="BI31" s="145"/>
-      <c r="BJ31" s="145"/>
-      <c r="BK31" s="145"/>
-      <c r="BL31" s="145"/>
-      <c r="BM31" s="145"/>
-      <c r="BN31" s="145"/>
-      <c r="BO31" s="145"/>
-      <c r="BP31" s="145"/>
-      <c r="BQ31" s="145"/>
-      <c r="BR31" s="145"/>
-      <c r="BS31" s="145"/>
-      <c r="BT31" s="145"/>
-      <c r="BU31" s="145"/>
-      <c r="BV31" s="145"/>
-      <c r="BW31" s="145"/>
-      <c r="BX31" s="145"/>
-      <c r="BY31" s="145"/>
-      <c r="BZ31" s="145"/>
-      <c r="CA31" s="145"/>
-      <c r="CB31" s="145"/>
-      <c r="CC31" s="145"/>
-      <c r="CD31" s="145"/>
-      <c r="CE31" s="145"/>
-      <c r="CF31" s="145"/>
-      <c r="CG31" s="145"/>
-      <c r="CH31" s="145"/>
-      <c r="CI31" s="145"/>
-      <c r="CJ31" s="145"/>
-      <c r="CK31" s="145"/>
-      <c r="CL31" s="146"/>
+      <c r="AI12" s="147"/>
+      <c r="AJ12" s="147"/>
+      <c r="AK12" s="147"/>
+      <c r="AL12" s="147"/>
+      <c r="AM12" s="147"/>
+      <c r="AN12" s="147"/>
+      <c r="AO12" s="147"/>
+      <c r="AP12" s="147"/>
+      <c r="AQ12" s="147"/>
+      <c r="AR12" s="147"/>
+      <c r="AS12" s="147"/>
+      <c r="AT12" s="147"/>
+      <c r="AU12" s="147"/>
+      <c r="AV12" s="147"/>
+      <c r="AW12" s="147"/>
+      <c r="AX12" s="147"/>
+      <c r="AY12" s="147"/>
+      <c r="AZ12" s="147"/>
+      <c r="BA12" s="147"/>
+      <c r="BB12" s="147"/>
+      <c r="BC12" s="147"/>
+      <c r="BD12" s="147"/>
+      <c r="BE12" s="147"/>
+      <c r="BF12" s="147"/>
+      <c r="BG12" s="147"/>
+      <c r="BH12" s="147"/>
+      <c r="BI12" s="147"/>
+      <c r="BJ12" s="147"/>
+      <c r="BK12" s="147"/>
+      <c r="BL12" s="147"/>
+      <c r="BM12" s="147"/>
+      <c r="BN12" s="147"/>
+      <c r="BO12" s="147"/>
+      <c r="BP12" s="147"/>
+      <c r="BQ12" s="147"/>
+      <c r="BR12" s="147"/>
+      <c r="BS12" s="147"/>
+      <c r="BT12" s="147"/>
+      <c r="BU12" s="147"/>
+      <c r="BV12" s="147"/>
+      <c r="BW12" s="147"/>
+      <c r="BX12" s="147"/>
+      <c r="BY12" s="147"/>
+      <c r="BZ12" s="147"/>
+      <c r="CA12" s="147"/>
+      <c r="CB12" s="147"/>
+      <c r="CC12" s="147"/>
+      <c r="CD12" s="147"/>
+      <c r="CE12" s="147"/>
+      <c r="CF12" s="147"/>
+      <c r="CG12" s="147"/>
+      <c r="CH12" s="147"/>
+      <c r="CI12" s="147"/>
+      <c r="CJ12" s="147"/>
+      <c r="CK12" s="147"/>
+      <c r="CL12" s="148"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>

</xml_diff>

<commit_message>
test: refine SEL-082 provisional CASE layout
</commit_message>
<xml_diff>
--- a/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
+++ b/tests/SqlAnalysisFormatter.OutputExpectations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Macro\SqlAnalyzerFormatter\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{446614F3-D109-470D-9E37-CC1D8EBE18FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73084267-F110-4D6C-89E3-48B050EFE2C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-8340" windowWidth="29040" windowHeight="15720" firstSheet="71" activeTab="81" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-8340" windowWidth="29040" windowHeight="15720" firstSheet="61" activeTab="81" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SEL-001" sheetId="1" r:id="rId1"/>
@@ -101,7 +101,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1431" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1437" uniqueCount="320">
   <si>
     <t>＜DB入出力項目定義＞</t>
   </si>
@@ -1027,28 +1027,40 @@
     <t>tb1.状態 = 'PENDING')</t>
   </si>
   <si>
-    <t>tb1.削除日時 IS NULL) → (tb1.ランクコード = 'VIP'</t>
+    <t>tb1.削除日時 IS NULL)</t>
+  </si>
+  <si>
+    <t>→ (tb1.ランクコード = 'VIP'</t>
   </si>
   <si>
     <t>(tb1.評価点 &gt;= 90</t>
   </si>
   <si>
-    <t>tb1.優先フラグ = 1)) → 'ACTIVE_PRIORITY'</t>
+    <t>tb1.優先フラグ = 1))</t>
   </si>
   <si>
-    <t>ELSE → 'ACTIVE_STANDARD'</t>
+    <t>→ 'ACTIVE_PRIORITY'</t>
   </si>
   <si>
-    <t>ELSE → ((tb1.状態 = 'LOCKED'</t>
+    <t>ELSE</t>
+  </si>
+  <si>
+    <t>→ 'ACTIVE_STANDARD'</t>
+  </si>
+  <si>
+    <t>→ ((tb1.状態 = 'LOCKED'</t>
   </si>
   <si>
     <t>tb1.状態 = 'INACTIVE')</t>
   </si>
   <si>
-    <t>tb1.削除日時 IS NOT NULL) → 'INACTIVE_DELETED'</t>
+    <t>tb1.削除日時 IS NOT NULL)</t>
   </si>
   <si>
-    <t>ELSE → 'OTHER'</t>
+    <t>→ 'INACTIVE_DELETED'</t>
+  </si>
+  <si>
+    <t>→ 'OTHER'</t>
   </si>
 </sst>
 </file>
@@ -61416,7 +61428,7 @@
 
 <file path=xl/worksheets/sheet82.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-5100-000000000000}">
-  <dimension ref="A1:CL12"/>
+  <dimension ref="A1:CL15"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="90" width="1.75" customWidth="1"/>
@@ -61652,13 +61664,13 @@
       <c r="AE3" s="142" t="s">
         <v>33</v>
       </c>
-      <c r="AF3" s="142"/>
+      <c r="AF3" s="142" t="s">
+        <v>306</v>
+      </c>
       <c r="AG3" s="142"/>
       <c r="AH3" s="142"/>
       <c r="AI3" s="142"/>
-      <c r="AJ3" s="142" t="s">
-        <v>306</v>
-      </c>
+      <c r="AJ3" s="142"/>
       <c r="AK3" s="142"/>
       <c r="AL3" s="142"/>
       <c r="AM3" s="142"/>
@@ -61746,15 +61758,15 @@
       <c r="AC4" s="140"/>
       <c r="AD4" s="140"/>
       <c r="AE4" s="140"/>
-      <c r="AF4" s="140"/>
+      <c r="AF4" s="140" t="s">
+        <v>128</v>
+      </c>
       <c r="AG4" s="140"/>
       <c r="AH4" s="140" t="s">
-        <v>128</v>
+        <v>307</v>
       </c>
       <c r="AI4" s="140"/>
-      <c r="AJ4" s="140" t="s">
-        <v>307</v>
-      </c>
+      <c r="AJ4" s="140"/>
       <c r="AK4" s="140"/>
       <c r="AL4" s="140"/>
       <c r="AM4" s="140"/>
@@ -61940,17 +61952,15 @@
       <c r="AE6" s="140"/>
       <c r="AF6" s="140"/>
       <c r="AG6" s="140"/>
-      <c r="AH6" s="140"/>
+      <c r="AH6" s="140" t="s">
+        <v>309</v>
+      </c>
       <c r="AI6" s="140"/>
-      <c r="AJ6" s="140" t="s">
-        <v>10</v>
-      </c>
+      <c r="AJ6" s="140"/>
       <c r="AK6" s="140"/>
       <c r="AL6" s="140"/>
       <c r="AM6" s="140"/>
-      <c r="AN6" s="140" t="s">
-        <v>309</v>
-      </c>
+      <c r="AN6" s="140"/>
       <c r="AO6" s="140"/>
       <c r="AP6" s="140"/>
       <c r="AQ6" s="140"/>
@@ -62038,15 +62048,15 @@
       <c r="AG7" s="140"/>
       <c r="AH7" s="140"/>
       <c r="AI7" s="140"/>
-      <c r="AJ7" s="140"/>
+      <c r="AJ7" s="140" t="s">
+        <v>10</v>
+      </c>
       <c r="AK7" s="140"/>
       <c r="AL7" s="140" t="s">
-        <v>128</v>
+        <v>310</v>
       </c>
       <c r="AM7" s="140"/>
-      <c r="AN7" s="140" t="s">
-        <v>310</v>
-      </c>
+      <c r="AN7" s="140"/>
       <c r="AO7" s="140"/>
       <c r="AP7" s="140"/>
       <c r="AQ7" s="140"/>
@@ -62134,13 +62144,15 @@
       <c r="AG8" s="140"/>
       <c r="AH8" s="140"/>
       <c r="AI8" s="140"/>
-      <c r="AJ8" s="140" t="s">
+      <c r="AJ8" s="140"/>
+      <c r="AK8" s="140"/>
+      <c r="AL8" s="140" t="s">
+        <v>128</v>
+      </c>
+      <c r="AM8" s="140"/>
+      <c r="AN8" s="140" t="s">
         <v>311</v>
       </c>
-      <c r="AK8" s="140"/>
-      <c r="AL8" s="140"/>
-      <c r="AM8" s="140"/>
-      <c r="AN8" s="140"/>
       <c r="AO8" s="140"/>
       <c r="AP8" s="140"/>
       <c r="AQ8" s="140"/>
@@ -62224,15 +62236,15 @@
       <c r="AC9" s="140"/>
       <c r="AD9" s="140"/>
       <c r="AE9" s="140"/>
-      <c r="AF9" s="140" t="s">
-        <v>312</v>
-      </c>
+      <c r="AF9" s="140"/>
       <c r="AG9" s="140"/>
       <c r="AH9" s="140"/>
       <c r="AI9" s="140"/>
       <c r="AJ9" s="140"/>
       <c r="AK9" s="140"/>
-      <c r="AL9" s="140"/>
+      <c r="AL9" s="140" t="s">
+        <v>312</v>
+      </c>
       <c r="AM9" s="140"/>
       <c r="AN9" s="140"/>
       <c r="AO9" s="140"/>
@@ -62323,11 +62335,11 @@
       <c r="AH10" s="140"/>
       <c r="AI10" s="140"/>
       <c r="AJ10" s="140" t="s">
-        <v>128</v>
+        <v>313</v>
       </c>
       <c r="AK10" s="140"/>
       <c r="AL10" s="140" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="AM10" s="140"/>
       <c r="AN10" s="140"/>
@@ -62414,15 +62426,15 @@
       <c r="AC11" s="140"/>
       <c r="AD11" s="140"/>
       <c r="AE11" s="140"/>
-      <c r="AF11" s="140"/>
+      <c r="AF11" s="140" t="s">
+        <v>313</v>
+      </c>
       <c r="AG11" s="140"/>
       <c r="AH11" s="140" t="s">
-        <v>10</v>
+        <v>315</v>
       </c>
       <c r="AI11" s="140"/>
-      <c r="AJ11" s="140" t="s">
-        <v>314</v>
-      </c>
+      <c r="AJ11" s="140"/>
       <c r="AK11" s="140"/>
       <c r="AL11" s="140"/>
       <c r="AM11" s="140"/>
@@ -62479,98 +62491,386 @@
       <c r="CL11" s="145"/>
     </row>
     <row r="12" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="137"/>
-      <c r="B12" s="138"/>
-      <c r="C12" s="138"/>
-      <c r="D12" s="138"/>
-      <c r="E12" s="138"/>
-      <c r="F12" s="139"/>
-      <c r="G12" s="146"/>
-      <c r="H12" s="147"/>
-      <c r="I12" s="147"/>
-      <c r="J12" s="147"/>
-      <c r="K12" s="147"/>
-      <c r="L12" s="147"/>
-      <c r="M12" s="147"/>
-      <c r="N12" s="147"/>
-      <c r="O12" s="147"/>
-      <c r="P12" s="147"/>
-      <c r="Q12" s="147"/>
-      <c r="R12" s="147"/>
-      <c r="S12" s="147"/>
-      <c r="T12" s="147"/>
-      <c r="U12" s="147"/>
-      <c r="V12" s="147"/>
-      <c r="W12" s="147"/>
-      <c r="X12" s="147"/>
-      <c r="Y12" s="147"/>
-      <c r="Z12" s="147"/>
-      <c r="AA12" s="147"/>
-      <c r="AB12" s="147"/>
-      <c r="AC12" s="147"/>
-      <c r="AD12" s="147"/>
-      <c r="AE12" s="147"/>
-      <c r="AF12" s="147"/>
-      <c r="AG12" s="147"/>
-      <c r="AH12" s="147" t="s">
-        <v>315</v>
-      </c>
-      <c r="AI12" s="147"/>
-      <c r="AJ12" s="147"/>
-      <c r="AK12" s="147"/>
-      <c r="AL12" s="147"/>
-      <c r="AM12" s="147"/>
-      <c r="AN12" s="147"/>
-      <c r="AO12" s="147"/>
-      <c r="AP12" s="147"/>
-      <c r="AQ12" s="147"/>
-      <c r="AR12" s="147"/>
-      <c r="AS12" s="147"/>
-      <c r="AT12" s="147"/>
-      <c r="AU12" s="147"/>
-      <c r="AV12" s="147"/>
-      <c r="AW12" s="147"/>
-      <c r="AX12" s="147"/>
-      <c r="AY12" s="147"/>
-      <c r="AZ12" s="147"/>
-      <c r="BA12" s="147"/>
-      <c r="BB12" s="147"/>
-      <c r="BC12" s="147"/>
-      <c r="BD12" s="147"/>
-      <c r="BE12" s="147"/>
-      <c r="BF12" s="147"/>
-      <c r="BG12" s="147"/>
-      <c r="BH12" s="147"/>
-      <c r="BI12" s="147"/>
-      <c r="BJ12" s="147"/>
-      <c r="BK12" s="147"/>
-      <c r="BL12" s="147"/>
-      <c r="BM12" s="147"/>
-      <c r="BN12" s="147"/>
-      <c r="BO12" s="147"/>
-      <c r="BP12" s="147"/>
-      <c r="BQ12" s="147"/>
-      <c r="BR12" s="147"/>
-      <c r="BS12" s="147"/>
-      <c r="BT12" s="147"/>
-      <c r="BU12" s="147"/>
-      <c r="BV12" s="147"/>
-      <c r="BW12" s="147"/>
-      <c r="BX12" s="147"/>
-      <c r="BY12" s="147"/>
-      <c r="BZ12" s="147"/>
-      <c r="CA12" s="147"/>
-      <c r="CB12" s="147"/>
-      <c r="CC12" s="147"/>
-      <c r="CD12" s="147"/>
-      <c r="CE12" s="147"/>
-      <c r="CF12" s="147"/>
-      <c r="CG12" s="147"/>
-      <c r="CH12" s="147"/>
-      <c r="CI12" s="147"/>
-      <c r="CJ12" s="147"/>
-      <c r="CK12" s="147"/>
-      <c r="CL12" s="148"/>
+      <c r="A12" s="135"/>
+      <c r="B12" s="131"/>
+      <c r="C12" s="131"/>
+      <c r="D12" s="131"/>
+      <c r="E12" s="131"/>
+      <c r="F12" s="136"/>
+      <c r="G12" s="144"/>
+      <c r="H12" s="140"/>
+      <c r="I12" s="140"/>
+      <c r="J12" s="140"/>
+      <c r="K12" s="140"/>
+      <c r="L12" s="140"/>
+      <c r="M12" s="140"/>
+      <c r="N12" s="140"/>
+      <c r="O12" s="140"/>
+      <c r="P12" s="140"/>
+      <c r="Q12" s="140"/>
+      <c r="R12" s="140"/>
+      <c r="S12" s="140"/>
+      <c r="T12" s="140"/>
+      <c r="U12" s="140"/>
+      <c r="V12" s="140"/>
+      <c r="W12" s="140"/>
+      <c r="X12" s="140"/>
+      <c r="Y12" s="140"/>
+      <c r="Z12" s="140"/>
+      <c r="AA12" s="140"/>
+      <c r="AB12" s="140"/>
+      <c r="AC12" s="140"/>
+      <c r="AD12" s="140"/>
+      <c r="AE12" s="140"/>
+      <c r="AF12" s="140"/>
+      <c r="AG12" s="140"/>
+      <c r="AH12" s="140" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI12" s="140"/>
+      <c r="AJ12" s="140" t="s">
+        <v>316</v>
+      </c>
+      <c r="AK12" s="140"/>
+      <c r="AL12" s="140"/>
+      <c r="AM12" s="140"/>
+      <c r="AN12" s="140"/>
+      <c r="AO12" s="140"/>
+      <c r="AP12" s="140"/>
+      <c r="AQ12" s="140"/>
+      <c r="AR12" s="140"/>
+      <c r="AS12" s="140"/>
+      <c r="AT12" s="140"/>
+      <c r="AU12" s="140"/>
+      <c r="AV12" s="140"/>
+      <c r="AW12" s="140"/>
+      <c r="AX12" s="140"/>
+      <c r="AY12" s="140"/>
+      <c r="AZ12" s="140"/>
+      <c r="BA12" s="140"/>
+      <c r="BB12" s="140"/>
+      <c r="BC12" s="140"/>
+      <c r="BD12" s="140"/>
+      <c r="BE12" s="140"/>
+      <c r="BF12" s="140"/>
+      <c r="BG12" s="140"/>
+      <c r="BH12" s="140"/>
+      <c r="BI12" s="140"/>
+      <c r="BJ12" s="140"/>
+      <c r="BK12" s="140"/>
+      <c r="BL12" s="140"/>
+      <c r="BM12" s="140"/>
+      <c r="BN12" s="140"/>
+      <c r="BO12" s="140"/>
+      <c r="BP12" s="140"/>
+      <c r="BQ12" s="140"/>
+      <c r="BR12" s="140"/>
+      <c r="BS12" s="140"/>
+      <c r="BT12" s="140"/>
+      <c r="BU12" s="140"/>
+      <c r="BV12" s="140"/>
+      <c r="BW12" s="140"/>
+      <c r="BX12" s="140"/>
+      <c r="BY12" s="140"/>
+      <c r="BZ12" s="140"/>
+      <c r="CA12" s="140"/>
+      <c r="CB12" s="140"/>
+      <c r="CC12" s="140"/>
+      <c r="CD12" s="140"/>
+      <c r="CE12" s="140"/>
+      <c r="CF12" s="140"/>
+      <c r="CG12" s="140"/>
+      <c r="CH12" s="140"/>
+      <c r="CI12" s="140"/>
+      <c r="CJ12" s="140"/>
+      <c r="CK12" s="140"/>
+      <c r="CL12" s="145"/>
+    </row>
+    <row r="13" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="135"/>
+      <c r="B13" s="131"/>
+      <c r="C13" s="131"/>
+      <c r="D13" s="131"/>
+      <c r="E13" s="131"/>
+      <c r="F13" s="136"/>
+      <c r="G13" s="144"/>
+      <c r="H13" s="140"/>
+      <c r="I13" s="140"/>
+      <c r="J13" s="140"/>
+      <c r="K13" s="140"/>
+      <c r="L13" s="140"/>
+      <c r="M13" s="140"/>
+      <c r="N13" s="140"/>
+      <c r="O13" s="140"/>
+      <c r="P13" s="140"/>
+      <c r="Q13" s="140"/>
+      <c r="R13" s="140"/>
+      <c r="S13" s="140"/>
+      <c r="T13" s="140"/>
+      <c r="U13" s="140"/>
+      <c r="V13" s="140"/>
+      <c r="W13" s="140"/>
+      <c r="X13" s="140"/>
+      <c r="Y13" s="140"/>
+      <c r="Z13" s="140"/>
+      <c r="AA13" s="140"/>
+      <c r="AB13" s="140"/>
+      <c r="AC13" s="140"/>
+      <c r="AD13" s="140"/>
+      <c r="AE13" s="140"/>
+      <c r="AF13" s="140"/>
+      <c r="AG13" s="140"/>
+      <c r="AH13" s="140"/>
+      <c r="AI13" s="140"/>
+      <c r="AJ13" s="140" t="s">
+        <v>10</v>
+      </c>
+      <c r="AK13" s="140"/>
+      <c r="AL13" s="140" t="s">
+        <v>317</v>
+      </c>
+      <c r="AM13" s="140"/>
+      <c r="AN13" s="140"/>
+      <c r="AO13" s="140"/>
+      <c r="AP13" s="140"/>
+      <c r="AQ13" s="140"/>
+      <c r="AR13" s="140"/>
+      <c r="AS13" s="140"/>
+      <c r="AT13" s="140"/>
+      <c r="AU13" s="140"/>
+      <c r="AV13" s="140"/>
+      <c r="AW13" s="140"/>
+      <c r="AX13" s="140"/>
+      <c r="AY13" s="140"/>
+      <c r="AZ13" s="140"/>
+      <c r="BA13" s="140"/>
+      <c r="BB13" s="140"/>
+      <c r="BC13" s="140"/>
+      <c r="BD13" s="140"/>
+      <c r="BE13" s="140"/>
+      <c r="BF13" s="140"/>
+      <c r="BG13" s="140"/>
+      <c r="BH13" s="140"/>
+      <c r="BI13" s="140"/>
+      <c r="BJ13" s="140"/>
+      <c r="BK13" s="140"/>
+      <c r="BL13" s="140"/>
+      <c r="BM13" s="140"/>
+      <c r="BN13" s="140"/>
+      <c r="BO13" s="140"/>
+      <c r="BP13" s="140"/>
+      <c r="BQ13" s="140"/>
+      <c r="BR13" s="140"/>
+      <c r="BS13" s="140"/>
+      <c r="BT13" s="140"/>
+      <c r="BU13" s="140"/>
+      <c r="BV13" s="140"/>
+      <c r="BW13" s="140"/>
+      <c r="BX13" s="140"/>
+      <c r="BY13" s="140"/>
+      <c r="BZ13" s="140"/>
+      <c r="CA13" s="140"/>
+      <c r="CB13" s="140"/>
+      <c r="CC13" s="140"/>
+      <c r="CD13" s="140"/>
+      <c r="CE13" s="140"/>
+      <c r="CF13" s="140"/>
+      <c r="CG13" s="140"/>
+      <c r="CH13" s="140"/>
+      <c r="CI13" s="140"/>
+      <c r="CJ13" s="140"/>
+      <c r="CK13" s="140"/>
+      <c r="CL13" s="145"/>
+    </row>
+    <row r="14" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="135"/>
+      <c r="B14" s="131"/>
+      <c r="C14" s="131"/>
+      <c r="D14" s="131"/>
+      <c r="E14" s="131"/>
+      <c r="F14" s="136"/>
+      <c r="G14" s="144"/>
+      <c r="H14" s="140"/>
+      <c r="I14" s="140"/>
+      <c r="J14" s="140"/>
+      <c r="K14" s="140"/>
+      <c r="L14" s="140"/>
+      <c r="M14" s="140"/>
+      <c r="N14" s="140"/>
+      <c r="O14" s="140"/>
+      <c r="P14" s="140"/>
+      <c r="Q14" s="140"/>
+      <c r="R14" s="140"/>
+      <c r="S14" s="140"/>
+      <c r="T14" s="140"/>
+      <c r="U14" s="140"/>
+      <c r="V14" s="140"/>
+      <c r="W14" s="140"/>
+      <c r="X14" s="140"/>
+      <c r="Y14" s="140"/>
+      <c r="Z14" s="140"/>
+      <c r="AA14" s="140"/>
+      <c r="AB14" s="140"/>
+      <c r="AC14" s="140"/>
+      <c r="AD14" s="140"/>
+      <c r="AE14" s="140"/>
+      <c r="AF14" s="140"/>
+      <c r="AG14" s="140"/>
+      <c r="AH14" s="140"/>
+      <c r="AI14" s="140"/>
+      <c r="AJ14" s="140"/>
+      <c r="AK14" s="140"/>
+      <c r="AL14" s="140" t="s">
+        <v>318</v>
+      </c>
+      <c r="AM14" s="140"/>
+      <c r="AN14" s="140"/>
+      <c r="AO14" s="140"/>
+      <c r="AP14" s="140"/>
+      <c r="AQ14" s="140"/>
+      <c r="AR14" s="140"/>
+      <c r="AS14" s="140"/>
+      <c r="AT14" s="140"/>
+      <c r="AU14" s="140"/>
+      <c r="AV14" s="140"/>
+      <c r="AW14" s="140"/>
+      <c r="AX14" s="140"/>
+      <c r="AY14" s="140"/>
+      <c r="AZ14" s="140"/>
+      <c r="BA14" s="140"/>
+      <c r="BB14" s="140"/>
+      <c r="BC14" s="140"/>
+      <c r="BD14" s="140"/>
+      <c r="BE14" s="140"/>
+      <c r="BF14" s="140"/>
+      <c r="BG14" s="140"/>
+      <c r="BH14" s="140"/>
+      <c r="BI14" s="140"/>
+      <c r="BJ14" s="140"/>
+      <c r="BK14" s="140"/>
+      <c r="BL14" s="140"/>
+      <c r="BM14" s="140"/>
+      <c r="BN14" s="140"/>
+      <c r="BO14" s="140"/>
+      <c r="BP14" s="140"/>
+      <c r="BQ14" s="140"/>
+      <c r="BR14" s="140"/>
+      <c r="BS14" s="140"/>
+      <c r="BT14" s="140"/>
+      <c r="BU14" s="140"/>
+      <c r="BV14" s="140"/>
+      <c r="BW14" s="140"/>
+      <c r="BX14" s="140"/>
+      <c r="BY14" s="140"/>
+      <c r="BZ14" s="140"/>
+      <c r="CA14" s="140"/>
+      <c r="CB14" s="140"/>
+      <c r="CC14" s="140"/>
+      <c r="CD14" s="140"/>
+      <c r="CE14" s="140"/>
+      <c r="CF14" s="140"/>
+      <c r="CG14" s="140"/>
+      <c r="CH14" s="140"/>
+      <c r="CI14" s="140"/>
+      <c r="CJ14" s="140"/>
+      <c r="CK14" s="140"/>
+      <c r="CL14" s="145"/>
+    </row>
+    <row r="15" spans="1:90" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="137"/>
+      <c r="B15" s="138"/>
+      <c r="C15" s="138"/>
+      <c r="D15" s="138"/>
+      <c r="E15" s="138"/>
+      <c r="F15" s="139"/>
+      <c r="G15" s="146"/>
+      <c r="H15" s="147"/>
+      <c r="I15" s="147"/>
+      <c r="J15" s="147"/>
+      <c r="K15" s="147"/>
+      <c r="L15" s="147"/>
+      <c r="M15" s="147"/>
+      <c r="N15" s="147"/>
+      <c r="O15" s="147"/>
+      <c r="P15" s="147"/>
+      <c r="Q15" s="147"/>
+      <c r="R15" s="147"/>
+      <c r="S15" s="147"/>
+      <c r="T15" s="147"/>
+      <c r="U15" s="147"/>
+      <c r="V15" s="147"/>
+      <c r="W15" s="147"/>
+      <c r="X15" s="147"/>
+      <c r="Y15" s="147"/>
+      <c r="Z15" s="147"/>
+      <c r="AA15" s="147"/>
+      <c r="AB15" s="147"/>
+      <c r="AC15" s="147"/>
+      <c r="AD15" s="147"/>
+      <c r="AE15" s="147"/>
+      <c r="AF15" s="147"/>
+      <c r="AG15" s="147"/>
+      <c r="AH15" s="147"/>
+      <c r="AI15" s="147"/>
+      <c r="AJ15" s="147" t="s">
+        <v>313</v>
+      </c>
+      <c r="AK15" s="147"/>
+      <c r="AL15" s="147" t="s">
+        <v>319</v>
+      </c>
+      <c r="AM15" s="147"/>
+      <c r="AN15" s="147"/>
+      <c r="AO15" s="147"/>
+      <c r="AP15" s="147"/>
+      <c r="AQ15" s="147"/>
+      <c r="AR15" s="147"/>
+      <c r="AS15" s="147"/>
+      <c r="AT15" s="147"/>
+      <c r="AU15" s="147"/>
+      <c r="AV15" s="147"/>
+      <c r="AW15" s="147"/>
+      <c r="AX15" s="147"/>
+      <c r="AY15" s="147"/>
+      <c r="AZ15" s="147"/>
+      <c r="BA15" s="147"/>
+      <c r="BB15" s="147"/>
+      <c r="BC15" s="147"/>
+      <c r="BD15" s="147"/>
+      <c r="BE15" s="147"/>
+      <c r="BF15" s="147"/>
+      <c r="BG15" s="147"/>
+      <c r="BH15" s="147"/>
+      <c r="BI15" s="147"/>
+      <c r="BJ15" s="147"/>
+      <c r="BK15" s="147"/>
+      <c r="BL15" s="147"/>
+      <c r="BM15" s="147"/>
+      <c r="BN15" s="147"/>
+      <c r="BO15" s="147"/>
+      <c r="BP15" s="147"/>
+      <c r="BQ15" s="147"/>
+      <c r="BR15" s="147"/>
+      <c r="BS15" s="147"/>
+      <c r="BT15" s="147"/>
+      <c r="BU15" s="147"/>
+      <c r="BV15" s="147"/>
+      <c r="BW15" s="147"/>
+      <c r="BX15" s="147"/>
+      <c r="BY15" s="147"/>
+      <c r="BZ15" s="147"/>
+      <c r="CA15" s="147"/>
+      <c r="CB15" s="147"/>
+      <c r="CC15" s="147"/>
+      <c r="CD15" s="147"/>
+      <c r="CE15" s="147"/>
+      <c r="CF15" s="147"/>
+      <c r="CG15" s="147"/>
+      <c r="CH15" s="147"/>
+      <c r="CI15" s="147"/>
+      <c r="CJ15" s="147"/>
+      <c r="CK15" s="147"/>
+      <c r="CL15" s="148"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>

</xml_diff>